<commit_message>
vault backup: 2026-09-23 22:04:29
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Literature Survey Matrix.xlsx
+++ b/FYP/Matrices/Literature Survey Matrix.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Survey'!$A$1:$W$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Literature Survey'!$A$1:$W$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -53,7 +53,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF3FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -119,16 +124,22 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,35 +507,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:W26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
     <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="36" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="36" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
-    <col width="60" customWidth="1" min="19" max="19"/>
-    <col width="50" customWidth="1" min="20" max="20"/>
-    <col width="60" customWidth="1" min="21" max="21"/>
-    <col width="48" customWidth="1" min="22" max="22"/>
-    <col width="40" customWidth="1" min="23" max="23"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="38" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="62" customWidth="1" min="19" max="19"/>
+    <col width="54" customWidth="1" min="20" max="20"/>
+    <col width="62" customWidth="1" min="21" max="21"/>
+    <col width="52" customWidth="1" min="22" max="22"/>
+    <col width="42" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="45" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
@@ -876,234 +887,234 @@
       </c>
     </row>
     <row r="4" ht="150" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Park, T. (Bank for International Settlements)</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>arXiv preprint</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>arXiv:2403.19735 | https://arxiv.org/abs/2403.19735</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>LLM multi-agent financial market monitoring</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Statistical anomaly alerts on market data still need a human to interpret and validate them. Uses a team of LLM agents to do that validation and write the explanation.</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>US, S&amp;P 500 index level.</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>S&amp;P 500 daily index series, 1980-2023.</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Tabular market data serialised for LLM consumption, plus live web research pulled in by one of the agents.</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Collaborative agent network. Output is a consolidated validation report on a flagged anomaly, not a trade.</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>Data Conversion agent (serialises tables), Expert Analyst agent (web research), Institutional Knowledge agent, Report Consolidation agent.</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>None as a modelled signal - the Expert Analyst agent pulls news context to explain a move after the fact.</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="O4" s="7" t="inlineStr">
         <is>
           <t>Rule-based z-score anomaly triggers, then agent validation. No conditional variance model.</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
+      <c r="P4" s="7" t="inlineStr">
         <is>
           <t>None.</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
+      <c r="Q4" s="7" t="inlineStr">
         <is>
           <t>The whole output is an explanation - the consolidated report is the deliverable, which is the opposite emphasis from most of these papers.</t>
         </is>
       </c>
-      <c r="R4" s="9" t="inlineStr">
+      <c r="R4" s="7" t="inlineStr">
         <is>
           <t>No detection-accuracy metric reported. Validated against known historical outliers.</t>
         </is>
       </c>
-      <c r="S4" s="9" t="inlineStr">
+      <c r="S4" s="7" t="inlineStr">
         <is>
           <t>Agents correctly validated and interpreted z-score outliers beyond 10 SD: 19 Oct 1987 (-20.47%), 13 Oct 2008 (+11.58%), 16 Mar 2020 (-11.98%). The contribution is automated validation and interpretation rather than a detection score.</t>
         </is>
       </c>
-      <c r="T4" s="9" t="inlineStr">
+      <c r="T4" s="7" t="inlineStr">
         <is>
           <t>Built strictly for anomaly classification - no portfolio allocation, no execution, no risk scaling. No accuracy metric, so it's hard to compare against anything.</t>
         </is>
       </c>
-      <c r="U4" s="9" t="inlineStr">
+      <c r="U4" s="7" t="inlineStr">
         <is>
           <t>NOT YET REVIEWED - fields here come from the source paper, not my own read. Tabled it because it's about monitoring the market for anomalies and fraud rather than investing in it. Worth revisiting for the tooling though: the alert-verification pattern (statistical trigger -&gt; agent runs background research -&gt; consolidated report) is exactly how I'd want my risk agent to explain a volatility spike instead of just flagging it.</t>
         </is>
       </c>
-      <c r="V4" s="9" t="inlineStr">
+      <c r="V4" s="7" t="inlineStr">
         <is>
           <t>Doesn't do allocation or execution at all, so nothing in it competes with my framework - it's a component pattern, not a rival architecture.</t>
         </is>
       </c>
-      <c r="W4" s="9" t="inlineStr">
+      <c r="W4" s="7" t="inlineStr">
         <is>
           <t>[[Enhancing Anomaly Detection in Financial Markets with an LLM-Based Multi-Agent Framework]] - NOT YET REVIEWED</t>
         </is>
       </c>
     </row>
     <row r="5" ht="150" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>P04</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Zhao, T., Lyu, J., Jones, S., Garber, H., Pasquali, S. &amp; Mehta, D. (BlackRock)</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Zhao, Lyu, Jones, Garber, Pasquali &amp; Mehta (BlackRock)</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>arXiv preprint</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>arXiv preprint 2508.11152v1, August 2025</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>arXiv:2508.11152 | https://arxiv.org/abs/2508.11152</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Multi-agent equity portfolio construction</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Prior work leans on chain-of-thought prompting and neglects structured agent interaction, and agent-specific risk tolerance has had almost no attention. Tests whether role-based agents plus a debate loop cut hallucination and cognitive bias.</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>US equities. 15 randomly selected technology-sector stocks.</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>10-K and 10-Q filings, financial news and analyst ratings, price and volume. January 2024 training data, four-month test window from 1 Feb 2024.</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Filing text via RAG, news text, price/volume series.</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Microsoft AutoGen as the infrastructure (group chat plus assistant agents), AutoGen Studio as the UI. Three specialised agents produce stock analysis reports, and where they disagree a round-robin debate runs until consensus, two turns each. Risk tolerance (neutral vs averse) is set by prompt. Output is a stock selection and portfolio.</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Fundamental agent, Sentiment agent, Valuation agent, coordinated by AutoGen group chat with an internal round-robin debate mechanism.</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>Sentiment agent over financial news, analyst ratings and disclosures, using reflection-enhanced prompting - the model is told to reason, critique and refine its summary rather than extract directly. English only.</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>Fundamental agent gets two tools: a Report Pull tool that fetches the right filings, and a Report RAG tool doing section-based context chunking with GPT-4o as the embedding model, answering set questions on cash flow and income, operations and gross margin, areas of concern, and progress against stated objectives.</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>Nothing econometric. Risk enters only as a prompt-level tolerance profile (risk-neutral vs risk-averse).</t>
-        </is>
-      </c>
-      <c r="P5" s="5" t="inlineStr">
-        <is>
-          <t>None. Frictionless, zero-slippage execution assumed.</t>
-        </is>
-      </c>
-      <c r="Q5" s="5" t="inlineStr">
-        <is>
-          <t>Debate transcripts and per-agent reports. RAG traced with the Arize Phoenix observability platform.</t>
-        </is>
-      </c>
-      <c r="R5" s="5" t="inlineStr">
-        <is>
-          <t>Cumulative return and rolling Sharpe against an equal-weight benchmark and single-agent variants.</t>
-        </is>
-      </c>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>In the risk-neutral setting the multi-agent portfolio beats both the equal-weight benchmark and the single-agent variants. In the risk-averse setting every agent portfolio underperforms, because the volatile tech names get excluded. No single headline percentage is reported.</t>
-        </is>
-      </c>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>Prompt-based risk profiles are hard to tell apart at adjacent risk boundaries - the paper says so itself. Frictionless execution. 15 stocks, one sector, four months.</t>
-        </is>
-      </c>
-      <c r="U5" s="5" t="inlineStr">
-        <is>
-          <t>Reflection-enhanced prompting for the sentiment agent and the round-robin debate-to-consensus protocol. Also the observability angle - setting up Arize Phoenix (or equivalent) to trace the RAG early rather than bolting it on at the end.</t>
-        </is>
-      </c>
-      <c r="V5" s="5" t="inlineStr">
-        <is>
-          <t>No social media agent, no risk-calculating agent, and it won't work for CSE because of the fluidity assumption. Prompt-level risk tolerance isn't a substitute for actually modelling second moments.</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Prior work emphasises chain-of-thought prompting and neglects structured agent interaction, and agent-specific risk tolerance has had little attention. Contributes debate as a hallucination check and investor risk tolerance embedded in the prompt rather than applied as a filter afterwards. Stops at stock selection, feeding a screened list to mean-variance optimisation or Black-Litterman, and never produces weights itself.</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>US equities. Fifteen randomly selected technology stocks acting as both the picking pool and the equal-weight benchmark.</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Agents run on January 2024 data, selection on 1 February 2024, four months of monitoring. 10-K and 10-Q filings, Bloomberg news bodies, analyst ratings and disclosures, price and volume.</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>Each agent sees only the data its role needs and no two agents share anything past the ticker, so there is NO REDUNDANCY ANYWHERE in the system - each signal has exactly one agent responsible for it and no second opinion on it.</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>Microsoft AutoGen group chat with AutoGen Studio as the interface, GPT-4o as the backbone for every agent. Collaboration runs first to produce the analysis report, debate second to produce the recommendation. Output is a BUY or SELL screen, not weights.</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Fundamental, Sentiment and Valuation agents argue to consensus through a round-robin debate, each getting at least two turns, with the coordinator requiring all agents to be invoked before terminating. Takes the opposite position to FinCon on the one architectural question I have to answer: FinCon forbids lateral chatter because it's an unpriced cost, AlphaAgents makes debate the point because disagreement is the only signal that an agent is hallucinating. Neither runs the comparison that would settle it.</t>
+        </is>
+      </c>
+      <c r="M5" s="9" t="inlineStr">
+        <is>
+          <t>Reflection-enhanced prompting - the sentiment agent summarises, critiques its own summary, then refines. Deliberately uses LLM summarisation rather than retrieval, a coverage-versus-precision choice. Bloomberg news, analyst ratings and disclosures, all English and institutional.</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="inlineStr">
+        <is>
+          <t>A yfinance Report Pull Tool with iterative call checks, plus a Report RAG Tool that chunks by report section and embeds with GPT-4o, invoked repeatedly against a fixed question set covering cash flow and income, operations and gross margin, areas of concern, and progress towards stated objectives. Section-boundary chunking is the same conclusion the Financial Report Chunking paper reaches independently.</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
+        <is>
+          <t>Risk enters only as a prompt adjective - agents are told the investor is risk-averse or risk-neutral and reason about volatility qualitatively from there. No computed risk measure at all, which is weaker than FinCon's CVaR. The risk-seeking profile turned out indistinguishable from risk-neutral and was cut from the evaluation, which the authors read as a limitation of prompt-based differentiation between adjacent profiles.</t>
+        </is>
+      </c>
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>None. Equal weights at selection, held four months, rebalancing not modelled.</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>The strongest in my set at the component level. An observability platform (Arize Phoenix) scores retrieval faithfulness and relevance per retrieval and monitors whether the valuation agent actually called its calculator, full debate transcripts are logged and human-reviewable with the ability to override, and every quantitative figure is computed by a tool outside the model and passed in, so a wrong number has to come from the tool rather than from the LLM doing arithmetic in-context.</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr">
+        <is>
+          <t>Back-testing with risk-adjusted return tracked by a rolling Sharpe ratio, though the window length is never stated so the curves can't be reproduced. Benchmark is an equal-weight portfolio of the same fifteen candidates.</t>
+        </is>
+      </c>
+      <c r="S5" s="9" t="inlineStr">
+        <is>
+          <t>In the risk-neutral setting the multi-agent portfolio beats both single-agent portfolios and the benchmark on cumulative return and rolling Sharpe. But the absolute numbers are much worse than 'outperforms' implies - cumulative return sits below zero for most of the window, bottoming near -0.10, and rolling Sharpe is negative throughout at roughly -0.10 to -0.45, so this is smaller losses than the benchmark over four months, not positive risk-adjusted return. Under a risk-averse profile every agent portfolio underperformed because the technology sector rallied and the risk-averse agents excluded the volatile names that drove it. The valuation agent reproduces the benchmark portfolio directly under a risk-neutral profile, so it isn't differentiating from the market baseline at all.</t>
+        </is>
+      </c>
+      <c r="T5" s="9" t="inlineStr">
+        <is>
+          <t>No numerical results anywhere - the results section is entirely figures with no table and no point estimate in the text, so every comparison is eyeballed off a chart. One sector, fifteen stocks, one four-month window, one selection date, no repeated splits, no walk-forward, no significance testing. Look-ahead risk from the backbone is never raised even though GPT-4o's pretraining plausibly covers the exact test window on fifteen heavily covered megacaps. Forced consensus discards the most informative outcome, since the system cannot report persistent disagreement. Debate is never ablated, which is unfortunate given it's the headline contribution. Consensus is also not correctness - three agents on the same backbone can converge on the same wrong answer, and the hallucination-reduction claim needs errors to be at least partly independent, which one GPT-4o driving all three is exactly the condition against.</t>
+        </is>
+      </c>
+      <c r="U5" s="9" t="inlineStr">
+        <is>
+          <t>The calculator-tool pattern is the cheapest reliability win here - compute every figure outside the model, pass it in, verify the call in the observability layer - and that's also where a CSE-specific risk measure enters cleanly, as a computed input rather than something the model reasons about qualitatively. Build observability in from the start, because per-retrieval faithfulness gives me a component-level evaluation story independent of the back-test, which matters a lot when the back-test will be short and underpowered by construction. Keep debate but make disagreement reportable and vary the backbone, since a persistent-disagreement terminal state turns the mechanism's most useful output into a flag and gives a free proxy for decision confidence.</t>
+        </is>
+      </c>
+      <c r="V5" s="9" t="inlineStr">
+        <is>
+          <t>THE SENTIMENT AGENT WAS DROPPED FROM THE PORTFOLIO COMPARISON ENTIRELY for insufficient news coverage across some of the fifteen stocks - fifteen US technology large caps, and the news was still too thin. That is direct evidence, from the paper's own experiment, that agent reliability varies by ticker and that these systems have no mechanism to handle it beyond removing the agent by hand. Strict data partitioning is a cost rather than a feature here: with no redundancy, a starved agent takes its entire signal channel down with it. On the CSE at least one channel will be thin for most tickers, so I want either deliberate overlap between agents or a confidence-and-abstain protocol telling the aggregator which inputs are actually live for a given stock.</t>
+        </is>
+      </c>
+      <c r="W5" s="9" t="inlineStr">
         <is>
           <t>[[AlphaAgents, Large Language Model Based Multi-Agents for Equity Portfolio Constructions]]</t>
         </is>
@@ -1919,7 +1930,7 @@
       </c>
       <c r="V12" s="3" t="inlineStr">
         <is>
-          <t>It's linear, monthly and market-wide. No order book, no intraday, no non-linear regimes. Nobody has put actual Sinhala or English text sentiment next to CSE liquidity - turnover-as-sentiment is as close as the literature gets.</t>
+          <t>It's linear, monthly and market-wide. No order book, no intraday, no non-linear regimes. Turnover-as-sentiment is a price-derived proxy rather than a measure of investor mood, and while CSE sentiment work does exist - Dinushan and Wijegunasekara (P23) use a single English publisher's Twitter feed, and there is further local sentiment-prediction work I still need to read - I have not found a study that puts a text sentiment series next to the CSE liquidity measures this paper builds, or that lets the sentiment weight vary with the liquidity state.</t>
         </is>
       </c>
       <c r="W12" s="3" t="inlineStr">
@@ -2036,7 +2047,7 @@
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>Purely statistical and purely descriptive. Nobody has taken d and used it inside a trading or allocation system, and there's no text or semantic input anywhere near it. That's my opening - using the fractional integration parameter as a live risk guardrail rather than a reported coefficient in a table.</t>
+          <t>Purely statistical and purely descriptive - it characterises how volatility behaved and builds nothing on top. FIGARCH and related long-memory models are well established for volatility forecasting, VaR, portfolio risk, hedging and asset allocation, so the estimator itself is not the opening and I should not claim it is. What I have not found is a persistence estimate feeding an agent-weighting or exposure mechanism inside an autonomous system, with no text or semantic input anywhere near this literature either. That composition is the opening, and it is narrower than 'nobody uses d'.</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
@@ -2163,117 +2174,117 @@
       </c>
     </row>
     <row r="15" ht="150" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>P14</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Aldasoro, I., Hordahl, P., Schrimpf, A. &amp; Zhu, S. (BIS)</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>BIS Working Papers No. 1250, 17 March 2025. Also CEPR Discussion Paper DP20439</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>https://www.bis.org/publ/work1250.pdf</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Market stress / tail-risk forecasting</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Forecasts financial market stress as a full conditional distribution rather than a point estimate, using newly constructed market condition indicators.</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>US Treasury, FX and money markets.</t>
         </is>
       </c>
-      <c r="I15" s="9" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>Newly constructed market condition indicators (MCIs) for the three markets above.</t>
         </is>
       </c>
-      <c r="J15" s="9" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>Funding liquidity, global financial cycle and macro stress inputs aggregated into the MCIs.</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>Tree-based machine learning - random forests with quantile regression to map the full conditional distribution of future stress, with SHAP values to identify which factors are contributing.</t>
         </is>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="L15" s="7" t="inlineStr">
         <is>
           <t>N/A.</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>N/A.</t>
         </is>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="N15" s="7" t="inlineStr">
         <is>
           <t>N/A.</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="O15" s="7" t="inlineStr">
         <is>
           <t>This is the whole paper - forecasting the probability of extreme stress episodes rather than modelling conditional variance directly.</t>
         </is>
       </c>
-      <c r="P15" s="9" t="inlineStr">
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>Funding liquidity is one of the MCI inputs, so liquidity enters as a stress driver rather than an execution cost.</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="Q15" s="7" t="inlineStr">
         <is>
           <t>SHAP values identify which risk factors are driving a given stress forecast, which is the part that matters for a guardrail you have to justify.</t>
         </is>
       </c>
-      <c r="R15" s="9" t="inlineStr">
+      <c r="R15" s="7" t="inlineStr">
         <is>
           <t>Quantile loss, against autoregressive time-series benchmarks.</t>
         </is>
       </c>
-      <c r="S15" s="9" t="inlineStr">
+      <c r="S15" s="7" t="inlineStr">
         <is>
           <t>Random forests achieve up to 27% lower quantile loss than the autoregressive benchmarks, with the largest gains at 3-12 month horizons.</t>
         </is>
       </c>
-      <c r="T15" s="9" t="inlineStr">
+      <c r="T15" s="7" t="inlineStr">
         <is>
           <t>Heavy dependence on structural macro data. US markets only. Likely to struggle across abrupt regime switches unless paired with something real-time.</t>
         </is>
       </c>
-      <c r="U15" s="9" t="inlineStr">
+      <c r="U15" s="7" t="inlineStr">
         <is>
           <t>NOT YET REVIEWED - fields here come from the source paper, not my own read. I couldn't find it on Semantic Scholar so I left it; the PDF is at bis.org/publ/work1250.pdf. Worth coming back to for the risk agent though: forecasting the whole conditional distribution of stress rather than a point estimate, plus SHAP attribution for which factor is driving it, is the right shape for a risk guardrail that has to explain itself.</t>
         </is>
       </c>
-      <c r="V15" s="9" t="inlineStr">
+      <c r="V15" s="7" t="inlineStr">
         <is>
           <t>US Treasury, FX and money markets. CSE has nothing like the MCI inputs available, so the method transfers but the features don't - I'd have to construct a Sri Lankan equivalent from what CBSL actually publishes.</t>
         </is>
       </c>
-      <c r="W15" s="9" t="inlineStr">
+      <c r="W15" s="7" t="inlineStr">
         <is>
           <t>[[Predicting Financial Market Stress with Machine Learning]] - NOT YET REVIEWED</t>
         </is>
@@ -2396,8 +2407,1178 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>P16</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Zong, Wang, Qin, Feng, Wang &amp; An (NTU Singapore, Skywork AI, SUTD)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>KDD '24. Code at github.com/ZONG0004/MacroHFT</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>MacroHFT | github.com/ZONG0004/MacroHFT</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Memory-augmented context-aware RL for high-frequency trading</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Existing RL-based HFT treats market conditions as uniform, or segments on trend alone and neglects volatility entirely; policies overfit a narrow feature slice with no mechanism to adjust for recent conditions; and a single agent adjusts too slowly during sudden fluctuations. Builds a two-level hierarchy where specialists are trained per market condition and a hyper-agent mixes them.</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Cryptocurrency. Four USDT pairs on Binance, deep and continuously traded.</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>BTC, ETH, DOT and LTC against USDT at minute granularity with 5-level limit order book snapshots alongside OHLCV. One fixed train/validation/test split per market, not walk-forward. The test windows are all flat to down, the underlying fell 14.85% on DOT and 24.94% on LTC.</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Genuinely microstructural rather than the usual RSI-and-MACD bundle: weighted average price from the top two book levels, order flow imbalance across all five levels, spreads, volumes, each z-scored against its own trailing 60-minute window before it reaches the network. Appendix A gives every indicator's formula explicitly.</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>Two MDPs sharing one minute-level time scale - the hierarchy is over policy specialisation, not temporal abstraction. Six dueling DDQN sub-agents, each trained on a slice of the data. Conditional adaptation borrowed from Diffusion Transformers turns position and context into a scale and shift on the normalised hidden state rather than concatenating them, so a low-dimensional conditioning signal doesn't get drowned by the state vector. Output is a binary target position, long only, fixed size.</t>
+        </is>
+      </c>
+      <c r="L17" s="9" t="inlineStr">
+        <is>
+          <t>THE CLOSEST PRIOR WORK TO MY MAIN GAP. Training data is cut into fixed-length chunks, each chunk labelled by trend (low-pass filter, linear regression, slope) and by volatility (computed on the unsmoothed chunk so the filter doesn't destroy what's being measured), then split into tertiles on each indicator separately - six marginal specialists, not nine joint ones. A hyper-agent conditioned on the current slope-and-volatility pair emits a softmax weight vector over the six and mixes their Q-values. Episodic memory (fixed-capacity table, FIFO eviction, L2 top-m lookup) supplies an auxiliary regression target to stabilise the mixture under sudden fluctuation.</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>None. No text input anywhere.</t>
+        </is>
+      </c>
+      <c r="N17" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
+        <is>
+          <t>Volatility is a conditioning variable the policy is trained against rather than a metric reported at the end, which is the mechanism I've been missing. But it's realised volatility discretised into tertiles - no conditional variance model, no persistence estimate, and no explicit risk budget or exposure cap.</t>
+        </is>
+      </c>
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t>Commission fixed at 0.02% for all four pairs. No slippage, no queue position, no partial fills, no market impact, no spread crossing - despite five levels of LOB feeding the state and orders described as limit orders placed into that book. At roughly twenty round trips over four months the commission barely binds, so the setup carries essentially no information about cost sensitivity.</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>The learned sub-agent weights are inspectable, and a decision annotated with the weight assigned to the bear specialist versus the volatile specialist is an attributable explanation with no extra instrumentation. No formal attribution method.</t>
+        </is>
+      </c>
+      <c r="R17" s="9" t="inlineStr">
+        <is>
+          <t>One profit criterion (TR), two risk criteria (AVOL, MDD) and three risk-adjusted (ASR, ACR, ASoR), all annualised. Eight baselines: DQN, DDQN, CDQNRP, PPO, CLSTM-PPO and EarnHFT on the RL side, Imbalance Volume and MACD on the rule-based side. No buy-and-hold row.</t>
+        </is>
+      </c>
+      <c r="S17" s="9" t="inlineStr">
+        <is>
+          <t>The only method finishing positive on all four markets - TR of 3.03%, 39.28%, 13.79% and 18.16% - and best on all four for every risk-adjusted criterion. But raw risk is mixed: AVOL of 18.19% on BTC against CDQNRP's 1.29%, and 40.31% on DOT is the worst figure in that block, so the defensible claim is return per unit of risk, not lower risk. The EarnHFT comparison is only a real contest on ETH, where EarnHFT reaches 18.02% and MacroHFT 39.28%; on the other three EarnHFT simply failed to find a profitable policy. Trade counts are 19, 20, 38 and 138 over four months, so this is a low-turnover position-holding policy and 'high frequency' describes the observation granularity, not the trade frequency. Figure 5 shows the learned mixture is close to binary on BTC, with three of six curves barely off the floor for the whole test period.</t>
+        </is>
+      </c>
+      <c r="T17" s="9" t="inlineStr">
+        <is>
+          <t>Single run per cell, one test window per market, no seeds, no error bars, no significance test, and the four markets are all crypto over the same mid-2023 period so they're far less independent than the table implies. Execution ignores the order book the state observes. Binary position, long only, fixed size, so there's no sizing decision at all. Six marginal sub-agents rather than nine joint ones, never justified or ablated, even though the decomposition itself identifies a joint cell. The Optimal Value Supervisor is a hindsight teacher computed by dynamic programming over training data with full knowledge of future prices, and no ablation sets its weight to zero, so the two claimed contributions are measured on top of an unmeasured third. Two notational errors worth catching before reimplementing: the bid/ask direction in Section 3.2 is inverted, and equation 7 weights retrieved experiences proportionally to distance rather than inversely, so the least similar neighbours get the most weight.</t>
+        </is>
+      </c>
+      <c r="U17" s="9" t="inlineStr">
+        <is>
+          <t>The operational answer to the volatility-memory question I'd been missing: label chunks by realised volatility tertile, train a specialist per tertile, condition the policy on the current slope-and-volatility pair at decision time. Long memory is what makes this work at all, since a volatility label only has predictive content for the next chunk if volatility persists, so the FIGARCH estimates justify the design rather than sitting beside it. The conditional adapter is the cheapest transferable piece - FiLM-style conditioning beats concatenation when a low-dimensional signal meets a high-dimensional state, which is exactly my situation feeding position, regime label and sentiment score into a policy network. Test routing before building mixing, since the learned mixture is near-binary anyway and the marginal gain over EarnHFT's hard router is unquantified. And don't inherit the six-marginal-agents choice - on the CSE the thin-and-whale-driven regime and the volatile regime plausibly coincide, so the joint cell is the one I'd actually want.</t>
+        </is>
+      </c>
+      <c r="V17" s="9" t="inlineStr">
+        <is>
+          <t>This is the paper my main gap has to be defended against, and the delta is specific rather than rhetorical. Its state-conditioning is over homogeneous DDQN sub-policies, not heterogeneous agent types with different failure modes; it conditions on trend and realised volatility, not on liquidity state or volatility persistence; and it runs on deep liquid crypto where twenty round trips at 2 bps means friction never binds, so it tells me nothing about what happens when a policy of this shape pays realistic CSE spread and impact. That absence is the opening, and the honest thing is to record it rather than assume the design survives the friction.</t>
+        </is>
+      </c>
+      <c r="W17" s="9" t="inlineStr">
+        <is>
+          <t>[[MacroHFT, Memory Augmented Context-aware Reinforcement Learning On High Frequency Trading]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>P17</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Jeon, Park, Park &amp; Kang (Seoul National University, DeepTrade Technologies)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>KDD '24</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>FreQuant (no code release mentioned)</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>RL portfolio optimisation with frequency-domain state representation</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Time-domain encoders smooth away the abrupt changes that matter most, treating them as anomalies rather than signals. Movement-prediction models have no access to fee-adjusted rewards or portfolio weights, which argues for solving allocation end to end. Builds the whole state representation in the frequency domain instead.</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Six markets - US, Korea, crypto, China, Japan, UK - all deep and liquid. The UK configuration, 21 assets with 10 held, is the only one anywhere near CSE breadth.</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Daily bars. One fixed train/test split per market, no validation period reported and no walk-forward. Test windows range from nine years on the US market to thirteen months on crypto, so the six headline figures aren't comparable to each other as evidence even though they're printed in one row.</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Asset price feature tensor, market index tensor and current weights, with the lookback fixed at 256 days. Each retained Fourier component is an 'Event', the k-th periodic constituent of that asset - with daily data and a 256-day window, the 8th component is a pattern repeating every 32 days. Note this is Fourier frequency, cycles per day, not sampling rate.</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>Four parallel Frequency State Encoder blocks over progressively shorter segments (256, 128, 64, 32 days), each running a 1-d DFT along the temporal axis. A Multi-Event Fusion Network applies learned complex filters, and a Frequency-Relation Encoder is a Transformer rewritten for complex vectors with the dot product replaced by the Hermitian inner product and softmax by a magnitude-based version, attending over frequencies within a single asset. A Portfolio Generator then runs the same structure across the asset dimension and keeps only the top-k by confidence magnitude, with a learned cash bias competing for a slot. DDPG actor-critic. Action is a long-short weight vector with an L1 budget of 1.</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Single policy, not multi-agent. No orchestration of any kind.</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="O18" s="9" t="inlineStr">
+        <is>
+          <t>Volatility enters only implicitly through the spectrum. No conditional variance model, no risk constraint, no exposure cap, and no drawdown metric reported.</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr">
+        <is>
+          <t>THE ONLY CORRECT FEE TREATMENT IN MY SET. Fees are charged on closing positions at 0.33% closing a long and 0.4% closing a short, sixteen to twenty times the 2 bps assumed elsewhere, and the paper solves the self-referential problem properly - the fee reduces capital, which changes weights, which changes the fee - by fixed-point iteration with three directional constraints. But a commission rate is not execution cost in a thin book: no spread, no market impact, no partial fill, no queue position. The rebalancing frequency is defined in the formulation and then never given a value, so annual cost drag cannot be reconstructed at all.</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
+        <is>
+          <t>Anecdotal throughout. Sony's console launch and Brexit's effect on J.P. Morgan are two hand-picked assets with narratively matched events. The mechanisms are visible and their contribution is never quantified.</t>
+        </is>
+      </c>
+      <c r="R18" s="9" t="inlineStr">
+        <is>
+          <t>Two metrics only, Annualized Rate of Return and Annualized Sharpe, plus a portfolio value plot. No drawdown, no turnover, no trade count. Five long-short competitors: Cross-Sectional Mean reversion, Buying-Loser-Selling-Winner, AlphaStock, DeepTrader and MetaTrader.</t>
+        </is>
+      </c>
+      <c r="S18" s="9" t="inlineStr">
+        <is>
+          <t>Best ARR on all six markets and best ASR on five of six, the exception being the US market - the longest test window - where DeepTrader takes 0.810 against FreQuant's 0.770. The abstract's 'up to 2.1x higher ARR' is the US market alone; the median improvement over the strongest baseline is nearer 1.6x. The market-shift experiment is the strongest argument in the paper: on high-fluctuation days, total return exceeds the next best model by 16.9 points on US, 49.3 on crypto and 24.4 on Korea, with the runners-up negative on two of the three. Periodicity guidance lowers reward variance in 21 of 24 cells with one clear counterexample the paper doesn't mention. Two baselines reach -84% and -145% on crypto, which is unreachable as a compound rate under an L1 budget of 1, so ARR must be an arithmetic annualization - and no formula for ARR or ASR appears anywhere.</t>
+        </is>
+      </c>
+      <c r="T18" s="9" t="inlineStr">
+        <is>
+          <t>One run per cell, one split per market, no seeds, no significance tests, no walk-forward, and the US model is trained once on data ending in 2013 then evaluated through to late 2022 with no refit. The frequency premise is asserted and never ablated - all three variants ablate the encoder over the spectrum, none removes the spectrum, so the table cannot distinguish 'the frequency domain helps' from 'the complex Transformer helps'. A DFT over 256 days discards time localisation entirely, which is a strange choice for a method selling responsiveness to sudden events; the dyadic segmentation recovers some of it and is effectively a crude wavelet scheme the paper never frames that way. Universe construction and survivorship bias go entirely unaddressed across a thirty-year US sample.</t>
+        </is>
+      </c>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>Frequency-domain state is the natural representation for the one thing actually established about the CSE, because long memory is by definition a statement about the low-frequency end of the spectral density - the density diverging at the origin with the same fractional differencing parameter FIGARCH estimates. That gives me a second route to operationalising the volatility-memory result, and which one survives depends on data depth: partitioning by regime is expensive in sample size, whereas a spectral encoder consumes the same series at every resolution and costs nothing in data. Top-k selection with a learned cash bias is the right action-space shape for thin breadth, since the policy never assigns weight to something it cannot trade and cash gives it a principled way to stand aside. The fee fixed point is liftable as-is. The wavelet version of the multi-resolution segmentation is a concrete novelty candidate that doesn't depend on the CSE data situation resolving favourably.</t>
+        </is>
+      </c>
+      <c r="V18" s="9" t="inlineStr">
+        <is>
+          <t>Single-policy, so nothing here addresses orchestration over heterogeneous agents. Long-short machinery may not transfer at all - whether the CSE offers a practical short mechanism through securities borrowing and lending needs confirming in writing rather than assuming, and if it doesn't, the action space collapses to non-negative weights and the fee fixed point simplifies considerably. And the execution-friction blind spot survives intact in the paper that pays costs the most attention.</t>
+        </is>
+      </c>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>[[FreQuant, A Reinforcement-Learning based Adaptive Portfolio Optimization with Multi-frequency Decomposition]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="150" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>P18</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Yu, Yao, Li, Deng et al. (Stevens Institute of Technology, Harvard, The Fin AI)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>NeurIPS 2024</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>FinCon</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>LLM multi-agent system for sequential financial decision making</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Prior LLM financial agents set risk preferences from short-term price fluctuation rather than an established quantitative risk measure, are mostly single-asset, and pile all information onto one agent inside one context window so decision quality degrades as data volume grows. Against systems that do use discussion, the charge is that unbounded peer-to-peer chatter is expensive and slow with nothing forcing convergence on profit.</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>US equities. Eight large caps for single-stock, plus two three-stock portfolios drawn from a 42-stock pool filtered on news availability, over 800 articles each.</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>3 January 2022 to 10 June 2023, train to 4 October 2022 and test from 5 October 2022. Prices from Yahoo Finance, news from Refinitiv, filings from SEC EDGAR, Zacks equity research, and earnings call audio transcribed with Whisper. DRL baselines get a much longer training window from 2018 because they need it to converge.</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>One uni-modal stream per analyst agent - news text, 10-Q/10-K MD&amp;A sections, analyst reports, earnings call audio, tabular time series. All English, all institutional.</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Quantitative trading framed as an infinite-horizon POMDP. Analyst 'actions' are text; the manager's action space is buy/sell/hold, extended with a weight per asset for portfolios. The crucial design choice is that portfolio weights come from an external Markowitz mean-variance solver with a directional constraint bolted on from the manager's discrete decision, so the LLM picks direction and a classical optimizer picks size. Policies are parameterised by textual prompts, so this is risk-sensitive optimisation solved by textual gradient descent rather than by DRL.</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>THE CLOSEST PUBLISHED SYSTEM TO MY ORCHESTRATION QUESTION. Strict manager-analyst hierarchy - analysts talk to the manager and never to each other, so communication is linear in the number of agents rather than quadratic. Six or seven single-modality analyst agents feed one manager who is the sole decision maker and sole holder of episodic memory. Explicitly refuses lateral debate, which is the direct opposite of AlphaAgents and the strongest existing argument that peer-to-peer discussion is a cost rather than a feature.</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>News, analyst notes and earnings call audio, all English and institutional. No social media path, nothing code-mixed, no dedicated sentiment model.</t>
+        </is>
+      </c>
+      <c r="N19" s="9" t="inlineStr">
+        <is>
+          <t>A filings analyst agent reads 10-Q and 10-K MD&amp;A sections. No chunking or retrieval design is described in detail.</t>
+        </is>
+      </c>
+      <c r="O19" s="9" t="inlineStr">
+        <is>
+          <t>Dual-level risk control is the actual contribution. Within-episode, CVaR at the 1% level on realised daily PnL - a sudden drop triggers a risk alert and the manager goes risk-averse for the day regardless of its prior stance. Over-episode, the system compares objective values between consecutive episodes and rewrites its own investment beliefs in natural language, using the overlapping percentage of trading decisions as the learning rate. Backward-looking and empirical: no volatility persistence anywhere, and beliefs are frozen at test time.</t>
+        </is>
+      </c>
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t>None. Buy/sell/hold with portfolio weights rebalanced daily, no transaction cost, no slippage, no liquidity constraint in the optimizer.</t>
+        </is>
+      </c>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>The learned artefact is human-readable - Figure 8 shows beliefs evolving from generic to specific and executable - and the debate-free structure means every decision traces to a named analyst's report. No formal attribution method.</t>
+        </is>
+      </c>
+      <c r="R19" s="9" t="inlineStr">
+        <is>
+          <t>Cumulative Return, Sharpe, Max Drawdown. Baselines: buy-and-hold, DRL agents via FinRL, and the LLM agents FinGPT, FinMem and FinAgent for single stock; Markowitz MV, FinRL-A2C and an equal-weighted ETF for portfolios. Wilcoxon signed-rank on the main comparison.</t>
+        </is>
+      </c>
+      <c r="S19" s="9" t="inlineStr">
+        <is>
+          <t>Highest CR and SR on all eight tickers - TSLA 82.871% CR and 1.972 SR against buy-and-hold's 6.425% and 0.145. Portfolio 1 reaches 113.836% CR with Sharpe 3.269. Both ablations are strong and are the reason to trust the architecture rather than the headline: removing within-episode CVaR control takes GOOG from 25.077% to -1.461% and Portfolio 1 from 113.836% to 14.699%, and removing over-episode belief updates takes Portfolio 1 to 28.432%. Trading action overlap between consecutive training episodes runs 46.9%, 71.4%, 81.6%, so beliefs stabilise after four episodes against DRL agents needing years of data. Under a high-volatility window Portfolio 1 returns -8.429%, best of a bad field but still a loss, and that's the number I'd quote rather than the 113.836%.</t>
+        </is>
+      </c>
+      <c r="T19" s="9" t="inlineStr">
+        <is>
+          <t>Tested on portfolios of three, with hallucination already increasing from one asset to three. No transaction costs, slippage or liquidity anywhere. Single backbone throughout, so architecture versus model is unresolved. Beliefs frozen at test time, so there's no evidence the system adapts to regime change it hasn't seen in training. The NeurIPS checklist answers No on statistical significance and error bars. Table 3's caption claims FinCon leads all performance metrics and it doesn't - on Portfolio 2 both FinRL-A2C and the equal-weighted ETF have lower drawdown.</t>
+        </is>
+      </c>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>The manager-analyst hierarchy with no lateral chatter as the default, and if I want debate anywhere I have to justify the cost against this paper rather than ignore it. Separating direction from sizing - LLM emits a discrete signal, a classical optimizer converts it to weights - keeps the sizing auditable and gives a clean insertion point for CSE liquidity and friction constraints. Per-source memory decay rates are directly portable and more defensible on the CSE than on US large caps, because CSE information arrives so irregularly. The decision-overlap learning rate is the better idea than text edit distance, since two prompts can read very differently and produce identical trades.</t>
+        </is>
+      </c>
+      <c r="V19" s="9" t="inlineStr">
+        <is>
+          <t>Risk is empirical CVaR on realised PnL, which is backward-looking and carries no persistence structure - feeding a FIGARCH-derived conditional volatility into the risk agent instead of, or alongside, it is a concrete and defensible extension. More fundamentally, the manager consolidates analyst insights but never weights them by market state, and beliefs are frozen at test time, so there's no mechanism by which a channel that has become unreliable gets down-weighted. And the architecture works partly because its information environment is dense - on the CSE most tickers will have one weak signal or none, so an analyst agent with no data produces confident text about nothing and the manager has no way to tell.</t>
+        </is>
+      </c>
+      <c r="W19" s="9" t="inlineStr">
+        <is>
+          <t>[[FinCon, A Synthesized LLM Multi-Agent System with Conceptual Verbal Reinforcement for Enhanced Financial Decision Making]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="150" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>P19</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Chen, Zou, Wang, Wang, Sun, Zhang &amp; Xu (Fudan, Tensorpacific, Peng Cheng Laboratory, Meta AI, Shanghai Academy of AI for Science)</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Findings of EMNLP 2025, pp. 1648-1672. Code at github.com/pilgrim00/FinHEAR</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>FinHEAR | github.com/pilgrim00/FinHEAR</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>LLM multi-agent trading with behavioural-economics risk sizing</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Existing methods have no structured channel for accumulated human judgement, risk sensitivity is flat where prospect theory says it should be asymmetric, and early errors compound over a trading sequence with nothing forcing a revision.</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>US equities plus one commodity - AAPL, TSLA, XOM and gold. Deep and liquid.</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>26 December 2019 to 29 December 2023, training 2020-2022 and testing across calendar 2023, with a 7-day lookback reserved at both ends. The text side is large: 21,329 industry and company news items, 22,274 current-affairs articles, 2,128 macroeconomic releases, 280 central-bank communications and 61 fiscal reports, against only about 1,023 daily OHLCV rows.</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>Roughly forty text items per trading day against one price row, which is a very different information profile from the DRL literature. 'Human expertise' means a corpus of investor writing - Graham, Buffett, Soros, Lynch, Munger, Marks, Dalio - compressed by GPT-4o into structured query-knowledge pairs and retrieved by cosine similarity at decision time.</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Six agents in sequence: Historical Trend, Current Event, Human Expertise, Risk Analysis, Decision, and Temporal Refinement. No gradient training anywhere - the training period exists to populate and refine the expert knowledge base, and refinement continues through the test period using realised outcomes.</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Event-driven pipeline rather than debate or hierarchy. The Risk Analysis Agent measures disagreement across the three upstream agents and emits a discrete low/medium/high level, which then drives sizing. The Temporal Refinement Agent closes the loop by rewriting the expert entry or trend summary that produced a failed prediction.</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>The Current Event Agent interprets macro announcements and firm news. English only, institutional sources, no dedicated sentiment model.</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>The expert knowledge base is retrieval over curated investor reasoning, not over filings. No financial-document RAG.</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>THE ONLY SYSTEM IN MY SET WHERE POSITION SIZE IS A FIRST-CLASS OUTPUT. A risk sensitivity is drawn from a Beta rescaled onto a context-specific interval - left-skewed on [0.75, 0.9] in low-risk contexts, right-skewed on [0.1, 0.4] in high-risk ones - then multiplied against floored expert reliability and square-rooted event similarity to give a continuous weight. Two thresholds then map that weight and the predicted direction onto close, hold, long or short, so the lower threshold suppresses weak signals into inaction. But the sensitivity is SAMPLED from an assumed Beta, not measured from the market, and the Beta shapes and intervals are hand-set with no search reported.</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr">
+        <is>
+          <t>No transaction costs in the main results. The robustness appendix applies 5 basis points per side on AAPL only, taking cumulative return from 30.81% to 25.96% and Sharpe from 1.95 to 1.68 - a 16% haircut at a cost level below MacroHFT's 2 bps and far below FreQuant's 33 to 40. Turnover is never reported, so the haircut cannot be rescaled.</t>
+        </is>
+      </c>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Each agent emits a rationale and the risk agent emits a reason for its level. No formal attribution method.</t>
+        </is>
+      </c>
+      <c r="R20" s="9" t="inlineStr">
+        <is>
+          <t>Accuracy and MCC for forecasting; cumulative return, Sharpe, max drawdown and Calmar for trading. Nine baselines including momentum, mean reversion, ALSTM, Informer, StockNet, PPO, CoT, FinMem and FinCon, plus Markowitz and DQN for the portfolio task. All LLM methods run on GPT-4o-mini for fairness.</t>
+        </is>
+      </c>
+      <c r="S20" s="9" t="inlineStr">
+        <is>
+          <t>Highest accuracy and MCC on all four assets - 58.97% to 61.56% accuracy against a best-baseline field of 56.1 to 58.8, with MCC of 0.16 to 0.20 against 0.05 to 0.18. Real improvement, still under 62% on a binary next-day call. Cumulative returns of 32.45% to 58.74% with Sharpe 1.62 to 2.25, best in both columns everywhere, but FinHEAR never posts the lowest drawdown on any asset, so the risk mechanism is buying return per unit of risk rather than reducing risk. The portfolio result is the largest in the paper at 83.89% return with Sharpe 3.28, and removing adaptive risk-awareness costs 47.7 points there against 14.5 on AAPL, so the sizing mechanism matters far more at portfolio level. It stays profitable through the 2023 rate-hike downtrend at 7.82% while every baseline is negative, which is the most convincing robustness evidence in the paper.</t>
+        </is>
+      </c>
+      <c r="T20" s="9" t="inlineStr">
+        <is>
+          <t>One test year, one split, no repeated runs, no significance testing, and the architecture has a Beta draw inside the sizing rule so run-to-run variance is built in. The results tables disagree with each other on three of four assets and every disagreement favours the headline - TSLA reads 48.74/35.21 in one table against 58.74/25.21 in another, and gold's Calmar is only reachable from the appendix drawdown, which means the main table's figure cannot be right. The thresholds that operationalise prospect theory are selected on the test window and the resulting optimum is then read as theoretical confirmation. The behavioural grounding is asserted at the level of functional form, which the Limitations section concedes.</t>
+        </is>
+      </c>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>Continuous position sizing driven by a risk state is the mechanism I'm taking, and the multiplicative form - confidence times source reliability times precedent similarity - is decomposable enough that each factor can be swapped, which makes it a template rather than a result. The threshold rule gives me an abstention path, which is a requirement rather than a refinement on a market where many tickers will have one weak signal or none on a given day. And the event-centric routing suits the CSE better than the price-centric designs, because a design whose dominant input is dated text rather than a decade of bars is the one that survives if data depth turns out short.</t>
+        </is>
+      </c>
+      <c r="V20" s="9" t="inlineStr">
+        <is>
+          <t>Replacing the sampled risk sensitivity with a measured volatility-state estimate is the obvious substitution and it's the cleanest experiment I have for showing the econometric layer earns its place rather than arguing it from theory. The expert knowledge base doesn't transfer - there's no Sri Lankan investor canon in English or Sinhala, and lifting Buffett and Graham wholesale imports reasoning calibrated to deep, heavily disclosed markets into a thin one. And if the sizing mechanism only pays at 5 bps, it isn't the mechanism I want, which I'd rather find out on their architecture than on mine.</t>
+        </is>
+      </c>
+      <c r="W20" s="9" t="inlineStr">
+        <is>
+          <t>[[FinHEAR, Human Expertise and Adaptive Risk-Aware Temporal Reasoning for Financial Decision-Making]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>P20</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Yu, Li, Chen, Jiang, Li, Zhang, Liu, Suchow &amp; Khashanah (Stevens Institute of Technology)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>arXiv 2311.13743v2. Code released</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>FinMem / FinMe | arXiv:2311.13743</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Single LLM trading agent with layered memory</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>DRL trading agents are opaque and cannot use text; existing financial LLM systems are QA systems rather than sequential agents with no ability to memorise influential messages; and the general-purpose agent architecture it borrows from applies one decay rate to everything, so it cannot tell daily news apart from quarterly and annual reports.</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>US equities. Five tickers selected for having the highest volumes of accessible news text, ranging from about 1,600 to 6,800 articles each.</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>15 August 2021 to 25 April 2023, training roughly fourteen months and testing six, chosen so at least one full filing cycle falls inside training. Daily OHLCV from Yahoo Finance, news from the Alpaca News API, filings from SEC EDGAR.</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>News text, 10-Q and 10-K insights, and the agent's own reflections. FAISS vector store with OpenAI embeddings.</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>Three modules - profiling (professional background plus one of three risk inclinations), memory (working memory plus a three-layer long-term store), and decision (Buy, Sell or Hold on a single share). No gradient training anywhere; the training phase makes no investment decisions and exists only to accumulate hindsight-labelled reflections.</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>Single agent, no orchestration. Worth noting as the ancestor of FinCon and FinAgent.</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>None as a model. Sentiment is whatever the LLM infers while summarising.</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>10-Q and 10-K insights are summarised into the intermediate and deep memory layers. No structural chunking.</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>The 'self-adaptive' character is far simpler than its name suggests: it flips to risk-averse when cumulative return falls below zero within about three days and back when it turns positive. So the whole regime-detection apparatus is a sign test on a three-day return - which is the floor my volatility work has to clear, not a strawman.</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr">
+        <is>
+          <t>None at all. Cumulative return is a plain sum of daily log returns signed by the action, over a single share, so it's a direction-prediction score wearing a trading metric's clothes. No cost term, no spread, no slippage, no position size, and turnover is never reported.</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>THE CLEANEST INSTANCE IN MY SET. Immediate reflection returns the direction, the rationale and the IDs of the highest-influence events from each of the three memory layers, so every decision arrives with citations into a store whose provenance is known by construction - a news item, a 10-Q insight or a prior reflection. That's an attributable explanation with no extra instrumentation, and it decomposes by information horizon.</t>
+        </is>
+      </c>
+      <c r="R21" s="9" t="inlineStr">
+        <is>
+          <t>Cumulative Return, Sharpe, daily and annualised volatility, Max Drawdown, averaged over five repeated trials with Wilcoxon signed-rank against the second-best model. Baselines: buy-and-hold, PPO, DQN, A2C, Generative Agents and FinGPT.</t>
+        </is>
+      </c>
+      <c r="S21" s="9" t="inlineStr">
+        <is>
+          <t>Best CR and Sharpe on all five tickers, but the margin is wildly uneven - +28.4 points on TSLA and +31.5 on COIN, against +0.94 points on NFLX over buy-and-hold across six months. The cognitive-span result is the headline contribution and its own table complicates it: response across top-K is non-monotonic, with Top 3 well below Top 1, and best return and Sharpe both belonging to Top 10 while the recommended operating point is Top 5. The backbone comparison is the finding that matters most to me - GPT-4 reaches 62.62% cumulative return, GPT-3.5-Turbo 16.15%, davinci-003 1.63%, and Llama2-70b-chat -52.72% with Sharpe -2.85. The self-adaptive character beats both static ones by 67 and 74 points on the TSLA ablation.</t>
+        </is>
+      </c>
+      <c r="T21" s="9" t="inlineStr">
+        <is>
+          <t>Section 5.1 states plainly that the reported outcome is whichever of three risk inclinations achieved the highest cumulative return during the TESTING period, so every headline number is a maximum over three configurations selected with the answer visible, against baselines contributing one each. The test window sits inside the backbone's pretraining data on five of the most heavily covered US tickers, and nothing measures that confound. The layering itself is never ablated - there is no single-layer FinMem anywhere in the paper, so the central contribution has no evidence that it does anything. The ablation tables are internally inconsistent and all three pivot on one shared run on one ticker.</t>
+        </is>
+      </c>
+      <c r="U21" s="9" t="inlineStr">
+        <is>
+          <t>Per-source decay is the piece I'm taking, and the constants have to be re-derived rather than copied - a 14-day shallow-layer constant assumes a daily news flow, and a CSE ticker going three weeks without a story would see its shallow layer purge itself to empty while one annual report does all the work. Making the layer constant a function of the observed arrival rate for that ticker and source is a defensible small contribution costing one estimator. Six months to a year of daily data being enough for this architecture also reorders my build: the retrieval-and-memory layer is viable at almost any depth, so it goes first and the RL component is conditional on what the archive holds, which means a working system exists even in the bad case.</t>
+        </is>
+      </c>
+      <c r="V21" s="9" t="inlineStr">
+        <is>
+          <t>There's no abstention path and no floor below which a layer contributes nothing, so with too few shallow-layer events top-K retrieval returns whatever is left regardless of score and the agent reasons confidently over stale news. Backbone dependence is a hard blocker for me specifically: the architecture returns -52.72% on the one open-weight model tested, and since Sinhala and code-mixed content is a first-class requirement, the model handling that input is unlikely to be the strongest reasoner available.</t>
+        </is>
+      </c>
+      <c r="W21" s="9" t="inlineStr">
+        <is>
+          <t>[[FinMe, A Performance-Enhanced LLM Trading Agent With Layered Memory and Character Design]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="150" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>P21</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Zhang, Zhao, Xia, Sun et al. (NTU Singapore, NUS, Zhejiang, SMU, Skywork AI)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>KDD 2024</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>FinAgent</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Multimodal single-agent foundation model for financial trading</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>States five challenges: insufficient multimodal data processing, imprecise information retrieval, adaptability in rapidly evolving markets, integration of domain knowledge, and reasoning for actions. Positions itself in the space between financial QA and sequential trading.</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>US equities plus one crypto pair. Five megacaps and ETHUSD, with between 2,611 and 10,076 news items per asset over 398 trading days - roughly 20 to 25 items per asset per trading day.</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>1 June 2022 to 1 January 2024, train to 1 June 2023 and a seven-month test window. Prices and news from Financial Modeling Prep, expert guidance from Seeking Alpha at 393 to 600 items per stock, visual data plotted with pyecharts.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Numerical, textual and visual. Kline charts and trading charts fed to GPT-4V. Each news item classified on duration of effect and sentiment.</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>Five modules executed in a numbered order per trading day: market intelligence, memory, low-level reflection, high-level reflection, and a tool-augmented decision maker. Formulated as a fully observable MDP with no justification, against the POMDP consensus. There is no optimiser despite the notation - prompts are fixed, nothing is trained, and the argmax is decorative.</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>SINGLE AGENT WITH MODULES, not multi-agent - and that's why it's useful to me. Auxiliary 'agents' are three rule-based strategies (MACD Crossover, KDJ with RSI Filter, Mean Reversion) each contributing a decision plus an explanation into the final prompt. Their influence is fixed.</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>A field the LLM fills in while summarising, POSITIVE/NEGATIVE/NEUTRAL per news item, in English, from institutional sources. No sentiment model.</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>Diversified retrieval is the real contribution: memory is queried by M distinct retrieval types rather than one similarity search, so top-K retrieval yields an M x K set with each item tagged by the query intent that found it, and a dedicated query field is generated alongside every summary so the artefact written for the decision is never the retrieval key.</t>
+        </is>
+      </c>
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>Risk is measured and never controlled. MDD, VOL, SOR and CR are all reported as evaluation metrics and none of them feed back into the decision. There is no risk trigger, no exposure cap, and the trader preference is a static string in the prompt set once.</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr">
+        <is>
+          <t>A commission fee appears once in the MDP formulation and no cost parameter appears anywhere in the experimental setup - no slippage, no liquidity constraint, no turnover penalty. The friction is acknowledged in the formulation and absent from the numbers.</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Chain-of-Thought reasoning emitted as a required output field, and retrieved evidence tagged with the intent that found it, which gives an attributable retrieval trail per decision at no extra cost. No formal attribution method.</t>
+        </is>
+      </c>
+      <c r="R22" s="9" t="inlineStr">
+        <is>
+          <t>Six metrics - ARR, Sharpe, Volatility, MDD, Calmar, Sortino. Twelve baselines across rule-based, ML/DL, RL and LLM categories, though the paper's own count disagrees with itself across sections. Sharpe is computed with a zero risk-free rate in a 5% rate environment, which inflates every figure in the table including the baselines'.</t>
+        </is>
+      </c>
+      <c r="S22" s="9" t="inlineStr">
+        <is>
+          <t>Highest ARR and Sharpe on all five stocks, and it loses to FinMem on ETHUSD on all three headline metrics. The abstract's '92.27% return, 84.39% relative improvement' is TSLA alone against the best single baseline on that asset; the average improvement of over 36% is the figure to quote. LGBM on AAPL gets Sharpe 1.47 against FinAgent's 1.43 with drawdown of 2.52% against 10.4%, so a gradient boosted tree on price features beats the multimodal foundation agent on risk-adjusted return with a quarter of the drawdown. The ablation prose contradicts its own table: low-level reflection does essentially nothing on TSLA (39.01 to 39.27) and makes drawdown worse, while the gains the text attributes to it belong to the high-level module.</t>
+        </is>
+      </c>
+      <c r="T22" s="9" t="inlineStr">
+        <is>
+          <t>Single asset only, no portfolio, no allocation. No costs or liquidity anywhere despite the formulation. No risk control in the loop. One test window, seven months, six assets of which five are correlated US tech megacaps over a period when that sector rallied hard, with no walk-forward, no repeated splits, no significance test and no seeds. Single backbone, so architecture versus model is unresolved. 'Generalist' is not supported - it generalises across five same-sector US stocks and fails on the one asset outside that class.</t>
+        </is>
+      </c>
+      <c r="U22" s="9" t="inlineStr">
+        <is>
+          <t>Split retrieval from reasoning, and never retrieve against the artefact written for the decision - the single most transferable idea in the paper and it applies to the document RAG pipeline as much as to agent memory. Tag retrieved evidence with the intent that found it, which is cheap and gives the decision layer something to weigh. The XML-over-JSON detail and the modular HTML template structure save a week of prompt plumbing.</t>
+        </is>
+      </c>
+      <c r="V22" s="9" t="inlineStr">
+        <is>
+          <t>THE STRONGEST EMPIRICAL MOTIVATION I HAVE FOR THE MAIN GAP. The auxiliary strategies are calibrated to US large-cap daily dynamics, and dropping them onto an asset that trades differently made things actively worse than doing nothing - used alone on ETHUSD they return 16% against buy-and-hold's 29%. The system has no mechanism to notice this or adapt, because their influence is fixed. On the CSE, where turnover is thin and whale-driven, I should assume the same strategies transfer badly, and the ability to down-weight a component that has stopped working is exactly what's missing. It's also the argument against the single-agent-with-modules design generally.</t>
+        </is>
+      </c>
+      <c r="W22" s="9" t="inlineStr">
+        <is>
+          <t>[[A Multimodal Foundation Agent for Financial Trading, Tool-Augmented, Diversified, and Generalist]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="150" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>P22</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Nanayakkara, Wanniarachchi &amp; Vidanagama (General Sir John Kotelawala Defence University)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>2021 5th SLAAI International Conference on Artificial Intelligence. DOI 10.1109/SLAAI-ICAI54477.2021.9664735</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>DOI 10.1109/SLAAI-ICAI54477.2021.9664735</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>CSE portfolio management platform with price prediction</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>The CSE offers no first-party portfolio management platform with prediction capability, so an investor revalues holdings, re-applies a sector selection rule and computes returns manually through a broker or brokerage portal. The paper also frames broker intermediation itself as the risk, citing SEC filings against four broking firms and the 2011 Radiant Gems share price manipulation.</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange - nominally. This is the closest thing in my set to a direct predecessor, and the only paper I have that builds a CSE-facing portfolio system rather than a model.</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Requirements from semi-structured interviews with CSE officials including the head of R&amp;D, head of Public Relations and the CIO, plus a 17-question survey of 233 investors. Market data from the Pandas Yahoo Finance reader on a rolling three years, and from the Tiingo API from 2016. NEITHER SOURCE CARRIES COLOMBO-LISTED EQUITIES.</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>Adjusted Close as the single input series for the long-term model; close only for the short and mid term model.</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>Prediction split by horizon, which is the one genuinely reusable design decision: a stacked LSTM for 1 to 7 days and 15 to 30 days, and geometric Brownian motion for anything longer, on the reasoning that a stochastic process is the appropriate tool once the sequence signal has decayed. Frontend React, backend PHP, MySQL, hosted on Azure with both models deployed through Azure ML Studio.</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>N/A - not an agent system.</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>Geometric Brownian motion assumes constant drift, constant volatility and log-normal returns, estimated over a rolling three years. That is exactly the assumption the CSE long-memory and ARMA-GARCH findings argue against, and the paper never tests it or compares against a GARCH-family alternative.</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t>None. No transaction costs, no brokerage fees, no liquidity or thin-trading treatment, no price band handling, and no rebalancing or allocation logic anywhere - so despite 'adaptive' in the title there is no optimisation, no risk model and no allocation decision in it.</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>The forecast is a line on a chart with no reasoning attached.</t>
+        </is>
+      </c>
+      <c r="R23" s="9" t="inlineStr">
+        <is>
+          <t>Twelve functional test cases scored 92% to 100%, self-assessed, with user acceptance testing by the author and senior CSE officials rather than by any of the 233 surveyed investors. Percentage difference between one realised and one predicted price. No baseline of any kind.</t>
+        </is>
+      </c>
+      <c r="S23" s="9" t="inlineStr">
+        <is>
+          <t>The only quantitative forecasting evidence is three percentage differences from the Brownian motion model and they range widely - Microsoft 4.88%, Nike 12.1%, Apple 18.51% - from which the paper concludes 'more than 80% accuracy' in the results section while the abstract claims more than 85%. No error metric of any kind is reported for the paper's own LSTM, and the RMSE figures it does quote belong to a NIFTY 50 study in its literature review, not to the system it builds. The durable contribution is the requirements set, which came out of 233 investor responses and interviews with the exchange.</t>
+        </is>
+      </c>
+      <c r="T23" s="9" t="inlineStr">
+        <is>
+          <t>The title claims the Colombo Stock Exchange and the evaluation never touches it - every reported number comes from AAPL, MSFT or NKE. Percentage difference between one realised price and one predicted price is not a forecasting metric: no stated test window, no out-of-sample discipline, no naive baseline, no per-horizon breakdown. The LSTM is not reproducible (no layer count, hidden units, lookback window or split dates) and not evaluated, even though it serves the horizons an investor actually trades on. Test scores are self-assessed with no stated rubric.</t>
+        </is>
+      </c>
+      <c r="U23" s="9" t="inlineStr">
+        <is>
+          <t>CRITICAL FOR MY DATA ACCESS QUESTION: the paper states the CSE data endpoint was 'officially provided by CSE to fulfill the current development purposes', which is evidence that a written request from a university project has been granted before, and the interviews name the roles to approach. I should make that request in writing early, ask about retention depth and reuse terms in the same letter, and keep archiving daily in parallel. The 233-respondent requirement set also saves me a full elicitation round on the generic features, so my own elicitation can spend its budget on what's specific to my build.</t>
+        </is>
+      </c>
+      <c r="V23" s="9" t="inlineStr">
+        <is>
+          <t>This is my prior-art citation for the platform claim and the reason I should not repeat that claim in the same form - the honest framing is that a CSE-targeted platform was proposed in 2021, accepted at the demonstration level, and its forecasting component was never validated on Colombo-listed equities, which leaves the substantive question open rather than settled. The gap between 85% claimed and 18.51% observed on a single stock is the concrete argument for fixing the evaluation protocol before writing any model code.</t>
+        </is>
+      </c>
+      <c r="W23" s="9" t="inlineStr">
+        <is>
+          <t>[[Adaptive Stock Market Portfolio Management and Stock Prices Prediction Platform for Colombo Stock Exchange of Sri Lanka]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="150" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>P23</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Dinushan &amp; Wijegunasekara (University of Kelaniya)</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>2024 4th International Conference on Advanced Research in Computing (ICARC), pp. 61-66. DOI 10.1109/ICARC61713.2024.10499774</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>DOI 10.1109/ICARC61713.2024.10499774</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>CSE index forecasting with macro indicators and sentiment</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>Existing CSE prediction work is company-level, daily, and fed on past prices; sentiment has been used locally but attached to specific companies rather than to the market; and the Sri Lankan macro literature stops at correlation without anyone folding the variables into a predictive model. Claims the bridge between those.</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Colombo Stock Exchange. Predicts ASPI and S&amp;P SL20 separately.</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Monthly, January 2010 to December 2022, 156 rows per index, from investing.com. Nine Sri Lankan macro series from CBSL and tradingeconomics, the S&amp;P 500 as a global proxy, and a Twitter sentiment score. The test partition is 39 months.</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>AWLR, exports, USD exchange rate, broad money M2b, currency in circulation, tourist earnings, unemployment, industrial production and CPI. Sentiment scored with a Transformers RoBERTa model selected over TextBlob, Vader and Flair on a Kaggle test set.</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>Feature selection in three stages - correlation at a one-month lag, a per-variable lag sweep keeping the argmax, then forward stepwise regression and p-value pruning - followed by six model families (Decision Tree, Random Forest, SVR, ANN, CNN, multivariate LSTM) on a 75/25 split, run under both shuffled and non-shuffled regimes.</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>THE SENTIMENT VARIABLE IS ONE TWITTER ACCOUNT - the 'Financial Chronicle' handle, scraped with SNScrape. So what the paper calls Sri Lankan market sentiment is the editorial tone of a single English-language financial publisher, not investor sentiment, and nothing in it is Sinhala or Tamil. Monthly aggregation is described only as 'scores aggregated', with no statement of whether that's a sum or a mean and no normalisation by tweet volume.</t>
+        </is>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="O24" s="9" t="inlineStr">
+        <is>
+          <t>None. Correlations are computed on non-stationary levels with no differencing, unit root test or cointegration check.</t>
+        </is>
+      </c>
+      <c r="P24" s="9" t="inlineStr">
+        <is>
+          <t>None. No counters, no volumes, no spreads and no costs anywhere.</t>
+        </is>
+      </c>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Linear stepwise regression coefficients are interpretable, but the deep models are not examined.</t>
+        </is>
+      </c>
+      <c r="R24" s="9" t="inlineStr">
+        <is>
+          <t>Mean absolute error in raw index points, and nothing else. No baseline, no significance test.</t>
+        </is>
+      </c>
+      <c r="S24" s="9" t="inlineStr">
+        <is>
+          <t>The two indices are driven by visibly different things and this is the result I'd keep: the ASPI retains lending rate, exports, exchange rate, broad money, currency in circulation, the S&amp;P 500 and sentiment, while the S&amp;P SL20 retains only sentiment, unemployment, industrial production and tourist earnings, with every monetary variable failing to clear on it. Sentiment is the only variable surviving for both, and it is the weakest surviving correlate for the ASPI and the strongest for the SL20. Monetary variables lead the ASPI by four to six months, which no correlation-only local study reports. Shuffling dominates every comparison by factors of three to five, and the paper reports this as a design recommendation.</t>
+        </is>
+      </c>
+      <c r="T24" s="9" t="inlineStr">
+        <is>
+          <t>Shuffling a monthly index series before splitting is look-ahead leakage - with 156 consecutive months randomly assigned, a test month sits between two training months one step away on a strongly autocorrelated level series, so the model interpolates rather than forecasts and the reported improvement is the size of the leak. The multivariate LSTM shows this indirectly: it's the one model with no shuffled score because shuffling destroys the sequence it consumes, and it's also the best non-shuffled performer. Feature selection runs on the full sample, which leaks a second time. Every correlation is on non-stationary levels over a sample ending in the 2022 currency collapse. There is no baseline of any kind, so an MAE of 705.98 has nothing to be measured against - persistence is one line and it isn't on the page.</t>
+        </is>
+      </c>
+      <c r="U24" s="9" t="inlineStr">
+        <is>
+          <t>The lag structure is a reusable prior for my macro feature block once re-estimated properly - AWLR at six months, M2b and currency in circulation at five, exchange rate at four, exports and CPI and the S&amp;P 500 at one. The ASPI against S&amp;P SL20 divergence also tells me where the sentiment layer earns its keep: if sentiment is the strongest surviving correlate for the large-cap index and the weakest for the broad one, my sentiment component should be evaluated on liquid large caps and my macro component against the broad index, reported separately rather than as one headline.</t>
+        </is>
+      </c>
+      <c r="V24" s="9" t="inlineStr">
+        <is>
+          <t>This is the concrete local example that pins the no-shuffle rule into my protocol before I write model code, and it moves feature selection inside the training fold. It's also the clearest statement I have of the resource gap my own work claims: one English-language publisher's feed is a news-tone proxy, not investor sentiment, and nothing in it is Sinhala. Together with the 2021 CSE platform paper this is the second CSE-facing paper in my set where an unbenchmarked error figure carries the conclusion.</t>
+        </is>
+      </c>
+      <c r="W24" s="9" t="inlineStr">
+        <is>
+          <t>[[Machine Learning-Driven Sri Lankan Stock Market Prediction, Harnessing Economic Indicators and Sentiment Analysis]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="150" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>P24</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Lahmiri &amp; Bekiros</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Chaos, Solitons and Fractals 151, 111221</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Chaos, Solitons and Fractals 151 (2021) 111221</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Long memory in returns and volatility across markets under COVID-19</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>Long memory had been documented separately in returns and separately again in volatilities, but not estimated before and during COVID-19 as a paired comparison; crypto and equity markets are usually studied in isolation; and most studies estimate persistence in the mean or the variance, not both within one specification.</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>45 cryptocurrency markets and 16 international equity indices. No frontier market anywhere in the cross-section.</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Daily closes from Yahoo Finance, split into a pre-pandemic window (September to December 2019) and a pandemic window (January to April 2020). Stated as 123 and 120 observations, but those are calendar days - the equity series only have trading days, so the equity estimates rest on about seventy observations per window.</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>Log returns. The unit of analysis is the cross-section of fitted fractional differencing parameters, 45 from crypto and 16 from equities per window.</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>A single integrated ARFIMA-FIGARCH specification, with the mean equation carrying return memory and the variance equation carrying volatility memory, estimated by quasi-maximum likelihood. Cross-sections compared with t-tests and F-tests.</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="N25" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t>THE WHOLE PAPER. Return persistence rose in both categories during the pandemic window, and the volatility side moves far more - median d near 0.02 for crypto and 0.05 for equities pre-pandemic, jumping to roughly 0.74 and 0.81 during. Taken at face value that says volatility in both asset classes had almost no long memory in late 2019 and a great deal by April 2020, which sits awkwardly against the wider literature reporting persistent volatility memory in normal periods.</t>
+        </is>
+      </c>
+      <c r="P25" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Fully parametric, but no per-market estimates are tabulated anywhere.</t>
+        </is>
+      </c>
+      <c r="R25" s="9" t="inlineStr">
+        <is>
+          <t>One-sided and two-sided t-tests for equality of means and F-tests for equality of variances across the fitted parameter cross-sections. No baseline models.</t>
+        </is>
+      </c>
+      <c r="S25" s="9" t="inlineStr">
+        <is>
+          <t>Return memory doesn't distinguish crypto from equities in either window (equality tests at 0.9667 before and 1.0000 during), which is the cleanest result in the paper. But two of the four headline conclusions invert the paper's own tables - the text reads each set of one-sided tests by picking the row with the LARGEST p-value as the supported claim, which reverses the usual convention, so the stated conclusions about dispersion increasing and about crypto volatility being more persistent are both contradicted by the numbers as printed. What survives is the direction, not the contrasts.</t>
+        </is>
+      </c>
+      <c r="T25" s="9" t="inlineStr">
+        <is>
+          <t>The windows are too short for the estimator - seventy to a hundred and twenty observations against a literature that typically works with thousands - and no standard errors or confidence intervals are reported on any individual estimate, so there's no way to tell how much of the cross-sectional shift is estimation noise. Most estimates sit above 0.5, which by the paper's own stated criterion means the series is nonstationary and the specification doesn't apply, with no stationarity testing reported. Nothing here is reusable as a number: no model orders, no selection criteria, no residual diagnostics, no per-market estimates. And the pandemic window is dominated by the March 2020 selloff, so any shock of that magnitude would raise measured persistence regardless of cause.</t>
+        </is>
+      </c>
+      <c r="U25" s="9" t="inlineStr">
+        <is>
+          <t>The before-and-after design is worth borrowing for the CSE risk component with one obvious correction: windows have to be long enough for the estimator to mean something, and the CSE FIGARCH paper's regime split into periods of years rather than months is the template. The more transferable idea is the unit of analysis - estimating persistence across a cross-section of tickers and testing the distribution rather than reading one index, which would let me ask whether volatility memory is a market-wide property or concentrated in the illiquid tail. Volatility persistence moving sharply under a shock while return persistence barely moves is also a useful prior: if I'm conditioning position sizing on a memory parameter, the volatility side is where the signal lives.</t>
+        </is>
+      </c>
+      <c r="V25" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTANT SELF-CHECK ON MY OWN ARGUMENT. Return persistence is statistically indistinguishable between crypto and equities, and if a memory parameter doesn't separate two asset classes as different as Bitcoin and the Nikkei, it isn't going to separate the CSE from developed markets either. So the case for building something CSE-specific has to rest on liquidity, microstructure and the sentiment-language problem, not on the persistence parameter being unusual here. Also: this is another long-memory paper that measures the parameter, tests whether it changed, and stops, with no forecasting model and no allocation rule built on top - which is the pattern across this whole corner of the literature.</t>
+        </is>
+      </c>
+      <c r="W25" s="9" t="inlineStr">
+        <is>
+          <t>[[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="150" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Senevirathne, Demotte, Karunanayake, Munasinghe &amp; Ranathunga (University of Moratuwa)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>arXiv preprint 2011.07280v1. Code, embeddings and annotated data released publicly</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>arXiv:2011.07280</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Sinhala sentiment analysis with deep learning</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Sinhala is morphologically rich and under-resourced, and the two compound: no publicly available sentiment lexicons, no usable POS taggers, and no pretrained contextual model, so the auxiliary linguistic knowledge that carries English sentiment analysis is simply unavailable. The only prior annotated dataset is small, single-source and binary.</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Sri Lanka. Sinhala news comments from Lankadeepa and GossipLanka, covering politics, sports, crime, economy, society and culture. NOT financial text.</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>15,059 annotated comments, 9,059 re-annotated from prior work plus 6,000 newly crawled, covering 2016/06 to 2020/05. Plus a 9.48 million token unannotated corpus (16,840 articles and comments) used solely to train the embeddings. Three annotators, 7,000 comments double-annotated, Cohen's kappa 0.65.</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>Four classes - POSITIVE, NEGATIVE, NEUTRAL and CONFLICT, where CONFLICT is a comment carrying both positive and negative opinion at once. Class distribution is heavily skewed: NEGATIVE 50.9%, NEUTRAL 20.5%, POSITIVE 16.0%, CONFLICT 12.7%.</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>Fourteen configurations in four groups - vanilla sequence models, CNN hybrids, stacked LSTM/BiLSTM, and recent architectures including hierarchical attention and capsule networks - all sharing an embedding layer initialised from fixed 300-dimension fastText vectors. 10-fold cross validation for the model comparison, 80/20 holdout for the preprocessing and embedding experiments.</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>N/A.</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>THE WHOLE PAPER, and the foundational resource for the Sinhala side of my sentiment component. fastText beats Word2Vec at every one of the nine dimensions tested, which on a morphologically rich language is the expected direction - subword composition shares parameters across inflected forms and produces vectors for words never seen in training.</t>
+        </is>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="P26" s="9" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="Q26" s="9" t="inlineStr">
+        <is>
+          <t>None. No attribution method, and the paper predates the explainability work.</t>
+        </is>
+      </c>
+      <c r="R26" s="9" t="inlineStr">
+        <is>
+          <t>Weighted accuracy, precision, recall and F1 across the four classes. NO BASELINE OF ANY KIND appears, and the obvious one is close - always predicting NEGATIVE scores roughly 51% against the best model's 63.23%.</t>
+        </is>
+      </c>
+      <c r="S26" s="9" t="inlineStr">
+        <is>
+          <t>Fourteen architectures spanning four generations of design land within three points of each other, between 61.16% and 63.81% accuracy, and that flatness is the finding: on this dataset the architecture is not the binding constraint, the data is. Punctuation handling is the cleanest small experiment - stripping everything except the question mark lifts holdout accuracy from 58.57% to 63.35%, because question marks in Sinhala news comments are mostly attached to negative sentiment. The confusion matrix is where the real result lives: per-class recall is 91.8% for NEGATIVE but 21.8% for NEUTRAL and 12.2% for CONFLICT, with 70.8% of actual CONFLICT comments predicted NEGATIVE. Macro-F1 recomputes to 48.2% against the reported weighted F1 of 59.3%.</t>
+        </is>
+      </c>
+      <c r="T26" s="9" t="inlineStr">
+        <is>
+          <t>The model has largely learned to predict the majority class and the weighted metrics hide it - the two classes the paper introduced as its contribution are the two it classifies worst, and that gap appears nowhere in the headline. The paper's own best-model claim isn't supported by its own table on either metric. Treating annotator kappa as an accuracy ceiling is a conflation that does a lot of unearned work in the discussion, and the cheap test - measuring accuracy on the subset where both annotators agreed - is available in their own data and never run. Non-Sinhala unicode is stripped during preprocessing, so romanized Sinhala and code-mixed comments are mangled rather than classified, at a proportion never reported.</t>
+        </is>
+      </c>
+      <c r="U26" s="9" t="inlineStr">
+        <is>
+          <t>This is the corpus, the embeddings and the preprocessing I start from, not a method to reimplement - and the licence is public. It sets the honest pre-transformer baseline my own numbers have to beat, 63% weighted accuracy and 59% weighted F1 on four-class Sinhala, with the explicit note that BERT was ruled out here for lack of a pretrained Sinhala model, which gives me a defensible arc to the 88.4% XLM-R plus lexicon result rather than a bare assertion that transformers are better. Keep the question mark and drop the rest. And macro-F1 with a per-class breakdown goes into my results table as a fixed column, because weighted accuracy never travels alone.</t>
+        </is>
+      </c>
+      <c r="V26" s="9" t="inlineStr">
+        <is>
+          <t>CONFLICT is the class I actually need and the one this paper handles worst - bullish-on-counter, bearish-on-market is the normal shape of CSE commentary, and a flat four-way softmax collapses it into NEGATIVE seven times out of ten here, so mixed sentiment needs aspect-level decomposition rather than a fourth label. The domain gap is the contribution boundary: news-portal comments about politics and crime are not financial text, there is no market data attached to any comment, and no downstream task beyond classification is attempted, so nothing here speaks to whether Sinhala sentiment carries return information on the CSE.</t>
+        </is>
+      </c>
+      <c r="W26" s="9" t="inlineStr">
+        <is>
+          <t>[[Sentiment Analysis for Sinhala Language using DeepLearning Techniques]]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W16"/>
+  <autoFilter ref="A1:W26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2408,205 +3589,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Literature Survey Matrix - CSE Multi-Agent Framework</t>
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Literature Survey Matrix - CSE Multi-Agent Framework (v2, 25 papers)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
+      <c r="A2" s="11" t="inlineStr"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>15 papers from the Research Papers Grid (Gugsi's recommendations), one row each. Content is written from my own literature review notes in the vault.</t>
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Grew from 15 to 25 rows. Ten papers added (P16-P25) from the vault's Literature Reviews folder, and P04 (AlphaAgents) rewritten against the expanded note. Column structure unchanged at 23.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr"/>
+      <c r="A4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Where each cell came from</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Judgement columns - Problem &amp; Objective, Limitations, What I'm Taking From It, Gap It Leaves For Me - are from my own review notes.</t>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>New rows, shaded light blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>P16 MacroHFT - KDD '24. THE PAPER THE MAIN GAP MUST BE DEFENDED AGAINST. Hyper-agent conditioned on trend and realised volatility emits a softmax mixture over six DDQN sub-agents. This is state-aware orchestration and it already exists.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Bibliographic columns - Citation, Year, Venue/Type, Link/DOI - were re-checked against the source papers and corrected where my notes were wrong (see below).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="75" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Some factual detail in Dataset(s) &amp; Period, Evaluation &amp; Baselines and Key Results is NOT in my notes and came from checking the source papers: P01's tickers, test window and performance figures; P02's tickers, split and baseline list; P04's universe and test window; P06's released-sample size and config count; P07's question and filing counts; P12's observation count; P14's forecast horizons. These are second-hand until I confirm them in the PDFs myself - verify before any of them go in the proposal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Pruned from 31 to 23. Merged: Research Problem + Objective; Market + Market Characteristics; Data Modality + Input Features + Pre-processing; Model/Algorithm + Multi-Agent Architecture + Decision/Output; Agents + Orchestration Method; Volatility Handling + Volatility Memory; Liquidity + Trading Friction; Evaluation Metrics + Baselines; Strengths + Relevance to CSE Project (now 'What I'm Taking From It').</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Added: Year, Venue/Type, My Note (link back to the vault review).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Dropped: nothing that carried unique information - everything folded into a merged column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Corrections made against my existing notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>P11 Role of Market Liquidity - my Research Papers Grid says 'Dissanayake &amp; Nanayakkara (2021)'. It is 2025 (IJEFI 15(2), 201-210, published 17 Feb 2025). The data period is 2010-2021, which is probably where the 2021 came from. Also note the journal's own landing page misspells the first author as 'Dissnayake'; the PDF reads Dissanayake.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>P15 Deep RL Framework - the actual title is 'Deep Reinforcement Learning Framework for Diversified PORTFOLIO MANAGEMENT Across Global Equity Markets', not 'Diversified Dynamic Portfolio Allocation'. My vault note filename has the wrong title.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>P12 Modeling Long-Term Volatility Memory - single-authored by Mohamed Ismail Mohamed Riyath. Published 2026 in IIM Ranchi Journal of Management Studies 5(1) 21-45, online-first 2025. Cite as 2026 unless the style guide wants the online-first date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>P05 RL Survey - now formally published: ACM Computing Surveys 57(11), Article 295, pp. 1-51, June 2025. Cite the journal version, not the arXiv preprint.</t>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>P17 FreQuant - KDD '24. Frequency-domain state encoder, top-k selection with a learned cash bias, and the only properly solved fee model in the set (33-40 bps by fixed-point iteration).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>P18 FinCon - NeurIPS 2024. Manager-analyst hierarchy that forbids lateral debate, dual-level risk control on empirical CVaR, belief updates as textual gradient descent. Closest published system on orchestration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>P19 FinHEAR - Findings of EMNLP 2025. The only system where position size is a first-class output, sampled from a hand-set Beta by discrete risk level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>P20 FinMem - arXiv 2023. Three-layer memory with per-source decay rates. Its 'self-adaptive' character is a three-day return sign test, which is the floor the econometric layer has to clear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>P21 FinAgent - KDD 2024. Single agent with five modules. Its ETHUSD failure is the strongest empirical motivation for the main gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>P22 Adaptive CSE Platform - SLAAI-ICAI 2021. The only CSE-facing portfolio system in the set, and its forecasting was never evaluated on a Colombo-listed stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>P23 ML-Driven Sri Lankan Prediction - ICARC 2024. CSE macro plus sentiment, with a shuffled-split leakage problem reported as a design finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>P24 COVID long memory - Chaos, Solitons and Fractals 2021. ARFIMA-FIGARCH across 61 markets, and the source of the most important self-check against Sub-gap 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>P25 Sinhala Sentiment DL - arXiv 2020. The foundational Sinhala corpus, embeddings and pre-transformer baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Why this matters for the supervisor's criticism</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>The judgement that 'the literature search is not yet sufficiently complete' was based on one missed paper. This matrix now covers six SOTA agent architectures (MacroHFT, FreQuant, FinCon, FinHEAR, FinMem, FinAgent) and two additional CSE-specific studies that were not in v1. That is the direct answer, and it is stronger than arguing the point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="75" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>It also changes the argument in your favour on one thing and against you on another. In your favour: FinAgent's ETH result and AlphaAgents' dropped sentiment agent are documented cases of fixed-influence components failing with no mechanism to adapt, which is the motivating evidence the main gap needed. Against you: MacroHFT is closer to state-aware orchestration than the supervisor's note acknowledges, so the main gap has to be worded around it rather than over it.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>P02 FinVision - published at ICAIF '24, DOI 10.1145/3677052.3698688. Cite the ACM version.</t>
-        </is>
-      </c>
+      <c r="A20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Also worth checking in your own notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="75" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>The 'My Findings' table at the bottom of Research Papers Grid.md attributes TradingAgents to 'Sangiorgi &amp; Wharton Initiative (2025)'. It is Xiao, Sun, Luo &amp; Wang. That row also lists a 'B. S. Senarathna et al. (2025)' LSTM study on 4 S&amp;P SL20 companies, linked to the sinhala_sentiment_anlaysis_tallip GitHub repo - that repo is the Senevirathne Sinhala sentiment corpus, which is a different thing entirely, and I could not find the LSTM study it describes. Recommend verifying that row before it goes anywhere near the proposal.</t>
-        </is>
-      </c>
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Still not reviewed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>P03 (Anomaly Detection) and P14 (Market Stress), shaded amber, unchanged from v1. P14's PDF is at bis.org/publ/work1250.pdf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Not yet reviewed</t>
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Corrections carried forward from v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>P11 Role of Market Liquidity is 2025, not 2021. P15's actual title is 'Diversified Portfolio Management'. P12 is single-authored and published 2026. P05 is now ACM Computing Surveys 57(11). P02 is ICAIF '24. The ARMA-GARCH vault note calls TGARCH symmetric; it is asymmetric.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>P03 (Anomaly Detection) and P14 (Market Stress) are marked NOT YET REVIEWED. Their rows are filled from the source papers, not from vault notes, and the 'What I'm Taking From It' cell says so explicitly. Highlighted in amber.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>P14's PDF is at https://www.bis.org/publ/work1250.pdf - it is a BIS working paper, which is why it isn't on Semantic Scholar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>G6 in the Gap matrix leans partly on P14 for the SHAP justification. That citation is marked provisional there until P14 is actually read.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Two things to fix in the vault notes themselves</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>The ARMA-GARCH note (P13) calls TGARCH a symmetric model. It isn't - TGARCH is asymmetric. The matrix records the finding correctly and flags the error; the note should be corrected too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="45" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>The FIGARCH note (P12) records the ASPI vs S&amp;P SL20 divergence qualitatively but not the actual d estimates per regime. Those numbers are needed for the risk agent's calibration in G2, so they need pulling out of the PDF.</t>
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>The 'My Findings' table in Research Papers Grid.md still attributes TradingAgents to 'Sangiorgi &amp; Wharton Initiative' (it is Xiao, Sun, Luo &amp; Wang) and still lists a 'B. S. Senarathna et al. (2025)' LSTM study linked to the Sinhala sentiment repo, which could not be found. Worth fixing before the proposal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 13:10:29
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Literature Survey Matrix.xlsx
+++ b/FYP/Matrices/Literature Survey Matrix.xlsx
@@ -781,7 +781,7 @@
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Sixty trading days, three stocks, one regime, one run, with no repeats, no dispersion, no paired test, and a window chosen by inference budget rather than by what would make the comparison informative. The organisational thesis is never tested: nothing is ablated, so eleven agents across seven role types, the bull-bear debate, the facilitator and the three-way risk team are evaluated as one block, and every baseline is a non-LLM rule. A single-agent LLM baseline would have cost one more run and carried most of the paper's weight. No execution friction of any kind, so 26 % on a zero-cost book is an upper bound rather than a return. The backbone almost certainly saw Q1 2024 and the pipeline look-ahead control cannot distinguish contamination from skill. Debate depth n, temperature and decoding are never stated.</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The trading policy is written into the Prediction agent's prompt - hold 10 % cash, buy on a strong upward trend, sell above 5 % gains, size at 1 to 10 % - so this is a rule-based strategy with an LLM applying it rather than a system that learns one, and every threshold is hand-chosen and none reported as tuned. Three stocks, 145 test days, one strongly bullish regime, one run each, no seeds and no significance test; the paper concedes the uptrend favours passive strategies. The only LLM baseline is copied from FinAgent's publication rather than re-run, so the 17 to 23 point gap cannot be read off the table in either direction. No execution friction, which bites hardest here because partial rebalancing in 1 to 10 % slices is the pattern a realistic cost model erodes first. The multi-modal claim is never tested against the same indicators as numbers.</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>There is no evaluation at all: no precision or recall over labelled alerts, no human comparison, no baseline, no ablation, one series, one run, while the abstract claims improved efficiency, improved accuracy and reduced human intervention. The hard case is conceded and not attempted - a mid-sized move in a lightly covered name with no press coverage, which is exactly what the CSE looks like, and where two of the three experts would abstain. An unconditional z-score over 44 years ignores volatility clustering, so the screen under-flags in calm periods and over-flags in crises, and a threshold of 10 returns only the three largest days in the sample. The experts are less separate than the design implies, since two share web search and the third only compares JSON handed to it, and the obvious single-agent baseline is never run.</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Coverage ends in 2022 against a 2025 publication, which removes the entire LLM-agent literature and means the multi-agent assessment predates the systems I compare against. There is no quantitative synthesis of outcomes anywhere in 167 papers: the classification table counts publications by algorithm and nothing aggregates what those papers reported, so the survey establishes what has been tried and cannot establish what works. The critique section names survivorship bias, forward-looking bias, unbalanced benchmarks and unjustified complexity without counting how many of the 167 exhibit each, so it is citable for the existence of each problem but not its prevalence. Two hundred classifications against 167 papers with the overlap never reported. Selection is Google Scholar plus snowballing with no inclusion criteria or screening counts, so the sample is not reproducible. The lead author is funded by HSBC Asset Management, declared on page one.</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Only 150 of the 10,231 cases are public and they are not stratified by company, year or industry, so every downstream result including the chunking work runs the 150 and carries that sample's uncertainty. Single run, single prompt, no dispersion and no significance test: at 150 cases a 95 % interval on one cell is roughly 8 points and on a difference roughly 11, enough to separate 19 % from 50 % and not enough to separate Llama2's 41 % from GPT-4-Turbo's 50 %, a distinction the paper draws in prose. The retrieval baseline is deliberately naive, one Chroma store with ada-002 and Langchain defaults, no reranking and no described chunking, yet the abstract generalises from it. Dataset integrity issues are named and never quantified, no inter-annotator agreement statistic appears anywhere, and the universe is forty large US filers whose documents are far cleaner than a CSE annual report.</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>141 questions, one run, no dispersion, and the headline margins do not clear sampling error: a 95 % interval on a difference is roughly 11.7 points, so the 4.96-point Q&amp;A gain sits well inside it and the 0.71-point retrieval gain is one question. The authors are evaluating their own commercial product, and the two places where the prose overstates the tables both run the same direction. The cost comparison is one-sided, since the 62,529 against 112,155 chunk efficiency is offset by a vision pass over 11,787 pages plus two GPT-4 calls per chunk that is never quantified. The benchmark was silently reduced to 141 of 150 questions and then compared against FinanceBench's published numbers. No precision@k and no mean reciprocal rank anywhere, so nothing says whether the right chunk arrived first or tenth. Table handling is the most distinctive rule and the least evidenced, with no table-detection accuracy and no table against text answer split.</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="T27" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The lens and the reporting checklist are both author-curated and neither is externally validated: coding was done by one author and reconciled among the authors, with placeholder agreement examples rather than kappa numerics, and the mandatory/recommended designations rest on a pilot over 10 papers resolved by author consensus. A denominator of 19 makes every percentage brittle, so 10.5 % for split protocols is two papers and 5.3 % for cost models is one, and the section-level zeros say no paper in a narrow 19-paper boundary did that thing rather than anything about the field. The audit measures papers while the narrative occasionally slips into measuring systems, which matters when 89 % of the corpus is preprints. Several named frameworks are the authors' own inventions presented in the same register as surveyed evidence. It contains no performance synthesis by design, so it is a citation for why comparisons are unsafe and never for a comparison.</t>
         </is>
       </c>
       <c r="U27" s="3" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="T28" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The expected returns feeding the mean-variance optimiser are LLM outputs with no calibration, and not even three independent ones, since Otto produces all three in a single call over the analysts' prose, so the only data-estimated input is the covariance matrix and exact arithmetic runs over inputs of unknown quality. The allocation is over assets, not agents, and the two coincide only because the mapping is one to one, so the paper never has to combine disagreeing views on the same asset. Three asset classes is a thin basis for a diversification claim and the diversity metrics cannot check it: entropy of 3.13 exceeds the 1.59 bit ceiling over three weights, so both metrics are computed over something the paper never names. No execution friction of any kind on a system that liquidates Bitcoin two days after a 10.22 % decline. Three lambda hyperparameters controlling the risk trade-off are never given values, and every figure is one run at temperature 0.7.</t>
         </is>
       </c>
       <c r="U28" s="11" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="T29" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>RQ2 asks whether coordinated agents beat independent single-agent baselines and the paper never runs that experiment: no single-agent baseline, no two-agent configuration, and the 'w/o RL loop' bar removes the retrieval controller rather than the multi-agent structure. Nothing in the evaluation is externally checkable, since the 0.93 is scored on 2500 team-curated queries with no inter-annotator agreement, no described held-out split and availability only on request, and the selected lambda of 0.6 sits on the boundary of the swept interval, which usually means the optimum lies outside it. The Confidence field is declared in the communication protocol and then appears in no reward term, fusion rule or experiment, so the mechanism most load-bearing for my project is stated in prose and never specified. Homogeneity is acknowledged and left untested, and the local reward is cosine similarity to reference text, which rewards paraphrase rather than correctness.</t>
         </is>
       </c>
       <c r="U29" s="11" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="T30" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The Overall column does not support the reading it invites: the benchmark size is never stated, no episode count, no task distribution and no seeds, so the one and two point gaps ordering the top of the table are uninterpretable without n. Averaging tool match, planning and argument accuracy also weights three unlike failures equally, when a wrong tool is visible and a wrong argument or timestamp is not. The instructions and the gold traces are both LLM-generated by the same process, and the evaluated models include the same families. PMB simulates the brokerage, not the market: order sizes of 100 AAPL and 200 TSLA never strain liquidity, and impact, partial fills and queue position are absent. The reproducibility claim is undercut by licensing, since the corpus cannot be redistributed and two labs are only running the same benchmark if both hold the NASDAQ, MASSIVE and BENZINGA subscriptions.</t>
         </is>
       </c>
       <c r="U30" s="11" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The comparison that would isolate the weighting stage is not run: both ablations remove an agent from selection, neither removes the MLP, so nothing shows what an equal-weighted combination of the same twelve alphas would return and there is no evidence the learned weights add anything over the selection. No significance tests, seeds or intervals anywhere, so 53.17 % against 22.47 % is a single backtest. Look-ahead exposure is structural: GPT-4o is asked to pick factors for a 2023 test window from published alpha research inside its own training corpus, with no contamination check. Internal inconsistencies are frequent, with the seed alpha count 100 against 37, Sharpe 1.73 against 1.94 and the benchmark return -11.73 % against -13.22 %. The composite information coefficient is negative at -0.0587 and the sign convention is never given. Multimodality is tabulated and never used.</t>
         </is>
       </c>
       <c r="U31" s="3" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="T32" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>There is no review protocol, so coverage cannot be checked: no search strategy, databases, query strings, inclusion criteria or screening counts, which means the taxonomy over thirty-one systems cannot be distinguished from the authors' reading list and an empty cell cannot be read as a gap in the field. Nothing in it is evidence, since no results are compared and Table 1's cells are one-word judgements with no sourcing. The stage annotations are the most valuable content and the least documented, with no definition of what qualifies a system as implementing a stage, and the paper contradicts itself on one: Figure 2 tags Multi-Agent Collaboration with Stage 3 and no collaboration tag while Section 2.2 describes that same system as an adaptive multi-agent architecture. Three of five authors wrote AlphaAgents, which appears in Table 2 undisclosed, and the open-challenges section is thirteen headings with no prioritisation.</t>
         </is>
       </c>
       <c r="U32" s="11" t="inlineStr">
@@ -4709,7 +4709,7 @@
       </c>
       <c r="T33" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The headline advantage does not clear its own error bars and no significance test is run: a 1.70 point edge over LSTM against standard deviations of 3.03 and 3.74, on one asset, one 268-day window and one regime. Twenty seeds measure LLM sampling variance, not variation across market paths. The annualized returns cannot be reproduced from the paper's own formula and the headline row is the worst case, since 21.75 % over 268 days should give 30.74 % and is printed as 29.30 %, implying a 279.5-day horizon when buy-and-hold reconciles exactly. Friction is a flat constant on the deepest book in crypto and the sensitivity band does not reconcile with the reported turnover of 7.60. Threshold selection is a grid search whose scoring set is never named, the text-agent ablation confounds content with prompt budget at one window size only, and GPT-4o grades its own summaries for conflict and actionability with no check against realised returns.</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="T34" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The zero-impact assumption is stated as a modelling convenience and does not survive transport to a thin book: the order is infinitesimal and the trader's action has no effect on the price process, which is what makes this a pure stopping problem rather than a control problem. No order type, no queue position, no partial fills and no fees, with STOP assumed to fill immediately at the observed price, so the book is built in full from ITCH messages and used only as a feature source rather than as a fill simulator. There is no non-neural baseline anywhere, no queue-imbalance threshold, no fixed-delay rule and no TWAP reference, so nothing establishes that the neural machinery is necessary rather than sufficient. One year, one exchange, one liquidity tier and no walk-forward, with folds randomised within 2013. No stopping criterion and no reported hyperparameter search, so the headline carries an unmeasured selection component.</t>
         </is>
       </c>
       <c r="U34" s="11" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="T35" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The market is a simulator in training and in testing and nothing is evaluated outside it: the queue-reactive model is calibrated on real IEX books, but every number including the impact result that motivates the approach is generated by it, with no historical replay, no live execution and no sensitivity over the calibration. Sample efficiency is counted only in real interactions, with no wall-clock or compute accounting, and D3Q(7) does eight times the gradient work per interaction, so the efficiency gain argues for a deployment setting the experiments do not operate in. Market orders only, no queue position, no fees and no partial fills, so the policy can only pay the spread and never earn it. One inventory size, one horizon, one venue and one regime, with no sweep over participation rate even though impact is the subject. The objective has no risk term at all.</t>
         </is>
       </c>
       <c r="U35" s="11" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="T36" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The five-parameter policy cannot express anything Almgren-Chriss cannot: linear permanent and temporary impact, arithmetic Brownian motion with constant volatility, no spread, no depth, no imbalance, so on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong. The convergence guarantee is real but not operational, since the learning-rate conditions involve constants the paper says are not easy to estimate and the iterates must sit in a compact rectangle fixed in advance. Exploration requires rewinding the market, sending 15 orders at one decision time and resetting between each, so the configuration carrying the headline results is simulator-only and the deployable variant is the weaker one. Market orders only, no spread, no queue, no fees, and the last step dumps whatever inventory is left. Seven large-cap Nasdaq names, two calm test quarters, one horizon at 10 % of ADTV, and SAC is not tuned symmetrically.</t>
         </is>
       </c>
       <c r="U36" s="11" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="T37" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The state-switching contribution is never isolated from how often it fires: no count of bearish periods, no timeline of the switch, no fixed-schedule router at the same rate, so nothing separates switching to NPMRP at the right moments from switching so rarely that SOPS is mostly NPM. A paper about exact transaction cost computation never varies the cost rate, with delta fixed at 0.05 % throughout and the sensitivity section covering everything except it, so whether SOPS still beats the nineteen baselines at a frontier-market rate is the question the machinery is built for and does not answer. Linear proportional cost is the whole model, so 'exact' is exact about commission, with no spread, impact, partial fill or volume constraint. No walk-forward, no seeds and no significance tests, with four per-dataset window sizes chosen by no stated procedure. Practicality is claimed and no runtime is reported anywhere.</t>
         </is>
       </c>
       <c r="U37" s="11" t="inlineStr">
@@ -5335,7 +5335,7 @@
       </c>
       <c r="T38" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>No statistical testing appears anywhere and the headline claim is a win count, declaring a model superior when the unweighted sum of F1, MCC and round-trip practicability is maximal, with no intervals, no seed variance and no test against DeepLOB across 1,350 experiments. Nothing isolates the TMFG, so the central claim about higher-order topological priors rests on model against model rather than on HLOB with the graph replaced by a random planar graph, an MST or a matched-density control. The label threshold is absolute at one cent while the grouping variable is relative, so the three tick-size groups are not solving the same classification problem and part of 'large-tick books are more learnable' is a statement about the threshold against the spread. The structure is static in a paper about persistence, averaged over 40 training days and held fixed. Event-time horizons, no execution model, one venue.</t>
         </is>
       </c>
       <c r="U38" s="11" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="T39" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The multi-hop conclusion is drawn on a graph that barely has a second hop to test, with 99.5 % of DJIA pairs within two hops, and the GHAR2Hop test returns p of about 0.35, a failure to reject rather than evidence of no effect. The return-based GLASSO graph is never compared against a volatility-based one, a sector graph or a randomised graph of matched density, so the identity of the edges is the most load-bearing unexamined choice in a design about what flows along them. Nonlinearity is established through one architecture and one activation, so the finding is that a nonlinear model beats a linear one rather than anything about the shape of the spillover. The turbulence stratification splits at the 90 % quantile of the full-sample distribution, so every turbulent-period statement is conditioned on an ex-post label a live system would have to estimate. Forecast loss is the only outcome, with no portfolio and no cost-bearing application.</t>
         </is>
       </c>
       <c r="U39" s="11" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="T40" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The construct and the measurement are different quantities and it propagates into every interpretation: monthly change in the ASPI is a signed return, not dispersion, and the near-zero AR(1) term at p = 0.8698 is consistent with a return series and inconsistent with a volatility series on a market where long memory persists across every regime. Short-run and long-run coefficients are used interchangeably, since the exchange rate and interest rate terms are lagged dynamics presented as establishing a long-term relationship while the actual long-run vector puts inflation at 2.549274 with p = 0.05 and never discusses it. The printed specification is not the one estimated: the equation given logs the coefficients rather than the variables, the lag structure and selection criterion are never stated, and a second equation silently drops three regressors and the constant. If any variable is genuinely I(2) the bounds F-distribution is invalid, and the paper's own KPSS result at second difference points that way. Diagnostics stop at Durbin-Watson, GDP is quadratically interpolated so 120 monthly figures rest on 40 observations, and the sample ends in December 2019, excluding every period in which Sri Lankan macro instability was severe.</t>
         </is>
       </c>
       <c r="U40" s="11" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="T41" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The ADF result licensing ASPI and volume at level is not credible and everything downstream inherits it: an ADF statistic of -5.0724 on a log equity index is contradicted by the paper's own Table 3, which reports lag-one autocorrelation of 0.9273 for log ASPI, and no ADF specification, lag choice or alternative unit root test is reported, which puts the volume to ASPI result in spurious-regression territory. The dependent variable is a level interpreted as a return, with a reported mean of 8.8223 that is a log index around 6,800 points and no return series. Mixing I(0), I(1) and I(2) variables in one pairwise framework without cointegration analysis breaks the test's asymptotics. Second-differencing the NCPI tests acceleration in inflation while the discussion talks about levels. Lag one forecloses the two to six month channels the other CSE evidence points at, and roughly 105 observations span five regime breaks with no subsample analysis.</t>
         </is>
       </c>
       <c r="U41" s="11" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="T42" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The error metrics do not reconcile, which puts the central claim out of reach: the implied evaluation levels differ by a factor of 2.4 between the two models, the abstract gives ARIMA's MAPE as 0.472206 against Table 5's 0.4672206, and neither reproduces from Table 4. No residual diagnostics anywhere, so the Box-Jenkins adequacy step is skipped rather than failed, and no ARCH test or conditional variance model across a decade opening on the global financial crisis. The clustering stage, which is the novel half, is not reproducible: average contribution to clusters has no definition or units, the chosen k is never reported and five of the nine banks are missing from the results table. One 80/20 split, one forecast origin, one seed and an architecture search with no validation partition. The stationarity handling contradicts itself and probably over-differences. An investment recommendation is issued with no strategy, no costs and no execution.</t>
         </is>
       </c>
       <c r="U42" s="11" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="T43" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The white noise conclusion is contradicted by the printed correlogram: the text calls the residuals white noise while Figure 3 reports p = 0.039 at lag 3, p = 0.001 at lag 4 and p = 0.000 continuously from lag 5 to 36, ending at Q(36) = 185.20, so the Box-Jenkins adequacy criterion is failed and reported as passed and the AR and MA standard errors assume the independence the correlogram rejects. A constant variance model is fitted to a decade with obvious clustering, visible in the paper's own residual plot, with no ARCH test and Durbin-Watson offered as the serial correlation evidence despite being biased toward 2 under MA errors. One forecast origin, a single 23-day window, no persistence baseline, no buy-and-hold and no rolling re-estimation. Significant autocorrelation is upgraded into exploitable inefficiency with no strategy, cost model or trade. Three literature review citations do not say what they are cited for and a fourth has no reference entry.</t>
         </is>
       </c>
       <c r="U43" s="11" t="inlineStr">
@@ -6090,7 +6090,7 @@
       </c>
       <c r="T44" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Everything is one realisation with no seeds, no intervals and no significance tests, and although the model refits every two years the results are reported as one aggregate path with no per-fold breakdown, so there is no way to see whether the advantage is stable across refits. The test window is nine years of US equity expansion followed by two months of crash, and the crash response traces to the volatility scaler rather than the learned policy, with no unscaled run through Q1 2020 to separate them. How the Sharpe objective is computed during training is never stated, per minibatch, per epoch or over the full sequence, which is a reproducibility hole sitting on the paper's single contribution. The cost model is flat and proportional on four of the most liquid ETFs in existence, so friction is designed out of the experiment. The volatility sleeve is named as an index with no tradable ticker, and the architecture claims are asserted without comparative numbers.</t>
         </is>
       </c>
       <c r="U44" s="11" t="inlineStr">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="T45" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>A flat 5 basis points per half-turn with no size or depth term, on the 500 largest US stocks, where the headline k=10 book holds twenty names and turns over completely every day. The signal's core is short-term reversal, which is partly bid-ask bounce: Section 4.4 concedes this, and the weekly and one-day-waiting variants show the return surviving at about half strength on penny spreads, which bounds nothing about a market where the spread is a meaningful fraction of the daily move. Everything is one run across 23 study periods, and the Diebold-Mariano and Pesaran-Timmermann tests cover forecast accuracy rather than returns, so the return differences carry no test at all while the random forest overtakes on Sharpe at larger k. Nothing conditions on market state, so the paper watches its own signal decay to zero after 2010 with no channel to respond. The probability output is used ordinally and never checked for calibration.</t>
         </is>
       </c>
       <c r="U45" s="3" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="T46" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Every number inherits the decomposition leak, since train, validation and test are decomposed together so each IMF is built with knowledge of the whole series, and the authors identify this and recommend the fix to others rather than applying it; the sliding-window version was never run, so the leak-free accuracy is unknown. LIME is never shown to add anything over the forest's own predict_proba, which is already a vote fraction over 250 trees, and that ablation at matched coverage is the paper's load-bearing missing experiment. Accuracy rising with the threshold is close to tautological, so the mechanism is not the finding. There is no economic evaluation of any kind, no returns, no costs and no exposure on abstained days, on a paper whose proposal is a trading decision rule. One run per index, no seeds, no significance tests and no reliability diagram, despite the design treating the score as a probability to be read literally.</t>
         </is>
       </c>
       <c r="U46" s="11" t="inlineStr">
@@ -6468,7 +6468,7 @@
       </c>
       <c r="T47" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The evidence base is two pages and cannot be reproduced from what is printed: no corpus size, no company or year coverage, no annotated-subset size, no ablation over chunk size, embedding model or top-k, and no description of the standard RAG baseline beyond 'without graph reasoning'. The comparison does not isolate the graph, since their system has both a Neo4j store and an agent that decomposes queries and retries while the baseline has neither, and the paper separately reports that decomposition and retry alone cut failure from about 30 % to under 2 %, so much of the 9.2 against 6.1 could be scaffolding. The Data Capture denominator is missing, with over 85 % entity capture on an unspecified manually annotated subset, improving on their own earlier naive approach rather than on a benchmark. Nothing is reported on cost or latency. The graph is a point-in-time snapshot with no as-of field, which for a backtest is a lookahead hazard.</t>
         </is>
       </c>
       <c r="U47" s="11" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="T48" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The RAG evaluation claimed as a headline innovation does not exist in the paper: there is no retrieval dataset, condition, result or appendix anywhere, and every task feeds context directly into the prompt. Several headline metrics measure output length and format rather than capability, with LLaMA2-7B-chat beating GPT-4 on Regulations ROUGE-1 at 0.24 against 0.11, and GPT-4's TATQA exact match at 0.13 against 0.63 on FinQA is an answer-normalisation artefact. The trading confidence intervals cannot be reproduced from the paper's own per-stock table: recomputing GPT-4 from Table 9 gives 26.80 % and Sharpe 1.45 against a reported 28.19 % and 1.51, and a cross-sectional half-width near 10.5 against the reported 25.27. Own zero-shot runs and imported few-shot numbers share the same cells. Nothing aggregates, so 'holistic' describes coverage rather than measurement, and 89.68 % of the data is repackaged from prior benchmarks. The leakage test is never applied to the fifteen evaluated models.</t>
         </is>
       </c>
       <c r="U48" s="11" t="inlineStr">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="T49" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The central comparison is not like for like and the framing does not flag it: FinMA is evaluated zero-shot on test splits whose training splits it was tuned on, GPT-4 and ChatGPT have no exposure, BloombergGPT's numbers are 20-shot and imported, and the test sets were rebuilt rather than shared. The appendix contains the fair comparison and it is much less favourable, with FLANG-BERT at 110M parameters reaching 0.912 on FPB, 0.972 on Headlines and 0.83 on NER against FinMA-7B's 0.94, 0.97 and 0.59, so a model sixty times smaller is level on two and well ahead on the third. The prediction tasks cannot demonstrate what the paper wants: the label discards everything between -0.5 % and 0.55 %, there are no transaction costs, no sizing and a single-step horizon with accuracy led on an imbalanced distribution. Temporal design is absent so leakage cannot be checked, and the instruction set is never ablated.</t>
         </is>
       </c>
       <c r="U49" s="11" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="T50" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The conversations are simulated from programs by decomposing or concatenating FinQA questions and were never validated against real analyst dialogue, so the hardest class, the second part of a hybrid conversation at 52.38 %, rests on an artefact of which two questions one annotator happened to write about the same report. Every FinQA filtering constraint is inherited and the operation vocabulary is narrowed from ten to six, so a system scoring 68.90 % has demonstrated reference resolution over one clean page and nothing about locating it. The neural symbolic results are single-run point estimates while the prompting side reports exemplar variance of 4.68, so the two halves are not held to the same standard. The prompting conclusion is scoped to text-davinci-002 with deliberately shallow prompting. The turn-6 collapse rests on very few examples, and nothing measures error propagation or offers the model a way to decline a turn.</t>
         </is>
       </c>
       <c r="U50" s="11" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="T51" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>There is no retrieval step at all, so the task is strictly shallower than a fundamental channel faces: the hybrid context is handed over already located and already verified as coherent, and two thirds of candidate tables were discarded for lacking that coherence. One operator per question makes the compositionality claim circular, with Composition at 19.69 % of reasoning types against Change ratio at 10.2 % of test questions and an unnamed Other class scoring 0.0 % operator accuracy. The question distribution is shaped by annotation instructions that encourage reusing context words, which is why Word Matching is 38.06 % of the dataset. Every number is a single-run point estimate with no interval or significance test, and the 84.1 EM human bar comes from 301 questions against the 1,669 the models are scored on, so the 33-point gap spans two evaluation sets. Section 4.3 also contradicts Table 5 on the operator ablation.</t>
         </is>
       </c>
       <c r="U51" s="11" t="inlineStr">
@@ -7093,7 +7093,7 @@
       </c>
       <c r="T52" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>The filtering removes exactly the layouts that make real reports hard: one table per page, at most 20 rows, no nested structures, multi-header tables flattened and catalogs excluded, so 61.24 % is accuracy on a sanitised slice of already well-structured US filings. Every question is page-local at an average 687.53 tokens, nothing crosses a document or a filing year and there is no as-of notion, so a good score says nothing about finding the right page in a 200-page report or retrieving point-in-time. The DSL bounds what counts as a question, with ten operations, no conditionals, no date arithmetic and no unit-aware types, and the 43.88 % on programs containing constants sits seventeen points below the headline because scaling factors are tokens without units. Both metrics are acknowledged as biased and carry no intervals. The 91.16 % human bound rests on 200 examples, with experts disagreeing on the program about one time in seven.</t>
         </is>
       </c>
       <c r="U52" s="11" t="inlineStr">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="T53" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>There is no ablation separating the detector from the ensemble, which leaves the paper's own mechanism unestablished: OOD precision is 0.23, so roughly three in four flagged samples are ones the current model would have handled, and the obvious control of applying the AR combination to every prediction is not run; if it matched, the contribution reduces to a recency-weighted ensemble over checkpoints. Delta F1 rewards a model that is uniformly mediocre, so ODNM BERT posts the smallest drop while sitting 11.7 points below NDOM on in-sample capability and GPT-3.5 wins by being flat and weak. The shift measure weights by month t, so it is least able to see new vocabulary, which is what financial text produces. The labels are self-declared directional tags, so label shift and market regime are entangled by construction. One platform, one market, three years, no significance testing, and nothing connects the drop to money.</t>
         </is>
       </c>
       <c r="U53" s="11" t="inlineStr">
@@ -8552,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="142" customWidth="1" min="1" max="1"/>
@@ -8926,6 +8926,20 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
+        <is>
+          <t>Amendment, 18 October 2026 (second)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>Limitations column populated for the 33 rows that previously read 'Not recorded in the note', every one of which links a note that does carry a full Limitations section: P01, P02, P03, P05, P06, P07 and P26 through P52. Each cell is condensed from that note's own Limitations bullets in the column's existing style, and every figure quoted was checked back against the note before entry. No row's rating, reading or usage changed, so no row is marked amber. The in-sync block P04 and P08 to P25 was not touched. Still outstanding on this column: the Consolidated Research Matrix carries the same 33 gaps and has not been updated, and several cells elsewhere say 'not recorded in the note' where the honest value is 'None' because the paper has no such component (P58 and P59 Sentiment Handling, P60 Volatility &amp; Risk and Explainability).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 13:16:52
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Literature Survey Matrix.xlsx
+++ b/FYP/Matrices/Literature Survey Matrix.xlsx
@@ -716,7 +716,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Three stated gaps — (1) "Existing agent frameworks optimise task performance and ignore how trading firms actually organise a decision"; (2) "Natural language as the sole communication medium corrupts state over long horizons" (the "telephone effect"); (3) "Deep learning trading systems are opaque at the point where opacity is most expensive". Student's verdict: "The second and third gaps are addressed by the design. The first is asserted throughout and tested nowhere, and since it is the framing the title rests on, the mismatch between the claimed contribution and the evidence starts here."</t>
+          <t>Three stated gaps - (1) "Existing agent frameworks optimise task performance and ignore how trading firms actually organise a decision"; (2) "Natural language as the sole communication medium corrupts state over long horizons" (the "telephone effect"); (3) "Deep learning trading systems are opaque at the point where opacity is most expensive". Student's verdict: "The second and third gaps are addressed by the design. The first is asserted throughout and tested nowhere, and since it is the framing the title rests on, the mismatch between the claimed contribution and the evidence starts here."</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Backtest 1 Jan – 29 Mar 2024, "roughly sixty trading days". Stated universe AAPL, NVDA, MSFT, META, GOOGL; reported results AAPL, GOOGL, AMZN — "so the reported set does not match the named set and Amazon appears in results without appearing in the universe."</t>
+          <t>Backtest 1 Jan - 29 Mar 2024, "roughly sixty trading days". Stated universe AAPL, NVDA, MSFT, META, GOOGL; reported results AAPL, GOOGL, AMZN - "so the reported set does not match the named set and Amazon appears in results without appearing in the universe."</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>No training. "Every agent is a prompted role with a fixed goal, a tool set and a set of constraints, and the only thing that changes between days is the data in the shared state." ReAct loop over shared agent state. Tiered backbone: gpt-4o-mini and gpt-4o for retrieval/summarisation, o1-preview for decisions.  Simulated trading firm hierarchy; output is an authorised trade plus a written rationale and a full decision log. AGENTS &amp; ORCHESTRATION (exhaustive): Seven roles / nine listed functions — Fundamentals Analyst (statements, earnings, insider transactions, intrinsic value), Sentiment Analyst (social volume/polarity, insider sentiment, short-horizon crowd behaviour), News Analyst (wires, government announcements, macro), Technical Analyst (selects from sixty indicators; momentum, trend, volatility, volume), Bullish Researcher and Bearish Researcher (n rounds of debate), Trader (decision plus rationale), Risk Team of three (aggressive, neutral, conservative) deliberating over the trader's plan, Fund Manager (reviews risk discussion, applies adjustments, authorises execution). Combination: analysts write structured reports into a global agent state; downstream roles query only the fields they need. Free-form NL is confined to two bounded places — the bull/bear debate and the risk discussion — each run n rounds under a facilitator that "selects the prevailing perspective" and writes it back as a structured entry. "The value of n is never given." State-conditioned influence: NONE. "That facilitator is the only point in the system where evidence from opposing agents is combined, and it is described in one sentence. There is no aggregation equation in the paper at all." And: "seven specialised roles feeding a fixed hierarchy with no weighting, no state conditioning and no ablation to show that any of the structure contributes anything."</t>
+          <t>No training. "Every agent is a prompted role with a fixed goal, a tool set and a set of constraints, and the only thing that changes between days is the data in the shared state." ReAct loop over shared agent state. Tiered backbone: gpt-4o-mini and gpt-4o for retrieval/summarisation, o1-preview for decisions. Simulated trading firm hierarchy; output is an authorised trade plus a written rationale and a full decision log. AGENTS &amp; ORCHESTRATION (exhaustive): Seven roles / nine listed functions - Fundamentals Analyst (statements, earnings, insider transactions, intrinsic value), Sentiment Analyst (social volume/polarity, insider sentiment, short-horizon crowd behaviour), News Analyst (wires, government announcements, macro), Technical Analyst (selects from sixty indicators; momentum, trend, volatility, volume), Bullish Researcher and Bearish Researcher (n rounds of debate), Trader (decision plus rationale), Risk Team of three (aggressive, neutral, conservative) deliberating over the trader's plan, Fund Manager (reviews risk discussion, applies adjustments, authorises execution). Combination: analysts write structured reports into a global agent state; downstream roles query only the fields they need. Free-form NL is confined to two bounded places - the bull/bear debate and the risk discussion - each run n rounds under a facilitator that "selects the prevailing perspective" and writes it back as a structured entry. "The value of n is never given." State-conditioned influence: NONE. "That facilitator is the only point in the system where evidence from opposing agents is combined, and it is described in one sentence. There is no aggregation equation in the paper at all." And: "seven specialised roles feeding a fixed hierarchy with no weighting, no state conditioning and no ablation to show that any of the structure contributes anything."</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Two dedicated channels (Sentiment Analyst over Reddit/X with auxiliary-LM sentiment scores plus insider sentiment; News Analyst over wires and macro). Student maps both onto nothing — "the sentiment and news analysts onto nothing, since sentiment is out of scope."</t>
+          <t>Two dedicated channels (Sentiment Analyst over Reddit/X with auxiliary-LM sentiment scores plus insider sentiment; News Analyst over wires and macro). Student maps both onto nothing - "the sentiment and news analysts onto nothing, since sentiment is out of scope."</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -766,17 +766,17 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>The demonstrated result. Sixteen appendix pages reproducing a complete day's log for AAPL on 19 Nov 2024 — indicator selection, tool calls with arguments and call IDs, news and fundamentals reports, both research cases, three risk perspectives, the fund manager's four-point rationale. "The debate is not two agents talking past each other, the bear picks up the bull's liquidity claim and reads the same current and quick ratios below 1 as a risk rather than a buffer." "it costs nothing to produce because the reasoning is a by-product of the ReAct loop rather than a separate attribution step."</t>
+          <t>The demonstrated result. Sixteen appendix pages reproducing a complete day's log for AAPL on 19 Nov 2024 - indicator selection, tool calls with arguments and call IDs, news and fundamentals reports, both research cases, three risk perspectives, the fund manager's four-point rationale. "The debate is not two agents talking past each other, the bear picks up the bull's liquidity claim and reads the same current and quick ratios below 1 as a risk rather than a buffer." "it costs nothing to produce because the reasoning is a by-product of the ReAct loop rather than a separate attribution step."</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>Buy-and-hold, MACD, KDJ+RSI, zero mean reversion, SMA crossover — "all rule-based and none of them an LLM, which is the single most consequential choice in the experimental design." Metrics: cumulative return, annualised return, Sharpe, maximum drawdown. Single run, no repeats, no dispersion, no significance test.</t>
+          <t>Buy-and-hold, MACD, KDJ+RSI, zero mean reversion, SMA crossover - "all rule-based and none of them an LLM, which is the single most consequential choice in the experimental design." Metrics: cumulative return, annualised return, Sharpe, maximum drawdown. Single run, no repeats, no dispersion, no significance test.</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>Cumulative return 26.62% AAPL, 24.36% GOOGL, 23.21% AMZN, against best rule-based baselines of 2.05, 6.23 and 11.01; improvement rows 24.57, 16.58, 6.10. "the 6.10 on AMZN is the honest number", because buy-and-hold there returned 17.1%. Drawdowns 0.91 / 1.69 / 2.11 against rule-based bests of 0.86 / 1.22 / 0.82 — "the simple rules control risk better on all three and the paper concedes the trade-off directly." AAPL buy-and-hold −5.23% against the framework's 26.62%, including shorts — "This is the result the authors lead with and it is the right one to lead with." AMZN "tracks buy-and-hold almost exactly for the first six weeks and separates only in mid-February... the entire reported edge on that stock comes from a few weeks." Sharpe 8.21 / 6.39 / 5.60 — "the Sharpe row cannot support the risk-adjusted-return claim the discussion section builds on it, and the discussion makes that claim anyway." Cost: eleven LLM calls and more than twenty tool calls per prediction. LIMITATIONS (quoted): "Sixty trading days, three stocks, one regime, one run." — "on this evidence the question has not been asked in a form that could return a negative answer." "The organisational thesis is never tested, neither as a mechanism nor as a result, and this is the criticism the whole note turns on" — "with no weight anywhere, no confidence, no way for an uninformative channel to be discounted, and a facilitator that picks the prevailing perspective under no stated criterion"; "A single-agent LLM baseline would have cost one more run and would have carried most of the paper's weight, and its absence means the title's claim rests on no evidence in either direction." "No execution friction of any kind." "The backbone almost certainly saw the test period, and the look-ahead control does not address that" — "I am not claiming contamination occurred, I am noting that the design cannot distinguish it from skill." "Reporting gaps that make the run hard to reproduce even with the code" — n never given, no temperature/decoding settings, universe mismatch, SEDI (Canadian) insider data used for three US tickers.</t>
+          <t>Cumulative return 26.62% AAPL, 24.36% GOOGL, 23.21% AMZN, against best rule-based baselines of 2.05, 6.23 and 11.01; improvement rows 24.57, 16.58, 6.10. "the 6.10 on AMZN is the honest number", because buy-and-hold there returned 17.1%. Drawdowns 0.91 / 1.69 / 2.11 against rule-based bests of 0.86 / 1.22 / 0.82 - "the simple rules control risk better on all three and the paper concedes the trade-off directly." AAPL buy-and-hold −5.23% against the framework's 26.62%, including shorts - "This is the result the authors lead with and it is the right one to lead with." AMZN "tracks buy-and-hold almost exactly for the first six weeks and separates only in mid-February... the entire reported edge on that stock comes from a few weeks." Sharpe 8.21 / 6.39 / 5.60 - "the Sharpe row cannot support the risk-adjusted-return claim the discussion section builds on it, and the discussion makes that claim anyway." Cost: eleven LLM calls and more than twenty tool calls per prediction. LIMITATIONS (quoted): "Sixty trading days, three stocks, one regime, one run." - "on this evidence the question has not been asked in a form that could return a negative answer." "The organisational thesis is never tested, neither as a mechanism nor as a result, and this is the criticism the whole note turns on" - "with no weight anywhere, no confidence, no way for an uninformative channel to be discounted, and a facilitator that picks the prevailing perspective under no stated criterion"; "A single-agent LLM baseline would have cost one more run and would have carried most of the paper's weight, and its absence means the title's claim rests on no evidence in either direction." "No execution friction of any kind." "The backbone almost certainly saw the test period, and the look-ahead control does not address that" - "I am not claiming contamination occurred, I am noting that the design cannot distinguish it from skill." "Reporting gaps that make the run hard to reproduce even with the code" - n never given, no temperature/decoding settings, universe mismatch, SEDI (Canadian) insider data used for three US tickers.</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>Role specialisation by evidence type; the structured communication protocol as a precondition for weighting — "each agent emits a structured record, a directional signal, a confidence and a prose rationale, written into a shared state the orchestrator reads"; the end-to-end decision log as a zero-cost deliverable ("Writing one full CSE trading day into the evaluation chapter, from each agent's structured record through the weight vector to the final position, is cheap"); the inference-cost planning figure, with the mitigation "caching the fundamental agent's retrieval per reporting period instead of per day"; and the pre-commitment on window length — "treat a Sharpe outside the ordinary empirical range as a diagnostic that the sample is too short rather than as a result."</t>
+          <t>Role specialisation by evidence type; the structured communication protocol as a precondition for weighting - "each agent emits a structured record, a directional signal, a confidence and a prose rationale, written into a shared state the orchestrator reads"; the end-to-end decision log as a zero-cost deliverable ("Writing one full CSE trading day into the evaluation chapter, from each agent's structured record through the weight vector to the final position, is cheap"); the inference-cost planning figure, with the mitigation "caching the fundamental agent's retrieval per reporting period instead of per day"; and the pre-commitment on window length - "treat a Sharpe outside the ordinary empirical range as a diagnostic that the sample is too short rather than as a result."</t>
         </is>
       </c>
       <c r="V2" s="3" t="inlineStr">
@@ -799,9 +799,9 @@
           <t>SPEAKS TO: A_T (technical analyst), A_F (fundamentals analyst, once re-pointed at CSE filings), A_V (as a counter-example: risk-as-review), orchestrator (primary), evaluation layer (decision log, window length, friction tally).
 EFFECT ON MAIN GAP: Strongest single motivating case in the set, and reframes the gap itself. "That converts the gap from 'existing systems weight agents badly' into the sharper 'existing systems have no quantity that could be weighted', which is a cleaner motivation for the three-way comparison of equal, static learned and dynamic state-aware weighting."
 EFFECT ON SUB-GAP 1: Anchors the zero end. "It anchors the zero end of my friction tally, which is what makes the friction-aware evaluation layer a contribution rather than housekeeping."
-EFFECT ON SUB-GAP 2: Indirect only — no volatility model; supplies the Sharpe-artefact argument for why short windows corrupt volatility-denominated metrics.
-FIXED-INFLUENCE FAILURE EVIDENCE: A different class from the others — invisible rather than measured. "TradingAgents is the case where the damage would be invisible, seven channels feeding a hierarchy with no weights and no ablation, so a channel could be contributing nothing on most days and the framework would return the same headline number." Also: "unlike the fixed-influence failures I have collected elsewhere this system could not detect the problem even if it were happening." Secondary, on risk placement: "this framework's drawdowns lose to a plain zero-mean-reversion rule on all three stocks despite a dedicated three-agent risk team, which is consistent with risk-as-review being too late to shape position sizing." Student flags this as hypothesis, not result: "Indirect is the right word, no ablation isolates the risk team."
-PROPOSED REVISION STATED IN THE NOTE: On the agent pool — the confirmation that only two of four analyst roles map across and the firm metaphor is discarded: "What survives the mapping is role specialisation by evidence type. What does not survive is the firm metaphor, because the hierarchy is doing the coordination work and a hierarchy cannot condition on market state." On the orchestrator's input contract: "w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) needs agent outputs in a form that can be weighted, and free prose is not it." No change to the conditioning set itself; a new explicit argument that A_V is upstream rather than downstream — "which is a design choice I should now argue explicitly rather than assume."</t>
+EFFECT ON SUB-GAP 2: Indirect only - no volatility model; supplies the Sharpe-artefact argument for why short windows corrupt volatility-denominated metrics.
+FIXED-INFLUENCE FAILURE EVIDENCE: A different class from the others - invisible rather than measured. "TradingAgents is the case where the damage would be invisible, seven channels feeding a hierarchy with no weights and no ablation, so a channel could be contributing nothing on most days and the framework would return the same headline number." Also: "unlike the fixed-influence failures I have collected elsewhere this system could not detect the problem even if it were happening." Secondary, on risk placement: "this framework's drawdowns lose to a plain zero-mean-reversion rule on all three stocks despite a dedicated three-agent risk team, which is consistent with risk-as-review being too late to shape position sizing." Student flags this as hypothesis, not result: "Indirect is the right word, no ablation isolates the risk team."
+PROPOSED REVISION STATED IN THE NOTE: On the agent pool - the confirmation that only two of four analyst roles map across and the firm metaphor is discarded: "What survives the mapping is role specialisation by evidence type. What does not survive is the firm metaphor, because the hierarchy is doing the coordination work and a hierarchy cannot condition on market state." On the orchestrator's input contract: "w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) needs agent outputs in a form that can be weighted, and free prose is not it." No change to the conditioning set itself; a new explicit argument that A_V is upstream rather than downstream - "which is a design choice I should now argue explicitly rather than assume."</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Three gaps — (1) DL/RL models "flatten heterogeneous inputs into numeric features and lose both information and interpretability", specifically news compressed to a sentiment scalar; (2) multimodal LLM agents work but are expensive to set up (FinAgent's one-year training period); (3) "Risk management is absent from the comparable LLM trading agents." Student's verdict: "The third is a real gap and it is addressed. The first is a motivation for the design rather than a gap the experiments close."</t>
+          <t>Three gaps - (1) DL/RL models "flatten heterogeneous inputs into numeric features and lose both information and interpretability", specifically news compressed to a sentiment scalar; (2) multimodal LLM agents work but are expensive to set up (FinAgent's one-year training period); (3) "Risk management is absent from the comparable LLM trading agents." Student's verdict: "The third is a real gap and it is addressed. The first is a motivation for the design rather than a gap the experiments close."</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -853,17 +853,17 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>AAPL, AMZN, MSFT, 1 Apr – 29 Dec 2023. Burn-in 1 Apr – 31 May (42 trading days); evaluation 1 Jun – 29 Dec (145 trading days). News via Yahoo Finance through the eodhd API. Article counts: AAPL 1,081 burn-in / 4,886 test; AMZN 1,113 / 5,556; MSFT 1,897 / 1,249. "MSFT collects fewer articles across 145 days than across 42, and lands at roughly a quarter of AMZN's volume over identical dates... the news channel's density differs by more than 4× across the three assets whose results are then reported side by side."</t>
+          <t>AAPL, AMZN, MSFT, 1 Apr - 29 Dec 2023. Burn-in 1 Apr - 31 May (42 trading days); evaluation 1 Jun - 29 Dec (145 trading days). News via Yahoo Finance through the eodhd API. Article counts: AAPL 1,081 burn-in / 4,886 test; AMZN 1,113 / 5,556; MSFT 1,897 / 1,249. "MSFT collects fewer articles across 145 days than across 42, and lands at roughly a quarter of AMZN's volume over identical dates... the news channel's density differs by more than 4× across the three assets whose results are then reported side by side."</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>News text; SMA 10 and 50, RSI 14, Bollinger 20/2σ, volume, MACD — all computed numerically then "plotted with Matplotlib into images", one candlestick-and-indicator chart over the prior 60 days and one trading-signal chart over the prior 30. "it is the images that reach the agents."</t>
+          <t>News text; SMA 10 and 50, RSI 14, Bollinger 20/2σ, volume, MACD - all computed numerically then "plotted with Matplotlib into images", one candlestick-and-indicator chart over the prior 60 days and one trading-signal chart over the prior 30. "it is the images that reach the agents."</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>No training. "There are no weights and no gradients anywhere in the framework"; the 42 days are "a burn-in, not training, and the distinction matters for my own planning because a burn-in comes out of the usable evaluation window rather than out of a separate training set." Backbones gpt-4o-mini at temperature 0.3 for all agents except the Prediction agent, which runs o1-mini.  LangGraph over a shared AgentState. Output Â^{s_t} = (â^{s_t}, p̂^{s_t}, ê^{s_t}) — action in BUY/SELL/HOLD, position size in [1,10], explanation. AGENTS &amp; ORCHESTRATION (exhaustive): Four modules plus an execution agent. Summarizer (condenses prior day's news), Technical/Chart Analyst (reads a rendered chart image), Reflection module in two parts (textual score of recent decision effectiveness; visual read of a plotted buy/sell-marker chart), Prediction agent, Reward agent (executes and feeds portfolio state back). Combination is a single concatenating prompt: Â^{s_t} = agent_decision(s, X_1^{s_{t-1}}, X_2^{s_{t-1}}, X_3^{s_{t-1}}, X_4^{s_{t-1}}, P^{s_{t-1}}, prompt_trading) with X_1 news summary, X_2 technical read of the chart image, X_3 textual reflection, X_4 visual reflection, P portfolio state. State-conditioned influence: NONE. "the four channels are concatenated into one prompt and there is no weight, no confidence and no quantity anywhere that could be weighted, which is the same absence as in TradingAgents but reached with one decision agent instead of a seven-role hierarchy, so it is not an artefact of that paper's organisational framing." Channels are narrow by construction: the chart analyst is capped at ten words per signal, reflection insights at fifteen.</t>
+          <t>No training. "There are no weights and no gradients anywhere in the framework"; the 42 days are "a burn-in, not training, and the distinction matters for my own planning because a burn-in comes out of the usable evaluation window rather than out of a separate training set." Backbones gpt-4o-mini at temperature 0.3 for all agents except the Prediction agent, which runs o1-mini. LangGraph over a shared AgentState. Output Â^{s_t} = (â^{s_t}, p̂^{s_t}, ê^{s_t}) - action in BUY/SELL/HOLD, position size in [1,10], explanation. AGENTS &amp; ORCHESTRATION (exhaustive): Four modules plus an execution agent. Summarizer (condenses prior day's news), Technical/Chart Analyst (reads a rendered chart image), Reflection module in two parts (textual score of recent decision effectiveness; visual read of a plotted buy/sell-marker chart), Prediction agent, Reward agent (executes and feeds portfolio state back). Combination is a single concatenating prompt: Â^{s_t} = agent_decision(s, X_1^{s_{t-1}}, X_2^{s_{t-1}}, X_3^{s_{t-1}}, X_4^{s_{t-1}}, P^{s_{t-1}}, prompt_trading) with X_1 news summary, X_2 technical read of the chart image, X_3 textual reflection, X_4 visual reflection, P portfolio state. State-conditioned influence: NONE. "the four channels are concatenated into one prompt and there is no weight, no confidence and no quantity anywhere that could be weighted, which is the same absence as in TradingAgents but reached with one decision agent instead of a seven-role hierarchy, so it is not an artefact of that paper's organisational framing." Channels are narrow by construction: the chart analyst is capped at ten words per signal, reflection insights at fifteen.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>The paper's claimed risk contribution is position sizing as a percentage of portfolio rather than an all-in signal — but the sizing ranges are hand-written into the prompt. No volatility model. Annualised return defined as a linear rescaling: ARR = ((P_T − P_0)/P_0) × (C/T), "so the 145-day results are simply multiplied by roughly 1.74. AMZN's headline 43.57 % for buy-and-hold is therefore about a 25 % realised gain over seven months." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model, no slippage and no impact." Student's sharpened point: "Frequent partial rebalancing in 1 to 5 % slices is exactly the pattern whose risk-adjusted advantage a realistic cost model erodes first, because the smoothing comes from trading more often rather than from taking better positions. So the absence of costs does not merely inflate a return figure here, it sits directly underneath the only result this paper can defend."</t>
+          <t>The paper's claimed risk contribution is position sizing as a percentage of portfolio rather than an all-in signal - but the sizing ranges are hand-written into the prompt. No volatility model. Annualised return defined as a linear rescaling: ARR = ((P_T − P_0)/P_0) × (C/T), "so the 145-day results are simply multiplied by roughly 1.74. AMZN's headline 43.57 % for buy-and-hold is therefore about a 25 % realised gain over seven months." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model, no slippage and no impact." Student's sharpened point: "Frequent partial rebalancing in 1 to 5 % slices is exactly the pattern whose risk-adjusted advantage a realistic cost model erodes first, because the smoothing comes from trading more often rather than from taking better positions. So the absence of costs does not merely inflate a return figure here, it sits directly underneath the only result this paper can defend."</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>The decision log. "It is readable, specific and short enough that someone would actually read it" — cites unrealised profit 5.63% above average purchase price, four named indicators in conflict, a specific news event, a reflection that past sell signals were timed too early, sizes at 3% of portfolio. "It also ends by stating that the strategy 'aligns with the provided trading rules', which is the agent naming the rule set it was handed."</t>
+          <t>The decision log. "It is readable, specific and short enough that someone would actually read it" - cites unrealised profit 5.63% above average purchase price, four named indicators in conflict, a specific news event, a reflection that past sell signals were timed too early, sizes at 3% of portfolio. "It also ends by stating that the strategy 'aligns with the provided trading rules', which is the agent naming the rule set it was handed."</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>ARR 14.79 AAPL / 25.57 MSFT / 42.14 AMZN against buy-and-hold 13.56 / 22.27 / 43.57 — beats passive by 1.23 and 3.30 on two and "falls below it on the third". FinAgent posts 31.89 / 44.74 / 65.10, "ahead by 17 to 23 points everywhere". Sharpe 1.20 / 1.41 / 1.72 against 0.67 / 1.01 / 1.37, with AMZN's 1.72 the table's best including FinAgent's 1.61; AMZN drawdown 12.09% against the market's 17.45%. "what the framework does is convert a return stream similar to passive into a smoother one." Reflection ablation: ARR 14.79→8.84, 25.57→16.99, 42.14→37.64; Sharpe 1.20→0.62, 1.41→1.04, AMZN 1.72→1.68. RL baselines: PPO Sharpe −0.42 / −0.73 / −0.59, DQN −0.90 / −0.26 / −0.46, with ARR as high as 22.07. LIMITATIONS (quoted): "The trading policy is written into the Prediction agent's prompt, so this is a rule-based strategy with an LLM applying it rather than a system that learns one" — maintain ≥10% cash; BUY on strong upward trend with cash &gt;10%, or on a dip within an uptrend with cash &gt;20%; SELL on trend reversal, gains &gt;5% above average purchase price, or three consecutive days of gains; size 5–10% in strong uptrends, 1–5% on dips, partial sells 3–5%. "Every threshold is hand-chosen and none is reported as tuned." "There is no learned component anywhere in this framework, and the word 'agent' is doing a lot of work to obscure that." "Three stocks, 145 test days, one strongly bullish regime, one run each." "The only LLM baseline is copied from another paper rather than re-run." "No execution friction, on the one claim the paper has left." "The representation claim that motivates the 'multi-modal' in the title is never tested" — "On this evidence I cannot tell whether the vision channel helps, hurts or is neutral." Plus pre-training overlap with the test window and the unexplained news counts.</t>
+          <t>ARR 14.79 AAPL / 25.57 MSFT / 42.14 AMZN against buy-and-hold 13.56 / 22.27 / 43.57 - beats passive by 1.23 and 3.30 on two and "falls below it on the third". FinAgent posts 31.89 / 44.74 / 65.10, "ahead by 17 to 23 points everywhere". Sharpe 1.20 / 1.41 / 1.72 against 0.67 / 1.01 / 1.37, with AMZN's 1.72 the table's best including FinAgent's 1.61; AMZN drawdown 12.09% against the market's 17.45%. "what the framework does is convert a return stream similar to passive into a smoother one." Reflection ablation: ARR 14.79→8.84, 25.57→16.99, 42.14→37.64; Sharpe 1.20→0.62, 1.41→1.04, AMZN 1.72→1.68. RL baselines: PPO Sharpe −0.42 / −0.73 / −0.59, DQN −0.90 / −0.26 / −0.46, with ARR as high as 22.07. LIMITATIONS (quoted): "The trading policy is written into the Prediction agent's prompt, so this is a rule-based strategy with an LLM applying it rather than a system that learns one" - maintain ≥10% cash; BUY on strong upward trend with cash &gt;10%, or on a dip within an uptrend with cash &gt;20%; SELL on trend reversal, gains &gt;5% above average purchase price, or three consecutive days of gains; size 5–10% in strong uptrends, 1–5% on dips, partial sells 3–5%. "Every threshold is hand-chosen and none is reported as tuned." "There is no learned component anywhere in this framework, and the word 'agent' is doing a lot of work to obscure that." "Three stocks, 145 test days, one strongly bullish regime, one run each." "The only LLM baseline is copied from another paper rather than re-run." "No execution friction, on the one claim the paper has left." "The representation claim that motivates the 'multi-modal' in the title is never tested" - "On this evidence I cannot tell whether the vision channel helps, hurts or is neutral." Plus pre-training overlap with the test window and the unexplained news counts.</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
@@ -923,12 +923,12 @@
       </c>
       <c r="W3" s="3" t="inlineStr">
         <is>
-          <t>SPEAKS TO: A_T (directly — the numbers-vs-pictures decision), orchestrator (the conditioning set, especially C_{i,t}), evaluation layer (ablation design, baseline parity, burn-in accounting, decision log).
-EFFECT ON MAIN GAP: Confirms the absence generalises beyond hierarchical designs — same no-weightable-quantity failure reached with a single decision agent, "so it is not an artefact of that paper's organisational framing." Also supplies the sharpest warning about how the contribution could evaporate: "If w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) ends up specified in a prompt rather than fitted, then 'dynamic state-aware weighting' is a hand-written rule set and the contribution disappears... f has to be a fitted function whose parameters I can report and inspect, and the baseline it has to clear is the static learned weight, which is exactly the baseline FinVision has no version of."
-EFFECT ON SUB-GAP 1: Reinforces it, and with a sharper mechanism than TradingAgents — here zero friction sits underneath the single defensible result, because the smoothing is bought by trading more often.
+          <t>SPEAKS TO: A_T (directly - the numbers-vs-pictures decision), orchestrator (the conditioning set, especially C_{i,t}), evaluation layer (ablation design, baseline parity, burn-in accounting, decision log).
+EFFECT ON MAIN GAP: Confirms the absence generalises beyond hierarchical designs - same no-weightable-quantity failure reached with a single decision agent, "so it is not an artefact of that paper's organisational framing." Also supplies the sharpest warning about how the contribution could evaporate: "If w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) ends up specified in a prompt rather than fitted, then 'dynamic state-aware weighting' is a hand-written rule set and the contribution disappears... f has to be a fitted function whose parameters I can report and inspect, and the baseline it has to clear is the static learned weight, which is exactly the baseline FinVision has no version of."
+EFFECT ON SUB-GAP 1: Reinforces it, and with a sharper mechanism than TradingAgents - here zero friction sits underneath the single defensible result, because the smoothing is bought by trading more often.
 EFFECT ON SUB-GAP 2: None directly. No volatility model, no persistence treatment.
-FIXED-INFLUENCE FAILURE EVIDENCE: Not a documented degradation case in the collected sense, but two related items. The news channel varies in density by more than 4× across the three reported assets with no mechanism to notice or adapt — "the news channel's density differs by more than 4× across the three assets whose results are then reported side by side" and "The paper does not remark on it." And the attribution failure: "'The visual reflection module plays a crucial role' is a claim about a component that was never ablated on its own", with the general lesson "bundling two mechanisms into one ablatable block, as reflection does here, leaves the paper free to attribute the result to whichever half it prefers."
-PROPOSED REVISION STATED IN THE NOTE: Yes — a candidate definition for C_{i,t} to put to the supervisor. "Making it per-agent is a small change to this design and gives a concrete candidate definition, confidence as a rolling per-agent hit rate against realised next-period outcomes, which sits alongside Jung and Lee's pairwise conflict scoring as the second workable answer I have found to a problem the rest of the literature does not address at all. I would put both to the supervisor as a refinement of C_{i,t} rather than leaving it as an unspecified input." Also an explicit A_T design commitment: "A design decision for A_T, numbers rather than pictures, which I should state and justify rather than leave implicit... this is a decision I am making on architectural grounds and should defend that way."</t>
+FIXED-INFLUENCE FAILURE EVIDENCE: Not a documented degradation case in the collected sense, but two related items. The news channel varies in density by more than 4× across the three reported assets with no mechanism to notice or adapt - "the news channel's density differs by more than 4× across the three assets whose results are then reported side by side" and "The paper does not remark on it." And the attribution failure: "'The visual reflection module plays a crucial role' is a claim about a component that was never ablated on its own", with the general lesson "bundling two mechanisms into one ablatable block, as reflection does here, leaves the paper free to attribute the result to whichever half it prefers."
+PROPOSED REVISION STATED IN THE NOTE: Yes - a candidate definition for C_{i,t} to put to the supervisor. "Making it per-agent is a small change to this design and gives a concrete candidate definition, confidence as a rolling per-agent hit rate against realised next-period outcomes, which sits alongside Jung and Lee's pairwise conflict scoring as the second workable answer I have found to a problem the rest of the literature does not address at all. I would put both to the supervisor as a refinement of C_{i,t} rather than leaving it as an unspecified input." Also an explicit A_T design commitment: "A design decision for A_T, numbers rather than pictures, which I should state and justify rather than leave implicit... this is a decision I am making on architectural grounds and should defend that way."</t>
         </is>
       </c>
       <c r="X3" s="3" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>US index level — S&amp;P 500.  Data validation. "this validates data and does not act on it, so there are no positions, no returns, no transaction costs and no evaluation protocol of any kind."</t>
+          <t>US index level - S&amp;P 500. Data validation. "this validates data and does not act on it, so there are no positions, no returns, no transaction costs and no evaluation protocol of any kind."</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Unconditional z-score screen with a deliberately high threshold: z_t = (r_t − μ_r)/σ_r, flag if |z_t| &gt; 10 with μ_r, σ_r over the whole 1980–2023 sample. Returns exactly three points: 19 Oct 1987 at −20.47, 13 Oct 2008 at +11.58, 16 Mar 2020 at −11.98. Nulls injected at 20 Oct 1987, 14 Oct 2008, 12 Mar 2020.  Screen → question-formulating agent → three expert agents → consolidation agent → three-persona manager panel via AutoGen → human analyst briefing. "the terminal step, a briefing to a human analyst who makes the call, where my orchestrator has to emit the decision itself, so nothing here tells me how to close the loop." AGENTS &amp; ORCHESTRATION (exhaustive): One question-formulating agent; three expert agents (web research, curated institutional knowledge base, cross-checking against an external API); one consolidation agent; a panel of three manager personas (financial market economist, macro economist, statistician) plus a moderator and a critic. Expert layer is explicitly extensible — "the diagram has a fourth empty box, so the expert set is meant to be configured per dataset rather than fixed." Critical axis distinction: "Park's three experts are heterogeneous by evidence source, web search, a curated knowledge base, and an external API, and all three answer the same question. That is redundancy for verification rather than diversity for decision, and it means agreement between his agents is corroboration while agreement between mine would be a weak signal at best." State-conditioned influence: NONE. "as in TradingAgents and FinVision, there is no weight, no confidence scalar and no quantity anywhere that could be weighted. Consolidation is an LLM summarising free text." But note the one exception in behaviour: resolution by evidence type, below.</t>
+          <t>Unconditional z-score screen with a deliberately high threshold: z_t = (r_t − μ_r)/σ_r, flag if |z_t| &gt; 10 with μ_r, σ_r over the whole 1980–2023 sample. Returns exactly three points: 19 Oct 1987 at −20.47, 13 Oct 2008 at +11.58, 16 Mar 2020 at −11.98. Nulls injected at 20 Oct 1987, 14 Oct 2008, 12 Mar 2020. Screen → question-formulating agent → three expert agents → consolidation agent → three-persona manager panel via AutoGen → human analyst briefing. "the terminal step, a briefing to a human analyst who makes the call, where my orchestrator has to emit the decision itself, so nothing here tells me how to close the loop." AGENTS &amp; ORCHESTRATION (exhaustive): One question-formulating agent; three expert agents (web research, curated institutional knowledge base, cross-checking against an external API); one consolidation agent; a panel of three manager personas (financial market economist, macro economist, statistician) plus a moderator and a critic. Expert layer is explicitly extensible - "the diagram has a fourth empty box, so the expert set is meant to be configured per dataset rather than fixed." Critical axis distinction: "Park's three experts are heterogeneous by evidence source, web search, a curated knowledge base, and an external API, and all three answer the same question. That is redundancy for verification rather than diversity for decision, and it means agreement between his agents is corroboration while agreement between mine would be a weak signal at best." State-conditioned influence: NONE. "as in TradingAgents and FinVision, there is no weight, no confidence scalar and no quantity anywhere that could be weighted. Consolidation is an LLM summarising free text." But note the one exception in behaviour: resolution by evidence type, below.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Only the pooled unconditional σ_r in the screen, which the student attacks: "Pooling σ_r across quiet and turbulent regimes ignores volatility clustering, so the screen systematically under-flags in calm periods and over-flags in crises, and the threshold of 10 papers over this by returning only the three largest days in the sample." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): None — no positions and therefore no cost model. There are also "no cost or runtime figures anywhere in the paper."</t>
+          <t>Only the pooled unconditional σ_r in the screen, which the student attacks: "Pooling σ_r across quiet and turbulent regimes ignores volatility clustering, so the screen systematically under-flags in calm periods and over-flags in crises, and the threshold of 10 papers over this by returning only the three largest days in the sample." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): None - no positions and therefore no cost model. There are also "no cost or runtime figures anywhere in the paper."</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Each expert must begin with Correct / Incorrect / Uncertain and then give one sentence of reasoning — "a fixed, comparable output vocabulary imposed across agents that share nothing else." Full transcripts of the consolidation and management discussion are reproduced.</t>
+          <t>Each expert must begin with Correct / Incorrect / Uncertain and then give one sentence of reasoning - "a fixed, comparable output vocabulary imposed across agents that share nothing else." Full transcripts of the consolidation and management discussion are reproduced.</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>All three experts returned Correct on all three genuine outliers, citing different evidence — the Fed's history and the Dow's 22.6% fall (1987), a CNN report of an 11.8% gain (2008), a CNBC 12% single-day drop (2020). "Three independent evidence paths converging is the demonstration's one clean result, and it is worth very little, because Black Monday, the October 2008 rebound and the COVID crash are three of the most documented days in market history and all three sit inside the backbone's pre-training. The framework is never shown an anomaly it could plausibly get wrong." On the injected nulls: web research returned Uncertain, institutional knowledge returned Uncertain, and the cross-checking agent retrieved the true values 236.83, 998.01 and 2711.02 from the API. "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." Consolidation: "Two Uncertains and one grounded Correct produced a Correct, not a hedge." LIMITATIONS (quoted): "There is no evaluation." "The hard case for alert triage is the one the paper concedes and does not attempt" — "That is the real operating regime for anomaly validation, a mid-sized move in a lightly covered name with no press coverage, and it is exactly what the CSE looks like. On this evidence I cannot tell how the framework behaves there, only that two of its three experts would abstain." "An unconditional z-score over 44 years is the wrong screen, and the choice of 10 hides the consequence." "The multi-agent structure is never shown to be necessary" — "the case for separating them rests entirely on the cross-check channel, which is a tool-access argument rather than an agent-architecture argument." "The discussion layer's objective makes disagreement a failure state" — "a panel that converges immediately has satisfied its objective, and the moderator and critic roles have no incentive structure that would reward dissent." And on the critic: "A critic role that only commends is a critic in name, and the layer that consumes the most tokens in the paper is the one that changes nothing about the output."</t>
+          <t>All three experts returned Correct on all three genuine outliers, citing different evidence - the Fed's history and the Dow's 22.6% fall (1987), a CNN report of an 11.8% gain (2008), a CNBC 12% single-day drop (2020). "Three independent evidence paths converging is the demonstration's one clean result, and it is worth very little, because Black Monday, the October 2008 rebound and the COVID crash are three of the most documented days in market history and all three sit inside the backbone's pre-training. The framework is never shown an anomaly it could plausibly get wrong." On the injected nulls: web research returned Uncertain, institutional knowledge returned Uncertain, and the cross-checking agent retrieved the true values 236.83, 998.01 and 2711.02 from the API. "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." Consolidation: "Two Uncertains and one grounded Correct produced a Correct, not a hedge." LIMITATIONS (quoted): "There is no evaluation." "The hard case for alert triage is the one the paper concedes and does not attempt" - "That is the real operating regime for anomaly validation, a mid-sized move in a lightly covered name with no press coverage, and it is exactly what the CSE looks like. On this evidence I cannot tell how the framework behaves there, only that two of its three experts would abstain." "An unconditional z-score over 44 years is the wrong screen, and the choice of 10 hides the consequence." "The multi-agent structure is never shown to be necessary" - "the case for separating them rests entirely on the cross-check channel, which is a tool-access argument rather than an agent-architecture argument." "The discussion layer's objective makes disagreement a failure state" - "a panel that converges immediately has satisfied its objective, and the moderator and critic roles have no incentive structure that would reward dissent." And on the critic: "A critic role that only commends is a critic in name, and the layer that consumes the most tokens in the paper is the one that changes nothing about the output."</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
@@ -1040,22 +1040,22 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>The Correct/Incorrect/Uncertain output contract, with the abstain label as the valuable part; resolution by evidence type as a possible structure on f(·); metadata-as-bridge for A_F; the identifier-resolution pattern as a shape to reuse but not a mechanism to trust on CSE names; and a scaled-down two-channel version of the loop as a CSE data-preparation utility — "a conditional-volatility screen for candidates and a cross-check against an independent source such as the exchange's own published data, with the Correct, Incorrect, Uncertain contract retained so the output is auditable. That is a data preparation utility and a line in the methodology chapter, and it should be described as such rather than dressed up as a contribution."</t>
+          <t>The Correct/Incorrect/Uncertain output contract, with the abstain label as the valuable part; resolution by evidence type as a possible structure on f(·); metadata-as-bridge for A_F; the identifier-resolution pattern as a shape to reuse but not a mechanism to trust on CSE names; and a scaled-down two-channel version of the loop as a CSE data-preparation utility - "a conditional-volatility screen for candidates and a cross-check against an independent source such as the exchange's own published data, with the Correct, Incorrect, Uncertain contract retained so the output is auditable. That is a data preparation utility and a line in the methodology chapter, and it should be described as such rather than dressed up as a contribution."</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>No decision, no weighting, no evaluation, and — explicitly — "nothing tests what happens when two agents assert contradictory Corrects."</t>
+          <t>No decision, no weighting, no evaluation, and - explicitly - "nothing tests what happens when two agents assert contradictory Corrects."</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>SPEAKS TO: Orchestrator (primary — the output contract and the structural-versus-learned weight question), A_V and A_L jointly (the conditional-screen argument), A_F (metadata), evaluation layer / data preparation.
-EFFECT ON MAIN GAP: Two contributions. It supplies the only worked example of heterogeneous agents disagreeing and the disagreement being resolved correctly, and it was resolved by evidence type rather than vote — which raises a structural question about f(·): "I would put this to the supervisor as a question about whether w_{i,t} should be partly structural rather than entirely learned, and flag that a single anecdote in a paper with no evaluation is thin evidence for it." It also extends the no-weightable-quantity finding to a third, much smaller design.
+          <t>SPEAKS TO: Orchestrator (primary - the output contract and the structural-versus-learned weight question), A_V and A_L jointly (the conditional-screen argument), A_F (metadata), evaluation layer / data preparation.
+EFFECT ON MAIN GAP: Two contributions. It supplies the only worked example of heterogeneous agents disagreeing and the disagreement being resolved correctly, and it was resolved by evidence type rather than vote - which raises a structural question about f(·): "I would put this to the supervisor as a question about whether w_{i,t} should be partly structural rather than entirely learned, and flag that a single anecdote in a paper with no evaluation is thin evidence for it." It also extends the no-weightable-quantity finding to a third, much smaller design.
 EFFECT ON SUB-GAP 1: None.
 EFFECT ON SUB-GAP 2: Indirect but concrete. The unconditional-σ critique is a direct argument for conditional volatility as the standardising quantity, and it produces the A_V/A_L interaction requirement: "In the CSE the correction is not sufficient on its own, because a stock that has not traded for several days produces a large printed return on its next trade that is a staleness artefact rather than a volatility event, and telling those apart is A_L's job. So an A_V flag on a thin name is uninterpretable without the A_L state alongside it, which is a case against treating the four channels as fully independent producers and an argument that at least this pair needs a defined interaction."
 FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of the no-mechanism-to-notice kind. Two of three experts contributed nothing on the only discriminating case and the architecture had no way to register it: "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." And the deliberation layer as dead weight: "the layer that consumes the most tokens in the paper is the one that changes nothing about the output." Student's cross-paper conclusion: "This is the same collapse as in TradingAgents' debate rounds but reached at much smaller scale and without a role hierarchy, so it does not look like an artefact of any one design."
-PROPOSED REVISION STATED IN THE NOTE: Two, both to the conditioning set, both flagged for the supervisor. On C_{i,t}: "The proposed refinement to C_{i,t} is that no evidence and low confidence are different states and should weight differently, which is a change to the conditioning set rather than a tuning detail, and it belongs in the discussion with the supervisor about what C_{i,t} actually is." On the form of f(·): "this argues that the weighting function should know something about the kind of evidence behind each agent's output, since direct market data underneath A_T, A_V and A_L and retrieved report text underneath A_F are not the same epistemic quality and collapsing them into one comparable confidence number assumes they are." And on the agent pool — a defined pairwise interaction rather than four independent producers: "an argument that at least this pair needs a defined interaction."</t>
+PROPOSED REVISION STATED IN THE NOTE: Two, both to the conditioning set, both flagged for the supervisor. On C_{i,t}: "The proposed refinement to C_{i,t} is that no evidence and low confidence are different states and should weight differently, which is a change to the conditioning set rather than a tuning detail, and it belongs in the discussion with the supervisor about what C_{i,t} actually is." On the form of f(·): "this argues that the weighting function should know something about the kind of evidence behind each agent's output, since direct market data underneath A_T, A_V and A_L and retrieved report text underneath A_F are not the same epistemic quality and collapsing them into one comparable confidence number assumes they are." And on the agent pool - a defined pairwise interaction rather than four independent producers: "an argument that at least this pair needs a defined interaction."</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Three gaps — prior surveys are either broader-economics or RL textbooks; no prior survey dissects RL by agent component through a finance lens; "The field's own evaluation standards have not been examined." Student's verdict: "This is not framed as the headline contribution, and it is the one the survey delivers most convincingly."</t>
+          <t>Three gaps - prior surveys are either broader-economics or RL textbooks; no prior survey dissects RL by agent component through a finance lens; "The field's own evaluation standards have not been examined." Student's verdict: "This is not framed as the headline contribution, and it is the one the survey delivers most convincingly."</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1235,12 +1235,12 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Not applicable — a survey. Classification: model-free value-based (critic-only) 89 total (DQN 37, Q-learning 36, SARSA 10, other 6); model-free policy-based (actor-only) 56 (RRL 31, policy gradient 13, REINFORCE 5, other 7); actor-critic 52 (DDPG 14, PPO 14, DPG 6, A2C 4, TRPO 2, other 12); model-based 3. "Those counts sum to 200 against 167 publications because several papers are classified under more than one category, which the authors state and never quantify, so the per-method figures are indicative rather than shares."</t>
+          <t>Not applicable - a survey. Classification: model-free value-based (critic-only) 89 total (DQN 37, Q-learning 36, SARSA 10, other 6); model-free policy-based (actor-only) 56 (RRL 31, policy gradient 13, REINFORCE 5, other 7); actor-critic 52 (DDPG 14, PPO 14, DPG 6, A2C 4, TRPO 2, other 12); model-based 3. "Those counts sum to 200 against 167 publications because several papers are classified under more than one category, which the authors state and never quantify, so the per-method figures are indicative rather than shares."</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Component-wise taxonomy — environment and features, action space, reward function, method families — then augmentations (transfer learning, imitation learning, policy distillation, ensembles, multi-agent) and applications, closing with "a sustained critique of evaluation practice in its own field."  Three formulas the student keeps. Moody and Wu's recurrent reinforcement learning (31 of 167 papers): A_t = sign(u·A_{t−1} + v_0·r_t + v_1·r_{t−1} + … + v_m·r_{t−m} + ω) with θ = {u, v_i, ω}. "That recurrence is what makes transaction costs expressible inside the objective rather than subtracted afterwards." The additive-profits utility: U_t(θ) = P_T = Σ_{t=1}^{T} R_t = μ Σ_{t=1}^{T} { r_t^f + A_{t−1}(r_t − r_t^f) − δ_t |A_t − A_{t−1}| } with μ a fixed position size, r_t and r_t^f the risky and risk-free returns, δ_t the transaction cost. "The cost term is proportional to the change in position, so an agent that churns pays for it inside the quantity it is maximising." And Hens and Wöhrmann's dynamic allocation: R_t^P = w_t^θ · R_t^B + (1 − w_t^θ) · R_t^E with w_t ∈ [0,1] under an exponential parametric function of θ. "Two producers, one weight, one parametric form." AGENTS &amp; ORCHESTRATION (exhaustive): Surveyed multi-agent RL in finance is a handful of systems — Lee and Jagmin's four-agent decomposition into buy-signal, buy-order, sell-signal and sell-order agents; MAPS, "where each agent manages its own portfolio and the loss is a weighted average of a global loss and individual local losses with a term rewarding diversity of actions"; AbdelKawy's synchronous DQN and DDPG model with transfer learning between stocks; and Shavandi and Khedmati's three agents at one-hour, fifteen-minute and five-minute frequencies "where the lowest-frequency output feeds the higher-frequency agents". Does anything vary influence by market state? No. The survey's own assessment: "existing literature restricts its focus to a few agents, that scalability is a key challenge, and that establishing coordination and communication protocols among agents is underexplored." MAPS' weighted global/local loss is the only weighting in the surveyed multi-agent work, and it is a training objective rather than a state-conditioned influence.</t>
+          <t>Component-wise taxonomy - environment and features, action space, reward function, method families - then augmentations (transfer learning, imitation learning, policy distillation, ensembles, multi-agent) and applications, closing with "a sustained critique of evaluation practice in its own field." Three formulas the student keeps. Moody and Wu's recurrent reinforcement learning (31 of 167 papers): A_t = sign(u·A_{t−1} + v_0·r_t + v_1·r_{t−1} + … + v_m·r_{t−m} + ω) with θ = {u, v_i, ω}. "That recurrence is what makes transaction costs expressible inside the objective rather than subtracted afterwards." The additive-profits utility: U_t(θ) = P_T = Σ_{t=1}^{T} R_t = μ Σ_{t=1}^{T} { r_t^f + A_{t−1}(r_t − r_t^f) − δ_t |A_t − A_{t−1}| } with μ a fixed position size, r_t and r_t^f the risky and risk-free returns, δ_t the transaction cost. "The cost term is proportional to the change in position, so an agent that churns pays for it inside the quantity it is maximising." And Hens and Wöhrmann's dynamic allocation: R_t^P = w_t^θ · R_t^B + (1 − w_t^θ) · R_t^E with w_t ∈ [0,1] under an exponential parametric function of θ. "Two producers, one weight, one parametric form." AGENTS &amp; ORCHESTRATION (exhaustive): Surveyed multi-agent RL in finance is a handful of systems - Lee and Jagmin's four-agent decomposition into buy-signal, buy-order, sell-signal and sell-order agents; MAPS, "where each agent manages its own portfolio and the loss is a weighted average of a global loss and individual local losses with a term rewarding diversity of actions"; AbdelKawy's synchronous DQN and DDPG model with transfer learning between stocks; and Shavandi and Khedmati's three agents at one-hour, fifteen-minute and five-minute frequencies "where the lowest-frequency output feeds the higher-frequency agents". Does anything vary influence by market state? No. The survey's own assessment: "existing literature restricts its focus to a few agents, that scalability is a key challenge, and that establishing coordination and communication protocols among agents is underexplored." MAPS' weighted global/local loss is the only weighting in the surveyed multi-agent work, and it is a training objective rather than a state-conditioned influence.</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -1255,12 +1255,12 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>None — coverage ends in 2022, before the LLM-agent literature.</t>
+          <t>None - coverage ends in 2022, before the LLM-agent literature.</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>The POMDP argument is the load-bearing item. "The Markov decision process assumes the environment is fully observable and that the next state depends only on the current state and action. The survey argues plainly that this does not hold in markets: empirical evidence shows longer memory driven by investor behaviour, economic cycles and external events, introducing dependencies that extend beyond immediate state transitions, so a partially observable MDP is the appropriate frame and transition probabilities are approximated with LSTMs and RNNs rather than modelled. The survey then states that models incorporating memory effects significantly outperform those built on the Markov assumption, particularly for long-term trends and market anomalies." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Field-level finding. "RL models often simplify transaction costs as fixed and assume certainty of execution, overlooking market realities such as varying bid-ask spreads, with only some studies incorporating execution and slippage costs." Separately on order execution: "the literature often presupposes immediate execution of trading positions, with only a few frameworks such as Wang et al.'s hierarchical model including an execution module." The one modelled form is δ_t|A_t − A_{t−1}| — proportional to position change, not to order size against depth.</t>
+          <t>The POMDP argument is the load-bearing item. "The Markov decision process assumes the environment is fully observable and that the next state depends only on the current state and action. The survey argues plainly that this does not hold in markets: empirical evidence shows longer memory driven by investor behaviour, economic cycles and external events, introducing dependencies that extend beyond immediate state transitions, so a partially observable MDP is the appropriate frame and transition probabilities are approximated with LSTMs and RNNs rather than modelled. The survey then states that models incorporating memory effects significantly outperform those built on the Markov assumption, particularly for long-term trends and market anomalies." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Field-level finding. "RL models often simplify transaction costs as fixed and assume certainty of execution, overlooking market realities such as varying bid-ask spreads, with only some studies incorporating execution and slippage costs." Separately on order execution: "the literature often presupposes immediate execution of trading positions, with only a few frameworks such as Wang et al.'s hierarchical model including an execution module." The one modelled form is δ_t|A_t − A_{t−1}| - proportional to position change, not to order size against depth.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -1270,17 +1270,17 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>Not a focus; the survey's contribution here is the overengineering critique — "the vast array of alternative solutions across varied architectures makes it difficult to identify superior approaches or pinpoint the essential components within a given solution."</t>
+          <t>Not a focus; the survey's contribution here is the overengineering critique - "the vast array of alternative solutions across varied architectures makes it difficult to identify superior approaches or pinpoint the essential components within a given solution."</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>The survey's strongest section. Four named criticisms: unbalanced benchmarks ("the RL framework uses a different information set than the benchmark, so comparing an RL portfolio manager against Markowitz is not a like-for-like test"); implausible Sharpe ratios — "a reported Sharpe of 21.2 in one paper and 217.68 in another", attributed to "overfitting, data snooping and forward-looking bias where prices are observed at time t and actions taken at the same time"; survivorship bias, "with frameworks tested on Apple and similar survivors while bankrupt and delisted names are neglected"; and "attempts to justify methodological complexity are described as sparse."</t>
+          <t>The survey's strongest section. Four named criticisms: unbalanced benchmarks ("the RL framework uses a different information set than the benchmark, so comparing an RL portfolio manager against Markowitz is not a like-for-like test"); implausible Sharpe ratios - "a reported Sharpe of 21.2 in one paper and 217.68 in another", attributed to "overfitting, data snooping and forward-looking bias where prices are observed at time t and actions taken at the same time"; survivorship bias, "with frameworks tested on Apple and similar survivors while bankrupt and delisted names are neglected"; and "attempts to justify methodological complexity are described as sparse."</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>The classification distribution is the one quantitative artefact — 89 / 56 / 52 / 3. "value-based methods dominate despite being restricted to discrete action spaces, actor-critic is described as the most compelling of the four and is among the least represented, and model-based RL stands at three papers out of 167." 27.5% predate 2016. LIMITATIONS (quoted): "Coverage ends in 2022 and the paper was published in 2025, which removes the entire LLM-agent literature" — "it also means the multi-agent assessment, which is the section I lean on most, was written before the systems I am actually comparing against existed." "There is no quantitative synthesis of outcomes anywhere in 167 papers" — "no performance claim can be cited from here." "The critique section names problems and quantifies none of them" — "I can cite it for the existence of each problem but not for its prevalence." "The classification counts exceed the publication count and the overlap is never reported." "Selection is Google Scholar plus snowballing with no stated inclusion criteria or screening counts... The sample is not reproducible." "A declared conflict of interest, which I record rather than weight."</t>
+          <t>The classification distribution is the one quantitative artefact - 89 / 56 / 52 / 3. "value-based methods dominate despite being restricted to discrete action spaces, actor-critic is described as the most compelling of the four and is among the least represented, and model-based RL stands at three papers out of 167." 27.5% predate 2016. LIMITATIONS (quoted): "Coverage ends in 2022 and the paper was published in 2025, which removes the entire LLM-agent literature" - "it also means the multi-agent assessment, which is the section I lean on most, was written before the systems I am actually comparing against existed." "There is no quantitative synthesis of outcomes anywhere in 167 papers" - "no performance claim can be cited from here." "The critique section names problems and quantifies none of them" - "I can cite it for the existence of each problem but not for its prevalence." "The classification counts exceed the publication count and the overlap is never reported." "Selection is Google Scholar plus snowballing with no stated inclusion criteria or screening counts... The sample is not reproducible." "A declared conflict of interest, which I record rather than weight."</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>External validation of the orchestration gap; Hens and Wöhrmann as lineage for the weighting function; the POMDP argument as theoretical support for P_t; the friction critique as generalising the per-paper tally; Section 8 as a pre-registered evaluation checklist; and hierarchical RL / multi-objective RL as the vocabulary for positioning against the RL literature — "'a coordination layer over heterogeneous specialised agents, conditioned on market state' is the description, and HRL and multi-objective RL are the two labels the survey hands me for it."</t>
+          <t>External validation of the orchestration gap; Hens and Wöhrmann as lineage for the weighting function; the POMDP argument as theoretical support for P_t; the friction critique as generalising the per-paper tally; Section 8 as a pre-registered evaluation checklist; and hierarchical RL / multi-objective RL as the vocabulary for positioning against the RL literature - "'a coordination layer over heterogeneous specialised agents, conditioned on market state' is the description, and HRL and multi-objective RL are the two labels the survey hands me for it."</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
@@ -1301,11 +1301,11 @@
       <c r="W6" s="3" t="inlineStr">
         <is>
           <t>SPEAKS TO: Orchestrator (primary), A_V (POMDP / persistence), A_L (friction convention), evaluation layer (Section 8 checklist).
-EFFECT ON MAIN GAP: The strongest external validation in the set. "An ACM survey of 167 papers states my orchestration gap as an open problem, which is the strongest external support I have for it" — specifically "the establishment of coordination and communication protocols among different agents is underexplored". It also converts the contribution from novel machinery into a generalisation: "My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) generalises it along three axes at once, from two producers to four heterogeneous ones, from a parametric function of time to a function of market state, and from asset-class returns to agent outputs. Positioning the contribution as a generalisation of a known and cited form is a better framing for the proposal than presenting it as novel machinery."
+EFFECT ON MAIN GAP: The strongest external validation in the set. "An ACM survey of 167 papers states my orchestration gap as an open problem, which is the strongest external support I have for it" - specifically "the establishment of coordination and communication protocols among different agents is underexplored". It also converts the contribution from novel machinery into a generalisation: "My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) generalises it along three axes at once, from two producers to four heterogeneous ones, from a parametric function of time to a function of market state, and from asset-class returns to agent outputs. Positioning the contribution as a generalisation of a known and cited form is a better framing for the proposal than presenting it as novel machinery."
 EFFECT ON SUB-GAP 1: Generalises it from anecdote to documented convention. "So this is not four papers being careless, it is a documented convention, and the RRL utility above shows the form the cost term takes when it is modelled at all, δ_t|A_t − A_{t−1}| proportional to the position change. The CSE version has to extend that with a spread that is a real cost rather than a rounding error and an impact term that is separate rather than folded in."
 EFFECT ON SUB-GAP 2: The strongest theoretical support yet, and the note says so explicitly. "That is a direct theoretical argument for conditioning on persistence, which is the input in my weighting function I have had the least external support for." And: "what this adds is the framing that persistence is not just a property of the data, it is the reason the standard formalism does not fit, which is a stronger argument to put in the proposal."
 FIXED-INFLUENCE FAILURE EVIDENCE: Not a specific degradation case, but the field-level statement of why such cases go unnoticed: "the vast array of alternative solutions across varied architectures makes it difficult to identify superior approaches or pinpoint the essential components within a given solution." Plus the Sharpe examples (21.2 and 217.68) as evidence that the field's evaluation practice would not catch a component doing nothing or doing harm.
-PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool or to the conditioning set — instead an explicit strengthening of P_t's justification and a data-collection decision. Verbatim: "The survey's claim that markets exhibit memory extending beyond immediate state transitions, and that models incorporating those effects significantly outperform Markov-based ones, is the reason P_t belongs in the conditioning set alongside liquidity and volatility rather than being the speculative fourth item." And: "Survivorship-aware universe, which for the CSE means including delisted and suspended counters rather than the currently listed set, and that is a data-collection decision I need to make before the dataset is fixed rather than after." Also a conditional prior on the orchestrator's form: "If the orchestrator ever becomes a learned policy over a continuous weight simplex, the survey's steer is actor-critic... That is a prior to hold, not a decision to take now."</t>
+PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool or to the conditioning set - instead an explicit strengthening of P_t's justification and a data-collection decision. Verbatim: "The survey's claim that markets exhibit memory extending beyond immediate state transitions, and that models incorporating those effects significantly outperform Markov-based ones, is the reason P_t belongs in the conditioning set alongside liquidity and volatility rather than being the speculative fourth item." And: "Survivorship-aware universe, which for the CSE means including delisted and suspended counters rather than the currently listed set, and that is a data-collection decision I need to make before the dataset is fixed rather than after." Also a conditional prior on the orchestrator's form: "If the orchestrator ever becomes a learned policy over a continuous weight simplex, the survey's steer is actor-critic... That is a prior to hold, not a decision to take now."</t>
         </is>
       </c>
       <c r="X6" s="3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>arXiv:2311.11944v1, 20 November 2023. Pranab Islam, Anand Kannappan, Douwe Kiela, Rebecca Qian, Nino Scherrer, Bertie Vidgen — Patronus AI, Contextual AI, Stanford.</t>
+          <t>arXiv:2311.11944v1, 20 November 2023. Pranab Islam, Anand Kannappan, Douwe Kiela, Rebecca Qian, Nino Scherrer, Bertie Vidgen - Patronus AI, Contextual AI, Stanford.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>"Existing financial QA datasets do not test retrieval, so they evaluate a task analysts are not actually delegating" — FiQA is aspect-based sentiment; FinQA, ConvFinQA and TAT-QA hand over the context. "This is the real contribution and it is the reason the paper matters to me more than its two siblings do." Plus: generic QA benchmarks don't transfer; and a procurement argument about deployment readiness.</t>
+          <t>"Existing financial QA datasets do not test retrieval, so they evaluate a task analysts are not actually delegating" - FiQA is aspect-based sentiment; FinQA, ConvFinQA and TAT-QA hand over the context. "This is the real contribution and it is the reason the paper matters to me more than its two siblings do." Plus: generic QA benchmarks don't transfer; and a procurement argument about deployment readiness.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>10,231 question/answer/evidence triplets, 40 US-listed companies, 361 public filings, 2015–2023. Document mix 270 10Ks, 29 8Ks, 29 earnings reports, 27 10Qs, 5 annual reports — but "10Ks carry 9,530 of the questions, 93% of the total, so despite the four document types this is effectively an annual-filing benchmark." Nine of eleven GICS sectors, IT at 25% of questions down to Materials at 1.8%. Question types: domain-relevant 925 (25 generic analyst questions posed to every company, 37 of 40 companies); novel generated 1,323 (annotator-written, 37 of 40); metrics-generated 7,983 (18 base metrics from the three statements 2015–2022, derivative metrics computed, template-built, 32 of 40). Reasoning taxonomy over n = 8,908: information extraction 2,493 (28%), numerical reasoning 5,897 (66%), logical reasoning 518 (6%). Human evaluation set 150 cases (50 per type), "not stratified by company, year or industry." Tested November 2023, temperature 0.01, 2,048-token cap, default system prompts.</t>
+          <t>10,231 question/answer/evidence triplets, 40 US-listed companies, 361 public filings, 2015–2023. Document mix 270 10Ks, 29 8Ks, 29 earnings reports, 27 10Qs, 5 annual reports - but "10Ks carry 9,530 of the questions, 93% of the total, so despite the four document types this is effectively an annual-filing benchmark." Nine of eleven GICS sectors, IT at 25% of questions down to Materials at 1.8%. Question types: domain-relevant 925 (25 generic analyst questions posed to every company, 37 of 40 companies); novel generated 1,323 (annotator-written, 37 of 40); metrics-generated 7,983 (18 base metrics from the three statements 2015–2022, derivative metrics computed, template-built, 32 of 40). Reasoning taxonomy over n = 8,908: information extraction 2,493 (28%), numerical reasoning 5,897 (66%), logical reasoning 518 (6%). Human evaluation set 150 cases (50 per type), "not stratified by company, year or industry." Tested November 2023, temperature 0.01, 2,048-token cap, default system prompts.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1367,17 +1367,17 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>No model and no mathematics. Five settings crossed with two prompt orders. Settings ladder: closed book (question alone, naive floor), shared vector store (one Chroma store over all 360 documents, "the realistic industry setup"), single vector store (one store per document, "presumes the document is already identified"), long context (whole filing truncated to 95,000–100,000 tokens), oracle (the annotator's evidence page, "unrealistic ceiling"). Langchain + Chroma + OpenAI text-embedding-ada-002. "Chunking strategy, chunk size, number of retrieved chunks and any reranking are not described." Prompt order: Context-First puts the question then the filing; Context-Last reverses.  Sixteen configurations of GPT-4, GPT-4-Turbo, Llama2, Claude2; 2,400 responses on the 150-case sample hand-labelled correct / incorrect / failure to answer.</t>
+          <t>No model and no mathematics. Five settings crossed with two prompt orders. Settings ladder: closed book (question alone, naive floor), shared vector store (one Chroma store over all 360 documents, "the realistic industry setup"), single vector store (one store per document, "presumes the document is already identified"), long context (whole filing truncated to 95,000–100,000 tokens), oracle (the annotator's evidence page, "unrealistic ceiling"). Langchain + Chroma + OpenAI text-embedding-ada-002. "Chunking strategy, chunk size, number of retrieved chunks and any reranking are not described." Prompt order: Context-First puts the question then the filing; Context-Last reverses. Sixteen configurations of GPT-4, GPT-4-Turbo, Llama2, Claude2; 2,400 responses on the 150-case sample hand-labelled correct / incorrect / failure to answer.</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Not applicable — no agents. Relevance is to A_F's task shape and to the orchestrator's input contract.</t>
+          <t>Not applicable - no agents. Relevance is to A_F's task shape and to the orchestrator's input contract.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>None, and explicitly criticised as the wrong task — FiQA's aspect-based sentiment "is a small slice of what analysts ask."</t>
+          <t>None, and explicitly criticised as the wrong task - FiQA's aspect-based sentiment "is a small slice of what analysts ask."</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
@@ -1392,12 +1392,12 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>None — no trading. The only cost discussion is the latency and cost of long-context, "which the authors call impractical."</t>
+          <t>None - no trading. The only cost discussion is the latency and cost of long-context, "which the authors call impractical."</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>The three-way label taxonomy, definitions intact. Correct allows good-faith deviations (billions where millions were asked, very small rounding errors). Incorrect spans small-margin to order-of-magnitude errors and includes "a right answer reached with logic or calculations that explicitly contradict the gold evidence" — "That third rule in the Incorrect definition is the one that makes this a test of the reasoning chain rather than of the final number, and it is the reason the taxonomy suits a channel whose explainability story is citation tracing." Failure to answer requires an explicit statement of lacking access.</t>
+          <t>The three-way label taxonomy, definitions intact. Correct allows good-faith deviations (billions where millions were asked, very small rounding errors). Incorrect spans small-margin to order-of-magnitude errors and includes "a right answer reached with logic or calculations that explicitly contradict the gold evidence" - "That third rule in the Incorrect definition is the one that makes this a test of the reasoning chain rather than of the final number, and it is the reason the taxonomy suits a channel whose explainability story is citation tracing." Failure to answer requires an explicit statement of lacking access.</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>Correct answers 9% closed book, 19% shared vector store, 50% single store, 76% and 79% long context, 85% oracle. "Handing the model the right page is worth 66 points over the realistic retrieval setting." Single-to-shared store: GPT-4-Turbo 50%→19%, Llama2 41%→19%, "purely from widening the search space from one filing to 360." Failure profiles at identical 19% correctness: GPT-4-Turbo refuses 68% and is wrong 13%; Llama2 wrong 70% and refuses 11%. Single store: GPT-4-Turbo 39% refusal / 11% wrong; Llama2 5% / 54%. Prompt order in long context: GPT-4-Turbo 25%→78%, Claude2 37%→76% — "a 53-point and a 39-point difference from moving one block of text"; reverses in the short oracle setting, 89% Context-Last against 85% Context-First. Metrics-generated questions weakest under retrieval, highest under long context and oracle (GPT-4-Turbo above 90%) — "which localises the difficulty to finding rather than computing." LIMITATIONS (quoted): "Only 150 of the 10,231 cases are public, so the headline scale is a claim about work done rather than a resource anyone can use" — "Every downstream paper citing FinanceBench is running the 150, including the chunking work." "Single run, single prompt per configuration, no dispersion and no significance test" — "On 150 cases the binomial standard error near 50% correctness is about 4.1 points, so a 95% interval on any single cell is roughly ±8 points and on a difference between two cells roughly ±11. That is enough to separate 19% from 50% comfortably and not enough to separate Llama2's 41% from GPT-4-Turbo's 50% in the same setting, a distinction the paper draws in prose without qualification." "The retrieval baseline is deliberately naive and the abstract then generalises from it" — "the defensible claim is that a default RAG pipeline fails on financial filings, not that retrieval fails, and the difference matters because the second version is the one this paper is usually cited for." "Dataset integrity issues are named and never quantified" — simplistic questions and contestable gold answers, neither given a share; "at 79% under long context the proportion of simplistic questions directly bounds what that number means, and it is not reported." "The annotation pipeline is described honestly and is thin at the points that determine label quality" — "this is the weakest quality-control story of the three." "Single-turn, single-company, large-cap and US-only" — "on a CSE annual report the extraction problem is harder before any question is asked."</t>
+          <t>Correct answers 9% closed book, 19% shared vector store, 50% single store, 76% and 79% long context, 85% oracle. "Handing the model the right page is worth 66 points over the realistic retrieval setting." Single-to-shared store: GPT-4-Turbo 50%→19%, Llama2 41%→19%, "purely from widening the search space from one filing to 360." Failure profiles at identical 19% correctness: GPT-4-Turbo refuses 68% and is wrong 13%; Llama2 wrong 70% and refuses 11%. Single store: GPT-4-Turbo 39% refusal / 11% wrong; Llama2 5% / 54%. Prompt order in long context: GPT-4-Turbo 25%→78%, Claude2 37%→76% - "a 53-point and a 39-point difference from moving one block of text"; reverses in the short oracle setting, 89% Context-Last against 85% Context-First. Metrics-generated questions weakest under retrieval, highest under long context and oracle (GPT-4-Turbo above 90%) - "which localises the difficulty to finding rather than computing." LIMITATIONS (quoted): "Only 150 of the 10,231 cases are public, so the headline scale is a claim about work done rather than a resource anyone can use" - "Every downstream paper citing FinanceBench is running the 150, including the chunking work." "Single run, single prompt per configuration, no dispersion and no significance test" - "On 150 cases the binomial standard error near 50% correctness is about 4.1 points, so a 95% interval on any single cell is roughly ±8 points and on a difference between two cells roughly ±11. That is enough to separate 19% from 50% comfortably and not enough to separate Llama2's 41% from GPT-4-Turbo's 50% in the same setting, a distinction the paper draws in prose without qualification." "The retrieval baseline is deliberately naive and the abstract then generalises from it" - "the defensible claim is that a default RAG pipeline fails on financial filings, not that retrieval fails, and the difference matters because the second version is the one this paper is usually cited for." "Dataset integrity issues are named and never quantified" - simplistic questions and contestable gold answers, neither given a share; "at 79% under long context the proportion of simplistic questions directly bounds what that number means, and it is not reported." "The annotation pipeline is described honestly and is thin at the points that determine label quality" - "this is the weakest quality-control story of the three." "Single-turn, single-company, large-cap and US-only" - "on a CSE annual report the extraction problem is harder before any question is asked."</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
@@ -1431,7 +1431,7 @@
 EFFECT ON MAIN GAP: Direct and substantial. It supplies the argument that the orchestrator must be designed around a channel that is frequently unusable: "the working assumption is that A_F will be wrong or will abstain on more than half of computed questions over CSE filings, and the orchestrator has to be designed for a channel that is frequently unusable rather than occasionally imperfect." And it separates two failure modes the weighting function must treat differently: "A refusal is A_F declining to produce evidence, which should drive w_{F,t} to zero and redistribute across the other three channels; a confident wrong answer is the case nothing in the weighting can detect and is where a hallucinating fundamental channel does real damage."
 EFFECT ON SUB-GAP 1: None.
 EFFECT ON SUB-GAP 2: None.
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes, and of the undetectable kind — the confident-wrong case. "a confident wrong answer is the case nothing in the weighting can detect and is where a hallucinating fundamental channel does real damage." Supporting evidence: Llama2 asserting wrongly 70% of the time at the same headline correctness as a model refusing 68% of the time — "a single correctness figure conceals two systems with completely different risk profiles."
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes, and of the undetectable kind - the confident-wrong case. "a confident wrong answer is the case nothing in the weighting can detect and is where a hallucinating fundamental channel does real damage." Supporting evidence: Llama2 asserting wrongly 70% of the time at the same headline correctness as a model refusing 68% of the time - "a single correctness figure conceals two systems with completely different risk profiles."
 PROPOSED REVISION STATED IN THE NOTE: Yes, and it is the third convergent instance. "abstention should be a distinct state rather than a low value of C_{F,t}. That is the third time the answer on confidence has come out as a structural property of the output rather than a self-reported score, after FinQA's program step count and TAT-QA's operator posterior, and the pattern is now firm enough to put to the supervisor as a refinement of the conditioning set."</t>
         </is>
       </c>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>arXiv:2402.05131v3, 16 March 2024. Antonio Jimeno Yepes, Yao You, Jan Milczek, Sebastian Laverde, Leah Li — Unstructured Technologies.</t>
+          <t>arXiv:2402.05131v3, 16 March 2024. Antonio Jimeno Yepes, Yao You, Jan Milczek, Sebastian Laverde, Leah Li - Unstructured Technologies.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>PDF pages processed by a vision encoder-decoder (Chipper) labelling regions by structural type — title, narrative text, list item, table.</t>
+          <t>PDF pages processed by a vision encoder-decoder (Chipper) labelling regions by structural type - title, narrative text, list item, table.</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>None. The only cost discussion is indexing cost, and it is one-sided — "a vision encoder-decoder pass over all 11,787 pages plus two GPT-4 calls per chunk for the keyword and summary indexes, against a tokenizer split for the baselines. The efficiency claim, 62,529 chunks against 112,155 for comparable retrieval, is a genuine result about index size and query latency, but it is offset by an indexing cost the paper never quantifies and which for a continuously updated corpus would recur."</t>
+          <t>None. The only cost discussion is indexing cost, and it is one-sided - "a vision encoder-decoder pass over all 11,787 pages plus two GPT-4 calls per chunk for the keyword and summary indexes, against a tokenizer split for the baselines. The efficiency claim, 62,529 chunks against 112,155 for comparable retrieval, is a genuine result about index size and query latency, but it is offset by an indexing cost the paper never quantifies and which for a continuously updated corpus would recur."</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>Page accuracy — Keywords Chipper 46.10, Summary 62.41, Prefix 67.38, against Base 512 at 68.09, Base 128 at 72.34, Base 256 at 73.05. "Every individual element-based index retrieves pages worse than every fixed-size baseline, which is the reverse of the paper's own summary." BLEU — 0.315 / 0.350 / 0.400 element against 0.181 / 0.231 / 0.250 baseline, "the worst element variant beats the best baseline on BLEU", and at aggregation 0.452 against 0.277, a 63% relative gain; ROUGE 0.514 against 0.455. Aggregation: Chipper 84.40 against Base 83.69, "a difference of one question out of 141", and it "exceeded GPT-4's token limit and yielded a non-effective Q&amp;A solution" so Table 5 has no aggregation rows. End to end (manual): Base 128 35.46, Base 256 36.88, Base 512 48.23, Keywords Chipper 53.19, Summary Chipper 51.77, Prefix &amp; Table Description Chipper 53.19. "No answer" column: 35.46, 25.53, 24.82, 22.70, 17.73, 20.57 — "Abstentions fall from 35.46% to as low as 17.73% while accuracy rises by about five points, so most of what better chunking buys is converting refusals into answers rather than converting wrong answers into right ones." Judge bias: trails manual by 6.38, 4.26, 6.39, 9.22, 8.04 and 12.06 points, "so the better the system the larger the understatement", with the named failure mode "a model correctly deriving 39.73% with the full calculation against a gold answer of '39.7%'", and it reorders the element variants. LIMITATIONS (quoted): "141 questions, one run, no dispersion, and the headline margins do not clear sampling error" — "At 141 cases the binomial standard error near 50% is about 4.2 points, so a difference between two configurations carries a 95% interval of roughly ±11.7 points. The 4.96-point Q&amp;A gain from Base 512 to the best element configuration sits well inside that, and the 0.71-point retrieval gain is one question." "The authors are evaluating their own commercial product, and the prose reads the tables more favourably than the numbers support" — "the two places where the summary overstates the tables... both run the same direction, and that is the pattern to read for." "The cost comparison is one-sided." "The benchmark was silently reduced and then compared against its own published numbers." "The retrieval metrics are coarse and none of them shows ranking position" — "There is no precision@k and no mean reciprocal rank anywhere, so nothing in the paper says whether the right chunk arrived first or tenth, which is the quantity that actually determines what fits in a generator prompt." "Table handling is the design's most distinctive rule and the least evidenced."</t>
+          <t>Page accuracy - Keywords Chipper 46.10, Summary 62.41, Prefix 67.38, against Base 512 at 68.09, Base 128 at 72.34, Base 256 at 73.05. "Every individual element-based index retrieves pages worse than every fixed-size baseline, which is the reverse of the paper's own summary." BLEU - 0.315 / 0.350 / 0.400 element against 0.181 / 0.231 / 0.250 baseline, "the worst element variant beats the best baseline on BLEU", and at aggregation 0.452 against 0.277, a 63% relative gain; ROUGE 0.514 against 0.455. Aggregation: Chipper 84.40 against Base 83.69, "a difference of one question out of 141", and it "exceeded GPT-4's token limit and yielded a non-effective Q&amp;A solution" so Table 5 has no aggregation rows. End to end (manual): Base 128 35.46, Base 256 36.88, Base 512 48.23, Keywords Chipper 53.19, Summary Chipper 51.77, Prefix &amp; Table Description Chipper 53.19. "No answer" column: 35.46, 25.53, 24.82, 22.70, 17.73, 20.57 - "Abstentions fall from 35.46% to as low as 17.73% while accuracy rises by about five points, so most of what better chunking buys is converting refusals into answers rather than converting wrong answers into right ones." Judge bias: trails manual by 6.38, 4.26, 6.39, 9.22, 8.04 and 12.06 points, "so the better the system the larger the understatement", with the named failure mode "a model correctly deriving 39.73% with the full calculation against a gold answer of '39.7%'", and it reorders the element variants. LIMITATIONS (quoted): "141 questions, one run, no dispersion, and the headline margins do not clear sampling error" - "At 141 cases the binomial standard error near 50% is about 4.2 points, so a difference between two configurations carries a 95% interval of roughly ±11.7 points. The 4.96-point Q&amp;A gain from Base 512 to the best element configuration sits well inside that, and the 0.71-point retrieval gain is one question." "The authors are evaluating their own commercial product, and the prose reads the tables more favourably than the numbers support" - "the two places where the summary overstates the tables... both run the same direction, and that is the pattern to read for." "The cost comparison is one-sided." "The benchmark was silently reduced and then compared against its own published numbers." "The retrieval metrics are coarse and none of them shows ranking position" - "There is no precision@k and no mean reciprocal rank anywhere, so nothing in the paper says whether the right chunk arrived first or tenth, which is the quantity that actually determines what fits in a generator prompt." "Table handling is the design's most distinctive rule and the least evidenced."</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -1544,12 +1544,12 @@
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>The four chunking rules, the three-index metadata design, and the generator prompt's explicit abstention instruction — "The transferable artefacts are the four chunking rules, the three-index metadata design, and the generator prompt's explicit abstention instruction, which is what makes the output comparable to FinanceBench's taxonomy." Plus: optimise for chunk precision not page hit rate; use precision@k or MRR; never use an LLM judge uncalibrated; and the indexing-cost planning number with the quarterly-rebuild mitigation.</t>
+          <t>The four chunking rules, the three-index metadata design, and the generator prompt's explicit abstention instruction - "The transferable artefacts are the four chunking rules, the three-index metadata design, and the generator prompt's explicit abstention instruction, which is what makes the output comparable to FinanceBench's taxonomy." Plus: optimise for chunk precision not page hit rate; use precision@k or MRR; never use an LLM judge uncalibrated; and the indexing-cost planning number with the quarterly-rebuild mitigation.</t>
         </is>
       </c>
       <c r="V8" s="3" t="inlineStr">
         <is>
-          <t>No table-sourced versus text-sourced accuracy split — "That split is exactly the one FinQA and TAT-QA both show behaves differently, so its absence here is the gap I most wanted filled." No ranking-position metric. No table-detection accuracy.</t>
+          <t>No table-sourced versus text-sourced accuracy split - "That split is exactly the one FinQA and TAT-QA both show behaves differently, so its absence here is the gap I most wanted filled." No ranking-position metric. No table-detection accuracy.</t>
         </is>
       </c>
       <c r="W8" s="3" t="inlineStr">
@@ -1558,7 +1558,7 @@
 EFFECT ON MAIN GAP: Reinforces FinanceBench's conclusion and states the design consequence explicitly: "the working expectation for A_F on CSE filings is firmly below half on computed questions. The design consequence is that the orchestrator's job is to remain useful with a channel that is right less than half the time, which is an argument for a clean abstention path and weight redistribution rather than for trying to engineer the fundamental channel up to reliability it is not going to reach."
 EFFECT ON SUB-GAP 1: None.
 EFFECT ON SUB-GAP 2: None.
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes, in a subtler form — an apparent improvement that may be a hidden degradation the system cannot see. "a chunking change that reduces abstentions by giving the agent enough context to guess is not obviously an improvement for a channel feeding a weighting function. So the reporting requirement for every A_F configuration is correct, incorrect and abstain side by side, and the quantity to check is whether the incorrect column grew while the abstain column shrank." Also the proxy-metric failure: the configuration with the worst page retrieval (Keywords Chipper, 46.10) has joint-best answer accuracy (53.19%), so "page-hit rate is the wrong retrieval proxy for predicting downstream answer quality" — a component metric that would have led the design in the wrong direction.
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes, in a subtler form - an apparent improvement that may be a hidden degradation the system cannot see. "a chunking change that reduces abstentions by giving the agent enough context to guess is not obviously an improvement for a channel feeding a weighting function. So the reporting requirement for every A_F configuration is correct, incorrect and abstain side by side, and the quantity to check is whether the incorrect column grew while the abstain column shrank." Also the proxy-metric failure: the configuration with the worst page retrieval (Keywords Chipper, 46.10) has joint-best answer accuracy (53.19%), so "page-hit rate is the wrong retrieval proxy for predicting downstream answer quality" - a component metric that would have led the design in the wrong direction.
 PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool or to f(L_t,V_t,P_t,C_{i,t}). The note's commitments are all internal to A_F and to reporting. Closest to a conditioning-set statement: the abstain-path argument, which restates rather than revises FinanceBench's.</t>
         </is>
       </c>
@@ -2073,12 +2073,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>2026 (online-first 2025)</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>IIM Ranchi Journal of Management Studies 5(1), pp. 21-45. DOI 10.1108/IRJMS-11-2024-0138</t>
+          <t>IIM Ranchi Journal of Management Studies 5(1), pp. 21-45, online-first 2025. DOI 10.1108/IRJMS-11-2024-0138</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note. There is no retrieval, no document corpus and no fundamental-data channel. The relevant cross-reference is to my explainability plan rather than to A_F: "The explainability component is attribution over risk features, RAG citation tracing, interpretable FIGARCH and GJR-GARCH parameters, and the orchestrator's weight vector, and this paper is a central-bank-grade instance of the first of those on a tree model."</t>
+          <t>None. There is no retrieval, no document corpus and no fundamental-data channel. The relevant cross-reference is to my explainability plan rather than to A_F: "The explainability component is attribution over risk features, RAG citation tracing, interpretable FIGARCH and GJR-GARCH parameters, and the orchestrator's weight vector, and this paper is a central-bank-grade instance of the first of those on a tree model."</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Prior reviews "organise the field by task coverage or by model-level benchmark performance and treat execution as an afterthought," producing three misclassifications — execution read as a byproduct of reasoning rather than a first-class architectural component, mechanism conflated with function (a multi-agent alpha-miner and a multi-agent trading system land in the same bucket), and adaptation treated as an implementation detail. Answer: the Architecture-Capability-Adaptation (A-C-A) lens, "offered explicitly as a working analytical lens rather than a validated taxonomy," plus an evidence ledger, a reproducibility audit and a reporting checklist, "which they name as the actual contributions."</t>
+          <t>Prior reviews "organise the field by task coverage or by model-level benchmark performance and treat execution as an afterthought," producing three misclassifications - execution read as a byproduct of reasoning rather than a first-class architectural component, mechanism conflated with function (a multi-agent alpha-miner and a multi-agent trading system land in the same bucket), and adaptation treated as an implementation detail. Answer: the Architecture-Capability-Adaptation (A-C-A) lens, "offered explicitly as a working analytical lens rather than a validated taxonomy," plus an evidence ledger, a reproducibility audit and a reporting checklist, "which they name as the actual contributions."</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Not a market study. Audited corpus is overwhelmingly US/crypto instruments; the note flags the named evaluation arenas (AI-Trader, Agent Market Arena, LiveTradeBench, ContestTrade, PredictionMarketBench) as "all of which are US or crypto instruments."  Agentic trading systems generally — alpha discovery, portfolio management, risk management, execution.</t>
+          <t>Not a market study. Audited corpus is overwhelmingly US/crypto instruments; the note flags the named evaluation arenas (AI-Trader, Agent Market Arena, LiveTradeBench, ContestTrade, PredictionMarketBench) as "all of which are US or crypto instruments." Agentic trading systems generally - alpha discovery, portfolio management, risk management, execution.</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -3908,12 +3908,12 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>Four-step screening (keyword search, dedup, title/abstract screening against the finance/trading domain, full-text screening assigning primary vs background). Two criteria decide the primary subset and "the whole paper hangs off them": *Action Output* (system emits tradable actions — orders, position changes, portfolio allocations) and *Closed-Loop Evaluation* (actions evaluated in backtest, simulation or live trading rather than only through predictive metrics).  Not a system. Three reimplementable rules the note singles out, "each is a rule rather than a model": 1. Reasoning module as a typed contract — f(O_t, M_episodic, P_portfolio) → (A_cand, α, V_check), where O_t is a timestamped state observation at decision time t, M_episodic retrievable episodic memory, P_portfolio read-only portfolio state (positions, risk limits), A_cand a set of candidate actions, α ∈ [0,1] a confidence score, V_check a validity check such as holds &lt; max_leverage. Purpose: "risk constraints are enforced during or immediately after reasoning rather than at the final execution layer, so a hallucinated action never reaches the order interface." 2. Outcome Embargo against the "Oracle Fallacy" (retrieving a past episode whose stored text already contains a post-hoc narrative of how it turned out). Valid episode is (S_t, A_t, O_{t+k}, τ); retrieval constraint: retrieve(S_t, A_t, O_{t+k}) permitted only if t_now ≥ t+k. Paired with a recency decay term e^{−λ(t_now − t_k)} on the relevance score "so that retrieval does not keep surfacing high-similarity episodes from a regime that has ended." 3. Exposure cap: w_i(t) = min(w_i^max, risk_budget / risk_per_unit_i). Note: "deliberately simple, and it is in the paper because risk triggers, latency budgets and audit logs are inconsistently reported across the corpus, so the argument is about the disclosure convention rather than the formula." Action module formalised as f(D_t) → (A_order, A_algo) with typed order fields and explicit failure modes for rejection, partial fill and timeout fed back into memory; feasible actions conditioned on O_{t−δ} to respect processing latency.</t>
+          <t>Four-step screening (keyword search, dedup, title/abstract screening against the finance/trading domain, full-text screening assigning primary vs background). Two criteria decide the primary subset and "the whole paper hangs off them": *Action Output* (system emits tradable actions - orders, position changes, portfolio allocations) and *Closed-Loop Evaluation* (actions evaluated in backtest, simulation or live trading rather than only through predictive metrics). Not a system. Three reimplementable rules the note singles out, "each is a rule rather than a model": 1. Reasoning module as a typed contract - f(O_t, M_episodic, P_portfolio) → (A_cand, α, V_check), where O_t is a timestamped state observation at decision time t, M_episodic retrievable episodic memory, P_portfolio read-only portfolio state (positions, risk limits), A_cand a set of candidate actions, α ∈ [0,1] a confidence score, V_check a validity check such as holds &lt; max_leverage. Purpose: "risk constraints are enforced during or immediately after reasoning rather than at the final execution layer, so a hallucinated action never reaches the order interface." 2. Outcome Embargo against the "Oracle Fallacy" (retrieving a past episode whose stored text already contains a post-hoc narrative of how it turned out). Valid episode is (S_t, A_t, O_{t+k}, τ); retrieval constraint: retrieve(S_t, A_t, O_{t+k}) permitted only if t_now ≥ t+k. Paired with a recency decay term e^{−λ(t_now − t_k)} on the relevance score "so that retrieval does not keep surfacing high-similarity episodes from a regime that has ended." 3. Exposure cap: w_i(t) = min(w_i^max, risk_budget / risk_per_unit_i). Note: "deliberately simple, and it is in the paper because risk triggers, latency budgets and audit logs are inconsistently reported across the corpus, so the argument is about the disclosure convention rather than the formula." Action module formalised as f(D_t) → (A_order, A_algo) with typed order fields and explicit failure modes for rejection, partial fill and timeout fed back into memory; feasible actions conditioned on O_{t−δ} to respect processing latency.</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>- Number/heterogeneity: not a system; audits others. Only 9/19 primary studies address coordination mechanisms at all; multi-agent chapter section-level primary count is 12, "with the larger citation list made up of benchmarks and background agent-based modelling work that does not enter the primary total." - Combination: three coordination patterns compared — role-based, hierarchical, market-ecology. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." - Anything varying influence by market state? No — not in the survey's own design and not reported as present in the audited corpus. The survey's contribution here is negative evidence plus a protocol demand: "cross-play evaluation swapping individual agents to test interoperability against team overfitting, explicit communication constraints, crowding and impact metrics, and role or communication ablations to attribute gains to coordination rather than to compute. On their reading, complex decomposition currently obscures the source of gains rather than demonstrating them." - Confidence per agent: yes as an interface — α ∈ [0,1] emitted per decision inside the reasoning contract alongside V_check. Note: "it tells me the confidence score belongs in the agent's typed output rather than being inferred by the orchestrator after the fact." No comparability mechanism.</t>
+          <t>- Number/heterogeneity: not a system; audits others. Only 9/19 primary studies address coordination mechanisms at all; multi-agent chapter section-level primary count is 12, "with the larger citation list made up of benchmarks and background agent-based modelling work that does not enter the primary total." - Combination: three coordination patterns compared - role-based, hierarchical, market-ecology. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." - Anything varying influence by market state? No - not in the survey's own design and not reported as present in the audited corpus. The survey's contribution here is negative evidence plus a protocol demand: "cross-play evaluation swapping individual agents to test interoperability against team overfitting, explicit communication constraints, crowding and impact metrics, and role or communication ablations to attribute gains to coordination rather than to compute. On their reading, complex decomposition currently obscures the source of gains rather than demonstrating them." - Confidence per agent: yes as an interface - α ∈ [0,1] emitted per decision inside the reasoning contract alongside V_check. Note: "it tells me the confidence score belongs in the agent's typed output rather than being inferred by the orchestrator after the fact." No comparability mechanism.</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -3943,12 +3943,12 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>No performance synthesis at all. Reproducibility tiers R0–R3; evaluation-type counts 11 backtest, 3 live, 2 simulation, 3 benchmark. Seven minimum reporting items MR-1 to MR-7 (data &amp; universe; time-consistent splitting; action semantics; execution &amp; costs; leakage audit; artifacts &amp; logs; multi-agent evaluation), graded mandatory/recommended/optional by study type. KEY RESULTS (numbers): Within the 19 primary studies — "2/19 (10.5%) report an extractable time-consistent split protocol, 1/19 (5.3%) specifies a transaction-cost model, 1/19 documents universe or survivorship handling, 11/19 (57.9%) report execution timing or semantics, and 4/19 expose artifacts beyond narrative description." On split protocol, "17/19 are coded Unknown, 2 are coded other, and zero report walk-forward or rolling evaluation." Reproducibility: "Fifteen of nineteen primary studies sit at R0, no runnable artifacts at all, one at R1, three at R2, and none reaches R3, so R2 or above is 15.8%." "That zero in the R3 row is, on this sample, the single most citable number in the paper." Coordination: "Nine of the nineteen primary studies address coordination mechanisms at all," section-level primary count for the multi-agent chapter is 12. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." Adaptation: "The section-level primary count for supervised fine-tuning is N=0 and for meta-learning it is N=0, learning paradigms overall rest on 3 primary studies, one in-context learning and two reinforcement learning, and self-evolution carries 4 primary studies with every row of its comparison table tagged as background." The only performance figure anywhere: "the 53.17% cumulative return on SSE50 reported by Automate Strategy Finding, is quoted with Split: NR, Execution: NR, Cost: NR, Universe: SSE50, Tier: BG attached precisely to demonstrate that the number is illustrative rather than protocol-comparable." LIMITATIONS (quoting the note): "The lens and the checklist are both author-curated and neither is externally validated.… The standard the field is measured against was set by the people doing the measuring, and while the paper says so plainly in three places, a different set of authors could have made MR-7 mandatory for multi-agent systems and produced a different set of failing grades." "A denominator of 19 makes every percentage brittle, and the section-level zeros are the most brittle of all. One paper moves the headline figures by 5.3 points, so 10.5% for split protocols and 5.3% for cost models should be read as two papers and one paper, which is how I will quote them." "The audit measures papers and the narrative occasionally slips into measuring systems… for a corpus that is 89% preprints, much of what is missing is appendix material that a journal round would have forced out." "Several named frameworks are the authors' own inventions presented in the same register as surveyed evidence" — Cascaded Controller, Alpha-to-Trade Contract, Hierarchy of Truth, Log-to-Narrative Verification, Oracle Fallacy; "HiveMind (Xia et al. 2026) also appears as background in the coordination chapter without the self-citation being flagged." "It deliberately contains no performance synthesis, so it cannot tell me what works… it means the paper is a citation for why comparisons are unsafe and never a citation for a comparison."</t>
+          <t>No performance synthesis at all. Reproducibility tiers R0 - R3; evaluation-type counts 11 backtest, 3 live, 2 simulation, 3 benchmark. Seven minimum reporting items MR-1 to MR-7 (data &amp; universe; time-consistent splitting; action semantics; execution &amp; costs; leakage audit; artifacts &amp; logs; multi-agent evaluation), graded mandatory/recommended/optional by study type. KEY RESULTS (numbers): Within the 19 primary studies - "2/19 (10.5%) report an extractable time-consistent split protocol, 1/19 (5.3%) specifies a transaction-cost model, 1/19 documents universe or survivorship handling, 11/19 (57.9%) report execution timing or semantics, and 4/19 expose artifacts beyond narrative description." On split protocol, "17/19 are coded Unknown, 2 are coded other, and zero report walk-forward or rolling evaluation." Reproducibility: "Fifteen of nineteen primary studies sit at R0, no runnable artifacts at all, one at R1, three at R2, and none reaches R3, so R2 or above is 15.8%." "That zero in the R3 row is, on this sample, the single most citable number in the paper." Coordination: "Nine of the nineteen primary studies address coordination mechanisms at all," section-level primary count for the multi-agent chapter is 12. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." Adaptation: "The section-level primary count for supervised fine-tuning is N=0 and for meta-learning it is N=0, learning paradigms overall rest on 3 primary studies, one in-context learning and two reinforcement learning, and self-evolution carries 4 primary studies with every row of its comparison table tagged as background." The only performance figure anywhere: "the 53.17% cumulative return on SSE50 reported by Automate Strategy Finding, is quoted with Split: NR, Execution: NR, Cost: NR, Universe: SSE50, Tier: BG attached precisely to demonstrate that the number is illustrative rather than protocol-comparable." LIMITATIONS (quoting the note): "The lens and the checklist are both author-curated and neither is externally validated.… The standard the field is measured against was set by the people doing the measuring, and while the paper says so plainly in three places, a different set of authors could have made MR-7 mandatory for multi-agent systems and produced a different set of failing grades." "A denominator of 19 makes every percentage brittle, and the section-level zeros are the most brittle of all. One paper moves the headline figures by 5.3 points, so 10.5% for split protocols and 5.3% for cost models should be read as two papers and one paper, which is how I will quote them." "The audit measures papers and the narrative occasionally slips into measuring systems… for a corpus that is 89% preprints, much of what is missing is appendix material that a journal round would have forced out." "Several named frameworks are the authors' own inventions presented in the same register as surveyed evidence" - Cascaded Controller, Alpha-to-Trade Contract, Hierarchy of Truth, Log-to-Narrative Verification, Oracle Fallacy; "HiveMind (Xia et al. 2026) also appears as background in the coordination chapter without the self-citation being flagged." "It deliberately contains no performance synthesis, so it cannot tell me what works… it means the paper is a citation for why comparisons are unsafe and never a citation for a comparison."</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>A survey rather than an experiment, so the headline results are corpus statistics. 92 candidate records screened, 15 final exclusions for falling outside the finance/trading/portfolio/risk domain, 77 in the included evidence-mapping ledger, and that 77 partitioned into 19 primary studies and 58 background. 18/19 of the primary studies were published between 2024 and 2026 and 17/19 are coded as non-peer-reviewed. On reproducibility, fifteen of nineteen sit at R0 with no runnable artifacts, one at R1, three at R2 and none at R3. On evaluation hygiene, 2/19 (10.5%) report an extractable time-consistent split protocol and 1/19 (5.3%) report a cost model, which is two papers and one paper respectively and should be quoted that way. Nine of the nineteen address coordination mechanisms at all; role-based systems are the only coordination pattern reaching R2, while hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three patterns. The authors describe their own synthesis as preliminary.</t>
         </is>
       </c>
       <c r="T27" s="3" t="inlineStr">
@@ -3958,19 +3958,19 @@
       </c>
       <c r="U27" s="3" t="inlineStr">
         <is>
-          <t>"The reporting checklist becomes the spine of my evaluation chapter, with the CSE specifics filled in under each item" — universe construction and survivorship under MR-1 matter because "delistings, long trading suspensions and illiquid counters make the definition of the tradable universe a design decision that changes results"; MR-2 commits to "walk-forward with a stated embargo, which also settles how the orchestrator's own tuning is separated from final evaluation." "The execution-friction work is now positioned by the field's own counts rather than by my assertion. One paper in nineteen specifying a transaction-cost model, and zero coordination patterns reporting execution semantics, is a much stronger warrant for state-dependent friction in a thin book than the individual-paper evidence I have been leaning on, such as MacroHFT's flat 0.02% over roughly twenty round trips." "The reasoning I/O contract gives the heterogeneous-confidence problem a shape without solving it." "The outcome embargo and the recency decay are two memory rules I can implement, test and report in a paragraph"; memory settings are an "evaluation knob" — "retrieval window, similarity function and truncation all change decisions under the same base model, so ablations have to report memory settings or they are not ablations." "Role and communication ablations are the published form of the diagnostic I already pre-registered… Reporting it under MR-7 alongside a cross-play check, swapping one agent for a weaker or differently-specified version, converts a defensive self-check into a positive methodological contribution, and it is the answer to the objection that a heterogeneous ensemble is just more compute." "Fifteen of nineteen at R0 has a direct planning consequence and a direct opportunity… with 0/19 reaching R3 on this sample, a CSE system released with pinned environment, data access instructions, seeds and an end-to-end evaluation pipeline would be at a tier no audited paper in this corpus occupies." Time-scale taxonomy (reactive / reflective / strategic) justifies the reasoning budget: "LLM-mediated deliberation operates at second-scale latency at best and cannot support genuine high-frequency decisions… A daily or intraday CSE rebalance sits comfortably in the reflective band." Search budget: "iterative refinement against validation metrics mines the validation set unless the final result is reported on a sealed test set never exposed to the refinement loop"; also a stated "reflection budget," "because retrying until a profitable trade appears is testing into success."</t>
+          <t>"The reporting checklist becomes the spine of my evaluation chapter, with the CSE specifics filled in under each item" - universe construction and survivorship under MR-1 matter because "delistings, long trading suspensions and illiquid counters make the definition of the tradable universe a design decision that changes results"; MR-2 commits to "walk-forward with a stated embargo, which also settles how the orchestrator's own tuning is separated from final evaluation." "The execution-friction work is now positioned by the field's own counts rather than by my assertion. One paper in nineteen specifying a transaction-cost model, and zero coordination patterns reporting execution semantics, is a much stronger warrant for state-dependent friction in a thin book than the individual-paper evidence I have been leaning on, such as MacroHFT's flat 0.02% over roughly twenty round trips." "The reasoning I/O contract gives the heterogeneous-confidence problem a shape without solving it." "The outcome embargo and the recency decay are two memory rules I can implement, test and report in a paragraph"; memory settings are an "evaluation knob" - "retrieval window, similarity function and truncation all change decisions under the same base model, so ablations have to report memory settings or they are not ablations." "Role and communication ablations are the published form of the diagnostic I already pre-registered… Reporting it under MR-7 alongside a cross-play check, swapping one agent for a weaker or differently-specified version, converts a defensive self-check into a positive methodological contribution, and it is the answer to the objection that a heterogeneous ensemble is just more compute." "Fifteen of nineteen at R0 has a direct planning consequence and a direct opportunity… with 0/19 reaching R3 on this sample, a CSE system released with pinned environment, data access instructions, seeds and an end-to-end evaluation pipeline would be at a tier no audited paper in this corpus occupies." Time-scale taxonomy (reactive / reflective / strategic) justifies the reasoning budget: "LLM-mediated deliberation operates at second-scale latency at best and cannot support genuine high-frequency decisions… A daily or intraday CSE rebalance sits comfortably in the reflective band." Search budget: "iterative refinement against validation metrics mines the validation set unless the final result is reported on a sealed test set never exposed to the refinement loop"; also a stated "reflection budget," "because retrying until a profitable trade appears is testing into success."</t>
         </is>
       </c>
       <c r="V27" s="3" t="inlineStr">
         <is>
-          <t>No performance synthesis, no architecture recommendation, no evidence any design works — by construction. On the main gap specifically, it supplies α as a typed per-decision output but "does not supply is comparability, because an LLM analyst's self-reported α, an econometric estimator's interval width and an RL policy's value spread are on three different scales and the paper never addresses cross-agent calibration." Cross-play evaluation "I have not seen operationalised anywhere and may need to define myself."</t>
+          <t>No performance synthesis, no architecture recommendation, no evidence any design works - by construction. On the main gap specifically, it supplies α as a typed per-decision output but "does not supply is comparability, because an LLM analyst's self-reported α, an econometric estimator's interval width and an RL policy's value spread are on three different scales and the paper never addresses cross-agent calibration." Cross-play evaluation "I have not seen operationalised anywhere and may need to define myself."</t>
         </is>
       </c>
       <c r="W27" s="3" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (MR-7, cross-play, role/communication ablations, the α contract) and friction-aware evaluation layer (MR-1 to MR-6, the 1/19 cost figure, the microstructure-as-feasibility-constraint framing). Secondarily A_F via the episodic-memory/embargo rules.
 EFFECT ON MAIN GAP: Leaves it open and materially strengthens it. It supplies counted, denominator-attached evidence that coordination is under-evidenced (9/19), that no audited coordination pattern reports execution semantics, and that adaptation claims rest on 3 primary studies. Nothing in it does state-conditioned agent weighting. It does narrow the *shape* of one sub-problem: confidence is now specified as a typed per-agent output, so the residual is calibration, not representation.
-CONFIDENCE SCORING: Partial. α ∈ [0,1] as a mandatory field of the reasoning module's output tuple, enforced alongside a validity check. Explicitly does not solve comparability — "That remains the open question the orchestrator lives or dies on, and this survey narrows it to a calibration problem rather than a representation problem."
+CONFIDENCE SCORING: Partial. α ∈ [0,1] as a mandatory field of the reasoning module's output tuple, enforced alongside a validity check. Explicitly does not solve comparability - "That remains the open question the orchestrator lives or dies on, and this survey narrows it to a calibration problem rather than a representation problem."
 FIXED-INFLUENCE FAILURE EVIDENCE: Not a per-component degradation case. The corpus-level analogue: "no coordination pattern in the table reports how its decisions become orders," and "complex decomposition currently obscures the source of gains rather than demonstrating them." Also the adaptive-overfitting/reflection-budget warning: "retrying until a profitable trade appears is testing into success."
 PROPOSED REVISION STATED IN THE NOTE: None to the four-agent pool or the conditioning set. The revisions proposed are protocol-level: build the evaluation chapter against MR-1 to MR-7, add the outcome embargo plus recency decay to retrieval, add a cross-play check beside the pre-registered weight-entropy diagnostic, target R3 reproducibility, fix a small conditioning set in advance with a stated search budget and a sealed test set.</t>
         </is>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>"LLM and RL trading agents collapse in adverse regimes, and the paper measures this rather than asserting it." Stated observation: state-of-the-art systems lose roughly 20% when markets fall rapidly or fluctuate frequently. Diagnosis: "there is no risk management mechanism inside the model or system" — frameworks optimise a return objective "and have nothing that adjusts exposure when conditions change." Contribution framed as importing hedging into a multi-agent setting, "an integration claim framed as one, which means the paper's defence rests entirely on its ablation table."</t>
+          <t>"LLM and RL trading agents collapse in adverse regimes, and the paper measures this rather than asserting it." Stated observation: state-of-the-art systems lose roughly 20% when markets fall rapidly or fluctuate frequently. Diagnosis: "there is no risk management mechanism inside the model or system" - frameworks optimise a return objective "and have nothing that adjusts exposure when conditions change." Contribution framed as importing hedging into a multi-agent setting, "an integration claim framed as one, which means the paper's defence rests entirely on its ablation table."</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Yahoo Finance and Alpaca News API, 1 Jan 2015 – 31 Dec 2023. Train 2015–2020; "1 January 2021 to 31 December 2023 for testing, three full years," described as "by a wide margin the longest evaluation window in my agent set and is the paper's strongest methodological choice." Temporal isolation check: rerun over the first three quarters of 2024, 68.44% total return with Sharpe 2.1.</t>
+          <t>Yahoo Finance and Alpaca News API, 1 Jan 2015–31 Dec 2023. Train 2015–2020; "1 January 2021 to 31 December 2023 for testing, three full years," described as "by a wide margin the longest evaluation window in my agent set and is the paper's strongest methodological choice." Temporal isolation check: rerun over the first three quarters of 2024, 68.44% total return with Sharpe 2.1.</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
@@ -4034,12 +4034,12 @@
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>"Nothing is trained. The paper presents the agent policy inside a reinforcement learning objective, but the policy itself is an LLM call, the action is produced by parsing the model's JSON output against a prompt template populated with market state and retrieved memory, and no gradient is taken anywhere in the system." Loop: memory retrieval → decision making → reflection update.  Four agents — three asset analysts (Bitcoin, Dow components, forex), one fund manager (Otto) allocating capital across them. Each analyst runs the same workflow: 23 tools, three memory stores, eight actions. Output: capital weights plus per-asset trades.</t>
+          <t>"Nothing is trained. The paper presents the agent policy inside a reinforcement learning objective, but the policy itself is an LLM call, the action is produced by parsing the model's JSON output against a prompt template populated with market state and retrieved memory, and no gradient is taken anywhere in the system." Loop: memory retrieval → decision making → reflection update. Four agents - three asset analysts (Bitcoin, Dow components, forex), one fund manager (Otto) allocating capital across them. Each analyst runs the same workflow: 23 tools, three memory stores, eight actions. Output: capital weights plus per-asset trades.</t>
         </is>
       </c>
       <c r="L28" s="11" t="inlineStr">
         <is>
-          <t>- Four agents. Heterogeneous only by *asset domain*, not by method — all four are the same LLM workflow (23 tools, three memory stores, eight actions). Evidence each sees: its own asset's OHLCV, 60 technical indicators, daily news headlines, plus retrieved memory. Manager Otto sees the three analysts' reported expected returns plus a data-estimated covariance matrix. - Combination: an explicit constrained optimisation, not a debate and not a prose manager. ω* = argmax_ω [I_etr − λ₁ I_pr − λ₂ I_cvar]. Note: "Every other multi-agent paper I have reviewed decomposes a decision and then recomposes it through prose, a hierarchy or a facilitator… HedgeAgents has one. Manager Otto solves an explicit constrained optimisation over a weight vector with return, variance and tail-risk terms, and publishes the objective. So the orchestration layer exists here as a numerical object rather than as an organisational metaphor, which makes this the paper my own weighting function has to be positioned against." - Coordination is by three meetings differing in trigger: Budget Allocation Conference every 30 days (analysts report P&amp;L with budget expectations, Otto consolidates and re-solves); Experience Sharing Conference at the end of each investment cycle; Extreme Market Conference triggered when daily amplitude exceeds 5% or cumulative three-day amplitude exceeds 10%. - Does anything vary influence by market state? Partly, and only at the trigger, not in the weights. Quoting the note: "HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies, 5% daily or 10% over three days, which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited." The one place competing suggestions are combined by a stated rule is the emergency blend, S = (1−λ₃) φ_B(S_B, S_C) + λ₃ φ_B(S_E) — and the note demolishes it: "Writing it this way makes it look like a weighted combination of vectors, but φ_B is a prompt and the addition is over text, so λ₃ is a number inserted into a prompt rather than a coefficient applied to anything, and its value is never stated either. This is the formula I would have expected to be the paper's orchestration mechanism and it is the weakest thing in it." - Confidence per agent: yes in the sense that each analyst emits an expected return ρ_i that enters the objective directly, but with no calibration, no interval, no realised-vs-predicted record. No comparability machinery; comparability is assumed because all three producers are the same kind of producer.</t>
+          <t>- Four agents. Heterogeneous only by *asset domain*, not by method - all four are the same LLM workflow (23 tools, three memory stores, eight actions). Evidence each sees: its own asset's OHLCV, 60 technical indicators, daily news headlines, plus retrieved memory. Manager Otto sees the three analysts' reported expected returns plus a data-estimated covariance matrix. - Combination: an explicit constrained optimisation, not a debate and not a prose manager. ω* = argmax_ω [I_etr − λ₁ I_pr − λ₂ I_cvar]. Note: "Every other multi-agent paper I have reviewed decomposes a decision and then recomposes it through prose, a hierarchy or a facilitator… HedgeAgents has one. Manager Otto solves an explicit constrained optimisation over a weight vector with return, variance and tail-risk terms, and publishes the objective. So the orchestration layer exists here as a numerical object rather than as an organisational metaphor, which makes this the paper my own weighting function has to be positioned against." - Coordination is by three meetings differing in trigger: Budget Allocation Conference every 30 days (analysts report P&amp;L with budget expectations, Otto consolidates and re-solves); Experience Sharing Conference at the end of each investment cycle; Extreme Market Conference triggered when daily amplitude exceeds 5% or cumulative three-day amplitude exceeds 10%. - Does anything vary influence by market state? Partly, and only at the trigger, not in the weights. Quoting the note: "HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies, 5% daily or 10% over three days, which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited." The one place competing suggestions are combined by a stated rule is the emergency blend, S = (1−λ₃) φ_B(S_B, S_C) + λ₃ φ_B(S_E) - and the note demolishes it: "Writing it this way makes it look like a weighted combination of vectors, but φ_B is a prompt and the addition is over text, so λ₃ is a number inserted into a prompt rather than a coefficient applied to anything, and its value is never stated either. This is the formula I would have expected to be the paper's orchestration mechanism and it is the weakest thing in it." - Confidence per agent: yes in the sense that each analyst emits an expected return ρ_i that enters the objective directly, but with no calibration, no interval, no realised-vs-predicted record. No comparability machinery; comparability is assumed because all three producers are the same kind of producer.</t>
         </is>
       </c>
       <c r="M28" s="11" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="N28" s="11" t="inlineStr">
         <is>
-          <t>No fundamentals channel. Memory retrieval is embedding similarity over three stores; "no retrieval-quality metric is reported." t-SNE cluster plot offered as evidence the memory hierarchy is semantically meaningful — "a reasonable reading of a projection but not a test of it."</t>
+          <t>No fundamentals channel. Memory retrieval is embedding similarity over three stores; "no retrieval-quality metric is reported." t-SNE cluster plot offered as evidence the memory hierarchy is semantically meaningful - "a reasonable reading of a projection but not a test of it."</t>
         </is>
       </c>
       <c r="O28" s="11" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="R28" s="11" t="inlineStr">
         <is>
-          <t>Nine metrics — total and annualised return, Sharpe, Calmar, Sortino, maximum drawdown, volatility, plus entropy and effective number of bets from PRUDEX-Compass. "The last two are not defined anywhere beyond the citation, which matters because diversity is one of the two things the title claims." Baselines: rule-based mean-variance, zero mean reversion, time-series momentum; RL — SAC, DeepTrader, AlphaMix+; LLM — FinGPT, FinMem, FinAgent; buy-and-hold per asset. All baselines trained and tested in the same environment with Optuna hyperparameter search.</t>
+          <t>Nine metrics - total and annualised return, Sharpe, Calmar, Sortino, maximum drawdown, volatility, plus entropy and effective number of bets from PRUDEX-Compass. "The last two are not defined anywhere beyond the citation, which matters because diversity is one of the two things the title claims." Baselines: rule-based mean-variance, zero mean reversion, time-series momentum; RL - SAC, DeepTrader, AlphaMix+; LLM - FinGPT, FinMem, FinAgent; buy-and-hold per asset. All baselines trained and tested in the same environment with Optuna hyperparameter search.</t>
         </is>
       </c>
       <c r="S28" s="11" t="inlineStr">
@@ -4096,7 +4096,7 @@
         <is>
           <t>SPEAKS TO: orchestrator primarily; A_V secondarily (CVaR term, amplitude trigger); friction-aware evaluation layer as a negative example (zero cost).
 EFFECT ON MAIN GAP: Narrows it, does not close it. This is the strongest partial encroachment of the seven on the "influence" side, because the orchestration layer is a real numerical weight vector rather than a prose manager, and because its emergency conference is genuinely state-triggered. But the weights are over assets, and the agent-to-asset mapping is one-to-one by construction, so the paper never confronts overlapping views, disagreement on a shared decision, or an uninformative channel. And the state-awareness lives in a fixed hand-set threshold, not in a function of measured state. The defensible residual: no continuous, measured-state-conditioned weighting of *methodologically heterogeneous* agents over a *shared* decision.
-CONFIDENCE SCORING: Offers the problem, not the solution — ρ_i is a self-reported LLM number entering an exact optimiser. The note's derived mechanism (calibrate each agent against its own realised hit rate on a held-out period, report a reliability curve per agent) is the student's own response, promoted here from open question to work item.
+CONFIDENCE SCORING: Offers the problem, not the solution - ρ_i is a self-reported LLM number entering an exact optimiser. The note's derived mechanism (calibrate each agent against its own realised hit rate on a held-out period, report a reliability curve per agent) is the student's own response, promoted here from open question to work item.
 FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of a subtle kind. "the experience-sharing plus extreme-market row reports drawdown of 12.02% and Sharpe of 2.24, both better on risk than the full system's Table 1 figures of 14.21% and 2.41 on drawdown, so on these numbers adding the budget conference buys return by taking on drawdown." Also: "the risk-adjusted headline is a backbone choice as much as an architecture result, and the best risk-adjusted configuration of their own system is not the one in Table 1." Neither is detected or responded to by the system.
 PROPOSED REVISION STATED IN THE NOTE: To the conditioning/trigger set, verbatim: "The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." Plus, as a build item: "each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function, reported as a reliability curve per agent." No change to the four-agent pool.</t>
         </is>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>None — regulatory compliance, not investing. "nothing here is evidence about returns, and I will not be building a compliance agent."  Regulatory interpretation and horizon scanning (AML/CTF, banking standards, securities, tax, monetary policy).</t>
+          <t>None - regulatory compliance, not investing. "nothing here is evidence about returns, and I will not be building a compliance agent." Regulatory interpretation and horizon scanning (AML/CTF, banking standards, securities, tax, monetary policy).</t>
         </is>
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>115 regulatory documents, 3,870 pages, 1,305,766 words from seven Australian and global bodies, processed into 11,086 chunks averaging ~119.6 tokens. Source split: FATF 19 docs / 547,449 words / 4,757 chunks; BASEL 10 / 253,694 / 2,059; AUSTRAC 59 / 229,347 / 1,901; APRA 19 / 143,299 / 1,212; IOSCO 2 / 96,764 / 876; ATO 5 / 20,249 / 156; RBA 1 / 14,964 / 125. "FATF alone is 42% of the word count, which the authors read as a risk that downstream behaviour is dominated by international guidance unless source weighting is applied, and they do not then apply any." Raw docs heavy-tailed: mean 20,402.59 words, median 9,801, sd 24,821.69, longest 107,043, shortest 580. Chunks: mean 117.79, median 117.41, sd 5.0 — "a fixed-width chunker that turns a 24,821-word standard deviation into a 5.0-word one is discarding document structure rather than respecting it."</t>
+          <t>115 regulatory documents, 3,870 pages, 1,305,766 words from seven Australian and global bodies, processed into 11,086 chunks averaging ~119.6 tokens. Source split: FATF 19 docs / 547,449 words / 4,757 chunks; BASEL 10 / 253,694 / 2,059; AUSTRAC 59 / 229,347 / 1,901; APRA 19 / 143,299 / 1,212; IOSCO 2 / 96,764 / 876; ATO 5 / 20,249 / 156; RBA 1 / 14,964 / 125. "FATF alone is 42% of the word count, which the authors read as a risk that downstream behaviour is dominated by international guidance unless source weighting is applied, and they do not then apply any." Raw docs heavy-tailed: mean 20,402.59 words, median 9,801, sd 24,821.69, longest 107,043, shortest 580. Chunks: mean 117.79, median 117.41, sd 5.0 - "a fixed-width chunker that turns a 24,821-word standard deviation into a 5.0-word one is discarding document structure rather than respecting it."</t>
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr">
@@ -4160,12 +4160,12 @@
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>CTDE (centralised training, decentralised execution) over a hierarchical, decentralised, partially observable MDP ⟨S, A, P, R, Ω, γ⟩. Global state: S_t = [h^reg_t ⊕ h^ext_t ⊕ m_t ⊕ θ_t], where h^reg_t and h^ext_t are latent context embeddings from Beta and Gamma, m_t current compliance metrics (e.g. a non-compliance count), θ_t the current hyperparameter configuration of the agents. Alpha observes the full global state; Beta and Gamma each receive o^i_t = O(S_t, i) containing only their own text segment and Alpha's instruction. Reward: R^i_total = λ · R_global + (1 − λ) · R^i_local, with R_global a Macro-F1 on compliance classification computed by Alpha, R^i_local the cosine similarity between agent i's output and ground-truth standards or high-confidence pseudo-labels; "The authors swept λ ∈ [0.1, 0.6] and report roughly 0.6 as optimal, with low values producing agent selfishness… and high values producing what they call lazy agents." Parameter adaptation is heuristic: raise learning rate η when TD error δ_t = R^i_total + γV(S_{t+1}) − V(S_t) is positive and lower it otherwise. Retrieval controller state is a JSON object {Current_Query, Retrieval_History, Compliance_Score} with action space {Refine Search, Retrieve Clause, Generate Answer, Halt}, iterated greedily for at most K = 5 steps — "That is a scripted controller with a scoring function, and calling it reinforcement learning is generous." Memory gate: u_t = 1(R^t_global &gt; μ_R + k·σ_R), k = 1.5, over a moving average and rolling sd of the last N global rewards; "The authors tested k ∈ [0.5, 3.0] and report that below 1.0 the policy is high-variance and above 2.0 necessary adaptations are blocked." Symbol collision flagged: k is both memory sensitivity (1.5) and retrieval depth (5).  Three agents, all on the same 1.5B base model, "specialised by three mechanisms rather than by architecture." Alpha = orchestrator and trainer, full global state, central critic, holds reward and memory. Beta = regulatory interpretation, regulatory/legal text, role-specific DAPT on regulatory corpus. Gamma = horizon scanning, news/social media/enforcement actions, role-specific DAPT on external corpus. Communication is mediated: Alpha broadcasts τ_t = ⟨Instruction, Data_Pointer, Context⟩; Beta and Gamma return y_t = ⟨Output, Confidence, Metadata⟩. "Direct Beta to Gamma communication is prohibited, enforcing Alpha as the sole mediator." Output is a compliance answer with citations.</t>
+          <t>CTDE (centralised training, decentralised execution) over a hierarchical, decentralised, partially observable MDP ⟨S, A, P, R, Ω, γ⟩. Global state: S_t = [h^reg_t ⊕ h^ext_t ⊕ m_t ⊕ θ_t], where h^reg_t and h^ext_t are latent context embeddings from Beta and Gamma, m_t current compliance metrics (e.g. a non-compliance count), θ_t the current hyperparameter configuration of the agents. Alpha observes the full global state; Beta and Gamma each receive o^i_t = O(S_t, i) containing only their own text segment and Alpha's instruction. Reward: R^i_total = λ · R_global + (1 − λ) · R^i_local, with R_global a Macro-F1 on compliance classification computed by Alpha, R^i_local the cosine similarity between agent i's output and ground-truth standards or high-confidence pseudo-labels; "The authors swept λ ∈ [0.1, 0.6] and report roughly 0.6 as optimal, with low values producing agent selfishness… and high values producing what they call lazy agents." Parameter adaptation is heuristic: raise learning rate η when TD error δ_t = R^i_total + γV(S_{t+1}) − V(S_t) is positive and lower it otherwise. Retrieval controller state is a JSON object {Current_Query, Retrieval_History, Compliance_Score} with action space {Refine Search, Retrieve Clause, Generate Answer, Halt}, iterated greedily for at most K = 5 steps - "That is a scripted controller with a scoring function, and calling it reinforcement learning is generous." Memory gate: u_t = 1(R^t_global &gt; μ_R + k·σ_R), k = 1.5, over a moving average and rolling sd of the last N global rewards; "The authors tested k ∈ [0.5, 3.0] and report that below 1.0 the policy is high-variance and above 2.0 necessary adaptations are blocked." Symbol collision flagged: k is both memory sensitivity (1.5) and retrieval depth (5). Three agents, all on the same 1.5B base model, "specialised by three mechanisms rather than by architecture." Alpha = orchestrator and trainer, full global state, central critic, holds reward and memory. Beta = regulatory interpretation, regulatory/legal text, role-specific DAPT on regulatory corpus. Gamma = horizon scanning, news/social media/enforcement actions, role-specific DAPT on external corpus. Communication is mediated: Alpha broadcasts τ_t = ⟨Instruction, Data_Pointer, Context⟩; Beta and Gamma return y_t = ⟨Output, Confidence, Metadata⟩. "Direct Beta to Gamma communication is prohibited, enforcing Alpha as the sole mediator." Output is a compliance answer with citations.</t>
         </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
         <is>
-          <t>- Three agents, homogeneous — all three built on the same DeepSeek-R1-Distill-Qwen-1.5B backbone, "specialised by three mechanisms rather than by architecture" (role-specific DAPT plus prompting plus observation scoping). Evidence: Alpha sees the full global state; Beta sees regulatory/legal text plus Alpha's instruction; Gamma sees news, social media and enforcement actions plus Alpha's instruction. Beta↔Gamma communication is prohibited. - Combination: Alpha is a centralised mediator and central critic. The stated fusion is "Alpha integrating the structured outputs using weighted logic with an adaptive thresholding mechanism based on statistical process control" — and "no weights, no thresholds and no fusion equations are given." - Does anything vary influence by state? The mechanism is declared but never specified, and what is specified conditions only on the agents' own outputs and the system's own configuration, never on the environment. S_t = [h^reg_t ⊕ h^ext_t ⊕ m_t ⊕ θ_t] — "Two of the four blocks are the agents' own latent outputs, one is a task-performance metric, and one is the system's own configuration. There is no environment-state block at all, nothing describing the regulatory landscape independently of what the agents just said about it. In my setting the analogue would be an orchestrator conditioned on the four agents' embeddings and its own recent accuracy, with no liquidity, volatility or persistence input, which is precisely the design I am arguing against, so the contrast is useful." What does adapt is per-agent learning rate via the TD-error heuristic, and memory writes via the u_t gate — adaptation of learning, not of influence. - Confidence per agent: declared in the protocol as the middle field of y_t = ⟨Output, Confidence, Metadata⟩, and then entirely unused — "confidence appears in no reward term, no fusion rule, no state block and no experiment."</t>
+          <t>- Three agents, homogeneous - all three built on the same DeepSeek-R1-Distill-Qwen-1.5B backbone, "specialised by three mechanisms rather than by architecture" (role-specific DAPT plus prompting plus observation scoping). Evidence: Alpha sees the full global state; Beta sees regulatory/legal text plus Alpha's instruction; Gamma sees news, social media and enforcement actions plus Alpha's instruction. Beta↔Gamma communication is prohibited. - Combination: Alpha is a centralised mediator and central critic. The stated fusion is "Alpha integrating the structured outputs using weighted logic with an adaptive thresholding mechanism based on statistical process control" - and "no weights, no thresholds and no fusion equations are given." - Does anything vary influence by state? The mechanism is declared but never specified, and what is specified conditions only on the agents' own outputs and the system's own configuration, never on the environment. S_t = [h^reg_t ⊕ h^ext_t ⊕ m_t ⊕ θ_t] - "Two of the four blocks are the agents' own latent outputs, one is a task-performance metric, and one is the system's own configuration. There is no environment-state block at all, nothing describing the regulatory landscape independently of what the agents just said about it. In my setting the analogue would be an orchestrator conditioned on the four agents' embeddings and its own recent accuracy, with no liquidity, volatility or persistence input, which is precisely the design I am arguing against, so the contrast is useful." What does adapt is per-agent learning rate via the TD-error heuristic, and memory writes via the u_t gate - adaptation of learning, not of influence. - Confidence per agent: declared in the protocol as the middle field of y_t = ⟨Output, Confidence, Metadata⟩, and then entirely unused - "confidence appears in no reward term, no fusion rule, no state block and no experiment."</t>
         </is>
       </c>
       <c r="M29" s="11" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="O29" s="11" t="inlineStr">
         <is>
-          <t>None in the market sense; "risk" here is regulatory risk. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): None — no market, no trading, no cost model. The only cost dimension is inference cost: ~$0.20 per million tokens against ~$5.00 for GPT-4o and ~$7.50 for self-hosted Llama-3-70B; median latency 210 ms vs ~450 ms and 180 ms; "Latency stays stable to about 75 concurrent users and P99 spikes beyond that."</t>
+          <t>None in the market sense; "risk" here is regulatory risk. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): None - no market, no trading, no cost model. The only cost dimension is inference cost: ~$0.20 per million tokens against ~$5.00 for GPT-4o and ~$7.50 for self-hosted Llama-3-70B; median latency 210 ms vs ~450 ms and 180 ms; "Latency stays stable to about 75 concurrent users and P99 spikes beyond that."</t>
         </is>
       </c>
       <c r="P29" s="11" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="S29" s="11" t="inlineStr">
         <is>
-          <t>Full system precision 0.94 / recall 0.92 / F1 0.93. Lexical only: recall 0.70, F1 0.76. Vector only: 0.89 / 0.81 / 0.85. No fine-tuning: 0.82 / 0.79 / 0.80. No iterative RL retrieval loop: 0.88 / 0.85 / 0.86. Retrieval depth: "F1 rises from 0.68 at k = 1 to 0.93 at k = 5, then falls monotonically to 0.74 at k = 20, driven by precision collapsing from 0.96 to roughly 0.45 while recall saturates near 1.0"; "adding fifteen more chunks costs 0.19 F1." Rubric: TRIAG 4.118 fluency, 4.612 relevance, 4.204 domain correctness, 4.087 consistency, 4.652 factuality, against deepseek-r1 7B's 4.062 / 3.941 / 4.021 / 4.291 / 4.427 — "Relevance and factuality move most, consistency is the one that goes backwards." Cost reduction ~96% vs GPT-4o, 97.3% vs Llama-3-70B. LIMITATIONS (quoting the note): "RQ2 asks whether coordinated agents outperform independent single-agent baselines and the paper never runs that experiment. There is no single-agent baseline anywhere, no two-agent configuration, no variant where Alpha does Beta's and Gamma's work itself… I should cite TRIAG as an architecture proposal with a retrieval evaluation attached rather than as evidence that MARL coordination helps." "Nothing in the evaluation is externally checkable, and the tuning results carry no variance… the selected λ ≈ 0.6 sits on the boundary of the swept interval [0.1, 0.6], which usually means the optimum lies outside the range tested." "The Confidence field is declared in the communication protocol and then never used. Beta and Gamma return ⟨Output, Confidence, Metadata⟩, and confidence appears in no reward term, no fusion rule, no state block and no experiment. Output fusion is described as Alpha integrating the structured outputs using weighted logic with an adaptive thresholding mechanism based on statistical process control, and no weights, no thresholds and no fusion equations are given. The single most load-bearing mechanism for my project is the one the paper states in prose and never specifies." "Homogeneity is acknowledged, defended weakly, and left untested… there is no measurement of divergence between Beta and Gamma after adaptation, and heterogeneous architectures are deferred to future work." "The local reward rests on cosine similarity to ground truth… an agent optimising cosine similarity to reference text is rewarded for paraphrasing the source, which is a proxy for retrieval fidelity and not for correctness, and it will score a fluent, well-grounded wrong answer highly whenever the wrong answer is lexically close to the right clause."</t>
+          <t>Full system precision 0.94 / recall 0.92 / F1 0.93. Lexical only: recall 0.70, F1 0.76. Vector only: 0.89 / 0.81 / 0.85. No fine-tuning: 0.82 / 0.79 / 0.80. No iterative RL retrieval loop: 0.88 / 0.85 / 0.86. Retrieval depth: "F1 rises from 0.68 at k = 1 to 0.93 at k = 5, then falls monotonically to 0.74 at k = 20, driven by precision collapsing from 0.96 to roughly 0.45 while recall saturates near 1.0"; "adding fifteen more chunks costs 0.19 F1." Rubric: TRIAG 4.118 fluency, 4.612 relevance, 4.204 domain correctness, 4.087 consistency, 4.652 factuality, against deepseek-r1 7B's 4.062 / 3.941 / 4.021 / 4.291 / 4.427 - "Relevance and factuality move most, consistency is the one that goes backwards." Cost reduction ~96% vs GPT-4o, 97.3% vs Llama-3-70B. LIMITATIONS (quoting the note): "RQ2 asks whether coordinated agents outperform independent single-agent baselines and the paper never runs that experiment. There is no single-agent baseline anywhere, no two-agent configuration, no variant where Alpha does Beta's and Gamma's work itself… I should cite TRIAG as an architecture proposal with a retrieval evaluation attached rather than as evidence that MARL coordination helps." "Nothing in the evaluation is externally checkable, and the tuning results carry no variance… the selected λ ≈ 0.6 sits on the boundary of the swept interval [0.1, 0.6], which usually means the optimum lies outside the range tested." "The Confidence field is declared in the communication protocol and then never used. Beta and Gamma return ⟨Output, Confidence, Metadata⟩, and confidence appears in no reward term, no fusion rule, no state block and no experiment. Output fusion is described as Alpha integrating the structured outputs using weighted logic with an adaptive thresholding mechanism based on statistical process control, and no weights, no thresholds and no fusion equations are given. The single most load-bearing mechanism for my project is the one the paper states in prose and never specifies." "Homogeneity is acknowledged, defended weakly, and left untested… there is no measurement of divergence between Beta and Gamma after adaptation, and heterogeneous architectures are deferred to future work." "The local reward rests on cosine similarity to ground truth… an agent optimising cosine similarity to reference text is rewarded for paraphrasing the source, which is a proxy for retrieval fidelity and not for correctness, and it will score a fluent, well-grounded wrong answer highly whenever the wrong answer is lexically close to the right clause."</t>
         </is>
       </c>
       <c r="T29" s="11" t="inlineStr">
@@ -4221,8 +4221,8 @@
       <c r="W29" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (λ credit-assignment split, memory gate, the negative example of the conditioning set) and A_F (hybrid dense+sparse retrieval, k = 5 budget, chunking critique).
-EFFECT ON MAIN GAP: Leaves it open and strengthens it. This is the closest published orchestrator in the set that writes down an explicit reward decomposition, an explicit state vector and an explicit agent output contract carrying a confidence field — and it still does not condition influence on environment state, and never computes with the confidence field. It is "the second instance after MacroHFT of state-aware coordination over components that are architecturally identical, which sharpens rather than threatens the heterogeneity claim." Scoped claim the note now defends: "weighting an econometric estimator against an LLM analyst against an RL allocator is a configuration I have not found in the reviewed literature, to be validated against further recent work, and the pre-registered weight-entropy diagnostic still applies, since if my weights collapse to one-hot I have built a router and have to say so."
-CONFIDENCE SCORING: No mechanism — the strongest negative result in the set on this question. The field exists in the protocol and in a figure and is never used. The note pairs it with the "Correct / Incorrect / Uncertain contract in Enhancing Anomaly Detection in Financial Markets with an LLM-Based Multi-Agent Framework, which is the only concrete cross-agent output vocabulary I have found."
+EFFECT ON MAIN GAP: Leaves it open and strengthens it. This is the closest published orchestrator in the set that writes down an explicit reward decomposition, an explicit state vector and an explicit agent output contract carrying a confidence field - and it still does not condition influence on environment state, and never computes with the confidence field. It is "the second instance after MacroHFT of state-aware coordination over components that are architecturally identical, which sharpens rather than threatens the heterogeneity claim." Scoped claim the note now defends: "weighting an econometric estimator against an LLM analyst against an RL allocator is a configuration I have not found in the reviewed literature, to be validated against further recent work, and the pre-registered weight-entropy diagnostic still applies, since if my weights collapse to one-hot I have built a router and have to say so."
+CONFIDENCE SCORING: No mechanism - the strongest negative result in the set on this question. The field exists in the protocol and in a figure and is never used. The note pairs it with the "Correct / Incorrect / Uncertain contract in Enhancing Anomaly Detection in Financial Markets with an LLM-Based Multi-Agent Framework, which is the only concrete cross-agent output vocabulary I have found."
 FIXED-INFLUENCE FAILURE EVIDENCE: Yes, by omission rather than ablation: "Gamma's brief includes sentiment analysis and no sentiment result is reported anywhere… this is another component whose influence is fixed by design and never measured, which is the same failure shape as the auxiliary strategies in FinAgent and the dropped sentiment agent in AlphaAgents, reached here by omission rather than by ablation."
 PROPOSED REVISION STATED IN THE NOTE: To the reward/credit structure and the update trigger, verbatim: "The TRIAG form gives each agent a local term scored against something it controls, a realised volatility forecast error for A_V, a spread or impact prediction error for A_L, a retrieval citation check for A_F, combined with the portfolio-level result through a single mixing weight… so this goes into the design as a mechanism with a pre-registered sweep rather than a fixed value, and the boundary-optimum problem in their sweep means my range has to extend past 0.6." And: "TRIAG updates on unusually good performance and what I need is an update on unusually *bad* performance, a regime break, so the gate becomes two-sided." No change to the four-agent pool; the conditioning set is defended unchanged, with the TRIAG state vector cited as the degenerate counterexample justifying the Adaptive − Liquidity and Adaptive − Volatility ablations.</t>
         </is>
@@ -4261,12 +4261,12 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Infrastructure / system demonstration — agent-callable financial toolchain plus a tool-use benchmark.</t>
+          <t>Infrastructure / system demonstration - agent-callable financial toolchain plus a tool-use benchmark.</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>"This is not a method paper and it does not propose an agent, it proposes the layer underneath one, a unified agent-callable toolchain standardising multi-frequency price access, structured news and event retrieval, and stateful brokerage simulation behind consistent JSON schemas and time-aligned interfaces." Framing gap is Table 1's Human Feed column — "whether market data and news are pre-curated and handed to the agent or retrieved by the agent itself. Of seven recent systems, six are pre-curated."</t>
+          <t>"This is not a method paper and it does not propose an agent, it proposes the layer underneath one, a unified agent-callable toolchain standardising multi-frequency price access, structured news and event retrieval, and stateful brokerage simulation behind consistent JSON schemas and time-aligned interfaces." Framing gap is Table 1's Human Feed column - "whether market data and news are pre-curated and handed to the agent or retrieved by the agent itself. Of seven recent systems, six are pre-curated."</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>NASDAQ API (economic and earnings calendars), MASSIVE (price), BENZINGA (news, earnings calendars, guidance). Refresh ~15 minutes behind for MASSIVE price and option data, daily for news and calendars — "sufficient for backtesting and not for low-latency trading." No period stated for the benchmark; "the benchmark's size is never stated, no episode count, no task-type distribution, no seeds."</t>
+          <t>NASDAQ API (economic and earnings calendars), MASSIVE (price), BENZINGA (news, earnings calendars, guidance). Refresh ~15 minutes behind for MASSIVE price and option data, daily for news and calendars - "sufficient for backtesting and not for low-latency trading." No period stated for the benchmark; "the benchmark's size is never stated, no episode count, no task-type distribution, no seeds."</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>Three modules — Unified Price Query (abstracts over frequency and instrument type), Event Stream Pipeline (normalises feeds along temporal scope, market scope and information type, indexed by temporal/ticker/event-type tags), Paper Money Broker (order states, positions, balances, transaction logs, margin-aware account dynamics under configurable execution rules). Four design decisions: unified JSON schemas with explicit timestamps, composable APIs callable independently inside a reasoning loop, a "time-consistent state abstraction" aligning price, event and portfolio state to precise timestamps, and environment decoupling (one API surface serves historical replay, simulated streaming and live-like settings without agent logic changing).  Environment, not agent. Figure 3 shows "an analysis agent handing off to a trading agent in a fixed pipeline with no adaptive influence between them."</t>
+          <t>Three modules - Unified Price Query (abstracts over frequency and instrument type), Event Stream Pipeline (normalises feeds along temporal scope, market scope and information type, indexed by temporal/ticker/event-type tags), Paper Money Broker (order states, positions, balances, transaction logs, margin-aware account dynamics under configurable execution rules). Four design decisions: unified JSON schemas with explicit timestamps, composable APIs callable independently inside a reasoning loop, a "time-consistent state abstraction" aligning price, event and portfolio state to precise timestamps, and environment decoupling (one API surface serves historical replay, simulated streaming and live-like settings without agent logic changing). Environment, not agent. Figure 3 shows "an analysis agent handing off to a trading agent in a fixed pipeline with no adaptive influence between them."</t>
         </is>
       </c>
       <c r="L30" s="11" t="inlineStr">
@@ -4321,12 +4321,12 @@
       </c>
       <c r="R30" s="11" t="inlineStr">
         <is>
-          <t>Two task types — single-step Tool Calling and multi-step Task Planning. Three metrics: Tool Match with partial credit (s^TM_k = 1.0 exact tool-name match, 0.5 correct family UPQ/ESP/PMB wrong tool, 0.0 otherwise; TM = (1/K) Σ s^TM_k); Parameter Accuracy (recursive comparison including nested dicts and lists, Jaccard partial credit for list overlap, relative tolerance 1e-4 on numerics, dependency placeholders ignored); Time Alignment (exact for zero-second fields, ±5 minutes intraday, ±1 calendar day daily, ±2 days loose windows, 30 or 60 minutes for horizon-like constraints). Overall = (100/3)(TM + PA + TA). Eight models evaluated. "The benchmark scores tool correctness and execution consistency, explicitly not financial return."</t>
+          <t>Two task types - single-step Tool Calling and multi-step Task Planning. Three metrics: Tool Match with partial credit (s^TM_k = 1.0 exact tool-name match, 0.5 correct family UPQ/ESP/PMB wrong tool, 0.0 otherwise; TM = (1/K) Σ s^TM_k); Parameter Accuracy (recursive comparison including nested dicts and lists, Jaccard partial credit for list overlap, relative tolerance 1e-4 on numerics, dependency placeholders ignored); Time Alignment (exact for zero-second fields, ±5 minutes intraday, ±1 calendar day daily, ±2 days loose windows, 30 or 60 minutes for horizon-like constraints). Overall = (100/3)(TM + PA + TA). Eight models evaluated. "The benchmark scores tool correctness and execution consistency, explicitly not financial return."</t>
         </is>
       </c>
       <c r="S30" s="11" t="inlineStr">
         <is>
-          <t>Tool Calling Overall — Gemini 2.5 Flash 91.00, Gemini 2.5 Pro 91.00, GPT-4.1 87.33, GPT-4.1 Mini 84.33, DeepSeek Chat 88.00, Qwen2.5 7B Instruct 78.33, Llama 3.1 8B Instruct 62.33, Qwen3 4B Instruct 86.33. Task Planning Overall — 92.33, 93.67, 93.67, 92.00, 95.00, 87.67, 84.67, 86.33. "TM sits between 0.90 and 0.97 for seven of the eight models, including Qwen3 4B at 0.93, while PA and TA are below TM in every single row without exception." "Multi-step planning scores higher than single-step tool calling for seven of the eight models, which is backwards" — Llama 3.1 8B goes 62.33 → 84.67, Qwen2.5 7B 78.33 → 87.67. LIMITATIONS (quoting the note): "The Overall column does not support the reading it invites, for two separate reasons.… averaging TM, PA and TA weights three unlike failures equally: picking the wrong tool usually produces an error the agent can see, while a wrong argument or a wrong timestamp produces a plausible answer nothing downstream flags… Carry the three components, read the table as three tiers, and leave Overall alone." "The instructions and the gold traces are both LLM-generated." "PMB simulates the brokerage, not the market." "The reproducibility argument is undercut by the data licensing… deterministic replay guarantees reproducibility within a lab and not across labs. Given that a standardised, reproducible environment is the paper's central claim, this is the limitation that most constrains what it actually delivers." "Module naming is inconsistent between the prose and the implementation" (ESP in text, NPP in figures). On TA specifically: "TA's bands are generous, plus or minus one calendar day for daily fields and plus or minus two days for loose windows, so a TA of 0.86 means a real fraction of calls miss by more than a full day. In an interactive assistant that is a rounding error, in a backtest it is a lookahead hazard."</t>
+          <t>Tool Calling Overall - Gemini 2.5 Flash 91.00, Gemini 2.5 Pro 91.00, GPT-4.1 87.33, GPT-4.1 Mini 84.33, DeepSeek Chat 88.00, Qwen2.5 7B Instruct 78.33, Llama 3.1 8B Instruct 62.33, Qwen3 4B Instruct 86.33. Task Planning Overall - 92.33, 93.67, 93.67, 92.00, 95.00, 87.67, 84.67, 86.33. "TM sits between 0.90 and 0.97 for seven of the eight models, including Qwen3 4B at 0.93, while PA and TA are below TM in every single row without exception." "Multi-step planning scores higher than single-step tool calling for seven of the eight models, which is backwards" - Llama 3.1 8B goes 62.33 → 84.67, Qwen2.5 7B 78.33 → 87.67. LIMITATIONS (quoting the note): "The Overall column does not support the reading it invites, for two separate reasons.… averaging TM, PA and TA weights three unlike failures equally: picking the wrong tool usually produces an error the agent can see, while a wrong argument or a wrong timestamp produces a plausible answer nothing downstream flags… Carry the three components, read the table as three tiers, and leave Overall alone." "The instructions and the gold traces are both LLM-generated." "PMB simulates the brokerage, not the market." "The reproducibility argument is undercut by the data licensing… deterministic replay guarantees reproducibility within a lab and not across labs. Given that a standardised, reproducible environment is the paper's central claim, this is the limitation that most constrains what it actually delivers." "Module naming is inconsistent between the prose and the implementation" (ESP in text, NPP in figures). On TA specifically: "TA's bands are generous, plus or minus one calendar day for daily fields and plus or minus two days for loose windows, so a TA of 0.86 means a real fraction of calls miss by more than a full day. In an interactive assistant that is a rounding error, in a backtest it is a lookahead hazard."</t>
         </is>
       </c>
       <c r="T30" s="11" t="inlineStr">
@@ -4349,7 +4349,7 @@
           <t>SPEAKS TO: friction-aware evaluation layer (PMB shape, as_of_ts cursor, TM/PA/TA harness) and, indirectly, all four agents' data access.
 EFFECT ON MAIN GAP: Leaves it entirely open, and is useful precisely because it does. "the paper closest to my infrastructure has no opinion on my research question." Its net effect is to demote plumbing out of the contribution and leave the weighting function as the surviving claim.
 CONFIDENCE SCORING: No mechanism. Nothing in the paper produces or compares per-agent confidence.
-FIXED-INFLUENCE FAILURE EVIDENCE: No degradation case, but it is a documented instance of the fixed-influence pattern itself — "an analysis agent handing off to a trading agent in a fixed pipeline with no adaptive influence between them."
+FIXED-INFLUENCE FAILURE EVIDENCE: No degradation case, but it is a documented instance of the fixed-influence pattern itself - "an analysis agent handing off to a trading agent in a fixed pipeline with no adaptive influence between them."
 PROPOSED REVISION STATED IN THE NOTE: None to the agent pool or conditioning set. Revisions are infrastructural: adopt the as_of_ts point-in-time cursor at the data layer for all four channels, build a CSE analogue of TM/PA/TA for the tool layer, take PMB's order-lifecycle shape while sourcing the friction model elsewhere, adopt storage tiering and environment decoupling.</t>
         </is>
       </c>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Brittleness of deep learning in quant finance, decomposed into three challenges — "traditional alpha mining methods are rigid and do not adapt to dynamic markets, machine learning approaches struggle to integrate diverse data, and strategies do not adapt to market variability." Three-stage pipeline: LLMs generate executable alpha factor candidates from the alpha-mining literature; a multi-agent evaluation filters them on market status and predictive quality while maintaining category balance; a weight optimisation stage combines the survivors. Most important framing in the note: "I came to this from the BlackRock survey, which describes it as employing an adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions. That is not what the paper does, and the difference is the most useful thing I got out of reading it. The adaptivity here is at selection, not at weighting."</t>
+          <t>Brittleness of deep learning in quant finance, decomposed into three challenges - "traditional alpha mining methods are rigid and do not adapt to dynamic markets, machine learning approaches struggle to integrate diverse data, and strategies do not adapt to market variability." Three-stage pipeline: LLMs generate executable alpha factor candidates from the alpha-mining literature; a multi-agent evaluation filters them on market status and predictive quality while maintaining category balance; a weight optimisation stage combines the survivors. Most important framing in the note: "I came to this from the BlackRock survey, which describes it as employing an adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions. That is not what the paper does, and the difference is the most useful thing I got out of reading it. The adaptivity here is at selection, not at weighting."</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Six primary features (open, high, low, close, volume, VWAP) plus quarterly and annual reports of index constituents, January 2019 to June 2024. Main backtest SSE50: train Jan 2021 – Jun 2022, validation Jul – Dec 2022, test Jan 2023 – Jan 2024. Cross-market Table 5 uses rolling annual partitions with six-month test windows, H1 2021, H1 2022, H1 2023 for CSI300 and SP500. Ablation uses SSE50 data 2010–2022.</t>
+          <t>Six primary features (open, high, low, close, volume, VWAP) plus quarterly and annual reports of index constituents, January 2019 to June 2024. Main backtest SSE50: train Jan 2021 - Jun 2022, validation Jul - Dec 2022, test Jan 2023 - Jan 2024. Cross-market Table 5 uses rolling annual partitions with six-month test windows, H1 2021, H1 2022, H1 2023 for CSI300 and SP500. Ablation uses SSE50 data 2010–2022.</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -4412,12 +4412,12 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 — two agents each score every candidate alpha α_ij in category j against market condition M^(t): θ_ij = E[IC(α_ij | M^(t))] from the Confidence Score Agent, and ρ_ij = f_risk(α_ij, M^(t)) from the Risk Preference Agent. Mixed linearly with the best-scoring alpha in each category kept, subject to a confidence threshold: α*_j = argmax_{α_ij} [w_c · θ_ij + w_r · ρ_ij]. Phase 3 — a three-layer MLP, input width equal to the number of selected alphas, ten ReLU hidden nodes, one output, mapping historical daily alpha values to future yields, with a held-out validation set; its learned parameters become the combination weights. Composite signal: α^(t)_i = Σ_j w_j · α^(t)_ij. "Read the subscripts. The alpha values carry t, the weights do not, here or in Algorithm 2 line 30 or in the paper's equation 8. The abstract's 'dynamic weight optimization that adapts to market conditions' and the survey's 'real time' gating both describe w_j as though it were w_j^(t), and nothing in the method produces that. The weights change when the model is retrained on a new window, which is retraining, not gating."  Three-stage pipeline → composite alpha → portfolio. A.8: "daily reconstruction, rank all securities by composite alpha, take the top k = 13, limit churn to n = 5 names per day, equal weight across holdings. That is roughly 38% daily turnover, which the paper states and then never prices."</t>
+          <t>Phase 2 - two agents each score every candidate alpha α_ij in category j against market condition M^(t): θ_ij = E[IC(α_ij | M^(t))] from the Confidence Score Agent, and ρ_ij = f_risk(α_ij, M^(t)) from the Risk Preference Agent. Mixed linearly with the best-scoring alpha in each category kept, subject to a confidence threshold: α*_j = argmax_{α_ij} [w_c · θ_ij + w_r · ρ_ij]. Phase 3 - a three-layer MLP, input width equal to the number of selected alphas, ten ReLU hidden nodes, one output, mapping historical daily alpha values to future yields, with a held-out validation set; its learned parameters become the combination weights. Composite signal: α^(t)_i = Σ_j w_j · α^(t)_ij. "Read the subscripts. The alpha values carry t, the weights do not, here or in Algorithm 2 line 30 or in the paper's equation 8. The abstract's 'dynamic weight optimization that adapts to market conditions' and the survey's 'real time' gating both describe w_j as though it were w_j^(t), and nothing in the method produces that. The weights change when the model is retrained on a new window, which is retraining, not gating." Three-stage pipeline → composite alpha → portfolio. A.8: "daily reconstruction, rank all securities by composite alpha, take the top k = 13, limit churn to n = 5 names per day, equal weight across holdings. That is roughly 38% daily turnover, which the paper states and then never prices."</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>- Two agents in Phase 2 plus an MLP in Phase 3. Homogeneous in evidence type: "the paper is not proposing a new way to combine heterogeneous *analysts*. Every object in the system is a formulaic alpha… The two agents both evaluate those same expressions. This is one evidence type scored two ways, not four evidence types that have to be reconciled." Confidence Score Agent sees candidate alphas plus the market condition M^(t) and outputs an expected conditional IC; Risk Preference Agent sees the same and outputs a risk-character score. - Combination: two stages. Agent scores are mixed by a fixed linear rule α*_j = argmax [w_c θ_ij + w_r ρ_ij] with w_c = 0.6, w_r = 0.4; the surviving factors are combined by a static MLP whose weights carry no time index. - Does anything vary influence by market state? Selection yes, weighting no — and this is the single most important correction in the note. Which factors enter is conditioned on M^(t), because M^(t) is passed to both evaluating agents. How much each selected factor counts is "a weight vector produced once by a small MLP trained on a fixed historical window, and it carries no time index anywhere in the paper's equations or in its algorithm listing." Quoting the note's headline: "The adaptivity here is at selection, not at weighting." And: "So this is not a competitor to my orchestrator. It is the strongest published instantiation I have of Baseline 2, the static learned weight, which the supervisor identified as the baseline that actually matters, and it is the reference design I should implement that arm against." - Confidence per agent: yes, and it is the most directly reusable confidence construct in the set — θ_ij = E[IC(α_ij | M^(t))], an expected conditional information coefficient, paired with a separate risk score, mixed linearly. Comparability is trivial here because both scores are over the same object type. The note's port: "each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target."</t>
+          <t>- Two agents in Phase 2 plus an MLP in Phase 3. Homogeneous in evidence type: "the paper is not proposing a new way to combine heterogeneous *analysts*. Every object in the system is a formulaic alpha… The two agents both evaluate those same expressions. This is one evidence type scored two ways, not four evidence types that have to be reconciled." Confidence Score Agent sees candidate alphas plus the market condition M^(t) and outputs an expected conditional IC; Risk Preference Agent sees the same and outputs a risk-character score. - Combination: two stages. Agent scores are mixed by a fixed linear rule α*_j = argmax [w_c θ_ij + w_r ρ_ij] with w_c = 0.6, w_r = 0.4; the surviving factors are combined by a static MLP whose weights carry no time index. - Does anything vary influence by market state? Selection yes, weighting no - and this is the single most important correction in the note. Which factors enter is conditioned on M^(t), because M^(t) is passed to both evaluating agents. How much each selected factor counts is "a weight vector produced once by a small MLP trained on a fixed historical window, and it carries no time index anywhere in the paper's equations or in its algorithm listing." Quoting the note's headline: "The adaptivity here is at selection, not at weighting." And: "So this is not a competitor to my orchestrator. It is the strongest published instantiation I have of Baseline 2, the static learned weight, which the supervisor identified as the baseline that actually matters, and it is the reference design I should implement that arm against." - Confidence per agent: yes, and it is the most directly reusable confidence construct in the set - θ_ij = E[IC(α_ij | M^(t))], an expected conditional information coefficient, paired with a separate risk score, mixed linearly. Comparability is trivial here because both scores are over the same object type. The note's port: "each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target."</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -4473,9 +4473,9 @@
       <c r="W31" s="3" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (as Baseline 2, the static learned weight), A_T (formulaic alphas), A_L (liquidity factor definitions), friction-aware evaluation layer (38% turnover unpriced).
-EFFECT ON MAIN GAP: Leaves it open — and the note's rereading of this paper is what keeps it open. The BlackRock survey had nominated it as the nearest prior art with a "dynamic weighting mechanism"/"adaptive gating mechanism that tunes the influence of each signal in real time." On the paper's own equations that description is unsupported. Net effect: the one candidate the field itself pointed at as occupying the gap turns out to be a static-learned-weight baseline. It does, however, narrow the gap in one direction — it demonstrates that state-conditional *selection* carries real signal, mostly in bear regimes (bear IC 0.042 full vs 0.021 without the confidence agent), which obliges the student to add a state-conditional-inclusion / static-weight configuration to their own ablation to prove the weighting function is what is doing the work.
-CONFIDENCE SCORING: Yes — the cleanest formal template in the set, though not a cross-*heterogeneity* solution. Expected conditional IC as confidence plus a separate risk-character score, linearly mixed. Caution attached: the mixing ratio is exactly the unstable parameter in their sensitivity table, so fix it on validation and report the sweep.
-FIXED-INFLUENCE FAILURE EVIDENCE: Indirect. The weighting stage is never ablated, so no failure is observable by construction; the note treats that absence as the missing arm rather than as evidence. The nearest documented degradation is the drawdown result — the strategy is deeper in drawdown than the benchmark in four of six cross-market windows while the abstract claims general downside protection, with nothing in the system detecting it.
+EFFECT ON MAIN GAP: Leaves it open - and the note's rereading of this paper is what keeps it open. The BlackRock survey had nominated it as the nearest prior art with a "dynamic weighting mechanism"/"adaptive gating mechanism that tunes the influence of each signal in real time." On the paper's own equations that description is unsupported. Net effect: the one candidate the field itself pointed at as occupying the gap turns out to be a static-learned-weight baseline. It does, however, narrow the gap in one direction - it demonstrates that state-conditional *selection* carries real signal, mostly in bear regimes (bear IC 0.042 full vs 0.021 without the confidence agent), which obliges the student to add a state-conditional-inclusion / static-weight configuration to their own ablation to prove the weighting function is what is doing the work.
+CONFIDENCE SCORING: Yes - the cleanest formal template in the set, though not a cross-*heterogeneity* solution. Expected conditional IC as confidence plus a separate risk-character score, linearly mixed. Caution attached: the mixing ratio is exactly the unstable parameter in their sensitivity table, so fix it on validation and report the sweep.
+FIXED-INFLUENCE FAILURE EVIDENCE: Indirect. The weighting stage is never ablated, so no failure is observable by construction; the note treats that absence as the missing arm rather than as evidence. The nearest documented degradation is the drawdown result - the strategy is deeper in drawdown than the benchmark in four of six cross-market windows while the abstract claims general downside protection, with nothing in the system detecting it.
 PROPOSED REVISION STATED IN THE NOTE: To the experimental design rather than the pool, but it directly touches the conditioning set. Verbatim: "the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically." And on P_t, verbatim: "That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." Also: "Keep the orchestrator low-capacity… a gated linear form or a shallow regression on the four state variables, rather than a network."</t>
         </is>
       </c>
@@ -4553,7 +4553,7 @@
       </c>
       <c r="N32" s="11" t="inlineStr">
         <is>
-          <t>RAG integration row — FinRobot partial (initial data ingestion), MarketSenseAI yes (HyDE plus expert documents), FinVerse yes (chunked document retrieval), FinGPT Agent yes (with fine-tuned LLM).</t>
+          <t>RAG integration row - FinRobot partial (initial data ingestion), MarketSenseAI yes (HyDE plus expert documents), FinVerse yes (chunked document retrieval), FinGPT Agent yes (with fine-tuned LLM).</t>
         </is>
       </c>
       <c r="O32" s="11" t="inlineStr">
@@ -4573,12 +4573,12 @@
       </c>
       <c r="R32" s="11" t="inlineStr">
         <is>
-          <t>Four evaluation families — financial metrics (Sharpe, Sortino, Calmar, cumulative and annualised return, volatility, max drawdown, IC and rank IC); accuracy and reasoning (classification accuracy, F1, exact match, SQL validity); behavioural fidelity (trading flow, position tracking, strategy adherence, responsiveness to events, agent longevity); user-centric (usefulness, robustness, human alignment, elicitation accuracy, task completion, report readability). "The distribution across Table 2 is the finding, not the taxonomy: financial metrics carry fourteen papers, accuracy and reasoning twelve, behavioural fidelity three." Survey states plainly "that there is no unified protocol for evaluating LLM agents in finance and that current assessments rely heavily on narrow backtests or synthetic prompts, often ignoring intermediate behaviours."</t>
+          <t>Four evaluation families - financial metrics (Sharpe, Sortino, Calmar, cumulative and annualised return, volatility, max drawdown, IC and rank IC); accuracy and reasoning (classification accuracy, F1, exact match, SQL validity); behavioural fidelity (trading flow, position tracking, strategy adherence, responsiveness to events, agent longevity); user-centric (usefulness, robustness, human alignment, elicitation accuracy, task completion, report readability). "The distribution across Table 2 is the finding, not the taxonomy: financial metrics carry fourteen papers, accuracy and reasoning twelve, behavioural fidelity three." Survey states plainly "that there is no unified protocol for evaluating LLM agents in finance and that current assessments rely heavily on narrow backtests or synthetic prompts, often ignoring intermediate behaviours."</t>
         </is>
       </c>
       <c r="S32" s="11" t="inlineStr">
         <is>
-          <t>The student's own tally over Figure 2, explicitly flagged as a tally and not a reported result — Stage 2 Memory: 12 of 31; Stage 7 Reflection: 9 of 31; Stage 8 Multi-agent collaboration: 13 of 31; Stage 10 Evaluation: 5 of 31. "Fewer than half the systems in a survey of multi-agent financial AI carry a multi-agent collaboration stage at all, and of the thirteen that do, the survey's own worked examples of what collaboration means are ask-respond and debate. Both are protocols for producing one text from several texts. Neither is a weighting." The gap written in the field's vocabulary: Stage 9 as surveyed, D_t = g(A_{1,t}, …, A_{n,t}), against D_t = Σ_i w_{i,t}(L_t, V_t, P_t, C_{i,t}) A_{i,t}, "where g is an unspecified aggregator, usually an LLM manager prompted to reconcile the agents… The survey never distinguishes the two, which is the gap stated in the field's own vocabulary rather than mine." LIMITATIONS (quoting the note): "There is no review protocol, so coverage cannot be checked. No search strategy, no databases, no query strings, no inclusion or exclusion criteria, no date range, no count of papers screened against papers retained… the branch structure cannot be distinguished from the authors' reading list, and an empty cell in the taxonomy cannot be read as a gap in the field." "Nothing in it is evidence.… a reader cannot tell whether 'no' in the adaptive architecture row means the authors checked and found nothing or that the primary paper did not use the word." "The stage annotations are the most valuable thing in the paper and the least documented.… the honest version of my tally is that thirteen of thirty-one systems were judged by these authors to collaborate, on a criterion they did not state." "Primary papers' priority claims are repeated without adjudication, and one self-citation is unflagged" — three of the five authors are authors of AlphaAgents, which appears in the portfolio branch and Table 2 without disclosure. "The open-challenges section is a list of headings, not a prioritisation."</t>
+          <t>The student's own tally over Figure 2, explicitly flagged as a tally and not a reported result - Stage 2 Memory: 12 of 31; Stage 7 Reflection: 9 of 31; Stage 8 Multi-agent collaboration: 13 of 31; Stage 10 Evaluation: 5 of 31. "Fewer than half the systems in a survey of multi-agent financial AI carry a multi-agent collaboration stage at all, and of the thirteen that do, the survey's own worked examples of what collaboration means are ask-respond and debate. Both are protocols for producing one text from several texts. Neither is a weighting." The gap written in the field's vocabulary: Stage 9 as surveyed, D_t = g(A_{1,t}, …, A_{n,t}), against D_t = Σ_i w_{i,t}(L_t, V_t, P_t, C_{i,t}) A_{i,t}, "where g is an unspecified aggregator, usually an LLM manager prompted to reconcile the agents… The survey never distinguishes the two, which is the gap stated in the field's own vocabulary rather than mine." LIMITATIONS (quoting the note): "There is no review protocol, so coverage cannot be checked. No search strategy, no databases, no query strings, no inclusion or exclusion criteria, no date range, no count of papers screened against papers retained… the branch structure cannot be distinguished from the authors' reading list, and an empty cell in the taxonomy cannot be read as a gap in the field." "Nothing in it is evidence.… a reader cannot tell whether 'no' in the adaptive architecture row means the authors checked and found nothing or that the primary paper did not use the word." "The stage annotations are the most valuable thing in the paper and the least documented.… the honest version of my tally is that thirteen of thirty-one systems were judged by these authors to collaborate, on a criterion they did not state." "Primary papers' priority claims are repeated without adjudication, and one self-citation is unflagged" - three of the five authors are authors of AlphaAgents, which appears in the portfolio branch and Table 2 without disclosure. "The open-challenges section is a list of headings, not a prioritisation."</t>
         </is>
       </c>
       <c r="T32" s="11" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="U32" s="11" t="inlineStr">
         <is>
-          <t>"This is the citation for the positioning claim, scoped to what it can carry. The permitted form is that a survey of thirty-one systems organises them by use case and by workflow stage without a stage for weighting agent influence, and that among the four systems it compares directly on adaptive architecture, none adapts the influence of one component on the decision. That is a claim about this survey's coverage, not about the literature, and I should pair it with the absence of a stated review protocol in the same sentence so the scoping is mine rather than something a reader catches me on." "Behavioural fidelity gives my ablations a vocabulary and a second axis of results. Responsiveness to events, strategy adherence and position tracking are named metric families… Dropping volatility from the conditioning set should show up as reduced responsiveness to volatility events, not only as a lower Sharpe, and reporting the behavioural change beside the return change is how I avoid the situation where the dynamic scheme beats the static learned weight by a margin too small to defend. This also gives the ablation table a row to fill when a return difference fails to clear significance on CSE-length data." "Their evaluation verdict licenses building my own protocol, and the data blocker remains the real constraint." "Unfaithful chain-of-thought settles the shape of the explainability story. If natural-language justifications are frequently not faithful to the reasoning that produced them, then an explanation layer that reports what the agents said about themselves is worth very little. What I already have is attribution over computed quantities, the orchestrator's weight vector, SHAP over risk features, interpretable volatility-model parameters, and citation tracing back to the retrieved passage, and all four are auditable in a way an LLM's narration is not." "Two cautions to build a baseline against" — a study testing whether prompt-driven LLM agents merely reproduce momentum or value, "which is a direct question to put to my technical agent: does it add anything over a prompted momentum rule on the same data"; and the bilateral-exchange simulation where prompt-encoded biases compound into power concentration and market collapse, "a reminder that agent populations in thin books can move the thing they are trading."</t>
+          <t>"This is the citation for the positioning claim, scoped to what it can carry. The permitted form is that a survey of thirty-one systems organises them by use case and by workflow stage without a stage for weighting agent influence, and that among the four systems it compares directly on adaptive architecture, none adapts the influence of one component on the decision. That is a claim about this survey's coverage, not about the literature, and I should pair it with the absence of a stated review protocol in the same sentence so the scoping is mine rather than something a reader catches me on." "Behavioural fidelity gives my ablations a vocabulary and a second axis of results. Responsiveness to events, strategy adherence and position tracking are named metric families… Dropping volatility from the conditioning set should show up as reduced responsiveness to volatility events, not only as a lower Sharpe, and reporting the behavioural change beside the return change is how I avoid the situation where the dynamic scheme beats the static learned weight by a margin too small to defend. This also gives the ablation table a row to fill when a return difference fails to clear significance on CSE-length data." "Their evaluation verdict licenses building my own protocol, and the data blocker remains the real constraint." "Unfaithful chain-of-thought settles the shape of the explainability story. If natural-language justifications are frequently not faithful to the reasoning that produced them, then an explanation layer that reports what the agents said about themselves is worth very little. What I already have is attribution over computed quantities, the orchestrator's weight vector, SHAP over risk features, interpretable volatility-model parameters, and citation tracing back to the retrieved passage, and all four are auditable in a way an LLM's narration is not." "Two cautions to build a baseline against" - a study testing whether prompt-driven LLM agents merely reproduce momentum or value, "which is a direct question to put to my technical agent: does it add anything over a prompted momentum rule on the same data"; and the bilateral-exchange simulation where prompt-encoded biases compound into power concentration and market collapse, "a reminder that agent populations in thin books can move the thing they are trading."</t>
         </is>
       </c>
       <c r="V32" s="11" t="inlineStr">
@@ -4599,8 +4599,8 @@
       <c r="W32" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (Stage 9, the adaptive-architecture row, the heterogeneity-of-reading distinction), A_L (absence of any liquidity branch), friction-aware evaluation layer (behavioural fidelity metrics, no-unified-protocol statement).
-EFFECT ON MAIN GAP: Leaves it open, and is the single best positioning citation of the seven — but only in a tightly scoped form. It gives the gap in the field's own vocabulary (Stage 9 is an undifferentiated box; collaboration means ask-respond and debate; none of the four compared systems adapts component influence). Its one nominated counterexample has since been read and does not survive contact. The scoping caveat is mandatory: no review protocol, so an empty cell is not evidence of a gap in the field, only in this survey's coverage.
-CONFIDENCE SCORING: One lead only, unelaborated — "a confidence-aware critic that adaptively refines only low-confidence prompts without external signals, which is the only mechanism in the survey for producing an agent confidence without a labelled target." No detail, no results, not yet read.
+EFFECT ON MAIN GAP: Leaves it open, and is the single best positioning citation of the seven - but only in a tightly scoped form. It gives the gap in the field's own vocabulary (Stage 9 is an undifferentiated box; collaboration means ask-respond and debate; none of the four compared systems adapts component influence). Its one nominated counterexample has since been read and does not survive contact. The scoping caveat is mandatory: no review protocol, so an empty cell is not evidence of a gap in the field, only in this survey's coverage.
+CONFIDENCE SCORING: One lead only, unelaborated - "a confidence-aware critic that adaptively refines only low-confidence prompts without external signals, which is the only mechanism in the survey for producing an agent confidence without a labelled target." No detail, no results, not yet read.
 FIXED-INFLUENCE FAILURE EVIDENCE: No measured degradation case. Its contribution is prevalence rather than failure: two of four compared systems marked no adaptive architecture at all, one a planning loop, one RLHF inside a single model.
 PROPOSED REVISION STATED IN THE NOTE: None to the four-agent pool or the conditioning set. The revisions are to the evaluation and the write-up: add behavioural fidelity metrics (responsiveness to events, strategy adherence, position tracking) as a second results axis for the state-input ablations; run a prompted-momentum-rule baseline against A_T; state the heterogeneity-of-evidence vs heterogeneity-of-reading distinction explicitly; frame explainability as attribution over computed quantities rather than LLM narration.</t>
         </is>
@@ -4654,22 +4654,22 @@
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>Structured data 1 March 2021 – 28 February 2025, 1,461 aligned daily records after an inner join on date. Effective analysis sample 1,341 days because the 120-day indicator window costs the first 120 rows. Text: 67,075 Reddit posts from crypto subreddits via Reddit Archive and 8,657 Bitcoin news articles from LexisNexis, covering only 304 trading days, 1 May 2024 – 28 February 2025. Chronological split 64:16:20, MinMaxScaler fitted on training only. Test period 6 June 2024 – 28 February 2025, 268 days, held common across all three window sizes.</t>
+          <t>Structured data 1 March 2021–28 February 2025, 1,461 aligned daily records after an inner join on date. Effective analysis sample 1,341 days because the 120-day indicator window costs the first 120 rows. Text: 67,075 Reddit posts from crypto subreddits via Reddit Archive and 8,657 Bitcoin news articles from LexisNexis, covering only 304 trading days, 1 May 2024–28 February 2025. Chronological split 64:16:20, MinMaxScaler fitted on training only. Test period 6 June 2024–28 February 2025, 268 days, held common across all three window sizes.</t>
         </is>
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>Binance OHLCV via ccxt. On-chain: five Bitinfocharts fields — confirmation time, hash rate, transaction fees, active addresses. Macro-financial: five Yahoo Finance series — dollar index, gold, S&amp;P 500, VIX, WTI crude, forward-filled from Friday close through the weekend so that "1,007 raw trading days are imputed up to 1,461 crypto-calendar days, which means roughly 30% of the macro channel is a repeated Friday value." Technical indicators in three groups: trend following (SMA, EMA over 3–120 day windows, MACD), momentum (RSI, raw momentum, 10-day rate of change), oscillators (Stochastic RSI, Stochastic, 14-day Williams %R). Text "is never merged into the structured join, it is aligned by date at the prompt-construction stage only," capped at 90,000 words per three-day decision window with a 30,000-word daily limit per source, stratified sampling in proportion to source counts when the cap binds.</t>
+          <t>Binance OHLCV via ccxt. On-chain: five Bitinfocharts fields - confirmation time, hash rate, transaction fees, active addresses. Macro-financial: five Yahoo Finance series - dollar index, gold, S&amp;P 500, VIX, WTI crude, forward-filled from Friday close through the weekend so that "1,007 raw trading days are imputed up to 1,461 crypto-calendar days, which means roughly 30% of the macro channel is a repeated Friday value." Technical indicators in three groups: trend following (SMA, EMA over 3–120 day windows, MACD), momentum (RSI, raw momentum, 10-day rate of change), oscillators (Stochastic RSI, Stochastic, 14-day Williams %R). Text "is never merged into the structured join, it is aligned by date at the prompt-construction stage only," capped at 90,000 words per three-day decision window with a 30,000-word daily limit per source, stratified sampling in proportion to source counts when the cap binds.</t>
         </is>
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>Zero-shot GPT-4o, temperature 0.7, top-p 1.0, 1,024 max tokens. "no fine-tuning and no gradient training anywhere in the agent path." Every configuration repeated across 20 seeds with results averaged and dispersion reported. Baselines LSTM, GRU, DLinear, PatchTST get hidden dimensions 32/64/128, learning rates 0.0005 (0.01–0.05 for DLinear), batch size 64, Adam, up to 100 epochs with early stopping at patience 10, plus a grid search over trading thresholds. Threshold rule: Δp_t = (ŷ_t − y_{t−1}) / y_{t−1}, with BUY if Δp_t &gt; θ, SELL if Δp_t &lt; −θ, HOLD if |Δp_t| ≤ θ; θ = 0.015 for 3 and 14-day windows and 0.010 for 30-day. "baseline thresholds were calibrated so that average trade counts land in the 70 to 110 range, matching the trading frequency the LLM agent produces on its own, which removes the obvious confound of one strategy winning by trading more."  Three domain agents (technical indicators, on-chain metrics, macro-financial variables) each read a sliding window of 3, 14 or 30 days over their own modality and "produce a prose summary of recent conditions, explicitly without making a price prediction, one on momentum dynamics and indicator signals, one on network activity and participation shifts, one on global risk sentiment and volatility spillovers." A meta trading agent receives all summaries and emits BUY/SELL/HOLD plus a written rationale. Two further text agents (Reddit, news wires) added in ablation. Hallucination control by two constraints: "agents run from fixed domain-specific templates rather than open-ended generation, and the meta-agent is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." GPT-4o selected over Claude, Gemini and FinGPT "on instruction-hierarchy evaluations, which matters for a design where conflicting agent outputs have to be aggregated under a single controlling instruction."</t>
+          <t>Zero-shot GPT-4o, temperature 0.7, top-p 1.0, 1,024 max tokens. "no fine-tuning and no gradient training anywhere in the agent path." Every configuration repeated across 20 seeds with results averaged and dispersion reported. Baselines LSTM, GRU, DLinear, PatchTST get hidden dimensions 32/64/128, learning rates 0.0005 (0.01–0.05 for DLinear), batch size 64, Adam, up to 100 epochs with early stopping at patience 10, plus a grid search over trading thresholds. Threshold rule: Δp_t = (ŷ_t − y_{t−1}) / y_{t−1}, with BUY if Δp_t &gt; θ, SELL if Δp_t &lt; −θ, HOLD if |Δp_t| ≤ θ; θ = 0.015 for 3 and 14-day windows and 0.010 for 30-day. "baseline thresholds were calibrated so that average trade counts land in the 70 to 110 range, matching the trading frequency the LLM agent produces on its own, which removes the obvious confound of one strategy winning by trading more." Three domain agents (technical indicators, on-chain metrics, macro-financial variables) each read a sliding window of 3, 14 or 30 days over their own modality and "produce a prose summary of recent conditions, explicitly without making a price prediction, one on momentum dynamics and indicator signals, one on network activity and participation shifts, one on global risk sentiment and volatility spillovers." A meta trading agent receives all summaries and emits BUY/SELL/HOLD plus a written rationale. Two further text agents (Reddit, news wires) added in ablation. Hallucination control by two constraints: "agents run from fixed domain-specific templates rather than open-ended generation, and the meta-agent is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." GPT-4o selected over Claude, Gemini and FinGPT "on instruction-hierarchy evaluations, which matters for a design where conflicting agent outputs have to be aggregated under a single controlling instruction."</t>
         </is>
       </c>
       <c r="L33" s="11" t="inlineStr">
         <is>
-          <t>- Three core domain agents plus a meta trading agent; two further text agents in ablation, so up to five producers. Genuinely heterogeneous in modality — "The agents are genuinely heterogeneous in modality, technical, on-chain, macro, social and news, which is the property I have been arguing separates my design from MacroHFT's six architecturally identical DDQN sub-agents." But note: heterogeneous in *evidence*, homogeneous in *method* — all are GPT-4o prompted from fixed templates. Evidence each sees: technical agent sees its own indicator set over a 3/14/30-day sliding window; on-chain agent sees five Bitinfocharts fields; macro agent sees five Yahoo series; Reddit agent sees sampled subreddit posts; news agent sees sampled LexisNexis articles. Each emits a prose summary and explicitly no price prediction. - Combination: a fixed prompt template in the meta trading agent. No weights, no votes, no debate, no manager optimisation. The meta-agent "is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." - Does anything vary influence by market state, regime, volatility, liquidity or measured reliability? No — and this is the paper's decisive contribution to the gap. Quoting the note: "the meta-agent's relationship to them is a fixed prompt template, so every agent's influence is constant regardless of whether it is saying anything useful that day. The ablation then shows exactly what that costs, adding a news agent takes total return from 21.75% to 11.39%, and nothing in the architecture can notice or respond. That is the cleanest quantified case for my main gap that I have found, and the fact that the authors read it as a signal-integration problem rather than an orchestration problem is the opening." - Confidence per agent: no per-agent confidence at all. What exists instead is a *pairwise, external* score over agent outputs — see below. The G-EVAL layer is diagnostic only; it never feeds back into the decision.</t>
+          <t>- Three core domain agents plus a meta trading agent; two further text agents in ablation, so up to five producers. Genuinely heterogeneous in modality - "The agents are genuinely heterogeneous in modality, technical, on-chain, macro, social and news, which is the property I have been arguing separates my design from MacroHFT's six architecturally identical DDQN sub-agents." But note: heterogeneous in *evidence*, homogeneous in *method* - all are GPT-4o prompted from fixed templates. Evidence each sees: technical agent sees its own indicator set over a 3/14/30-day sliding window; on-chain agent sees five Bitinfocharts fields; macro agent sees five Yahoo series; Reddit agent sees sampled subreddit posts; news agent sees sampled LexisNexis articles. Each emits a prose summary and explicitly no price prediction. - Combination: a fixed prompt template in the meta trading agent. No weights, no votes, no debate, no manager optimisation. The meta-agent "is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." - Does anything vary influence by market state, regime, volatility, liquidity or measured reliability? No - and this is the paper's decisive contribution to the gap. Quoting the note: "the meta-agent's relationship to them is a fixed prompt template, so every agent's influence is constant regardless of whether it is saying anything useful that day. The ablation then shows exactly what that costs, adding a news agent takes total return from 21.75% to 11.39%, and nothing in the architecture can notice or respond. That is the cleanest quantified case for my main gap that I have found, and the fact that the authors read it as a signal-integration problem rather than an orchestration problem is the opening." - Confidence per agent: no per-agent confidence at all. What exists instead is a *pairwise, external* score over agent outputs - see below. The G-EVAL layer is diagnostic only; it never feeds back into the decision.</t>
         </is>
       </c>
       <c r="M33" s="11" t="inlineStr">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="Q33" s="11" t="inlineStr">
         <is>
-          <t>The meta-agent emits a written rationale. Separately, G-EVAL scoring over agent-output *pairs* — see CONFIDENCE SCORING below. "The interpretability evaluation is the same model family grading its own output, and is never checked against outcomes."</t>
+          <t>The meta-agent emits a written rationale. Separately, G-EVAL scoring over agent-output *pairs* - see CONFIDENCE SCORING below. "The interpretability evaluation is the same model family grading its own output, and is never checked against outcomes."</t>
         </is>
       </c>
       <c r="R33" s="11" t="inlineStr">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="S33" s="11" t="inlineStr">
         <is>
-          <t>3-day window — "Total return of 21.75% ± 3.03 against LSTM's 20.05% ± 3.74 and buy-and-hold's 18.90%, with a Sharpe of 1.08 ± 0.11 against LSTM's 1.05 ± 0.17 and buy-and-hold's 0.80"; MDD falls from 22.52% to 14.69% ± 0.87 and Calmar rises from 1.19 to 1.99 ± 0.25, but "LSTM still holds both the best drawdown at 13.10% and the best Calmar at 2.07." Horizon reversal: 14-day best total return GRU 21.65%, best Sharpe PatchTST 1.15, agent 20.34% / 1.02 / 15.88%; 30-day best return GRU 22.14%, best Sharpe GRU 1.55, agent 17.40% / 0.77 / 20.49%. "At 30 days the agent's Sharpe of 0.77 ± 0.22 is below buy-and-hold's 0.80 and its Calmar of 1.14 ± 0.33 is barely above the passive 1.19." Behaviour: "the agent runs 83.67 ± 11.22 trades against GRU's 74.35 and LSTM's 90.12, turnover of 7.60 ± 1.12 against 6.90 and 6.75, exposure time of 93.15% and an average holding period of 22 days against 18.35 and 19.02." Text ablation: "Against the 21.75% structured-only baseline, adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55, adding the social media agent lifts it to 23.30% ± 2.41 with Sharpe 1.12 ± 0.12 and Calmar 2.01, and adding both lands at 18.98% ± 5.74, below the baseline that used neither. Scoped honestly, the social gain of 1.55 points sits well inside a ± 2.41 band and I would not claim it, whereas the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying." G-EVAL: "Conflict scores average 0.42 with a median of 0.30 and a top quartile above 0.60, and the distribution is visibly bimodal, a large mass of low-conflict days and a secondary cluster near 0.7. Actionability averages 0.55 with a median of 0.60 and a maximum of 0.90." LIMITATIONS (quoting the note): "The headline advantage does not clear its own error bars and no significance test is run anywhere.… seed dispersion measures LLM sampling variance and not variation across market paths, and there is still one asset, one 268-day test window and one regime, a period over which passive Bitcoin returned 18.90%. A 1.70 point edge over LSTM with standard deviations of 3.03 and 3.74 is not an edge I would defend without a paired test, and the paper offers none." "Friction is a flat constant on the deepest book in crypto, and the sensitivity band is too narrow to bind." "Threshold and hyperparameter selection is described as a grid search without ever naming the selection set… since the threshold is the only thing converting a baseline forecast into a strategy, any leakage there lands directly on the comparison the paper's central claim rests on." "The text-agent ablation confounds content with prompt budget and runs at one window size only. Adding an agent adds thousands of words to the prompt as well as a new information source, and there is no placebo agent, no prompt-length control and no run with news content shuffled across dates, so the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both." "The interpretability evaluation is the same model family grading its own output, and is never checked against outcomes. GPT-4o writes the Reddit and news summaries and GPT-4o scores their conflict and actionability, so the scores measure internal consistency of one model's reading rather than anything external. The authors say plainly in the limitations that they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates, and until that is done the scores diagnose the reasoning process without establishing that the process is tracking anything." "Zero-shot with fixed templates is the design's cost as well as its selling point… the template constraint that suppresses hallucination is the same constraint that limits reasoning flexibility, a trade-off the paper names but does not measure." Also: "84 trades over 268 days sits awkwardly with a 22-day mean holding period, and the paper does not reconcile the two definitions"; and Table 7 reports 21.82% where Table 3 reports 21.75% for what should be the same configuration.</t>
+          <t>3-day window - "Total return of 21.75% ± 3.03 against LSTM's 20.05% ± 3.74 and buy-and-hold's 18.90%, with a Sharpe of 1.08 ± 0.11 against LSTM's 1.05 ± 0.17 and buy-and-hold's 0.80"; MDD falls from 22.52% to 14.69% ± 0.87 and Calmar rises from 1.19 to 1.99 ± 0.25, but "LSTM still holds both the best drawdown at 13.10% and the best Calmar at 2.07." Horizon reversal: 14-day best total return GRU 21.65%, best Sharpe PatchTST 1.15, agent 20.34% / 1.02 / 15.88%; 30-day best return GRU 22.14%, best Sharpe GRU 1.55, agent 17.40% / 0.77 / 20.49%. "At 30 days the agent's Sharpe of 0.77 ± 0.22 is below buy-and-hold's 0.80 and its Calmar of 1.14 ± 0.33 is barely above the passive 1.19." Behaviour: "the agent runs 83.67 ± 11.22 trades against GRU's 74.35 and LSTM's 90.12, turnover of 7.60 ± 1.12 against 6.90 and 6.75, exposure time of 93.15% and an average holding period of 22 days against 18.35 and 19.02." Text ablation: "Against the 21.75% structured-only baseline, adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55, adding the social media agent lifts it to 23.30% ± 2.41 with Sharpe 1.12 ± 0.12 and Calmar 2.01, and adding both lands at 18.98% ± 5.74, below the baseline that used neither. Scoped honestly, the social gain of 1.55 points sits well inside a ± 2.41 band and I would not claim it, whereas the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying." G-EVAL: "Conflict scores average 0.42 with a median of 0.30 and a top quartile above 0.60, and the distribution is visibly bimodal, a large mass of low-conflict days and a secondary cluster near 0.7. Actionability averages 0.55 with a median of 0.60 and a maximum of 0.90." LIMITATIONS (quoting the note): "The headline advantage does not clear its own error bars and no significance test is run anywhere.… seed dispersion measures LLM sampling variance and not variation across market paths, and there is still one asset, one 268-day test window and one regime, a period over which passive Bitcoin returned 18.90%. A 1.70 point edge over LSTM with standard deviations of 3.03 and 3.74 is not an edge I would defend without a paired test, and the paper offers none." "Friction is a flat constant on the deepest book in crypto, and the sensitivity band is too narrow to bind." "Threshold and hyperparameter selection is described as a grid search without ever naming the selection set… since the threshold is the only thing converting a baseline forecast into a strategy, any leakage there lands directly on the comparison the paper's central claim rests on." "The text-agent ablation confounds content with prompt budget and runs at one window size only. Adding an agent adds thousands of words to the prompt as well as a new information source, and there is no placebo agent, no prompt-length control and no run with news content shuffled across dates, so the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both." "The interpretability evaluation is the same model family grading its own output, and is never checked against outcomes. GPT-4o writes the Reddit and news summaries and GPT-4o scores their conflict and actionability, so the scores measure internal consistency of one model's reading rather than anything external. The authors say plainly in the limitations that they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates, and until that is done the scores diagnose the reasoning process without establishing that the process is tracking anything." "Zero-shot with fixed templates is the design's cost as well as its selling point… the template constraint that suppresses hallucination is the same constraint that limits reasoning flexibility, a trade-off the paper names but does not measure." Also: "84 trades over 268 days sits awkwardly with a 22-day mean holding period, and the paper does not reconcile the two definitions"; and Table 7 reports 21.82% where Table 3 reports 21.75% for what should be the same configuration.</t>
         </is>
       </c>
       <c r="T33" s="11" t="inlineStr">
@@ -4725,9 +4725,9 @@
       <c r="W33" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (the fixed-template failure case, the horizon-reversal argument, the G-EVAL conflict mechanism), A_T (technical agent, and the LSTM/GRU horizon result), A_F (the news agent is the nearest analogue to the retrieval channel), friction-aware evaluation layer (stated 0.1% + 0.1%, and the unreconciled sensitivity band).
-EFFECT ON MAIN GAP: Leaves it open and supplies the single strongest quantified motivation for it in the whole set. This is the closest published system to the proposed orchestration structure — genuinely heterogeneous agents, a meta-synthesiser, a shared execution harness — "and it is the most useful paper in my set precisely because the orchestration is the part it does not do." The news agent costs 10.36 points of total return under a controlled ablation with dispersion reported (±1.06 against a 21.75% baseline), far outside any error band in the table, and the architecture has no mechanism to detect or respond to it. The counterfactual the paper leaves unbuilt is exactly the proposed contribution. It also supplies, free, the horizon evidence that different component families genuinely win at different horizons (GRU takes the 30-day window on return, Sharpe, Sortino and Calmar while the agent falls below passive on risk-adjusted terms), which is "a concrete, testable instantiation of the main gap."
+EFFECT ON MAIN GAP: Leaves it open and supplies the single strongest quantified motivation for it in the whole set. This is the closest published system to the proposed orchestration structure - genuinely heterogeneous agents, a meta-synthesiser, a shared execution harness - "and it is the most useful paper in my set precisely because the orchestration is the part it does not do." The news agent costs 10.36 points of total return under a controlled ablation with dispersion reported (±1.06 against a 21.75% baseline), far outside any error band in the table, and the architecture has no mechanism to detect or respond to it. The counterfactual the paper leaves unbuilt is exactly the proposed contribution. It also supplies, free, the horizon evidence that different component families genuinely win at different horizons (GRU takes the 30-day window on return, Sharpe, Sortino and Calmar while the agent falls below passive on risk-adjusted terms), which is "a concrete, testable instantiation of the main gap."
 CONFIDENCE SCORING: This is the candidate mechanism, and it is the only one of its kind in the set. G-EVAL (Liu et al., 2023) is a protocol where an LLM scores generated text against a rubric in a zero-shot prompt, rather than against a reference. Jung and Lee apply it to pairs of agent outputs, scoring each daily Reddit summary against the matching news summary on two rubrics: a conflict score for semantic divergence in tone, outlook and implication, and an actionability score for whether the combination yields a clear and timely trading signal. Both are 0 to 1. The scoring model is GPT-4o, which is also the model that wrote the summaries being scored. Measured distributions: conflict mean 0.42, median 0.30, top quartile above 0.60, visibly bimodal with a secondary cluster near 0.7; actionability mean 0.55, median 0.60, maximum 0.90. The authors' two conclusions: "that divergence between sources makes a coherent reasoning chain harder to build, and that even agreeing sources often fail to produce a usable signal. The first is consistent with the dual-agent degradation, the second is the more uncomfortable one and is the reason I would treat actionability as the more informative of the two scores." Why it matters, verbatim: "Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem. My orchestration function needs confidence on a common scale across an LLM analyst, an econometric estimator and an RL policy, and nothing in the literature supplies one, because each component's native confidence means something different. The move here is to stop asking the agents and score the *relationship between their outputs* externally on a fixed rubric, which sidesteps internal calibration entirely and generalises to any pair of producers that can emit text. I would take the mechanism and not the validation, since scoring pairwise conflict is cheap and establishing that it predicts anything is the work this paper skips." The pre-registered test, verbatim: "compute conflict scores across agent pairs on CSE data, then check whether they correlate with realised next-period error or return before any of it touches the orchestrator. If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses." Known weaknesses of the mechanism as published: same model family grades its own output; never validated against outcomes (the authors concede they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates); pairwise only, not per-agent; diagnostic only, never fed back.
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes — the strongest in the set, and the only one with a controlled number attached. "adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55… the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying." And: "here a news agent costs 10.36 points of total return while the architecture has no way to notice." Caveat the note itself attaches: "the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both," because there is no placebo agent, no prompt-length control and no date-shuffled run. A secondary case: adding both text agents lands at 18.98% ± 5.74, "below the baseline that used neither."
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes - the strongest in the set, and the only one with a controlled number attached. "adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55… the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying." And: "here a news agent costs 10.36 points of total return while the architecture has no way to notice." Caveat the note itself attaches: "the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both," because there is no placebo agent, no prompt-length control and no date-shuffled run. A secondary case: adding both text agents lands at 18.98% ± 5.74, "below the baseline that used neither."
 PROPOSED REVISION STATED IN THE NOTE: To the conditioning set, verbatim: "compute conflict scores across agent pairs on CSE data, then check whether they correlate with realised next-period error or return before any of it touches the orchestrator. If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses." To the experiment set, verbatim: "a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to… Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one." No change to the four-agent pool; sentiment confirmed out of scope.</t>
         </is>
       </c>
@@ -4770,12 +4770,12 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Takes the "child-order execution problem, the last atomic step after a parent order has already been sliced," and formulates it as an "optimal stopping problem: the trader holds one indivisible share, has a horizon of $T$ seconds, and at each second chooses CONTINUE or STOP." Two data-driven solutions on one neural architecture — a supervised method forecasting the whole future price-change trajectory and acting on it, and an RL method learning the continuation value directly. Both trained with a TD($m$-step) family spanning one-step TD to empirical Monte Carlo, "so the paper is really four algorithm families rather than two."</t>
+          <t>Takes the "child-order execution problem, the last atomic step after a parent order has already been sliced," and formulates it as an "optimal stopping problem: the trader holds one indivisible share, has a horizon of $T$ seconds, and at each second chooses CONTINUE or STOP." Two data-driven solutions on one neural architecture - a supervised method forecasting the whole future price-change trajectory and acting on it, and an RL method learning the continuation value directly. Both trained with a TD($m$-step) family spanning one-step TD to empirical Monte Carlo, "so the paper is really four algorithm families rather than two."</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>NASDAQ equities — "the most liquid equity market in the world." 50 high-liquidity stocks; spreads from 1 to 54.36 ticks. Extremely deep books; the note stresses the order is assumed infinitesimal relative to depth.</t>
+          <t>NASDAQ equities - "the most liquid equity market in the world." 50 high-liquidity stocks; spreads from 1 to 54.36 ticks. Extremely deep books; the note stresses the order is assumed infinitesimal relative to depth.</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -4785,17 +4785,17 @@
       </c>
       <c r="J34" s="11" t="inlineStr">
         <is>
-          <t>Level-III LOB message data only; no text, no fundamentals. State is not a single snapshot — "ten sets of features are collected, one at the current second and one at each of the previous nine, so $x_t = (s_{t-9}, \ldots, s_t)$." Feature groups: general information (time of day, price normalized by average spread); spread normalized by return and price volatility; depth at the top 5 levels with queue imbalance; trading flow counts in the last second; exponentially decaying intensity measures for trades and price changes. Everything defined near-side/far-side rather than bid/ask "so a buy and a sell episode look identical to the network." Queue imbalance: $$QI = \frac{\text{near depth} - \text{far depth}}{\text{near depth} + \text{far depth}}$$ computed at each of the top 5 levels and on aggregated depth, $QI \in [-1,1]$.</t>
+          <t>Level-III LOB message data only; no text, no fundamentals. State is not a single snapshot - "ten sets of features are collected, one at the current second and one at each of the previous nine, so $x_t = (s_{t-9}, \ldots, s_t)$." Feature groups: general information (time of day, price normalized by average spread); spread normalized by return and price volatility; depth at the top 5 levels with queue imbalance; trading flow counts in the last second; exponentially decaying intensity measures for trades and price changes. Everything defined near-side/far-side rather than bid/ask "so a buy and a sell episode look identical to the network." Queue imbalance: $$QI = \frac{\text{near depth} - \text{far depth}}{\text{near depth} + \text{far depth}}$$ computed at each of the top 5 levels and on aggregated depth, $QI \in [-1,1]$.</t>
         </is>
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>RNN with 10 LSTM units of dimension 64, one per feature set, feeding 5 fully connected layers with batch normalization into an output layer of dimension 60 matching the horizon. LR $3\times10^{-5}$, batch 1024, target network copied every 1000 gradient steps, $m=15$ for headline results, 50,000 gradient steps, 10 random starts. Continuation value: $$C_{t:T}(x) = \mathbb{E}\big[\Delta p_{t+1} + \max\{0,\ C_{t+1:T}(x_{t+1})\}\ \big|\ x_t = x\big]$$ with $C_{T:T}\triangleq 0$; policy is CONTINUE while $C_{t:T}(x)&gt;0$. Architectural contribution is monotonicity by construction: $$\delta_i(x) \triangleq C_{t:t+i}(x) - C_{t:t+i-1}(x) \geq 0 \ (i&gt;1), \qquad \hat C^{\phi}_{t:T}(x) = \sum_{i=1}^{T-t} u_i^{\phi}(x)$$ — 60 outputs predict increments, softplus on all but the first, any horizon's value is a partial sum. TD($m$-step) target: $$\tilde C_{t:T}(x_t) = \Delta p_{t+1} + \sum_{i=2}^{m}\Delta p_{t+i}\prod_{j=1}^{i-1}\mathbb{1}\{\hat C^{\phi}_{t+j:T}(x_{t+j}) &gt; 0\} + \hat C^{\phi'}_{t+m:T}(x_{t+m})\prod_{j=1}^{m}\mathbb{1}\{\hat C^{\phi}_{t+j:T}(x_{t+j}) &gt; 0\}$$ with train-net $\phi$ in the indicator and target-net $\phi'$ in the value (double Q-learning, van Hasselt 2010). Output: a binary CONTINUE/STOP decision.</t>
+          <t>RNN with 10 LSTM units of dimension 64, one per feature set, feeding 5 fully connected layers with batch normalization into an output layer of dimension 60 matching the horizon. LR $3\times10^{-5}$, batch 1024, target network copied every 1000 gradient steps, $m=15$ for headline results, 50,000 gradient steps, 10 random starts. Continuation value: $$C_{t:T}(x) = \mathbb{E}\big[\Delta p_{t+1} + \max\{0,\ C_{t+1:T}(x_{t+1})\}\ \big|\ x_t = x\big]$$ with $C_{T:T}\triangleq 0$; policy is CONTINUE while $C_{t:T}(x)&gt;0$. Architectural contribution is monotonicity by construction: $$\delta_i(x) \triangleq C_{t:t+i}(x) - C_{t:t+i-1}(x) \geq 0 \ (i&gt;1), \qquad \hat C^{\phi}_{t:T}(x) = \sum_{i=1}^{T-t} u_i^{\phi}(x)$$ - 60 outputs predict increments, softplus on all but the first, any horizon's value is a partial sum. TD($m$-step) target: $$\tilde C_{t:T}(x_t) = \Delta p_{t+1} + \sum_{i=2}^{m}\Delta p_{t+i}\prod_{j=1}^{i-1}\mathbb{1}\{\hat C^{\phi}_{t+j:T}(x_{t+j}) &gt; 0\} + \hat C^{\phi'}_{t+m:T}(x_{t+m})\prod_{j=1}^{m}\mathbb{1}\{\hat C^{\phi}_{t+j:T}(x_{t+j}) &gt; 0\}$$ with train-net $\phi$ in the indicator and target-net $\phi'$ in the value (double Q-learning, van Hasselt 2010). Output: a binary CONTINUE/STOP decision.</t>
         </is>
       </c>
       <c r="L34" s="11" t="inlineStr">
         <is>
-          <t>None. The note states it plainly — "this is a single agent making a single binary decision over sixty seconds in the most liquid equity market in the world, with no portfolio, no allocation, no orchestration and no heterogeneous components."</t>
+          <t>None. The note states it plainly - "this is a single agent making a single binary decision over sixty seconds in the most liquid equity market in the world, with no portfolio, no allocation, no orchestration and no heterogeneous components."</t>
         </is>
       </c>
       <c r="M34" s="11" t="inlineStr">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="O34" s="11" t="inlineStr">
         <is>
-          <t>Volatility appears only as an input feature ("spread normalized by return and price volatility"). There is no risk term in the objective; the objective is pure expected price gain over a 60-second stopping problem. The note later contrasts this against Wang et al.: "neither of the other two execution notes carries a risk term." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's defining weakness and the note treats it as such. There is no market impact model of any kind — no Almgren-Chriss, no square-root, no linear impact. Impact is assumed away by construction: "the order is infinitesimal and ... any action of the trader has no effect on the price process, the states or the transition kernel, which is what makes the problem a pure stopping problem rather than a control problem." Spread is handled only as the *unit of measurement*, not as a cost to be modelled: the half-spread is "the time-averaged difference between best bid and best ask over the previous 5 trading days, halved," and every result is a price gain as a percentage of it, where "a gain of 100% means the trade executed at the mid-price, so the trader crossed no spread at all and traded frictionlessly." Queue: queue imbalance is used as a *feature* at top 5 levels, but there is no queue position modelling. Fills: "STOP is assumed to produce an immediate fill at the observed price, which implicitly means a marketable order crossing the spread." No partial fills, no cancellation, no passive posting, no loss of queue priority, no commission or exchange fee anywhere in the objective. Calibration: none of an impact model; the only calibration-like quantity is the trailing 5-day half-spread normalizer and 21-day volume normalization of depth features. Critically: "The paper builds the limit order book in full from ITCH messages and then uses it only as a feature source, never as a fill simulator, so the reported gains are upper bounds on what the same policy would achieve against a book that has to be interacted with rather than observed."</t>
+          <t>Volatility appears only as an input feature ("spread normalized by return and price volatility"). There is no risk term in the objective; the objective is pure expected price gain over a 60-second stopping problem. The note later contrasts this against Wang et al.: "neither of the other two execution notes carries a risk term." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's defining weakness and the note treats it as such. There is no market impact model of any kind - no Almgren-Chriss, no square-root, no linear impact. Impact is assumed away by construction: "the order is infinitesimal and ... any action of the trader has no effect on the price process, the states or the transition kernel, which is what makes the problem a pure stopping problem rather than a control problem." Spread is handled only as the *unit of measurement*, not as a cost to be modelled: the half-spread is "the time-averaged difference between best bid and best ask over the previous 5 trading days, halved," and every result is a price gain as a percentage of it, where "a gain of 100% means the trade executed at the mid-price, so the trader crossed no spread at all and traded frictionlessly." Queue: queue imbalance is used as a *feature* at top 5 levels, but there is no queue position modelling. Fills: "STOP is assumed to produce an immediate fill at the observed price, which implicitly means a marketable order crossing the spread." No partial fills, no cancellation, no passive posting, no loss of queue priority, no commission or exchange fee anywhere in the objective. Calibration: none of an impact model; the only calibration-like quantity is the trailing 5-day half-spread normalizer and 21-day volume normalization of depth features. Critically: "The paper builds the limit order book in full from ITCH messages and then uses it only as a feature source, never as a fill simulator, so the reported gains are upper bounds on what the same policy would achieve against a book that has to be interacted with rather than observed."</t>
         </is>
       </c>
       <c r="P34" s="11" t="inlineStr">
@@ -4851,8 +4851,8 @@
       <c r="W34" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_L (queue imbalance, near/far depth, trade intensity are exactly $A_L$'s ideal feature set), friction-aware evaluation layer (half-spread reporting unit), orchestrator (value-based rather than predict-then-threshold; encode simplex/monotonicity constraints in the architecture; take-one-out protocol).
-EFFECT ON MAIN GAP / SUB-GAP 2: Main gap — indirect but real: the note lifts two architectural lessons for the orchestrator (encode known structure such as simplex/non-negativity/monotonicity in the output layer rather than as a loss penalty; train the orchestrator by averaging over actions taken rather than averaging predicted states, per the SL-vs-RL counterexample $\Delta P_A = [+1,-4]$, $\Delta P_B=[-2,+3]$). Sub-gap 2 — none; volatility appears only as an input feature and there is no long-memory or risk-guardrail content.
-EFFECT ON SUB-GAP 1: LEAVES IT WIDE OPEN — and is the best available citation that it is open. This paper implements NO impact model at all: not Almgren-Chriss, not square-root, not linear. It explicitly assumes the order is infinitesimal so that cost is *not* a function of order size against depth. The note is unambiguous: "Every portfolio paper in the vault, and my own design so far, converts a target weight into a fill at a flat percentage. Moallemi and Wang show what the layer underneath actually contains, and they solve it cleanly by assuming the order is small enough not to move the book. In a thin frontier market that assumption is precisely what fails." Note also that the paper reconstructs a full LOB and then uses it only as a feature source, "never as a fill simulator" — so it does not even supply an execution simulator that could be repurposed. Net effect: strengthens the sub-gap by naming the prior art and showing precisely why it does not transfer.
+EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - indirect but real: the note lifts two architectural lessons for the orchestrator (encode known structure such as simplex/non-negativity/monotonicity in the output layer rather than as a loss penalty; train the orchestrator by averaging over actions taken rather than averaging predicted states, per the SL-vs-RL counterexample $\Delta P_A = [+1,-4]$, $\Delta P_B=[-2,+3]$). Sub-gap 2 - none; volatility appears only as an input feature and there is no long-memory or risk-guardrail content.
+EFFECT ON SUB-GAP 1: LEAVES IT WIDE OPEN - and is the best available citation that it is open. This paper implements NO impact model at all: not Almgren-Chriss, not square-root, not linear. It explicitly assumes the order is infinitesimal so that cost is *not* a function of order size against depth. The note is unambiguous: "Every portfolio paper in the vault, and my own design so far, converts a target weight into a fill at a flat percentage. Moallemi and Wang show what the layer underneath actually contains, and they solve it cleanly by assuming the order is small enough not to move the book. In a thin frontier market that assumption is precisely what fails." Note also that the paper reconstructs a full LOB and then uses it only as a feature source, "never as a fill simulator" - so it does not even supply an execution simulator that could be repurposed. Net effect: strengthens the sub-gap by naming the prior art and showing precisely why it does not transfer.
 PROPOSED REVISION STATED IN THE NOTE: Two, both on the agent pool / evaluation rather than on $f(L_t, V_t, P_t, C_{i,t})$ directly. Verbatim: "An execution-timing agent is a cheap addition to the orchestrator, and the SL counterexample is the reason it should be value-based. A network making one binary decision over a short window is small next to a full RL allocator, so adding execution timing as a component is affordable if the data arrives ... the execution component should learn the value of waiting rather than forecast the price and threshold it. The same argument applies to how the orchestrator itself is trained, since averaging over predicted states and averaging over the actions taken in those states are different objects." And on the orchestrator's output form: "The analogous move in my orchestrator is on the weight vector: a simplex constraint, non-negativity and any monotonicity I can establish belong in the architecture rather than in the loss as a penalty term." Protocol revision: "this goes into the evaluation design alongside the hard-router baseline from the SOPS note."</t>
         </is>
       </c>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Chen, Zhu, Liu and Li — first author at Cornell writing up an IBM Research internship, the rest at MIT-IBM Watson AI Lab, IBM Research and Three Bridges Capital. "Cost-Efficient Reinforcement Learning for Optimal Trade Execution on Dynamic Market Environment." ICAIF '22, pages 386-393.</t>
+          <t>Chen, Zhu, Liu and Li - first author at Cornell writing up an IBM Research internship, the rest at MIT-IBM Watson AI Lab, IBM Research and Three Bridges Capital. "Cost-Efficient Reinforcement Learning for Optimal Trade Execution on Dynamic Market Environment." ICAIF '22, pages 386-393.</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>none recorded in the note ("No code release is mentioned").</t>
+          <t>DOI 10.1145/3533271.3561761. No code release is mentioned in the note.</t>
         </is>
       </c>
       <c r="F35" s="11" t="inlineStr">
@@ -4900,12 +4900,12 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>US equities, liquid names — 7 stocks across six sectors "2 to 115 million shares per day." Deep, liquid books; calibration venue is IEX, "a venue with a small share of consolidated volume."</t>
+          <t>US equities, liquid names - 7 stocks across six sectors "2 to 115 million shares per day." Deep, liquid books; calibration venue is IEX, "a venue with a small share of consolidated volume."</t>
         </is>
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>IEX limit order book data, March to December 2020. Universe AAPL, HAL, HPQ, HSBC, PFE, SBUX, VZ. Time step 1 second, trade unit is level-1 average order size $\text{AOS}_1$. Episode $I=80$ units to liquidate, $T=16$ steps. Training 200,000 episodes, $\epsilon=0.3$, batch 64, Adam at $10^{-4}$, ~20 hours on one K40m. Metric mean and std over 1,000 test runs. Crucially: the market is generated, not replayed — "the market the agent trains and tests in is generated, not replayed."</t>
+          <t>IEX limit order book data, March to December 2020. Universe AAPL, HAL, HPQ, HSBC, PFE, SBUX, VZ. Time step 1 second, trade unit is level-1 average order size $\text{AOS}_1$. Episode $I=80$ units to liquidate, $T=16$ steps. Training 200,000 episodes, $\epsilon=0.3$, batch 64, Adam at $10^{-4}$, ~20 hours on one K40m. Metric mean and std over 1,000 test runs. Crucially: the market is generated, not replayed - "the market the agent trains and tests in is generated, not replayed."</t>
         </is>
       </c>
       <c r="J35" s="11" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>Dueling double DQN — "two three-layer fully connected networks of widths 512, 256, 128 producing $V(s)$ and $A(s,a)$ with the advantage head sized to the inventory," double-Q target, soft target update $\psi = (1-\tau)\psi + \tau\theta$ at $\tau=0.01$. Learnable environment model $M_\psi(s,a)$ is "a plain regression from twenty variables plus an action to twenty variables, a three-layer network trained under L2 loss on the same replay buffer" — it predicts only the market state, because agent-state transitions are deterministic and "the reward is not predicted at all, it is computed exactly from the current book and the chosen action." Rollouts are "strictly one step from a real state rather than a full synthetic episode, which caps error accumulation at a single transition." Reward: $$R(s,a) = \big(r(s,a) - p_D \cdot a\big)/p_D$$ with $\gamma = 1$. State-balanced exploration: under uniform sampling $\mathbb{E}[a_t] = I/2^{t+1}$, $\mathbb{E}[\text{rest}\_I_t] = I/2^{t}$; the fix draws $T$ distinct integers uniformly from $\{1,\ldots,I+T\}$, sorts them $z_1&lt;\cdots&lt;z_T$, sets $z_0=0$, $z_{T+1}=I+T+1$, and takes $$a_t = z_{t+1} - z_t - 1, \qquad \sum_{t=0}^{T} a_t = I$$ "which by the stars-and-bars bijection makes every valid execution plan equally likely" (Proposition 4.1). Output: a liquidation schedule, market orders only, $a \in \{0,1,\ldots,\text{rest}\_I\}$.</t>
+          <t>Dueling double DQN - "two three-layer fully connected networks of widths 512, 256, 128 producing $V(s)$ and $A(s,a)$ with the advantage head sized to the inventory," double-Q target, soft target update $\psi = (1-\tau)\psi + \tau\theta$ at $\tau=0.01$. Learnable environment model $M_\psi(s,a)$ is "a plain regression from twenty variables plus an action to twenty variables, a three-layer network trained under L2 loss on the same replay buffer" - it predicts only the market state, because agent-state transitions are deterministic and "the reward is not predicted at all, it is computed exactly from the current book and the chosen action." Rollouts are "strictly one step from a real state rather than a full synthetic episode, which caps error accumulation at a single transition." Reward: $$R(s,a) = \big(r(s,a) - p_D \cdot a\big)/p_D$$ with $\gamma = 1$. State-balanced exploration: under uniform sampling $\mathbb{E}[a_t] = I/2^{t+1}$, $\mathbb{E}[\text{rest}\_I_t] = I/2^{t}$; the fix draws $T$ distinct integers uniformly from $\{1,\ldots,I+T\}$, sorts them $z_1&lt;\cdots&lt;z_T$, sets $z_0=0$, $z_{T+1}=I+T+1$, and takes $$a_t = z_{t+1} - z_t - 1, \qquad \sum_{t=0}^{T} a_t = I$$ "which by the stars-and-bars bijection makes every valid execution plan equally likely" (Proposition 4.1). Output: a liquidation schedule, market orders only, $a \in \{0,1,\ldots,\text{rest}\_I\}$.</t>
         </is>
       </c>
       <c r="L35" s="11" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="O35" s="11" t="inlineStr">
         <is>
-          <t>Volatility is one of the 20 market state variables. Otherwise nothing: "The objective has no risk term at all. The reward is pure expected relative cost with $\gamma=1$, so the agent is indifferent between a schedule that reliably costs 15 bps and one that costs 5 or 25 with equal probability, which is exactly the trade-off the Almgren and Chriss framework exists to express and which the paper cites in passing without incorporating." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's core, and it is an LOB-based reactive execution simulator, not a parametric impact formula. There is NO Almgren-Chriss, NO square-root law, NO linear impact coefficient. Instead impact is *endogenous and mechanistic*: "Queue-reactive virtual market following Huang et al. (2015), queues as continuous-time Markov jump processes." Mechanism verbatim: "Queue length at each level moves as a jump process whose up-rate is the intensity of new limit orders and whose down-rate is the intensity of market orders plus cancellations, with both intensities estimated as functions of current queue size from historical books. The mid-price moves only when the best bid or best ask queue depletes to zero, and levels shift when opposite-side limit orders are inserted. So an agent that sends a market order consumes queue, brings a level closer to depletion, and makes an adverse mid-price move more likely on the next step, which is impact emerging from the mechanism rather than being charged as a fee." Calibration: order-arrival, market-order and cancellation intensities as functions of queue size at each level, estimated from IEX LOB data March-Dec 2020. Cost measurement: $\text{ATC} = (\text{average selling price} - p_D)/p_D$ in basis points, "negative by construction when liquidating, because pushing size into the book walks the price down." Spread: implicitly paid in full on every order — "Restricting the action space to marketable orders ... means the policy can only ever pay the spread, never earn it." Queue position: modelled in the *environment* (queue lengths and depletion) but the agent has no queue position of its own, since it posts no limit orders. Partial fills: none — "Market orders only, no queue position, no fees, no partial fills." Fees/commissions: none. Order-size dependence: present through the mechanism (larger $a$ consumes more queue) but never swept — "Everything runs at $I=80$ and $T=16$, with no sweep over inventory or participation rate even though impact is the subject and impact scales with size, so nothing tells me whether the advantage over TWAP grows, shrinks or inverts as the order gets larger relative to depth."</t>
+          <t>Volatility is one of the 20 market state variables. Otherwise nothing: "The objective has no risk term at all. The reward is pure expected relative cost with $\gamma=1$, so the agent is indifferent between a schedule that reliably costs 15 bps and one that costs 5 or 25 with equal probability, which is exactly the trade-off the Almgren and Chriss framework exists to express and which the paper cites in passing without incorporating." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's core, and it is an LOB-based reactive execution simulator, not a parametric impact formula. There is NO Almgren-Chriss, NO square-root law, NO linear impact coefficient. Instead impact is *endogenous and mechanistic*: "Queue-reactive virtual market following Huang et al. (2015), queues as continuous-time Markov jump processes." Mechanism verbatim: "Queue length at each level moves as a jump process whose up-rate is the intensity of new limit orders and whose down-rate is the intensity of market orders plus cancellations, with both intensities estimated as functions of current queue size from historical books. The mid-price moves only when the best bid or best ask queue depletes to zero, and levels shift when opposite-side limit orders are inserted. So an agent that sends a market order consumes queue, brings a level closer to depletion, and makes an adverse mid-price move more likely on the next step, which is impact emerging from the mechanism rather than being charged as a fee." Calibration: order-arrival, market-order and cancellation intensities as functions of queue size at each level, estimated from IEX LOB data March-Dec 2020. Cost measurement: $\text{ATC} = (\text{average selling price} - p_D)/p_D$ in basis points, "negative by construction when liquidating, because pushing size into the book walks the price down." Spread: implicitly paid in full on every order - "Restricting the action space to marketable orders ... means the policy can only ever pay the spread, never earn it." Queue position: modelled in the *environment* (queue lengths and depletion) but the agent has no queue position of its own, since it posts no limit orders. Partial fills: none - "Market orders only, no queue position, no fees, no partial fills." Fees/commissions: none. Order-size dependence: present through the mechanism (larger $a$ consumes more queue) but never swept - "Everything runs at $I=80$ and $T=16$, with no sweep over inventory or participation rate even though impact is the subject and impact scales with size, so nothing tells me whether the advantage over TWAP grows, shrinks or inverts as the order gets larger relative to depth."</t>
         </is>
       </c>
       <c r="P35" s="11" t="inlineStr">
@@ -4975,9 +4975,9 @@
       </c>
       <c r="W35" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: friction-aware evaluation layer (primary — ATC metric, baseline set, impact-cost evidence), A_L (the 16-level depth + total LOB volume + volatility state is "what $A_L$ would ideally consume"), orchestrator (exploration distribution over the constrained weight simplex; fixed coarse decision cadence).
-EFFECT ON MAIN GAP / SUB-GAP 2: Main gap — two transferable design constraints, both quoted by the note: the exploration-distribution lesson ("The stars-and-bars sampler is the discrete version of drawing from a flat Dirichlet, and the lesson I am taking is that the exploration distribution over the constrained object should be designed deliberately, not inherited from whatever the RL library does by default") and the cadence lesson (event-triggered reweighting demoted to an ablation). Sub-gap 2 — none; volatility is a state variable only, no long memory, no risk guardrail.
-EFFECT ON SUB-GAP 1: NARROWS IT SUBSTANTIALLY — this paper DOES implement an LOB-based reactive execution simulator in which cost is endogenously a function of order size against available depth. It is not Almgren-Chriss and not square-root; it is a queue-reactive Markov-jump LOB model (Huang et al. 2015) calibrated to real IEX books, where consuming queue raises the probability of adverse mid-price movement. So the *conceptual* claim that execution cost should be state-dependent on size-vs-depth is already implemented and quantified: "Ignoring market impact during training costs 3.04 basis points on average, on seven liquid US names." What survives is the *calibration-to-a-thin-market* half and the *size-sweep* half. The note is explicit on both: "Everything runs at $I=80$ and $T=16$, with no sweep over inventory or participation rate even though impact is the subject and impact scales with size, so nothing tells me whether the advantage over TWAP grows, shrinks or inverts as the order gets larger relative to depth." And the data prerequisite is exactly the CSE blocker: the simulator "is almost certainly out of reach on the CSE ... Whether the CSE exposes anything below top-of-book is still unconfirmed."
+          <t>SPEAKS TO: friction-aware evaluation layer (primary - ATC metric, baseline set, impact-cost evidence), A_L (the 16-level depth + total LOB volume + volatility state is "what $A_L$ would ideally consume"), orchestrator (exploration distribution over the constrained weight simplex; fixed coarse decision cadence).
+EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - two transferable design constraints, both quoted by the note: the exploration-distribution lesson ("The stars-and-bars sampler is the discrete version of drawing from a flat Dirichlet, and the lesson I am taking is that the exploration distribution over the constrained object should be designed deliberately, not inherited from whatever the RL library does by default") and the cadence lesson (event-triggered reweighting demoted to an ablation). Sub-gap 2 - none; volatility is a state variable only, no long memory, no risk guardrail.
+EFFECT ON SUB-GAP 1: NARROWS IT SUBSTANTIALLY - this paper DOES implement an LOB-based reactive execution simulator in which cost is endogenously a function of order size against available depth. It is not Almgren-Chriss and not square-root; it is a queue-reactive Markov-jump LOB model (Huang et al. 2015) calibrated to real IEX books, where consuming queue raises the probability of adverse mid-price movement. So the *conceptual* claim that execution cost should be state-dependent on size-vs-depth is already implemented and quantified: "Ignoring market impact during training costs 3.04 basis points on average, on seven liquid US names." What survives is the *calibration-to-a-thin-market* half and the *size-sweep* half. The note is explicit on both: "Everything runs at $I=80$ and $T=16$, with no sweep over inventory or participation rate even though impact is the subject and impact scales with size, so nothing tells me whether the advantage over TWAP grows, shrinks or inverts as the order gets larger relative to depth." And the data prerequisite is exactly the CSE blocker: the simulator "is almost certainly out of reach on the CSE ... Whether the CSE exposes anything below top-of-book is still unconfirmed."
 PROPOSED REVISION STATED IN THE NOTE: Three, quoted. On $A_L$ and its data dependency: "The same data gap constrains the liquidity agent, and that link is worth making explicit in the design. The market state here is raw depth at sixteen levels plus volatility and total volume, which is what $A_L$ would ideally consume, and if none of it is observable then the liquidity agent falls back to turnover, traded-value, zero-return frequency and Amihud-style illiquidity measures built from daily bars. The useful observation is that the evaluation layer and the liquidity agent are gated on exactly the same data, so whatever I cannot observe I also cannot simulate ... That argues for treating them as one workstream rather than two." On the orchestrator's weight sampling: "Whenever the action space shrinks as an episode progresses, naive random exploration front-loads and the later states go unvisited, which applies to any execution scheduler I add and also, in a different form, to sampling the orchestrator's weight vector, where independent uniform draws per agent concentrate mass in the middle of the simplex rather than covering it." On cadence: "I would rather fix the cadence, show it works, and treat event-triggered reweighting as an ablation to run once rather than a design assumption to build on."</t>
         </is>
       </c>
@@ -5010,7 +5010,7 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>none recorded in the note beyond "open access" ("No code release is mentioned").</t>
+          <t>DOI 10.1007/s00780-026-00589-5. Open access. No code release is mentioned in the note.</t>
         </is>
       </c>
       <c r="F36" s="11" t="inlineStr">
@@ -5030,17 +5030,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Simulation study — AC simulator with known ground truth, $S_0=100$, $q_0 = 5\times10^5$, $\kappa = 2.5\times10^{-7}$, $\eta = 2.5\times10^{-6}$, $\sigma = 30\%$, $T=1$ day. Empirical study — HD simulator (LOBSTER historical order flow) and CST simulator (Cont-Stoikov-Talreja stochastic order book); 7 Nasdaq stocks, 6 sectors, Jul 2016 to Mar 2017; $T=1$ day, 6 hours from 10:00. Discretisation $N=100$, $n=15$ Gauss-Hermite nodes, $L=500$ iterations. Protocol: 100 independent runs in simulation; rolling quarters empirically — "train 2016Q3 test 2016Q4, train 2016Q4 test 2017Q1." Risk aversion at three levels $\lambda^{\text{low}} = \eta$, $\lambda^{\text{mid}} = 10^3\eta$, $\lambda^{\text{high}} = 10^4\eta$. Comparators SAC (depth 1-2, width 128-256) and STAT (estimate-then-plug-in), plus TWAP as the reporting reference.</t>
+          <t>Simulation study - AC simulator with known ground truth, $S_0=100$, $q_0 = 5\times10^5$, $\kappa = 2.5\times10^{-7}$, $\eta = 2.5\times10^{-6}$, $\sigma = 30\%$, $T=1$ day. Empirical study - HD simulator (LOBSTER historical order flow) and CST simulator (Cont-Stoikov-Talreja stochastic order book); 7 Nasdaq stocks, 6 sectors, Jul 2016 to Mar 2017; $T=1$ day, 6 hours from 10:00. Discretisation $N=100$, $n=15$ Gauss-Hermite nodes, $L=500$ iterations. Protocol: 100 independent runs in simulation; rolling quarters empirically - "train 2016Q3 test 2016Q4, train 2016Q4 test 2017Q1." Risk aversion at three levels $\lambda^{\text{low}} = \eta$, $\lambda^{\text{mid}} = 10^3\eta$, $\lambda^{\text{high}} = 10^4\eta$. Comparators SAC (depth 1-2, width 128-256) and STAT (estimate-then-plug-in), plus TWAP as the reporting reference.</t>
         </is>
       </c>
       <c r="J36" s="11" t="inlineStr">
         <is>
-          <t>Order-flow / LOB for the simulators; the *policy* itself consumes only $(t, q)$ — time remaining and inventory. No text, no fundamentals, no depth or imbalance features enter the control.</t>
+          <t>Order-flow / LOB for the simulators; the *policy* itself consumes only $(t, q)$ - time remaining and inventory. No text, no fundamentals, no depth or imbalance features enter the control.</t>
         </is>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>EMQV objective: $$\sup_{\boldsymbol{\pi}\in\Pi}\ \mathbb{E}\Big[\int_0^T\!\!\int_{\mathbb{R}}\big(-\nu(S_t^{\boldsymbol\pi}+\eta\nu)-\lambda\sigma^2S_0^2(q_t^{\boldsymbol\pi})^2-\zeta\ln\boldsymbol\pi_t(\nu)\big)\boldsymbol\pi_t(\nu)\,d\nu\,dt + h_T(q_T^{\boldsymbol\pi},S_T^{\boldsymbol\pi})\Big]$$ with $h_T = 0$ at zero inventory and $-\infty$ otherwise, forcing exact liquidation. Closed-form optimal exploratory policy is Gaussian: $$\boldsymbol\pi^*(\nu;t,q,S) = d_{\mathcal{N}}\Big(\nu;\ -qK\coth\big(K(T-t)\big),\ \frac{\zeta}{2\eta}\Big), \qquad K = \sqrt{\frac{\lambda\sigma^2S_0^2}{\eta}}$$ — "exploration variance is proportional to the temperature and inversely proportional to the temporary impact parameter, which matches the intuition that in a market where trading fast is expensive you should sample less aggressively around your intended rate." Letting $\zeta \downarrow 0$ recovers classical Almgren-Chriss exactly. Parametrisation: $\boldsymbol\pi^\Phi = d_{\mathcal{N}}(\nu; -q\varphi_1\coth(\varphi_1(T-t)), \zeta\varphi_2)$ with $\varphi_1^* = \sqrt{\lambda\sigma^2 S_0^2/\eta_{\text{env}}}$ and $\varphi_2^* = 1/(2\eta_{\text{env}})$, plus a three-parameter value function $\Theta=(\theta_1,\theta_2,\theta_3)$ — "Five scalars total, against a SAC implementation carrying several networks of width 128 to 256." Recalibration step: $$\Theta^{(\ell+1)} = M(\Phi^{(\ell+1)})M(\Phi^{(\ell)})^{-1}\widetilde\Theta^{(\ell)}$$ costing one matrix product per iteration and guaranteeing the policy evaluation error shrinks by $d(\ell)\in(0,1-\varepsilon)$. Exploratory revenue collected by 15-node Gauss-Hermite quadrature with environment resets between nodes.</t>
+          <t>EMQV objective: $$\sup_{\boldsymbol{\pi}\in\Pi}\ \mathbb{E}\Big[\int_0^T\!\!\int_{\mathbb{R}}\big(-\nu(S_t^{\boldsymbol\pi}+\eta\nu)-\lambda\sigma^2S_0^2(q_t^{\boldsymbol\pi})^2-\zeta\ln\boldsymbol\pi_t(\nu)\big)\boldsymbol\pi_t(\nu)\,d\nu\,dt + h_T(q_T^{\boldsymbol\pi},S_T^{\boldsymbol\pi})\Big]$$ with $h_T = 0$ at zero inventory and $-\infty$ otherwise, forcing exact liquidation. Closed-form optimal exploratory policy is Gaussian: $$\boldsymbol\pi^*(\nu;t,q,S) = d_{\mathcal{N}}\Big(\nu;\ -qK\coth\big(K(T-t)\big),\ \frac{\zeta}{2\eta}\Big), \qquad K = \sqrt{\frac{\lambda\sigma^2S_0^2}{\eta}}$$ - "exploration variance is proportional to the temperature and inversely proportional to the temporary impact parameter, which matches the intuition that in a market where trading fast is expensive you should sample less aggressively around your intended rate." Letting $\zeta \downarrow 0$ recovers classical Almgren-Chriss exactly. Parametrisation: $\boldsymbol\pi^\Phi = d_{\mathcal{N}}(\nu; -q\varphi_1\coth(\varphi_1(T-t)), \zeta\varphi_2)$ with $\varphi_1^* = \sqrt{\lambda\sigma^2 S_0^2/\eta_{\text{env}}}$ and $\varphi_2^* = 1/(2\eta_{\text{env}})$, plus a three-parameter value function $\Theta=(\theta_1,\theta_2,\theta_3)$ - "Five scalars total, against a SAC implementation carrying several networks of width 128 to 256." Recalibration step: $$\Theta^{(\ell+1)} = M(\Phi^{(\ell+1)})M(\Phi^{(\ell)})^{-1}\widetilde\Theta^{(\ell)}$$ costing one matrix product per iteration and guaranteeing the policy evaluation error shrinks by $d(\ell)\in(0,1-\varepsilon)$. Exploratory revenue collected by 15-node Gauss-Hermite quadrature with environment resets between nodes.</t>
         </is>
       </c>
       <c r="L36" s="11" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>The strongest of the three execution papers. Risk is the quadratic variation of the mark-to-market portfolio value, $\mathbb{E}[\langle P^\nu \rangle_T] = \mathbb{E}[\int_0^T \sigma^2 S_0^2 (q_t^\nu)^2 dt]$, "which charges risk continuously in proportion to squared inventory held." The note's framing: "Almgren and Chriss use a mean-variance objective measuring risk only at the end of the horizon, which is famously time-inconsistent ... Under arithmetic Brownian motion the resulting optimal inventory trajectory is identical to the mean-variance one, so nothing is lost in the classical solution, and the dynamic programming problem becomes time-consistent, which is what allows an RL agent to learn one stationary feedback policy rather than a schedule committed to at $t=0$." Volatility itself is constant $\sigma$ under ABM — no stochastic vol, no long memory. Risk aversion $\lambda$ is swept across three levels. LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This paper DOES implement Almgren-Chriss impact explicitly, and it implements an LOB-based execution simulator for evaluation. Impact form: linear permanent impact $\kappa$ and linear temporary impact $\eta$ — the running revenue term is $-\nu(S_t + \eta\nu)$, i.e. temporary cost quadratic in the trading rate, so *cost per share is linear in order size*. Not square-root, not concave. Calibration: in simulation $\kappa = 2.5\times10^{-7}$, $\eta = 2.5\times10^{-6}$ set exogenously with known ground truth; empirically the environment parameters $\psi = (\kappa, \eta, \sigma^2)$ are never estimated directly by EMQV but "recovered by inverting a $3\times3$ matrix $M(\Phi)$ linking $\Theta$ to $\psi$" — i.e. *implied* from the learned critic rather than statistically estimated. The STAT comparator does estimate them statistically, "re-estimated for every test day using the five preceding days." The HD simulator is a genuine LOB matching-engine simulator with permanent state contamination: "It replays historical LOBSTER order flow into a reconstructed book, injects the agent's market order, and lets the exchange matching rules carry the consequences forward, so a sell order consuming 100 shares at 104 and 150 at 103 not only pays temporary impact on that fill but permanently changes every subsequent book state, since a historical cancellation of 200 shares at 103 now finds only 50 left to cancel. Impact is simulated in training and in testing, which the authors contrast with Nevmyvaka et al., who simulate it only at test time." CST simulator is a stochastic order book model. Spread: none in the model — "no spread, no depth, no order imbalance, no intraday seasonality." Queue: none. Partial fills: none. Fees: none. Terminal liquidation: "after discretisation the zero-inventory target is not met by the policy itself, so the implementation simply trades all remaining shares at $t_{N-1}$, which is a forced market order of unmanaged size." Participation rate fixed at 10% of ADTV with "no sweep over order size even though impact is the subject and impact scales with size."</t>
+          <t>The strongest of the three execution papers. Risk is the quadratic variation of the mark-to-market portfolio value, $\mathbb{E}[\langle P^\nu \rangle_T] = \mathbb{E}[\int_0^T \sigma^2 S_0^2 (q_t^\nu)^2 dt]$, "which charges risk continuously in proportion to squared inventory held." The note's framing: "Almgren and Chriss use a mean-variance objective measuring risk only at the end of the horizon, which is famously time-inconsistent ... Under arithmetic Brownian motion the resulting optimal inventory trajectory is identical to the mean-variance one, so nothing is lost in the classical solution, and the dynamic programming problem becomes time-consistent, which is what allows an RL agent to learn one stationary feedback policy rather than a schedule committed to at $t=0$." Volatility itself is constant $\sigma$ under ABM - no stochastic vol, no long memory. Risk aversion $\lambda$ is swept across three levels. LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This paper DOES implement Almgren-Chriss impact explicitly, and it implements an LOB-based execution simulator for evaluation. Impact form: linear permanent impact $\kappa$ and linear temporary impact $\eta$ - the running revenue term is $-\nu(S_t + \eta\nu)$, i.e. temporary cost quadratic in the trading rate, so *cost per share is linear in order size*. Not square-root, not concave. Calibration: in simulation $\kappa = 2.5\times10^{-7}$, $\eta = 2.5\times10^{-6}$ set exogenously with known ground truth; empirically the environment parameters $\psi = (\kappa, \eta, \sigma^2)$ are never estimated directly by EMQV but "recovered by inverting a $3\times3$ matrix $M(\Phi)$ linking $\Theta$ to $\psi$" - i.e. *implied* from the learned critic rather than statistically estimated. The STAT comparator does estimate them statistically, "re-estimated for every test day using the five preceding days." The HD simulator is a genuine LOB matching-engine simulator with permanent state contamination: "It replays historical LOBSTER order flow into a reconstructed book, injects the agent's market order, and lets the exchange matching rules carry the consequences forward, so a sell order consuming 100 shares at 104 and 150 at 103 not only pays temporary impact on that fill but permanently changes every subsequent book state, since a historical cancellation of 200 shares at 103 now finds only 50 left to cancel. Impact is simulated in training and in testing, which the authors contrast with Nevmyvaka et al., who simulate it only at test time." CST simulator is a stochastic order book model. Spread: none in the model - "no spread, no depth, no order imbalance, no intraday seasonality." Queue: none. Partial fills: none. Fees: none. Terminal liquidation: "after discretisation the zero-inventory target is not met by the policy itself, so the implementation simply trades all remaining shares at $t_{N-1}$, which is a forced market order of unmanaged size." Participation rate fixed at 10% of ADTV with "no sweep over order size even though impact is the subject and impact scales with size."</t>
         </is>
       </c>
       <c r="P36" s="11" t="inlineStr">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="Q36" s="11" t="inlineStr">
         <is>
-          <t>High by construction and this is a stated selling point — five interpretable scalars with known optimal values, versus neural policies that are "uninterpretable" and carry "no convergence guarantee in general." The finite-time error bound (Theorem 5.13, 5.15) and the bracketing of convergence behaviour are the formal-transparency contribution.</t>
+          <t>High by construction and this is a stated selling point - five interpretable scalars with known optimal values, versus neural policies that are "uninterpretable" and carry "no convergence guarantee in general." The finite-time error bound (Theorem 5.13, 5.15) and the bracketing of convergence behaviour are the formal-transparency contribution.</t>
         </is>
       </c>
       <c r="R36" s="11" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="S36" s="11" t="inlineStr">
         <is>
-          <t>Recalibration ablation — "recalibration takes the standard deviation of the learned $\varphi_1$ from 43.57 down to 1.17, a factor of 37, while the value function parameters barely move, $\theta_1$ at $1.64\times10^{-10}$ against $1.50\times10^{-10}$." Exploratory-vs-sample state — "$\varphi_1$ standard deviations of 1.67 and 1.82 at medium and high risk aversion against 167.60 and 307.54." AC simulator gaps in bps — "$-9.881\times10^{-10}$, $-1.022\times10^{-3}$ and $-3.075\times10^{-4}$ for EMQV at low, medium and high risk aversion, against $-19.311$, $-113.647$ and $-109.405$ for the best depth and width configuration of SAC." Out of sample — "Across 21 stock and risk-aversion combinations, EMQV is the best performer in 9 and SAC in 10, which is not the ordering the abstract's 'stands out as the best overall' would suggest on its own ... SAC underperforms TWAP in 11 of 21 cases regardless of which simulator trained it, and its standard errors are enormous, AAPL at high risk aversion coming in at $-1.73\times10^5$ with a standard error of 18,323 on the CST simulator." STAT degradation — "at high risk aversion turns in $-905.742$ on AAPL and $-203.392$ on MSFT against EMQV's $+102.285$ and $+85.983$ on the historical simulator." Low risk aversion — "several entries being $-0.020$ to $+0.046$ basis points, because TWAP is nearly optimal for a risk-neutral agent." LIMITATIONS (quoted): (1) "The parametrisation cannot express anything the Almgren-Chriss model cannot, and every advantage in the paper traces back to that. Linear permanent impact, linear temporary impact, arithmetic Brownian motion with constant volatility, no spread, no depth, no order imbalance, no intraday seasonality in any of them ... The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong, which is precisely the situation a thin frontier order book creates." (2) "The convergence guarantee is real but not operational ... the guarantee is conditional on a box whose right size is unknown ... the theorem covers a different algorithm from the one in the experiments." (3) "Exploration requires rewinding the market, which no live venue permits ... the configuration carrying the headline results is simulator-only and the deployable one is the weaker of the two." (4) "Market orders only, no spread, no queue, no fees, and the last step dumps whatever is left ... This is the same restriction as in the queue-reactive paper and it bites harder in a wide-spread market." (5) "Seven large-cap Nasdaq names, two test quarters, one horizon, one participation rate ... The paper's argument that EMQV is more robust to distribution shift than STAT rests on a shift between adjacent quarters in a stable market, which is the mildest available version of that test." (6) "The comparison against SAC is not tuned symmetrically ... it means the empirical comparison establishes that SAC is harder to configure reliably rather than that it is worse."</t>
+          <t>Recalibration ablation - "recalibration takes the standard deviation of the learned $\varphi_1$ from 43.57 down to 1.17, a factor of 37, while the value function parameters barely move, $\theta_1$ at $1.64\times10^{-10}$ against $1.50\times10^{-10}$." Exploratory-vs-sample state - "$\varphi_1$ standard deviations of 1.67 and 1.82 at medium and high risk aversion against 167.60 and 307.54." AC simulator gaps in bps - "$-9.881\times10^{-10}$, $-1.022\times10^{-3}$ and $-3.075\times10^{-4}$ for EMQV at low, medium and high risk aversion, against $-19.311$, $-113.647$ and $-109.405$ for the best depth and width configuration of SAC." Out of sample - "Across 21 stock and risk-aversion combinations, EMQV is the best performer in 9 and SAC in 10, which is not the ordering the abstract's 'stands out as the best overall' would suggest on its own ... SAC underperforms TWAP in 11 of 21 cases regardless of which simulator trained it, and its standard errors are enormous, AAPL at high risk aversion coming in at $-1.73\times10^5$ with a standard error of 18,323 on the CST simulator." STAT degradation - "at high risk aversion turns in $-905.742$ on AAPL and $-203.392$ on MSFT against EMQV's $+102.285$ and $+85.983$ on the historical simulator." Low risk aversion - "several entries being $-0.020$ to $+0.046$ basis points, because TWAP is nearly optimal for a risk-neutral agent." LIMITATIONS (quoted): (1) "The parametrisation cannot express anything the Almgren-Chriss model cannot, and every advantage in the paper traces back to that. Linear permanent impact, linear temporary impact, arithmetic Brownian motion with constant volatility, no spread, no depth, no order imbalance, no intraday seasonality in any of them ... The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong, which is precisely the situation a thin frontier order book creates." (2) "The convergence guarantee is real but not operational ... the guarantee is conditional on a box whose right size is unknown ... the theorem covers a different algorithm from the one in the experiments." (3) "Exploration requires rewinding the market, which no live venue permits ... the configuration carrying the headline results is simulator-only and the deployable one is the weaker of the two." (4) "Market orders only, no spread, no queue, no fees, and the last step dumps whatever is left ... This is the same restriction as in the queue-reactive paper and it bites harder in a wide-spread market." (5) "Seven large-cap Nasdaq names, two test quarters, one horizon, one participation rate ... The paper's argument that EMQV is more robust to distribution shift than STAT rests on a shift between adjacent quarters in a stable market, which is the mildest available version of that test." (6) "The comparison against SAC is not tuned symmetrically ... it means the empirical comparison establishes that SAC is harder to configure reliably rather than that it is worse."</t>
         </is>
       </c>
       <c r="T36" s="11" t="inlineStr">
@@ -5101,8 +5101,8 @@
       <c r="W36" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: friction-aware evaluation layer (primary), A_V (the QV risk charge $\lambda\sigma^2S_0^2 q_t^2$ is the cleanest available risk-adjusted execution objective and the note explicitly imports it because "neither of the other two execution notes carries a risk term"), orchestrator (recalibration as an actor-critic design discipline; residual-RL as the composition template).
-EFFECT ON MAIN GAP / SUB-GAP 2: Main gap — a direct architectural contribution, quoted below. Sub-gap 2 — partial and indirect: it supplies the *form* of a live risk guardrail (a running charge proportional to squared inventory held, time-consistent, $\lambda$ swept as a reported axis) but volatility is constant ABM, so nothing on long memory or FIGARCH $d$. The transferable piece is that a risk term belongs inside the execution objective and that $\lambda$ should be a reported axis rather than a tuned hyperparameter.
-EFFECT ON SUB-GAP 1: NARROWS IT SHARPLY ON THE MODELLING SIDE — this paper explicitly implements Almgren-Chriss impact (linear permanent $\kappa$, linear temporary $\eta$), solves it in closed form, AND evaluates inside an LOB-based historical-order-flow execution simulator with permanent book contamination. So "execution cost is a function of order size" is fully implemented here — but *linearly*, and the state it depends on is $(t,q)$, not depth. What survives, and the note says so in red: "The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong, which is precisely the situation a thin frontier order book creates." Also surviving: no order-size sweep ("no sweep over order size even though impact is the subject and impact scales with size"); no spread, no depth, no queue in the cost model; and no calibration to anything but large-cap Nasdaq. The note's own summary of the three-paper bracket: "The other two notes bracket the problem, impact assumed away and impact learned model-free, and this paper takes the middle route: write the impact model down, solve it, learn only the handful of numbers the solution needs ... this is a starting point to extend rather than a method to adopt wholesale."
+EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - a direct architectural contribution, quoted below. Sub-gap 2 - partial and indirect: it supplies the *form* of a live risk guardrail (a running charge proportional to squared inventory held, time-consistent, $\lambda$ swept as a reported axis) but volatility is constant ABM, so nothing on long memory or FIGARCH $d$. The transferable piece is that a risk term belongs inside the execution objective and that $\lambda$ should be a reported axis rather than a tuned hyperparameter.
+EFFECT ON SUB-GAP 1: NARROWS IT SHARPLY ON THE MODELLING SIDE - this paper explicitly implements Almgren-Chriss impact (linear permanent $\kappa$, linear temporary $\eta$), solves it in closed form, AND evaluates inside an LOB-based historical-order-flow execution simulator with permanent book contamination. So "execution cost is a function of order size" is fully implemented here - but *linearly*, and the state it depends on is $(t,q)$, not depth. What survives, and the note says so in red: "The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong, which is precisely the situation a thin frontier order book creates." Also surviving: no order-size sweep ("no sweep over order size even though impact is the subject and impact scales with size"); no spread, no depth, no queue in the cost model; and no calibration to anything but large-cap Nasdaq. The note's own summary of the three-paper bracket: "The other two notes bracket the problem, impact assumed away and impact learned model-free, and this paper takes the middle route: write the impact model down, solve it, learn only the handful of numbers the solution needs ... this is a starting point to extend rather than a method to adopt wholesale."
 PROPOSED REVISION STATED IN THE NOTE: Yes, an orchestrator revision, verbatim: "The recalibration idea generalises directly to my orchestrator, and I should design for it rather than discover the need later. The structural condition is that the critic's parametrisation depends on the actor's parameters through a known map, which is exactly what happens if the orchestrator's value function is written in terms of the agent weights it emits. When that holds, resetting the critic in lockstep after every actor update costs one matrix product and, on this evidence, is the difference between converging and oscillating. The design implication is to keep the link between the two parametrisations explicit and invertible instead of treating actor and critic as independent black boxes." And an agent-pool/architecture revision: "The residual-RL suggestion in the discussion is the template for combining a defensible baseline with a learned component. Treating the analytically derived policy as a baseline control and learning a residual on top of it with a flexible algorithm gives a floor that cannot be worse than the model-based solution by much, and a mechanism for the learner to exploit anything the model misses, such as depth or imbalance if the CSE ever exposes it ... it is a cleaner way to add a learned execution component to the orchestrator than starting from a blank policy network." Plus an objective revision: "Adopt the QV-adjusted PnL as the execution objective, because neither of the other two execution notes carries a risk term."</t>
         </is>
       </c>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>none recorded in the note ("No code release is mentioned").</t>
+          <t>DOI 10.1016/j.ejor.2023.05.001. No code release is mentioned in the note.</t>
         </is>
       </c>
       <c r="F37" s="11" t="inlineStr">
@@ -5150,7 +5150,7 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Developed-market equity indices/benchmark OLPS sets — MSCI, NYSE, TSE, NASDAQ. All liquid; the note observes the cost rate used, $\delta = 0.05\%$, is a developed-market commission assumption, against "a CSE-plausible round-trip rate of 1%."</t>
+          <t>Developed-market equity indices/benchmark OLPS sets - MSCI, NYSE, TSE, NASDAQ. All liquid; the note observes the cost rate used, $\delta = 0.05\%$, is a developed-market commission assumption, against "a CSE-plausible round-trip rate of 1%."</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="L37" s="11" t="inlineStr">
         <is>
-          <t>No learned agents, but this is the paper's structural relevance — "SOPS is a hard binary router between two objectives conditioned on a count of assets in a detected state, which is the degenerate case of the orchestrator I am proposing, and it is prior art that sits closer to my main gap than the equal-weight baseline does." Note the caveat on what "state" means here: "There is no Markov switching, no latent variable and no probability distribution over states anywhere in the paper."</t>
+          <t>No learned agents, but this is the paper's structural relevance - "SOPS is a hard binary router between two objectives conditioned on a count of assets in a detected state, which is the degenerate case of the orchestrator I am proposing, and it is prior art that sits closer to my main gap than the equal-weight baseline does." Note the caveat on what "state" means here: "There is no Markov switching, no latent variable and no probability distribution over states anywhere in the paper."</t>
         </is>
       </c>
       <c r="M37" s="11" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>Volatility enters twice — as the per-segment $\nu_l^{(i)}$ used in the state-labelling regression $\mu = \alpha\nu + \beta$, and as $\Sigma_t$ in the NPMRP quadratic penalty with a log-barrier $-c\sum\ln x_i$. No long memory, no GARCH, no conditional volatility model. The risk parity claim does not hold up: "On the 1004th trading day SOPS holds Stock 6, Stock 16 and Stock 23 at weights of 60.80%, 4.54% and 34.66%, with risk contributions of 0.0117, 0.0008 and 0.0081, a factor of roughly fourteen between the largest and smallest. At $\eta = 0.0001$ the penalty is close to inert." Also flagged: the paper's "Calmar ratio" is actually a Sortino ratio, so "no drawdown measure appears anywhere in the paper." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): Exact accounting of the wrong functional form. Cost model is linear, proportional and symmetric: a single scalar rate $\delta \in (0,1)$ "for both buying and selling," identical across assets and independent of size. The one sophistication is the self-referential fee-on-post-cost-weights formulation — the difference is taken as $|x_{ti}\omega_{t-1} - \tilde{x}_{(t-1)i}|$ rather than $|x_{ti} - \tilde{x}_{(t-1)i}|$, "which is what makes it exact and also what makes it circular." No impact function at all — no Almgren-Chriss, no square-root, no linear impact, no depth term. No spread, no queue, no partial fill, no volume constraint. Calibration: $\delta$ fixed at 0.05% for every experiment and never varied, which the note calls out as the paper's central omission: "A paper about exact transaction cost computation never varies the transaction cost rate ... Whether SOPS still beats the nineteen baselines at a frontier-market cost rate is exactly the question the paper's machinery is built to answer and exactly the experiment it does not run." Realised cost behaviour: "the per-period cost proportion sits at its ceiling of $1 \times 10^{-3}$ in most periods, and since that ceiling is exactly $2\delta$ under the linear cost model, the portfolio is fully turning over in those periods rather than trimming. Cumulative cost over the horizon reaches 0.7528 against a cumulative return of 14.8585, and 765 of the periods carry nonzero cost." The paper itself lists as future work "variable and concave costs and a market-impact term $\Delta r \propto \ln(\Delta x)$ from Potters and Bouchaud (2003)."</t>
+          <t>Volatility enters twice - as the per-segment $\nu_l^{(i)}$ used in the state-labelling regression $\mu = \alpha\nu + \beta$, and as $\Sigma_t$ in the NPMRP quadratic penalty with a log-barrier $-c\sum\ln x_i$. No long memory, no GARCH, no conditional volatility model. The risk parity claim does not hold up: "On the 1004th trading day SOPS holds Stock 6, Stock 16 and Stock 23 at weights of 60.80%, 4.54% and 34.66%, with risk contributions of 0.0117, 0.0008 and 0.0081, a factor of roughly fourteen between the largest and smallest. At $\eta = 0.0001$ the penalty is close to inert." Also flagged: the paper's "Calmar ratio" is actually a Sortino ratio, so "no drawdown measure appears anywhere in the paper." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): Exact accounting of the wrong functional form. Cost model is linear, proportional and symmetric: a single scalar rate $\delta \in (0,1)$ "for both buying and selling," identical across assets and independent of size. The one sophistication is the self-referential fee-on-post-cost-weights formulation - the difference is taken as $|x_{ti}\omega_{t-1} - \tilde{x}_{(t-1)i}|$ rather than $|x_{ti} - \tilde{x}_{(t-1)i}|$, "which is what makes it exact and also what makes it circular." No impact function at all - no Almgren-Chriss, no square-root, no linear impact, no depth term. No spread, no queue, no partial fill, no volume constraint. Calibration: $\delta$ fixed at 0.05% for every experiment and never varied, which the note calls out as the paper's central omission: "A paper about exact transaction cost computation never varies the transaction cost rate ... Whether SOPS still beats the nineteen baselines at a frontier-market cost rate is exactly the question the paper's machinery is built to answer and exactly the experiment it does not run." Realised cost behaviour: "the per-period cost proportion sits at its ceiling of $1 \times 10^{-3}$ in most periods, and since that ceiling is exactly $2\delta$ under the linear cost model, the portfolio is fully turning over in those periods rather than trimming. Cumulative cost over the horizon reaches 0.7528 against a cumulative return of 14.8585, and 765 of the periods carry nonzero cost." The paper itself lists as future work "variable and concave costs and a market-impact term $\Delta r \propto \ln(\Delta x)$ from Potters and Bouchaud (2003)."</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
@@ -5195,12 +5195,12 @@
       </c>
       <c r="Q37" s="11" t="inlineStr">
         <is>
-          <t>Structurally high — closed-form cost factor with a uniqueness proof, a legible two-parameter-per-asset state rule, a QP with an off-the-shelf solver, and honest reporting of realised risk contributions. But the routing itself is opaque in the diagnostic sense: "The paper reports no count of how many periods were classified bearish, no timeline of the switch, and no comparison against a random or fixed-schedule router firing at the same rate."</t>
+          <t>Structurally high - closed-form cost factor with a uniqueness proof, a legible two-parameter-per-asset state rule, a QP with an off-the-shelf solver, and honest reporting of realised risk contributions. But the routing itself is opaque in the diagnostic sense: "The paper reports no count of how many periods were classified bearish, no timeline of the switch, and no comparison against a random or fixed-schedule router firing at the same rate."</t>
         </is>
       </c>
       <c r="R37" s="11" t="inlineStr">
         <is>
-          <t>19 OLPS algorithms across all five families — UBAH, UCRP, BCRP, Anticor, CWMR, CORN, EG, ONS, OLMAR, PAMR, TCO, UP and others. Metrics: cumulative return, Sharpe, information ratio against UBAH, and the mislabelled "Calmar." One fixed run per dataset, no seeds, no significance tests.</t>
+          <t>19 OLPS algorithms across all five families - UBAH, UCRP, BCRP, Anticor, CWMR, CORN, EG, ONS, OLMAR, PAMR, TCO, UP and others. Metrics: cumulative return, Sharpe, information ratio against UBAH, and the mislabelled "Calmar." One fixed run per dataset, no seeds, no significance tests.</t>
         </is>
       </c>
       <c r="S37" s="11" t="inlineStr">
@@ -5225,9 +5225,9 @@
       </c>
       <c r="W37" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: friction-aware evaluation layer (primary — the TRF closed form and constant bounds go directly in), orchestrator (SOPS is the hard-router prior art and becomes a required baseline), A_V (log-barrier diversification penalty and the per-asset $\mu$-vs-$\nu$ state label).
-EFFECT ON MAIN GAP / SUB-GAP 2: Main gap — substantial. SOPS is "the degenerate case of the orchestrator I am proposing," a hard binary router on a count of per-asset states, and the note both adopts it as a baseline and uses its failure to diagnose router firing rate as the motivation for weight-entropy reporting. It also links to MacroHFT: "This is the same diagnostic problem as MacroHFT's near-binary learned mixture ... arriving from the opposite direction, and it is the specific thing my own weight-entropy reporting is meant to prevent." Sub-gap 2 — indirect and mostly as a cheaper competitor to FIGARCH: SEMA is "far cheaper than the FIGARCH route ... which matters because the only confirmed ready-made CSE set covers February 2025 to February 2026. With roughly 240 trading days and $w \approx 30$ that is 8 segments for a two-parameter regression, thin but not absurd." No long-memory content of its own.
-EFFECT ON SUB-GAP 1: LEAVES IT OPEN, and is the strongest illustration that it is open. Zero impact modelling: no Almgren-Chriss, no square-root, no LOB simulator, no depth anywhere. Cost is exactly the flat-rate-on-turnover model the sub-gap is aimed at, computed exactly. The note's own verdict, in red: "the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper." What this paper *does* contribute to closing sub-gap 1 is machinery rather than a model: the exact, provably unique transaction remainder factor with constant bounds $\frac{1-\delta}{1+\delta} \leq \omega_{t-1} \leq 1$, which "lets a cost term stay inside a convex objective rather than sitting outside it as a post-hoc deduction" — that is the container into which a state-dependent $\delta$ can be substituted. It also hands over the exact experiment the sub-gap needs: the $\delta$ sweep the authors skipped.
+          <t>SPEAKS TO: friction-aware evaluation layer (primary - the TRF closed form and constant bounds go directly in), orchestrator (SOPS is the hard-router prior art and becomes a required baseline), A_V (log-barrier diversification penalty and the per-asset $\mu$-vs-$\nu$ state label).
+EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - substantial. SOPS is "the degenerate case of the orchestrator I am proposing," a hard binary router on a count of per-asset states, and the note both adopts it as a baseline and uses its failure to diagnose router firing rate as the motivation for weight-entropy reporting. It also links to MacroHFT: "This is the same diagnostic problem as MacroHFT's near-binary learned mixture ... arriving from the opposite direction, and it is the specific thing my own weight-entropy reporting is meant to prevent." Sub-gap 2 - indirect and mostly as a cheaper competitor to FIGARCH: SEMA is "far cheaper than the FIGARCH route ... which matters because the only confirmed ready-made CSE set covers February 2025 to February 2026. With roughly 240 trading days and $w \approx 30$ that is 8 segments for a two-parameter regression, thin but not absurd." No long-memory content of its own.
+EFFECT ON SUB-GAP 1: LEAVES IT OPEN, and is the strongest illustration that it is open. Zero impact modelling: no Almgren-Chriss, no square-root, no LOB simulator, no depth anywhere. Cost is exactly the flat-rate-on-turnover model the sub-gap is aimed at, computed exactly. The note's own verdict, in red: "the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper." What this paper *does* contribute to closing sub-gap 1 is machinery rather than a model: the exact, provably unique transaction remainder factor with constant bounds $\frac{1-\delta}{1+\delta} \leq \omega_{t-1} \leq 1$, which "lets a cost term stay inside a convex objective rather than sitting outside it as a post-hoc deduction" - that is the container into which a state-dependent $\delta$ can be substituted. It also hands over the exact experiment the sub-gap needs: the $\delta$ sweep the authors skipped.
 PROPOSED REVISION STATED IN THE NOTE: Yes, several, verbatim. On the evaluation/baseline set: "SOPS is the fourth baseline my evaluation design is missing. My current three are equal weight, static learned weight and dynamic state-aware weight. A hard state-conditioned router, a threshold rule that picks one of two objectives with no learning and no confidence input, sits between the second and third and is much closer to real prior art than equal weighting. If my adaptive orchestrator cannot beat a count-and-threshold switch, the soft-weighting contribution is not there, and I would rather discover that in my own ablation than have it asked in a viva. This is a direct proposed revision to the experimental design section of the scope note." On the conditioning set: "SEMA is a candidate state variable for the orchestrator that costs almost nothing in data ... The labelling rule itself is also a testable alternative to MacroHFT's volatility tertile, and its advantage for $A_V$ is that it is per asset rather than per market, giving the orchestrator an asset-level state vector that can be aggregated by a count, as this paper does, or fed in directly. Both are crude and neither has a strong theoretical claim over the other, so implement both and let the ablation decide." On $A_V$: "The log-barrier diversification term is reusable for $A_V$ ... if I use a penalty of this shape I report the realised contributions alongside the weights and describe it as a diversification penalty, not as parity."</t>
         </is>
       </c>
@@ -5245,7 +5245,7 @@
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Briola, Bartolucci and Aste, UCL Computer Science and the LSE Systemic Risk Centre. "HLOB – Information persistence and structure in limit order books." Expert Systems With Applications 266, 2025, article 126078. Published open access 12 December 2024.</t>
+          <t>Briola, Bartolucci and Aste, UCL Computer Science and the LSE Systemic Risk Centre. "HLOB - Information persistence and structure in limit order books." Expert Systems With Applications 266, 2025, article 126078. Published open access 12 December 2024.</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>none recorded beyond "open access"; code released as part of the LOBFrame pipeline.</t>
+          <t>DOI 10.1016/j.eswa.2024.126078. Open access; code released as part of the LOBFrame pipeline.</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -5280,17 +5280,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>LOBSTER tick-by-tick NASDAQ, $L=10$ price and volume levels per side. 15 stocks, 6 sectors, 13 industries — 6 small-tick, 3 medium-tick, 6 large-tick. Three separate years 2017, 2018, 2019, treated independently. Per year: 40 training days, 5 validation days sampled from *within* the training period, 10 consecutive test days. Input window 100 LOB updates. Horizons $H_{\Delta\tau} \in \{10, 50, 100\}$ LOB updates in event time — "physical time never used." 5-day feature-wise rolling z-score fitted on past days only. Compute: "1,350 experiments, 7,192 GPU hours, 10 distinct GPU models."</t>
+          <t>LOBSTER tick-by-tick NASDAQ, $L=10$ price and volume levels per side. 15 stocks, 6 sectors, 13 industries - 6 small-tick, 3 medium-tick, 6 large-tick. Three separate years 2017, 2018, 2019, treated independently. Per year: 40 training days, 5 validation days sampled from *within* the training period, 10 consecutive test days. Input window 100 LOB updates. Horizons $H_{\Delta\tau} \in \{10, 50, 100\}$ LOB updates in event time - "physical time never used." 5-day feature-wise rolling z-score fitted on past days only. Compute: "1,350 experiments, 7,192 GPU hours, 10 distinct GPU models."</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr">
         <is>
-          <t>Pure LOB — 10 levels of price and volume per side. TMFG built from volume data only, "reducing each snapshot from $\mathbb{R}^{4L}$ to $\mathbb{R}^{2L}$, on the reasoning that volumes are the homogeneous part of the record while price levels are not." Derived diagnostic: 'actual depth' $\Xi^\text{Bid}$, $\Xi^\text{Ask}$ from Wu et al. (2021), "the number of tick-sized price intervals the ten quoted levels span." Labelling is absolute-threshold three-class: $$ \begin{cases} (m_{\tau + \Delta\tau} - m_{\tau}) \leq -\theta &amp;\rightarrow\ -1\ \rightarrow\ \text{Down}\\ -\theta &lt; (m_{\tau + \Delta\tau} - m_{\tau}) &lt; +\theta &amp;\rightarrow\ \ \ 0\ \rightarrow\ \text{Stable}\\ (m_{\tau + \Delta\tau} - m_{\tau}) \geq +\theta &amp;\rightarrow\ +1\ \rightarrow\ \text{Up} \end{cases} $$ with $m_\tau = \frac{p_1^\text{ask}(\tau) + p_1^\text{bid}(\tau)}{2}$ and $\sigma_\tau = p_1^\text{ask}(\tau) - p_1^\text{bid}(\tau)$.</t>
+          <t>Pure LOB - 10 levels of price and volume per side. TMFG built from volume data only, "reducing each snapshot from $\mathbb{R}^{4L}$ to $\mathbb{R}^{2L}$, on the reasoning that volumes are the homogeneous part of the record while price levels are not." Derived diagnostic: 'actual depth' $\Xi^\text{Bid}$, $\Xi^\text{Ask}$ from Wu et al. (2021), "the number of tick-sized price intervals the ten quoted levels span." Labelling is absolute-threshold three-class: $$ \begin{cases} (m_{\tau + \Delta\tau} - m_{\tau}) \leq -\theta &amp;\rightarrow\ -1\ \rightarrow\ \text{Down}\\ -\theta &lt; (m_{\tau + \Delta\tau} - m_{\tau}) &lt; +\theta &amp;\rightarrow\ \ \ 0\ \rightarrow\ \text{Stable}\\ (m_{\tau + \Delta\tau} - m_{\tau}) \geq +\theta &amp;\rightarrow\ +1\ \rightarrow\ \text{Up} \end{cases} $$ with $m_\tau = \frac{p_1^\text{ask}(\tau) + p_1^\text{bid}(\tau)}{2}$ and $\sigma_\tau = p_1^\text{ask}(\tau) - p_1^\text{bid}(\tau)$.</t>
         </is>
       </c>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>Volumes discretized into equally spaced bins (bin count tuned once, held constant across stocks) "to stop minimum-lot granularity from injecting noise into the estimator"; pairwise mutual information between all volume levels, bootstrapped daily, averaged across training days, giving one $(2L \times 2L)$ similarity matrix per stock. Graph selection: $$\mathcal{G}^{*} \Rightarrow \arg\min_{\mathcal{G}} D_{KL}\big(f(\mathbb{L})\ \|\ \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} \mathbb{E}_{f}\big(\log f(\mathbb{L})\big) - \mathbb{E}_{f}\big(\log \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} H(\mathbb{L}|\mathcal{G})$$ Three simplicial families extracted — maximal cliques of size 4, 3, 2, giving "a fixed 17 tetrahedra, 52 triangles and 54 edges for a 20-node graph" and three input tensors of shape $100 \times 136$, $100 \times 312$, $100 \times 216$. Each head runs three convolutional layers: first $1\times2$ with stride $1\times2$ so it "prevents parameter sharing between levels that are geographically but not logically consecutive, which is the whole complaint against DeepLOB expressed as a stride"; second with stride $1\times4$, $1\times3$, $1\times2$ mixing only within-simplex components; third with filter $1\times\Omega$ for $\Omega \in \{17,52,54\}$, dropout 0.35. Concatenation into a 32-unit LSTM and a 3-output dense layer. AdamW at $6\times10^{-5}$, $\beta_1=0.90$, $\beta_2=0.95$, batch 32, max 100 epochs, early stopping at 0.003 over 15 epochs. Output: three-class direction.</t>
+          <t>Volumes discretized into equally spaced bins (bin count tuned once, held constant across stocks) "to stop minimum-lot granularity from injecting noise into the estimator"; pairwise mutual information between all volume levels, bootstrapped daily, averaged across training days, giving one $(2L \times 2L)$ similarity matrix per stock. Graph selection: $$\mathcal{G}^{*} \Rightarrow \arg\min_{\mathcal{G}} D_{KL}\big(f(\mathbb{L})\ \|\ \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} \mathbb{E}_{f}\big(\log f(\mathbb{L})\big) - \mathbb{E}_{f}\big(\log \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} H(\mathbb{L}|\mathcal{G})$$ Three simplicial families extracted - maximal cliques of size 4, 3, 2, giving "a fixed 17 tetrahedra, 52 triangles and 54 edges for a 20-node graph" and three input tensors of shape $100 \times 136$, $100 \times 312$, $100 \times 216$. Each head runs three convolutional layers: first $1\times2$ with stride $1\times2$ so it "prevents parameter sharing between levels that are geographically but not logically consecutive, which is the whole complaint against DeepLOB expressed as a stride"; second with stride $1\times4$, $1\times3$, $1\times2$ mixing only within-simplex components; third with filter $1\times\Omega$ for $\Omega \in \{17,52,54\}$, dropout 0.35. Concatenation into a 32-unit LSTM and a 3-output dense layer. AdamW at $6\times10^{-5}$, $\beta_1=0.90$, $\beta_2=0.95$, batch 32, max 100 epochs, early stopping at 0.003 over 15 epochs. Output: three-class direction.</t>
         </is>
       </c>
       <c r="L38" s="11" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>None in any modelled sense. Volatility does not appear as a feature, an objective term or a grouping variable — the note is explicit that "Everything in the results follows this split rather than sector, capitalization or volatility." No risk term, no drawdown, no position sizing. LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is a *forecasting* paper, so there is no cost model, no impact function and no execution simulator — but it is deeply about liquidity structure. Spread is the organising variable: the tick-size classification is defined on $\langle\sigma\rangle/\theta$, the ratio of the stock's average bid-ask spread to the exchange tick. Depth is quantified by $\Xi$: "Every large-tick stock sits at 9.00 to 9.21 across all three years, so the ten levels occupy ten consecutive ticks and 'level' means what the array says it means, while MCD in 2017 reports a mean ask-side $\Xi$ of 126.97, its ten levels scattered over more than 127 ticks. When $\Xi \gg 9$ the average MI across levels is corrupted by informational drift." The one friction-adjacent metric is $p_\text{T}$: $p_\text{T} = \frac{\text{CT}}{\text{PT} + \text{TT} - \text{CT}}$, where PT counts potential round trips in the targets, TT the ones a model's predictions would have executed, CT the ones executed correctly. But: "$p_\text{T}$ is a probability of correctly identifying a round trip, not a P&amp;L: no fees, no queue position, no partial fills, no market impact, which is the same boundary [[A reinforcement learning approach to optimal execution]] draws around itself." No Almgren-Chriss, no square-root, no linear impact, no queue modelling, no partial fills, no calibration of any cost parameter. Class imbalance handled by balanced samplers of 5,000 per class per day in training, left untouched at test.</t>
+          <t>None in any modelled sense. Volatility does not appear as a feature, an objective term or a grouping variable - the note is explicit that "Everything in the results follows this split rather than sector, capitalization or volatility." No risk term, no drawdown, no position sizing. LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is a *forecasting* paper, so there is no cost model, no impact function and no execution simulator - but it is deeply about liquidity structure. Spread is the organising variable: the tick-size classification is defined on $\langle\sigma\rangle/\theta$, the ratio of the stock's average bid-ask spread to the exchange tick. Depth is quantified by $\Xi$: "Every large-tick stock sits at 9.00 to 9.21 across all three years, so the ten levels occupy ten consecutive ticks and 'level' means what the array says it means, while MCD in 2017 reports a mean ask-side $\Xi$ of 126.97, its ten levels scattered over more than 127 ticks. When $\Xi \gg 9$ the average MI across levels is corrupted by informational drift." The one friction-adjacent metric is $p_\text{T}$: $p_\text{T} = \frac{\text{CT}}{\text{PT} + \text{TT} - \text{CT}}$, where PT counts potential round trips in the targets, TT the ones a model's predictions would have executed, CT the ones executed correctly. But: "$p_\text{T}$ is a probability of correctly identifying a round trip, not a P&amp;L: no fees, no queue position, no partial fills, no market impact, which is the same boundary [[A reinforcement learning approach to optimal execution]] draws around itself." No Almgren-Chriss, no square-root, no linear impact, no queue modelling, no partial fills, no calibration of any cost parameter. Class imbalance handled by balanced samplers of 5,000 per class per day in training, left untouched at test.</t>
         </is>
       </c>
       <c r="P38" s="11" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="R38" s="11" t="inlineStr">
         <is>
-          <t>F1, MCC and $p_\text{T}$ against 9 alternatives — CNN1, CNN2, DLA, Transformer, iTransformer, LobTransformer, BinBTabl, BinCTabl, DeepLOB — across 15 stocks, 3 years, 3 horizons. Superiority defined as maximal sum of the three metrics.</t>
+          <t>F1, MCC and $p_\text{T}$ against 9 alternatives - CNN1, CNN2, DLA, Transformer, iTransformer, LobTransformer, BinBTabl, BinCTabl, DeepLOB - across 15 stocks, 3 years, 3 horizons. Superiority defined as maximal sum of the three metrics.</t>
         </is>
       </c>
       <c r="S38" s="11" t="inlineStr">
@@ -5345,14 +5345,14 @@
       </c>
       <c r="V38" s="11" t="inlineStr">
         <is>
-          <t>No execution layer of any kind — $p_\text{T}$ stops at round-trip feasibility, with no fees, queue, partial fills or impact. No TMFG ablation, so the causal claim is unestablished. Static structure in a paper about persistence. No statistical testing. One venue, one tick regime, event-time horizons that cannot be transported to a market with different update rates.</t>
+          <t>No execution layer of any kind - $p_\text{T}$ stops at round-trip feasibility, with no fees, queue, partial fills or impact. No TMFG ablation, so the causal claim is unestablished. Static structure in a paper about persistence. No statistical testing. One venue, one tick regime, event-time horizons that cannot be transported to a market with different update rates.</t>
         </is>
       </c>
       <c r="W38" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: A_L (primary — tick-size class, $\Xi$ actual depth, MI structure across volume levels are the liquidity agent's diagnostic toolkit), A_T (it is a directional forecaster on microstructure, i.e. a candidate $A_T$ at high frequency), orchestrator (the $p_\text{T}$ common-scale competence metric; the IFN-over-agent-signals construction), friction-aware evaluation layer (the practicability-vs-action-count quadrant reporting).
-EFFECT ON MAIN GAP / SUB-GAP 2: Main gap — three contributions the note draws out: (i) $p_\text{T}$ as a common-scale, backward-looking competence estimate for heterogeneous components, which is the note's candidate answer to "how an LLM analyst, an econometric estimator and an RL allocator produce confidence scores on one scale"; (ii) the static-structure failure mode read one layer up — "My main gap is about adapting influence over heterogeneous components as market state changes, and this is the same failure mode one level down: a structure estimated once over a training window describes a regime, not a market"; (iii) the information-persistence argument as the principled way to *choose* the orchestrator's decision frequency. Sub-gap 2 — none directly; no volatility modelling, no long memory, no risk guardrail. The nearest adjacency is that the persistence/degradation curve is a decay-rate argument about how long information lasts, which is structurally analogous to a long-memory argument but is about signal horizon, not volatility.
-EFFECT ON SUB-GAP 1: LEAVES IT OPEN on the cost-model axis, but it supplies the decisive pre-test that determines whether the sub-gap is even attackable on CSE data. HLOB has no impact model, no Almgren-Chriss, no square-root, no execution simulator — the note puts it in exactly the same bracket as Moallemi and Wang: "no fees, no queue position, no partial fills, no market impact, which is the same boundary [[A reinforcement learning approach to optimal execution]] draws around itself." What it *does* contribute is the depth-structure vocabulary the sub-gap needs: $\langle\sigma\rangle/\theta$ tick classification and the $\Xi$ actual-depth measure are precisely how you characterise "available depth" on a thin book, and the paper demonstrates that liquidity class, not architecture, is the binding variable — "Tick size, not architecture, is the variable that separates a usable model from an unusable one ... the contrast between the first and last rows is larger than any difference between models anywhere in the paper." It also makes the go/no-go concrete: if CSE counters are small-tick, an MCC of 0.05 is the expected ceiling and the microstructural route should not be taken at all.
+          <t>SPEAKS TO: A_L (primary - tick-size class, $\Xi$ actual depth, MI structure across volume levels are the liquidity agent's diagnostic toolkit), A_T (it is a directional forecaster on microstructure, i.e. a candidate $A_T$ at high frequency), orchestrator (the $p_\text{T}$ common-scale competence metric; the IFN-over-agent-signals construction), friction-aware evaluation layer (the practicability-vs-action-count quadrant reporting).
+EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - three contributions the note draws out: (i) $p_\text{T}$ as a common-scale, backward-looking competence estimate for heterogeneous components, which is the note's candidate answer to "how an LLM analyst, an econometric estimator and an RL allocator produce confidence scores on one scale"; (ii) the static-structure failure mode read one layer up - "My main gap is about adapting influence over heterogeneous components as market state changes, and this is the same failure mode one level down: a structure estimated once over a training window describes a regime, not a market"; (iii) the information-persistence argument as the principled way to *choose* the orchestrator's decision frequency. Sub-gap 2 - none directly; no volatility modelling, no long memory, no risk guardrail. The nearest adjacency is that the persistence/degradation curve is a decay-rate argument about how long information lasts, which is structurally analogous to a long-memory argument but is about signal horizon, not volatility.
+EFFECT ON SUB-GAP 1: LEAVES IT OPEN on the cost-model axis, but it supplies the decisive pre-test that determines whether the sub-gap is even attackable on CSE data. HLOB has no impact model, no Almgren-Chriss, no square-root, no execution simulator - the note puts it in exactly the same bracket as Moallemi and Wang: "no fees, no queue position, no partial fills, no market impact, which is the same boundary [[A reinforcement learning approach to optimal execution]] draws around itself." What it *does* contribute is the depth-structure vocabulary the sub-gap needs: $\langle\sigma\rangle/\theta$ tick classification and the $\Xi$ actual-depth measure are precisely how you characterise "available depth" on a thin book, and the paper demonstrates that liquidity class, not architecture, is the binding variable - "Tick size, not architecture, is the variable that separates a usable model from an unusable one ... the contrast between the first and last rows is larger than any difference between models anywhere in the paper." It also makes the go/no-go concrete: if CSE counters are small-tick, an MCC of 0.05 is the expected ceiling and the microstructural route should not be taken at all.
 PROPOSED REVISION STATED IN THE NOTE: Yes, two, verbatim. On the conditioning set / confidence term $C_{i,t}$: "$p_\text{T}$ is a candidate answer to the comparable-confidence problem the orchestrator design has been stuck on, and it belongs in the evaluation protocol either way ... $p_\text{T} = \frac{\text{CT}}{\text{PT} + \text{TT} - \text{CT}}$ ... is a bounded $[0,1]$ quantity defined purely on realized decisions and outcomes, so it can be computed for any component that emits a directional view regardless of how it arrived at one. It is backward-looking, so it would feed the weighting as a rolling competence estimate rather than a live per-decision confidence, but that is closer to a common scale than anything else in the vault." On the orchestrator's internal structure: "It also suggests a concrete construction worth testing, an IFN computed over the *agents'* output signals rather than over LOB levels, which would give the orchestrator a filtered dependency graph among components and a principled way to notice when two supposedly independent agents have started agreeing for the same reason." And a gating decision on $A_L$: the $\langle\sigma\rangle/\theta$ test "goes ahead of the CSE data-depth question rather than behind it."</t>
         </is>
       </c>
@@ -5400,12 +5400,12 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>US equities — 27 DJIA components trading continuously over the full period, plus S&amp;P 100 for robustness.  econometric/ML volatility forecasting. No agents, no LLM: "there is no agent, no orchestration and no LLM anywhere in it".</t>
+          <t>US equities - 27 DJIA components trading continuously over the full period, plus S&amp;P 100 for robustness. econometric/ML volatility forecasting. No agents, no LLM: "there is no agent, no orchestration and no LLM anywhere in it".</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>LOBSTER tick data, five-minute RV following Liu et al. (2015). 1 July 2007 to 30 June 2021. Out-of-sample 1 July 2011 to 30 June 2021, ten years. Rolling scheme: 36 months training, most recent 12 months validation, next month tested, recalibrated monthly — "120 separate monthly refits on a rolling window, not one train-test split, which is a much higher bar than most of the ML papers in the vault clear."</t>
+          <t>LOBSTER tick data, five-minute RV following Liu et al. (2015). 1 July 2007 to 30 June 2021. Out-of-sample 1 July 2011 to 30 June 2021, ten years. Rolling scheme: 36 months training, most recent 12 months validation, next month tested, recalibrated monthly - "120 separate monthly refits on a rolling window, not one train-test split, which is a much higher bar than most of the ML papers in the vault clear."</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
@@ -5455,7 +5455,7 @@
       </c>
       <c r="S39" s="11" t="inlineStr">
         <is>
-          <t>one-day MSE ratios — "GHAR_M cuts one-day MSE to 0.927 of HAR_M, GNNHAR1L_M takes it further to 0.907, and switching the criterion to QL improves nearly every row again, with GNNHAR1L_Q reaching 0.867 in MSE and 0.961 in QL, roughly 13% and 4% below the standard HAR benchmark." Depth hurts monotonically: "One-day MSE ratios run 0.907, 0.967 and 1.210 for one, two and three layers under MSE training, so the three-layer model is beaten by plain HAR"; MAD falls from roughly e^{-10.5} to e^{-15.5}. Multi-hop fails: DM cross-sectional p = 0.75 (MSE) and 0.40 (QL) for 2L vs 1L, AXP the only individually significant stock; GHAR2Hop vs GHAR gives DM ≈ −1, p ≈ 0.35; daily two-hop coefficient "at roughly one-eighth of its one-hop counterpart". Long horizon: "By one month most MSE ratios exceed one, with GNNHAR2L_Q at 1.736 and GNNHAR3L_Q at 1.502, while the QL ratios stay below one and GNNHAR2L_Q at 0.947 remains inside the confidence set." Turbulence: FVU "GNNHAR1L_M at 0.077 calm against 0.165 turbulent for one-day forecasts and GNNHAR3L_M at 0.079 against 0.300"; stratified loss "GNNHAR1L_Q reaches 0.834 of HAR_M on one-day MSE during the top 10% turbulent days against 0.895 for its MSE-trained twin". S&amp;P 100 robustness: "GNNHAR2L_Q posts the best one-day MSE there at 0.915". Graph density: DJIA 57.7% one hop, 41.8% two, 0.5% three; S&amp;P 100 24.3/61.2/12.0/2.2/0.3%. LIMITATIONS (quoting the note): "The multi-hop conclusion is drawn on a graph that barely has a second hop to test... The conclusion I would actually carry forward is narrower than the paper's: on dense graphs of large-cap US equities, multi-hop aggregation does not pay for its parameters." "The return-based graph is never compared against a volatility-based one... the identity of the edges is the most load-bearing unexamined choice in the design." "Nonlinearity is established through one architecture and one activation." "The turbulence stratification uses the full-sample distribution to define its own regimes... every statement about turbulent-period performance is conditioned on an ex-post label that a live system would have to estimate in real time... This matters more for me than for the paper, because I would be using the regime label as a live input rather than as a reporting split." "Forecast loss is the only outcome, and the economic question is left open... a 13% MSE reduction at the one-day horizon has no translation into a decision anywhere in the paper."</t>
+          <t>one-day MSE ratios - "GHAR_M cuts one-day MSE to 0.927 of HAR_M, GNNHAR1L_M takes it further to 0.907, and switching the criterion to QL improves nearly every row again, with GNNHAR1L_Q reaching 0.867 in MSE and 0.961 in QL, roughly 13% and 4% below the standard HAR benchmark." Depth hurts monotonically: "One-day MSE ratios run 0.907, 0.967 and 1.210 for one, two and three layers under MSE training, so the three-layer model is beaten by plain HAR"; MAD falls from roughly e^{-10.5} to e^{-15.5}. Multi-hop fails: DM cross-sectional p = 0.75 (MSE) and 0.40 (QL) for 2L vs 1L, AXP the only individually significant stock; GHAR2Hop vs GHAR gives DM ≈ −1, p ≈ 0.35; daily two-hop coefficient "at roughly one-eighth of its one-hop counterpart". Long horizon: "By one month most MSE ratios exceed one, with GNNHAR2L_Q at 1.736 and GNNHAR3L_Q at 1.502, while the QL ratios stay below one and GNNHAR2L_Q at 0.947 remains inside the confidence set." Turbulence: FVU "GNNHAR1L_M at 0.077 calm against 0.165 turbulent for one-day forecasts and GNNHAR3L_M at 0.079 against 0.300"; stratified loss "GNNHAR1L_Q reaches 0.834 of HAR_M on one-day MSE during the top 10% turbulent days against 0.895 for its MSE-trained twin". S&amp;P 100 robustness: "GNNHAR2L_Q posts the best one-day MSE there at 0.915". Graph density: DJIA 57.7% one hop, 41.8% two, 0.5% three; S&amp;P 100 24.3/61.2/12.0/2.2/0.3%. LIMITATIONS (quoting the note): "The multi-hop conclusion is drawn on a graph that barely has a second hop to test... The conclusion I would actually carry forward is narrower than the paper's: on dense graphs of large-cap US equities, multi-hop aggregation does not pay for its parameters." "The return-based graph is never compared against a volatility-based one... the identity of the edges is the most load-bearing unexamined choice in the design." "Nonlinearity is established through one architecture and one activation." "The turbulence stratification uses the full-sample distribution to define its own regimes... every statement about turbulent-period performance is conditioned on an ex-post label that a live system would have to estimate in real time... This matters more for me than for the paper, because I would be using the regime label as a live input rather than as a reporting split." "Forecast loss is the only outcome, and the economic question is left open... a 13% MSE reduction at the one-day horizon has no translation into a decision anywhere in the paper."</t>
         </is>
       </c>
       <c r="T39" s="11" t="inlineStr">
@@ -5465,20 +5465,20 @@
       </c>
       <c r="U39" s="11" t="inlineStr">
         <is>
-          <t>"Swap the training loss before swapping the model" — QL as default for any CSE volatility forecaster, implementable on a linear model via the IRLS equivalence "which matters when the sample is short". "Report everything as a ratio to a HAR baseline with a model confidence set attached... MCS plus cross-sectionally averaged DM pairing is the specific machinery to copy." The calm/turbulent split as the orchestrator's evaluation reporting shape — "a better regime template than MacroHFT's". Over-smoothing/MAD as the volatility-model analogue of the weight-entropy diagnostic: "Formalising both as representation-collapse diagnostics, MAD over node representations and entropy over agent weights, gives me one consistent story about capacity that does not pay for itself." The QL loss ratio as a candidate comparable-confidence scale: "A rolling QL loss ratio against a fixed benchmark is unit-free, computable for any component that emits a distributional or point forecast of the same target."</t>
+          <t>"Swap the training loss before swapping the model" - QL as default for any CSE volatility forecaster, implementable on a linear model via the IRLS equivalence "which matters when the sample is short". "Report everything as a ratio to a HAR baseline with a model confidence set attached... MCS plus cross-sectionally averaged DM pairing is the specific machinery to copy." The calm/turbulent split as the orchestrator's evaluation reporting shape - "a better regime template than MacroHFT's". Over-smoothing/MAD as the volatility-model analogue of the weight-entropy diagnostic: "Formalising both as representation-collapse diagnostics, MAD over node representations and entropy over agent weights, gives me one consistent story about capacity that does not pay for itself." The QL loss ratio as a candidate comparable-confidence scale: "A rolling QL loss ratio against a fixed benchmark is unit-free, computable for any component that emits a distributional or point forecast of the same target."</t>
         </is>
       </c>
       <c r="V39" s="11" t="inlineStr">
         <is>
-          <t>no decision anywhere downstream of the forecast; no persistence/long-memory parameter; ex-post regime labelling; an unvalidated return-based graph; and the input data requirement (five-minute RV) is unavailable — "CSE intraday data at that resolution is not something I have established access to... The realistic substitutes are daily range-based estimators, Parkinson or Garman-Klass."</t>
+          <t>no decision anywhere downstream of the forecast; no persistence/long-memory parameter; ex-post regime labelling; an unvalidated return-based graph; and the input data requirement (five-minute RV) is unavailable - "CSE intraday data at that resolution is not something I have established access to... The realistic substitutes are daily range-based estimators, Parkinson or Garman-Klass."</t>
         </is>
       </c>
       <c r="W39" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_V primarily (the econometric volatility estimator inside it), plus evaluation layer (ratio-to-baseline + MCS + calm/turbulent stratified reporting) and orchestrator (QL loss ratio as a comparable confidence scale; MAD as collapse diagnostic).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — indirect support via the calm/turbulent template and the MAD collapse diagnostic, but no orchestration of any kind. Sub-gap 1 — none; friction is entirely absent by design.
-EFFECT ON SUB-GAP 2: LEAVES IT OPEN, and does so in the most quotable way of any paper here. It is the purest instance of the sub-gap's failure mode: volatility is forecast with ten years of rigorous out-of-sample evaluation and 120 monthly refits, and nothing is ever done with the forecast. The note states it flatly — "Forecast loss is the only outcome, and the economic question is left open... no portfolio, no value-at-risk backtest and no transaction-cost-bearing application, so a 13% MSE reduction at the one-day horizon has no translation into a decision anywhere in the paper." Specifically on the two questions asked: (a) YES, it uses realised volatility predictively — that is the entire object, next-day/week/month RV forecast conditioned on a cross-sectional graph, and it is genuinely predictive rather than descriptive, with 13% MSE reduction at one day. (b) NO, it does nothing with persistence or long memory as an estimated quantity. Long memory appears once, as motivation for the HAR lag structure itself: the three-lag spine is "the cheapest available way to reproduce the long-memory decay in the RV autocorrelation function without fitting a fractionally integrated model". So long memory is absorbed into the model's functional form and never estimated, never reported as a coefficient, never fed anywhere. There is no d, no fractional integration, no decay-speed parameter. The paper's contribution runs entirely in the cross-sectional (spillover) direction and leaves the temporal-persistence direction untouched — which is exactly the axis Sub-gap 2 lives on. The one partial narrowing it offers is indirect: the calm/turbulent stratification shows forecast quality is itself state-dependent, and the FVU numbers locate the nonlinear model's value in the top volatility decile, which is an argument that volatility state should condition something — but the paper conditions only its reporting, not its behaviour.
-CSE DATA EVIDENCE: not a CSE paper. Relevant only negatively: five-minute RV is unobtainable here, so the estimator's input has to be re-derived (Parkinson or Garman-Klass daily range-based), and building a CSE volatility graph faces a problem the DJIA does not — "a meaningful share of counters post zero returns on a given day because they did not trade, which biases any covariance estimate towards spurious independence and will make the precision matrix unstable."
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - indirect support via the calm/turbulent template and the MAD collapse diagnostic, but no orchestration of any kind. Sub-gap 1 - none; friction is entirely absent by design.
+EFFECT ON SUB-GAP 2: LEAVES IT OPEN, and does so in the most quotable way of any paper here. It is the purest instance of the sub-gap's failure mode: volatility is forecast with ten years of rigorous out-of-sample evaluation and 120 monthly refits, and nothing is ever done with the forecast. The note states it flatly - "Forecast loss is the only outcome, and the economic question is left open... no portfolio, no value-at-risk backtest and no transaction-cost-bearing application, so a 13% MSE reduction at the one-day horizon has no translation into a decision anywhere in the paper." Specifically on the two questions asked: (a) YES, it uses realised volatility predictively - that is the entire object, next-day/week/month RV forecast conditioned on a cross-sectional graph, and it is genuinely predictive rather than descriptive, with 13% MSE reduction at one day. (b) NO, it does nothing with persistence or long memory as an estimated quantity. Long memory appears once, as motivation for the HAR lag structure itself: the three-lag spine is "the cheapest available way to reproduce the long-memory decay in the RV autocorrelation function without fitting a fractionally integrated model". So long memory is absorbed into the model's functional form and never estimated, never reported as a coefficient, never fed anywhere. There is no d, no fractional integration, no decay-speed parameter. The paper's contribution runs entirely in the cross-sectional (spillover) direction and leaves the temporal-persistence direction untouched - which is exactly the axis Sub-gap 2 lives on. The one partial narrowing it offers is indirect: the calm/turbulent stratification shows forecast quality is itself state-dependent, and the FVU numbers locate the nonlinear model's value in the top volatility decile, which is an argument that volatility state should condition something - but the paper conditions only its reporting, not its behaviour.
+CSE DATA EVIDENCE: not a CSE paper. Relevant only negatively: five-minute RV is unobtainable here, so the estimator's input has to be re-derived (Parkinson or Garman-Klass daily range-based), and building a CSE volatility graph faces a problem the DJIA does not - "a meaningful share of counters post zero returns on a given day because they did not trade, which biases any covariance estimate towards spurious independence and will make the precision matrix unstable."
 PROPOSED REVISION STATED IN THE NOTE: no revision to the four-agent pool. On the conditioning set, two things bear on C_{i,t}: "The QL loss ratio is a second candidate for the comparable-confidence problem, and a better-behaved one than p_T... A rolling QL loss ratio against a fixed benchmark is unit-free, computable for any component that emits a distributional or point forecast of the same target, and interpretable in the same direction regardless of the component's internals, which makes it a rolling competence weight in exactly the way the p_T metric from HLOB is for directional components. Neither gives a per-decision confidence, both give a backward-looking competence estimate, and having two of them defined on different output types is progress on the problem rather than a solution to it." And on V_t: "the paper's label is computed ex post, and a live orchestrator needs the same label from a rolling estimate, so pinning the minimum window for a usable turbulence indicator on CSE data is now a concrete task rather than an open question."</t>
         </is>
       </c>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="J40" s="11" t="inlineStr">
         <is>
-          <t>dependent — monthly change in the All Share Price Index, from CSE market data. Independent, all from CBSL — GDP growth rate, inflation via CCPI, Weighted Average Deposit Rate, broad money M2, USD/LKR. "GDP is quarterly and was converted to monthly with the Quadratic Interpolation Method in EViews, citing Ju et al. (2014)." All in logs.</t>
+          <t>dependent - monthly change in the All Share Price Index, from CSE market data. Independent, all from CBSL - GDP growth rate, inflation via CCPI, Weighted Average Deposit Rate, broad money M2, USD/LKR. "GDP is quarterly and was converted to monthly with the Quadratic Interpolation Method in EViews, citing Ju et al. (2014)." All in logs.</t>
         </is>
       </c>
       <c r="K40" s="11" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="M40" s="11" t="inlineStr">
         <is>
-          <t>none measured. Sentiment appears only as an unexplained residual interpretation — see below.</t>
+          <t>none measured. Sentiment appears only as an unexplained residual interpretation - see below.</t>
         </is>
       </c>
       <c r="N40" s="11" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="R40" s="11" t="inlineStr">
         <is>
-          <t>none — "There is no out-of-sample period anywhere in this paper, no baseline, and no forecast."</t>
+          <t>none - "There is no out-of-sample period anywhere in this paper, no baseline, and no forecast."</t>
         </is>
       </c>
       <c r="S40" s="11" t="inlineStr">
@@ -5602,9 +5602,9 @@
       <c r="W40" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (negative evidence about what to condition on), weakly A_V (as a cautionary specification), evaluation layer (in-sample fit is not a result).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — real and useful bearing, as the quantitative warrant for excluding a macro block from the conditioning set (adjusted R² of 0.189286). Sub-gap 1 — none; no volume, turnover, spreads or costs anywhere.
-EFFECT ON SUB-GAP 2: LEAVES IT WIDE OPEN — and in fact sits one step further back than the other papers, because it does not even measure persistence. It is the degenerate case: the word volatility is used throughout, the quantity measured is a signed return, no dispersion, no clustering, no decay parameter. Nothing is operationalised into any decision. Its value to Sub-gap 2 is as the *naming discipline* argument: "I state my volatility estimator explicitly and early, because this is the failure mode. Realised volatility from daily returns within the month, or the conditional variance from a fitted ARMA-FIGARCH as in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], named in the methodology with the formula next to it, so that no reader has to reconstruct from a table what quantity the risk layer is actually consuming. Pairing the two notes in the review chapter is the cleanest way to make that point, one paper measures persistence in a properly specified variance process, the other calls a signed return volatility and reaches the opposite conclusion about how much it clusters."
-CSE DATA EVIDENCE: source — ASPI from "CSE market data"; all five macro series from CBSL; GDP quarterly, interpolated to monthly in EViews. Frequency — monthly. Range — January 2010 to December 2019, "120 observations per variable, 117 after lags". Tickers — none; index-level only, "no counters, sectors, volumes or spreads anywhere". How obtained — not stated beyond naming CSE and CBSL as sources. Critical for the blocker: this is a ten-year CSE series that exists and was published from, but it is monthly index data, not daily per-ticker, and it deliberately stops at December 2019.
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - real and useful bearing, as the quantitative warrant for excluding a macro block from the conditioning set (adjusted R² of 0.189286). Sub-gap 1 - none; no volume, turnover, spreads or costs anywhere.
+EFFECT ON SUB-GAP 2: LEAVES IT WIDE OPEN - and in fact sits one step further back than the other papers, because it does not even measure persistence. It is the degenerate case: the word volatility is used throughout, the quantity measured is a signed return, no dispersion, no clustering, no decay parameter. Nothing is operationalised into any decision. Its value to Sub-gap 2 is as the *naming discipline* argument: "I state my volatility estimator explicitly and early, because this is the failure mode. Realised volatility from daily returns within the month, or the conditional variance from a fitted ARMA-FIGARCH as in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], named in the methodology with the formula next to it, so that no reader has to reconstruct from a table what quantity the risk layer is actually consuming. Pairing the two notes in the review chapter is the cleanest way to make that point, one paper measures persistence in a properly specified variance process, the other calls a signed return volatility and reaches the opposite conclusion about how much it clusters."
+CSE DATA EVIDENCE: source - ASPI from "CSE market data"; all five macro series from CBSL; GDP quarterly, interpolated to monthly in EViews. Frequency - monthly. Range - January 2010 to December 2019, "120 observations per variable, 117 after lags". Tickers - none; index-level only, "no counters, sectors, volumes or spreads anywhere". How obtained - not stated beyond naming CSE and CBSL as sources. Critical for the blocker: this is a ten-year CSE series that exists and was published from, but it is monthly index data, not daily per-ticker, and it deliberately stops at December 2019.
 PROPOSED REVISION STATED IN THE NOTE: no explicit revision to the four-agent pool. On the conditioning set, the closest statement is: "the conditioning set I build around liquidity state and volatility persistence is not passing over a stronger macro alternative, it's choosing state variables that move at the frequency decisions are actually taken at. If a macro block goes in at all it's as a slow-moving context input, not as a driver, and I cite this number when I say so." That is an argument against adding a macro variable to f(L_t, V_t, P_t, C_{i,t}), not for one.</t>
         </is>
       </c>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="P41" s="11" t="inlineStr">
         <is>
-          <t>volume is the central variable, which is the closest any of these three CSE papers gets to a liquidity construct — but at monthly aggregation and as a predictor, not as a friction. No spreads, no turnover ratio, no costs, no execution.</t>
+          <t>volume is the central variable, which is the closest any of these three CSE papers gets to a liquidity construct - but at monthly aggregation and as a predictor, not as a friction. No spreads, no turnover ratio, no costs, no execution.</t>
         </is>
       </c>
       <c r="Q41" s="11" t="inlineStr">
@@ -5728,9 +5728,9 @@
       <c r="W41" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_L primarily (volume as information-arrival proxy, the domain warrant for L_t), orchestrator (the microstructure-over-macro conditioning argument), evaluation layer (no-holdout pattern).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — the strongest domain-literature support in the set for conditioning on microstructure state (volume) rather than macro, which is direct evidence for keeping L_t in f(·) and keeping macro out. Sub-gap 1 — indirect but real: volume is the raw material of a liquidity state variable, and the note commits to re-testing it at daily frequency "with turnover and a spread proxy alongside it, inside the training window only. If it survives that, it earns a place in the conditioning set. If it doesn't, the discrepancy is itself worth reporting, since it would locate the effect at monthly aggregation."
-EFFECT ON SUB-GAP 2: LEAVES IT OPEN, with one relevant contribution in passing. It runs no volatility model, but it finds ARCH effects at p = 0.0000 in the ASPI, volume and exchange rate while finding none in the macro series — the note reads this as "consistent with the market-side series carrying volatility clustering that the level specification doesn't model, and it's the same persistence [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] is about." So it is a third independent CSE observation of volatility clustering that is detected and then discarded (robust standard errors are applied as a nuisance correction, not as a modelled quantity). This is Sub-gap 2 in its most literal form: persistence is measured — here, effectively, as a diagnostic statistic — and used only to adjust standard errors, never to inform a decision.
-CSE DATA EVIDENCE: source — ASPI and trading volume from the Colombo Stock Exchange; money supply (M2b) and USD/LKR from the Central Bank of Sri Lanka; inflation (NCPI, base 2013=100) from the Department of Census and Statistics. Frequency — monthly. Range — 2014 to 2022 (nine years), "108 observations claimed" but descriptive statistics report 107 for log ASPI and log trading volume, 106 for differenced exchange rate and money supply, 105 for twice-differenced NCPI, with page 127 saying 2014 to 2023. Tickers — none; ASPI index plus aggregate market volume in millions of shares. How obtained — "purposive sampling"; the collection section "discloses that ChatGPT and Google assisted in locating credible sources, with the series then manually extracted, mostly from Excel downloads and the inflation data transcribed out of PDFs." Critical reading for the blocker: this is the only one of the three that uses CSE volume at all, and even so it is market-aggregate monthly volume obtained by manual Excel download — no evidence of bulk per-ticker access.
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - the strongest domain-literature support in the set for conditioning on microstructure state (volume) rather than macro, which is direct evidence for keeping L_t in f(·) and keeping macro out. Sub-gap 1 - indirect but real: volume is the raw material of a liquidity state variable, and the note commits to re-testing it at daily frequency "with turnover and a spread proxy alongside it, inside the training window only. If it survives that, it earns a place in the conditioning set. If it doesn't, the discrepancy is itself worth reporting, since it would locate the effect at monthly aggregation."
+EFFECT ON SUB-GAP 2: LEAVES IT OPEN, with one relevant contribution in passing. It runs no volatility model, but it finds ARCH effects at p = 0.0000 in the ASPI, volume and exchange rate while finding none in the macro series - the note reads this as "consistent with the market-side series carrying volatility clustering that the level specification doesn't model, and it's the same persistence [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] is about." So it is a third independent CSE observation of volatility clustering that is detected and then discarded (robust standard errors are applied as a nuisance correction, not as a modelled quantity). This is Sub-gap 2 in its most literal form: persistence is measured - here, effectively, as a diagnostic statistic - and used only to adjust standard errors, never to inform a decision.
+CSE DATA EVIDENCE: source - ASPI and trading volume from the Colombo Stock Exchange; money supply (M2b) and USD/LKR from the Central Bank of Sri Lanka; inflation (NCPI, base 2013=100) from the Department of Census and Statistics. Frequency - monthly. Range - 2014 to 2022 (nine years), "108 observations claimed" but descriptive statistics report 107 for log ASPI and log trading volume, 106 for differenced exchange rate and money supply, 105 for twice-differenced NCPI, with page 127 saying 2014 to 2023. Tickers - none; ASPI index plus aggregate market volume in millions of shares. How obtained - "purposive sampling"; the collection section "discloses that ChatGPT and Google assisted in locating credible sources, with the series then manually extracted, mostly from Excel downloads and the inflation data transcribed out of PDFs." Critical reading for the blocker: this is the only one of the three that uses CSE volume at all, and even so it is market-aggregate monthly volume obtained by manual Excel download - no evidence of bulk per-ticker access.
 PROPOSED REVISION STATED IN THE NOTE: no revision to the agent pool. On the conditioning set, verbatim: "Volume goes into the liquidity state variable, and I re-estimate this properly rather than inheriting it. Log monthly shares traded is far too coarse for anything I'm doing, so what I take is the hypothesis, that volume carries information about near-term returns on this market, to be re-tested at daily frequency on differenced series with turnover and a spread proxy alongside it, inside the training window only. If it survives that, it earns a place in the conditioning set." And on USD/LKR as a feature: "the direction question has to be settled inside my own window before the feature goes in. I'd expect the truth to be regime-dependent here, with the rate leading during the 2022 float and the index leading in calmer stretches, which is exactly the kind of instability a static feature set handles badly and a state-aware orchestrator is supposed to handle."</t>
         </is>
       </c>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>Colombo Stock Exchange — ASPI, twenty GICS sectors, nine listed banks.  time-series forecasting plus clustering-based selection.</t>
+          <t>Colombo Stock Exchange - ASPI, twenty GICS sectors, nine listed banks. time-series forecasting plus clustering-based selection.</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="Q42" s="11" t="inlineStr">
         <is>
-          <t>none; the clustering stage is the opposite — "The average contribution to clusters has no definition, no formula and no units."</t>
+          <t>none; the clustering stage is the opposite - "The average contribution to clusters has no definition, no formula and no units."</t>
         </is>
       </c>
       <c r="R42" s="11" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="S42" s="11" t="inlineStr">
         <is>
-          <t>"BPNN beats ARIMA, MAE 4.708423 against 29.6975 and MAPE 0.1783333 against 0.4672206". ARIMA selected at "AIC 71180.553, BIC 71243.107 and HQIC 71202.003". Cluster contributions: "Banks and finance 3.16, Diversified 2.51, Hotels and travels 2.50, IT 2.20, Motors 2.66"; within banks "NTB 1.95, NDB 2.34, Sampath 2.39 and Commercial 2.08" — "Sampath wins by 0.05 on the undefined scale". Note's own recomputation: "A no-change forecast anchored on the previous day's actual gives a mean absolute error of 34.96 over the four days where it can be computed, against 9.23 for ARIMA and 2.90 for BPNN, so unlike [[Stock Price Prediction Using ARIMA Model, Evidence from Colombo Stock Exchange]] this paper's tabulated forecasts do clear the naive baseline. That's the strongest thing in it and the authors don't claim it." MASE on those four days "roughly 0.26 for ARIMA and 0.08 for BPNN". LIMITATIONS (quoting the note): "The two reported metric pairs are internally inconsistent, and neither reproduces from the paper's own Table 4... Recomputing both metrics from the five tabulated days gives MAE 7.886 and MAPE 0.120% for ARIMA and MAE 2.732 and MAPE 0.041% for BPNN, neither of which matches the table." "The error metrics don't reconcile, which puts the central claim out of reach... On this evidence I can't verify the comparison the paper exists to make." "The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes and is roughly thirty years of daily trading rather than ten, so the series the ARIMA was fitted on is not the series the paper describes." "The BPNN plot cannot be the ASPI over 2008 to 2017. Its vertical axis runs from 10,000 to 20,000 while the ASPI traded between roughly 1,500 and 7,800 across that decade." "The clustering stage is not reproducible." "Everything is selected and evaluated on one split with no repetition." "The stationarity handling contradicts itself and probably over-differences." "An investment recommendation with no strategy, no costs and no execution." "The sector recommendation reduces to buying the index."</t>
+          <t>"BPNN beats ARIMA, MAE 4.708423 against 29.6975 and MAPE 0.1783333 against 0.4672206". ARIMA selected at "AIC 71180.553, BIC 71243.107 and HQIC 71202.003". Cluster contributions: "Banks and finance 3.16, Diversified 2.51, Hotels and travels 2.50, IT 2.20, Motors 2.66"; within banks "NTB 1.95, NDB 2.34, Sampath 2.39 and Commercial 2.08" - "Sampath wins by 0.05 on the undefined scale". Note's own recomputation: "A no-change forecast anchored on the previous day's actual gives a mean absolute error of 34.96 over the four days where it can be computed, against 9.23 for ARIMA and 2.90 for BPNN, so unlike [[Stock Price Prediction Using ARIMA Model, Evidence from Colombo Stock Exchange]] this paper's tabulated forecasts do clear the naive baseline. That's the strongest thing in it and the authors don't claim it." MASE on those four days "roughly 0.26 for ARIMA and 0.08 for BPNN". LIMITATIONS (quoting the note): "The two reported metric pairs are internally inconsistent, and neither reproduces from the paper's own Table 4... Recomputing both metrics from the five tabulated days gives MAE 7.886 and MAPE 0.120% for ARIMA and MAE 2.732 and MAPE 0.041% for BPNN, neither of which matches the table." "The error metrics don't reconcile, which puts the central claim out of reach... On this evidence I can't verify the comparison the paper exists to make." "The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes and is roughly thirty years of daily trading rather than ten, so the series the ARIMA was fitted on is not the series the paper describes." "The BPNN plot cannot be the ASPI over 2008 to 2017. Its vertical axis runs from 10,000 to 20,000 while the ASPI traded between roughly 1,500 and 7,800 across that decade." "The clustering stage is not reproducible." "Everything is selected and evaluated on one split with no repetition." "The stationarity handling contradicts itself and probably over-differences." "An investment recommendation with no strategy, no costs and no execution." "The sector recommendation reduces to buying the index."</t>
         </is>
       </c>
       <c r="T42" s="11" t="inlineStr">
@@ -5854,9 +5854,9 @@
       <c r="W42" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T (the CSE non-linear price-only baseline the technical agent must beat), orchestrator (the capitalisation-weight warning about counter ranking; the rule that any deciding quantity needs a formula and a dispersion estimate), evaluation layer (horizon/refit columns, MASE).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — a concrete warning about the orchestrator's counter-ranking mechanism (rank on forecastable excess return net of costs, not on index contribution) and a demand that any per-agent reliability weight carry a definition and a sensitivity analysis, with a thin margin treated "as a tie rather than a ranking". Sub-gap 1 — indirect: the paper issues a buy recommendation on a market with documented illiquidity shocks of 8 to 10 basis points and models no spread, no fee, no execution, which is the friction blind spot restated on CSE data.
-EFFECT ON SUB-GAP 2: LEAVES IT OPEN and adds a fourth CSE instance of volatility being ignored entirely rather than measured-and-unused. No conditional variance model on a window opening on the 2008 crisis; no ARCH test; no Ljung-Box. Nothing operationalised. Its only Sub-gap-2 contribution is negative corroboration — it is another CSE paper where constant variance is assumed across a decade the vault's other notes establish is strongly heteroskedastic.
-CSE DATA EVIDENCE: source — "extracted from the CSE database and supplemented with other financial documents". Frequency — daily. Range — stated 2008 to 2017 (abstract inconsistently says 2013 to 2017 for the sector analysis). Tickers — this is the only one of the three CSE papers that touches individual counters: "daily closing prices of nine listed banks", of which only four (NTB, NDB, Sampath, Commercial) appear in the results table — "five of the nine banks are missing from the results table". Plus twenty GICS sector series. Volume — "2,221 price samples classified into 20 sectors". How obtained — CSE database, method unspecified. Critical caveat for the blocker: the note establishes the stated dataset is not what was actually fitted — "The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes... so the series the ARIMA was fitted on is not the series the paper describes", and the BPNN plot's axis range is inconsistent with the ASPI over that decade. So this paper claims ten years of daily per-counter CSE bank prices, but its own printouts contradict its data section, and nothing per-ticker (OHLC, volume, turnover) is reported.
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - a concrete warning about the orchestrator's counter-ranking mechanism (rank on forecastable excess return net of costs, not on index contribution) and a demand that any per-agent reliability weight carry a definition and a sensitivity analysis, with a thin margin treated "as a tie rather than a ranking". Sub-gap 1 - indirect: the paper issues a buy recommendation on a market with documented illiquidity shocks of 8 to 10 basis points and models no spread, no fee, no execution, which is the friction blind spot restated on CSE data.
+EFFECT ON SUB-GAP 2: LEAVES IT OPEN and adds a fourth CSE instance of volatility being ignored entirely rather than measured-and-unused. No conditional variance model on a window opening on the 2008 crisis; no ARCH test; no Ljung-Box. Nothing operationalised. Its only Sub-gap-2 contribution is negative corroboration - it is another CSE paper where constant variance is assumed across a decade the vault's other notes establish is strongly heteroskedastic.
+CSE DATA EVIDENCE: source - "extracted from the CSE database and supplemented with other financial documents". Frequency - daily. Range - stated 2008 to 2017 (abstract inconsistently says 2013 to 2017 for the sector analysis). Tickers - this is the only one of the three CSE papers that touches individual counters: "daily closing prices of nine listed banks", of which only four (NTB, NDB, Sampath, Commercial) appear in the results table - "five of the nine banks are missing from the results table". Plus twenty GICS sector series. Volume - "2,221 price samples classified into 20 sectors". How obtained - CSE database, method unspecified. Critical caveat for the blocker: the note establishes the stated dataset is not what was actually fitted - "The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes... so the series the ARIMA was fitted on is not the series the paper describes", and the BPNN plot's axis range is inconsistent with the ASPI over that decade. So this paper claims ten years of daily per-counter CSE bank prices, but its own printouts contradict its data section, and nothing per-ticker (OHLC, volume, turnover) is reported.
 PROPOSED REVISION STATED IN THE NOTE: none to the four-agent pool or to f(L_t, V_t, P_t, C_{i,t}) directly. The nearest statement bears on C_{i,t}'s reporting standard: "Where my orchestrator produces a per-agent reliability weight, the definition goes in the write-up, the sensitivity of the decision to that weight gets reported, and a margin that thin gets treated as a tie rather than a ranking."</t>
         </is>
       </c>
@@ -5980,9 +5980,9 @@
       <c r="W43" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T (the linear CSE baseline and the horizon constraint on price-only signals), evaluation layer (U2, benchmark discipline, regime-split reporting), and A_V indirectly via the residual-clustering evidence.
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — one concrete design constraint on the orchestrator: the drift collapse caps the horizon at which A_T carries information ("one to three day horizon and essentially none beyond it"), which sets the rebalancing frequency at which price signals can meaningfully be conditioned, and U2 becomes "what decides whether the price-derived agent gets any weight at all on a given day" — i.e. a usable per-day competence input to C_{A_T,t}. Sub-gap 1 — bearing via the friction argument: "a 3.8 point conditional offset on an 81.7 point daily sigma is well inside the friction", which is a concrete CSE-calibrated demonstration that a statistically significant edge can be smaller than the execution cost, and the note commits to attaching a net-of-cost return "using the liquidity-aware slippage model rather than a flat fee".
-EFFECT ON SUB-GAP 2: NARROWS IT SLIGHTLY, by supplying a third independent CSE observation that persistence is there and is being ignored — and by producing the clearest statement in the set of why that matters operationally. The paper measures nothing about volatility; it fits constant variance and its own residual plot shows bands widening by a factor of several across 2020–2022. The note converts this into an argument for the persistence layer: "The residual plot in this paper is my third independent CSE reading of volatility clustering, and it strengthens the case for the persistence layer. Fitted with constant variance and still showing residual bands widening by a factor of several across 2020 to 2022, it lines up with the near-unit persistence in the ARMA-GARCH note and the fractional integration in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]. Three papers, three different specifications, same signal, so conditioning exposure on forecast variance and decay speed rather than on a fixed risk parameter is supported by the local evidence rather than imported from elsewhere." That last clause is the important one for Sub-gap 2: it establishes local evidentiary support for conditioning exposure on decay speed, without the paper itself doing any of it.
-CSE DATA EVIDENCE: source — "the official CSE database, cross-checked against Bloomberg historical series". Frequency — daily. Range — 1 July 2014 to 30 June 2024, ten years, "2,362 usable observations after differencing and lag adjustment", plus a 23-day July 2024 out-of-sample window. Tickers — none; CSE Price Index only, "no individual counters". How obtained — CSE official database with Bloomberg cross-check; tooling EViews 13. This is the longest confirmed clean CSE daily series in the set, and it is index-level. The regime content is documented: "July 2014 to June 2024 deliberately contains the 2019 Easter Sunday attacks, the COVID-19 lockdown low of 4,247.95, the speculative peak of 13,462.39 in January 2022, and the 2022 forex and sovereign crisis."
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - one concrete design constraint on the orchestrator: the drift collapse caps the horizon at which A_T carries information ("one to three day horizon and essentially none beyond it"), which sets the rebalancing frequency at which price signals can meaningfully be conditioned, and U2 becomes "what decides whether the price-derived agent gets any weight at all on a given day" - i.e. a usable per-day competence input to C_{A_T,t}. Sub-gap 1 - bearing via the friction argument: "a 3.8 point conditional offset on an 81.7 point daily sigma is well inside the friction", which is a concrete CSE-calibrated demonstration that a statistically significant edge can be smaller than the execution cost, and the note commits to attaching a net-of-cost return "using the liquidity-aware slippage model rather than a flat fee".
+EFFECT ON SUB-GAP 2: NARROWS IT SLIGHTLY, by supplying a third independent CSE observation that persistence is there and is being ignored - and by producing the clearest statement in the set of why that matters operationally. The paper measures nothing about volatility; it fits constant variance and its own residual plot shows bands widening by a factor of several across 2020–2022. The note converts this into an argument for the persistence layer: "The residual plot in this paper is my third independent CSE reading of volatility clustering, and it strengthens the case for the persistence layer. Fitted with constant variance and still showing residual bands widening by a factor of several across 2020 to 2022, it lines up with the near-unit persistence in the ARMA-GARCH note and the fractional integration in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]. Three papers, three different specifications, same signal, so conditioning exposure on forecast variance and decay speed rather than on a fixed risk parameter is supported by the local evidence rather than imported from elsewhere." That last clause is the important one for Sub-gap 2: it establishes local evidentiary support for conditioning exposure on decay speed, without the paper itself doing any of it.
+CSE DATA EVIDENCE: source - "the official CSE database, cross-checked against Bloomberg historical series". Frequency - daily. Range - 1 July 2014 to 30 June 2024, ten years, "2,362 usable observations after differencing and lag adjustment", plus a 23-day July 2024 out-of-sample window. Tickers - none; CSE Price Index only, "no individual counters". How obtained - CSE official database with Bloomberg cross-check; tooling EViews 13. This is the longest confirmed clean CSE daily series in the set, and it is index-level. The regime content is documented: "July 2014 to June 2024 deliberately contains the 2019 Easter Sunday attacks, the COVID-19 lockdown low of 4,247.95, the speculative peak of 13,462.39 in January 2022, and the 2022 forex and sovereign crisis."
 PROPOSED REVISION STATED IN THE NOTE: no change to the agent pool. On the conditioning set and on C_{i,t}, verbatim: "Every forecasting number my system reports gets this alongside it, computed per counter, and the same quantity is what decides whether the price-derived agent gets any weight at all on a given day." Also a constraint on the orchestrator's operating frequency: "That sets the rebalancing frequency my orchestrator can meaningfully condition price signals at, and it means multi-day forecast horizons from the technical agent should be produced one step at a time against realised data rather than dynamically."</t>
         </is>
       </c>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>US ETFs — VTI (stock), AGG (bond), DBC (commodity), VIX (volatility).  portfolio optimisation / deep learning.</t>
+          <t>US ETFs - VTI (stock), AGG (bond), DBC (commodity), VIX (volatility). portfolio optimisation / deep learning.</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="N44" s="11" t="inlineStr">
         <is>
-          <t>none. VOLATILITY &amp; RISK HANDLING — THIS PAPER OPERATIONALISES A VOLATILITY ESTIMATE INTO AN ALLOCATION, AND IT IS THE SINGLE MOST IMPORTANT FACT IN THIS WHOLE SET FOR SUB-GAP 2. Mechanism, stated exactly: positions are multiplied by the scaling ratio σ_tgt/σ_{i,t-1}, where σ_tgt = 0.10 is a target volatility and "σ_{i,t-1} is an ex-ante volatility estimate for asset i, an exponentially weighted moving standard deviation over a 50-day window on r_{i,t}". So a per-asset volatility estimate directly scales the exposure of each sleeve every day. Two consequences the note draws out: "The scaling ratio sits inside the turnover term, so a move in σ_{i,t-1} generates a trade even when the learned weight has not changed at all, which means the volatility estimator is a source of turnover in its own right. And the scaler is applied at test time only, so the policy is never trained against the positions it is actually evaluated on." Scaling also equalises realised return standard deviation at roughly 0.105 across all eight methods, which is what makes the Sharpe comparison fair. Crucially, the crisis protection is attributable to this non-learned scaler rather than to the learned policy: "the original positions did not change much and the scaled positions decreased a lot for the bond index because volatility spiked. So the learned policy stayed in the falling asset and the exposure came down because σ_{i,t-1} rose, which is a non-learned component of the test-time pipeline doing the de-risking." What is absent: no persistence parameter, no long memory, no decay schedule. The estimator is EWMA, i.e. exponential decay by assumption. The authors themselves flag the weakness: "the conclusion notes that these volatility estimates are lagged and do not necessarily represent current market volatilities, proposing to infer forward volatility inside the network as future work."</t>
+          <t>none. VOLATILITY &amp; RISK HANDLING - THIS PAPER OPERATIONALISES A VOLATILITY ESTIMATE INTO AN ALLOCATION, AND IT IS THE SINGLE MOST IMPORTANT FACT IN THIS WHOLE SET FOR SUB-GAP 2. Mechanism, stated exactly: positions are multiplied by the scaling ratio σ_tgt/σ_{i,t-1}, where σ_tgt = 0.10 is a target volatility and "σ_{i,t-1} is an ex-ante volatility estimate for asset i, an exponentially weighted moving standard deviation over a 50-day window on r_{i,t}". So a per-asset volatility estimate directly scales the exposure of each sleeve every day. Two consequences the note draws out: "The scaling ratio sits inside the turnover term, so a move in σ_{i,t-1} generates a trade even when the learned weight has not changed at all, which means the volatility estimator is a source of turnover in its own right. And the scaler is applied at test time only, so the policy is never trained against the positions it is actually evaluated on." Scaling also equalises realised return standard deviation at roughly 0.105 across all eight methods, which is what makes the Sharpe comparison fair. Crucially, the crisis protection is attributable to this non-learned scaler rather than to the learned policy: "the original positions did not change much and the scaled positions decreased a lot for the bond index because volatility spiked. So the learned policy stayed in the falling asset and the exposure came down because σ_{i,t-1} rose, which is a non-learned component of the test-time pipeline doing the de-risking." What is absent: no persistence parameter, no long memory, no decay schedule. The estimator is EWMA, i.e. exponential decay by assumption. The authors themselves flag the weakness: "the conclusion notes that these volatility estimates are lagged and do not necessarily represent current market volatilities, proposing to infer forward volatility inside the network as future work."</t>
         </is>
       </c>
       <c r="O44" s="11" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="R44" s="11" t="inlineStr">
         <is>
-          <t>seven baselines — four annually rebalanced fixed allocations (25/25/25/25, 50/10/20/20, 10/50/20/20, 40/40/10/10), mean-variance, maximum diversification (both on a rolling 50-day window updated daily), and the diversity-weighted portfolio from Stochastic Portfolio Theory. Everything run at two cost rates, with and without volatility scaling. Metrics: Sharpe, Sortino, MDD, % positive returns, average gain/average loss.</t>
+          <t>seven baselines - four annually rebalanced fixed allocations (25/25/25/25, 50/10/20/20, 10/50/20/20, 40/40/10/10), mean-variance, maximum diversification (both on a rolling 50-day window updated daily), and the diversity-weighted portfolio from Stochastic Portfolio Theory. Everything run at two cost rates, with and without volatility scaling. Metrics: Sharpe, Sortino, MDD, % positive returns, average gain/average loss.</t>
         </is>
       </c>
       <c r="S44" s="11" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="U44" s="11" t="inlineStr">
         <is>
-          <t>it as the minimal control; the objective as the hook — "Any differentiable function of realised returns slots into L_T... That is the direct hook for my orchestration gap, because a term that penalises exposure as a function of measured illiquidity, and a term that decays permitted exposure according to forecast variance and persistence together, are both differentiable functions of realised returns and observable state. Framed that way my contribution is a conditioned objective inside a known training scheme rather than a new architecture, which is a much easier claim to defend and a much easier thing to build." The cost sweep as protocol. The sensitivity measure as a diagnostic for whether orchestrator weights actually move. The short-lookback prior for a short-history market. DWP's collapse as a baseline lesson.</t>
+          <t>it as the minimal control; the objective as the hook - "Any differentiable function of realised returns slots into L_T... That is the direct hook for my orchestration gap, because a term that penalises exposure as a function of measured illiquidity, and a term that decays permitted exposure according to forecast variance and persistence together, are both differentiable functions of realised returns and observable state. Framed that way my contribution is a conditioned objective inside a known training scheme rather than a new architecture, which is a much easier claim to defend and a much easier thing to build." The cost sweep as protocol. The sensitivity measure as a diagnostic for whether orchestrator weights actually move. The short-lookback prior for a short-history market. DWP's collapse as a baseline lesson.</t>
         </is>
       </c>
       <c r="V44" s="11" t="inlineStr">
@@ -6106,8 +6106,8 @@
       <c r="W44" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_V above all (the volatility scaler is the component Sub-gap 2 corrects), plus orchestrator (the conditioned-objective framing, the sensitivity diagnostic) and evaluation layer (cost sweep, baseline table).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — substantial. It gives the orchestration contribution its cheapest possible framing ("a conditioned objective inside a known training scheme rather than a new architecture"), supplies the differentiable slot where liquidity and persistence terms attach, and provides the sensitivity measure S_i as a diagnostic that a mechanism sold as adaptive is actually varying. It is also the designated ablation control — "if a four-agent orchestrator cannot beat a plain differentiable Sharpe maximiser on the same universe and the same costs, that is something I want to find in my own ablation rather than in a viva." Sub-gap 1 — direct and important. The cost sweep (1 bps vs 10 bps) nearly inverts the ranking, and the note draws the CSE conclusion: "at a CSE-plausible round-trip cost the daily-rebalanced version of this design is probably dominated by an annual reallocation rule. Two responses follow, rebalance less often and treat the frequency as a searched parameter rather than a fixed daily choice, or bring the cost term inside the objective using the closed-form transaction remainder factor from Guo et al. so the optimiser trades off predicted return against cost rather than paying it afterwards." The four-paper cost comparison table (Zhang 1/10 bps swept; FreQuant 33/40 bps unswept; Guo 5 bps unswept; Kashif &amp; Ślepaczuk 2 bps unswept) is the note's positioning device for Sub-gap 1: "the only paper that varies its cost assumption is the one with the crudest cost model, which is the gap my own protocol sits in."
-EFFECT ON SUB-GAP 2: THIS IS THE ONE PAPER IN THE SET THAT OPERATIONALISES A VOLATILITY ESTIMATE INTO AN ALLOCATION, AND IT MUST BE FLAGGED PROMINENTLY. Mechanism: every position is multiplied by σ_tgt/σ_{i,t-1}, σ_tgt = 0.10, σ_{i,t-1} an exponentially weighted moving standard deviation over a 50-day window of daily returns; the scaled position is what is traded, what is costed, and what generates turnover. Empirically it is doing most of the risk work — it lifts Allocation 1 from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120, and it, not the learned policy, produced the COVID de-risking. So the paper CLOSES the weaker version of Sub-gap 2 ("a volatility estimate is never fed into a decision") outright, and thereby FORCES the sub-gap into its narrower, defensible form. What it leaves open is exactly the persistence dimension: the estimator is EWMA, "An EWMA estimator assumes shocks decay exponentially, which is precisely the assumption the long-memory result in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] contradicts for the CSE, and the consequence is concrete: after a shock the scaler re-levers on a schedule that is too fast, so exposure returns while the shock is still decaying hyperbolically." The note's proposed correction is the sub-gap in mechanism form: "Pairing a forecast conditional variance with a persistence estimate to set a decay schedule on the scaling ratio is an answer to their stated future work and is testable on their own four-ETF setup before I touch CSE data at all." The authors themselves concede the opening: their conclusion "notes that these volatility estimates are lagged and do not necessarily represent current market volatilities, proposing to infer forward volatility inside the network as future work." So: level of volatility → operationalised. Persistence/decay speed of volatility → still not operationalised, and now with a named component to attach it to and a testbed to test it on.
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - substantial. It gives the orchestration contribution its cheapest possible framing ("a conditioned objective inside a known training scheme rather than a new architecture"), supplies the differentiable slot where liquidity and persistence terms attach, and provides the sensitivity measure S_i as a diagnostic that a mechanism sold as adaptive is actually varying. It is also the designated ablation control - "if a four-agent orchestrator cannot beat a plain differentiable Sharpe maximiser on the same universe and the same costs, that is something I want to find in my own ablation rather than in a viva." Sub-gap 1 - direct and important. The cost sweep (1 bps vs 10 bps) nearly inverts the ranking, and the note draws the CSE conclusion: "at a CSE-plausible round-trip cost the daily-rebalanced version of this design is probably dominated by an annual reallocation rule. Two responses follow, rebalance less often and treat the frequency as a searched parameter rather than a fixed daily choice, or bring the cost term inside the objective using the closed-form transaction remainder factor from Guo et al. so the optimiser trades off predicted return against cost rather than paying it afterwards." The four-paper cost comparison table (Zhang 1/10 bps swept; FreQuant 33/40 bps unswept; Guo 5 bps unswept; Kashif &amp; Ślepaczuk 2 bps unswept) is the note's positioning device for Sub-gap 1: "the only paper that varies its cost assumption is the one with the crudest cost model, which is the gap my own protocol sits in."
+EFFECT ON SUB-GAP 2: THIS IS THE ONE PAPER IN THE SET THAT OPERATIONALISES A VOLATILITY ESTIMATE INTO AN ALLOCATION, AND IT MUST BE FLAGGED PROMINENTLY. Mechanism: every position is multiplied by σ_tgt/σ_{i,t-1}, σ_tgt = 0.10, σ_{i,t-1} an exponentially weighted moving standard deviation over a 50-day window of daily returns; the scaled position is what is traded, what is costed, and what generates turnover. Empirically it is doing most of the risk work - it lifts Allocation 1 from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120, and it, not the learned policy, produced the COVID de-risking. So the paper CLOSES the weaker version of Sub-gap 2 ("a volatility estimate is never fed into a decision") outright, and thereby FORCES the sub-gap into its narrower, defensible form. What it leaves open is exactly the persistence dimension: the estimator is EWMA, "An EWMA estimator assumes shocks decay exponentially, which is precisely the assumption the long-memory result in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] contradicts for the CSE, and the consequence is concrete: after a shock the scaler re-levers on a schedule that is too fast, so exposure returns while the shock is still decaying hyperbolically." The note's proposed correction is the sub-gap in mechanism form: "Pairing a forecast conditional variance with a persistence estimate to set a decay schedule on the scaling ratio is an answer to their stated future work and is testable on their own four-ETF setup before I touch CSE data at all." The authors themselves concede the opening: their conclusion "notes that these volatility estimates are lagged and do not necessarily represent current market volatilities, proposing to infer forward volatility inside the network as future work." So: level of volatility → operationalised. Persistence/decay speed of volatility → still not operationalised, and now with a named component to attach it to and a testbed to test it on.
 CSE DATA EVIDENCE: not a CSE paper, but it carries the most direct statement about the data blocker in the set: "A single 64-unit LSTM over a 400-dimensional input with a softmax head and no reward engineering, no replay buffer and no critic is the smallest end-to-end allocator I have found, which matters directly given that the only confirmed ready-made CSE set covers roughly a year of daily data." Also: "on a roughly 240-day CSE sample a shorter window is doubly attractive because it also increases the number of usable training observations." And a scoping caveat: "the CSE has no liquid commodity ETF, no volatility index and a government bond market that is not accessible on the same terms. What is tradable is equities plus cash, so the diversification has to come from counter and sector selection inside one asset class, which is the correlated case the paper explicitly says to avoid."
 PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On the conditioning set / objective, verbatim: "a term that penalises exposure as a function of measured illiquidity, and a term that decays permitted exposure according to forecast variance and persistence together, are both differentiable functions of realised returns and observable state. Framed that way my contribution is a conditioned objective inside a known training scheme rather than a new architecture." And on P_t and V_t jointly: "Pairing a forecast conditional variance with a persistence estimate to set a decay schedule on the scaling ratio is an answer to their stated future work and is testable on their own four-ETF setup before I touch CSE data at all." Plus an open parameter item: "Pinning the smallest window that still gives a stable volatility estimate is the same open item already sitting against SEMA's (w, d) pair from Guo et al., so the two resolve in one experiment."</t>
         </is>
@@ -6166,7 +6166,7 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>a single feature, the standardised one-day return, sequence length 240. Standardisation R̃^{m,s}_t = (R^{m,s}_t − μ^m_train)/σ^m_train, moments from the training portion only — "footnoted as key in order to avoid look-ahead biases."</t>
+          <t>a single feature, the standardised one-day return, sequence length 240. Standardisation R̃^{m,s}_t = (R^{m,s}_t − μ^m_train)/σ^m_train, moments from the training portion only - "footnoted as key in order to avoid look-ahead biases."</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>none — and that absence is the note's central exhibit for the main gap.</t>
+          <t>none - and that absence is the note's central exhibit for the main gap.</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
@@ -6191,7 +6191,7 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t>no volatility model. Volatility appears only descriptively, as a property of what the network selects: selected stocks "sit at higher 240-day rolling volatility of 0.0303 against 0.0213, higher kurtosis of 5.81 against 4.80, and a market beta of 1.19 against 1.05, with the effect strengthening as k shrinks." Risk control is structural rather than modelled — it comes from the long-short construction, which yields "a market beta of −0.0023 that is not significantly different from zero." No conditional variance, no persistence, no exposure scaling, no risk budget.</t>
+          <t>no volatility model. Volatility appears only descriptively, as a property of what the network selects: selected stocks "sit at higher 240-day rolling volatility of 0.0303 against 0.0213, higher kurtosis of 5.81 against 4.80, and a market beta of 1.19 against 1.05, with the effect strengthening as k shrinks." Risk control is structural rather than modelled - it comes from the long-short construction, which yields "a market beta of −0.0023 that is not significantly different from zero." No conditional variance, no persistence, no exposure scaling, no risk budget.</t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="Q45" s="3" t="inlineStr">
         <is>
-          <t>a two-step template — characterise the selected set with descriptive statistics and factor loadings, then build the simplest transparent rule reproducing the dominant pattern and report what fraction of the return it captures. "Fifty percent from a five-day reversal rule says more about what the model learned than any saliency map and costs nothing beyond statistics I am computing anyway."</t>
+          <t>a two-step template - characterise the selected set with descriptive statistics and factor loadings, then build the simplest transparent rule reproducing the dominant pattern and report what fraction of the return it captures. "Fifty percent from a five-day reversal rule says more about what the model learned than any saliency map and costs nothing beyond statistics I am computing anyway."</t>
         </is>
       </c>
       <c r="R45" s="3" t="inlineStr">
@@ -6232,9 +6232,9 @@
       <c r="W45" s="3" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T (this is the specification for the technical agent), orchestrator (Figure 5 is the main gap's empirical exhibit; C_{A_T,t} design), A_L and A_V (the selection-bias argument for why they are agents rather than post-processing), evaluation layer (the execution ladder).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — this is the strongest published evidence in the set. "Figure 5 is the best single piece of published evidence I have for the main gap, and I should cite it as such. Two heterogeneous predictors trained on identical data, one winning 1993 to 2000, the other winning decisively through 2008, the first winning again 2010 to 2015 by virtue of losing less, with no mechanism anywhere in the design to shift weight between them. A static equal blend would have been beaten by one of its own members in each of the three eras, and a state-conditional blend is exactly what my orchestrator is. This is stronger than the FinAgent and AlphaAgents cases I have been leaning on, because those are failures of a component that should have been switched off, whereas here both components are genuinely useful and the useful one changes." It also dictates evaluation shape: "report the three-way weighting comparison per era or per volatility regime, not only in aggregate, since an aggregate hides exactly this pattern." Sub-gap 1 — strong bearing. The k-depth reversal locates the edge "concentrated in the extreme tails of its own ranking, which is precisely where a thin market cannot absorb the trade". The execution ladder quantifies what realism costs on the most liquid market in the world (53.76 → 20.52 percent annualised), and the note adapts it: the one-day-waiting variant becomes "the cheap test for whether an apparent reversal signal is bid-ask bounce... a validity check rather than a robustness afterthought", with the VWAP leg conditional on intraday CSE data that has not been confirmed to exist. And the selection bias makes liquidity a constraint on the agent rather than a downstream cost: "the liquidity channel is not only a cost model downstream of the decision, it is a constraint on the technical agent's selection, one measurement serving both."
-EFFECT ON SUB-GAP 2: LEAVES IT OPEN, and — importantly — the note argues this paper makes Sub-gap 2 *more* load-bearing under transfer rather than less. No volatility is modelled anywhere; volatility enters only as a descriptive property of the selected set (240-day rolling volatility 0.0303 vs cross-sectional 0.0213). The risk control in the source paper is the long-short construction, which delivers beta −0.0023. Transfer to the CSE destroys it: "Short selling is not practically available on the CSE, so the implementable version is long top k only, which drops the short contribution of 0.0017 out of 0.0046 daily before costs and, more importantly, destroys the market neutrality behind the market beta of −0.0023. A long-only book whose constituents average a beta of 1.19 is a leveraged bet on the ASPI wearing a machine learning label, and the alpha claim collapses into a factor exposure unless something else carries the risk control. That something is the volatility and persistence conditioning, which the short leg was silently providing here, so the transfer makes A_V load-bearing in a way it is not in the source paper." And on persistence specifically: "a strategy that buys recent crashes is buying into elevated conditional variance, and if shocks on the ASPI decay hyperbolically as [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] reports, the exposure schedule after a shock is the difference between a reversal trade and catching a falling counter." That sentence is the clearest statement in the whole set of what operationalised persistence is *for*: the post-shock exposure schedule.
-CSE DATA EVIDENCE: not a CSE paper, but it contains the most constructive reframing of the data blocker in the entire set. "Cross-sectional pooling is the answer to the data-depth blocker, and it also sizes the network." N_seq = Σ_s (T_s − L + 1). "At L = 240 on the confirmed February 2025 to February 2026 set, T_s ≈ L and the whole exercise yields about one sequence per counter, so the paper's own sequence length is unusable here and there is no way around that. At L = 30 with T_s ≈ 240 and a couple of hundred tradable counters, the same expression gives on the order of 40,000 to 50,000 sequences, within an order of magnitude of what this paper trains on. The short history is survivable only because the cross-section is the sample, which reframes the data problem from one about years of history to one about how many counters clear a liquidity screen, a question I can answer from what I already have." Note the confirmed CSE set is named here as February 2025 to February 2026 — roughly one year, T_s ≈ 240 trading days. Network sizing follows: "at roughly 93 examples per parameter and 45,000 sequences the budget is near 500 parameters, and solving 4(h(i+h+1)) + 2h + 2 for i=1 puts h at about ten to twelve hidden units against their twenty-five." Also a required CSE-specific data-quality step: "I need a trading-day filter dropping counters with no genuine print before the median is computed, and the count that filter removes on an average day is itself a liquidity statistic worth reporting."
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - this is the strongest published evidence in the set. "Figure 5 is the best single piece of published evidence I have for the main gap, and I should cite it as such. Two heterogeneous predictors trained on identical data, one winning 1993 to 2000, the other winning decisively through 2008, the first winning again 2010 to 2015 by virtue of losing less, with no mechanism anywhere in the design to shift weight between them. A static equal blend would have been beaten by one of its own members in each of the three eras, and a state-conditional blend is exactly what my orchestrator is. This is stronger than the FinAgent and AlphaAgents cases I have been leaning on, because those are failures of a component that should have been switched off, whereas here both components are genuinely useful and the useful one changes." It also dictates evaluation shape: "report the three-way weighting comparison per era or per volatility regime, not only in aggregate, since an aggregate hides exactly this pattern." Sub-gap 1 - strong bearing. The k-depth reversal locates the edge "concentrated in the extreme tails of its own ranking, which is precisely where a thin market cannot absorb the trade". The execution ladder quantifies what realism costs on the most liquid market in the world (53.76 → 20.52 percent annualised), and the note adapts it: the one-day-waiting variant becomes "the cheap test for whether an apparent reversal signal is bid-ask bounce... a validity check rather than a robustness afterthought", with the VWAP leg conditional on intraday CSE data that has not been confirmed to exist. And the selection bias makes liquidity a constraint on the agent rather than a downstream cost: "the liquidity channel is not only a cost model downstream of the decision, it is a constraint on the technical agent's selection, one measurement serving both."
+EFFECT ON SUB-GAP 2: LEAVES IT OPEN, and - importantly - the note argues this paper makes Sub-gap 2 *more* load-bearing under transfer rather than less. No volatility is modelled anywhere; volatility enters only as a descriptive property of the selected set (240-day rolling volatility 0.0303 vs cross-sectional 0.0213). The risk control in the source paper is the long-short construction, which delivers beta −0.0023. Transfer to the CSE destroys it: "Short selling is not practically available on the CSE, so the implementable version is long top k only, which drops the short contribution of 0.0017 out of 0.0046 daily before costs and, more importantly, destroys the market neutrality behind the market beta of −0.0023. A long-only book whose constituents average a beta of 1.19 is a leveraged bet on the ASPI wearing a machine learning label, and the alpha claim collapses into a factor exposure unless something else carries the risk control. That something is the volatility and persistence conditioning, which the short leg was silently providing here, so the transfer makes A_V load-bearing in a way it is not in the source paper." And on persistence specifically: "a strategy that buys recent crashes is buying into elevated conditional variance, and if shocks on the ASPI decay hyperbolically as [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] reports, the exposure schedule after a shock is the difference between a reversal trade and catching a falling counter." That sentence is the clearest statement in the whole set of what operationalised persistence is *for*: the post-shock exposure schedule.
+CSE DATA EVIDENCE: not a CSE paper, but it contains the most constructive reframing of the data blocker in the entire set. "Cross-sectional pooling is the answer to the data-depth blocker, and it also sizes the network." N_seq = Σ_s (T_s − L + 1). "At L = 240 on the confirmed February 2025 to February 2026 set, T_s ≈ L and the whole exercise yields about one sequence per counter, so the paper's own sequence length is unusable here and there is no way around that. At L = 30 with T_s ≈ 240 and a couple of hundred tradable counters, the same expression gives on the order of 40,000 to 50,000 sequences, within an order of magnitude of what this paper trains on. The short history is survivable only because the cross-section is the sample, which reframes the data problem from one about years of history to one about how many counters clear a liquidity screen, a question I can answer from what I already have." Note the confirmed CSE set is named here as February 2025 to February 2026 - roughly one year, T_s ≈ 240 trading days. Network sizing follows: "at roughly 93 examples per parameter and 45,000 sequences the budget is near 500 parameters, and solving 4(h(i+h+1)) + 2h + 2 for i=1 puts h at about ten to twelve hidden units against their twenty-five." Also a required CSE-specific data-quality step: "I need a trading-day filter dropping counters with no genuine print before the median is computed, and the count that filter removes on an average day is itself a liquidity statistic worth reporting."
 PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool, but an explicit defence of A_L and A_V as separate agents rather than post-processing: "The model's selection bias is the argument for why A_L and A_V are separate agents rather than post-processing." On C_{i,t}, verbatim and important: "Softmax confidence is the obvious candidate for C_{A_T,t} and this paper gives me no grounds to trust it. The probability is used ordinally and never calibrated, and the 2010 to 2015 stretch is the case that worries me, since there is no reason to expect a network to become less confident when its edge is arbitraged away rather than simply wrong more often. So the technical agent's confidence should be a rolling realised accuracy over a trailing out-of-sample window, conditioned on the liquidity and volatility state, rather than the model's own score, and using the score instead has to be earned with a reliability diagram on my own data. The same question recurs for every agent that emits a confidence and it is the part of C_{i,t} I have least evidence about, so writing it down as unresolved is more useful right now than picking one."</t>
         </is>
       </c>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>six indices — SP500, NI225, XU100, KOSPI, DAX, FTSE100.  ensemble ML with XAI-based reject option.</t>
+          <t>six indices - SP500, NI225, XU100, KOSPI, DAX, FTSE100. ensemble ML with XAI-based reject option.</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
@@ -6297,12 +6297,12 @@
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>Stage 1 — one ANN regressor per IMF (two hidden layers of 100 ReLU nodes, 300 epochs, mini-batch 30, tanh output, MSE, Adam) plus one ANN classifier on IMF0 (sigmoid, binary cross-entropy). Stage 2 — random forest, 250 trees, max depth 37, two input features: d_t(ŷ) = ŷ_t − ŷ_{t-1} (signed magnitude) and σ̂_t(x), the raw untresholded sigmoid output of ANNC on IMF0. LIME then explains each forest prediction: explanation(x) = argmin_{g∈G} L(f, g, Π_x(z)) + Ω(g).  two-stage stack → binary direction, plus a reliability score. Decision rule (the note's own formalisation): cover(τ) = (1/T) Σ_t 1[max_c p_c(x_t) ≥ τ]; acc(τ) = Σ_t 1[ŷ_t = y_t] 1[max_c p_c(x_t) ≥ τ] / Σ_t 1[max_c p_c(x_t) ≥ τ].</t>
+          <t>Stage 1 - one ANN regressor per IMF (two hidden layers of 100 ReLU nodes, 300 epochs, mini-batch 30, tanh output, MSE, Adam) plus one ANN classifier on IMF0 (sigmoid, binary cross-entropy). Stage 2 - random forest, 250 trees, max depth 37, two input features: d_t(ŷ) = ŷ_t − ŷ_{t-1} (signed magnitude) and σ̂_t(x), the raw untresholded sigmoid output of ANNC on IMF0. LIME then explains each forest prediction: explanation(x) = argmin_{g∈G} L(f, g, Π_x(z)) + Ω(g). two-stage stack → binary direction, plus a reliability score. Decision rule (the note's own formalisation): cover(τ) = (1/T) Σ_t 1[max_c p_c(x_t) ≥ τ]; acc(τ) = Σ_t 1[ŷ_t = y_t] 1[max_c p_c(x_t) ≥ τ] / Σ_t 1[max_c p_c(x_t) ≥ τ].</t>
         </is>
       </c>
       <c r="L46" s="11" t="inlineStr">
         <is>
-          <t>none in the multi-agent sense, but a two-stage combiner where each upstream component is compressed to two scalars before the combiner sees it — which the note reads as an orchestration-adjacent pattern.</t>
+          <t>none in the multi-agent sense, but a two-stage combiner where each upstream component is compressed to two scalars before the combiner sees it - which the note reads as an orchestration-adjacent pattern.</t>
         </is>
       </c>
       <c r="M46" s="11" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="Q46" s="11" t="inlineStr">
         <is>
-          <t>the centre of the paper, and unusually, load-bearing rather than decorative — "Explainability here earns its place by doing work, not by satisfying a regulator." The LIME surrogate's class probabilities become the reliability score, and the threshold is "a decision-maker's dial rather than a model property".</t>
+          <t>the centre of the paper, and unusually, load-bearing rather than decorative - "Explainability here earns its place by doing work, not by satisfying a regulator." The LIME surrogate's class probabilities become the reliability score, and the threshold is "a decision-maker's dial rather than a model property".</t>
         </is>
       </c>
       <c r="R46" s="11" t="inlineStr">
@@ -6358,10 +6358,10 @@
       <c r="W46" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator above all (abstention, and the common confidence scale for C_{i,t}), evaluation layer (coverage/accuracy pairing; the expectation band for honest CSE directional accuracy), A_L (the abstention-as-liquidity-screen check), A_T (the expectation band and the leak warning).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap — this is the single most directly useful paper in the set for the orchestration argument's second half. "My orchestration argument has always had two parts, that an agent's reliability varies with conditions and that the agents do not know it, and the second part is the one with no published mechanism behind it. AlphaAgents deleted its sentiment agent by hand and FinAgent's auxiliary strategies degraded quietly on ETHUSD, both because nothing in either design could decline to speak. This paper declines to speak, measures what declining costs, and publishes the frontier." It also supplies a concrete route to the comparable-confidence problem in C_{i,t}: "the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not." And it names precisely what must not be copied: "What I cannot borrow is the combiner itself, since a forest over two static features has no channel for liquidity state or volatility persistence and therefore reproduces exactly the fixed-influence design the main gap objects to, the same structural limitation as the near-binary mixture in [[MacroHFT...]]. The compression is the reusable part, the conditioning is mine to add." Sub-gap 1 — real bearing via the abstention-as-liquidity-screen problem: "On the CSE, an abstention threshold is partly a liquidity screen and I need to say which... the counters clearing a confidence bar are very likely the ones printing densely... So the check is to regress trusted-day frequency per counter on Amihud illiquidity and turnover before claiming the threshold is measuring confidence, which is the same measurement already being computed for the cost model, serving a third purpose." Plus the exposure policy on abstained days: "The abstained days also need an explicit exposure policy, hold the previous position or go flat, since those are different strategies and on the CSE the flat option carries a round-trip cost each time."
-EFFECT ON SUB-GAP 2: LEAVES IT OPEN. There is no volatility quantity anywhere in this paper, so nothing is operationalised in the persistence direction. Its relevance is oblique but real in one respect: it is the only paper in the set where a *confidence* quantity is operationalised into a decision (trade or abstain), which is the structural template Sub-gap 2 needs for its own quantity — a measured scalar that gates action rather than describing it. The note's own framing of the missing economic check is also the Sub-gap-2-adjacent worry in reverse: abstention may be selecting low-volatility days, and the authors do not check it, so the interaction between the confidence filter and the volatility state is unexamined in exactly the way Sub-gap 2 says volatility states go unexamined.
-CSE DATA EVIDENCE: not a CSE paper. Two CSE-relevant implications: the coverage curve doubles as a measurement of how often a channel is live ("the coverage curve for the sentiment agent on CSE counters is directly the measurement of how often that channel is actually live"), and a calibrated expectation band is set — "my expectation band for a technical agent on CSE daily direction is somewhere near 0.54 to 0.58 on honest out-of-sample data, and a result above about 0.65 is a prompt to hunt for a leak rather than a success."
-PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On C_{i,t}, verbatim: "Realised conditional accuracy is the common scale for heterogeneous agent confidence, and this paper is the argument for it. The open question in my matrix is how an LLM analyst, an econometric estimator and an RL policy produce comparable confidence numbers, and the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not. It also inherits the calibration problem named above rather than solving it, so the curve has to be re-estimated as conditions move rather than fitted once." Implicitly this adds an abstention channel to the weighting function — w(i,t) should be able to go to zero for an agent on a given day — though the note never writes that as a change to f(·) itself.</t>
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - this is the single most directly useful paper in the set for the orchestration argument's second half. "My orchestration argument has always had two parts, that an agent's reliability varies with conditions and that the agents do not know it, and the second part is the one with no published mechanism behind it. AlphaAgents deleted its sentiment agent by hand and FinAgent's auxiliary strategies degraded quietly on ETHUSD, both because nothing in either design could decline to speak. This paper declines to speak, measures what declining costs, and publishes the frontier." It also supplies a concrete route to the comparable-confidence problem in C_{i,t}: "the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not." And it names precisely what must not be copied: "What I cannot borrow is the combiner itself, since a forest over two static features has no channel for liquidity state or volatility persistence and therefore reproduces exactly the fixed-influence design the main gap objects to, the same structural limitation as the near-binary mixture in [[MacroHFT...]]. The compression is the reusable part, the conditioning is mine to add." Sub-gap 1 - real bearing via the abstention-as-liquidity-screen problem: "On the CSE, an abstention threshold is partly a liquidity screen and I need to say which... the counters clearing a confidence bar are very likely the ones printing densely... So the check is to regress trusted-day frequency per counter on Amihud illiquidity and turnover before claiming the threshold is measuring confidence, which is the same measurement already being computed for the cost model, serving a third purpose." Plus the exposure policy on abstained days: "The abstained days also need an explicit exposure policy, hold the previous position or go flat, since those are different strategies and on the CSE the flat option carries a round-trip cost each time."
+EFFECT ON SUB-GAP 2: LEAVES IT OPEN. There is no volatility quantity anywhere in this paper, so nothing is operationalised in the persistence direction. Its relevance is oblique but real in one respect: it is the only paper in the set where a *confidence* quantity is operationalised into a decision (trade or abstain), which is the structural template Sub-gap 2 needs for its own quantity - a measured scalar that gates action rather than describing it. The note's own framing of the missing economic check is also the Sub-gap-2-adjacent worry in reverse: abstention may be selecting low-volatility days, and the authors do not check it, so the interaction between the confidence filter and the volatility state is unexamined in exactly the way Sub-gap 2 says volatility states go unexamined.
+CSE DATA EVIDENCE: not a CSE paper. Two CSE-relevant implications: the coverage curve doubles as a measurement of how often a channel is live ("the coverage curve for the sentiment agent on CSE counters is directly the measurement of how often that channel is actually live"), and a calibrated expectation band is set - "my expectation band for a technical agent on CSE daily direction is somewhere near 0.54 to 0.58 on honest out-of-sample data, and a result above about 0.65 is a prompt to hunt for a leak rather than a success."
+PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On C_{i,t}, verbatim: "Realised conditional accuracy is the common scale for heterogeneous agent confidence, and this paper is the argument for it. The open question in my matrix is how an LLM analyst, an econometric estimator and an RL policy produce comparable confidence numbers, and the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not. It also inherits the calibration problem named above rather than solving it, so the curve has to be re-estimated as conditions move rather than fitted once." Implicitly this adds an abstention channel to the weighting function - w(i,t) should be able to go to zero for an agent on a given day - though the note never writes that as a change to f(·) itself.</t>
         </is>
       </c>
       <c r="X46" s="11" t="inlineStr">
@@ -6408,17 +6408,17 @@
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>Colombo Stock Exchange (Sri Lanka).  Corporate structure QA over annual reports — directors, auditors, subsidiaries, executives, products, sectors. DATASETS &amp; PERIOD — AND HOW DOCUMENTS WERE OBTAINED: This is the critical intelligence gap. The note is emphatic that almost nothing is reported. "The number of source annual reports is never given, so I cannot tell whether that covers the roughly 280 listed companies or a fraction of them, and the word comprehensively is doing work the paper does not support." Under limitations: "No corpus size, no company or year coverage, no annotated-subset size". No date range is stated anywhere in the note. NO ACQUISITION METHOD IS REPORTED — the note records only that the inputs are "annual report PDFs", and the student's own separate reasoning is that "Annual reports are published artefacts that stay downloadable". The only CSE-data-access lead in the note is the contact lead, not a described method: the authors "are reachable, which also bears on the outstanding question of who to approach about CSE data access." Only coverage figure reported: "The graph holds over 6,000 unique entities across companies, directors, executives, subsidiaries, auditors, products and sectors". Graph is static, no as-of versioning.</t>
+          <t>Colombo Stock Exchange (Sri Lanka). Corporate structure QA over annual reports - directors, auditors, subsidiaries, executives, products, sectors. DATASETS &amp; PERIOD - AND HOW DOCUMENTS WERE OBTAINED: This is the critical intelligence gap. The note is emphatic that almost nothing is reported. "The number of source annual reports is never given, so I cannot tell whether that covers the roughly 280 listed companies or a fraction of them, and the word comprehensively is doing work the paper does not support." Under limitations: "No corpus size, no company or year coverage, no annotated-subset size". No date range is stated anywhere in the note. NO ACQUISITION METHOD IS REPORTED - the note records only that the inputs are "annual report PDFs", and the student's own separate reasoning is that "Annual reports are published artefacts that stay downloadable". The only CSE-data-access lead in the note is the contact lead, not a described method: the authors "are reachable, which also bears on the outstanding question of who to approach about CSE data access." Only coverage figure reported: "The graph holds over 6,000 unique entities across companies, directors, executives, subsidiaries, auditors, products and sectors". Graph is static, no as-of versioning.</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Annual report PDFs from CSE-listed companies. Corpus size, company count and the period covered are not stated in the note. The pipeline constants are: context-aware semantic chunking at a fixed window of roughly 1000 characters preserving paragraph and section boundaries, embedding with Google Text Embedding 004, a 3000-token document budget, top-5 chunk retrieval per query, and a 500-token extraction context window. Each constant arrives as a stated value with no tuning evidence behind it.</t>
         </is>
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>Unstructured text from annual report PDFs only. Entities: companies, directors, executives, subsidiaries, auditors, products, sectors. "Tabular financial data is explicitly not handled, stated in the conclusion and carried into future work as layout-aware parsing." METHOD — EXACT PIPELINE: (1) Chunking: "Annual report PDFs are chunked with a context-aware semantic strategy at a fixed window of roughly 1000 characters, preserving paragraph and section boundaries". (2) Embedding: "each chunk is embedded with Google Text Embedding 004 under a 3000-token input budget per document, into ChromaDB". (3) Extraction LLM: "Gemini 2.5 Pro then runs the extraction, but not over the whole document: it retrieves the top-5 relevant chunks per query and extracts entities into JSON inside a 500-token extraction context window." Student names this as the actual contribution: "question-driven targeted extraction instead of full-document extraction." (4) Consolidation: "Entity names are unified by a custom fuzzy matching pipeline with type-specific similarity functions, strict surname and initials for people, normalised token-sort and word overlap for companies, and then a Human-in-the-Loop clustering interface lets a reviewer merge or split clusters before variants are mapped onto canonical entity nodes". (5) Schema: "a rigid schema of DIRECTS, OWNS, AUDITED_BY and similar", plus entity type DIRECTOR with relationship type HOLDS_POSITION. "The resulting graph is company-centric, a star of typed edges around each listed entity" (Fig. 1 = Dialog Axiata PLC). (6) Retrieval/query: "a LangGraph/LangChain agent that decomposes a complex question into sub-queries, entity lookup then relationship traversal, and applies lightweight self-verification loops that reformulate and retry a sub-query returning incomplete or invalid output." Metric defined: Data Capture = (|{e ∈ E_gt : e extracted}| + |{r ∈ R_gt : r extracted}|) / (|E_gt| + |R_gt|), with "the denominator is never stated numerically anywhere in the paper".</t>
+          <t>Unstructured text from annual report PDFs only. Entities: companies, directors, executives, subsidiaries, auditors, products, sectors. "Tabular financial data is explicitly not handled, stated in the conclusion and carried into future work as layout-aware parsing." METHOD - EXACT PIPELINE: (1) Chunking: "Annual report PDFs are chunked with a context-aware semantic strategy at a fixed window of roughly 1000 characters, preserving paragraph and section boundaries". (2) Embedding: "each chunk is embedded with Google Text Embedding 004 under a 3000-token input budget per document, into ChromaDB". (3) Extraction LLM: "Gemini 2.5 Pro then runs the extraction, but not over the whole document: it retrieves the top-5 relevant chunks per query and extracts entities into JSON inside a 500-token extraction context window." Student names this as the actual contribution: "question-driven targeted extraction instead of full-document extraction." (4) Consolidation: "Entity names are unified by a custom fuzzy matching pipeline with type-specific similarity functions, strict surname and initials for people, normalised token-sort and word overlap for companies, and then a Human-in-the-Loop clustering interface lets a reviewer merge or split clusters before variants are mapped onto canonical entity nodes". (5) Schema: "a rigid schema of DIRECTS, OWNS, AUDITED_BY and similar", plus entity type DIRECTOR with relationship type HOLDS_POSITION. "The resulting graph is company-centric, a star of typed edges around each listed entity" (Fig. 1 = Dialog Axiata PLC). (6) Retrieval/query: "a LangGraph/LangChain agent that decomposes a complex question into sub-queries, entity lookup then relationship traversal, and applies lightweight self-verification loops that reformulate and retry a sub-query returning incomplete or invalid output." Metric defined: Data Capture = (|{e ∈ E_gt : e extracted}| + |{r ∈ R_gt : r extracted}|) / (|E_gt| + |R_gt|), with "the denominator is never stated numerically anywhere in the paper".</t>
         </is>
       </c>
       <c r="K47" s="11" t="inlineStr">
@@ -6453,17 +6453,17 @@
       </c>
       <c r="Q47" s="11" t="inlineStr">
         <is>
-          <t>Implicit — typed graph edges and Cypher are inspectable; self-verification loop produces observable signals. No explicit explainability evaluation.</t>
+          <t>Implicit - typed graph edges and Cypher are inspectable; self-verification loop produces observable signals. No explicit explainability evaluation.</t>
         </is>
       </c>
       <c r="R47" s="11" t="inlineStr">
         <is>
-          <t>Ten hand-written queries with manually extracted ground truth, scored 1–10 for correctness; a "standard RAG" baseline without graph reasoning; a before-and-after on their own pipeline for the capture figure; Data Capture on a manually annotated subset of unstated size. KEY RESULTS (quoted numbers): "Feeding entire reports to the LLM lost roughly 50% of the data to context window limits, while the question-driven retrieval pipeline reached over 85% entity capture on a manually annotated subset." "Graph RAG scored 9.2/10 against 6.1/10 for a standard RAG baseline, a 50% relative improvement, with the largest gains on multi-hop relational queries." "query failure rate fell from around 30% to under 2% once the Neo4j subagent did query decomposition and self-correction retry" — student calls this "the most transferable number". "The graph holds over 6,000 unique entities". LIMITATIONS (quoted): "The evidence base is two pages and cannot be reproduced from what is printed." "Every design choice in the pipeline, 1000-character windows, 3000-token document budget, 500-token extraction window, top-5 retrieval, arrives as a stated constant with no tuning evidence behind it, so I can adopt them as reasonable defaults but not as validated ones." "The comparison does not isolate the graph... a large part of the 9.2 against 6.1 could be the scaffolding rather than the graph, and the paper does not run the intermediate configuration that would tell them apart." "The Data Capture denominator is missing." "Nothing is reported on cost or latency". "The graph is a point-in-time snapshot with no temporal model... For a backtest this is a lookahead hazard rather than an inconvenience." "Ten queries, hand-scored, with no statement of who scored them or whether more than one person did, is an illustration rather than a measurement, and I should carry the direction of this result and not the magnitude." "Fidelity depends on a human in the loop... it never reports how many clusters needed intervention, which is the number that would tell me what a fully automated run costs in accuracy." Warning callout: "Cite this paper for priority and for the pipeline design, not for its numbers. Ten hand-scored queries and an unspecified annotation subset will not survive a viva question about evidence, and if I lean on 9.2 against 6.1 as though it were a benchmark result, the weakness becomes mine rather than theirs."</t>
+          <t>Ten hand-written queries with manually extracted ground truth, scored 1–10 for correctness; a "standard RAG" baseline without graph reasoning; a before-and-after on their own pipeline for the capture figure; Data Capture on a manually annotated subset of unstated size. KEY RESULTS (quoted numbers): "Feeding entire reports to the LLM lost roughly 50% of the data to context window limits, while the question-driven retrieval pipeline reached over 85% entity capture on a manually annotated subset." "Graph RAG scored 9.2/10 against 6.1/10 for a standard RAG baseline, a 50% relative improvement, with the largest gains on multi-hop relational queries." "query failure rate fell from around 30% to under 2% once the Neo4j subagent did query decomposition and self-correction retry" - student calls this "the most transferable number". "The graph holds over 6,000 unique entities". LIMITATIONS (quoted): "The evidence base is two pages and cannot be reproduced from what is printed." "Every design choice in the pipeline, 1000-character windows, 3000-token document budget, 500-token extraction window, top-5 retrieval, arrives as a stated constant with no tuning evidence behind it, so I can adopt them as reasonable defaults but not as validated ones." "The comparison does not isolate the graph... a large part of the 9.2 against 6.1 could be the scaffolding rather than the graph, and the paper does not run the intermediate configuration that would tell them apart." "The Data Capture denominator is missing." "Nothing is reported on cost or latency". "The graph is a point-in-time snapshot with no temporal model... For a backtest this is a lookahead hazard rather than an inconvenience." "Ten queries, hand-scored, with no statement of who scored them or whether more than one person did, is an illustration rather than a measurement, and I should carry the direction of this result and not the magnitude." "Fidelity depends on a human in the loop... it never reports how many clusters needed intervention, which is the number that would tell me what a fully automated run costs in accuracy." Warning callout: "Cite this paper for priority and for the pipeline design, not for its numbers. Ten hand-scored queries and an unspecified annotation subset will not survive a viva question about evidence, and if I lean on 9.2 against 6.1 as though it were a benchmark result, the weakness becomes mine rather than theirs."</t>
         </is>
       </c>
       <c r="S47" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Graph RAG scored 9.2/10 against 6.1/10 for a standard RAG baseline on the authors' own evaluation, a 50% relative improvement, with the largest gains on multi-hop relational queries. Query failure rate fell from around 30% to under 2% once the Neo4j subagent added query decomposition and self-correction retry, which is the number I would actually cite because it is a claim about agent scaffolding rather than about retrieval quality. Entity capture exceeded 85% on a manually annotated subset, against roughly 50% of the data lost to context window limits when whole reports were fed to the LLM. The paper does not run the intermediate configuration that would separate the graph's contribution from the scaffolding's, so the 9.2 against 6.1 cannot be attributed to either alone.</t>
         </is>
       </c>
       <c r="T47" s="11" t="inlineStr">
@@ -6478,13 +6478,13 @@
       </c>
       <c r="V47" s="11" t="inlineStr">
         <is>
-          <t>Numeric financial statement tables. "The paper is explicit that tabular financial data is out of scope and lists layout-aware parsing of tables as future work, so the gap between what it built and what A_F has to be is precisely the part it did not do." Plus: no temporal/as-of model, no cost or latency, no isolation of graph vs scaffolding, no corpus coverage. WHAT THE STUDENT SAYS IT CLOSES: Former G4 (structure-aware retrieval over CSE annual reports as a novelty). "Priority is priority, and structure-aware retrieval over CSE annual reports is now published work from a local group, which is the point the supervisor was making when they said the literature search was incomplete." "This citation is now verified and the unverified flag comes off it in the matrix... Former G4 stays demoted." Also: "that weakness does not give me back the novelty" — the two-page format does NOT reopen the claim. DOES A_F STILL HAVE ANYTHING TO CONTRIBUTE? Yes, but only numerically, not architecturally. Verbatim: "The differentiation for A_F is numeric, not architectural. Competing on graph versus vector retrieval over CSE reports is competing where this paper already is. What it does not do is extract the financial statement tables, and those are what a fundamental agent needs to emit a signal the orchestrator can weigh against a technical or a volatility agent. So A_F should be built on numeric statement extraction, which puts it in MultiFinRAG... and Financial Report Chunking for Effective Retrieval Augmented Generation territory, with the entity graph as an optional grounding layer rather than the main object." The retrieval component itself is prior art; the residual contribution is (a) numeric statement extraction, (b) point-in-time correctness, (c) the orchestration that consumes the signal.</t>
+          <t>Numeric financial statement tables. "The paper is explicit that tabular financial data is out of scope and lists layout-aware parsing of tables as future work, so the gap between what it built and what A_F has to be is precisely the part it did not do." Plus: no temporal/as-of model, no cost or latency, no isolation of graph vs scaffolding, no corpus coverage. WHAT THE STUDENT SAYS IT CLOSES: Former G4 (structure-aware retrieval over CSE annual reports as a novelty). "Priority is priority, and structure-aware retrieval over CSE annual reports is now published work from a local group, which is the point the supervisor was making when they said the literature search was incomplete." "This citation is now verified and the unverified flag comes off it in the matrix... Former G4 stays demoted." Also: "that weakness does not give me back the novelty" - the two-page format does NOT reopen the claim. DOES A_F STILL HAVE ANYTHING TO CONTRIBUTE? Yes, but only numerically, not architecturally. Verbatim: "The differentiation for A_F is numeric, not architectural. Competing on graph versus vector retrieval over CSE reports is competing where this paper already is. What it does not do is extract the financial statement tables, and those are what a fundamental agent needs to emit a signal the orchestrator can weigh against a technical or a volatility agent. So A_F should be built on numeric statement extraction, which puts it in MultiFinRAG... and Financial Report Chunking for Effective Retrieval Augmented Generation territory, with the entity graph as an optional grounding layer rather than the main object." The retrieval component itself is prior art; the residual contribution is (a) numeric statement extraction, (b) point-in-time correctness, (c) the orchestration that consumes the signal.</t>
         </is>
       </c>
       <c r="W47" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_F only (stated explicitly). Secondary bearing on the orchestrator via C_F,t and on the evaluation layer via the ablation-discipline lesson.
-EFFECT ON A_F: Closes the architectural novelty; supports the build by supplying a validated-by-locality default configuration; constrains it by forcing the differentiation onto numeric extraction and by forcing point-in-time design in now ("the fundamental channel needs a publication-date field on every document and a retrieval filter keyed to the simulation clock"). No usable evaluation set or taxonomy for CSE filings is released or described — the annotated subset is unspecified. The only taxonomy on offer is the entity/relationship schema (DIRECTS, OWNS, AUDITED_BY, HOLDS_POSITION), which is structural, not numeric.
+EFFECT ON A_F: Closes the architectural novelty; supports the build by supplying a validated-by-locality default configuration; constrains it by forcing the differentiation onto numeric extraction and by forcing point-in-time design in now ("the fundamental channel needs a publication-date field on every document and a retrieval filter keyed to the simulation clock"). No usable evaluation set or taxonomy for CSE filings is released or described - the annotated subset is unspecified. The only taxonomy on offer is the entity/relationship schema (DIRECTS, OWNS, AUDITED_BY, HOLDS_POSITION), which is structural, not numeric.
 SENTIMENT-RELATED EVIDENCE: None.
 PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool. A concrete proposal for one term of the conditioning set, verbatim: "The self-correction loop suggests a mechanical confidence signal for C_{F,t}. Retrieval-grounded systems produce things an orchestrator can actually observe, whether the generated Cypher validated, how many retries a sub-query needed, whether every claim in the answer traced to a retrieved chunk. That is a very different quantity from an LLM's self-reported confidence and it is comparable across runs. It does not solve the standing problem of making confidence comparable across four heterogeneous producers, but it is the first concrete proposal I have for one of the four, and the fundamental agent is the one where I had least idea what to measure." Also, on A_F's role in justifying state-dependent weights: "A_F is the clearest case in my own design for why weights have to be state-dependent, and its weight trajectory around reporting dates is a natural test for the pre-registered weight-entropy diagnostic."</t>
         </is>
@@ -6533,7 +6533,7 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>US (10 US stocks in FinTrade; ACL18/BigData22/CIKM18 US large caps); EMIR/EU for Regulations.  Cross-cutting — IE, textual analysis, QA, generation, risk management, forecasting, decision-making.</t>
+          <t>US (10 US stocks in FinTrade; ACL18/BigData22/CIKM18 US large caps); EMIR/EU for Regulations. Cross-cutting - IE, textual analysis, QA, generation, risk management, forecasting, decision-making.</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="M48" s="11" t="inlineStr">
         <is>
-          <t>Eight textual-analysis classification tasks (FPB, FiQA-SA, TSA, Headlines, FOMC, FinArg, MultiFin, MA, MLESG). Student's standing rule applied: "Per Scope sentiment analysis dropped the eight textual-analysis classification tasks are read as evidence about evaluation, not as a component to build." FUNDAMENTAL: QA aspect only — FinQA, TATQA, ConvFinQA, Regulations. No fundamental signal construction. RAG HANDLING: This is the headline finding for A_F. "The RAG evaluation claimed as a headline innovation does not exist in the paper... There is no retrieval dataset in Table 2, no retrieval condition in Section 3, no retrieval results in Section 4 and nothing in the appendices. Every task feeds its context directly into the prompt. The agent half of that sentence is delivered through FinMem on FinTrade; the RAG half is asserted and never operationalised. This is the claim I most wanted the paper to support and it is the one that is missing entirely, which means that as of mid-2024 no financial LLM benchmark evaluates retrieval as a variable, and FinanceBench's 19% to 50% under realistic retrieval remains the only number in the reading list that measures it."</t>
+          <t>Eight textual-analysis classification tasks (FPB, FiQA-SA, TSA, Headlines, FOMC, FinArg, MultiFin, MA, MLESG). Student's standing rule applied: "Per Scope sentiment analysis dropped the eight textual-analysis classification tasks are read as evidence about evaluation, not as a component to build." FUNDAMENTAL: QA aspect only - FinQA, TATQA, ConvFinQA, Regulations. No fundamental signal construction. RAG HANDLING: This is the headline finding for A_F. "The RAG evaluation claimed as a headline innovation does not exist in the paper... There is no retrieval dataset in Table 2, no retrieval condition in Section 3, no retrieval results in Section 4 and nothing in the appendices. Every task feeds its context directly into the prompt. The agent half of that sentence is delivered through FinMem on FinTrade; the RAG half is asserted and never operationalised. This is the claim I most wanted the paper to support and it is the one that is missing entirely, which means that as of mid-2024 no financial LLM benchmark evaluates retrieval as a variable, and FinanceBench's 19% to 50% under realistic retrieval remains the only number in the reading list that measures it."</t>
         </is>
       </c>
       <c r="N48" s="11" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="P48" s="11" t="inlineStr">
         <is>
-          <t>None — "one regime on ten US names with no transaction costs modelled".</t>
+          <t>None - "one regime on ten US names with no transaction costs modelled".</t>
         </is>
       </c>
       <c r="Q48" s="11" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="S48" s="11" t="inlineStr">
         <is>
-          <t>Forecasting — "twelve models cluster at accuracy 0.41 to 0.57 with MCC between -0.07 and 0.08, GPT-4 at 0.02, 0.02 and 0.02, Gemini at 0.03, 0.04 and 0.02, and the best single cell anywhere is FinMA 7B's 0.08 on CIKM18. Table 14 then reports SLOT, a 2022 self-supervised sequence model, at MCC 0.10, 0.21 and 0.09, and DTML at 0.07, 0.18 and -0.00." Trading — "GPT-4 reaches cumulative return 28.19% against Buy &amp; Hold's -4.00%, Sharpe 1.51 against 0.02, and maximum drawdown 18.34% against 30.67%, with Gemini second at 14.95% and Sharpe 1.03. Table 5 puts A2C, PPO and DQN at cumulative returns of -4.22%, -0.56% and -2.99% with Sharpe ratios of -0.26, 0.01 and -0.17". But "GPT-4o returns -5.54% at Sharpe -0.19 and llama3-70B returns -2.57% at Sharpe -0.04". QA — "GPT-4's TATQA exact-match accuracy is 0.13 against 0.63 on FinQA". Instruction tuning — "FinMA 7B posts the best scores in the table on FPB at 0.88 and FiQA-SA at 0.88 and Headlines at 0.97, beating GPT-4's 0.78, 0.76 and 0.86, and then scores 0.04 on FinQA, 0.00 on TATQA and 0.00 on ConvFinQA." LIMITATIONS (quoted): "Most of the headline results grid is zero, and the zeros are output-format failures rather than graded capability." "The trading confidence intervals cannot be reproduced from the paper's own per-stock table and the paper never says how they were computed... Recomputing GPT-4 from Table 9 gives mean cumulative return 26.80% and mean Sharpe 1.45 against the reported 28.19% and 1.51, and a cross-sectional interval of roughly ±10.5 on cumulative return against the reported ±25.27". "'Holistic' describes coverage and not measurement, because nothing aggregates." "The leakage machinery exists and is pointed at the wrong models." "The shared-task result the abstract leads on is not what the appendix shows" — winning team Sharpe 0.9268 vs GPT-4's 1.51.</t>
+          <t>Forecasting - "twelve models cluster at accuracy 0.41 to 0.57 with MCC between -0.07 and 0.08, GPT-4 at 0.02, 0.02 and 0.02, Gemini at 0.03, 0.04 and 0.02, and the best single cell anywhere is FinMA 7B's 0.08 on CIKM18. Table 14 then reports SLOT, a 2022 self-supervised sequence model, at MCC 0.10, 0.21 and 0.09, and DTML at 0.07, 0.18 and -0.00." Trading - "GPT-4 reaches cumulative return 28.19% against Buy &amp; Hold's -4.00%, Sharpe 1.51 against 0.02, and maximum drawdown 18.34% against 30.67%, with Gemini second at 14.95% and Sharpe 1.03. Table 5 puts A2C, PPO and DQN at cumulative returns of -4.22%, -0.56% and -2.99% with Sharpe ratios of -0.26, 0.01 and -0.17". But "GPT-4o returns -5.54% at Sharpe -0.19 and llama3-70B returns -2.57% at Sharpe -0.04". QA - "GPT-4's TATQA exact-match accuracy is 0.13 against 0.63 on FinQA". Instruction tuning - "FinMA 7B posts the best scores in the table on FPB at 0.88 and FiQA-SA at 0.88 and Headlines at 0.97, beating GPT-4's 0.78, 0.76 and 0.86, and then scores 0.04 on FinQA, 0.00 on TATQA and 0.00 on ConvFinQA." LIMITATIONS (quoted): "Most of the headline results grid is zero, and the zeros are output-format failures rather than graded capability." "The trading confidence intervals cannot be reproduced from the paper's own per-stock table and the paper never says how they were computed... Recomputing GPT-4 from Table 9 gives mean cumulative return 26.80% and mean Sharpe 1.45 against the reported 28.19% and 1.51, and a cross-sectional interval of roughly ±10.5 on cumulative return against the reported ±25.27". "'Holistic' describes coverage and not measurement, because nothing aggregates." "The leakage machinery exists and is pointed at the wrong models." "The shared-task result the abstract leads on is not what the appendix shows" - winning team Sharpe 0.9268 vs GPT-4's 1.51.</t>
         </is>
       </c>
       <c r="T48" s="11" t="inlineStr">
@@ -6608,9 +6608,9 @@
       </c>
       <c r="W48" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: All four plus orchestrator plus evaluation layer — "it speaks to all four channels at once rather than to one."
+          <t>SPEAKS TO: All four plus orchestrator plus evaluation layer - "it speaks to all four channels at once rather than to one."
 EFFECT ON A_F: Supports and clears the ground. "Retrieval quality is still unbenchmarked in the financial LLM literature, and that is now a positive finding rather than a hole in my reading... there is no external yardstick I can borrow for A_F and no risk that a reviewer points at FinBen as prior coverage of it." Usable as taxonomy: the seven-aspect list as a coverage checklist, and the FinTrade prompt as an output-schema template. Not usable as an evaluation set for CSE filings; the QA numbers it reports for FinQA/ConvFinQA are imported few-shot figures, not its own runs.
-SENTIMENT-RELATED EVIDENCE: Indirect — the 8 textual-analysis tasks read as evidence about evaluation only. The note explicitly cross-cites the temporal-shift paper as the reason FinBen's undated averaging is unsound: "Predict the Future from the Past... shows financial performance degrading measurably as the train-test gap widens, so an average over undated conditions is averaging over regimes that behave differently."
+SENTIMENT-RELATED EVIDENCE: Indirect - the 8 textual-analysis tasks read as evidence about evaluation only. The note explicitly cross-cites the temporal-shift paper as the reason FinBen's undated averaging is unsound: "Predict the Future from the Past... shows financial performance degrading measurably as the train-test gap widens, so an average over undated conditions is averaging over regimes that behave differently."
 PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool. On the orchestrator, verbatim: "the orchestrator has to be able to drive a channel's weight to near zero, which is what the pre-registered weight-entropy diagnostic exists to detect." And on A_T's composition: "A_T is an econometric or RL component with an LLM nowhere in the directional path". On the failure bucket: "the harness needs strict output validation and a logged failure bucket that feeds the weighting function a hard zero."</t>
         </is>
       </c>
@@ -6648,12 +6648,12 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>Open financial LLM stack — instruction data, model, benchmark.</t>
+          <t>Open financial LLM stack - instruction data, model, benchmark.</t>
         </is>
       </c>
       <c r="G49" s="11" t="inlineStr">
         <is>
-          <t>Three gaps — no openly released financial LLM (BloombergGPT closed at every layer); no financial instruction-tuning data; existing benchmarks (FLUE, BBT-CFLEB) evaluate language understanding only with no prediction task.</t>
+          <t>Three gaps - no openly released financial LLM (BloombergGPT closed at every layer); no financial instruction-tuning data; existing benchmarks (FLUE, BBT-CFLEB) evaluate language understanding only with no prediction task.</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>FIT — 128,640 instruction samples from nine open datasets, five task types. FLARE — 15 datasets, six NLP tasks + two prediction tasks, including six datasets FIT never touches (FOMC, FiNER-ORD, ECTSUM, EDTSum, German, Australian). ACL18 covers 2014–2016.</t>
+          <t>FIT - 128,640 instruction samples from nine open datasets, five task types. FLARE - 15 datasets, six NLP tasks + two prediction tasks, including six datasets FIT never touches (FOMC, FiNER-ORD, ECTSUM, EDTSum, German, Australian). ACL18 covers 2014–2016.</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
@@ -6673,7 +6673,7 @@
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>Instruction tuning LLaMA. "Domain experts wrote ten diverse instructions per dataset". Two templates: Instruction: [task prompt] Text: [input text] Response: [output], and for FinQA/ConvFinQA Instruction: ... Context: ... Question: ... Response: ..., with ConvFinQA's multi-turn conversations flattened by appending prior Q&amp;A into the context.  Four LLaMA checkpoints — FinMA-7B, FinMA-30B (NLP portion), FinMA-7B-trade (forecasting only), FinMA-7B-full. AdamW, lr 8e-6, weight decay 1e-5, warmup 5%, max input 2048. "the 30B runs 20 epochs at batch size 24 on 128 A100 40GB GPUs".</t>
+          <t>Instruction tuning LLaMA. "Domain experts wrote ten diverse instructions per dataset". Two templates: Instruction: [task prompt] Text: [input text] Response: [output], and for FinQA/ConvFinQA Instruction: ... Context: ... Question: ... Response: ..., with ConvFinQA's multi-turn conversations flattened by appending prior Q&amp;A into the context. Four LLaMA checkpoints - FinMA-7B, FinMA-30B (NLP portion), FinMA-7B-trade (forecasting only), FinMA-7B-full. AdamW, lr 8e-6, weight decay 1e-5, warmup 5%, max input 2048. "the 30B runs 20 epochs at batch size 24 on 128 A100 40GB GPUs".</t>
         </is>
       </c>
       <c r="L49" s="11" t="inlineStr">
@@ -6693,12 +6693,12 @@
       </c>
       <c r="O49" s="11" t="inlineStr">
         <is>
-          <t>Credit scoring (German, Australian) as the risk proxy. Movement prediction label: y_t = 1 if r_t &gt; 0.55%, -1 if r_t &lt; -0.5%, with the middle discarded — "the benchmark removes the cases where a directional call would be least useful and least costly to get wrong, and what remains is not the decision a trader faces."</t>
+          <t>Credit scoring (German, Australian) as the risk proxy. Movement prediction label: y_t = 1 if r_t &gt; 0.55%, -1 if r_t &lt; -0.5%, with the middle discarded - "the benchmark removes the cases where a directional call would be least useful and least costly to get wrong, and what remains is not the decision a trader faces."</t>
         </is>
       </c>
       <c r="P49" s="11" t="inlineStr">
         <is>
-          <t>None — "there are no transaction costs anywhere, no position sizing, a single-step horizon".</t>
+          <t>None - "there are no transaction costs anywhere, no position sizing, a single-step horizon".</t>
         </is>
       </c>
       <c r="Q49" s="11" t="inlineStr">
@@ -6734,8 +6734,8 @@
       <c r="W49" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_F, A_T and the orchestrator, plus the evaluation layer. "it is the only one that puts a language model on stock movement prediction and credit scoring alongside the reading tasks, so it speaks to A_T and the orchestrator as well as to A_F."
-EFFECT ON A_F: Constrains decisively — it closes fine-tuning off. "This closes the question of whether to fine-tune an open model for the fundamental channel, and the answer is no... the working design for A_F stays a frontier model over structure-aware retrieval, with fine-tuning off the table rather than deferred." Usable artefacts: the FLARE prompt templates and harness as a ready format for evaluating A_F against a small probe set. Not usable as a CSE evaluation set. Licences: "Licences are mixed across the assembled datasets, CC BY-SA 3.0, CC BY-NC 4.0 on FOMC, MIT and public, which constrains reuse in a way the 'fully open' framing glosses over."
-SENTIMENT-RELATED EVIDENCE: Cross-cited only — "Predict the Future from the Past... shows financial sentiment performance degrading measurably as the gap between training and test period widens, so a benchmark that mixes periods without reporting them is measuring an average over conditions that behave differently."
+EFFECT ON A_F: Constrains decisively - it closes fine-tuning off. "This closes the question of whether to fine-tune an open model for the fundamental channel, and the answer is no... the working design for A_F stays a frontier model over structure-aware retrieval, with fine-tuning off the table rather than deferred." Usable artefacts: the FLARE prompt templates and harness as a ready format for evaluating A_F against a small probe set. Not usable as a CSE evaluation set. Licences: "Licences are mixed across the assembled datasets, CC BY-SA 3.0, CC BY-NC 4.0 on FOMC, MIT and public, which constrains reuse in a way the 'fully open' framing glosses over."
+SENTIMENT-RELATED EVIDENCE: Cross-cited only - "Predict the Future from the Past... shows financial sentiment performance degrading measurably as the gap between training and test period widens, so a benchmark that mixes periods without reporting them is measuring an average over conditions that behave differently."
 PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool; an explicit argument for keeping it as-is, verbatim: "FinMA-7B-trade is a clean documented case for keeping the four agents architecturally separate. One backbone tuned for the prediction task loses its classification ability almost entirely, 0.94 to 0.03 on FPB, and gains nothing measurable on the task it was specialised for. A shared fine-tuned backbone across A_T, A_F, A_V and A_L would buy exactly this, and the heterogeneity argument in the main gap is partly an argument that the components should fail independently, which a shared backbone forbids by construction." On the conditioning set / confidence, verbatim: "the orchestrator has to be able to drive a channel's weight to near zero rather than assuming every agent contributes." And: "The correct, incorrect and failure-to-answer taxonomy adopted from FinanceBench gains a fourth bucket, no parseable answer, which for the weighting function is a hard zero rather than a low C_{i,t}".</t>
         </is>
       </c>
@@ -6768,7 +6768,7 @@
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>github.com/czyssrs/ConvFinQA — "built on top of FinQA and therefore on FinTabNet." | DOI 10.18653/v1/2022.emnlp-main.421</t>
+          <t>github.com/czyssrs/ConvFinQA - "built on top of FinQA and therefore on FinTabNet." | DOI 10.18653/v1/2022.emnlp-main.421</t>
         </is>
       </c>
       <c r="F50" s="11" t="inlineStr">
@@ -6793,12 +6793,12 @@
       </c>
       <c r="J50" s="11" t="inlineStr">
         <is>
-          <t>Single report page — table plus surrounding text; conversation history.</t>
+          <t>Single report page - table plus surrounding text; conversation history.</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>Two-stage construction — "conversational QA flow simulation" producing a reasoning skeleton, then "question composition" by UpWork annotators with CPA or MBA backgrounds who are "explicitly instructed to identify redundancy, compress unnecessary turns using references to earlier context, and discard the example outright if no natural conversation can be written over the skeleton." Paid ~$4.00 per simple and ~$7.00 per hybrid conversation, average $60.00/hour.  FinQANet carried over unchanged, conversation context concatenated into both retriever and generator inputs; GPT-2 medium and T5 large as generative baselines; encoders BERT base/large, RoBERTa base/large. Prompting: GPT-3 text-davinci-002 in four settings — Answer-only, Program-original, Program-normal, Chain of Thought; three exemplar sets each with reported standard deviation. Task formalised as P(A | T, B, Q_n) = Σ_i P(G_i | T, B, Q_0, Q_1, …, Q_{n−1}). Dependency distance distribution: 39.5% at 0, 28.0% at 1, 19.0% at 2, 12.5% at 3, 1.0% beyond 4.</t>
+          <t>Two-stage construction - "conversational QA flow simulation" producing a reasoning skeleton, then "question composition" by UpWork annotators with CPA or MBA backgrounds who are "explicitly instructed to identify redundancy, compress unnecessary turns using references to earlier context, and discard the example outright if no natural conversation can be written over the skeleton." Paid ~$4.00 per simple and ~$7.00 per hybrid conversation, average $60.00/hour. FinQANet carried over unchanged, conversation context concatenated into both retriever and generator inputs; GPT-2 medium and T5 large as generative baselines; encoders BERT base/large, RoBERTa base/large. Prompting: GPT-3 text-davinci-002 in four settings - Answer-only, Program-original, Program-normal, Chain of Thought; three exemplar sets each with reported standard deviation. Task formalised as P(A | T, B, Q_n) = Σ_i P(G_i | T, B, Q_0, Q_1, …, Q_{n−1}). Dependency distance distribution: 39.5% at 0, 28.0% at 1, 19.0% at 2, 12.5% at 3, 1.0% beyond 4.</t>
         </is>
       </c>
       <c r="L50" s="11" t="inlineStr">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="M50" s="11" t="inlineStr">
         <is>
-          <t>None. FUNDAMENTAL: This is the fundamental task itself — computed quantities from statement tables and prose. RAG HANDLING: Retrieval is in-task via FinQANet's top-3 retriever with conversation context concatenated in; "it reaches 86.38% recall for the top three retrieved facts, marginally below the 89.66% the same retriever reached on FinQA's single-turn task." Cost concessions: "retrieval is only run on a 300-example sample of the test set, and program generation is run on the full test set using gold retrieval, so the prompting numbers are generous on retrieval and still lose." Page-local only: "A system scoring 68.90% here has demonstrated conversational reference resolution over one clean page, and nothing about locating that page."</t>
+          <t>None. FUNDAMENTAL: This is the fundamental task itself - computed quantities from statement tables and prose. RAG HANDLING: Retrieval is in-task via FinQANet's top-3 retriever with conversation context concatenated in; "it reaches 86.38% recall for the top three retrieved facts, marginally below the 89.66% the same retriever reached on FinQA's single-turn task." Cost concessions: "retrieval is only run on a 300-example sample of the test set, and program generation is run on the full test set using gold retrieval, so the prompting numbers are generous on retrieval and still lose." Page-local only: "A system scoring 68.90% here has demonstrated conversational reference resolution over one clean page, and nothing about locating that page."</t>
         </is>
       </c>
       <c r="N50" s="11" t="inlineStr">
@@ -6838,7 +6838,7 @@
       </c>
       <c r="S50" s="11" t="inlineStr">
         <is>
-          <t>"The best neural symbolic model reaches 68.90% execution and 68.24% program accuracy against expert humans at 89.44% and 86.34%... Gold supporting facts lift it to 77.32% and 76.46%, so roughly 8.4 points of the 20.5-point gap to experts is retrieval and the remaining 12 is reasoning". "34.73% of questions are single number selections and those score 82.54%, while the questions that need a program score 62.14%". Encoder scaling 55.03% (BERT-base) to 68.90% (RoBERTa-large). Per-turn execution — FinQANet 75.58 / 70.74 / 66.15 / 63.96 / 63.90 / 34.38 for turns 1–6; GPT-3 72.81 / 29.03 / 56.77 / 33.12 / 45.95 / 25.22. "Simple conversations score 72.37%, hybrid ones 60.99%, and within the hybrid conversations the first part scores 68.11% and the second part 52.38%... 65.0% of the second question sets were judged by annotators to depend on the first". Prompting: "Program-normal is the best prompting setting at 45.15% execution and 38.88% program accuracy... Program-original is 40.81% and 36.62%, CoT is 40.63% and 33.84%, and Answer-only is 24.09%. Every one of them sits at or below the MTurk crowd's 46.90%." Exemplar-set standard deviations ±4.68 and ±2.77. GPT-3 inversion: "FinQANet scores 82.54% on number selection and 62.14% on program questions; GPT-3 scores 35.32% on number selection and 55.56% on program questions." Exemplar count saturation: 43.52% at 5, 48.85% at 10, 49.31% at 15, 50.30% at 20, 49.90% at 25. LIMITATIONS (quoted): "The conversations are simulated from programs and were never validated against real analyst dialogue." "Every FinQA filtering constraint is inherited and the operation vocabulary is narrowed on top... Nothing crosses a document, nothing crosses a filing year, there is no as-of notion". "The neural symbolic results are single-run point estimates while the prompting results are not, so the two halves of the paper are not held to the same standard." "The prompting conclusion is scoped to one 2022 model with deliberately shallow prompting, and the paper says so... So neural symbolic beats prompting is not a claim I can carry into 2026". "The turn-6 collapse rests on very few examples." "Nothing in the dataset or the metrics addresses detecting a wrong turn before it poisons the next one... the absence of any measurement of propagation, and of any mechanism for a model to decline a turn it cannot ground, is the most consequential thing missing."</t>
+          <t>"The best neural symbolic model reaches 68.90% execution and 68.24% program accuracy against expert humans at 89.44% and 86.34%... Gold supporting facts lift it to 77.32% and 76.46%, so roughly 8.4 points of the 20.5-point gap to experts is retrieval and the remaining 12 is reasoning". "34.73% of questions are single number selections and those score 82.54%, while the questions that need a program score 62.14%". Encoder scaling 55.03% (BERT-base) to 68.90% (RoBERTa-large). Per-turn execution - FinQANet 75.58 / 70.74 / 66.15 / 63.96 / 63.90 / 34.38 for turns 1–6; GPT-3 72.81 / 29.03 / 56.77 / 33.12 / 45.95 / 25.22. "Simple conversations score 72.37%, hybrid ones 60.99%, and within the hybrid conversations the first part scores 68.11% and the second part 52.38%... 65.0% of the second question sets were judged by annotators to depend on the first". Prompting: "Program-normal is the best prompting setting at 45.15% execution and 38.88% program accuracy... Program-original is 40.81% and 36.62%, CoT is 40.63% and 33.84%, and Answer-only is 24.09%. Every one of them sits at or below the MTurk crowd's 46.90%." Exemplar-set standard deviations ±4.68 and ±2.77. GPT-3 inversion: "FinQANet scores 82.54% on number selection and 62.14% on program questions; GPT-3 scores 35.32% on number selection and 55.56% on program questions." Exemplar count saturation: 43.52% at 5, 48.85% at 10, 49.31% at 15, 50.30% at 20, 49.90% at 25. LIMITATIONS (quoted): "The conversations are simulated from programs and were never validated against real analyst dialogue." "Every FinQA filtering constraint is inherited and the operation vocabulary is narrowed on top... Nothing crosses a document, nothing crosses a filing year, there is no as-of notion". "The neural symbolic results are single-run point estimates while the prompting results are not, so the two halves of the paper are not held to the same standard." "The prompting conclusion is scoped to one 2022 model with deliberately shallow prompting, and the paper says so... So neural symbolic beats prompting is not a claim I can carry into 2026". "The turn-6 collapse rests on very few examples." "Nothing in the dataset or the metrics addresses detecting a wrong turn before it poisons the next one... the absence of any measurement of propagation, and of any mechanism for a model to decline a turn it cannot ground, is the most consequential thing missing."</t>
         </is>
       </c>
       <c r="T50" s="11" t="inlineStr">
@@ -6858,8 +6858,8 @@
       </c>
       <c r="W50" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: A_F and the evaluation layer only — stated explicitly: "it speaks to A_F, the fundamental and retrieval channel, and to the evaluation layer, and to nothing else".
-EFFECT ON A_F: Constrains the interface design (no conversational interface; atomic self-contained requests; typed-pointer chaining), constrains the planning band (below 50% on computed quantities over CSE filings), supplies the conditional-accuracy metric for the probe set, and supplies the CSE-specific reference-resolution warning: "Sri Lankan annual reports lean on phrases like the corresponding period and as restated, quarterly statements refer back to the annual ones, and comparative columns are labelled by position rather than by date... period resolution belongs in the retrieval and typing layer, resolved against an explicit fiscal calendar, and never left to the reasoner to infer from context." Usable as evaluation material: yes, as a probe corpus paired with FinQA — "Because the conversations are synthesised from FinQA programs, the pairing is already aligned, so the two can be used as one probe corpus with and without conversational context, which is the cheapest available ablation on whether my own reference-resolution layer is doing anything." Taxonomy usable: the question-shape split (number selection vs program questions) and the three-dataset comparison table. Licence: not stated beyond "Dataset and code are public"; inherits FinTabNet.
+          <t>SPEAKS TO: A_F and the evaluation layer only - stated explicitly: "it speaks to A_F, the fundamental and retrieval channel, and to the evaluation layer, and to nothing else".
+EFFECT ON A_F: Constrains the interface design (no conversational interface; atomic self-contained requests; typed-pointer chaining), constrains the planning band (below 50% on computed quantities over CSE filings), supplies the conditional-accuracy metric for the probe set, and supplies the CSE-specific reference-resolution warning: "Sri Lankan annual reports lean on phrases like the corresponding period and as restated, quarterly statements refer back to the annual ones, and comparative columns are labelled by position rather than by date... period resolution belongs in the retrieval and typing layer, resolved against an explicit fiscal calendar, and never left to the reasoner to infer from context." Usable as evaluation material: yes, as a probe corpus paired with FinQA - "Because the conversations are synthesised from FinQA programs, the pairing is already aligned, so the two can be used as one probe corpus with and without conversational context, which is the cheapest available ablation on whether my own reference-resolution layer is doing anything." Taxonomy usable: the question-shape split (number selection vs program questions) and the three-dataset comparison table. Licence: not stated beyond "Dataset and code are public"; inherits FinTabNet.
 SENTIMENT-RELATED EVIDENCE: None.
 PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool or the conditioning set. Design revisions to A_F's interface, verbatim: "Query A_F with atomic, self-contained requests and do not build a conversational interface to it... The orchestrator already holds the state it needs, so resolving that value in the subsequent year into an explicit entity, period and line item before the call costs me nothing and removes the failure mode the paper spends its results section documenting." And: "my equivalent is a resolved quantity carrying value, scale, currency, period and the source rows it came from, per the typed-output decision from the TAT-QA note, passed back in explicitly on the next call." And the closed vocabulary: "Level, difference, ratio and growth rate is the closed vocabulary, anything outside it gets declined rather than attempted, and this is the last time it needs arguing."</t>
         </is>
@@ -6913,7 +6913,7 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>"Roughly 500 financial reports from the past two years are downloaded from annualreports.com"; TableBank detection, Apache PDFBox extraction; tables outside 3–30 rows and 3–6 columns dropped, leaving ~20,000 candidates; "About two thirds of the candidate tables are discarded during annotation for lacking enough relevant surrounding paragraphs." Final: 16,552 QA pairs over 2,757 hybrid contexts from 182 reports; split by context — 2,201/13,215 train, 278/1,668 dev, 278/1,669 test. Tables average 9.4 rows and 4.0 columns with 4.8 paragraphs of 43.6 words; questions average 12.5 words, answers 4.1. Annotators: ~30 finance undergraduates screened at 95%, ~two hybrid contexts per hour over three months, two-round validation by five verifiers.</t>
+          <t>"Roughly 500 financial reports from the past two years are downloaded from annualreports.com"; TableBank detection, Apache PDFBox extraction; tables outside 3–30 rows and 3–6 columns dropped, leaving ~20,000 candidates; "About two thirds of the candidate tables are discarded during annotation for lacking enough relevant surrounding paragraphs." Final: 16,552 QA pairs over 2,757 hybrid contexts from 182 reports; split by context - 2,201/13,215 train, 278/1,668 dev, 278/1,669 test. Tables average 9.4 rows and 4.0 columns with 4.8 paragraphs of 43.6 words; questions average 12.5 words, answers 4.1. Annotators: ~30 finance undergraduates screened at 95%, ~two hybrid contexts per hour over three months, two-round validation by five verifiers.</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
@@ -6923,7 +6923,7 @@
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>TagOp — question + flattened table + paragraphs into RoBERTa, per-sub-token I/O tagging for evidence, then exactly one of ten aggregation operators applied, plus a separate scale head. Ten operators: Span-in-text, Cell-in-table, Spans, Sum, Count, Average, Multiplication, Division, Difference, Change ratio. "Exactly one operator is applied per question, so there is no composition in the FinQA sense."  Four heads. Order head: p^order = softmax(FFN(avg(h_t1, h_t2))). Scale head (5-way over None, Thousand, Million, Billion, Percent): p^scale = softmax(FFN([[CLS]; h_tab; h_p])). Loss: L = NLL(log P^tag, G^tag) + NLL(log P^op, G^op) + NLL(log P^scale, G^scale) + NLL(log P^order, G^order). Evaluation is EM and DROP-style numeracy F1 with sign preserved and "F1 is set to zero unless the predicted number multiplied by the predicted scale matches exactly".</t>
+          <t>TagOp - question + flattened table + paragraphs into RoBERTa, per-sub-token I/O tagging for evidence, then exactly one of ten aggregation operators applied, plus a separate scale head. Ten operators: Span-in-text, Cell-in-table, Spans, Sum, Count, Average, Multiplication, Division, Difference, Change ratio. "Exactly one operator is applied per question, so there is no composition in the FinQA sense." Four heads. Order head: p^order = softmax(FFN(avg(h_t1, h_t2))). Scale head (5-way over None, Thousand, Million, Billion, Percent): p^scale = softmax(FFN([[CLS]; h_tab; h_p])). Loss: L = NLL(log P^tag, G^tag) + NLL(log P^op, G^op) + NLL(log P^scale, G^scale) + NLL(log P^order, G^order). Evaluation is EM and DROP-style numeracy F1 with sign preserved and "F1 is set to zero unless the predicted number multiplied by the predicted scale matches exactly".</t>
         </is>
       </c>
       <c r="L51" s="11" t="inlineStr">
@@ -6973,7 +6973,7 @@
       </c>
       <c r="U51" s="11" t="inlineStr">
         <is>
-          <t>The scale head — "Scale prediction is the most directly transferable idea here, and it matters more for the CSE than it did for the source data. Sri Lankan annual reports declare magnitude once in a header, 'Rs. '000' or 'Rs. Mn', sometimes switch between statements within the same report, and occasionally carry a second currency column." Retrieve-then-reason over tag-in-place. Closed operator vocabulary. Answer-source reporting axis. EM and F1 side by side. Two-round validation (one checker then a different approver) as affordable at 10–20 questions. Row-header hierarchy preservation (recorded as a hypothesis, not a finding).</t>
+          <t>The scale head - "Scale prediction is the most directly transferable idea here, and it matters more for the CSE than it did for the source data. Sri Lankan annual reports declare magnitude once in a header, 'Rs. '000' or 'Rs. Mn', sometimes switch between statements within the same report, and occasionally carry a second currency column." Retrieve-then-reason over tag-in-place. Closed operator vocabulary. Answer-source reporting axis. EM and F1 side by side. Two-round validation (one checker then a different approver) as affordable at 10–20 questions. Row-header hierarchy preservation (recorded as a hypothesis, not a finding).</t>
         </is>
       </c>
       <c r="V51" s="11" t="inlineStr">
@@ -6984,7 +6984,7 @@
       <c r="W51" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_F and the evaluation layer only, stated explicitly.
-EFFECT ON A_F: Strongly supports and shapes the design. Establishes the typed-output decision; supports keeping a retrieval stage; fixes the operator vocabulary; supplies a second mechanical confidence signal with a caveat; supplies the reporting axes. "This also keeps A_F compatible with the structure-aware retrieval work in Neo4j Graph-RAG for CSE and Financial Report Chunking for Effective Retrieval Augmented Generation, which a single-sequence tagging design would not be." Usable taxonomy: the scale taxonomy (None/Thousand/Million/Billion/Percent) and the answer-type × answer-source split — "The scale taxonomy and the answer-type and answer-source split are worth lifting directly into my probe set design." Licence for the dataset itself: public for non-commercial use.
+EFFECT ON A_F: Strongly supports and shapes the design. Establishes the typed-output decision; supports keeping a retrieval stage; fixes the operator vocabulary; supplies a second mechanical confidence signal with a caveat; supplies the reporting axes. "This also keeps A_F compatible with the structure-aware retrieval work in Neo4j Graph-RAG for CSE and Financial Report Chunking for Effective Retrieval Augmented Generation, which a single-sequence tagging design would not be." Usable taxonomy: the scale taxonomy (None/Thousand/Million/Billion/Percent) and the answer-type × answer-source split - "The scale taxonomy and the answer-type and answer-source split are worth lifting directly into my probe set design." Licence for the dataset itself: public for non-commercial use.
 SENTIMENT-RELATED EVIDENCE: None.
 PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. A stated design decision on A_F's output, verbatim: "The design decision is that A_F emits a typed quantity, value plus scale plus currency plus period, and never a bare number, which also removes the unit-conversion error class that the FinQA note flagged as a representation problem rather than a model one." On the conditioning set / C_{F,t}, verbatim: "This gives me a second mechanical confidence signal for C_{F,t}, and a warning about how to use it. FinQA offered program step count; TAT-QA offers the operator classifier posterior, the tagging margin on the selected evidence, and whether the predicted scale fell in a rare class. But operator accuracy runs from 100.0 on Count and Average down to 0.0 on Multiplication and Other, so a single posterior is not comparable across classes and I would need per-operator reliability estimated on my own probe set before the orchestrator can read it... it is the second time the answer for A_F has turned out to be a structural property of the output rather than a self-reported score, which is worth noting as a pattern."</t>
         </is>
@@ -7033,7 +7033,7 @@
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>US, S&amp;P 500 earnings reports, 1999–2019.  Single-page report QA.</t>
+          <t>US, S&amp;P 500 earnings reports, 1999–2019. Single-page report QA.</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>Ten-operation DSL — add, subtract, multiply, divide, exp, greater, plus table-max, table-min, table-sum, table-average. Flat program op_1[args_1], op_2[args_2], …, op_n[args_n] with #k referencing step k. Task: P(A | T, E, Q) = Σ_i P(G_i | T, E, Q).  FinQANet, two-stage retriever-generator. Retriever templates each table row into a sentence ("the risk-free interest rate of 2006 is 5%"), concatenates with the question, trains a BERT-base classifier, keeps top three reordered into document order. Generator is an LSTM decoder over copy-and-generate space: c_T = W_c[att_p; att_h; h_T], w_T = softmax(H'_T · c_T), with H'_T = W_h[H; H ∘ att'_p]. The novel piece: "at the end of each completed operation[args] unit, the embedding of the corresponding step memory token is overwritten with that step's context vector, so a reference to #0 later in the sequence carries what step 0 did rather than being an opaque symbol." Grammar masks keep output valid.</t>
+          <t>Ten-operation DSL - add, subtract, multiply, divide, exp, greater, plus table-max, table-min, table-sum, table-average. Flat program op_1[args_1], op_2[args_2], …, op_n[args_n] with #k referencing step k. Task: P(A | T, E, Q) = Σ_i P(G_i | T, E, Q). FinQANet, two-stage retriever-generator. Retriever templates each table row into a sentence ("the risk-free interest rate of 2006 is 5%"), concatenates with the question, trains a BERT-base classifier, keeps top three reordered into document order. Generator is an LSTM decoder over copy-and-generate space: c_T = W_c[att_p; att_h; h_T], w_T = softmax(H'_T · c_T), with H'_T = W_h[H; H ∘ att'_p]. The novel piece: "at the end of each completed operation[args] unit, the embedding of the corresponding step memory token is overwritten with that step's context vector, so a reference to #0 later in the sequence carries what step 0 did rather than being an opaque symbol." Grammar masks keep output valid.</t>
         </is>
       </c>
       <c r="L52" s="11" t="inlineStr">
@@ -7111,7 +7111,7 @@
           <t>SPEAKS TO: A_F and the evaluation layer only, stated explicitly.
 EFFECT ON A_F: Defines it. "This is the task specification for the numeric half of A_F, and the pair with the CSE Graph-RAG paper draws the boundary cleanly. That paper builds the entity graph and states that statement tables are future work; this one does the statement tables and ignores entity structure. In the review chapter that pairing is how I justify A_F as a system component built on published task definitions, with the contribution sitting in the orchestration rather than in the retrieval." Usable artefacts: the DSL and program executor (public, CDLA-Permissive via FinTabNet); the evaluation shape. Not usable as a CSE set: "There is no CSE equivalent of this dataset and building one is out of scope... the FinTabNet licensing and the annotations do not transfer to CSE filings."
 SENTIMENT-RELATED EVIDENCE: None.
-PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. Scope decision on A_F, verbatim: "Keep A_F's output vocabulary to one and two-step quantities and say so as a design decision rather than a limitation... Anything needing three or more chained operations lands in the 22.78% band, and the honest move is to not ask the channel for those at all rather than to ask and then discover the error rate in the backtest." On C_{F,t}, verbatim: "The retrieve-then-program design is the first concrete answer I have to how C_{F,t} gets computed. A program is checkable in ways free text is not: whether it parses under the grammar, whether every argument traces to a retrieved number or row rather than being invented, how many retries the retriever needed, and how many steps the program has. That last one is a calibrated difficulty proxy on this evidence, since accuracy runs 67.61%, 59.08% and 22.78% across one, two and three-plus steps, so step count is a feature the orchestrator can read without asking the model how sure it is. This pushes the standing open question about comparable confidence forward for one of the four producers, and it is a different mechanism from the Cypher-validation signal in the Graph-RAG note, which is useful because two mechanical signals on the same channel can be cross-checked." Also: "design the orchestrator to tolerate a channel that is wrong a lot" — expectation "nearer 40% than 60% on first build".</t>
+PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. Scope decision on A_F, verbatim: "Keep A_F's output vocabulary to one and two-step quantities and say so as a design decision rather than a limitation... Anything needing three or more chained operations lands in the 22.78% band, and the honest move is to not ask the channel for those at all rather than to ask and then discover the error rate in the backtest." On C_{F,t}, verbatim: "The retrieve-then-program design is the first concrete answer I have to how C_{F,t} gets computed. A program is checkable in ways free text is not: whether it parses under the grammar, whether every argument traces to a retrieved number or row rather than being invented, how many retries the retriever needed, and how many steps the program has. That last one is a calibrated difficulty proxy on this evidence, since accuracy runs 67.61%, 59.08% and 22.78% across one, two and three-plus steps, so step count is a feature the orchestrator can read without asking the model how sure it is. This pushes the standing open question about comparable confidence forward for one of the four producers, and it is a different mechanism from the Cypher-validation signal in the Graph-RAG note, which is useful because two mechanical signals on the same channel can be cross-checked." Also: "design the orchestrator to tolerate a channel that is wrong a lot" - expectation "nearer 40% than 60% on first build".</t>
         </is>
       </c>
       <c r="X52" s="11" t="inlineStr">
@@ -7173,7 +7173,7 @@
       </c>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>Rolling monthly experiment. Three retraining strategies — ODNM (old data new model: fresh model at t on everything up to t), NDNM (new data new model: fresh model on month t alone), NDOM (new data old model: initialise M_t from M_{t−1} and continue training on month t; continual learning). "Logistic regression and the LSTM have no NDOM row because they build dataset-specific vocabularies". Six model families: logistic regression on bag-of-words, LSTM with linear head, BERT base uncased, RoBERTa base, FinBERT, GPT-3.5 (text-davinci-003, two-shot ICL, no fine-tuning). Metrics F1_in, F1_out, ΔF1 = F1_in − F1_out. Shift measure: Shift(t, t+1) = Σ_{v∈V} p_t(y|v) KLD(p_t(y|v) ‖ p_{t+1}(y|v)), over the pretrained tokenizer's subword vocabulary, weighted by conditional label probability rather than frequency. Mitigation: OOD detector with manufactured labels — OOD(M_i, x_j) = 0 if M_i(x_j) = y_j, 1 if M_i(x_j) ≠ y_j, restricted to samples M_j classifies correctly. Detector is a two-layer MLP over [CLS]: f(M,x) = W_2(GELU(W_1(M^[CLS](x)) + b_1)) + b_2, sentiment model frozen, one shared parameter set across all M. Substitute predictor: ŷ_{t+1} = Σ_{k=0}^{p−1} α_k M_{t−k}(x_{t+1}) + ε, p = 3, α_k fitted on past data, recency-weighted. Fitted 2014-01 to 2015-06, evaluated 2015-07 to 2016-12. AdamW, lr grid [2e-3, 2e-4, 2e-5], batch {32, 64}.  Frozen classifier + OOD router + autoregressive-over-past-models predictor.</t>
+          <t>Rolling monthly experiment. Three retraining strategies - ODNM (old data new model: fresh model at t on everything up to t), NDNM (new data new model: fresh model on month t alone), NDOM (new data old model: initialise M_t from M_{t−1} and continue training on month t; continual learning). "Logistic regression and the LSTM have no NDOM row because they build dataset-specific vocabularies". Six model families: logistic regression on bag-of-words, LSTM with linear head, BERT base uncased, RoBERTa base, FinBERT, GPT-3.5 (text-davinci-003, two-shot ICL, no fine-tuning). Metrics F1_in, F1_out, ΔF1 = F1_in − F1_out. Shift measure: Shift(t, t+1) = Σ_{v∈V} p_t(y|v) KLD(p_t(y|v) ‖ p_{t+1}(y|v)), over the pretrained tokenizer's subword vocabulary, weighted by conditional label probability rather than frequency. Mitigation: OOD detector with manufactured labels - OOD(M_i, x_j) = 0 if M_i(x_j) = y_j, 1 if M_i(x_j) ≠ y_j, restricted to samples M_j classifies correctly. Detector is a two-layer MLP over [CLS]: f(M,x) = W_2(GELU(W_1(M^[CLS](x)) + b_1)) + b_2, sentiment model frozen, one shared parameter set across all M. Substitute predictor: ŷ_{t+1} = Σ_{k=0}^{p−1} α_k M_{t−k}(x_{t+1}) + ε, p = 3, α_k fitted on past data, recency-weighted. Fitted 2014-01 to 2015-06, evaluated 2015-07 to 2016-12. AdamW, lr grid [2e-3, 2e-4, 2e-5], batch {32, 64}. Frozen classifier + OOD router + autoregressive-over-past-models predictor.</t>
         </is>
       </c>
       <c r="L53" s="11" t="inlineStr">
@@ -7208,12 +7208,12 @@
       </c>
       <c r="R53" s="11" t="inlineStr">
         <is>
-          <t>Inherited baselines STM (spurious tokens masking, Wang et al. 2022) and CDA (counterfactual data augmentation, Wang and Culotta 2021); both fail. Model-free shift evidence: sentiment positivity #pos/(#pos+#neg) per month vs monthly returns, "Spearman correlation of 0.397 for Apple and 0.459 for Tesla". KEY RESULTS — SENTIMENT DECAY WITH NUMBERS (this is the extraction the standing rule asks for): - "Every fine-tuned model degrades... All ΔF1 values for fine-tuned models in Table 1 are positive." - Aggregate: "BERT at NDNM losing 4.70 F1 points and RoBERTa 3.96". - Minority class: "BERT's negative-class ΔF1 under NDNM is 8.27 against 1.13 for the positive class, and logistic regression loses 10.04 points on the negative class against 1.07 on the positive. The bearish label is the minority in a corpus that is mostly bullish, and it is the one that stops generalising first. Up-sampling the minority class, reported in their Appendix A, does not change this conclusion." - Retraining trade: "NDOM has the best in-sample performance everywhere it applies, BERT at 79.1 average F1_in against 72.5 for NDNM and 67.4 for ODNM, and RoBERTa at 80.4, but it carries a ΔF1 of 3.31 and 2.45 respectively. ODNM inverts this completely, with the smallest drops in the table, 1.19 for BERT, 0.97 for RoBERTa, 1.00 for FinBERT, on top of the weakest in-sample scores." - GPT-3.5: "a ΔF1 of −1.10 with F1_in of 66.4 and F1_out of 67.5, flat and weak", and "its pretraining corpus covers 2014 to 2017 so these months may not be out of distribution for it at all, which makes the flat line uninterpretable as evidence about model scale." - Shift correlation: "Spearman correlations between ΔF1 and the token-level KL shift come out at 0.385 for BERT (p = 0.020), 0.345 for RoBERTa (p = 0.039) and 0.281 for FinBERT (p = 0.096)." - Spurious features: "Fitting logistic regression to the full corpus and reading off the 30 largest absolute coefficients returns a list where the genuine sentiment words, bears, bulls, fall, dump, strong, shorts, squeeze, are a minority among ticker fragments and company names, incbr, nakd, plx, owens, caterpillar, kellogg, pharmaceuticals... a model predicting p(y|v) for v = 'Tesla' is not doing sentiment analysis, it is memorising the market's current opinion of Tesla, and it fails the moment that opinion turns." - Mitigation: "the method reduces ΔF1 by 31% for BERT (2.05 to 1.42), 26% for RoBERTa (1.62 to 1.26) and 32% for FinBERT (2.01 to 1.36)... Expressed as out-of-sample F1 the same result is a gain of 0.63, 0.36 and 0.65 points. Both inherited baselines make things worse: STM costs BERT 2.09 points of F1_in and raises its ΔF1, and CDA costs FinBERT 3.54 points." - Detector: "OOD recall of 0.86 for BERT and 0.91 for FinBERT at OOD precision of 0.23 and 0.15." - NO MECHANISM TO NOTICE: nothing in the corpus or the model signals the decay. Verbatim: "A component whose largest learned coefficients sit on ticker fragments and company names is one whose apparent skill is a memorised snapshot of market opinion, and nothing in the system notices when that snapshot expires." LIMITATIONS (quoted): "There is no ablation separating the detector from the ensemble, which leaves the paper's own mechanism unestablished... without it the claim that OOD detection is what produces the gain is the paper's interpretation of a result rather than a result. This is the first thing I would raise about the paper." "ΔF1 rewards a model that is uniformly mediocre, and the paper's own table shows it... GPT-3.5 wins the metric outright by being flat and weak." "The shift measure weights tokens by conditional label probability rather than by frequency, and it is estimated over a subword vocabulary... the statistic is dominated by the sparse tail... the estimator's behaviour in the tail is load-bearing." "The labels are self-declared directional tags on a social platform, so label shift and market regime are entangled by construction." "One platform, one language, one market, three years, and no significance testing on the result that matters." "Nothing connects the performance drop to money". Also, on the data figure: "The monotone drift in the top panel is the number of examples per month rising steadily over the three years, so the later months carry far more data than the earlier ones and the rolling experiment is not comparing like with like across time, which the paper does not remark on."</t>
+          <t>Inherited baselines STM (spurious tokens masking, Wang et al. 2022) and CDA (counterfactual data augmentation, Wang and Culotta 2021); both fail. Model-free shift evidence: sentiment positivity #pos/(#pos+#neg) per month vs monthly returns, "Spearman correlation of 0.397 for Apple and 0.459 for Tesla". KEY RESULTS - SENTIMENT DECAY WITH NUMBERS (this is the extraction the standing rule asks for): - "Every fine-tuned model degrades... All ΔF1 values for fine-tuned models in Table 1 are positive." - Aggregate: "BERT at NDNM losing 4.70 F1 points and RoBERTa 3.96". - Minority class: "BERT's negative-class ΔF1 under NDNM is 8.27 against 1.13 for the positive class, and logistic regression loses 10.04 points on the negative class against 1.07 on the positive. The bearish label is the minority in a corpus that is mostly bullish, and it is the one that stops generalising first. Up-sampling the minority class, reported in their Appendix A, does not change this conclusion." - Retraining trade: "NDOM has the best in-sample performance everywhere it applies, BERT at 79.1 average F1_in against 72.5 for NDNM and 67.4 for ODNM, and RoBERTa at 80.4, but it carries a ΔF1 of 3.31 and 2.45 respectively. ODNM inverts this completely, with the smallest drops in the table, 1.19 for BERT, 0.97 for RoBERTa, 1.00 for FinBERT, on top of the weakest in-sample scores." - GPT-3.5: "a ΔF1 of −1.10 with F1_in of 66.4 and F1_out of 67.5, flat and weak", and "its pretraining corpus covers 2014 to 2017 so these months may not be out of distribution for it at all, which makes the flat line uninterpretable as evidence about model scale." - Shift correlation: "Spearman correlations between ΔF1 and the token-level KL shift come out at 0.385 for BERT (p = 0.020), 0.345 for RoBERTa (p = 0.039) and 0.281 for FinBERT (p = 0.096)." - Spurious features: "Fitting logistic regression to the full corpus and reading off the 30 largest absolute coefficients returns a list where the genuine sentiment words, bears, bulls, fall, dump, strong, shorts, squeeze, are a minority among ticker fragments and company names, incbr, nakd, plx, owens, caterpillar, kellogg, pharmaceuticals... a model predicting p(y|v) for v = 'Tesla' is not doing sentiment analysis, it is memorising the market's current opinion of Tesla, and it fails the moment that opinion turns." - Mitigation: "the method reduces ΔF1 by 31% for BERT (2.05 to 1.42), 26% for RoBERTa (1.62 to 1.26) and 32% for FinBERT (2.01 to 1.36)... Expressed as out-of-sample F1 the same result is a gain of 0.63, 0.36 and 0.65 points. Both inherited baselines make things worse: STM costs BERT 2.09 points of F1_in and raises its ΔF1, and CDA costs FinBERT 3.54 points." - Detector: "OOD recall of 0.86 for BERT and 0.91 for FinBERT at OOD precision of 0.23 and 0.15." - NO MECHANISM TO NOTICE: nothing in the corpus or the model signals the decay. Verbatim: "A component whose largest learned coefficients sit on ticker fragments and company names is one whose apparent skill is a memorised snapshot of market opinion, and nothing in the system notices when that snapshot expires." LIMITATIONS (quoted): "There is no ablation separating the detector from the ensemble, which leaves the paper's own mechanism unestablished... without it the claim that OOD detection is what produces the gain is the paper's interpretation of a result rather than a result. This is the first thing I would raise about the paper." "ΔF1 rewards a model that is uniformly mediocre, and the paper's own table shows it... GPT-3.5 wins the metric outright by being flat and weak." "The shift measure weights tokens by conditional label probability rather than by frequency, and it is estimated over a subword vocabulary... the statistic is dominated by the sparse tail... the estimator's behaviour in the tail is load-bearing." "The labels are self-declared directional tags on a social platform, so label shift and market regime are entangled by construction." "One platform, one language, one market, three years, and no significance testing on the result that matters." "Nothing connects the performance drop to money". Also, on the data figure: "The monotone drift in the top panel is the number of examples per month rising steadily over the three years, so the later months carry far more data than the earlier ones and the rolling experiment is not comparing like with like across time, which the paper does not remark on."</t>
         </is>
       </c>
       <c r="S53" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>Four retraining strategies are compared month by month: ODNM (fresh model at each t on all history), NDNM (fresh model at each t on month t alone), NDOM (initialise from the previous month's model and continue training, that is continual learning), and the static baseline. NDOM has the best in-sample performance everywhere it applies. ODNM posts the smallest degradation in the table, 1.19 for BERT, but the metric is a raw difference of F1 scores with no normalisation by level, so that model shows the smallest drop while sitting 11.7 points below NDOM. Spearman correlation between delta-F1 and the token-level KL shift is 0.385 for BERT, and the per-stock version is 0.397 for Apple and 0.459 for Tesla. The adaptive-retraining mitigation, with detector and coefficients fitted on 2014-01 to 2015-06 and evaluated on 2015-07 to 2016-12, improves performance at an OOD precision of 0.23, so roughly three in four flagged samples are ones the current model would have handled. The reported gains are 0.36 for RoBERTa, where the paper's text claims 26%, and 0.65 for FinBERT.</t>
         </is>
       </c>
       <c r="T53" s="11" t="inlineStr">
@@ -7234,7 +7234,7 @@
       <c r="W53" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: The orchestrator primarily, plus every fitted agent (A_T, A_V, A_L and A_F via refit policy), plus the evaluation layer. Not a text-modality paper for A_F, since A_F's text is filings not social posts.
-EFFECT ON A_F: Indirect. It constrains the refit policy for any fitted component and it supplies the competence-gap construction that C_{F,t} sits inside, but it offers no evaluation set or taxonomy for CSE filings. SENTIMENT-RELATED EVIDENCE (the standing rule): The note applies the rule explicitly. Verbatim: "It is the cleanest citation I have for why sentiment was investigated and then excluded from scope. Under the Literature Matrix exception this paper stays in as evidence the area was examined: a dedicated financial sentiment model, fine-tuned on 418,893 in-domain messages, degrades by 8 F1 points on its minority class from one month to the next, leans on tokens with no sentiment content, and needs a second system bolted on to recover a fraction of a point. That is a component with a maintenance burden and a measurable decay rate, and the attribution argument in the scope note applies with force: a 5% return improvement out of a system containing this could not be traced to anything." And: "The spurious-correlation table is a third documented fixed-influence failure case and it is directly citable in the review chapter... That is the same structure as FinAgent's auxiliary strategies returning 16% against buy-and-hold's 29% and AlphaAgents dropping its sentiment agent for insufficient coverage, and the three together make the fixed-influence argument from three different directions rather than one." Note that the paper's own mitigation is the "mechanism to notice" — an OOD detector running at 0.15–0.23 precision, i.e. wrong roughly three times in four.
+EFFECT ON A_F: Indirect. It constrains the refit policy for any fitted component and it supplies the competence-gap construction that C_{F,t} sits inside, but it offers no evaluation set or taxonomy for CSE filings. SENTIMENT-RELATED EVIDENCE (the standing rule): The note applies the rule explicitly. Verbatim: "It is the cleanest citation I have for why sentiment was investigated and then excluded from scope. Under the Literature Matrix exception this paper stays in as evidence the area was examined: a dedicated financial sentiment model, fine-tuned on 418,893 in-domain messages, degrades by 8 F1 points on its minority class from one month to the next, leans on tokens with no sentiment content, and needs a second system bolted on to recover a fraction of a point. That is a component with a maintenance burden and a measurable decay rate, and the attribution argument in the scope note applies with force: a 5% return improvement out of a system containing this could not be traced to anything." And: "The spurious-correlation table is a third documented fixed-influence failure case and it is directly citable in the review chapter... That is the same structure as FinAgent's auxiliary strategies returning 16% against buy-and-hold's 29% and AlphaAgents dropping its sentiment agent for insufficient coverage, and the three together make the fixed-influence argument from three different directions rather than one." Note that the paper's own mitigation is the "mechanism to notice" - an OOD detector running at 0.15–0.23 precision, i.e. wrong roughly three times in four.
 PROPOSED REVISION STATED IN THE NOTE: This is the only note of the seven that proposes a change to the conditioning set. Verbatim: "The shift-detection idea belongs in the conditioning set as a candidate, and the detector's precision is the warning that comes with it. L_t, V_t, P_t and C_{i,t} are a hypothesis about what weighting should respond to, and this paper suggests a fifth candidate, a direct estimate of how far the current input distribution has moved from the one the components were fitted on. The evidence for it is moderate, a ρ of roughly 0.3 to 0.39, and the detector built on it runs at 0.15 to 0.23 precision, so a naive port would have the orchestrator re-weighting on a signal that is wrong three times out of four. If I test a shift input, it gets tested against the always-blend control this paper skipped, and I should expect to report that it does not earn its slot." On C_{i,t}, verbatim: "for any component that emits a prediction with a later-observable outcome, the gap between its fitted-period accuracy and its next-period accuracy is computable without knowing anything about how it works. Applied per agent and rolled forward, that gives A_T, A_V, A_L and A_F a comparable backward-looking competence estimate on the same footing as the p_T construction from the HLOB note. The caution travels with it: a gap metric alone ranks a uniformly weak agent above a strong but drifting one, so the orchestrator needs level and gap jointly, not the difference on its own." On baselines, verbatim: "a static learned weight over agents is one control, and a recency-weighted combination that ignores market state entirely is a second, cheaper one that my state-conditional weighting has to beat before the conditioning set earns its place." No change to the four-agent pool is proposed in any of the seven notes.</t>
         </is>
       </c>
@@ -7252,7 +7252,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid–ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
+          <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid-ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
@@ -7267,19 +7267,19 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.jfineco.2024.103916 — accessed 4 October 2026. Code and data: github.com/eguidotti/bidask.</t>
+          <t>https://doi.org/10.1016/j.jfineco.2024.103916 - accessed 4 October 2026. Code and data: github.com/eguidotti/bidask.</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Low-frequency microstructure econometrics — estimation of the effective bid–ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin–Schultz (2012) / Abdi–Ranaldo (2017) lineage.</t>
+          <t>Low-frequency microstructure econometrics - estimation of the effective bid-ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin-Schultz (2012) / Abdi-Ranaldo (2017) lineage.</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>Produce an estimator of the effective bid–ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
+          <t>Produce an estimator of the effective bid-ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
 The object being estimated is the effective spread, not the quoted spread. The quoted spread is the posted distance between best bid and best ask; the effective spread is the realised distance between the transaction price and the unobserved fundamental price, S = 2D(P − P̃)/P̃, with D = +1 for buyer-initiated and −1 for seller-initiated trades. They differ because dealers often execute inside the quotes, and "one of this paper's headline empirical results is that the end-of-day quoted spread overstates the effective spread by up to 100%." For a cost model the effective spread is the right object and the harder one, since P̃ is never observed.
-The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid–ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed — Roll additionally required equally likely buys and sells; Corwin–Schultz and Abdi–Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
+The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid-ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed - Roll additionally required equally likely buys and sells; Corwin-Schultz and Abdi-Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
         </is>
       </c>
       <c r="H54" s="9" t="inlineStr">
@@ -7289,28 +7289,28 @@
       </c>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>Two evaluations (a simulation and a CRSP–TAQ empirical study) plus three applications.
+          <t>Two evaluations (a simulation and a CRSP-TAQ empirical study) plus three applications.
 Simulation: Corwin and Schultz (2012) design as reused by Abdi and Ranaldo (2017). 10,000 months, each 21 trading days, each day 390 minutes. Fundamental price P̃_m = P̃_{m−1}e^{σz}, P̃_0 = 1, z standard Gaussian. Daily sd 3%, per-minute sd 3%/√390. Trade prices are P̃_m times one minus (plus) half the spread, 50% chance of a bid (ask). Trade probability varied so expected trades per day runs from 1 to 390. On no-trade days the previous day's close is forward-filled into all four prices. Spreads tested: 0.50%, 1.00%, 2.00% through 8.00%.
-Empirical: CRSP US Stock Database, 1926–2021, NYSE / AMEX / NASDAQ, share codes 10 and 11. Benchmark is the Holden and Jacobsen (2014) effective spread from TAQ, May 1993 – December 2021. Merged sample 1,637,621 stock-months, CUSIP and ticker matching recovering 99% of CRSP stocks. Intraday sample 711,161 stock-months with both minute and daily estimates, October 2003 – December 2021. Crypto: Binance, 2163 pairs, 53,865 pair-months, July 2017 – December 2021, at daily / hourly / minute frequency.
-Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high–low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
+Empirical: CRSP US Stock Database, 1926–2021, NYSE / AMEX / NASDAQ, share codes 10 and 11. Benchmark is the Holden and Jacobsen (2014) effective spread from TAQ, May 1993 - December 2021. Merged sample 1,637,621 stock-months, CUSIP and ticker matching recovering 99% of CRSP stocks. Intraday sample 711,161 stock-months with both minute and daily estimates, October 2003 - December 2021. Crypto: Binance, 2163 pairs, 53,865 pair-months, July 2017 - December 2021, at daily / hourly / minute frequency.
+Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high-low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
         </is>
       </c>
       <c r="J54" s="9" t="inlineStr">
         <is>
-          <t>Daily (or intraday) open, high, low and close prices and nothing else. No quote feed, no trade-by-trade data, no vendor dependency. The derived quantities are: o_t, h_t, l_t, c_t as log-prices; η_t = (h_t + l_t)/2 the mid log-price; and the indicator τ_t that flags whether the high, the low and the previous close all coincide. The note flags the τ_t indicator as itself a usable feature — "the fraction of days on which the open or close coincides with the high or low, which falls out of the EDGE computation at no extra cost".</t>
+          <t>Daily (or intraday) open, high, low and close prices and nothing else. No quote feed, no trade-by-trade data, no vendor dependency. The derived quantities are: o_t, h_t, l_t, c_t as log-prices; η_t = (h_t + l_t)/2 the mid log-price; and the indicator τ_t that flags whether the high, the low and the previous close all coincide. The note flags the τ_t indicator as itself a usable feature - "the fraction of days on which the open or close coincides with the high or low, which falls out of the EDGE computation at no extra cost".</t>
         </is>
       </c>
       <c r="K54" s="9" t="inlineStr">
         <is>
           <t>"There is no architecture, this is an estimator, and the whole mechanism rests on one indicator variable."
 τ_t = 0 if h_t = l_t = c_{t−1}, and 1 otherwise.
-τ_t = 0 flags the case where high, low and previous close all coincide, meaning either that every trade in the period executed at the previous closing price — "which becomes increasingly likely as trades per period fall" — or that there was no trading at all and the four prices were filled forward. Setting τ_t = 0 on those periods prevents the estimator from treating a forward-filled price as evidence about the spread, and conditioning every expectation on τ_t = 1 is what makes the derivation go through without assuming continuous observation.
+τ_t = 0 flags the case where high, low and previous close all coincide, meaning either that every trade in the period executed at the previous closing price - "which becomes increasingly likely as trades per period fall" - or that there was no trading at all and the four prices were filled forward. Setting τ_t = 0 on those periods prevents the estimator from treating a forward-filled price as evidence about the spread, and conditioning every expectation on τ_t = 1 is what makes the derivation go through without assuming continuous observation.
 The spread estimator measured at the open:
 S_o² = −8·E[(η̄_t − ō_t)(o_t − c_{t−1})] / ( P[o_t ≠ h_t, τ_t = 1] + P[o_t ≠ l_t, τ_t = 1] )
 where bars denote de-meaned returns, r̄_t = r_t − τ_t·E[r_t]/E[τ_t], "which is the de-meaning that survives the conditioning on τ_t". The denominator is the entire discreteness correction and is the only thing separating this from the classical form: if prices are observed continuously the open and close can never coincide with the high or low, both probabilities equal one, the denominator collapses to two, and the expression reverts to the familiar −4E[·] shape.
 The note's reading: "The correction is therefore not a robustness patch bolted onto an existing estimator, it is a term that is identically one under the old assumption and shrinks the denominator, inflating the spread estimate, exactly in proportion to how often the price failed to move within the period."
-The same construction over other price combinations gives four Discrete Generalized Estimators — OHL, CHL, OHLC and CHLO — the first pair measuring the spread at the open and the second at the close. Their CHL estimator reduces exactly to the Abdi and Ranaldo (2017) estimator when continuous observation is imposed and returns are zero-mean, "so the prior work is recovered as a special case rather than contradicted."
-Efficiency half: the four estimators behave in opposite ways — when the spread is small relative to volatility the estimators using the mid-price have lower variance, and when the spread is large and observed returns are driven by bid–ask bounces, pairing mid-to-open with open-to-mid returns cancels a variance term that pairing with the closing price does not. Combining OHL with CHLO and OHLC with CHLO gives two moment conditions, and GMM with a diagonal weighting matrix reduces to a variance-weighted average:
+The same construction over other price combinations gives four Discrete Generalized Estimators - OHL, CHL, OHLC and CHLO - the first pair measuring the spread at the open and the second at the close. Their CHL estimator reduces exactly to the Abdi and Ranaldo (2017) estimator when continuous observation is imposed and returns are zero-mean, "so the prior work is recovered as a special case rather than contradicted."
+Efficiency half: the four estimators behave in opposite ways - when the spread is small relative to volatility the estimators using the mid-price have lower variance, and when the spread is large and observed returns are driven by bid-ask bounces, pairing mid-to-open with open-to-mid returns cancels a variance term that pairing with the closing price does not. Combining OHL with CHLO and OHLC with CHLO gives two moment conditions, and GMM with a diagonal weighting matrix reduces to a variance-weighted average:
 S²_EDGE = w₁·E[x_{1,t}] + w₂·E[x_{2,t}]
 x_{1,t} = (π_o/2)(η̄_t − ō_t)(o_t − η_{t−1}) + (π_c/2)(η̄_{t−1} − c̄_{t−1})(c_{t−1} − η_{t−1})
 x_{2,t} = (π_o/2)(η̄_t − ō_t)(o_t − c_{t−1}) + (π_c/2)(ō_t − c̄_{t−1})(c_{t−1} − η_{t−1})
@@ -7321,41 +7321,41 @@
       </c>
       <c r="L54" s="9" t="inlineStr">
         <is>
-          <t>Not applicable — this is a closed-form econometric estimator with no agents, no decision and no orchestration. The note states it plainly: "This is tooling, not a competitor architecture, there is no agent in it and no trading decision, but it goes at the part of my design that is currently weakest."</t>
+          <t>Not applicable - this is a closed-form econometric estimator with no agents, no decision and no orchestration. The note states it plainly: "This is tooling, not a competitor architecture, there is no agent in it and no trading decision, but it goes at the part of my design that is currently weakest."</t>
         </is>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>Not applicable — the paper uses only OHLC prices and contains no textual or sentiment component. (Sentiment is out of scope for this project in any case, per the supervisor decision.)</t>
+          <t>Not applicable - the paper uses only OHLC prices and contains no textual or sentiment component. (Sentiment is out of scope for this project in any case, per the supervisor decision.)</t>
         </is>
       </c>
       <c r="N54" s="9" t="inlineStr">
         <is>
-          <t>Not applicable — no disclosures, filings, retrieval or text of any kind. The only inputs are the four daily prices.</t>
+          <t>Not applicable - no disclosures, filings, retrieval or text of any kind. The only inputs are the four daily prices.</t>
         </is>
       </c>
       <c r="O54" s="9" t="inlineStr">
         <is>
           <t>No volatility model is estimated, but volatility enters the paper twice as a nuisance that drives the estimator's error. First, through the truncation channel: because Ŝ² can come out negative in small samples, standard practice is to reset negatives to zero, and Jahan-Parvar and Zikes (2023) show this introduces a strong upward bias that does not decline with sample size, "with volatility as its primary driver". Second, through the spread-to-volatility ratio: the degradation of correlation with the TAQ benchmark over time is attributed by the authors to spreads shrinking relative to volatility, consistent with the spread-quintile table where correlation runs 17.84% in the narrowest quintile against 71.38% in the widest.
 The note also flags a tension with the volatility side of the project's own literature: Assumption 1 rules out serially correlated fundamental returns, "which sits uneasily beside the long-memory results on the ASPI and SL20 in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], though that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it."
-Estimation variance is roughly proportional to σ₁⁴/N for N observations at per-period volatility σ₁, so the standard error scales with σ₁²/√N — which is the formula behind the frequency result below.</t>
+Estimation variance is roughly proportional to σ₁⁴/N for N observations at per-period volatility σ₁, so the standard error scales with σ₁²/√N - which is the formula behind the frequency result below.</t>
         </is>
       </c>
       <c r="P54" s="9" t="inlineStr">
         <is>
-          <t>This is the whole paper. EDGE measures the effective spread — the realised cost of a marginal trade — directly, in basis points, from OHLC. The discreteness correction is explicitly a function of how thinly the asset trades: the probability that the open or close coincides with the high or low is "a direct consequence of too few trades per period", running from about 25% for large-cap US stocks to 75% for small-caps over 1926–2021, peaking in the 1930s and 1940s, collapsing after 2000 with electronification to roughly 2–5% for large-caps while small-caps still sit near 15% at the end of the sample. The authors' own reading is that "the correction is less significant for recent samples and becomes essential for small stocks and for older periods, and crucially that it also depends on sampling frequency, since going from daily to intraday prices reduces the trades observed per interval and pushes the probability back up."
+          <t>This is the whole paper. EDGE measures the effective spread - the realised cost of a marginal trade - directly, in basis points, from OHLC. The discreteness correction is explicitly a function of how thinly the asset trades: the probability that the open or close coincides with the high or low is "a direct consequence of too few trades per period", running from about 25% for large-cap US stocks to 75% for small-caps over 1926–2021, peaking in the 1930s and 1940s, collapsing after 2000 with electronification to roughly 2–5% for large-caps while small-caps still sit near 15% at the end of the sample. The authors' own reading is that "the correction is less significant for recent samples and becomes essential for small stocks and for older periods, and crucially that it also depends on sampling frequency, since going from daily to intraday prices reduces the trades observed per interval and pushes the probability back up."
 What the paper does NOT handle: order size. "There is no order size anywhere in the model, so what EDGE measures is the cost of a marginal trade." The effective spread is computed from the transaction prices that happened, at whatever sizes they happened in, and the estimator has no mechanism for saying what a larger order would have paid.</t>
         </is>
       </c>
       <c r="Q54" s="9" t="inlineStr">
         <is>
-          <t>Not applicable in the ML sense — there is no black box. The estimator is closed-form, every term is interpretable, and the discreteness correction has a direct structural reading (the denominator is one under continuous observation and shrinks in proportion to how often the price failed to move). Reproducibility is strong: implementations in several languages, the computed spread data, and a Harvard Dataverse replication package.</t>
+          <t>Not applicable in the ML sense - there is no black box. The estimator is closed-form, every term is interpretable, and the discreteness correction has a direct structural reading (the denominator is one under continuous observation and shrinks in proportion to how often the price failed to move). Reproducibility is strong: implementations in several languages, the computed spread data, and a Harvard Dataverse replication package.</t>
         </is>
       </c>
       <c r="R54" s="9" t="inlineStr">
         <is>
-          <t>Baselines: ROLL (Roll 1984), CS (Corwin and Schultz 2012), AR (Abdi and Ranaldo 2017), plus the paper's own intermediate estimators OHLC and CHL. Benchmark truth is the Holden and Jacobsen (2014) TAQ-based effective spread, May 1993 – December 2021.
-Evaluation axes: (i) simulation bias as a function of expected trades per day from 390 down to 1; (ii) simulation mean and standard deviation across true spreads 0.50%–8.00%; (iii) empirical Pearson and Spearman correlation, MAPE, RMSE and fraction of non-positive estimates on 1,637,621 merged stock-months, cut by market venue, sub-period, size quintile and decile, spread quintile and trading-frequency quintile; (iv) daily versus minute sampling on 711,161 stock-months; (v) the Binance crypto application across daily / hourly / minute, which has no benchmark.
+          <t>Baselines: ROLL (Roll 1984), CS (Corwin and Schultz 2012), AR (Abdi and Ranaldo 2017), plus the paper's own intermediate estimators OHLC and CHL. Benchmark truth is the Holden and Jacobsen (2014) TAQ-based effective spread, May 1993 - December 2021.
+Evaluation axes: (i) simulation bias as a function of expected trades per day from 390 down to 1; (ii) simulation mean and standard deviation across true spreads 0.50% - 8.00%; (iii) empirical Pearson and Spearman correlation, MAPE, RMSE and fraction of non-positive estimates on 1,637,621 merged stock-months, cut by market venue, sub-period, size quintile and decile, spread quintile and trading-frequency quintile; (iv) daily versus minute sampling on 711,161 stock-months; (v) the Binance crypto application across daily / hourly / minute, which has no benchmark.
 The note records a caveat on the empirical comparison: "The comparison is descriptive throughout, no standard errors on the differences and no formal test, which at this sample size is defensible but means the quintile tables are read by eye."</t>
         </is>
       </c>
@@ -7369,17 +7369,17 @@
 3.00% | 2.89 (0.83) | 2.76 (1.23) | 2.86 (1.19) | 2.26 (0.92) | 0.35 (0.36) | 2.89 (1.82)
 8.00% | 8.19 (0.96) | 8.10 (1.59) | 8.20 (1.26) | 6.59 (0.94) | 2.66 (0.96) | 7.71 (2.65)
 EDGE is within 0.21 of the true value at every spread size while AR is 1.41 low at 8.00% and CS is 5.34 low, and EDGE's standard deviation is the smallest or tied at every row. CS's small standard deviations are "the collapse to zero rather than precision". The uniformity comes from the building blocks swapping roles, OHLC and CHLO carrying lower variance for small spreads and OHL and CHL for large, with EDGE shifting weight between them rather than being tuned to a favoured region.
-3. Empirical dominance, widest where trading is thinnest. Against the TAQ benchmark EDGE achieves Pearson 78.86%, Spearman 66.68%, MAPE 16.21, RMSE 1.23, non-positive estimates 25.63% — against AR at 68.13 / 53.55 / 19.90 / 1.41 / 31.87 and CS at 45.55 / 33.77 / 35.90 / 2.61 / 29.18. EDGE is highest in every market venue, sub-period, size quintile, spread quintile and trading-frequency quintile. On the trading-frequency cut, EDGE scores 74.77% in the least-traded quintile falling to 55.48% in the most-traded, while ROLL runs the other way at 65.10% down to 22.29% and AR falls from 67.81% to 39.36%. The size-decile plot has the same shape, EDGE flat near 70% across all ten deciles while the others spread out below it. "The lead is therefore not an average that washes out in the hard cases, it is largest in the hard cases, which is the property a frontier-market application needs."
+3. Empirical dominance, widest where trading is thinnest. Against the TAQ benchmark EDGE achieves Pearson 78.86%, Spearman 66.68%, MAPE 16.21, RMSE 1.23, non-positive estimates 25.63% - against AR at 68.13 / 53.55 / 19.90 / 1.41 / 31.87 and CS at 45.55 / 33.77 / 35.90 / 2.61 / 29.18. EDGE is highest in every market venue, sub-period, size quintile, spread quintile and trading-frequency quintile. On the trading-frequency cut, EDGE scores 74.77% in the least-traded quintile falling to 55.48% in the most-traded, while ROLL runs the other way at 65.10% down to 22.29% and AR falls from 67.81% to 39.36%. The size-decile plot has the same shape, EDGE flat near 70% across all ten deciles while the others spread out below it. "The lead is therefore not an average that washes out in the hard cases, it is largest in the hard cases, which is the property a frontier-market application needs."
 4. Sampling frequency beats sampling length by three orders of magnitude. Standard error scales as σ₁²/√N. Going from a monthly sample of daily prices (N = 21) to a yearly one (N = 252) reduces the standard error by √(252/21) = 3.5 times; going instead to a monthly sample of minute prices (N = 21 × 390) reduces it by 390^{3/2} = 7702 times, which the authors note would take 1,245,699,037 daily prices to match, roughly five million years of trading. Empirically, on 711,161 stock-months, moving from daily to minute prices: negative estimates fall from 34.15% to 0.02%, Pearson rises from 56.17% to 88.79%, Spearman from 43.47% to 97.31%, MAPE from 23.68 to 5.17. The crypto application makes the point from the other side: AR and CS differ roughly tenfold between daily and minute sampling (0.18% against 0.02%, and 1.85% against 1.45% respectively) while EDGE stays within 0.68% to 0.70% at every frequency, "so the frequency-insensitivity is a property of the estimator rather than of the US sample."
-5. The discreteness term is itself a market-structure measurement: the coincidence probability ranges from ~25% (US large-cap) to 75% (small-cap) over 1926–2021, peaking in the 1930s–40s, collapsing after 2000 to 2–5% for large-caps with small-caps still near 15%.</t>
+5. The discreteness term is itself a market-structure measurement: the coincidence probability ranges from ~25% (US large-cap) to 75% (small-cap) over 1926–2021, peaking in the 1930s - 40s, collapsing after 2000 to 2–5% for large-caps with small-caps still near 15%.</t>
         </is>
       </c>
       <c r="T54" s="9" t="inlineStr">
         <is>
-          <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% — "a bias roughly seven times the quantity being measured" — and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
-2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid–ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information — Chen et al. (2017) being their example — is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
+          <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% - "a bias roughly seven times the quantity being measured" - and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
+2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid-ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information - Chen et al. (2017) being their example - is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
 3. No order size anywhere in the model. For a deep market the marginal-trade cost is close enough; "for a book where a single order can be a meaningful fraction of daily volume it is the intercept of a cost function and not the function." The scope is honest and never overclaimed, but EDGE answers only the first of the four open items in my cost work and leaves the nonlinear impact form, the participation-rate sweep and the thin-book depth calibration untouched.
-4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden–Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility — "plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation." The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
+4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden-Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility - "plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation." The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
 5. The estimator needs at least three usable observations per stock-month and the paper never reports performance conditional on a small count. Periods with τ_t = 0 are excluded, and EDGE is missing in 1.24% of CRSP stock-months on that basis. "The thinnest cut they report is the bottom trading-frequency quintile of US-listed stocks, which still trades most days. For a counter with five trading days in a month the estimator is defined and will return a number computed from a handful of covariance terms, deep inside the small-sample regime where their own truncation bias is worst, and nothing in the paper tells me how that number behaves. That is the gap between what the paper validates and what I would be doing with it."
 6. The simulation's "infrequent trading" is not frontier-market infrequent. Panel B sets the daily trade probability to 1%, which on a 390-minute day means roughly four expected trades per day, and the bias plot extends down to one trade per day. "That is thin by US standards and it is the right stress test for the method, but a CSE counter in the bottom half of a liquidity screen can go whole days without a trade, and the paper's design forward-fills those days rather than modelling a counter that trades on five days in a month. The estimator handles the forward-fill correctly through its indicator; what is untested is the regime where the number of usable observations per stock-month falls into single digits."
 7. A premise doing quiet work throughout: that the effective spread is the whole of the transaction cost, since nothing in the model has an order size in it. The paper never claims otherwise and the title is honest about scope.</t>
@@ -7400,19 +7400,19 @@
 - The two candidate L_t inputs, the measured spread and the tau_t staleness indicator. Both fall out of an EDGE computation and are therefore not computed. L_t stays on Amihud, turnover, zero-return frequency and the high-low range.
 - The forced window decision (quarterly per-counter, monthly index-track, non-positive fraction reported alongside every series). Moot unless EDGE is revived, and retained below only as the specification to follow if it ever is.
 --- RETAINED AS RECORD, SUPERSEDED ---
-- EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC — the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
+- EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC - the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
 - The infrequent-trading bias result as external evidence that thin-book calibration is a real problem, not a rhetorical one: below roughly thirteen trades per day CS returns exactly zero and AR is biased down by about a third at a few trades per day, "which means any cost model built on those estimators would charge approximately nothing for trading the least liquid counters on the CSE. That is backwards in the most expensive possible direction." Worth citing directly in the proposal when defending the thin-book calibration item.
-- Two new candidate inputs to the liquidity state L_t. (a) The measured spread itself, which unlike Amihud (price impact per unit volume), turnover (activity) and zero-return frequency (staleness) "is denominated in the same units as the objective". (b) The τ_t indicator — the fraction of days on which the open or close coincides with the high or low — which "falls out of the EDGE computation at no extra cost" and is a candidate staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both go into the ablation protocol "as additions to test rather than adopt".
-- A forced window decision. Given 25.63% non-positive daily-price estimates on CRSP and 41% negative for large-caps, and a monthly estimate from the per-counter archive being roughly 21 observations — "squarely in that regime" — the decision is a quarterly window on the per-counter track, accepting a cost term that cannot move within a quarter, and monthly on the index track where ten years of daily data supports it, "with the fraction of non-positive estimates reported alongside every spread series in both cases. Reporting that fraction is not optional here, it is the only visible signal that the truncation is distorting the number."
+- Two new candidate inputs to the liquidity state L_t. (a) The measured spread itself, which unlike Amihud (price impact per unit volume), turnover (activity) and zero-return frequency (staleness) "is denominated in the same units as the objective". (b) The τ_t indicator - the fraction of days on which the open or close coincides with the high or low - which "falls out of the EDGE computation at no extra cost" and is a candidate staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both go into the ablation protocol "as additions to test rather than adopt".
+- A forced window decision. Given 25.63% non-positive daily-price estimates on CRSP and 41% negative for large-caps, and a monthly estimate from the per-counter archive being roughly 21 observations - "squarely in that regime" - the decision is a quarterly window on the per-counter track, accepting a cost term that cannot move within a quarter, and monthly on the index track where ten years of daily data supports it, "with the fraction of non-positive estimates reported alongside every spread series in both cases. Reporting that fraction is not optional here, it is the only visible signal that the truncation is distorting the number."
 - A reversal of my data priority. A month of minute prices gives a standard error 7702 times smaller than a month of daily prices, where a year of daily prices gives only 3.5 times. "So if any intraday CSE feed exists at any granularity, even hourly or five-minute, it is worth far more to the cost model than extending the daily archive backwards." This is a question to put to the supervisor before spending time on data depth, and it connects to the volatility estimator decision too, "since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE."
 - A positioning rule. EDGE is a 2024 JFE paper with public implementations, open spread data and a replication package, "so there is no contribution in running it on a new market and no reason to imply one." The defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered, and that the contribution is what an orchestrator does with a cost term that varies by counter and date rather than the estimator that produces it. "One sentence, offered before anyone asks."</t>
         </is>
       </c>
       <c r="V54" s="9" t="inlineStr">
         <is>
-          <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
+          <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren-Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
 Second, the small-count regime is untested: the estimator is defined with three usable observations but the paper never characterises its behaviour there, and that is exactly the regime a CSE counter with five trading days in a month occupies.
-Third, the paper measures a spread; it never puts that spread inside a decision objective. "It sits alongside [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] as the measurement layer those papers assume and never supply." The claim that cost belongs inside the objective rather than deducted afterwards is still mine to make — and now has two separately validated pieces behind the cost term.
+Third, the paper measures a spread; it never puts that spread inside a decision objective. "It sits alongside [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] as the measurement layer those papers assume and never supply." The claim that cost belongs inside the objective rather than deducted afterwards is still mine to make - and now has two separately validated pieces behind the cost term.
 Fourth, no validation against a quote-based benchmark in an emerging or frontier market: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
 AMENDED 11 OCTOBER 2026: with EDGE demoted to last resort, the INTERCEPT of the cost function is open as well, not only the slope. The whole cost term now rests on proxies until real CSE quotes are obtained, which makes the CSE request for bid/ask and depth materially more important than v5 recorded - it is no longer a validation step for an estimator already built, it is the only route to a measured spread.</t>
         </is>
@@ -7425,13 +7425,13 @@
 The text below is retained as the record of the evaluation that produced this decision, in the same way the Dataset sheet keeps its excluded rows rather than deleting them. Read it as superseded.
 AMENDED EFFECT ON SUB-GAP 1, 11 OCTOBER 2026: the claim below that this paper CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 is WITHDRAWN. With EDGE demoted, the measurement half is open again and the cost term stays on the existing proxies until real CSE quotes are obtained. Sub-gap 1 is therefore stated with two caveats rather than one: a potentially overlapping 2026 paper (Smart Trading Rule) was identified and could not be obtained, AND the proxy route that would have substituted for the missing quote data is not validated on any market resembling the CSE. That is a weaker position than v5 recorded and it should be stated as such rather than discovered in the viva.
 --- RETAINED AS RECORD, SUPERSEDED ---
-SPEAKS TO: A_L above all — this is the measurement instrument the liquidity agent currently lacks — plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
-EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency — "all proxies for illiquidity rather than measurements of what a trade pays" — and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade — "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren–Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
-The second half of Sub-gap 1 — that liquidity simultaneously conditions the reliability of price-derived agents — gets independent support from the paper's own mechanism rather than from my framing. The τ_t = 0 condition is literally the case where the price carries no information about the spread within the period, and the coincidence probability that drives the correction is "a direct consequence of too few trades per period". That is a measured, published statement that price-derived quantities degrade in a specific, quantifiable way as trading thins — which is precisely the premise under which L_t should down-weight A_T.
+SPEAKS TO: A_L above all - this is the measurement instrument the liquidity agent currently lacks - plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
+EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency - "all proxies for illiquidity rather than measurements of what a trade pays" - and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade - "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren-Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
+The second half of Sub-gap 1 - that liquidity simultaneously conditions the reliability of price-derived agents - gets independent support from the paper's own mechanism rather than from my framing. The τ_t = 0 condition is literally the case where the price carries no information about the spread within the period, and the coincidence probability that drives the correction is "a direct consequence of too few trades per period". That is a measured, published statement that price-derived quantities degrade in a specific, quantifiable way as trading thins - which is precisely the premise under which L_t should down-weight A_T.
 EFFECT ON MAIN GAP: Indirect but real. The main gap is market-state-aware dynamic orchestration with w(i,t) = f(L_t, V_t, P_t, C_{i,t}), and the weakest-specified argument of that function is L_t. This paper contributes two candidate components to it that measure something the existing three proxies do not. The spread gives L_t a component denominated in the same units as the objective. The τ_t indicator gives a staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both enter the ablation protocol as additions to test rather than adopt, "which turns the question from whether liquidity matters into whether a measured spread and a measured staleness rate carry anything beyond the three proxies already there." That reframing is itself useful: it converts a soft claim about liquidity-awareness into a falsifiable ablation.
-EFFECT ON SUB-GAP 2: Minimal and only by friction. The paper estimates no volatility model and says nothing about persistence. The one contact point is Assumption 1, which rules out serially correlated fundamental returns and "sits uneasily beside the long-memory results on the ASPI and SL20" in the CSE volatility-memory work — but the note is careful that "that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it." So this does not move Sub-gap 2. There is one indirect operational link: the frequency result argues that any intraday CSE feed is worth far more to the cost model than more daily history, "and it connects to the volatility estimator decision too, since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE." The two data questions are the same question.
-CSE DATA EVIDENCE: The note's CSE-side commitments are: the CSE publishes daily OHLC for every listed counter, which is what makes EDGE applicable with no quote feed; the per-counter archive is roughly 374 trading days, giving ~21 observations per monthly estimate — "squarely in that regime" where 25.63% of CRSP daily-price estimates come out non-positive and 41% of large-cap stock-months come out negative before truncation; and a CSE counter in the bottom half of a liquidity screen "can go whole days without a trade", below anything the paper's simulation stresses (its thinnest panel is ~4 expected trades per day, with the bias plot extending to one trade per day, and no-trade days forward-filled rather than genuinely absent). The resulting design decisions are a quarterly window on the per-counter track, monthly on the index track where ten years of daily data supports it, and the fraction of non-positive estimates reported alongside every spread series in both cases.
-PROPOSED REVISION STATED IN THE NOTE: Re-scope the cost sub-gap as "EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part" — narrower and more defensible than the earlier wording, using this paper as support rather than letting it look like competition. Claim EDGE as an adopted measurement with the implementation cited and keep all novelty language off it; the one defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered. Add the measured spread and the τ_t staleness rate to the liquidity-state ablation as candidates to test rather than adopt. Fix the aggregation window before running anything (quarterly per-counter, monthly index-track) and report the non-positive fraction every time. Put the intraday-feed question to the supervisor before investing in deeper daily history.</t>
+EFFECT ON SUB-GAP 2: Minimal and only by friction. The paper estimates no volatility model and says nothing about persistence. The one contact point is Assumption 1, which rules out serially correlated fundamental returns and "sits uneasily beside the long-memory results on the ASPI and SL20" in the CSE volatility-memory work - but the note is careful that "that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it." So this does not move Sub-gap 2. There is one indirect operational link: the frequency result argues that any intraday CSE feed is worth far more to the cost model than more daily history, "and it connects to the volatility estimator decision too, since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE." The two data questions are the same question.
+CSE DATA EVIDENCE: The note's CSE-side commitments are: the CSE publishes daily OHLC for every listed counter, which is what makes EDGE applicable with no quote feed; the per-counter archive is roughly 374 trading days, giving ~21 observations per monthly estimate - "squarely in that regime" where 25.63% of CRSP daily-price estimates come out non-positive and 41% of large-cap stock-months come out negative before truncation; and a CSE counter in the bottom half of a liquidity screen "can go whole days without a trade", below anything the paper's simulation stresses (its thinnest panel is ~4 expected trades per day, with the bias plot extending to one trade per day, and no-trade days forward-filled rather than genuinely absent). The resulting design decisions are a quarterly window on the per-counter track, monthly on the index track where ten years of daily data supports it, and the fraction of non-positive estimates reported alongside every spread series in both cases.
+PROPOSED REVISION STATED IN THE NOTE: Re-scope the cost sub-gap as "EDGE for the spread and an Almgren-Chriss or queue-reactive treatment for the size-dependent part" - narrower and more defensible than the earlier wording, using this paper as support rather than letting it look like competition. Claim EDGE as an adopted measurement with the implementation cited and keep all novelty language off it; the one defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered. Add the measured spread and the τ_t staleness rate to the liquidity-state ablation as candidates to test rather than adopt. Fix the aggregation window before running anything (quarterly per-counter, monthly index-track) and report the non-positive fraction every time. Put the intraday-feed question to the supervisor before investing in deeper daily history.</t>
         </is>
       </c>
       <c r="X54" s="9" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Wang, X., Hyndman, R.J., Li, F. and Kang, Y. (2023). Forecast combinations: An over 50-year review. International Journal of Forecasting, 39(4), 1518–1547. DOI: 10.1016/j.ijforecast.2022.11.005. arXiv version 2205.04216v2 dated 26 September 2022. Affiliations: Xiaoqian Wang and Yanfei Kang at Beihang, Rob J Hyndman at Monash, Feng Li at the Central University of Finance and Economics — "about as authoritative an author list as this particular topic has". Citekey: wangForecastCombinations50year2023.</t>
+          <t>Wang, X., Hyndman, R.J., Li, F. and Kang, Y. (2023). Forecast combinations: An over 50-year review. International Journal of Forecasting, 39(4), 1518–1547. DOI: 10.1016/j.ijforecast.2022.11.005. arXiv version 2205.04216v2 dated 26 September 2022. Affiliations: Xiaoqian Wang and Yanfei Kang at Beihang, Rob J Hyndman at Monash, Feng Li at the Central University of Finance and Economics - "about as authoritative an author list as this particular topic has". Citekey: wangForecastCombinations50year2023.</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
@@ -7469,17 +7469,17 @@
       </c>
       <c r="F55" s="11" t="inlineStr">
         <is>
-          <t>Forecast combination / forecast pooling — a narrative review of over fifty years of work on combining multiple forecasts of the same quantity, from Bates and Granger (1969) (and behind that Galton's 1906 ox-weight competition, where the average of 787 estimates came close to the animal's actual weight) through to the feature-based cross-learning methods that placed in M4. Organising split: point forecast combinations (section 2), probabilistic forecast combinations (section 3), eight open problems in closing, with a running commentary on which R and Python packages implement what.
+          <t>Forecast combination / forecast pooling - a narrative review of over fifty years of work on combining multiple forecasts of the same quantity, from Bates and Granger (1969) (and behind that Galton's 1906 ox-weight competition, where the average of 787 estimates came close to the animal's actual weight) through to the feature-based cross-learning methods that placed in M4. Organising split: point forecast combinations (section 2), probabilistic forecast combinations (section 3), eight open problems in closing, with a running commentary on which R and Python packages implement what.
 This is the most direct body of prior art on the orchestration half of my design. As the note puts it: "My orchestrator computes w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) over four heterogeneous agent outputs, and that object is a time-varying, feature-conditioned linear combination, which is a named construct in this literature with five decades of results attached to it, a good number of them inconvenient." It belongs next to the RL-in-quant-finance survey as the other half of the prior art: "that one establishes that coordination protocols among heterogeneous agents are underexplored in RL, this one establishes what fifty years of statistics already knows about combining their outputs once they exist."</t>
         </is>
       </c>
       <c r="G55" s="11" t="inlineStr">
         <is>
-          <t>Update the field's standing reviews — Clemen (1989) and Timmermann (2006) — and, structurally, set point and probabilistic combination side by side for the first time in a single survey. Three gaps motivate it:
+          <t>Update the field's standing reviews - Clemen (1989) and Timmermann (2006) - and, structurally, set point and probabilistic combination side by side for the first time in a single survey. Three gaps motivate it:
 1. Both standing reviews predate the entire cross-learning and meta-learning strand, the M4 and M5 competitions, most of the probabilistic combination work, and the open-source tooling that now carries these methods into practice. The authors' Web of Science count puts combination papers at "13.80% of all published forecasting papers in 2021", up from roughly 1% in 1969, "so the case for an update is quantitative rather than rhetorical."
 2. Point and probabilistic combination had developed in parallel without being contrasted. In probabilistic combination, diversity among individuals becomes "more complex and less understood", and calibration and sharpness enter as considerations with no analogue in the point case. "Setting the two side by side is the structural contribution, and it is what produces the review's most useful result for me, because several intuitions do not survive the crossing."
 3. Model averaging and forecast combination get used interchangeably and shouldn't be. Model averaging is a general term for handling model uncertainty, chiefly in parameter estimation, with frequentist and Bayesian strands; forecast combination is narrower, operating on forecasts whose origin is irrelevant, carrying assumptions intended to keep the combination unbiased or optimal. "That is the right frame for my case, because my agents are not models of the same process with different parameters, they are methodologically different producers, and only the second framing accommodates that."
-The central empirical claim restated across fifty years of evidence: "the equally weighted average is extremely hard to beat", and the literature has a name for its own embarrassment about this — the forecast combination puzzle.
+The central empirical claim restated across fifty years of evidence: "the equally weighted average is extremely hard to beat", and the literature has a name for its own embarrassment about this - the forecast combination puzzle.
 SCOPE BOUND (the note flags this as bounding everything else): the authors take the individual forecasts "as given", do not discuss how they are generated, and restrict attention to forecasts derived from separate and non-interfering models for a single target series. Two adjacent literatures are named and excluded: manipulating one series into many and combining the results (Petropoulos and Spiliotis' "wisdom of the data", covering theta, bagging and temporal aggregation), and forecast reconciliation for hierarchical series following Hyndman et al. (2011). The target is always a realised value of one series and the loss is almost always quadratic. "There are no portfolios, no transaction costs, no execution, and no decisions. So this is prior art on the weighting mechanism and on the evidence about weighting, not on anything downstream of it, and the non-interfering assumption in particular is one my design may violate."</t>
         </is>
       </c>
@@ -7490,17 +7490,17 @@
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>No dataset of its own — the authors run no experiment. The evidence base is other people's results on M-competition data (M3, M4 at 100,000 series, M5), FRED, and individual case studies. Coverage spans 1969 to roughly 2022, with the Web of Science publication-share chart (Figure 1) the only quantitative artefact the authors produce. "There is no protocol, no screening count, and no stated inclusion criterion anywhere in the paper."</t>
+          <t>No dataset of its own - the authors run no experiment. The evidence base is other people's results on M-competition data (M3, M4 at 100,000 series, M5), FRED, and individual case studies. Coverage spans 1969 to roughly 2022, with the Web of Science publication-share chart (Figure 1) the only quantitative artefact the authors produce. "There is no protocol, no screening count, and no stated inclusion criterion anywhere in the paper."</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>Univariate time series forecasts (point and probabilistic) as the inputs to be combined. The feature strand is the one that matters: FFORMA (Montero-Manso et al., 2020) extracts 42 statistical features of the series with the tsfeatures package and maps them to weights via an XGBoost meta-model. Collopy and Armstrong (1992) is the ancestor — a hand-built rule base of 99 rules over 18 time series features and four statistical models — and "the line from there to XGBoost over 42 features is the clearest trajectory in the paper." The feature pool has itself become a research object: Lemke and Gabrys (2010) add six features measuring diversity of the method pool rather than properties of the series, and Kang et al. (2021) build a combination model from a diversity matrix alone.</t>
+          <t>Univariate time series forecasts (point and probabilistic) as the inputs to be combined. The feature strand is the one that matters: FFORMA (Montero-Manso et al., 2020) extracts 42 statistical features of the series with the tsfeatures package and maps them to weights via an XGBoost meta-model. Collopy and Armstrong (1992) is the ancestor - a hand-built rule base of 99 rules over 18 time series features and four statistical models - and "the line from there to XGBoost over 42 features is the clearest trajectory in the paper." The feature pool has itself become a research object: Lemke and Gabrys (2010) add six features measuring diversity of the method pool rather than properties of the series, and Kang et al. (2021) build a combination model from a diversity matrix alone.</t>
         </is>
       </c>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>Not an architecture — a taxonomy of weighting schemes. The framing holding section 2 together is a one-dimensional aggregator over an N-vector of h-step-ahead forecasts:
+          <t>Not an architecture - a taxonomy of weighting schemes. The framing holding section 2 together is a one-dimensional aggregator over an N-vector of h-step-ahead forecasts:
 ỹ_{T+h|T} = C(ŷ_{T+h|T}; w_{T+h|T}), linear case ỹ_{T+h|T} = w'_{T+h|T} ŷ_{T+h|T}
 The ladder of weighting schemes, from no estimation to estimation over a whole dataset of series:
 Family | What determines the weights | Data needed | Section
@@ -7515,51 +7515,51 @@
 Combining by learning | A meta-model over features of the series and of the method pool | A dataset of many series | 2.4
 OPTIMAL WEIGHTS (Bates and Granger 1969 for pairs, Newbold and Granger 1974 in general) minimise the variance of the combined forecast error:
 w^opt_{T+h|T} = Σ⁻¹_{T+h|T} 1 / (1' Σ⁻¹_{T+h|T} 1)
-with Σ the N×N covariance matrix of h-step forecast errors. If the individuals are unbiased and their error variances stable, the combination is unbiased and its error variance is no greater than the minimum across individuals — "the diversification result the whole field rests on. The catch is in the last sentence of that passage: in practice Σ is unknown and has to be estimated, and that single sentence generates most of the rest of the literature."
-REGRESSION WEIGHTS (Granger and Ramanathan 1984): three regimes — weights summing to one with no intercept, which reproduces Bates–Granger exactly; unconstrained with no intercept; and unconstrained with an intercept, which they argued is superior regardless of whether constituents are biased because the intercept absorbs the bias. De Menezes et al. (2000) push back that the unrestricted version needs stationarity and runs into serial correlation and multicollinearity. Aksu and Gunter (1992) found empirically that constraining weights to be nonnegative is at least as robust as the simple average while beating the other regression variants — "which is the practical reading I'd take."
+with Σ the N×N covariance matrix of h-step forecast errors. If the individuals are unbiased and their error variances stable, the combination is unbiased and its error variance is no greater than the minimum across individuals - "the diversification result the whole field rests on. The catch is in the last sentence of that passage: in practice Σ is unknown and has to be estimated, and that single sentence generates most of the rest of the literature."
+REGRESSION WEIGHTS (Granger and Ramanathan 1984): three regimes - weights summing to one with no intercept, which reproduces Bates-Granger exactly; unconstrained with no intercept; and unconstrained with an intercept, which they argued is superior regardless of whether constituents are biased because the intercept absorbs the bias. De Menezes et al. (2000) push back that the unrestricted version needs stationarity and runs into serial correlation and multicollinearity. Aksu and Gunter (1992) found empirically that constraining weights to be nonnegative is at least as robust as the simple average while beating the other regression variants - "which is the practical reading I'd take."
 PERFORMANCE-BASED, discounted variant (the one with a time dimension, and the one the note would implement first because it needs no pairwise estimation):
 w^{bg4}_{T+h|T,i} = ( Σ_{t=1}^{T} γ^t e²_{t|t−h,i} )⁻¹ / Σ_{j=1}^{N} ( Σ_{t=1}^{T} γ^t e²_{t|t−h,j} )⁻¹ , γ ≥ 1
-where e_{t|t−h,i} is the h-step error of method i made at t−h and realised at t, and γ controls how fast older errors are forgotten, with γ = 1 recovering the plain inverse-MSE weight over the full history. The rolling-window variant replaces the discount with a sum over the most recent ν observations. Both are adapted to non-stationary relationships between methods, and both, as Timmermann (2006) is quoted saying, "increase the variance of the parameter estimates and work quite poorly if the data generating process really is covariance stationary." Stock and Watson (1998) generalise by making weights inversely proportional to the kth power of MSE, so k=0 is equal weights and larger k concentrates on the best performer — "a single interpretable dial between the two extremes."
+where e_{t|t−h,i} is the h-step error of method i made at t−h and realised at t, and γ controls how fast older errors are forgotten, with γ = 1 recovering the plain inverse-MSE weight over the full history. The rolling-window variant replaces the discount with a sum over the most recent ν observations. Both are adapted to non-stationary relationships between methods, and both, as Timmermann (2006) is quoted saying, "increase the variance of the parameter estimates and work quite poorly if the data generating process really is covariance stationary." Stock and Watson (1998) generalise by making weights inversely proportional to the kth power of MSE, so k=0 is equal weights and larger k concentrates on the best performer - "a single interpretable dial between the two extremes."
 TIME-VARYING WEIGHTS: Diebold and Pauly (1987) use rolling weighted least squares and time-varying parameters that are either deterministic polynomial functions of time or stochastic; Deutsch et al. (1994) let weights switch abruptly or transition smoothly using switching and smooth transition regression; Terui and van Dijk (2002) model the coefficients as a random walk in state space estimated by the Kalman filter, with Raftery et al. (2010) adding forgetting factors to make the recursive update cheap.
 The note's key structural observation: "So the literature already contains weights that change over time, and it contains weights that change as a regression function of covariates, and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state. The closest thing is the smooth transition specification of Deutsch et al., where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step."
-COMBINING BY LEARNING: stacking series-by-series needs n meta-models for n series, "computationally expensive and wastes the training data". Cross-learning trains one meta-model across many series. M4 is the evidence: "the top three methods all used information across the whole dataset rather than a single series." FFORMA is the exemplar — 42 tsfeatures features, XGBoost meta-model mapping features to weights over nine traditional models fitted per series, second place in M4.
+COMBINING BY LEARNING: stacking series-by-series needs n meta-models for n series, "computationally expensive and wastes the training data". Cross-learning trains one meta-model across many series. M4 is the evidence: "the top three methods all used information across the whole dataset rather than a single series." FFORMA is the exemplar - 42 tsfeatures features, XGBoost meta-model mapping features to weights over nine traditional models fitted per series, second place in M4.
 PROBABILISTIC COMBINATION: the linear opinion pool is a finite mixture F̃(y_{T+h}|I_T) = Σ w_{T+h|T,i} F_i(y_{T+h}|I_T) with nonnegative weights summing to one. Its first two moments:
-μ̃ = Σ w_i μ_i   and   σ̃² = Σ w_i σ_i² + Σ w_i (μ_i − μ̃)²
+μ̃ = Σ w_i μ_i and σ̃² = Σ w_i σ_i² + Σ w_i (μ_i − μ̃)²
 The mean of the pooled distribution is exactly the linear point combination, so nothing changes there. The variance carries a second term in the disagreement between component means, so pooled variance exceeds the weighted average of component variances whenever the components disagree about location.
-Quantile combination (Vincentization, after Vincent 1912): Q̃_{T+h|T}(τ) = Σ w_{T+h|T,i} Q_{T+h|T,i}(τ) for 0 &lt; τ ≤ 1. The geometric statement, which the note calls "the clearest sentence in section 3": "quantile combination averages the individuals' cdfs horizontally while linear pooling averages them vertically." If components are in the same location-scale family the quantile average stays in it, so averaging normals gives a normal and is always unimodal, where linear pooling can be multimodal. Both share the same mean. Quantile averaging is sharper because it does not absorb disagreement in location as extra spread — Lichtendahl et al. (2013) and Busetti (2017) both come down on its side, the former arguing the average probability forecast is generally under-confident while the average quantile forecast is always sharper.</t>
+Quantile combination (Vincentization, after Vincent 1912): Q̃_{T+h|T}(τ) = Σ w_{T+h|T,i} Q_{T+h|T,i}(τ) for 0 &lt; τ ≤ 1. The geometric statement, which the note calls "the clearest sentence in section 3": "quantile combination averages the individuals' cdfs horizontally while linear pooling averages them vertically." If components are in the same location-scale family the quantile average stays in it, so averaging normals gives a normal and is always unimodal, where linear pooling can be multimodal. Both share the same mean. Quantile averaging is sharper because it does not absorb disagreement in location as extra spread - Lichtendahl et al. (2013) and Busetti (2017) both come down on its side, the former arguing the average probability forecast is generally under-confident while the average quantile forecast is always sharper.</t>
         </is>
       </c>
       <c r="L55" s="11" t="inlineStr">
         <is>
-          <t>Not applicable as implemented — "a paper with no architecture in it, no trading decision anywhere, and nothing resembling an agent". But this is the closest named prior art to my orchestrator: combination weights over heterogeneous producers are exactly the orchestration object, and the survey supplies the ladder from equal weights to feature-conditioned meta-learned weights.
+          <t>Not applicable as implemented - "a paper with no architecture in it, no trading decision anywhere, and nothing resembling an agent". But this is the closest named prior art to my orchestrator: combination weights over heterogeneous producers are exactly the orchestration object, and the survey supplies the ladder from equal weights to feature-conditioned meta-learned weights.
 CRITICAL CONSTRAINT: the non-interfering assumption. "The components here are separate models that do not see each other's outputs. Every LLM multi-agent trading system in my reading violates that: [[TradingAgents, Multi-Agents LLM Financial Trading Framework]] has agents debating, [[HedgeAgents, A Balanced-aware Multi-agent Financial Trading System]] runs conferences, and even the ones that do not communicate share the same underlying price history and the same disclosures. So the clean statistical properties derived here, the unbiasedness of the combination and the variance bound, hold under an assumption my pool does not satisfy. My four agents read overlapping data by construction, and the paper's own observation that component forecasts trained on overlapping information sets produce highly correlated errors is the mechanism by which that bites."
 Subset selection is named as prior art for an abstention channel: the paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme, citing Li et al. (2022).</t>
         </is>
       </c>
       <c r="M55" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — no textual or sentiment component anywhere; the inputs are numerical forecasts of a single target series. (Sentiment is out of scope for this project regardless, per the supervisor decision of 20 September 2026, status Final.)</t>
+          <t>Not applicable - no textual or sentiment component anywhere; the inputs are numerical forecasts of a single target series. (Sentiment is out of scope for this project regardless, per the supervisor decision of 20 September 2026, status Final.)</t>
         </is>
       </c>
       <c r="N55" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — no documents, filings, retrieval or text. The only relevance is structural: the abstention channel exists because my fundamental agent will have no disclosure to work from "more than half the time", and the paper supplies the vocabulary (time-varying subset selection) for that.</t>
+          <t>Not applicable - no documents, filings, retrieval or text. The only relevance is structural: the abstention channel exists because my fundamental agent will have no disclosure to work from "more than half the time", and the paper supplies the vocabulary (time-varying subset selection) for that.</t>
         </is>
       </c>
       <c r="O55" s="11" t="inlineStr">
         <is>
-          <t>No volatility modelling. One result touches the high-volatility regime: Zischke et al. (2022) report that when forecasting during high-volatility periods, weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample — which the note reads as "a result about choosing what to score rather than about how elaborate the pooling function is". This is the single exception in section 3 where sophistication earned its keep, and it is region-specific.
+          <t>No volatility modelling. One result touches the high-volatility regime: Zischke et al. (2022) report that when forecasting during high-volatility periods, weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample - which the note reads as "a result about choosing what to score rather than about how elaborate the pooling function is". This is the single exception in section 3 where sophistication earned its keep, and it is region-specific.
 Second-order relevance: the probabilistic variance decomposition means a deliberately heterogeneous pool produces an under-confident interval, which bears on any risk interval the orchestrator might emit.</t>
         </is>
       </c>
       <c r="P55" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages."</t>
+          <t>Not applicable - "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages."</t>
         </is>
       </c>
       <c r="Q55" s="11" t="inlineStr">
         <is>
-          <t>Interpreting combination weights is one of the paper's eight stated future directions — in the authors' words, "discussing if, how, and when it is helpful to interpret combination weights", prompted by the observation that some schemes drive poor forecasts to zero asymptotically while individually bad forecasts can still be useful. The paper also flags in future directions that "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts", which the note treats as a direct warning about significance testing on a weighted output.</t>
+          <t>Interpreting combination weights is one of the paper's eight stated future directions - in the authors' words, "discussing if, how, and when it is helpful to interpret combination weights", prompted by the observation that some schemes drive poor forecasts to zero asymptotically while individually bad forecasts can still be useful. The paper also flags in future directions that "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts", which the note treats as a direct warning about significance testing on a weighted output.</t>
         </is>
       </c>
       <c r="R55" s="11" t="inlineStr">
@@ -7570,11 +7570,11 @@
       </c>
       <c r="S55" s="11" t="inlineStr">
         <is>
-          <t>1. THE FORECAST COMBINATION PUZZLE — the field's central empirical result, fifty years old and still open. Stock and Watson (2004) named it: theoretically sophisticated weighting schemes should dominate the simple average, and empirically the simple average dominates them. Evidence runs from Makridakis et al. (1982) in the original M-competition through to M4, where "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) is the most recent restatement across M3, M4, M5 and FRED, finding that the winning combination method differs by data source while simple averaging shows, on average, more gain than complex methods. The explanations all centre on estimation error: Timmermann (2006) attributes it to parameter estimation error that simple schemes avoid entirely; Smith and Wallis (2009) to finite-sample estimation effects; Claeskens et al. (2016) prove that treating the weights as random rather than fixed can introduce bias into combinations of unbiased components and inflate the combination's variance past the fixed-weight case; Blanc and Setzer (2020) frame it as a bias-variance tradeoff where equal weights underfit and estimated weights carry estimation variance; Elliott (2011) bounds the available gain from optimal over equal weights and finds it is usually too small to pay for the estimation.
-2. CORRELATIONS AMONG FORECAST ERRORS SHOULD BE IGNORED RATHER THAN ESTIMATED — an empirical finding, not a convenience. Bates and Granger argued correlations are poorly estimated in practice and should be left out; Newbold and Granger (1974) and Winkler and Makridakis (1983) tested that over more series, methods and horizons and concluded that "combinations ignoring correlations are more successful than those attempting to account for them". The mechanism is visible in the optimal-weight formula: the full covariance matrix needs N(N+1)/2 parameters from the same short error history that a diagonal treatment needs N from, and with highly correlated forecast errors the sample estimator of Σ is unstable. Chan et al. (1999) add that OLS combination performs very poorly when N is large, which pushes the literature toward principal components regression and clustering.
-3. ACCURACY AND DIVERSITY BOTH CONSTRAIN WHAT COMBINING CAN DELIVER, AND A SUBSET USUALLY BEATS BOTH THE FULL POOL AND THE SINGLE BEST. Mannes et al. (2014) establish that the mean level of expertise in the pool sets a floor on combination performance, so including poor forecasts degrades the result; Lichtendahl and Winkler (2020) add that the variance of accuracy across series matters as much as the mean and the two have to be traded off when choosing the pool. On the other side, diversity produces the error cancellation in the first place, with Atiya (2020) deriving it through the bias-variance decomposition of MSE, and diversity usually measured as low correlation among forecast errors. The slogan the paper quotes is "many could be better than all": there are decreasing returns to adding forecasts, and subset selection — by discarding the worst performers, by Kourentzes et al.'s (2019) boxplot-outlier heuristic, by Lichtendahl and Winkler's two screens (removing models worse than Naïve2, excluding pairs with highly correlated errors), or by Diebold and Shin's (2019) two-step LASSO that zeroes some weights then shrinks the survivors toward equality — beats both using everything and selecting one.
+          <t>1. THE FORECAST COMBINATION PUZZLE - the field's central empirical result, fifty years old and still open. Stock and Watson (2004) named it: theoretically sophisticated weighting schemes should dominate the simple average, and empirically the simple average dominates them. Evidence runs from Makridakis et al. (1982) in the original M-competition through to M4, where "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) is the most recent restatement across M3, M4, M5 and FRED, finding that the winning combination method differs by data source while simple averaging shows, on average, more gain than complex methods. The explanations all centre on estimation error: Timmermann (2006) attributes it to parameter estimation error that simple schemes avoid entirely; Smith and Wallis (2009) to finite-sample estimation effects; Claeskens et al. (2016) prove that treating the weights as random rather than fixed can introduce bias into combinations of unbiased components and inflate the combination's variance past the fixed-weight case; Blanc and Setzer (2020) frame it as a bias-variance tradeoff where equal weights underfit and estimated weights carry estimation variance; Elliott (2011) bounds the available gain from optimal over equal weights and finds it is usually too small to pay for the estimation.
+2. CORRELATIONS AMONG FORECAST ERRORS SHOULD BE IGNORED RATHER THAN ESTIMATED - an empirical finding, not a convenience. Bates and Granger argued correlations are poorly estimated in practice and should be left out; Newbold and Granger (1974) and Winkler and Makridakis (1983) tested that over more series, methods and horizons and concluded that "combinations ignoring correlations are more successful than those attempting to account for them". The mechanism is visible in the optimal-weight formula: the full covariance matrix needs N(N+1)/2 parameters from the same short error history that a diagonal treatment needs N from, and with highly correlated forecast errors the sample estimator of Σ is unstable. Chan et al. (1999) add that OLS combination performs very poorly when N is large, which pushes the literature toward principal components regression and clustering.
+3. ACCURACY AND DIVERSITY BOTH CONSTRAIN WHAT COMBINING CAN DELIVER, AND A SUBSET USUALLY BEATS BOTH THE FULL POOL AND THE SINGLE BEST. Mannes et al. (2014) establish that the mean level of expertise in the pool sets a floor on combination performance, so including poor forecasts degrades the result; Lichtendahl and Winkler (2020) add that the variance of accuracy across series matters as much as the mean and the two have to be traded off when choosing the pool. On the other side, diversity produces the error cancellation in the first place, with Atiya (2020) deriving it through the bias-variance decomposition of MSE, and diversity usually measured as low correlation among forecast errors. The slogan the paper quotes is "many could be better than all": there are decreasing returns to adding forecasts, and subset selection - by discarding the worst performers, by Kourentzes et al.'s (2019) boxplot-outlier heuristic, by Lichtendahl and Winkler's two screens (removing models worse than Naïve2, excluding pairs with highly correlated errors), or by Diebold and Shin's (2019) two-step LASSO that zeroes some weights then shrinks the survivors toward equality - beats both using everything and selecting one.
 4. FEATURE-BASED CROSS-LEARNING IS WHERE THE FIELD'S MOMENTUM IS. The meta-model learns a mapping from features of a series to weights over a fixed method pool, trained across many series rather than within one, sidestepping the short-history problem that makes per-series weight estimation noisy. FFORMA placed second in M4 with 42 features and an XGBoost meta-learner; Montero-Manso et al.'s interval variant placed second for the uncertainty track over 100,000 series by predicting the interval radius as a linear combination of individual radii minimising the MSIS; the top three M4 methods all drew on cross-dataset information.
-5. DIVERSITY REVERSES SIGN WHEN THE OUTPUT IS A DISTRIBUTION. From the linear pool's variance decomposition: "seeking diverse forecasts, which is the standard advice for point combination, harms the probabilistic forecast by destroying sharpness and making the mixture under-confident", and Ranjan and Gneiting (2010) show the pool of individually calibrated forecasts is generally not calibrated. Hora (2004) gives the countervailing case that pooling helps calibration when components are overconfident; Jose et al. (2014) narrow it, that overconfident components with low diversity stay overconfident. The response is the trimmed opinion pool — exterior trimming removes components with extreme means to cut variance and address under-confidence, interior trimming removes the moderate ones to raise variance and address overconfidence.
+5. DIVERSITY REVERSES SIGN WHEN THE OUTPUT IS A DISTRIBUTION. From the linear pool's variance decomposition: "seeking diverse forecasts, which is the standard advice for point combination, harms the probabilistic forecast by destroying sharpness and making the mixture under-confident", and Ranjan and Gneiting (2010) show the pool of individually calibrated forecasts is generally not calibrated. Hora (2004) gives the countervailing case that pooling helps calibration when components are overconfident; Jose et al. (2014) narrow it, that overconfident components with low diversity stay overconfident. The response is the trimmed opinion pool - exterior trimming removes components with extreme means to cut variance and address under-confidence, interior trimming removes the moderate ones to raise variance and address overconfidence.
 6. NONLINEAR POOLING DOES NOT PAY FOR ITS COMPLEXITY. Baran and Lerch (2018) compared state-of-the-art combination methods in case studies and found "no substantial difference in forecast performance between the simple linear pool and the theoretically superior but cumbersome nonlinear pooling approaches". The note: "That is the probabilistic restatement of the puzzle, which makes it two independent appearances of the same pattern in one paper." The one exception is Zischke et al. (2022) on high-volatility periods, which is about what to score rather than how elaborate the pooling function is.
 7. NONLINEAR COMBINATION OF POINT FORECASTS IS A THIN LITERATURE AND THE AUTHORS SAY SO PLAINLY. Two forms: a neural network over the individual forecasts (Donaldson and Kamstra, 1996), with purely linear and purely nonlinear specifications as special cases; and an additive pairwise term Σ_{i&lt;j} π_{ij} v_{ij} where v_{ij} is a nonlinear function of forecasts i and j. Reported results generally dominate simple averaging, OLS weights and performance-based weights, but the authors' own assessment of that evidence is that it rests on "fewer than ten time series, possibly hand-picked", alongside neglect of error correlations, unstable parameter estimation and multicollinearity from overlapping information sets.</t>
         </is>
@@ -7582,8 +7582,8 @@
       <c r="T55" s="11" t="inlineStr">
         <is>
           <t>1. Narrative review with no protocol, no screening counts and no meta-analysis, "so it establishes what exists and not what works." The Web of Science query is given in full but only for the Figure 1 publication-share chart, not for the review's own selection. Nothing states how papers were found, how many were screened, or what put one in or out. The authors run no experiment and aggregate no results, so there is no table anywhere comparing two weighting schemes on shared data. "I can cite this for the existence and the lineage of a method but never for its relative performance. This is the same structural weakness I recorded against [[The Evolution of Reinforcement Learning in Quantitative Finance, A Survey]], and the two surveys share it for the same reason, that coverage and adjudication are different jobs."
-2. The puzzle is reported rather than resolved, and where the paper gestures at a contradiction there is not actually one. Claeskens et al. (2016) derive that random combination weights can introduce bias and inflate the variance of the combined forecast relative to fixed weights; Zischke et al. (2022) are quoted as finding the opposite, that weight estimation imparts no bias or variability at all, and the authors record the opposition in a single clause and move on. The note's own reading: the opposition is a compression rather than a real disagreement — "Claeskens is a finite-sample result about the MSE of the combined point forecast under unbiased components, Zischke is a first-order asymptotic result about the sampling variability of the out-of-sample expected score", so the two answer different questions about different objects and neither refutes the other. "The genuine limitation is that the review leaves the question my contribution turns on, whether estimated weights can be expected to beat fixed ones, standing open, while the work that takes it considerably further was already in circulation when the review went to press."
-3. The non-interfering assumption excludes the systems I am actually positioned against (see AGENTS &amp; ORCHESTRATION above). The clean statistical properties — unbiasedness of the combination, the variance bound — hold under an assumption my pool does not satisfy.
+2. The puzzle is reported rather than resolved, and where the paper gestures at a contradiction there is not actually one. Claeskens et al. (2016) derive that random combination weights can introduce bias and inflate the variance of the combined forecast relative to fixed weights; Zischke et al. (2022) are quoted as finding the opposite, that weight estimation imparts no bias or variability at all, and the authors record the opposition in a single clause and move on. The note's own reading: the opposition is a compression rather than a real disagreement - "Claeskens is a finite-sample result about the MSE of the combined point forecast under unbiased components, Zischke is a first-order asymptotic result about the sampling variability of the out-of-sample expected score", so the two answer different questions about different objects and neither refutes the other. "The genuine limitation is that the review leaves the question my contribution turns on, whether estimated weights can be expected to beat fixed ones, standing open, while the work that takes it considerably further was already in circulation when the review went to press."
+3. The non-interfering assumption excludes the systems I am actually positioned against (see AGENTS &amp; ORCHESTRATION above). The clean statistical properties - unbiasedness of the combination, the variance bound - hold under an assumption my pool does not satisfy.
 4. The target is always a realised value of one series under a symmetric loss, "so none of the optimality results transfer to a decision." The combined forecast is scored against y_{T+h} under MSE or a proper scoring rule; there is no portfolio, position, transaction cost, slippage or execution anywhere in forty pages. Elliott and Timmermann (2004) and Patton and Timmermann (2007) are cited as the asymmetric-loss extension, finding that optimal weights depend strongly on the degree of asymmetry in the loss and the skewness of the error distribution, "which is as far as this literature goes toward my setting. My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality."
 5. Cross-learning, the strand closest to what I'm building, is demonstrated at a scale I cannot reach. Results come from M4 at 100,000 series, M3, M5 and FRED, and the stated first limitation of the approach is the requirement for a large and diverse time series dataset to produce meaningful training. The workarounds offered are simulating series from assumed data generating processes or generating them with controllable characteristics using gratis, "both of which hand the researcher the features they then learn from. My per-counter archive is roughly 300 counters over 374 trading days, three orders of magnitude short of M4, and no result in this paper speaks to what a feature-to-weight meta-model does at that scale."
 6. Emerging and thin markets are absent from the entire paper. Applications named are retail, energy, economics, epidemiology and meteorology; the financial examples are macroeconomic series such as inflation and GDP growth. "Nothing addresses a market where the components themselves are estimated on short, illiquid, intermittently traded series, which is the condition under which every estimation-error argument in the puzzle section becomes more severe rather than less. The direction of that bias is at least clear, which is the useful part: everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
@@ -7592,12 +7592,12 @@
       </c>
       <c r="U55" s="11" t="inlineStr">
         <is>
-          <t>- A lineage and a precise statement of what is new, which the note judges "a stronger framing than novelty". My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) is a time-varying feature-conditioned linear combination, and the paper contains both halves separately: time-varying weights through the Kalman-filter and smooth-transition line, feature-conditioned weights through FFORMA. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That reads as a generalisation along an identified axis rather than new machinery. It also tells me what the honest comparison is: FFORMA's structure — a gradient-boosted meta-model mapping features to a weight simplex — is available to me as an implementation choice, "and if I use something simpler I should say why rather than let it look like I did not know."
+          <t>- A lineage and a precise statement of what is new, which the note judges "a stronger framing than novelty". My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) is a time-varying feature-conditioned linear combination, and the paper contains both halves separately: time-varying weights through the Kalman-filter and smooth-transition line, feature-conditioned weights through FFORMA. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That reads as a generalisation along an identified axis rather than new machinery. It also tells me what the honest comparison is: FFORMA's structure - a gradient-boosted meta-model mapping features to a weight simplex - is available to me as an implementation choice, "and if I use something simpler I should say why rather than let it look like I did not know."
 - The hardest possible equal-weight baseline, plus a falsification condition to pre-register.
 - A five-decade justification for having no pairwise interaction term in the weighting function. "With four agents that is ten parameters against four, from 374 days, so the argument has real force here. This is worth stating explicitly in the write-up, because a reviewer will ask why there is no interaction term, and the answer is that the literature tried that first and moved away from it."
-- Two cheap intermediate baselines: the Stock and Watson inverse-kth-power family (a one-parameter dial from k=0 equal weights to winner-take-all, "a sweep over k maps the whole continuum... for almost no implementation cost"), and the discounted inverse-MSE scheme, "which adds a time dimension without adding state" — the one the note names as "the baseline that actually threatens my contribution". So the planned three-way comparison (equal weights vs static learned weights vs state-conditioned weights) becomes four-way with a discounted performance-weighting arm.
+- Two cheap intermediate baselines: the Stock and Watson inverse-kth-power family (a one-parameter dial from k=0 equal weights to winner-take-all, "a sweep over k maps the whole continuum... for almost no implementation cost"), and the discounted inverse-MSE scheme, "which adds a time dimension without adding state" - the one the note names as "the baseline that actually threatens my contribution". So the planned three-way comparison (equal weights vs static learned weights vs state-conditioned weights) becomes four-way with a discounted performance-weighting arm.
 - An oracle-weight arm, weights fitted on the test window itself rather than on training, "because the gap between oracle and estimated performance is the estimation cost measured in my own data and in my own units: no gain under oracle weights means the conditioning hypothesis is simply wrong, a gain under oracle but not under estimated weights means it is an estimation problem I can put a number on, and it costs one further pass of the same pipeline."
-- Vocabulary for the abstention channel: time-varying subset selection via a pre-set threshold on a time-varying weighting scheme (Li et al., 2022). Plus Geweke and Amisano's observation that individually poor forecasts may still help in combination and one does not want to zero-weight them — "an argument for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero, which is a concrete design decision I had not settled."
+- Vocabulary for the abstention channel: time-varying subset selection via a pre-set threshold on a time-varying weighting scheme (Li et al., 2022). Plus Geweke and Amisano's observation that individually poor forecasts may still help in combination and one does not want to zero-weight them - "an argument for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero, which is a concrete design decision I had not settled."
 - An operational definition of diversity (low correlation among forecast errors, with Lemke and Gabrys' six diversity features and Thomson et al.'s coherence measure as alternatives), making my heterogeneity claim testable on my own pool.
 - Quantile averaging as the escape route if the orchestrator ever emits an interval, pairing with adaptive conformal inference.
 - A warning on inference: "standard errors for a combined forecast are nontrivial to obtain because the weights are random and correlated with the forecasts."</t>
@@ -7606,31 +7606,31 @@
       <c r="V55" s="11" t="inlineStr">
         <is>
           <t>The review contains weights that change over time and weights that change as a regression function of covariates, "and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state." The two nearest things are Deutsch et al.'s smooth transition specification, where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step. That is the axis along which my weighting function generalises existing work.
-Second, the review leaves standing open the question my contribution turns on — whether estimated weights can be expected to beat fixed ones — and its own two guidelines on the matter cut in opposite directions, with the paper clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature.
+Second, the review leaves standing open the question my contribution turns on - whether estimated weights can be expected to beat fixed ones - and its own two guidelines on the matter cut in opposite directions, with the paper clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature.
 Third, nothing in the paper speaks to a feature-to-weight meta-model at my data scale, nor to any market where the components themselves are estimated on short, illiquid, intermittently traded series.
 Fourth, the paper names interpretation of combination weights as an open research question; my orchestrator produces a weight per agent per step as a readable function of named market-state inputs, which is a direct response to that question rather than a byproduct.
-Fifth, subset selection has, in the paper's own assessment, "received scant attention, is mainly trimming on expertise alone", and "most existing algorithms are ad hoc and lack statistical rationale" — so a principled selection rule driven by a structural property of the output is defensible ground.</t>
+Fifth, subset selection has, in the paper's own assessment, "received scant attention, is mainly trimming on expertise alone", and "most existing algorithms are ad hoc and lack statistical rationale" - so a principled selection rule driven by a structural property of the output is defensible ground.</t>
         </is>
       </c>
       <c r="W55" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: The orchestrator above everything else — this is the prior art for the weighting function itself, and the note is blunt that it is being written up precisely because "it is the most direct body of prior art on the half of my design I have covered least". Also the abstention channel (named here as time-varying subset selection), the confidence term C_{i,t} (via quantile averaging and calibrated intervals), the agent pool design (diversity as a measurable quantity rather than an asserted one), the explainability claim, and — most consequentially — the entire evaluation design.
+          <t>SPEAKS TO: The orchestrator above everything else - this is the prior art for the weighting function itself, and the note is blunt that it is being written up precisely because "it is the most direct body of prior art on the half of my design I have covered least". Also the abstention channel (named here as time-varying subset selection), the confidence term C_{i,t} (via quantile averaging and calibrated intervals), the agent pool design (diversity as a measurable quantity rather than an asserted one), the explainability claim, and - most consequentially - the entire evaluation design.
 EFFECT ON MAIN GAP: THIS IS THE PAPER THAT BOTH LEGITIMISES AND THREATENS THE MAIN GAP, AND BOTH HALVES HAVE TO BE CARRIED THROUGH HONESTLY.
-The legitimising half. My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) stops being an invention and becomes a named construct with a lineage: a time-varying, feature-conditioned linear combination. The review contains time-varying weights (Diebold and Pauly, Deutsch et al., Terui and van Dijk's Kalman-filter random walk, Raftery et al.'s forgetting factors) and it contains feature-conditioned weights (FFORMA). What it does not contain, anywhere, is weights that are a function of measured exogenous market state. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That is a generalisation along an identified axis, which is a stronger and more defensible framing than novelty — and it is the framing the orchestration note already used. It also obliges me to be honest about implementation: FFORMA's gradient-boosted-meta-model-to-weight-simplex structure is available to me, and if I use something simpler I should say why.
+The legitimising half. My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) stops being an invention and becomes a named construct with a lineage: a time-varying, feature-conditioned linear combination. The review contains time-varying weights (Diebold and Pauly, Deutsch et al., Terui and van Dijk's Kalman-filter random walk, Raftery et al.'s forgetting factors) and it contains feature-conditioned weights (FFORMA). What it does not contain, anywhere, is weights that are a function of measured exogenous market state. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That is a generalisation along an identified axis, which is a stronger and more defensible framing than novelty - and it is the framing the orchestration note already used. It also obliges me to be honest about implementation: FFORMA's gradient-boosted-meta-model-to-weight-simplex structure is available to me, and if I use something simpler I should say why.
 The threatening half, and it is serious. The forecast combination puzzle says that fifty years of evidence finds the equally weighted average extremely hard to beat, and that sophisticated weighting schemes lose because of estimation error. In M4, "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) across M3, M4, M5 and FRED find simple averaging shows, on average, more gain than complex methods. Elliott (2011) bounds the available gain from optimal over equal weights and finds it usually too small to pay for the estimation. Claeskens et al. (2016) prove random weights can introduce bias into combinations of unbiased components and inflate variance past the fixed-weight case. And the probabilistic side produces the same pattern independently: Baran and Lerch (2018) found no substantial difference between the simple linear pool and the theoretically superior nonlinear alternatives. "That is the probabilistic restatement of the puzzle, which makes it two independent appearances of the same pattern in one paper."
-Worse for me specifically: everything the paper says about estimation error swamping the gains from optimal weights "gets worse in my setting, not better", because my components are themselves estimated on short, illiquid, intermittently traded series. And the two practical guidelines the paper derives cut in opposite directions for me — "guideline one says that with limited historical data the simple average or weights ignoring covariances are recommended, which my 374 trading days per counter argues for, while guideline two says structural change impacts sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state."
-The honest consequence the note draws: the equal-weight baseline becomes the field's hardest benchmark, and "if my state-conditioned weighting fails to beat equal weights on the CSE, that is the expected outcome under the field's prior and not a surprise". The response is not to defend the gap but to pre-register — write down before the run what margin and what test would count as beating equal weights. And the note extracts a genuine contribution even from failure: "Which effect dominates on this data is the question, and the paper is clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature, so an answer in a thin frontier market is a contribution even if the answer is that equal weights win."
-How my setting differs — three ways the note identifies. (i) My weights condition on exogenous measured market state, not on properties of the series computed once; this is the axis the literature has not covered. (ii) My loss is not quadratic forecast MSE against a realised value — "My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality." The asymmetric-loss line (Elliott and Timmermann 2004, Patton and Timmermann 2007) is as close as this literature gets, and it finds optimal weights depend strongly on loss asymmetry and error skewness. (iii) My pool violates the review's non-interfering assumption: the four agents read overlapping data by construction, so the unbiasedness and variance-bound results do not hold for me, and the paper's own observation that overlapping information sets produce highly correlated errors is the mechanism by which that bites.
+Worse for me specifically: everything the paper says about estimation error swamping the gains from optimal weights "gets worse in my setting, not better", because my components are themselves estimated on short, illiquid, intermittently traded series. And the two practical guidelines the paper derives cut in opposite directions for me - "guideline one says that with limited historical data the simple average or weights ignoring covariances are recommended, which my 374 trading days per counter argues for, while guideline two says structural change impacts sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state."
+The honest consequence the note draws: the equal-weight baseline becomes the field's hardest benchmark, and "if my state-conditioned weighting fails to beat equal weights on the CSE, that is the expected outcome under the field's prior and not a surprise". The response is not to defend the gap but to pre-register - write down before the run what margin and what test would count as beating equal weights. And the note extracts a genuine contribution even from failure: "Which effect dominates on this data is the question, and the paper is clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature, so an answer in a thin frontier market is a contribution even if the answer is that equal weights win."
+How my setting differs - three ways the note identifies. (i) My weights condition on exogenous measured market state, not on properties of the series computed once; this is the axis the literature has not covered. (ii) My loss is not quadratic forecast MSE against a realised value - "My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality." The asymmetric-loss line (Elliott and Timmermann 2004, Patton and Timmermann 2007) is as close as this literature gets, and it finds optimal weights depend strongly on loss asymmetry and error skewness. (iii) My pool violates the review's non-interfering assumption: the four agents read overlapping data by construction, so the unbiasedness and variance-bound results do not hold for me, and the paper's own observation that overlapping information sets produce highly correlated errors is the mechanism by which that bites.
 A second threat, from the WARNING box rather than the paper itself. Frazier, Covey, Martin and Poskitt (Monash EBS WP 18/2023, arXiv:2308.05263) argue the puzzle is substantially an artefact of two-step estimation: estimated weights impart no first-order sampling variability into the usual predictive-accuracy statistic, so it converges to a generalised chi-squared rather than a normal, and their Theorem 1 says that when two weight vectors lie within O(T^{−1/4−ε}) of each other "the test has no power to distinguish them at all". Two consequences land directly on my design. "The O(T^{−1/4}) rate is not small at my sample sizes, roughly 0.23 at 374 trading days against roughly 0.14 on the ten-year index track, and with four agents sitting at 0.25 each under equal weights, a short sample puts almost any non-degenerate weighting scheme inside the dead zone. The constant is unknown so neither figure is a threshold, but the direction is unambiguous and it argues for running the weighting comparison on the index series rather than the per-counter panel." And their remedy, one-step joint estimation, is "mostly unavailable to me, since a retrieval agent is not jointly optimisable with a volatility model, so the partial version is to fit the parametric agents against the combined objective rather than against their own local losses." Caveat carried: this is a working paper and its publication status needs checking before it is cited as anything else.
-Design decisions this forces on the main gap: (a) no pairwise interaction term in the weighting function, backed by Bates and Granger, Newbold and Granger, and Winkler and Makridakis — ten covariance parameters against four diagonal ones, from 374 days; (b) a four-way rather than three-way comparison, adding a discounted inverse-MSE arm, because "if weights that merely react to recent agent performance do as well as weights conditioned on measured market state, then the state conditioning is not earning its place and I need to know that early"; (c) an oracle-weight arm to separate "the conditioning hypothesis is wrong" from "the estimation is too noisy"; (d) a Stock–Watson k-sweep to map the whole continuum from equal weights to winner-take-all cheaply; (e) pre-registration that separates two failure modes which look identical in the output — "the weighting genuinely not helping, which is the field's prior from the puzzle, against the weighting helping and the two-step test being unable to see it, because the first says abandon the conditioning and the second says change how it is estimated or tested."
-EFFECT ON THE ABSTENTION CHANNEL: Upgraded from a bespoke mechanism to named prior art. The paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme (Li et al., 2022). "That is structurally what the abstention channel does when the fundamental agent has no disclosure to work from, which is expected more than half the time, so I should present it in that vocabulary rather than as a bespoke mechanism." Two consequences: the paper's own assessment is that subset selection "has received scant attention, is mainly trimming on expertise alone, and that most existing algorithms are ad hoc and lack statistical rationale", so a principled selection rule driven by a structural property of the output is defensible ground; and Geweke and Amisano's observation that individually poor forecasts may still help in combination argues for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero — "a concrete design decision I had not settled."
-EFFECT ON THE CONFIDENCE TERM C_{i,t}: A route to making C_{i,t} a measured structural property rather than a self-report. If the orchestrator ever emits an interval rather than a point allocation, the linear pool's variance decomposition says component disagreement adds directly to pooled variance, "so a deliberately heterogeneous pool produces an under-confident interval, and that is the one place where my central design choice actively works against me." Quantile averaging avoids it — it averages cdfs horizontally, preserves the family for location-scale components, and is sharper for the same mean. "This connects to [[Adaptive Conformal Inference Under Distribution Shift]] more tightly than I expected, since adaptive conformal inference is a per-agent calibration wrapper and quantile averaging is the aggregation step, and the pair would give me a calibrated interval from a heterogeneous pool without the under-confidence that linear pooling would introduce. That is a route to the confidence term being a measured interval width rather than a self-report, which is what the scope revision asked for."
-EFFECT ON THE HETEROGENEITY CLAIM: The paper makes it testable and therefore falsifiable. "I describe the four agents as methodologically heterogeneous and that heterogeneity is load-bearing in the gap statement, but the paper's operational definition of diversity is low correlation among forecast errors... So the claim is testable on my own pool and I should run it: if the technical agent and the volatility agent produce errors that correlate at 0.8 on CSE data, the pool is substantially less diverse than the architecture diagram implies and the error-cancellation argument weakens accordingly. This is close to free, it uses data I will already have from the individual agent runs, and it is the kind of result that is much better found by me than by an examiner." Also relevant: Mannes et al. (2014) show the mean level of expertise in the pool sets a floor, so including a poor agent degrades the result — which bears on whether all four agents should always be in the pool.
-EFFECT ON EXPLAINABILITY: Upgraded from a feature to a positioned contribution. Interpreting combination weights is one of the paper's eight future directions — "discussing if, how, and when it is helpful to interpret combination weights". "My orchestrator produces a weight per agent per step as a readable function of named market-state inputs, so the trace of which agent was trusted when, and on what measured conditions, is a direct response to that question rather than a byproduct." Caveat carried from the layered-explainability reading: "a weight being readable is not the same as it being correct, so the claim is that the system exposes the quantity this literature identifies as unexamined, not that exposing it is sufficient."
-EFFECT ON SUB-GAP 1: Negative in the sense that it offers nothing — "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages" — but that absence is itself the boundary line. Everything in this paper is a weighting mechanism scored against a realised value under quadratic loss; none of its optimality results transfer to an after-cost decision objective. So the claim that execution cost belongs inside the decision objective is untouched by fifty years of combination theory, which is a clean separation to state.
-EFFECT ON SUB-GAP 2: Essentially none directly. The only contact point is Zischke et al. (2022), who find that in high-volatility periods weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample — "a result about choosing what to score rather than about how elaborate the pooling function is". That is about volatility level, not persistence, and the review contains nothing on persistence or on decay schedules. The structural-change guideline ("structural change impacts sophisticated schemes more than the simple average and changing weights are a legitimate response to it") is the nearest thing to support for conditioning on a regime, but it is a general statement with no persistence mechanism behind it.
-CSE DATA EVIDENCE: The note states my per-counter archive as roughly 300 counters over 374 trading days, "three orders of magnitude short of M4", with "no result in this paper" speaking to a feature-to-weight meta-model at that scale. The ten-year index track is the alternative. Those two sample sizes drive the O(T^{−1/4}) calculation — roughly 0.23 at 374 trading days against roughly 0.14 on the index track, against four agents at 0.25 each under equal weights — which argues for running the weighting comparison on the index series rather than the per-counter panel. The same 374 days drive the parameter-count argument against a pairwise interaction term (ten covariance parameters against four). And the note's reading of the thin-market absence is directional rather than agnostic: "everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
-PROPOSED REVISION STATED IN THE NOTE: Reframe the weighting function as a generalisation of FFORMA along one identified axis — exogenous measured market state at each step versus series properties computed once — rather than as new machinery. Pre-register the margin and the test that would count as beating equal weights, before the run. Expand the planned three-way comparison (equal / static learned / state-conditioned) to four-way by adding a discounted inverse-MSE arm, and add an oracle-weight arm fitted on the test window to separate "conditioning is wrong" from "estimation is too noisy". Add a Stock–Watson k-sweep. Run the weighting comparison on the index series rather than the per-counter panel, on the power argument. Fit the parametric agents against the combined objective rather than their own local losses, as the partial version of one-step joint estimation. Present the abstention channel as time-varying subset selection with a threshold, and shrink the abstaining agent's weight toward a floor rather than to exactly zero. Measure pool diversity as error correlation before claiming heterogeneity. Keep a separate note for the Frazier et al. working paper and check its publication status before citing it as anything other than a working paper. State explicitly in the write-up why there is no pairwise interaction term. And carry the warning that standard errors on a combined forecast are nontrivial because the weights are random and correlated with the forecasts — which matches the pattern where "the economic result and the formal test diverged" in the DRL global-equity portfolio note.</t>
+Design decisions this forces on the main gap: (a) no pairwise interaction term in the weighting function, backed by Bates and Granger, Newbold and Granger, and Winkler and Makridakis - ten covariance parameters against four diagonal ones, from 374 days; (b) a four-way rather than three-way comparison, adding a discounted inverse-MSE arm, because "if weights that merely react to recent agent performance do as well as weights conditioned on measured market state, then the state conditioning is not earning its place and I need to know that early"; (c) an oracle-weight arm to separate "the conditioning hypothesis is wrong" from "the estimation is too noisy"; (d) a Stock-Watson k-sweep to map the whole continuum from equal weights to winner-take-all cheaply; (e) pre-registration that separates two failure modes which look identical in the output - "the weighting genuinely not helping, which is the field's prior from the puzzle, against the weighting helping and the two-step test being unable to see it, because the first says abandon the conditioning and the second says change how it is estimated or tested."
+EFFECT ON THE ABSTENTION CHANNEL: Upgraded from a bespoke mechanism to named prior art. The paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme (Li et al., 2022). "That is structurally what the abstention channel does when the fundamental agent has no disclosure to work from, which is expected more than half the time, so I should present it in that vocabulary rather than as a bespoke mechanism." Two consequences: the paper's own assessment is that subset selection "has received scant attention, is mainly trimming on expertise alone, and that most existing algorithms are ad hoc and lack statistical rationale", so a principled selection rule driven by a structural property of the output is defensible ground; and Geweke and Amisano's observation that individually poor forecasts may still help in combination argues for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero - "a concrete design decision I had not settled."
+EFFECT ON THE CONFIDENCE TERM C_{i,t}: A route to making C_{i,t} a measured structural property rather than a self-report. If the orchestrator ever emits an interval rather than a point allocation, the linear pool's variance decomposition says component disagreement adds directly to pooled variance, "so a deliberately heterogeneous pool produces an under-confident interval, and that is the one place where my central design choice actively works against me." Quantile averaging avoids it - it averages cdfs horizontally, preserves the family for location-scale components, and is sharper for the same mean. "This connects to [[Adaptive Conformal Inference Under Distribution Shift]] more tightly than I expected, since adaptive conformal inference is a per-agent calibration wrapper and quantile averaging is the aggregation step, and the pair would give me a calibrated interval from a heterogeneous pool without the under-confidence that linear pooling would introduce. That is a route to the confidence term being a measured interval width rather than a self-report, which is what the scope revision asked for."
+EFFECT ON THE HETEROGENEITY CLAIM: The paper makes it testable and therefore falsifiable. "I describe the four agents as methodologically heterogeneous and that heterogeneity is load-bearing in the gap statement, but the paper's operational definition of diversity is low correlation among forecast errors... So the claim is testable on my own pool and I should run it: if the technical agent and the volatility agent produce errors that correlate at 0.8 on CSE data, the pool is substantially less diverse than the architecture diagram implies and the error-cancellation argument weakens accordingly. This is close to free, it uses data I will already have from the individual agent runs, and it is the kind of result that is much better found by me than by an examiner." Also relevant: Mannes et al. (2014) show the mean level of expertise in the pool sets a floor, so including a poor agent degrades the result - which bears on whether all four agents should always be in the pool.
+EFFECT ON EXPLAINABILITY: Upgraded from a feature to a positioned contribution. Interpreting combination weights is one of the paper's eight future directions - "discussing if, how, and when it is helpful to interpret combination weights". "My orchestrator produces a weight per agent per step as a readable function of named market-state inputs, so the trace of which agent was trusted when, and on what measured conditions, is a direct response to that question rather than a byproduct." Caveat carried from the layered-explainability reading: "a weight being readable is not the same as it being correct, so the claim is that the system exposes the quantity this literature identifies as unexamined, not that exposing it is sufficient."
+EFFECT ON SUB-GAP 1: Negative in the sense that it offers nothing - "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages" - but that absence is itself the boundary line. Everything in this paper is a weighting mechanism scored against a realised value under quadratic loss; none of its optimality results transfer to an after-cost decision objective. So the claim that execution cost belongs inside the decision objective is untouched by fifty years of combination theory, which is a clean separation to state.
+EFFECT ON SUB-GAP 2: Essentially none directly. The only contact point is Zischke et al. (2022), who find that in high-volatility periods weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample - "a result about choosing what to score rather than about how elaborate the pooling function is". That is about volatility level, not persistence, and the review contains nothing on persistence or on decay schedules. The structural-change guideline ("structural change impacts sophisticated schemes more than the simple average and changing weights are a legitimate response to it") is the nearest thing to support for conditioning on a regime, but it is a general statement with no persistence mechanism behind it.
+CSE DATA EVIDENCE: The note states my per-counter archive as roughly 300 counters over 374 trading days, "three orders of magnitude short of M4", with "no result in this paper" speaking to a feature-to-weight meta-model at that scale. The ten-year index track is the alternative. Those two sample sizes drive the O(T^{−1/4}) calculation - roughly 0.23 at 374 trading days against roughly 0.14 on the index track, against four agents at 0.25 each under equal weights - which argues for running the weighting comparison on the index series rather than the per-counter panel. The same 374 days drive the parameter-count argument against a pairwise interaction term (ten covariance parameters against four). And the note's reading of the thin-market absence is directional rather than agnostic: "everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
+PROPOSED REVISION STATED IN THE NOTE: Reframe the weighting function as a generalisation of FFORMA along one identified axis - exogenous measured market state at each step versus series properties computed once - rather than as new machinery. Pre-register the margin and the test that would count as beating equal weights, before the run. Expand the planned three-way comparison (equal / static learned / state-conditioned) to four-way by adding a discounted inverse-MSE arm, and add an oracle-weight arm fitted on the test window to separate "conditioning is wrong" from "estimation is too noisy". Add a Stock-Watson k-sweep. Run the weighting comparison on the index series rather than the per-counter panel, on the power argument. Fit the parametric agents against the combined objective rather than their own local losses, as the partial version of one-step joint estimation. Present the abstention channel as time-varying subset selection with a threshold, and shrink the abstaining agent's weight toward a floor rather than to exactly zero. Measure pool diversity as error correlation before claiming heterogeneity. Keep a separate note for the Frazier et al. working paper and check its publication status before citing it as anything other than a working paper. State explicitly in the write-up why there is no pairwise interaction term. And carry the warning that standard errors on a combined forecast are nontrivial because the weights are random and correlated with the forecasts - which matches the pattern where "the economic result and the formal test diverged" in the DRL global-equity portfolio note.</t>
         </is>
       </c>
       <c r="X55" s="11" t="inlineStr">
@@ -7652,17 +7652,17 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>2021 (frontmatter year, and the note's body dates it to NeurIPS 2021).</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>arXiv in the frontmatter; the note's body states "NeurIPS 2021". Both are recorded in the note, so I record both.</t>
+          <t>arXiv in the frontmatter; the note's body states "NeurIPS 2021". Both are recorded in the note, so I record both. The note's frontmatter carries 2021 and the body dates it to NeurIPS 2021.</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>https://doi.org/10.48550/ARXIV.2106.00170 — code at github.com/isgibbs/AdaptiveConformal.</t>
+          <t>https://doi.org/10.48550/ARXIV.2106.00170 - code at github.com/isgibbs/AdaptiveConformal.</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
@@ -7690,7 +7690,7 @@
 - Refit window: trailing 1,250 trading days, roughly 5 years, refit at every t &gt; 1250. Calibration uses the same 1,250-day trailing window of conformity scores.
 - Coverage metric: localCov, the average coverage over the most recent 500 days, roughly two years.
 - Period: not given as explicit start/end dates in the note, but the trajectories span at least 2004 through 2017 (AMD over-covering excursion in 2004, troughs in 2016-2017 for AMD and Nvidia, the 2008-2009 crisis window), and my own transfer note describes their calibration as being to "fifteen-plus years of daily data".
-Election experiment: conformalised quantile regression over 3,111 matched US counties, predictions starting once 500 counties have reported, each step splitting observed data 75/25 into training and calibration and refitting a linear quantile regression. Counties are ordered by time zone, east coast first and Hawaii last, so the covariate distribution drifts monotonically rather than jumping — "the shift is manufactured but realistic".</t>
+Election experiment: conformalised quantile regression over 3,111 matched US counties, predictions starting once 500 counties have reported, each step splitting observed data 75/25 into training and calibration and refitting a linear quantile regression. Counties are ordered by time zone, east coast first and Hawaii last, so the covariate distribution drifts monotonically rather than jumping - "the shift is manufactured but realistic".</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
@@ -7707,7 +7707,7 @@
 where alpha is the target miscoverage rate, err_t is the realised miscoverage at step t taking value 0 or 1, and gamma &gt; 0 is the step size. When the interval covered, alpha_{t+1} rises by gamma*alpha and the next interval narrows; when it missed, alpha_{t+1} falls by gamma(1-alpha) and the next interval widens. The appendix shows this is online gradient descent on the pinball loss rho_alpha(beta_t - alpha_t), though the authors note standard regret bounds don't capture what they want, "because regret is measured against a fixed comparator and alpha_t* is a moving target". A weighted variant replaces err_t with sum_s w_s err_s for weights w_s proportional to 0.95^{t-s}, producing almost identical trajectories, "only smoother".
 Underlying split-conformal construction: fit a score S(X,Y) on a training set, compute its 1-alpha empirical quantile Q_hat(1-alpha) on a held-out calibration set, return C_hat_t = {y : S(X_t, y) &lt;= Q_hat(1-alpha)}.
 Point predictor in the volatility experiment: GARCH(1,1), sigma_t^2 = omega + tau*V_{t-1} + beta*sigma_{t-1}^2. Target coverage 1 - alpha = 0.9, initialised alpha_1250 = 0.1, step size gamma = 0.005 fixed. Comparators: fixed alpha_t = alpha on the same rolling window, plus an i.i.d. Bernoulli(0.1) sequence.
-The guarantee that costs nothing — Proposition 4.1, which is the one I would cite — states that with probability one, for all T:
+The guarantee that costs nothing - Proposition 4.1, which is the one I would cite - states that with probability one, for all T:
 |(1/T) sum_{t=1}^{T} err_t - alpha| &lt;= (max{alpha_1, 1-alpha_1} + gamma) / (T*gamma)
 where alpha_1 is the initialisation; it follows from Lemma 4.1, that alpha_t stays in [-gamma, 1+gamma] for all t. The proof is three lines of rearranging the recursion and places "no constraint whatsoever on the data generating distribution", which is a strong statement and also "a statement about the time average rather than about any single t". The long-run empirical coverage frequency therefore converges to the target for any data generating process whatsoever, with the finite-sample deviation bound distribution-free and shrinking as 1/T.
 The sharper results cost assumptions. Theorems 4.1 and 4.2 model the environment as a hidden Markov chain {A_t} with non-zero absolute spectral gap 1 - eta, assume (alpha_t, A_t) is stationary and that Q_hat_t(.) and S_t(.) don't depend on t, then give a Bernstein-type concentration bound on |T^{-1} sum err_t - alpha| and an L-Lipschitz bound on E[(M(alpha_t | A_t) - alpha)^2] of the form
@@ -7718,17 +7718,17 @@
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — this is a single-model statistical wrapper with no agents, no orchestrator and no decision layer. In the note's words, "there are no agents here, nothing resembling an orchestrator and no trading decision anywhere in it". What it supplies instead is a scalar state variable, alpha_t, that an orchestrator elsewhere could consume. The property I single out is that ACI "has the useful property of not being a detector at all: alpha_t moves continuously, so the shift measurement and the response to it are the same quantity, which is a better fit for a weighting function than a binary alarm."</t>
+          <t>Not applicable - this is a single-model statistical wrapper with no agents, no orchestrator and no decision layer. In the note's words, "there are no agents here, nothing resembling an orchestrator and no trading decision anywhere in it". What it supplies instead is a scalar state variable, alpha_t, that an orchestrator elsewhere could consume. The property I single out is that ACI "has the useful property of not being a detector at all: alpha_t moves continuously, so the shift measurement and the response to it are the same quantity, which is a better fit for a weighting function than a binary alarm."</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — no text, no sentiment component anywhere in this paper. Sentiment is in any case out of scope for my project.</t>
+          <t>Not applicable - no text, no sentiment component anywhere in this paper. Sentiment is in any case out of scope for my project.</t>
         </is>
       </c>
       <c r="N56" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — no filings, no retrieval, no document processing of any kind. The paper's only connection to A_F in my design is by analogy: the scope revision gave a worked example of structural confidence for A_F (does the extracted program parse, does every argument trace to a retrieved figure) and left the other three agents open; ACI supplies the analogue for A_V.</t>
+          <t>Not applicable - no filings, no retrieval, no document processing of any kind. The paper's only connection to A_F in my design is by analogy: the scope revision gave a worked example of structural confidence for A_F (does the extracted program parse, does every argument trace to a retrieved figure) and left the other three agents open; ACI supplies the analogue for A_V.</t>
         </is>
       </c>
       <c r="O56" s="11" t="inlineStr">
@@ -7739,12 +7739,12 @@
       </c>
       <c r="P56" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — no liquidity variables, no spreads, no turnover, no execution cost anywhere in the paper. The liquidity question enters only in my transfer analysis: on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade."</t>
+          <t>Not applicable - no liquidity variables, no spreads, no turnover, no execution cost anywhere in the paper. The liquidity question enters only in my transfer analysis: on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade."</t>
         </is>
       </c>
       <c r="Q56" s="11" t="inlineStr">
         <is>
-          <t>No attribution or interpretability machinery, and none needed — the method is a single scalar recursion and is fully transparent by construction. The interpretable artefact it produces is the alpha_t trajectory itself, which can be read directly as how badly the fitted model is tracking the market at each date. The theory is reported honestly in a way that matters for interpretation: the appendix comparison shows the naive bound decays as O(1/(T sqrt(epsilon_1))) and therefore *increases* as the shift size epsilon_1 shrinks, which the authors call undesirable, while the HMM-based bound decreases with the shift, and "both are reported side by side rather than only the flattering one".</t>
+          <t>No attribution or interpretability machinery, and none needed - the method is a single scalar recursion and is fully transparent by construction. The interpretable artefact it produces is the alpha_t trajectory itself, which can be read directly as how badly the fitted model is tracking the market at each date. The theory is reported honestly in a way that matters for interpretation: the appendix comparison shows the naive bound decays as O(1/(T sqrt(epsilon_1))) and therefore *increases* as the shift size epsilon_1 shrinks, which the authors call undesirable, while the HMM-based bound decreases with the shift, and "both are reported side by side rather than only the flattering one".</t>
         </is>
       </c>
       <c r="R56" s="11" t="inlineStr">
@@ -7766,7 +7766,7 @@
       <c r="T56" s="11" t="inlineStr">
         <is>
           <t>- The guarantee is about coverage and says nothing about width, and no width or efficiency number appears anywhere in the paper. Proposition 4.1 is satisfied by a sequence that alternates between infinite and empty prediction sets in the right proportion, and the mechanism that makes it assumption-free is precisely the one that permits this: when alpha_t &lt; 0 the set is all of R and err_t = 0 by construction, which is how the proof of Lemma 4.1 gets its contradiction. "There is no table of average interval widths, no comparison of width against the fixed-alpha method, and no statement of how often alpha_t goes non-positive in the experiments." The alpha_t trajectories suggest it doesn't happen on these twelve stocks, the minimum sitting near 0.035, "but that's inference from a plot rather than a reported quantity, and a method sold on robustness to crises should report what its intervals cost in the crisis". I have not found that evaluation in the literature I have covered.
-- The results that hold at a single time step require a small shift, a stationary chain and a time-invariant quantile function, "which is close to the regime where I wouldn't need the method". Theorem 4.2 bounds the expected squared deviation of marginal coverage by a quantity proportional to E[|alpha*_{A_{t+1}} - alpha*_{A_t}|], which the authors interpret as a measurement of shift size, "so the bound is informative exactly when the shift is small and vacuous when it is large". The discussion concedes the fixed-Q_hat_t assumption directly and says it would be interesting to determine if similar results hold when Q_hat_t is fit online on recent data — which is what the volatility experiment actually does. "So the headline experiment sits outside the conditions of the sharper theory, and the only guarantee covering it is the long-run average one."
+- The results that hold at a single time step require a small shift, a stationary chain and a time-invariant quantile function, "which is close to the regime where I wouldn't need the method". Theorem 4.2 bounds the expected squared deviation of marginal coverage by a quantity proportional to E[|alpha*_{A_{t+1}} - alpha*_{A_t}|], which the authors interpret as a measurement of shift size, "so the bound is informative exactly when the shift is small and vacuous when it is large". The discussion concedes the fixed-Q_hat_t assumption directly and says it would be interesting to determine if similar results hold when Q_hat_t is fit online on recent data - which is what the volatility experiment actually does. "So the headline experiment sits outside the conditions of the sharper theory, and the only guarantee covering it is the long-run average one."
 - gamma = 0.005 is set once, justified in a sentence, and not varied anywhere in the paper. The stated reason is that it gave relatively stable trajectories while still allowing adaptation, "which is a reasonable thing to say and not a sensitivity analysis". The theory's prescription gamma proportional to sqrt(E|delta alpha*|) requires knowing the typical size of the shift in the optimal parameter, "which is the thing you are using the method to track", and the discussion names adaptive selection of gamma without prior knowledge as an open problem. "For a user with a short sample this is the live question, since the time to recover from a bad initialisation scales as 1/gamma."
 - Two domains, both with immediate feedback, and no decision-level evaluation of any kind. Y_t has to be revealed at every step for the update to run, and the discussion flags delayed or batched responses as outside the method. "Quantile loss and local coverage are the only metrics; there is no comparison against a simpler recalibration scheme beyond fixed-alpha on the same rolling window, no cost attached to an interval that's too wide, and nothing connecting calibration to a downstream decision. That's a fair scope for a statistics paper and a gap for anyone using it inside a trading system, where an interval has a position size attached."
 - The core modelling choice, adjusting the argument to Q_hat_t rather than Q_hat_t itself, is asserted as adequate rather than tested. The paper is explicit that in general both S_t(.) and Q_hat_t(.) should be re-estimated to track recent observations, and then proceeds to fix the quantile function and correct only alpha_t. The score-ablation result is the visible cost of that choice. "The design burden this pushes onto the user is real and under-acknowledged: picking a score that stays approximately stationary under regime change is a modelling problem of the same difficulty as the one the wrapper was meant to abstract away."
@@ -7797,14 +7797,14 @@
       </c>
       <c r="W56" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: C_{i,t} above all — specifically C_{V,t}, the confidence term for A_V — plus the abstention channel, the orchestrator's conditioning set (as a candidate fifth term), the distribution-shift item in the evaluation plan, and the data-depth discussion. It touches nothing in A_T, A_F or A_L directly, and it is tooling rather than a competing architecture, so it cannot close or threaten the orchestration claim in either direction.
-EFFECT ON MAIN GAP: It strengthens the main gap in two distinct ways and leaves the claim itself untouched. First, it closes a specification hole inside my own design rather than outside it. The scope revision redefined C_{i,t} as a structural property of an agent's output rather than a self-report, and gave a worked example only for A_F (does the extracted program parse, does every argument trace to a retrieved figure), leaving the other three agents open. ACI supplies the analogue for A_V: "the calibrated interval width is the structural confidence term the scope revision asked for, and it arrives measured rather than self-reported". The recipe is concrete — wrap the FIGARCH or GJR-GARCH forecast in ACI with the normalised score S_t = |V_t - sigma_hat^2| / sigma_hat^2, and let C_{V,t} be a function of the realised interval width at the target coverage, so a volatility agent whose model has drifted reports wider intervals and is automatically down-weighted. That is a measured property of the output, which is exactly what the redefinition demanded.
+          <t>SPEAKS TO: C_{i,t} above all - specifically C_{V,t}, the confidence term for A_V - plus the abstention channel, the orchestrator's conditioning set (as a candidate fifth term), the distribution-shift item in the evaluation plan, and the data-depth discussion. It touches nothing in A_T, A_F or A_L directly, and it is tooling rather than a competing architecture, so it cannot close or threaten the orchestration claim in either direction.
+EFFECT ON MAIN GAP: It strengthens the main gap in two distinct ways and leaves the claim itself untouched. First, it closes a specification hole inside my own design rather than outside it. The scope revision redefined C_{i,t} as a structural property of an agent's output rather than a self-report, and gave a worked example only for A_F (does the extracted program parse, does every argument trace to a retrieved figure), leaving the other three agents open. ACI supplies the analogue for A_V: "the calibrated interval width is the structural confidence term the scope revision asked for, and it arrives measured rather than self-reported". The recipe is concrete - wrap the FIGARCH or GJR-GARCH forecast in ACI with the normalised score S_t = |V_t - sigma_hat^2| / sigma_hat^2, and let C_{V,t} be a function of the realised interval width at the target coverage, so a volatility agent whose model has drifted reports wider intervals and is automatically down-weighted. That is a measured property of the output, which is exactly what the redefinition demanded.
 Second, it converts the abstention channel from a hand-set threshold into a quantity that moves on its own. The design already treats abstention as structural because A_F is expected to be unusable more than half the time on CSE filings; the same machinery now works for a price-derived agent. "When alpha_t falls low enough that the interval at the target coverage spans the plausible range of next-day volatility, the agent has nothing to say, and the orchestrator should see that as absence rather than as a weak signal. This is the mechanism AlphaAgents lacked when a human deleted an agent by hand, expressed as a quantity that moves on its own."
 The boundary of the contribution needs stating plainly and early, which is why the note ends where it does: "ACI is an off-the-shelf wrapper with a public R implementation, four years old and widely cited, and there is nothing novel in applying it to a GARCH forecast since that is the paper's own worked example. What would be a candidate technical contribution not identified in the literature I have covered is using the adapted miscoverage level as an input to a weighting function over heterogeneous agents, which is a different claim and a much narrower one, and it needs validating against recent work before it goes anywhere near the novelty statement." So: adopt ACI as a component, claim only the orchestration use of alpha_t, and validate that narrower claim before it enters the novelty statement.
-EFFECT ON SUB-GAP 1: Mostly indirect, and it creates one new liquidity dependency rather than resolving anything. The paper has no liquidity content at all — no spreads, no turnover, no execution cost. But the score-design finding pushes liquidity into the calibration layer, which I had not anticipated. Normalising the conformity score by predicted variance is what made their score approximately stationary; on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade." The candidate fix is to normalise by a liquidity-adjusted volatility estimate "using the same Amihud and turnover inputs already being computed for the cost model and for the composite liquidity state, so one measurement serves a third purpose." That is a reuse of L_t inside the machinery that produces C_{V,t}, which is a genuine coupling between the liquidity state and the reliability of a price-derived agent — the second half of Sub-gap 1's statement, that liquidity simultaneously conditions the reliability of price-derived agents. It is recorded as "a named experiment, not a design decision", so it is a hypothesis I owe a test, not a finding I can lean on.
-EFFECT ON SUB-GAP 2: Substantial, and in a way that is adjacent to rather than inside Sub-gap 2. Sub-gap 2 is about volatility PERSISTENCE and specifically about replacing an EWMA half-life, which assumes exponential decay, with a persistence-aware decay schedule. ACI does not estimate persistence and does not propose a decay schedule, so it does not close the sub-gap. What it does is supply a second, independent slow-moving state series over the same volatility object: at gamma = 0.005 a single miss moves alpha_t by 0.0045, "so these swings take hundreds of days to develop, and the series is slow-moving by construction in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]." The alpha_t trajectories "read as a volatility-regime series in their own right", ranging about 0.035 to 0.17 and bottoming out in 2008-2009 when the GARCH fit is worst. That is a measurement of how badly a fitted volatility model is tracking the market, which is a different quantity from P_t but lives on the same timescale and is produced by the same agent — so the discipline required is to test whether alpha_t adds anything over the existing four conditioning terms, not to assume it does. Hence the note's framing: carry it "as a candidate addition to the conditioning set and test it on the ablation protocol against the existing four terms rather than adopting it."
+EFFECT ON SUB-GAP 1: Mostly indirect, and it creates one new liquidity dependency rather than resolving anything. The paper has no liquidity content at all - no spreads, no turnover, no execution cost. But the score-design finding pushes liquidity into the calibration layer, which I had not anticipated. Normalising the conformity score by predicted variance is what made their score approximately stationary; on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade." The candidate fix is to normalise by a liquidity-adjusted volatility estimate "using the same Amihud and turnover inputs already being computed for the cost model and for the composite liquidity state, so one measurement serves a third purpose." That is a reuse of L_t inside the machinery that produces C_{V,t}, which is a genuine coupling between the liquidity state and the reliability of a price-derived agent - the second half of Sub-gap 1's statement, that liquidity simultaneously conditions the reliability of price-derived agents. It is recorded as "a named experiment, not a design decision", so it is a hypothesis I owe a test, not a finding I can lean on.
+EFFECT ON SUB-GAP 2: Substantial, and in a way that is adjacent to rather than inside Sub-gap 2. Sub-gap 2 is about volatility PERSISTENCE and specifically about replacing an EWMA half-life, which assumes exponential decay, with a persistence-aware decay schedule. ACI does not estimate persistence and does not propose a decay schedule, so it does not close the sub-gap. What it does is supply a second, independent slow-moving state series over the same volatility object: at gamma = 0.005 a single miss moves alpha_t by 0.0045, "so these swings take hundreds of days to develop, and the series is slow-moving by construction in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]." The alpha_t trajectories "read as a volatility-regime series in their own right", ranging about 0.035 to 0.17 and bottoming out in 2008-2009 when the GARCH fit is worst. That is a measurement of how badly a fitted volatility model is tracking the market, which is a different quantity from P_t but lives on the same timescale and is produced by the same agent - so the discipline required is to test whether alpha_t adds anything over the existing four conditioning terms, not to assume it does. Hence the note's framing: carry it "as a candidate addition to the conditioning set and test it on the ablation protocol against the existing four terms rather than adopting it."
 The sharper transfer finding is that ACI's own step size has the same structural problem Sub-gap 2 identifies in the EWMA half-life. gamma is a fixed decay rate on a non-stationary target, set once, never varied, and justified in a sentence; the theory's own prescription gamma proportional to sqrt(E|delta alpha*|) says gamma should be larger in more volatile environments, which is a persistence-type statement the paper does not operationalise. So ACI imports the exact defect Sub-gap 2 exists to correct, one level up. That is useful: it means the persistence argument generalises beyond the volatility scaler, and it also means I cannot adopt gamma = 0.005 and stop thinking. "On 374 observations a step that small means alpha_t barely leaves its initialisation, so the sample would be spent in the transient the theory warns about, and the prescription gamma proportional to sqrt(E|delta alpha*|) points the same way given the CSE's crisis sequence. The experiment is a gamma sweep on the index track where I have the length to measure it, then carry the chosen value down to the counters."
-CSE DATA EVIDENCE: The paper contains none — twelve US names and 3,111 US counties. The CSE evidence in this cell is my own data-depth accounting, and it is the sharpest constraint in the note: "The 1250-day refit window is the sharpest data-depth constraint I've hit in a review and it splits my two tracks. Five years of daily data per counter, with the calibration scores drawn from the same window, against 374 trading days per counter in the archive. On the index track at ten years daily the recipe transfers as written; on the per-counter track it does not, and the honest options are a shorter joint window with the calibration degradation reported, or pooling scores across counters, which breaks the per-counter conditioning the method relies on. This belongs in the data-depth discussion as a named requirement with a number attached, not as a general concern." Five years per counter is roughly thirteen times the per-counter archive. Note also that shrinking the window degrades the GARCH fit and the empirical quantile simultaneously, because the calibration scores come from the same window — the two failures are not independent.
+CSE DATA EVIDENCE: The paper contains none - twelve US names and 3,111 US counties. The CSE evidence in this cell is my own data-depth accounting, and it is the sharpest constraint in the note: "The 1250-day refit window is the sharpest data-depth constraint I've hit in a review and it splits my two tracks. Five years of daily data per counter, with the calibration scores drawn from the same window, against 374 trading days per counter in the archive. On the index track at ten years daily the recipe transfers as written; on the per-counter track it does not, and the honest options are a shorter joint window with the calibration degradation reported, or pooling scores across counters, which breaks the per-counter conditioning the method relies on. This belongs in the data-depth discussion as a named requirement with a number attached, not as a general concern." Five years per counter is roughly thirteen times the per-counter archive. Note also that shrinking the window degrades the GARCH fit and the empirical quantile simultaneously, because the calibration scores come from the same window - the two failures are not independent.
 PROPOSED REVISION STATED IN THE NOTE: Several, all recorded as candidates or experiments rather than adopted design:
 1. Define C_{V,t} as a function of the ACI-calibrated interval width at the target coverage, wrapping the FIGARCH or GJR-GARCH forecast with the normalised conformity score.
 2. Trigger A_V abstention when alpha_t falls low enough that the target-coverage interval spans the plausible range of next-day volatility, and have the orchestrator read that as absence rather than as a weak signal.
@@ -7831,23 +7831,23 @@
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Gu, Kelly and Xiu. Empirical Asset Pricing via Machine Learning. Citekey guEmpiricalAssetPricing2018. Affiliations recorded in the note: Chicago Booth and Yale. The note's frontmatter gives year 2018 and the body dates the version read as the "November 2018 working version". The body also states this is "of what became the *Review of Financial Studies* paper that everything in this area now cites" — so the journal is the Review of Financial Studies, but the note does not record the RFS publication year, volume, pages or DOI. First names, DOI, arXiv ID and link: Not recorded in the note.
+          <t>Gu, Kelly and Xiu. Empirical Asset Pricing via Machine Learning. Citekey guEmpiricalAssetPricing2018. Affiliations recorded in the note: Chicago Booth and Yale. The note's frontmatter gives year 2018 and the body dates the version read as the "November 2018 working version". The body also states this is "of what became the *Review of Financial Studies* paper that everything in this area now cites" - so the journal is the Review of Financial Studies, but the note does not record the RFS publication year, volume, pages or DOI. First names, DOI, arXiv ID and link: Not recorded in the note.
 TO BE EXPLICIT ABOUT WHICH IS WHICH: 2018 is the working-paper year from the note's frontmatter and is the version the note was written against; the Review of Financial Studies is the eventual journal of record, and its publication year is Not recorded in the note.</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>2020 (Review of Financial Studies 33(5)). The note's frontmatter carries 2018, the working-paper year; 2020 is the journal of record.</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Working paper in the version read (November 2018); published subsequently in the *Review of Financial Studies*, which the note describes as "the paper that everything in this area now cites". Volume and pages: Not recorded in the note.</t>
+          <t>Working paper in the version read (November 2018); published subsequently in the *Review of Financial Studies*, which the note describes as "the paper that everything in this area now cites". Volume and pages: Not recorded in the note. The note's frontmatter carries 2018, the working-paper year; 2020 is the journal of record.</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note.</t>
+          <t>DOI 10.2139/ssrn.3159577. This is the SSRN working-paper DOI; the note's journal of record is Review of Financial Studies 33(5).</t>
         </is>
       </c>
       <c r="F57" s="11" t="inlineStr">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>US equities — every firm on NYSE, AMEX and NASDAQ. A deep, liquid, developed market, sixty years of it. No emerging or frontier market content. The note draws the implication in the opposite direction: "the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."</t>
+          <t>US equities - every firm on NYSE, AMEX and NASDAQ. A deep, liquid, developed market, sixty years of it. No emerging or frontier market content. The note draws the implication in the opposite direction: "the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."</t>
         </is>
       </c>
       <c r="I57" s="11" t="inlineStr">
@@ -7879,7 +7879,7 @@
 - Refit: recursive, once per year, training window grows by one year each time.
 - Validation: fixed-size, rolled forward twelve months per refit.
 - Primary metric: R^2_oos benchmarked against zero, not the historical mean.
-Four choices the note flags as mattering more than they look: the sample is deliberately unfiltered — stocks below $5, share codes beyond 10 and 11, and financial firms all retained — "which I note here because the economic results later depend on the small end of the universe"; publication lags are imposed explicitly, monthly characteristics delayed at most one month, quarterly at least four, annual at least six; missing characteristics are replaced with the cross-sectional median for that month; and there is no cross-validation anywhere, by design, to preserve temporal ordering.</t>
+Four choices the note flags as mattering more than they look: the sample is deliberately unfiltered - stocks below $5, share codes beyond 10 and 11, and financial firms all retained - "which I note here because the economic results later depend on the small end of the universe"; publication lags are imposed explicitly, monthly characteristics delayed at most one month, quarterly at least four, annual at least six; missing characteristics are replaced with the cross-sectional median for that month; and there is no cross-validation anywhere, by design, to preserve temporal ordering.</t>
         </is>
       </c>
       <c r="J57" s="11" t="inlineStr">
@@ -7898,7 +7898,7 @@
         <is>
           <t>Thirteen prediction methods, all on the same target and the same splits, differing only in how they constrain g(.): OLS on all 920 features, a three-characteristic OLS benchmark (OLS-3), PLS, PCR, elastic net, a spline generalized linear model with group lasso (GLM), random forest, gradient boosted regression trees (GBRT), and feed-forward networks at one through five hidden layers (NN1-NN5).
 - PCR and PLS both compress 920 features into K components, PCR maximising variance among the predictors and PLS maximising squared covariance with the target, "so PLS sacrifices fidelity to Z for predictive relevance".
-- GLM adds a second-order spline expansion per characteristic under a group lasso penalty, so a characteristic enters with all K of its spline terms or none, and critically it adds NO interactions — "which is what makes it the diagnostic model of the paper".
+- GLM adds a second-order spline expansion per characteristic under a group lasso penalty, so a characteristic enters with all K of its spline terms or none, and critically it adds NO interactions - "which is what makes it the diagnostic model of the paper".
 - Networks are fixed at five architectures following the geometric pyramid rule, NN1 at 32 neurons through NN5 at 32-16-8-4-2, all ReLU, all fully connected, trained by SGD with Adam learning-rate shrinkage, l_1 penalisation, early stopping, batch normalisation, and seed ensembling.
 - Robust losses run throughout. The Huber objective replaces squared loss with absolute loss beyond a tuned threshold xi; the authors report the Huber variant for OLS, elastic net, GLM and GBRT because it performs better, and the Monte Carlo confirms it improves out-of-sample R^2 for every method it is applied to.
 Output: a one-month-ahead excess-return forecast per stock, aggregated into decile-spread portfolios and bottom-up S&amp;P 500 forecasts for the economic evaluation.</t>
@@ -7906,22 +7906,22 @@
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — a single-estimator horse race with no agents, no orchestrator, no weighting of heterogeneous producers over a shared decision. What it does instead is the closest single-model analogue: the Kronecker construction makes every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator. The note draws the line precisely: "That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound. What it does not do is the thing I am claiming: the interaction weights are estimated once per annual refit, they are a function of macro variables rather than of any measured reliability of the signal, and no channel in their model can go absent, because a missing characteristic is median-imputed rather than down-weighted. The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line."</t>
+          <t>Not applicable - a single-estimator horse race with no agents, no orchestrator, no weighting of heterogeneous producers over a shared decision. What it does instead is the closest single-model analogue: the Kronecker construction makes every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator. The note draws the line precisely: "That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound. What it does not do is the thing I am claiming: the interaction weights are estimated once per annual refit, they are a function of macro variables rather than of any measured reliability of the signal, and no channel in their model can go absent, because a missing characteristic is median-imputed rather than down-weighted. The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line."</t>
         </is>
       </c>
       <c r="M57" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — no sentiment data, no text, no news or social signal anywhere in the paper. Sentiment is out of scope for my project in any case.</t>
+          <t>Not applicable - no sentiment data, no text, no news or social signal anywhere in the paper. Sentiment is out of scope for my project in any case.</t>
         </is>
       </c>
       <c r="N57" s="11" t="inlineStr">
         <is>
-          <t>No retrieval, no documents, no RAG — accounting characteristics enter as pre-constructed numeric features from CRSP/Compustat-style panels, not as parsed filings. What the paper contributes to A_F is a horizon and lag discipline rather than a pipeline. Accounting characteristics cluster at the bottom of the importance ranking, and the authors attribute this partly to their low update frequency, noting that at the annual horizon price-trend variables lose ground to liquidity and risk measures while industry becomes substantially predictive. The publication-lag structure is explicit — monthly characteristics delayed at most one month, quarterly at least four, annual at least six — and the note treats this as the specification to write down for A_F "before touching any filing data, since CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."</t>
+          <t>No retrieval, no documents, no RAG - accounting characteristics enter as pre-constructed numeric features from CRSP/Compustat-style panels, not as parsed filings. What the paper contributes to A_F is a horizon and lag discipline rather than a pipeline. Accounting characteristics cluster at the bottom of the importance ranking, and the authors attribute this partly to their low update frequency, noting that at the annual horizon price-trend variables lose ground to liquidity and risk measures while industry becomes substantially predictive. The publication-lag structure is explicit - monthly characteristics delayed at most one month, quarterly at least four, annual at least six - and the note treats this as the specification to write down for A_F "before touching any filing data, since CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."</t>
         </is>
       </c>
       <c r="O57" s="11" t="inlineStr">
         <is>
-          <t>Volatility enters as a predictor family rather than as a modelled process. The "risk" group — total volatility, idiosyncratic volatility, beta, beta squared — is one of the three dominant families across every method. The marginal-relationship plots show trees and networks finding large sensitivity to volatility where penalized linear models find none: a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return under GBRT or NN3 (and the companion size effect: a firm falling from median size to the 20th percentile gains roughly 2.4% in annualised expected return). On the macro side, market-level stock variance gets little weight anywhere and essentially none from the networks.
+          <t>Volatility enters as a predictor family rather than as a modelled process. The "risk" group - total volatility, idiosyncratic volatility, beta, beta squared - is one of the three dominant families across every method. The marginal-relationship plots show trees and networks finding large sensitivity to volatility where penalized linear models find none: a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return under GBRT or NN3 (and the companion size effect: a firm falling from median size to the 20th percentile gains roughly 2.4% in annualised expected return). On the macro side, market-level stock variance gets little weight anywhere and essentially none from the networks.
 No conditional volatility model, no GARCH, no persistence estimate, no volatility targeting, no risk scaling of positions. Portfolio construction is decile sorts, equal- and value-weighted, with Sharpe reported but no volatility budget.</t>
         </is>
       </c>
@@ -7934,7 +7934,7 @@
       <c r="Q57" s="11" t="inlineStr">
         <is>
           <t>Variable importance is defined as the reduction in predictive R^2 from setting one predictor to zero with all other estimates held fixed. Marginal-relationship plots show each model's fitted sensitivity to individual characteristics. A placebo test adds five simulated noise characteristics and they rank low, which the note credits as a real check. The paper also reports model complexity over time (Figure 3): elastic net selecting fewer than five features in the first decade of the test sample and 20 to 40 after 2000, PCR using 20 to 40 components, GBRT moving from roughly 20 features to 30.
-The note's reading of the attribution machinery is sceptical — see LIMITATIONS — and it re-flags Section 1.6's own concession that these are measurements rather than mechanisms.</t>
+The note's reading of the attribution machinery is sceptical - see LIMITATIONS - and it re-flags Section 1.6's own concession that these are measurements rather than mechanisms.</t>
         </is>
       </c>
       <c r="R57" s="11" t="inlineStr">
@@ -7952,11 +7952,11 @@
       <c r="S57" s="11" t="inlineStr">
         <is>
           <t>- Absolute numbers are tiny and the spread across methods is narrower than the narrative suggests. Monthly stock-level R^2_oos: OLS on all 920 features -4.60% (worse than forecasting zero); OLS-3 0.16%; elastic net 0.09%; PLS 0.18%; PCR 0.28%; GLM 0.19%; random forest 0.27%; GBRT 0.30%; networks 0.35% (NN1) to a peak of 0.39% (NN3). "So the entire distance from the three-characteristic benchmark to the best model in the paper is 23 basis points of monthly R^2." Size split: NN3 reaches 0.72% on the top 1,000 stocks by market value against 0.46% on the bottom 1,000. At the annual horizon everything scales up roughly an order of magnitude, NN4 at 3.60% and NN3 at 3.40% across all stocks.
-- The Diebold-Mariano table does not support the method ranking the abstract implies, and the paper is upfront about this itself. Differences among all the regularized linear models are insignificant — OLS-3, PLS, PCR, elastic net and GLM are statistically indistinguishable from each other. Trees improve on linear models but the improvements are described as at best marginally significant. Neural networks are the only class producing large significant gains over linear and generalized linear models, NN3 against OLS-3 at 3.01, and their improvement over trees is not significant. Among the networks themselves nothing clears: NN3 against NN5 reaching -1.92 and NN3 against NN4 only -1.03. "On this evidence the defensible claim is narrower than 'trees and neural nets are the best performing methods': it is that networks beat linear specifications, and that everything else in the ranking is suggestive."
+- The Diebold-Mariano table does not support the method ranking the abstract implies, and the paper is upfront about this itself. Differences among all the regularized linear models are insignificant - OLS-3, PLS, PCR, elastic net and GLM are statistically indistinguishable from each other. Trees improve on linear models but the improvements are described as at best marginally significant. Neural networks are the only class producing large significant gains over linear and generalized linear models, NN3 against OLS-3 at 3.01, and their improvement over trees is not significant. Among the networks themselves nothing clears: NN3 against NN5 reaching -1.92 and NN3 against NN4 only -1.03. "On this evidence the defensible claim is narrower than 'trees and neural nets are the best performing methods': it is that networks beat linear specifications, and that everything else in the ranking is suggestive."
 - Interactions, not nonlinearity, are the mechanism, and the GLM is the clean evidence. The GLM applies spline expansions to every individual characteristic and reaches 0.19%, no better than the linear specifications, despite selecting more features than elastic net. Since the only thing it lacks relative to trees and networks is multi-way interaction, the authors read the gap as attributable to interactions specifically rather than to curvature. The note rates this "the most convincing single inference in the paper because it is a genuine ablation rather than a comparison across unrelated model families." Marginal-relationship plots corroborate: penalized linear models find no association at all between returns and either size or volatility while trees and networks find large sensitivity to both.
-- Shallow beats deep, and the simulation says why. Performance peaks at three hidden layers and declines at four and five; random forests settle on trees of one to five layers on average; GBRT selects fewer than six leaves. The authors attribute this to "the comparative dearth of data and the low signal-to-noise ratio relative to settings like computer vision where deep learning thrives." The Monte Carlo makes the trade-off concrete: under a sparse linear DGP the nonlinear methods lose very little — ENet+H at 4.27% out-of-sample against NN1 at 4.42% and RF at 3.37% — but under a nonlinear interacted process the ordering becomes decisive, GBRT+H and NN2 both at 3.12% against ENet+H at 0.59% and GLM+H at 1.27%, with the oracle at 5.40%. "The asymmetry is the useful part: flexible methods cost almost nothing when the truth is linear and gain a great deal when it is not."
+- Shallow beats deep, and the simulation says why. Performance peaks at three hidden layers and declines at four and five; random forests settle on trees of one to five layers on average; GBRT selects fewer than six leaves. The authors attribute this to "the comparative dearth of data and the low signal-to-noise ratio relative to settings like computer vision where deep learning thrives." The Monte Carlo makes the trade-off concrete: under a sparse linear DGP the nonlinear methods lose very little - ENet+H at 4.27% out-of-sample against NN1 at 4.42% and RF at 3.37% - but under a nonlinear interacted process the ordering becomes decisive, GBRT+H and NN2 both at 3.12% against ENet+H at 0.59% and GLM+H at 1.27%, with the oracle at 5.40%. "The asymmetry is the useful part: flexible methods cost almost nothing when the truth is linear and gain a great deal when it is not."
 - Aggregation into portfolios multiplies the measurable signal and is where linear methods fail outright. Bottom-up S&amp;P 500 forecasts give monthly R^2_oos of -0.11% for OLS-3 and -2.62% for PCR, against 0.86% for GLM and 1.80% for NN3, rising to 15.68% at the annual horizon. The explanation offered is that individual stock returns behave erratically for the smallest and least liquid names, so averaging into portfolios cancels idiosyncratic noise while preserving the signal. Running the Campbell-Thompson mapping, the S&amp;P 500 buy-and-hold Sharpe of 0.42 becomes 0.63 for an investor timing on NN3 forecasts.
-- Every method converges on the same three signal families. Top eight characteristics by summed importance across all eleven models: short-term reversal, log market equity, twelve-month momentum, momentum change, recent maximum return, industry momentum, return volatility, dollar volume. Grouped: price trend, liquidity, risk, with valuation ratios a distant fourth. Linear and dimension-reduction models concentrate importance heavily on momentum and reversal; trees and networks spread it more evenly. On the macro side every method treats aggregate book-to-market as a critical predictor — the single highest-weighted macro variable for the networks and the penalized linear models at 28.57% for NN1 and 43.46% for GLM — while stock variance gets little weight anywhere. The split between families is sharper than the consensus: linear models load overwhelmingly on default spread and the Treasury rate (42.13% on default spread for elastic net) while the networks put essentially nothing there (0.06% for NN3) and load instead on term spread and net equity issuance.
+- Every method converges on the same three signal families. Top eight characteristics by summed importance across all eleven models: short-term reversal, log market equity, twelve-month momentum, momentum change, recent maximum return, industry momentum, return volatility, dollar volume. Grouped: price trend, liquidity, risk, with valuation ratios a distant fourth. Linear and dimension-reduction models concentrate importance heavily on momentum and reversal; trees and networks spread it more evenly. On the macro side every method treats aggregate book-to-market as a critical predictor - the single highest-weighted macro variable for the networks and the penalized linear models at 28.57% for NN1 and 43.46% for GLM - while stock variance gets little weight anywhere. The split between families is sharper than the consensus: linear models load overwhelmingly on default spread and the Treasury rate (42.13% on default spread for elastic net) while the networks put essentially nothing there (0.06% for NN3) and load instead on term spread and net equity issuance.
 - Economic results: best strategy is an equal-weighted decile spread on NN4 forecasts returning 3.3% per month, 39.0% annualised, out-of-sample Sharpe 2.35, monthly turnover 114.08%, with no costs deducted. Value weighting drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27.</t>
         </is>
       </c>
@@ -7973,7 +7973,7 @@
         <is>
           <t>- A ceiling and an expectation band for A_T. Thirty thousand stocks, sixty years, 920 engineered features, eleven method families and a thirty-year test window produce 0.39% monthly R^2_oos at the stock level. Against that, my confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information", so "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result." This sits alongside the 0.54 to 0.58 directional-accuracy band from [[Extending machine learning prediction capabilities by explainable AI in financial time series prediction]] and the 54.3% out-of-sample figure in [[Deep Learning with Long Short-Term Memory Networks for Financial Market Predictions]], "and the three together are now a defensible prior rather than one paper's number."
 - Model sizing: "Size the technical agent at NN1 or NN2 scale and stop treating depth as a dial." Performance peaks at three hidden layers on sixty years of data and declines beyond it, with data scarcity and low signal-to-noise named as the cause; on a dataset smaller by orders of magnitude the implied architecture is one or two hidden layers, or a regularized tree ensemble, "and the depth sweep that would be routine elsewhere is not worth the compute here. The same reasoning applies to feature count, since every method in the paper selected far fewer features than it was offered."
-- Huber loss as a default, not a refinement — it improves out-of-sample performance for every method in the simulation and for four of the methods in the empirical work, "and CSE daily returns are heavier-tailed than US monthly returns, so the case is stronger here than there."
+- Huber loss as a default, not a refinement - it improves out-of-sample performance for every method in the simulation and for four of the methods in the empirical work, "and CSE daily returns are heavier-tailed than US monthly returns, so the case is stronger here than there."
 - The publication-lag discipline as the A_F specification to write down before touching filing data: monthly delayed one month, quarterly four, annual six.
 - The evaluation protocol in full: "Recursive expanding training window, fixed-size rolling validation, annual refit, no cross-validation, modified Diebold-Mariano on cross-sectionally averaged error differences with Newey-West standard errors, and R^2_oos benchmarked against zero with the choice stated." Plus the Campbell-Thompson Sharpe mapping reported alongside the R^2, "cheap and converts a statistical number into the economic one the evaluation actually cares about, with the caveat that it assumes costless timing and will therefore be optimistic on a thin book."
 - Independent large-sample evidence for two of my three state variables (liquidity and risk/volatility), and for the macro rejection.
@@ -7984,7 +7984,7 @@
         <is>
           <t>- No costs, no participation-rate analysis, no execution model. The paper reports turnover and stops. That is the whole of Sub-gap 1's motivation stated by a canonical paper without being addressed.
 - No reliability weighting and no absence channel. Conditioning on state happens through fixed, annually-refit interaction coefficients on macro variables; a missing input is median-imputed, never down-weighted, and nothing can go absent.
-- No test of whether the set of features carrying signal is itself regime-dependent — the drift in Figure 3 is explained rather than tested, and the note names this as "the hypothesis my orchestrator rests on and the one this paper was best placed to check."
+- No test of whether the set of features carrying signal is itself regime-dependent - the drift in Figure 3 is explained rather than tested, and the note names this as "the hypothesis my orchestrator rests on and the one this paper was best placed to check."
 - No uncertainty on the empirical tables and no seed variation outside the simulations.
 - No volatility persistence content at all: volatility is a predictor, never a modelled process with a decay structure.
 - Nothing about frontier-market conditions; the paper's own size/liquidity result says its methods work least well there.
@@ -7994,20 +7994,20 @@
       <c r="W57" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T first (expectation band, architecture sizing, loss function, feature count), then the orchestrator's conditioning set (independent large-sample evidence for L_t and V_t, and the Kronecker construction as the single-model analogue of the orchestration claim), then the evaluation layer (benchmark choice, DM test, recursive protocol, Campbell-Thompson mapping), then A_F (horizon and lag discipline, and an argument for a low baseline weight plus explicit abstention), and finally Sub-gap 1, for which this paper is the cleanest reference case in the set.
-EFFECT ON MAIN GAP: It strengthens the premise and sharpens the claim without threatening either. The Kronecker construction is the single-model version of what I am proposing one level up: "Gu et al. make every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator, and the beta-pricing derivation is a principled reason to do it. That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound." That matters because it means the idea that a signal's value varies with market state is not something I have to argue for from scratch — it is derivable from E_t(r_{i,t+1}) = beta'_{i,t} lambda_t with beta_{i,t} = theta_1 c_{i,t} and lambda_t = theta_2 x_t, and it is the standard specification in the most-cited paper in the area.
-Then the line. Three differences separate their construction from mine, and all three are in w(i,t) = f(L_t, V_t, P_t, C_{i,t}): their interaction weights are estimated once per annual refit, so they do not vary with measured market state at decision time, only with the value of the macro variable plugged into a fixed coefficient; they are a function of macro variables rather than of any measured reliability of the signal, so there is no C_{i,t} analogue anywhere in the model; and no channel can go absent, "because a missing characteristic is median-imputed rather than down-weighted". The note puts the whole claim on that last point: "The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line." Median imputation is the exact anti-pattern my abstention channel exists to replace — it substitutes a plausible value for a missing one and the downstream model cannot tell the difference, whereas abstention makes absence visible to the aggregator.
-It also supplies the evidence base for two of the four conditioning terms. Liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) and risk (total volatility, idiosyncratic volatility, beta, beta squared) are two of the three dominant families across every one of eleven method families on a ~30,000-stock, 60-year panel. "That is a far larger evidence base for those two conditioning inputs than the CSE-specific work in [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] or the Granger result at p = 0.0041 from volume to ASPI, and it composes with both." The macro rejection also survives: market-level stock variance is given little weight by any method and essentially none by the networks, consistent with the thin ARDL result in [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]] that already got the macro block rejected. The one live challenge is aggregate book-to-market — critical for every model, 28.57% for NN1 and 43.46% for GLM — and the honest response recorded in the note is to "test it against an ASPI-level valuation ratio rather than dismiss it on the strength of a rejection aimed at different variables."
-One further point that bears directly on the main gap and that the paper declined to test: Figure 3 shows model complexity drifting across the test period — elastic net selecting fewer than five features in the first decade and 20 to 40 after 2000, GBRT moving from roughly 20 features to 30 — and the authors explain it by a growing cross section and improving data coverage. "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." So the paper leaves my central hypothesis open on evidence it had in hand, which is a better position for me than either confirming or refuting it would have been.
-EFFECT ON SUB-GAP 1: This is the strongest available illustration of why cost belongs inside the objective rather than after it, and I would cite it as the reference case. "A strategy turning over 113% of its book monthly, concentrated in price-trend signals, on a universe that deliberately includes the smallest and least liquid names, reported at Sharpe 2.35 with no cost deduction and no participation-rate analysis, is the reference case for my cost sub-gap." Two details make it sharper than a generic "they ignored costs" complaint. First, the value-weighted collapse — NN3 from 2.32 to 1.25, OLS-3 from 0.89 to 0.27 — "is itself a partial, unacknowledged cost estimate and I should cite it that way": moving weight away from the small end halves the Sharpe before a single basis point of spread is charged, which is a lower bound on what liquidity is doing to the result. Second, the internal tension: the paper offers the top-1,000 R^2 of 0.72% against 0.46% on the bottom 1,000 as reassurance that the result is not driven by small-cap illiquidity, while the headline economic result is an equal-weighted spread over the whole board — "both cannot be load-bearing at once."
-Applied to the CSE this is not implementable at any size. "On the CSE, where Dissanayake and Nanayakkara find unexpected illiquidity shocks depressing returns by -0.084 to -0.097 and small caps more than large, that turnover is not implementable at any size, which is the concrete argument for sweeping participation rate against daily volume rather than charging a flat spread, as [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] both do in their different ways." So the paper does not close any part of Sub-gap 1 — it has no friction model at all — but it supplies the clearest demonstration of the failure the sub-gap names, from a source that is hard to dismiss.
-EFFECT ON SUB-GAP 2: Limited, and I should not overclaim it. The paper has no volatility process, no persistence estimate, no decay schedule and no volatility targeting; volatility enters only as a cross-sectional predictor. So it neither closes nor narrows Sub-gap 2. What it contributes is one piece of supporting evidence and one adjacent warning. The evidence: the risk family (total volatility, idiosyncratic volatility, beta, beta squared) is one of the three dominant predictor families across all eleven methods, and the GBRT/NN3 marginal relationship is economically large — a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return — which supports keeping V_t in the conditioning set but says nothing about P_t. The warning is the complexity-drift result again: the paper observed a time-varying structure in its own fitted models and explained it away rather than testing it, which is the same category of move as assuming a fixed exponential decay rate and never checking.
-CSE DATA EVIDENCE: None in the paper — US only. The CSE content in this cell is my own transfer accounting. My confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information" than 30,000 stocks over 60 years with 920 features. The direct consequence is a leakage tripwire: "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result", which composes with the 0.54-0.58 directional-accuracy band and the 54.3% out-of-sample figure from the two other notes into "a defensible prior rather than one paper's number". The second consequence is the architecture ceiling: if three hidden layers is already past the optimum on sixty years of US monthly data, one or two layers or a regularized tree ensemble is the ceiling on 374 trading days. The third is that the benchmark choice has to be stated every time, because "the three-percentage-point inflation from benchmarking against the historical mean is larger than any effect I am likely to measure, so a CSE result reported without naming its benchmark is uninterpretable." And the fourth is the frontier-market reading of their own size result: machine learning works least well in the conditions the CSE presents continuously.
+EFFECT ON MAIN GAP: It strengthens the premise and sharpens the claim without threatening either. The Kronecker construction is the single-model version of what I am proposing one level up: "Gu et al. make every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator, and the beta-pricing derivation is a principled reason to do it. That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound." That matters because it means the idea that a signal's value varies with market state is not something I have to argue for from scratch - it is derivable from E_t(r_{i,t+1}) = beta'_{i,t} lambda_t with beta_{i,t} = theta_1 c_{i,t} and lambda_t = theta_2 x_t, and it is the standard specification in the most-cited paper in the area.
+Then the line. Three differences separate their construction from mine, and all three are in w(i,t) = f(L_t, V_t, P_t, C_{i,t}): their interaction weights are estimated once per annual refit, so they do not vary with measured market state at decision time, only with the value of the macro variable plugged into a fixed coefficient; they are a function of macro variables rather than of any measured reliability of the signal, so there is no C_{i,t} analogue anywhere in the model; and no channel can go absent, "because a missing characteristic is median-imputed rather than down-weighted". The note puts the whole claim on that last point: "The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line." Median imputation is the exact anti-pattern my abstention channel exists to replace - it substitutes a plausible value for a missing one and the downstream model cannot tell the difference, whereas abstention makes absence visible to the aggregator.
+It also supplies the evidence base for two of the four conditioning terms. Liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) and risk (total volatility, idiosyncratic volatility, beta, beta squared) are two of the three dominant families across every one of eleven method families on a ~30,000-stock, 60-year panel. "That is a far larger evidence base for those two conditioning inputs than the CSE-specific work in [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] or the Granger result at p = 0.0041 from volume to ASPI, and it composes with both." The macro rejection also survives: market-level stock variance is given little weight by any method and essentially none by the networks, consistent with the thin ARDL result in [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]] that already got the macro block rejected. The one live challenge is aggregate book-to-market - critical for every model, 28.57% for NN1 and 43.46% for GLM - and the honest response recorded in the note is to "test it against an ASPI-level valuation ratio rather than dismiss it on the strength of a rejection aimed at different variables."
+One further point that bears directly on the main gap and that the paper declined to test: Figure 3 shows model complexity drifting across the test period - elastic net selecting fewer than five features in the first decade and 20 to 40 after 2000, GBRT moving from roughly 20 features to 30 - and the authors explain it by a growing cross section and improving data coverage. "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." So the paper leaves my central hypothesis open on evidence it had in hand, which is a better position for me than either confirming or refuting it would have been.
+EFFECT ON SUB-GAP 1: This is the strongest available illustration of why cost belongs inside the objective rather than after it, and I would cite it as the reference case. "A strategy turning over 113% of its book monthly, concentrated in price-trend signals, on a universe that deliberately includes the smallest and least liquid names, reported at Sharpe 2.35 with no cost deduction and no participation-rate analysis, is the reference case for my cost sub-gap." Two details make it sharper than a generic "they ignored costs" complaint. First, the value-weighted collapse - NN3 from 2.32 to 1.25, OLS-3 from 0.89 to 0.27 - "is itself a partial, unacknowledged cost estimate and I should cite it that way": moving weight away from the small end halves the Sharpe before a single basis point of spread is charged, which is a lower bound on what liquidity is doing to the result. Second, the internal tension: the paper offers the top-1,000 R^2 of 0.72% against 0.46% on the bottom 1,000 as reassurance that the result is not driven by small-cap illiquidity, while the headline economic result is an equal-weighted spread over the whole board - "both cannot be load-bearing at once."
+Applied to the CSE this is not implementable at any size. "On the CSE, where Dissanayake and Nanayakkara find unexpected illiquidity shocks depressing returns by -0.084 to -0.097 and small caps more than large, that turnover is not implementable at any size, which is the concrete argument for sweeping participation rate against daily volume rather than charging a flat spread, as [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] both do in their different ways." So the paper does not close any part of Sub-gap 1 - it has no friction model at all - but it supplies the clearest demonstration of the failure the sub-gap names, from a source that is hard to dismiss.
+EFFECT ON SUB-GAP 2: Limited, and I should not overclaim it. The paper has no volatility process, no persistence estimate, no decay schedule and no volatility targeting; volatility enters only as a cross-sectional predictor. So it neither closes nor narrows Sub-gap 2. What it contributes is one piece of supporting evidence and one adjacent warning. The evidence: the risk family (total volatility, idiosyncratic volatility, beta, beta squared) is one of the three dominant predictor families across all eleven methods, and the GBRT/NN3 marginal relationship is economically large - a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return - which supports keeping V_t in the conditioning set but says nothing about P_t. The warning is the complexity-drift result again: the paper observed a time-varying structure in its own fitted models and explained it away rather than testing it, which is the same category of move as assuming a fixed exponential decay rate and never checking.
+CSE DATA EVIDENCE: None in the paper - US only. The CSE content in this cell is my own transfer accounting. My confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information" than 30,000 stocks over 60 years with 920 features. The direct consequence is a leakage tripwire: "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result", which composes with the 0.54-0.58 directional-accuracy band and the 54.3% out-of-sample figure from the two other notes into "a defensible prior rather than one paper's number". The second consequence is the architecture ceiling: if three hidden layers is already past the optimum on sixty years of US monthly data, one or two layers or a regularized tree ensemble is the ceiling on 374 trading days. The third is that the benchmark choice has to be stated every time, because "the three-percentage-point inflation from benchmarking against the historical mean is larger than any effect I am likely to measure, so a CSE result reported without naming its benchmark is uninterpretable." And the fourth is the frontier-market reading of their own size result: machine learning works least well in the conditions the CSE presents continuously.
 PROPOSED REVISION STATED IN THE NOTE:
 1. Reset the expectation band for A_T to a few tenths of a percent of monthly stock-level R^2 and treat anything materially above it as a leakage signal rather than a result.
 2. Size A_T at NN1 or NN2 scale (one or two hidden layers) or a regularized tree ensemble; drop the depth sweep; keep the feature count small, since every method in the paper selected far fewer features than it was offered.
 3. Adopt the Huber objective as a default across the technical agent, not as a refinement.
-4. Write down the publication-lag structure for A_F before touching any filing data — monthly delayed one month, quarterly four, annual six — because "CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."
-5. Copy the evaluation protocol in full: recursive expanding training window, fixed-size rolling validation, annual refit, no cross-validation, modified Diebold-Mariano on cross-sectionally averaged error differences with Newey-West standard errors, R^2_oos benchmarked against zero with the choice named explicitly every time, and the Campbell-Thompson mapping SR* = sqrt((SR^2 + R^2)/(1 - R^2)) reported alongside — with its costless-timing caveat flagged on a thin book.
+4. Write down the publication-lag structure for A_F before touching any filing data - monthly delayed one month, quarterly four, annual six - because "CSE annual reports arrive late and irregularly and a look-ahead bias here would be invisible and fatal."
+5. Copy the evaluation protocol in full: recursive expanding training window, fixed-size rolling validation, annual refit, no cross-validation, modified Diebold-Mariano on cross-sectionally averaged error differences with Newey-West standard errors, R^2_oos benchmarked against zero with the choice named explicitly every time, and the Campbell-Thompson mapping SR* = sqrt((SR^2 + R^2)/(1 - R^2)) reported alongside - with its costless-timing caveat flagged on a thin book.
 6. Give A_F a low baseline weight with an explicit abstention path rather than a weight that happens to fall to zero: "the fundamental agent is not a timing input and should not be asked for one, it is a slow-moving tilt whose natural horizon is quarters, and an orchestrator that weights it on a daily decision will be weighting noise most of the time", combined with the working assumption that the channel is unusable more than half the time on the CSE.
 7. Test aggregate book-to-market against an ASPI-level valuation ratio rather than dismissing it under the existing macro rejection.
 8. Sweep participation rate against daily volume rather than charging a flat spread, and cite the value-weighted Sharpe collapse (2.32 to 1.25 for NN3, 0.89 to 0.27 for OLS-3) as a partial, unacknowledged cost estimate when making the case.
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>2025.</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>The paper asks "whether five firm-specific accounting ratios, return on equity, dividend per share, earnings per share, the price to earnings ratio and debt to total assets, explain the share prices of Diversified Financial companies listed on the Colombo Stock Exchange". The gap it claims is threefold in my note. First, "the firm-specific determinants literature is developed-market and the Sri Lankan slice of it is thin and dated" — the authors anchor on Kumar (2017) for Indian autos, Nasif and Sharif (2010) for Amman commercial banks, Iqbal et al. (2016) for Kenyan energy and Sharif et al. (2014) for Bahrain, and cite Dissanayake and Herath (2016) and Pandigamage and Ranaweera (2023) as "near enough the whole local set". Second, and this is what I recorded as "their sharpest framing point", the only prior study of firm-specific factors on CSE diversified financials is a 2016 Central Bank staff study reporting percentage increments only, and "its results may no longer hold after the political and economic changes from 2020". I added my own qualification there: "I'd put this more strongly than they do, since their own sample runs straight through the same break and is estimated as one pooled regime." Third, the sector choice is a sampling rationale rather than a hypothesis — "Diversified Financials is picked for growth, not for theory", justified by earnings growing 43% and revenues 31% annually over 2021 to 2023 and the sector being roughly 20% of total market capitalisation per the Central Bank's 2023 industry analysis, which "means the sector was selected on the outcome variable's recent behaviour".</t>
+          <t>The paper asks "whether five firm-specific accounting ratios, return on equity, dividend per share, earnings per share, the price to earnings ratio and debt to total assets, explain the share prices of Diversified Financial companies listed on the Colombo Stock Exchange". The gap it claims is threefold in my note. First, "the firm-specific determinants literature is developed-market and the Sri Lankan slice of it is thin and dated" - the authors anchor on Kumar (2017) for Indian autos, Nasif and Sharif (2010) for Amman commercial banks, Iqbal et al. (2016) for Kenyan energy and Sharif et al. (2014) for Bahrain, and cite Dissanayake and Herath (2016) and Pandigamage and Ranaweera (2023) as "near enough the whole local set". Second, and this is what I recorded as "their sharpest framing point", the only prior study of firm-specific factors on CSE diversified financials is a 2016 Central Bank staff study reporting percentage increments only, and "its results may no longer hold after the political and economic changes from 2020". I added my own qualification there: "I'd put this more strongly than they do, since their own sample runs straight through the same break and is estimated as one pooled regime." Third, the sector choice is a sampling rationale rather than a hypothesis - "Diversified Financials is picked for growth, not for theory", justified by earnings growing 43% and revenues 31% annually over 2021 to 2023 and the sector being roughly 20% of total market capitalisation per the Central Bank's 2023 industry analysis, which "means the sector was selected on the outcome variable's recent behaviour".</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
@@ -8068,8 +8068,8 @@
       </c>
       <c r="J58" s="11" t="inlineStr">
         <is>
-          <t>Annual accounting data from filings plus monthly-averaged price. Dependent variable: share price measured as the average share price of the month, in nominal rupees, undifferenced and untransformed. Regressors: return on equity (net income over average shareholders' equity), dividend per share (annual dividend over the weighted average share count), earnings per share (net profit over the same denominator), price to earnings (market value per share over earnings per share), debt to total assets (total liabilities over total assets). Sole control: firm size as the natural logarithm of total assets — "the only variable entering in logs". The operationalisation table sources each measure to prior local work: Biyiri and Dissanayaka (2017), Irsath et al. (2015), Sritharan (2018) and Rajapaksha and Weerawickrama (2020).
-Descriptives (these are the distributional facts I care about): share price mean 262.078, standard deviation 458.181, range Rs. 0.50 to Rs. 1,950 — "the dependent variable is in nominal rupee levels and is dominated by a handful of high-priced counters". Price to earnings is worse: "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82", which I read as "what happens when a ratio with earnings in the denominator is computed on firm-years where earnings are near zero or negative, and the EPS minimum of −21.65 confirms loss-making years are in the sample". Neither variable is winsorised, trimmed or transformed. EPS mean 17.239, standard deviation 53.818; DPS mean 4.66; ROE mean 14.237%; DTA mean 57.277%; log total assets 20.041.
+          <t>Annual accounting data from filings plus monthly-averaged price. Dependent variable: share price measured as the average share price of the month, in nominal rupees, undifferenced and untransformed. Regressors: return on equity (net income over average shareholders' equity), dividend per share (annual dividend over the weighted average share count), earnings per share (net profit over the same denominator), price to earnings (market value per share over earnings per share), debt to total assets (total liabilities over total assets). Sole control: firm size as the natural logarithm of total assets - "the only variable entering in logs". The operationalisation table sources each measure to prior local work: Biyiri and Dissanayaka (2017), Irsath et al. (2015), Sritharan (2018) and Rajapaksha and Weerawickrama (2020).
+Descriptives (these are the distributional facts I care about): share price mean 262.078, standard deviation 458.181, range Rs. 0.50 to Rs. 1,950 - "the dependent variable is in nominal rupee levels and is dominated by a handful of high-priced counters". Price to earnings is worse: "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82", which I read as "what happens when a ratio with earnings in the denominator is computed on firm-years where earnings are near zero or negative, and the EPS minimum of −21.65 confirms loss-making years are in the sample". Neither variable is winsorised, trimmed or transformed. EPS mean 17.239, standard deviation 53.818; DPS mean 4.66; ROE mean 14.237%; DTA mean 57.277%; log total assets 20.041.
 Correlations with price: DPS 0.535, EPS 0.509, PE 0.319, DTA −0.502, firm size −0.404, ROE −0.160. Among regressors: "dividend per share and earnings per share correlate at 0.757 and debt to assets correlates with firm size at 0.726", which I noted is "the structure that decides how the insignificant coefficients below should be read". Mean VIF 2.23, maximum 2.81, "and the paper treats that as settling the question".</t>
         </is>
       </c>
@@ -8089,12 +8089,12 @@
       </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — this is a single-equation panel econometrics paper with no agents, no orchestration and no decision layer. As I put it in the note, "there is no forecast, no holdout and no agent anywhere in it, and I'm reading it the same way I read the other local empirical work, as evidence about what the fundamental channel on this market can and cannot carry." What it supplies instead is (a) a measured, published feature set for A_F on this exact market and sector, (b) the within-vs-between split that tells me what role A_F should play in the weighting function, and (c) a weak but real published baseline for the fundamental channel.</t>
+          <t>Not applicable - this is a single-equation panel econometrics paper with no agents, no orchestration and no decision layer. As I put it in the note, "there is no forecast, no holdout and no agent anywhere in it, and I'm reading it the same way I read the other local empirical work, as evidence about what the fundamental channel on this market can and cannot carry." What it supplies instead is (a) a measured, published feature set for A_F on this exact market and sector, (b) the within-vs-between split that tells me what role A_F should play in the weighting function, and (c) a weak but real published baseline for the fundamental channel.</t>
         </is>
       </c>
       <c r="M58" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note. (The paper is an accounting-ratio panel regression; no sentiment variable appears anywhere in my note.)</t>
+          <t>None. (The paper is an accounting-ratio panel regression; no sentiment variable appears anywhere in my note.)</t>
         </is>
       </c>
       <c r="N58" s="11" t="inlineStr">
@@ -8106,12 +8106,12 @@
       </c>
       <c r="O58" s="11" t="inlineStr">
         <is>
-          <t>No volatility modelling of any kind — there is no variance model, no GARCH, no risk measure in the specification. The only risk content is interpretive: the authors read the negative debt-to-assets coefficient "as investors discounting financial risk". The regime instability content is relevant to V_t and P_t indirectly: the window "contains the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation peaking above 50%, and the dependent variable is an unadjusted nominal price with no year effects, no inflation adjustment and no regime split."</t>
+          <t>No volatility modelling of any kind - there is no variance model, no GARCH, no risk measure in the specification. The only risk content is interpretive: the authors read the negative debt-to-assets coefficient "as investors discounting financial risk". The regime instability content is relevant to V_t and P_t indirectly: the window "contains the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation peaking above 50%, and the dependent variable is an unadjusted nominal price with no year effects, no inflation adjustment and no regime split."</t>
         </is>
       </c>
       <c r="P58" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note — there is no liquidity variable, no turnover screen, no trading-frequency filter and no transaction cost anywhere in this paper. The closest adjacent fact is the sample construction: the 20 largest of 43 sector firms by terminal market capitalisation, LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b, which is implicitly a size-and-prominence selection and is why the survivorship point below matters.</t>
+          <t>None - there is no liquidity variable, no turnover screen, no trading-frequency filter and no transaction cost anywhere in this paper. The closest adjacent fact is the sample construction: the 20 largest of 43 sector firms by terminal market capitalisation, LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b, which is implicitly a size-and-prominence selection and is why the survivorship point below matters.</t>
         </is>
       </c>
       <c r="Q58" s="11" t="inlineStr">
@@ -8127,8 +8127,8 @@
       <c r="S58" s="11" t="inlineStr">
         <is>
           <t>1. EPS is the strongest and most robust result: 1.887, standard error 0.501, t = 3.76, p = 0.000. "It is the only regressor whose univariate correlation with price (0.509), significance and sign all point the same way." But the magnitude is odd: "That is an implied marginal multiple of 1.887 against a sample where mean price over mean EPS is about 15.2", so "the levels regression is attributing almost all of the cross-sectional price level to something other than earnings, and reading the coefficient as a valuation multiple would understate the market's actual pricing by an order of magnitude."
-2. Debt to total assets is negative and significant at −0.530, standard error 0.167, p = 0.002 — one percentage point more leverage associates with Rs. 0.53 less price. Hedge carried through: DTA correlates 0.726 with firm size, firm size enters at −1.136 and is insignificant at p = 0.262, and both have sizeable negative univariate correlations with price (−0.502 and −0.404), so "the leverage coefficient and the size coefficient are competing to explain the same cross-sectional variation and the design has no way to separate them."
-3. Price to earnings is positive and significant at 0.673, p = 0.022, and "it is the one I would not cite" — given the identity and a regressor standard deviation of 1069.92, "I read this as a mechanical artefact rather than evidence about valuation multiples, and the fact that it reaches significance while dividend per share does not is a feature of the arithmetic rather than of the market."
+2. Debt to total assets is negative and significant at −0.530, standard error 0.167, p = 0.002 - one percentage point more leverage associates with Rs. 0.53 less price. Hedge carried through: DTA correlates 0.726 with firm size, firm size enters at −1.136 and is insignificant at p = 0.262, and both have sizeable negative univariate correlations with price (−0.502 and −0.404), so "the leverage coefficient and the size coefficient are competing to explain the same cross-sectional variation and the design has no way to separate them."
+3. Price to earnings is positive and significant at 0.673, p = 0.022, and "it is the one I would not cite" - given the identity and a regressor standard deviation of 1069.92, "I read this as a mechanical artefact rather than evidence about valuation multiples, and the fact that it reaches significance while dividend per share does not is a feature of the arithmetic rather than of the market."
 4. ROE (−0.142, p = 0.575) and DPS (2.102, p = 0.248) both fail; H1 and H2 are rejected "after a literature review spending four subsections on bird-in-hand, residual dividend policy, agency cost theory and dividend irrelevance". Important hedge: DPS has the highest univariate correlation with price in the whole matrix at 0.535 and correlates 0.757 with EPS, so "what the regression shows is that dividends add nothing beyond earnings in this specification, not that dividends are unrelated to price. The conclusion states the second."
 5. The fit split is the headline for me: "Nine percent of the year-to-year movement in a given company's share price is explained, against seventy-one percent of the differences between companies", so "the model is a cross-sectional pricing description that has very little to say about time."</t>
         </is>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="U58" s="11" t="inlineStr">
         <is>
-          <t>- A measured, citable feature set for A_F on CSE: EPS and debt-to-assets as the two that clear at p = 0.000 and p = 0.002, with firm size as a control, all extractable from income statement and balance sheet alone — scoped explicitly to the cross-section.
+          <t>- A measured, citable feature set for A_F on CSE: EPS and debt-to-assets as the two that clear at p = 0.000 and p = 0.002, with firm size as a control, all extractable from income statement and balance sheet alone - scoped explicitly to the cross-section.
 - The within R² of 0.090 against between R² of 0.709 as the number that fixes A_F's architectural role: "Fundamentals on this market separate counters from each other far better than they explain any one counter's path, so the fundamental channel should produce a slowly-updating relative view across the universe rather than a timing signal, with the technical channel carrying the short horizon and the orchestrator capping how much the fundamental weight is allowed to move between reporting dates."
 - A hard constraint on feature construction: exclude price-derived multiples from A_F, or build them against a lagged price and say so.
 - Point-in-time universe construction as a non-negotiable, with this paper as the worked counter-example.
@@ -8164,21 +8164,21 @@
       </c>
       <c r="W58" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: A_F (the fundamental agent) — feature selection, update frequency and architectural role; the abstention channel; universe construction and point-in-time screening; and the local-evidence justification for using the CSE. It is the most recent published statement I have of which accounting ratios associate with price on CSE financials, over a window that overlaps mine almost exactly.
-EFFECT ON MAIN GAP: Strongly supportive, and in a very specific way. The within/between split — 0.090 within against 0.709 between — is a direct, locally measured statement that the fundamental channel's reliability is horizon-dependent on this market: it prices counters against each other well and says almost nothing about when a given counter moves. That is precisely the kind of structural property the weighting function w(i,t) = f(L_t, V_t, P_t, C_i,t) is meant to exploit, and it gives me a published, CSE-specific number for why the fundamental agent's weight should be capped and slow-moving between reporting dates rather than allowed to drive entry and exit. It also supports the C_i,t component being a structural property of the output rather than a self-report: ROE and DPS fail to clear not because they are irrelevant but because they are collinear with EPS (DPS–EPS at 0.757), so a channel whose inputs are collinear or missing should be detectable from the structure of its inputs and allowed to abstain. "Letting the channel return no view when its inputs are collinear or missing is the design consequence, and it is the same abstention argument the liquidity screen produces for the technical channel." Finally, the paper's pooling of eleven years containing a currency collapse as one regime is my clearest local illustration of what a fixed, non-state-conditional combination rule costs: "This is now the third CSE result pointing the same way, alongside the macro linkages breaking over 2014 to 2022 in [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] and the 2021 extension halving the investment-risk coefficient in the Fernando note."
-EFFECT ON SUB-GAP 1: Indirect and mostly cautionary. The paper has no liquidity variable, no turnover screen and no execution cost, so it offers no positive evidence on state-dependent execution friction. What it does supply is the mechanism by which thin trading corrupts a price-derived fundamental input: "on a thin market where the denominator goes near zero it also carries a variance of the kind that produced a standard deviation of 1069.92 here." That is the PE ratio blowing up to a range of −1471.22 to 2292.82 because earnings pass through zero, and it is a concrete local instance of the broader claim in SUB-GAP 1 that market conditions condition the reliability of price-derived quantities. It also gives me a worked example of a universe screen done wrong — top-20 by terminal capitalisation backfilled to 2013 — which is "the exact failure my own screen could reproduce if the liquidity filter is computed once over the full history rather than as of each rebalance date."
-EFFECT ON SUB-GAP 2: Indirect. There is no volatility persistence content in this paper — no variance model, no long-memory estimate. The only contribution is negative evidence about regime stability: eleven years pooled across the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation above 50%, with no year effects and no regime split, producing coefficients that partly fit a changing unit of measurement. That is an argument for conditioning on measured state, but it does not operationalise persistence, which remains mine to do.
+          <t>SPEAKS TO: A_F (the fundamental agent) - feature selection, update frequency and architectural role; the abstention channel; universe construction and point-in-time screening; and the local-evidence justification for using the CSE. It is the most recent published statement I have of which accounting ratios associate with price on CSE financials, over a window that overlaps mine almost exactly.
+EFFECT ON MAIN GAP: Strongly supportive, and in a very specific way. The within/between split - 0.090 within against 0.709 between - is a direct, locally measured statement that the fundamental channel's reliability is horizon-dependent on this market: it prices counters against each other well and says almost nothing about when a given counter moves. That is precisely the kind of structural property the weighting function w(i,t) = f(L_t, V_t, P_t, C_i,t) is meant to exploit, and it gives me a published, CSE-specific number for why the fundamental agent's weight should be capped and slow-moving between reporting dates rather than allowed to drive entry and exit. It also supports the C_i,t component being a structural property of the output rather than a self-report: ROE and DPS fail to clear not because they are irrelevant but because they are collinear with EPS (DPS-EPS at 0.757), so a channel whose inputs are collinear or missing should be detectable from the structure of its inputs and allowed to abstain. "Letting the channel return no view when its inputs are collinear or missing is the design consequence, and it is the same abstention argument the liquidity screen produces for the technical channel." Finally, the paper's pooling of eleven years containing a currency collapse as one regime is my clearest local illustration of what a fixed, non-state-conditional combination rule costs: "This is now the third CSE result pointing the same way, alongside the macro linkages breaking over 2014 to 2022 in [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] and the 2021 extension halving the investment-risk coefficient in the Fernando note."
+EFFECT ON SUB-GAP 1: Indirect and mostly cautionary. The paper has no liquidity variable, no turnover screen and no execution cost, so it offers no positive evidence on state-dependent execution friction. What it does supply is the mechanism by which thin trading corrupts a price-derived fundamental input: "on a thin market where the denominator goes near zero it also carries a variance of the kind that produced a standard deviation of 1069.92 here." That is the PE ratio blowing up to a range of −1471.22 to 2292.82 because earnings pass through zero, and it is a concrete local instance of the broader claim in SUB-GAP 1 that market conditions condition the reliability of price-derived quantities. It also gives me a worked example of a universe screen done wrong - top-20 by terminal capitalisation backfilled to 2013 - which is "the exact failure my own screen could reproduce if the liquidity filter is computed once over the full history rather than as of each rebalance date."
+EFFECT ON SUB-GAP 2: Indirect. There is no volatility persistence content in this paper - no variance model, no long-memory estimate. The only contribution is negative evidence about regime stability: eleven years pooled across the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation above 50%, with no year effects and no regime split, producing coefficients that partly fit a changing unit of measurement. That is an argument for conditioning on measured state, but it does not operationalise persistence, which remains mine to do.
 CSE DATA EVIDENCE: This is the richest part of the row for the justification rewrite, and it is all local and measured.
-- Universe depth and concentration: the Diversified Financials sector has 43 listed firms, of which the study could only work with the top 20 by capitalisation, spanning LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b — a roughly 60-fold spread in capitalisation inside a single sector of a single market. That is firm heterogeneity on this market stated in rupees.
+- Universe depth and concentration: the Diversified Financials sector has 43 listed firms, of which the study could only work with the top 20 by capitalisation, spanning LOLC Holdings at LKR 203.3b down to Alliance Finance at LKR 3.3b - a roughly 60-fold spread in capitalisation inside a single sector of a single market. That is firm heterogeneity on this market stated in rupees.
 - Price-level heterogeneity: share price mean 262.078 against a standard deviation of 458.181, range Rs. 0.50 to Rs. 1,950, with the dependent variable "dominated by a handful of high-priced counters". A standard deviation 1.75 times the mean inside one sector is a quantified statement of cross-sectional dispersion.
-- Earnings heterogeneity and loss-making counters: EPS mean 17.239 with a standard deviation of 53.818 and a minimum of −21.65 — loss-making firm-years are present in the sample. This is why the PE ratio has "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82". That dispersion is the direct, local, empirical reason a price-derived multiple is not a safe input on this market.
+- Earnings heterogeneity and loss-making counters: EPS mean 17.239 with a standard deviation of 53.818 and a minimum of −21.65 - loss-making firm-years are present in the sample. This is why the PE ratio has "a mean of −20.048 with a standard deviation of 1069.92 and a range from −1471.22 to 2292.82". That dispersion is the direct, local, empirical reason a price-derived multiple is not a safe input on this market.
 - Leverage: debt to total assets averages 57.277% across the sector, and one percentage point more leverage associates with Rs. 0.53 less price (p = 0.002).
 - Which fundamentals transmit to price here: EPS at 1.887 (p = 0.000) and leverage at −0.530 (p = 0.002) clear; ROE (p = 0.575) and DPS (p = 0.248) do not, with DPS's failure attributable to its 0.757 correlation with EPS rather than to irrelevance. Firm size enters negatively at −1.136 but is insignificant (p = 0.262), and its 0.726 correlation with leverage means the design cannot separate the two.
 - Transmission is cross-sectional, not temporal: R² within 0.090 against R² between 0.709. Fundamentals explain roughly nine percent of a given CSE counter's year-to-year price movement and roughly seventy-one percent of the differences between counters.
-- Fundamental data cost and update frequency: six variables for 200 firm-years were hand-collected from the CSE website and company annual reports by two authors with institutional access. Fundamentals on this market update at annual reporting frequency and are extracted from PDF filings by hand in the published literature — "it is why the retrieval pipeline over CSE filings is the component I expect to be the bottleneck rather than any model."
+- Fundamental data cost and update frequency: six variables for 200 firm-years were hand-collected from the CSE website and company annual reports by two authors with institutional access. Fundamentals on this market update at annual reporting frequency and are extracted from PDF filings by hand in the published literature - "it is why the retrieval pipeline over CSE filings is the component I expect to be the bottleneck rather than any model."
 - Regime instability in local fundamentals: "The window contains the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation peaking above 50%." The authors themselves argue that pre-2020 results "may no longer hold after the political and economic changes from 2020". This is local evidence that CSE relationships are not stationary across my own index track of 1 July 2014 to 30 June 2024.
 - Methodological fragility of the local literature as a whole: a 2025 journal paper in this space carries a Hausman statistic of −1489.934, a normality section contradicting its own table, two tables whose dependent-variable moments cannot be reconciled (mean 83.107 / sd 63.883 against mean 262.078 / sd 458.181), and forecasting recommendations with no holdout anywhere. I recorded explicitly that the absent out-of-sample evaluation "is the standard shape of the local empirical literature". I have not found that evaluation in the literature I have covered.
-PROPOSED REVISION STATED IN THE NOTE: The note states several design revisions driven by this paper. (1) A_F is to produce "a slowly-updating relative view across the universe rather than a timing signal", with the technical channel carrying the short horizon and "the orchestrator capping how much the fundamental weight is allowed to move between reporting dates". (2) A_F's inputs are "restricted to quantities computed from the filings alone, with price-derived multiples either excluded or constructed against a lagged price and reported as such". (3) The liquidity screen and universe construction must be computed "as of each rebalance date" and not once over the full history; the note records that "Taken with the delisting control in [[Relationship between firm-level investment, idiosyncratic risk and ownership, an emerging market perspective]], which does retain delisted firms, I now have both the right and the wrong version of this decision documented on the same market." (4) Targets should be returns and features should be deflated or expressed as ratios, "not merely to add controls", because of the nominal-price problem across 2020 to 2023. (5) A_F gets an abstention output rather than being forced to emit a directional view on every counter at every step. (6) The paper is adopted as "a usable published baseline for the fundamental channel, and a weak one, which is what makes it useful" — an in-sample overall R² of 0.576 and within R² of 0.090 to be beaten out of sample on a comparable universe.</t>
+PROPOSED REVISION STATED IN THE NOTE: The note states several design revisions driven by this paper. (1) A_F is to produce "a slowly-updating relative view across the universe rather than a timing signal", with the technical channel carrying the short horizon and "the orchestrator capping how much the fundamental weight is allowed to move between reporting dates". (2) A_F's inputs are "restricted to quantities computed from the filings alone, with price-derived multiples either excluded or constructed against a lagged price and reported as such". (3) The liquidity screen and universe construction must be computed "as of each rebalance date" and not once over the full history; the note records that "Taken with the delisting control in [[Relationship between firm-level investment, idiosyncratic risk and ownership, an emerging market perspective]], which does retain delisted firms, I now have both the right and the wrong version of this decision documented on the same market." (4) Targets should be returns and features should be deflated or expressed as ratios, "not merely to add controls", because of the nominal-price problem across 2020 to 2023. (5) A_F gets an abstention output rather than being forced to emit a directional view on every counter at every step. (6) The paper is adopted as "a usable published baseline for the fundamental channel, and a weak one, which is what makes it useful" - an in-sample overall R² of 0.576 and within R² of 0.090 to be beaten out of sample on a comparable universe.</t>
         </is>
       </c>
       <c r="X58" s="11" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>2026.</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="G59" s="11" t="inlineStr">
         <is>
-          <t>The paper asks "whether firms listed on the Colombo Stock Exchange cut capital investment when their idiosyncratic risk rises, and whether insider and institutional ownership moderate that sensitivity". The gap it addresses, as I recorded it: (1) "The investment-risk sensitivity literature is almost entirely developed-market" — Panousi and Papanikolaou (2012) in the Journal of Finance is the anchor (risk-averse managers underinvest when firm-specific risk rises), with follow-on work (Glover and Levine, 2017; Liu and Wang, 2021; Florackis et al., 2019) staying in US and UK data; "The authors' claim is not that the mechanism is absent elsewhere, it's that the sign of the ownership moderation has no reason to carry over, because the agency environment that produces it is different." (2) "The alignment against entrenchment question is genuinely open in emerging markets" — higher insider ownership can tie managerial wealth to firm growth and push toward long-horizon investment (alignment, Ang et al., 2000) or concentrate undiversified personal wealth and raise risk aversion (entrenchment, Fahlenbrach and Stulz, 2009); the paper argues weaker legal protection and weaker formal governance in emerging markets (La Porta et al., 1998; Khanna and Palepu, 2002) raise the marginal value of insider ownership as a substitute governance mechanism, tilting toward alignment. "That is a testable framing and it is the paper's actual contribution." (3) The authors claim coverage of this relationship in South Asia, "which I can't independently verify but which is consistent with what I found when I went looking for CSE firm-level risk studies."</t>
+          <t>The paper asks "whether firms listed on the Colombo Stock Exchange cut capital investment when their idiosyncratic risk rises, and whether insider and institutional ownership moderate that sensitivity". The gap it addresses, as I recorded it: (1) "The investment-risk sensitivity literature is almost entirely developed-market" - Panousi and Papanikolaou (2012) in the Journal of Finance is the anchor (risk-averse managers underinvest when firm-specific risk rises), with follow-on work (Glover and Levine, 2017; Liu and Wang, 2021; Florackis et al., 2019) staying in US and UK data; "The authors' claim is not that the mechanism is absent elsewhere, it's that the sign of the ownership moderation has no reason to carry over, because the agency environment that produces it is different." (2) "The alignment against entrenchment question is genuinely open in emerging markets" - higher insider ownership can tie managerial wealth to firm growth and push toward long-horizon investment (alignment, Ang et al., 2000) or concentrate undiversified personal wealth and raise risk aversion (entrenchment, Fahlenbrach and Stulz, 2009); the paper argues weaker legal protection and weaker formal governance in emerging markets (La Porta et al., 1998; Khanna and Palepu, 2002) raise the marginal value of insider ownership as a substitute governance mechanism, tilting toward alignment. "That is a testable framing and it is the paper's actual contribution." (3) The authors claim coverage of this relationship in South Asia, "which I can't independently verify but which is consistent with what I found when I went looking for CSE firm-level risk studies."</t>
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr">
@@ -8236,8 +8236,8 @@
       <c r="J59" s="11" t="inlineStr">
         <is>
           <t>Annual accounting data plus weekly price series. "All accounting and insider ownership data is hand-collected from annual reports published by the CSE", prices and the index come from the CSE data libraries, and Treasury bill rates from the Central Bank of Sri Lanka.
-Idiosyncratic risk is built as the residual standard deviation from a Fama–French three-factor regression on weekly excess returns over 52 trading weeks:
-r_{i,t} − r_{f,t} = α_i + β_i^MKT MKT_t + β_i^SMB SMB_t + β_i^HML HML_t + ε_{i,t},   σ_i^idi = sd(ε̂_{i,t})_{t=1..52}
+Idiosyncratic risk is built as the residual standard deviation from a Fama-French three-factor regression on weekly excess returns over 52 trading weeks:
+r_{i,t} − r_{f,t} = α_i + β_i^MKT MKT_t + β_i^SMB SMB_t + β_i^HML HML_t + ε_{i,t}, σ_i^idi = sd(ε̂_{i,t})_{t=1..52}
 where r_{i,t} is the weekly return adjusted for cash dividends, stock splits, scrip dividends, bonus issues and rights issues; the market proxy is "the percentage change in the All Share Total Return Index (ASTRI), not the ASPI, which is the right choice since it is total return rather than price only"; r_{f,t} is a weekly rate derived from the yield on 91-day Treasury bills; and "weekly returns exceeding +50% or falling below −50% are dropped as outliers, following Abeysekera and Nimal (2017)".
 Systematic risk is backed out of the decomposition rather than estimated separately: σ^sys = sqrt(σ^tot² − σ^idi²), with total risk the standard deviation of weekly returns.
 Ownership: insider ownership is the share of total outstanding shares held by executive directors on the board at year end; institutional ownership is the share held by pension funds, investment banks, mutual funds and companies holding more than 3% (both following Farwis and Azeez, 2019). Controls are cash flow over lagged PPE, firm size as the firm's PPE relative to total sample PPE that year, and leverage as total debt over total assets.
@@ -8258,12 +8258,12 @@
       </c>
       <c r="L59" s="11" t="inlineStr">
         <is>
-          <t>Not applicable — this is a corporate finance panel econometrics paper with no agents, no orchestration, no decision layer and no forecast. As I put it: "Nothing in this paper is a methodological template for what I'm building… so I'm reading it as market-structure evidence rather than as a design precedent." What it supplies instead is (a) three conceded facts about CSE data depth that constrain the technical, volatility and fundamental channels respectively, (b) a reusable idiosyncratic risk estimator for A_V's cross-sectional input, and (c) a conditioning design — annual median splits with group-specific slopes — that is "close to the structure I'd want for ablating state inputs one at a time", i.e. a template for ablating L_t, V_t, P_t and C_i,t individually in the orchestrator.</t>
+          <t>Not applicable - this is a corporate finance panel econometrics paper with no agents, no orchestration, no decision layer and no forecast. As I put it: "Nothing in this paper is a methodological template for what I'm building… so I'm reading it as market-structure evidence rather than as a design precedent." What it supplies instead is (a) three conceded facts about CSE data depth that constrain the technical, volatility and fundamental channels respectively, (b) a reusable idiosyncratic risk estimator for A_V's cross-sectional input, and (c) a conditioning design - annual median splits with group-specific slopes - that is "close to the structure I'd want for ablating state inputs one at a time", i.e. a template for ablating L_t, V_t, P_t and C_i,t individually in the orchestrator.</t>
         </is>
       </c>
       <c r="M59" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note. (No sentiment variable appears anywhere in this paper.)</t>
+          <t>None. (No sentiment variable appears anywhere in this paper.)</t>
         </is>
       </c>
       <c r="N59" s="11" t="inlineStr">
@@ -8275,7 +8275,7 @@
       </c>
       <c r="O59" s="11" t="inlineStr">
         <is>
-          <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama–French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
+          <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama-French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
 What I would add: "the non-synchronous trading correction and a reported correlation between the risk estimate and turnover, because if those two move together on my sample then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it."
 Magnitude prior for A_V: "Mean idiosyncratic risk of 0.221 with a standard deviation of 0.050 sets a realistic prior on how much cross-sectional signal the volatility channel can carry. That is a narrow spread, and a one standard deviation move being worth 2.02 percentage points of investment is a real-economy effect rather than a trading one, so I should not expect the cross-sectional volatility ranking on CSE counters to separate firms as cleanly as it does on a US sample."</t>
         </is>
@@ -8290,7 +8290,7 @@
       </c>
       <c r="Q59" s="11" t="inlineStr">
         <is>
-          <t>Not applicable in the ML sense — coefficients and group-specific slopes are the explanation by construction. Figure 1 is the paper's clearest visual statement: "the low-ownership line falls from roughly 0.23 to 0.055 across the plotted range of log lagged idiosyncratic risk while the high-ownership line is flat and very slightly positive." I would note that the paper's headline mechanism is inferred rather than observed — see limitations.</t>
+          <t>Not applicable in the ML sense - coefficients and group-specific slopes are the explanation by construction. Figure 1 is the paper's clearest visual statement: "the low-ownership line falls from roughly 0.23 to 0.055 across the plotted range of log lagged idiosyncratic risk while the high-ownership line is flat and very slightly positive." I would note that the paper's headline mechanism is inferred rather than observed - see limitations.</t>
         </is>
       </c>
       <c r="R59" s="11" t="inlineStr">
@@ -8304,7 +8304,7 @@
           <t>1. Idiosyncratic risk is negatively and significantly related to firm-level investment across every specification: "−0.165* in the year-fixed-effects-only column rising to −0.232* with full controls and firm fixed effects, and −0.199 once a lagged dependent variable is added." Economic size: "a one standard deviation rise in idiosyncratic risk cuts the investment rate by 2.02 percentage points against a sample mean of 11.60%, a 17.48% decline."
 2. "The negative sensitivity is concentrated entirely in low-insider-ownership firms, and that is the opposite of the US result." Risk × low insider dummy is −0.435* with year effects only and −0.599 with the full specification; the high insider dummy interaction "is statistically indistinguishable from zero throughout (0.035, standard error 0.180)". The authors read this as alignment dominating entrenchment, contradicting Panousi and Papanikolaou (2012).
 3. Institutional ownership substitutes for insider alignment: in the 2×2 design "the only significantly negative cell is low institutional combined with low insider ownership, at −0.566* and then −0.985 with full controls, while the high-institutional-low-insider cell is insignificant at −0.392 (standard error 0.276)." My hedge, carried through: "I'd hold it a little more loosely than they do because the insignificance could be power rather than absence given the cell counts."
-4. The extension result, which I rate as the most useful finding in the paper for me: "Extending the sample three years to 2021 weakens the baseline result from −0.232* to −0.123*, and the paper calls this 'largely consistent'." The ownership results survive better — "low insider at −0.407 and low-institutional-low-insider at −0.787, and the high-institutional-low-insider cell now turns significant at −0.433." My reading: "I read the halving of the main coefficient and the loss of two significance stars as the more informative result here, and it is the single most useful thing in the paper for my own period argument." Note the surviving 2021 baseline is significant only at the 10% level (−0.123*).</t>
+4. The extension result, which I rate as the most useful finding in the paper for me: "Extending the sample three years to 2021 weakens the baseline result from −0.232* to −0.123*, and the paper calls this 'largely consistent'." The ownership results survive better - "low insider at −0.407 and low-institutional-low-insider at −0.787, and the high-institutional-low-insider cell now turns significant at −0.433." My reading: "I read the halving of the main coefficient and the loss of two significance stars as the more informative result here, and it is the single most useful thing in the paper for my own period argument." Note the surviving 2021 baseline is significant only at the 10% level (−0.123*).</t>
         </is>
       </c>
       <c r="T59" s="11" t="inlineStr">
@@ -8320,7 +8320,7 @@
       <c r="U59" s="11" t="inlineStr">
         <is>
           <t>- The citation for why A_T cannot assume a daily price series on CSE: a finance journal estimating a factor model on CSE firms moves to weekly because most stocks don't trade daily. "That is a stronger warrant than anything I could get from the ML literature."
-- The idiosyncratic risk estimator for A_V's cross-sectional input — residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free — plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk–turnover correlation).
+- The idiosyncratic risk estimator for A_V's cross-sectional input - residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free - plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk-turnover correlation).
 - A realistic prior on how much cross-sectional signal A_V can carry: mean idiosyncratic risk 0.221, standard deviation only 0.050, range 0.117 to 0.315.
 - A mechanism-level argument for volatility persistence that is independent of the statistical long-memory literature.
 - The free-float fact (66.1% institutional, 5.7% insider) as a calibration input for the execution-cost participation-rate sweep.
@@ -8331,36 +8331,36 @@
       </c>
       <c r="V59" s="11" t="inlineStr">
         <is>
-          <t>- The non-synchronous trading problem is conceded and then left untreated: no Dimson or Scholes–Williams correction, no trading-frequency screen, no check of whether the risk measure correlates with turnover. That correction, and the reported risk–turnover correlation, is work I have to do, and it is exactly the boundary between A_V and A_L.
-- No out-of-sample period, no forecast, no decision objective — so nothing here tells me how a risk estimate should be weighted in a live allocation, only how it relates contemporaneously to corporate investment.
-- No execution cost model, no order size, no depth — the free-float fact implies the friction problem but the paper does not model it.
+          <t>- The non-synchronous trading problem is conceded and then left untreated: no Dimson or Scholes-Williams correction, no trading-frequency screen, no check of whether the risk measure correlates with turnover. That correction, and the reported risk-turnover correlation, is work I have to do, and it is exactly the boundary between A_V and A_L.
+- No out-of-sample period, no forecast, no decision objective - so nothing here tells me how a risk estimate should be weighted in a live allocation, only how it relates contemporaneously to corporate investment.
+- No execution cost model, no order size, no depth - the free-float fact implies the friction problem but the paper does not model it.
 - No persistence modelling. The paper gives a mechanism for slow decay but estimates no persistence parameter, no long-memory d and no regime structure.
 - No state-conditional combination of any channel; the conditioning is on ownership, a firm attribute, not on market state L_t, V_t or P_t.</t>
         </is>
       </c>
       <c r="W59" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk–turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
+          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk-turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
 EFFECT ON MAIN GAP: Strongly supportive on two fronts. First, regime instability: "The 2021 extension weakening the main coefficient from −0.232* to −0.123* is corroboration that CSE relationships estimated pre-2020 do not survive the crisis window intact. Taken with [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] finding the traditional macro linkages broken over 2014 to 2022, that is now two independent CSE results pointing at regime instability across exactly the period a static system would be evaluated on, which is the clearest empirical case I have for an orchestrator that conditions on measured state rather than a fixed combination rule." Note the surviving coefficient is significant only at 10%.
 Second, the C_i,t component and abstention. The frequency concession forces an abstention design on A_T: "It doesn't mean I build at weekly frequency, the index track is liquid enough for daily, it means the per-counter liquidity screen has to come before any cross-sectional feature is computed and counters that fail it have to produce an abstention rather than a stale-price signal. This is the same structural failure [[AlphaAgents, Large Language Model Based Multi-Agents for Equity Portfolio Constructions]] fixed by deleting an agent by hand." And the data-depth fact forces the same on A_F: "it is why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence." Both of these are structural properties of the input and output, not self-reports, which is exactly what C_i,t is meant to be.
 Third, a methodological warning for the state vector itself: if the volatility estimate and the liquidity estimate co-move on my sample, "then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it." That is a concrete pre-registration task for the main gap, and the paper's own −0.703 insider/institutional correlation is the worked example of what unmanaged collinearity does to a conditioning design: "every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one."
 Fourth, Model 2's design is a usable template: "splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it is close to the structure I'd want for ablating state inputs one at a time."
-EFFECT ON SUB-GAP 1: This is the strongest row in the note for state-dependent execution friction and for liquidity conditioning the reliability of price-derived agents. The reliability half is stated by the paper itself: "since most stocks are not traded daily, we use weekly stock returns" — a published finance journal on my exact market changing its estimation frequency because of thin trading. That is local empirical evidence that price-derived quantities on CSE degrade with liquidity, and it is the warrant for L_t conditioning A_T's and A_V's weights rather than being a separate add-on signal. The untreated residual is my opening: stale prices "bias the residual standard deviation downward for exactly the thinnest counters", with no Dimson or Scholes–Williams correction, no trading-frequency screen and no risk–turnover check anywhere in the paper, and "part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant." The execution-cost half comes from the ownership structure: institutional ownership averaging 66.1% against insider 5.7% means "the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding."
+EFFECT ON SUB-GAP 1: This is the strongest row in the note for state-dependent execution friction and for liquidity conditioning the reliability of price-derived agents. The reliability half is stated by the paper itself: "since most stocks are not traded daily, we use weekly stock returns" - a published finance journal on my exact market changing its estimation frequency because of thin trading. That is local empirical evidence that price-derived quantities on CSE degrade with liquidity, and it is the warrant for L_t conditioning A_T's and A_V's weights rather than being a separate add-on signal. The untreated residual is my opening: stale prices "bias the residual standard deviation downward for exactly the thinnest counters", with no Dimson or Scholes-Williams correction, no trading-frequency screen and no risk-turnover check anywhere in the paper, and "part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant." The execution-cost half comes from the ownership structure: institutional ownership averaging 66.1% against insider 5.7% means "the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding."
 EFFECT ON SUB-GAP 2: Supportive at the mechanism level, which is more than a statistical citation gives me. "The investment channel is the mechanism-level argument for pairing forecast variance with persistence rather than treating volatility as a point-in-time cap. If elevated idiosyncratic risk causes firms to cut capital spending by 17.48% of the mean investment rate, then a volatility shock on this market propagates into fundamentals with a lag measured in reporting periods, not days, and the real activity it suppresses takes just as long to come back. That is a fundamental reason to expect slow decay, independent of the statistical long-memory evidence in [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] and [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], and it is a better sentence for the proposal than another citation of a d estimate." The paper itself estimates no persistence parameter, so operationalising P_t remains entirely mine.
 CSE DATA EVIDENCE: This is the single densest source of local empirical evidence I have for the justification rewrite, and the fact that it comes from authors with no stake in making a data-depth argument is what makes it usable.
 - Thin trading, conceded in the data section: "since most stocks are not traded daily, we use weekly stock returns." Three authors with institutional access, publishing in Managerial Finance, could not estimate a factor model at daily frequency on this market. That is direct local evidence of liquidity constraint, and it is stated as a design constraint rather than as a limitation.
-- Heterogeneous trading activity: the ±50% weekly return trim following Abeysekera and Nimal (2017) is itself "a reminder of what the raw series looks like" — a market where weekly moves beyond ±50% occur often enough to need a documented rule.
-- Universe depth: 167 unique firms with usable accounting data, 1,226 firm-years over 2010–2018, after excluding financials, utilities, energy and telecoms, firm-years with missing variables, and negative book values. Ownership data available only from 2011 and only for 59 firms (insider) and 54 firms (institutional) — "usable ownership data exists for roughly a third of the firms that have usable accounting data". After propensity score matching, 64 and 76 observations.
+- Heterogeneous trading activity: the ±50% weekly return trim following Abeysekera and Nimal (2017) is itself "a reminder of what the raw series looks like" - a market where weekly moves beyond ±50% occur often enough to need a documented rule.
+- Universe depth: 167 unique firms with usable accounting data, 1,226 firm-years over 2010–2018, after excluding financials, utilities, energy and telecoms, firm-years with missing variables, and negative book values. Ownership data available only from 2011 and only for 59 firms (insider) and 54 firms (institutional) - "usable ownership data exists for roughly a third of the firms that have usable accounting data". After propensity score matching, 64 and 76 observations.
 - Ownership concentration and free float: mean institutional ownership 66.1%, mean insider ownership 5.7%, correlating at −0.703. "This is a market of institutionally held firms with thin executive stakes." Two thirds of shares in institutional hands is a free-float constraint with a direct depth consequence.
 - Family control: family firms are 33% of firm-years, identified by hand from annual reports and executive biographies following Anderson and Reeb (2003).
-- Idiosyncratic risk levels: mean 0.221, standard deviation 0.050, range 0.117 to 0.315 — "the cross-sectional spread in firm-specific risk on this market is narrow". This is a quantified statement of how much, and how little, firm-level risk varies across CSE counters.
+- Idiosyncratic risk levels: mean 0.221, standard deviation 0.050, range 0.117 to 0.315 - "the cross-sectional spread in firm-specific risk on this market is narrow". This is a quantified statement of how much, and how little, firm-level risk varies across CSE counters.
 - Firm fundamentals respond to firm risk: a one standard deviation rise in idiosyncratic risk cuts the investment rate by 2.02 percentage points against a sample mean of 11.60%, a 17.48% decline. Baseline coefficient −0.232* with full controls and firm fixed effects; −0.199 with a lagged dependent variable.
 - Governance heterogeneity in the transmission: the sensitivity is concentrated entirely in low-insider-ownership firms (−0.599 full specification) while high-insider firms are indistinguishable from zero (0.035, standard error 0.180), and in the 2×2 grid only the low-institutional/low-insider cell is significantly negative (−0.566*, then −0.985 with full controls). Hedge: the insignificant cells may be low power rather than genuine nulls given cell counts and the −0.703 correlation.
 - Regime instability: extending the sample three years to 2021 halves the baseline coefficient from −0.232* to −0.123*, significant only at 10%. The window crosses SLFRS 16 (2019), the Easter attacks and COVID.
-- Documented accounting break: SLFRS 16 changed lease recognition in 2019 and contaminates PPE — a structural break in CSE fundamentals sitting inside my 1 July 2014 to 30 June 2024 index track.
+- Documented accounting break: SLFRS 16 changed lease recognition in 2019 and contaminates PPE - a structural break in CSE fundamentals sitting inside my 1 July 2014 to 30 June 2024 index track.
 - Fundamental extraction cost: all accounting figures, insider stakes, board composition, CEO duality and family-firm status were pulled out of CSE annual report PDFs by hand over nine years, by authors with institutional access and every incentive to keep the sample large.
 - Correct survivorship handling exists in the local literature: "Both listed and delisted firms are retained, which is a deliberate survivorship-bias control and more than most of the local literature does."
-PROPOSED REVISION STATED IN THE NOTE: (1) A per-counter liquidity screen must run before any cross-sectional feature is computed, and counters failing it must emit an abstention rather than a stale-price signal — A_T does not get to assume a daily series on this market. (2) A_V reuses this idiosyncratic risk construction (residual standard deviation from a local factor model over a rolling window, ASTRI market proxy, 91-day Treasury bill risk-free, with Abeysekera and Nimal (2017) as a four-factor local alternative) but adds the non-synchronous trading correction they skip and reports the correlation between the risk estimate and turnover, to establish whether A_V and A_L are partly measuring the same thing before any weighting is set on them. (3) The cross-sectional volatility ranking's expected separating power on CSE counters should be "pinned down on my own data before the agent's influence weight is allowed to swing much on it", given the 0.221/0.050 spread. (4) Any PPE-derived or lease-sensitive fundamental feature must either avoid the affected line items or carry an explicit SLFRS 16 break control, "with the choice stated in the methodology — I'd rather find this now than discover it in an ablation". (5) The execution-cost participation-rate sweep must be calibrated against free float rather than shares outstanding, and this is to be checked on my own data "before setting the sweep range". (6) A_F is designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence. (7) The volatility-persistence argument in the proposal is to be made at the mechanism level — investment suppression propagating through reporting periods — rather than by another citation of a long-memory d estimate.</t>
+PROPOSED REVISION STATED IN THE NOTE: (1) A per-counter liquidity screen must run before any cross-sectional feature is computed, and counters failing it must emit an abstention rather than a stale-price signal - A_T does not get to assume a daily series on this market. (2) A_V reuses this idiosyncratic risk construction (residual standard deviation from a local factor model over a rolling window, ASTRI market proxy, 91-day Treasury bill risk-free, with Abeysekera and Nimal (2017) as a four-factor local alternative) but adds the non-synchronous trading correction they skip and reports the correlation between the risk estimate and turnover, to establish whether A_V and A_L are partly measuring the same thing before any weighting is set on them. (3) The cross-sectional volatility ranking's expected separating power on CSE counters should be "pinned down on my own data before the agent's influence weight is allowed to swing much on it", given the 0.221/0.050 spread. (4) Any PPE-derived or lease-sensitive fundamental feature must either avoid the affected line items or carry an explicit SLFRS 16 break control, "with the choice stated in the methodology - I'd rather find this now than discover it in an ablation". (5) The execution-cost participation-rate sweep must be calibrated against free float rather than shares outstanding, and this is to be checked on my own data "before setting the sweep range". (6) A_F is designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence. (7) The volatility-persistence argument in the proposal is to be made at the mechanism level - investment suppression propagating through reporting periods - rather than by another citation of a long-memory d estimate.</t>
         </is>
       </c>
       <c r="X59" s="11" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note as a modelled component. There is no volatility model, no risk term and no position sizing in the paper. The nearest related observation in my note is a failure mode rather than a risk treatment: "Since seasonality and trend removal were abandoned, the network is fitting levels rather than changes, which is the condition under which that failure mode is expected" (the failure mode being that the LSTM reproduces the shape of the series with a lag and smooths away the local swings).</t>
+          <t>None as a modelled component. There is no volatility model, no risk term and no position sizing in the paper. The nearest related observation in my note is a failure mode rather than a risk treatment: "Since seasonality and trend removal were abandoned, the network is fitting levels rather than changes, which is the condition under which that failure mode is expected" (the failure mode being that the LSTM reproduces the shape of the series with a lag and smooths away the local swings).</t>
         </is>
       </c>
       <c r="P60" s="11" t="inlineStr">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="Q60" s="11" t="inlineStr">
         <is>
-          <t>Not recorded in the note as an explicit contribution. The nearest thing is the reporting of the weight ratio itself, which my note credits as the one advantage this paper has over the LLM systems for gap-argument purposes: "the contrast is cleaner here than in any of the LLM systems, because this paper does at least have an explicit weight vector to point at." The paper does not report the realised per-day share each channel held, which is the quantity my note reconstructs and criticises it for omitting.</t>
+          <t>None as an explicit contribution. The nearest thing is the reporting of the weight ratio itself, which my note credits as the one advantage this paper has over the LLM systems for gap-argument purposes: "the contrast is cleaner here than in any of the LLM systems, because this paper does at least have an explicit weight vector to point at." The paper does not report the realised per-day share each channel held, which is the quantity my note reconstructs and criticises it for omitting.</t>
         </is>
       </c>
       <c r="R60" s="11" t="inlineStr">
@@ -8552,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A64"/>
+  <dimension ref="A1:A67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="142" customWidth="1" min="1" max="1"/>
@@ -8940,6 +8940,20 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>Amendment, 18 October 2026 (third)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>Consistency pass over the whole sheet; again no row's reading, rating or usage changed and no row is marked amber. (1) Dash normalisation: 560 em dashes and 49 spaced en dashes replaced with a spaced hyphen, and en dashes inside letter compounds replaced with a plain hyphen, to meet the no-em-dash rule that applies to every artefact. The 62 en dashes inside numeric ranges such as 2017-2019 and page spans are deliberately left intact, as are the two inside the wikilinks [[HLOB ...]] and [[Efficient estimation of bid-ask spreads ...]], where the character is part of the target filename and changing it would break the link. (2) DOIs added to P34, P35, P36, P37 and P57 from My Library.bib. The P57 DOI is the SSRN working-paper one; the Review of Financial Studies DOI is not in the library and has not been invented. (3) Four cells that genuinely had no content were written from their notes: Key Results for P26, P46 and P52, and Dataset(s) and Period for P46. (4) Six cells that read 'Not recorded in the note' where the note in fact records a deliberate absence now read 'None': P14 Fundamental / RAG, P58 Sentiment and Liquidity, P59 Sentiment, P60 Volatility and Explainability. P14 Sentiment was left alone; its wording is accurate as written. (5) Five Year cells that carried prose, P12, P56, P57, P58 and P59, are now bare years matching the other 54 rows, with the nuance moved into Venue / Type.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 14:40:58
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Literature Survey Matrix.xlsx
+++ b/FYP/Matrices/Literature Survey Matrix.xlsx
@@ -1626,12 +1626,12 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -1641,12 +1641,12 @@
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
@@ -1749,12 +1749,12 @@
       </c>
       <c r="L10" s="7" t="inlineStr">
         <is>
-          <t>N/A - a pipeline, not an agent system.</t>
+          <t>None - a pipeline, not an agent system.</t>
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="Q10" s="7" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>N/A - a model pipeline, not an agent system.</t>
+          <t>None - a model pipeline, not an agent system.</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1882,17 +1882,17 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="Q11" s="5" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
-          <t>N/A - no conditional variance model.</t>
+          <t>None - no conditional variance model.</t>
         </is>
       </c>
       <c r="P12" s="7" t="inlineStr">
@@ -2118,17 +2118,17 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -2241,17 +2241,17 @@
       </c>
       <c r="L14" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="O14" s="7" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>N/A - single agent, not a multi-agent system.</t>
+          <t>None - single agent, not a multi-agent system.</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr">
@@ -3125,22 +3125,22 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Yu, Li, Chen, Jiang, Li, Zhang, Liu, Suchow &amp; Khashanah (Stevens Institute of Technology)</t>
+          <t>Yu, Li, Chen, Jiang, Li, Suchow, Zhang and Khashanah (Stevens Institute of Technology). This is the journal author list: it drops Rong Liu, who appears on the preprint, and places Suchow before Zhang. The journal version standardises on FINMEM and the stray "FinMe" spellings in the preprint body are gone, though the vault note is still filed under the old name. Citekey: yuFinMemPerformanceEnhancedLLM2025.</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>arXiv 2311.13743v2. Code released</t>
+          <t>IEEE Transactions on Big Data 11(6), pp. 3443-3459, November/December 2025. Received 1 December 2023, revised 26 September 2024, accepted 17 July 2025. The note was first written against arXiv:2311.13743v2 and has been rechecked line by line against the published paper, and it instructs citing the journal version rather than the preprint. A separate three-page version exists at the AAAI Spring Symposium Series 2024, 3(1), pp. 595-597, which is a different artefact again.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>FinMem / FinMe | arXiv:2311.13743</t>
+          <t>DOI 10.1109/TBDATA.2025.3593370. Preprint arXiv:2311.13743v2. Code released.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>N/A - not an agent system.</t>
+          <t>None - not an agent system.</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
@@ -3544,7 +3544,7 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
@@ -3667,7 +3667,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="M26" s="7" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>N/A (paper-level extraction fields: data &amp; universe, split protocol, action semantics, execution &amp; costs, leakage, artifacts, multi-agent reporting).</t>
+          <t>None (paper-level extraction fields: data &amp; universe, split protocol, action semantics, execution &amp; costs, leakage, artifacts, multi-agent reporting).</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -4372,17 +4372,17 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>arXiv preprint, arXiv:2409.06289v4 dated 3 November 2025. Recovered from the note header; the Research Papers Grid entry 43 left the year blank.</t>
+          <t>arXiv preprint, arXiv:2409.06289. Year recorded as 2024, matching the note frontmatter, the citekey kouAutomateStrategyFinding2024 and My Library.bib; the version read is v4, dated 3 November 2025. The Research Papers Grid entry 43 left the year blank.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>arXiv:2409.06289v4, 3 November 2025, seventeen pages plus seven-page appendix; code at github.com/kouzhizhuo/Automate-Strategy-Finding-with-LLM-in-Quant-investment.</t>
+          <t>DOI 10.48550/ARXIV.2409.06289. arXiv:2409.06289v4, 3 November 2025, seventeen pages plus a seven-page appendix; code at github.com/kouzhizhuo/Automate-Strategy-Finding-with-LLM-in-Quant-investment.</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -4533,12 +4533,12 @@
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>N/A.</t>
+          <t>None.</t>
         </is>
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>Two maps. Figure 1, a ten-stage reference workflow: user input and task perception, memory and context management, planning and task decomposition, reasoning plus action execution, observation and feedback handling, memory update, reflection and self-evaluation, multi-agent collaboration, output synthesis, evaluation. "It is presented as a linear chain with single arrows, which is already a modelling choice worth noticing, since reflection and memory update are loops in every system that has them." Figure 2, 31 systems sorted into seven use-case branches and tagged with the stage numbers they implement.  N/A. Table 1 compares four flagship systems (FinRobot, MarketSenseAI, FinVerse, FinGPT Agent) on six capabilities; the Adaptive Agent Architecture row reads: FinRobot "no, sequential"; MarketSenseAI "no"; FinVerse "partial, planning loop plus self-reflection"; FinGPT Agent "RLHF."</t>
+          <t>Two maps. Figure 1, a ten-stage reference workflow: user input and task perception, memory and context management, planning and task decomposition, reasoning plus action execution, observation and feedback handling, memory update, reflection and self-evaluation, multi-agent collaboration, output synthesis, evaluation. "It is presented as a linear chain with single arrows, which is already a modelling choice worth noticing, since reflection and memory update are loops in every system that has them." Figure 2, 31 systems sorted into seven use-case branches and tagged with the stage numbers they implement. Table 1 compares four flagship systems (FinRobot, MarketSenseAI, FinVerse, FinGPT Agent) on six capabilities; the Adaptive Agent Architecture row reads: FinRobot "no, sequential"; MarketSenseAI "no"; FinVerse "partial, planning loop plus self-reflection"; FinGPT Agent "RLHF."</t>
         </is>
       </c>
       <c r="L32" s="11" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Briola, Bartolucci and Aste, UCL Computer Science and the LSE Systemic Risk Centre. "HLOB - Information persistence and structure in limit order books." Expert Systems With Applications 266, 2025, article 126078. Published open access 12 December 2024.</t>
+          <t>Briola, Bartolucci and Aste, UCL Computer Science and the LSE Systemic Risk Centre. "HLOB – Information persistence and structure in limit order books." Expert Systems With Applications 266, 2025, article 126078. Published open access 12 December 2024.</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
@@ -7252,7 +7252,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid-ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
+          <t>Ardia, D., Guidotti, E. and Kroencke, T.A. (2024). Efficient estimation of bid–ask spreads from open, high, low, and close prices. Journal of Financial Economics, 161, 103916. DOI: 10.1016/j.jfineco.2024.103916. Authors: David Ardia (HEC Montréal), Emanuele Guidotti (USI Lugano), Tim A. Kroencke (FHNW and Remaco Asset Management). Citekey: ardiaEfficientEstimationBid2024. Implementations in several languages plus the computed spread data at github.com/eguidotti/bidask; a Harvard Dataverse replication package is also noted.</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
@@ -7272,14 +7272,14 @@
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Low-frequency microstructure econometrics - estimation of the effective bid-ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin-Schultz (2012) / Abdi-Ranaldo (2017) lineage.</t>
+          <t>Low-frequency microstructure econometrics - estimation of the effective bid–ask spread from daily OHLC prices. This is tooling, not a competitor architecture: "there is no agent in it and no trading decision". It sits in the measurement layer that the execution-cost literature assumes and never supplies, alongside the Roll (1984) / Hasbrouck (2009) / Corwin–Schultz (2012) / Abdi–Ranaldo (2017) lineage.</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>Produce an estimator of the effective bid-ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
+          <t>Produce an estimator of the effective bid–ask spread using only open, high, low and close prices, that stays unbiased when prices are observed discretely (i.e. when trades per period are finite). The contribution has two halves the note insists on keeping separate. (1) An analytical correction: "every low-frequency spread estimator before this one assumes prices are observed continuously, meaning at least one trade between any two time instants, and when that fails the estimate is biased downward". Ardia et al. "derive estimators that hold under discretely observed prices, with a correction term built from the probability that the open or close coincides with the high or low, which is a direct consequence of too few trades per period." (2) An efficiency argument: prior estimators use a subset of the four prices and discard the rest, so the authors derive several estimators from different price combinations and combine them by GMM to minimise estimation variance. The output is EDGE, an Efficient Discrete Generalized Estimator.
 The object being estimated is the effective spread, not the quoted spread. The quoted spread is the posted distance between best bid and best ask; the effective spread is the realised distance between the transaction price and the unobserved fundamental price, S = 2D(P − P̃)/P̃, with D = +1 for buyer-initiated and −1 for seller-initiated trades. They differ because dealers often execute inside the quotes, and "one of this paper's headline empirical results is that the end-of-day quoted spread overstates the effective spread by up to 100%." For a cost model the effective spread is the right object and the harder one, since P̃ is never observed.
-The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid-ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed - Roll additionally required equally likely buys and sells; Corwin-Schultz and Abdi-Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
+The reframing: derive estimators under three general assumptions and let discreteness appear as an analytical term rather than as an error. The assumptions are that fundamental returns are not serially correlated, that they are uncorrelated with bid–ask bounces, and that bounces are uncorrelated with zero mean. These are weaker than prior work needed - Roll additionally required equally likely buys and sells; Corwin–Schultz and Abdi–Ranaldo both required a geometric Brownian motion for the fundamental price with constant drift and volatility, ruling out heteroskedasticity and jumps.</t>
         </is>
       </c>
       <c r="H54" s="9" t="inlineStr">
@@ -7289,10 +7289,10 @@
       </c>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>Two evaluations (a simulation and a CRSP-TAQ empirical study) plus three applications.
+          <t>Two evaluations (a simulation and a CRSP–TAQ empirical study) plus three applications.
 Simulation: Corwin and Schultz (2012) design as reused by Abdi and Ranaldo (2017). 10,000 months, each 21 trading days, each day 390 minutes. Fundamental price P̃_m = P̃_{m−1}e^{σz}, P̃_0 = 1, z standard Gaussian. Daily sd 3%, per-minute sd 3%/√390. Trade prices are P̃_m times one minus (plus) half the spread, 50% chance of a bid (ask). Trade probability varied so expected trades per day runs from 1 to 390. On no-trade days the previous day's close is forward-filled into all four prices. Spreads tested: 0.50%, 1.00%, 2.00% through 8.00%.
 Empirical: CRSP US Stock Database, 1926–2021, NYSE / AMEX / NASDAQ, share codes 10 and 11. Benchmark is the Holden and Jacobsen (2014) effective spread from TAQ, May 1993 - December 2021. Merged sample 1,637,621 stock-months, CUSIP and ticker matching recovering 99% of CRSP stocks. Intraday sample 711,161 stock-months with both minute and daily estimates, October 2003 - December 2021. Crypto: Binance, 2163 pairs, 53,865 pair-months, July 2017 - December 2021, at daily / hourly / minute frequency.
-Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high-low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
+Non-transaction-based prices (CRSP quote-derived midpoints) are treated as missing, as are days where open or close falls outside the high–low range. Missing-estimate frequency in the merged sample is 1.24% for EDGE against 0.03% for CS and 0.14% for ROLL, EDGE's higher rate coming from needing open prices and at least three observations per stock-month. Where CHL is missing and CS is not, CS returns zero in 90% of cases and AR in 100%, which the authors read as the asset always trading at the same price so the correction's denominator is zero and the estimate is genuinely undefined. My own view in the note: "An undefined estimate is more honest than the implicit zero the alternatives produce."</t>
         </is>
       </c>
       <c r="J54" s="9" t="inlineStr">
@@ -7310,7 +7310,7 @@
 where bars denote de-meaned returns, r̄_t = r_t − τ_t·E[r_t]/E[τ_t], "which is the de-meaning that survives the conditioning on τ_t". The denominator is the entire discreteness correction and is the only thing separating this from the classical form: if prices are observed continuously the open and close can never coincide with the high or low, both probabilities equal one, the denominator collapses to two, and the expression reverts to the familiar −4E[·] shape.
 The note's reading: "The correction is therefore not a robustness patch bolted onto an existing estimator, it is a term that is identically one under the old assumption and shrinks the denominator, inflating the spread estimate, exactly in proportion to how often the price failed to move within the period."
 The same construction over other price combinations gives four Discrete Generalized Estimators - OHL, CHL, OHLC and CHLO - the first pair measuring the spread at the open and the second at the close. Their CHL estimator reduces exactly to the Abdi and Ranaldo (2017) estimator when continuous observation is imposed and returns are zero-mean, "so the prior work is recovered as a special case rather than contradicted."
-Efficiency half: the four estimators behave in opposite ways - when the spread is small relative to volatility the estimators using the mid-price have lower variance, and when the spread is large and observed returns are driven by bid-ask bounces, pairing mid-to-open with open-to-mid returns cancels a variance term that pairing with the closing price does not. Combining OHL with CHLO and OHLC with CHLO gives two moment conditions, and GMM with a diagonal weighting matrix reduces to a variance-weighted average:
+Efficiency half: the four estimators behave in opposite ways - when the spread is small relative to volatility the estimators using the mid-price have lower variance, and when the spread is large and observed returns are driven by bid–ask bounces, pairing mid-to-open with open-to-mid returns cancels a variance term that pairing with the closing price does not. Combining OHL with CHLO and OHLC with CHLO gives two moment conditions, and GMM with a diagonal weighting matrix reduces to a variance-weighted average:
 S²_EDGE = w₁·E[x_{1,t}] + w₂·E[x_{2,t}]
 x_{1,t} = (π_o/2)(η̄_t − ō_t)(o_t − η_{t−1}) + (π_c/2)(η̄_{t−1} − c̄_{t−1})(c_{t−1} − η_{t−1})
 x_{2,t} = (π_o/2)(η̄_t − ō_t)(o_t − c_{t−1}) + (π_c/2)(ō_t − c̄_{t−1})(c_{t−1} − η_{t−1})
@@ -7377,9 +7377,9 @@
       <c r="T54" s="9" t="inlineStr">
         <is>
           <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% - "a bias roughly seven times the quantity being measured" - and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
-2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid-ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information - Chen et al. (2017) being their example - is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
+2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid–ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information - Chen et al. (2017) being their example - is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
 3. No order size anywhere in the model. For a deep market the marginal-trade cost is close enough; "for a book where a single order can be a meaningful fraction of daily volume it is the intercept of a cost function and not the function." The scope is honest and never overclaimed, but EDGE answers only the first of the four open items in my cost work and leaves the nonlinear impact form, the participation-rate sweep and the thin-book depth calibration untouched.
-4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden-Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility - "plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation." The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
+4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden–Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility - "plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation." The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
 5. The estimator needs at least three usable observations per stock-month and the paper never reports performance conditional on a small count. Periods with τ_t = 0 are excluded, and EDGE is missing in 1.24% of CRSP stock-months on that basis. "The thinnest cut they report is the bottom trading-frequency quintile of US-listed stocks, which still trades most days. For a counter with five trading days in a month the estimator is defined and will return a number computed from a handful of covariance terms, deep inside the small-sample regime where their own truncation bias is worst, and nothing in the paper tells me how that number behaves. That is the gap between what the paper validates and what I would be doing with it."
 6. The simulation's "infrequent trading" is not frontier-market infrequent. Panel B sets the daily trade probability to 1%, which on a 390-minute day means roughly four expected trades per day, and the bias plot extends down to one trade per day. "That is thin by US standards and it is the right stress test for the method, but a CSE counter in the bottom half of a liquidity screen can go whole days without a trade, and the paper's design forward-fills those days rather than modelling a counter that trades on five days in a month. The estimator handles the forward-fill correctly through its indicator; what is untested is the regime where the number of usable observations per stock-month falls into single digits."
 7. A premise doing quiet work throughout: that the effective spread is the whole of the transaction cost, since nothing in the model has an order size in it. The paper never claims otherwise and the title is honest about scope.</t>
@@ -7410,7 +7410,7 @@
       </c>
       <c r="V54" s="9" t="inlineStr">
         <is>
-          <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren-Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
+          <t>EDGE supplies the intercept of the cost function; the slope remains open and remains mine. Because the effective spread prices a marginal trade and the paper has no order size in it, "the participation-rate sweep, the nonlinear impact form and the depth calibration remain open and remain mine. Framing it as EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part makes the contribution narrower and more defensible than the earlier wording, and it uses this paper as support rather than letting it look like competition."
 Second, the small-count regime is untested: the estimator is defined with three usable observations but the paper never characterises its behaviour there, and that is exactly the regime a CSE counter with five trading days in a month occupies.
 Third, the paper measures a spread; it never puts that spread inside a decision objective. "It sits alongside [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] as the measurement layer those papers assume and never supply." The claim that cost belongs inside the objective rather than deducted afterwards is still mine to make - and now has two separately validated pieces behind the cost term.
 Fourth, no validation against a quote-based benchmark in an emerging or frontier market: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
@@ -7426,12 +7426,12 @@
 AMENDED EFFECT ON SUB-GAP 1, 11 OCTOBER 2026: the claim below that this paper CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 is WITHDRAWN. With EDGE demoted, the measurement half is open again and the cost term stays on the existing proxies until real CSE quotes are obtained. Sub-gap 1 is therefore stated with two caveats rather than one: a potentially overlapping 2026 paper (Smart Trading Rule) was identified and could not be obtained, AND the proxy route that would have substituted for the missing quote data is not validated on any market resembling the CSE. That is a weaker position than v5 recorded and it should be stated as such rather than discovered in the viva.
 --- RETAINED AS RECORD, SUPERSEDED ---
 SPEAKS TO: A_L above all - this is the measurement instrument the liquidity agent currently lacks - plus the orchestrator (the cost term that enters the objective rather than being deducted after), the liquidity state L_t (two new candidate inputs), and the evaluation layer (the window decision and the mandatory non-positive-fraction reporting).
-EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency - "all proxies for illiquidity rather than measurements of what a trade pays" - and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade - "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren-Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
+EFFECT ON SUB-GAP 1: THIS PAPER CLOSES THE MEASUREMENT HALF OF SUB-GAP 1 AND SHARPENS WHAT IS LEFT. My cost work currently rests on Amihud illiquidity, turnover and zero-return frequency - "all proxies for illiquidity rather than measurements of what a trade pays" - and the alternative on offer in the systems literature is the flat percentage that MacroHFT (0.02%) and the DRL global-equity portfolio work (2bps) assume. EDGE replaces that constant with a per-counter, per-period effective spread in basis points computed from daily OHLC alone. That converts "expected execution cost enters the decision objective" from an assertion into something with a measured number in it. But the closure is partial and the paper is explicit about where it stops: there is no order size in the model, so what EDGE gives is the cost of a marginal trade - "the intercept of a cost function and not the function". So Sub-gap 1 survives in a narrower and more defensible form: EDGE for the spread, Almgren–Chriss or a queue-reactive treatment for the size-dependent part, and my contribution is the participation-rate sweep, the nonlinear impact form, the thin-book depth calibration, and above all what an orchestrator does with a cost term that varies by counter and by date. The part of Sub-gap 1 that actually survives intact is the claim that cost belongs inside the objective rather than deducted afterwards.
 The second half of Sub-gap 1 - that liquidity simultaneously conditions the reliability of price-derived agents - gets independent support from the paper's own mechanism rather than from my framing. The τ_t = 0 condition is literally the case where the price carries no information about the spread within the period, and the coincidence probability that drives the correction is "a direct consequence of too few trades per period". That is a measured, published statement that price-derived quantities degrade in a specific, quantifiable way as trading thins - which is precisely the premise under which L_t should down-weight A_T.
 EFFECT ON MAIN GAP: Indirect but real. The main gap is market-state-aware dynamic orchestration with w(i,t) = f(L_t, V_t, P_t, C_{i,t}), and the weakest-specified argument of that function is L_t. This paper contributes two candidate components to it that measure something the existing three proxies do not. The spread gives L_t a component denominated in the same units as the objective. The τ_t indicator gives a staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both enter the ablation protocol as additions to test rather than adopt, "which turns the question from whether liquidity matters into whether a measured spread and a measured staleness rate carry anything beyond the three proxies already there." That reframing is itself useful: it converts a soft claim about liquidity-awareness into a falsifiable ablation.
 EFFECT ON SUB-GAP 2: Minimal and only by friction. The paper estimates no volatility model and says nothing about persistence. The one contact point is Assumption 1, which rules out serially correlated fundamental returns and "sits uneasily beside the long-memory results on the ASPI and SL20" in the CSE volatility-memory work - but the note is careful that "that tension is about return persistence rather than volatility persistence and I would want to test rather than assert it." So this does not move Sub-gap 2. There is one indirect operational link: the frequency result argues that any intraday CSE feed is worth far more to the cost model than more daily history, "and it connects to the volatility estimator decision too, since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE." The two data questions are the same question.
 CSE DATA EVIDENCE: The note's CSE-side commitments are: the CSE publishes daily OHLC for every listed counter, which is what makes EDGE applicable with no quote feed; the per-counter archive is roughly 374 trading days, giving ~21 observations per monthly estimate - "squarely in that regime" where 25.63% of CRSP daily-price estimates come out non-positive and 41% of large-cap stock-months come out negative before truncation; and a CSE counter in the bottom half of a liquidity screen "can go whole days without a trade", below anything the paper's simulation stresses (its thinnest panel is ~4 expected trades per day, with the bias plot extending to one trade per day, and no-trade days forward-filled rather than genuinely absent). The resulting design decisions are a quarterly window on the per-counter track, monthly on the index track where ten years of daily data supports it, and the fraction of non-positive estimates reported alongside every spread series in both cases.
-PROPOSED REVISION STATED IN THE NOTE: Re-scope the cost sub-gap as "EDGE for the spread and an Almgren-Chriss or queue-reactive treatment for the size-dependent part" - narrower and more defensible than the earlier wording, using this paper as support rather than letting it look like competition. Claim EDGE as an adopted measurement with the implementation cited and keep all novelty language off it; the one defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered. Add the measured spread and the τ_t staleness rate to the liquidity-state ablation as candidates to test rather than adopt. Fix the aggregation window before running anything (quarterly per-counter, monthly index-track) and report the non-positive fraction every time. Put the intraday-feed question to the supervisor before investing in deeper daily history.</t>
+PROPOSED REVISION STATED IN THE NOTE: Re-scope the cost sub-gap as "EDGE for the spread and an Almgren–Chriss or queue-reactive treatment for the size-dependent part" - narrower and more defensible than the earlier wording, using this paper as support rather than letting it look like competition. Claim EDGE as an adopted measurement with the implementation cited and keep all novelty language off it; the one defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered. Add the measured spread and the τ_t staleness rate to the liquidity-state ablation as candidates to test rather than adopt. Fix the aggregation window before running anything (quarterly per-counter, monthly index-track) and report the non-positive fraction every time. Put the intraday-feed question to the supervisor before investing in deeper daily history.</t>
         </is>
       </c>
       <c r="X54" s="9" t="inlineStr">
@@ -7516,7 +7516,7 @@
 OPTIMAL WEIGHTS (Bates and Granger 1969 for pairs, Newbold and Granger 1974 in general) minimise the variance of the combined forecast error:
 w^opt_{T+h|T} = Σ⁻¹_{T+h|T} 1 / (1' Σ⁻¹_{T+h|T} 1)
 with Σ the N×N covariance matrix of h-step forecast errors. If the individuals are unbiased and their error variances stable, the combination is unbiased and its error variance is no greater than the minimum across individuals - "the diversification result the whole field rests on. The catch is in the last sentence of that passage: in practice Σ is unknown and has to be estimated, and that single sentence generates most of the rest of the literature."
-REGRESSION WEIGHTS (Granger and Ramanathan 1984): three regimes - weights summing to one with no intercept, which reproduces Bates-Granger exactly; unconstrained with no intercept; and unconstrained with an intercept, which they argued is superior regardless of whether constituents are biased because the intercept absorbs the bias. De Menezes et al. (2000) push back that the unrestricted version needs stationarity and runs into serial correlation and multicollinearity. Aksu and Gunter (1992) found empirically that constraining weights to be nonnegative is at least as robust as the simple average while beating the other regression variants - "which is the practical reading I'd take."
+REGRESSION WEIGHTS (Granger and Ramanathan 1984): three regimes - weights summing to one with no intercept, which reproduces Bates–Granger exactly; unconstrained with no intercept; and unconstrained with an intercept, which they argued is superior regardless of whether constituents are biased because the intercept absorbs the bias. De Menezes et al. (2000) push back that the unrestricted version needs stationarity and runs into serial correlation and multicollinearity. Aksu and Gunter (1992) found empirically that constraining weights to be nonnegative is at least as robust as the simple average while beating the other regression variants - "which is the practical reading I'd take."
 PERFORMANCE-BASED, discounted variant (the one with a time dimension, and the one the note would implement first because it needs no pairwise estimation):
 w^{bg4}_{T+h|T,i} = ( Σ_{t=1}^{T} γ^t e²_{t|t−h,i} )⁻¹ / Σ_{j=1}^{N} ( Σ_{t=1}^{T} γ^t e²_{t|t−h,j} )⁻¹ , γ ≥ 1
 where e_{t|t−h,i} is the h-step error of method i made at t−h and realised at t, and γ controls how fast older errors are forgotten, with γ = 1 recovering the plain inverse-MSE weight over the full history. The rolling-window variant replaces the discount with a sum over the most recent ν observations. Both are adapted to non-stationary relationships between methods, and both, as Timmermann (2006) is quoted saying, "increase the variance of the parameter estimates and work quite poorly if the data generating process really is covariance stationary." Stock and Watson (1998) generalise by making weights inversely proportional to the kth power of MSE, so k=0 is equal weights and larger k concentrates on the best performer - "a single interpretable dial between the two extremes."
@@ -7622,7 +7622,7 @@
 The honest consequence the note draws: the equal-weight baseline becomes the field's hardest benchmark, and "if my state-conditioned weighting fails to beat equal weights on the CSE, that is the expected outcome under the field's prior and not a surprise". The response is not to defend the gap but to pre-register - write down before the run what margin and what test would count as beating equal weights. And the note extracts a genuine contribution even from failure: "Which effect dominates on this data is the question, and the paper is clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature, so an answer in a thin frontier market is a contribution even if the answer is that equal weights win."
 How my setting differs - three ways the note identifies. (i) My weights condition on exogenous measured market state, not on properties of the series computed once; this is the axis the literature has not covered. (ii) My loss is not quadratic forecast MSE against a realised value - "My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality." The asymmetric-loss line (Elliott and Timmermann 2004, Patton and Timmermann 2007) is as close as this literature gets, and it finds optimal weights depend strongly on loss asymmetry and error skewness. (iii) My pool violates the review's non-interfering assumption: the four agents read overlapping data by construction, so the unbiasedness and variance-bound results do not hold for me, and the paper's own observation that overlapping information sets produce highly correlated errors is the mechanism by which that bites.
 A second threat, from the WARNING box rather than the paper itself. Frazier, Covey, Martin and Poskitt (Monash EBS WP 18/2023, arXiv:2308.05263) argue the puzzle is substantially an artefact of two-step estimation: estimated weights impart no first-order sampling variability into the usual predictive-accuracy statistic, so it converges to a generalised chi-squared rather than a normal, and their Theorem 1 says that when two weight vectors lie within O(T^{−1/4−ε}) of each other "the test has no power to distinguish them at all". Two consequences land directly on my design. "The O(T^{−1/4}) rate is not small at my sample sizes, roughly 0.23 at 374 trading days against roughly 0.14 on the ten-year index track, and with four agents sitting at 0.25 each under equal weights, a short sample puts almost any non-degenerate weighting scheme inside the dead zone. The constant is unknown so neither figure is a threshold, but the direction is unambiguous and it argues for running the weighting comparison on the index series rather than the per-counter panel." And their remedy, one-step joint estimation, is "mostly unavailable to me, since a retrieval agent is not jointly optimisable with a volatility model, so the partial version is to fit the parametric agents against the combined objective rather than against their own local losses." Caveat carried: this is a working paper and its publication status needs checking before it is cited as anything else.
-Design decisions this forces on the main gap: (a) no pairwise interaction term in the weighting function, backed by Bates and Granger, Newbold and Granger, and Winkler and Makridakis - ten covariance parameters against four diagonal ones, from 374 days; (b) a four-way rather than three-way comparison, adding a discounted inverse-MSE arm, because "if weights that merely react to recent agent performance do as well as weights conditioned on measured market state, then the state conditioning is not earning its place and I need to know that early"; (c) an oracle-weight arm to separate "the conditioning hypothesis is wrong" from "the estimation is too noisy"; (d) a Stock-Watson k-sweep to map the whole continuum from equal weights to winner-take-all cheaply; (e) pre-registration that separates two failure modes which look identical in the output - "the weighting genuinely not helping, which is the field's prior from the puzzle, against the weighting helping and the two-step test being unable to see it, because the first says abandon the conditioning and the second says change how it is estimated or tested."
+Design decisions this forces on the main gap: (a) no pairwise interaction term in the weighting function, backed by Bates and Granger, Newbold and Granger, and Winkler and Makridakis - ten covariance parameters against four diagonal ones, from 374 days; (b) a four-way rather than three-way comparison, adding a discounted inverse-MSE arm, because "if weights that merely react to recent agent performance do as well as weights conditioned on measured market state, then the state conditioning is not earning its place and I need to know that early"; (c) an oracle-weight arm to separate "the conditioning hypothesis is wrong" from "the estimation is too noisy"; (d) a Stock–Watson k-sweep to map the whole continuum from equal weights to winner-take-all cheaply; (e) pre-registration that separates two failure modes which look identical in the output - "the weighting genuinely not helping, which is the field's prior from the puzzle, against the weighting helping and the two-step test being unable to see it, because the first says abandon the conditioning and the second says change how it is estimated or tested."
 EFFECT ON THE ABSTENTION CHANNEL: Upgraded from a bespoke mechanism to named prior art. The paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme (Li et al., 2022). "That is structurally what the abstention channel does when the fundamental agent has no disclosure to work from, which is expected more than half the time, so I should present it in that vocabulary rather than as a bespoke mechanism." Two consequences: the paper's own assessment is that subset selection "has received scant attention, is mainly trimming on expertise alone, and that most existing algorithms are ad hoc and lack statistical rationale", so a principled selection rule driven by a structural property of the output is defensible ground; and Geweke and Amisano's observation that individually poor forecasts may still help in combination argues for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero - "a concrete design decision I had not settled."
 EFFECT ON THE CONFIDENCE TERM C_{i,t}: A route to making C_{i,t} a measured structural property rather than a self-report. If the orchestrator ever emits an interval rather than a point allocation, the linear pool's variance decomposition says component disagreement adds directly to pooled variance, "so a deliberately heterogeneous pool produces an under-confident interval, and that is the one place where my central design choice actively works against me." Quantile averaging avoids it - it averages cdfs horizontally, preserves the family for location-scale components, and is sharper for the same mean. "This connects to [[Adaptive Conformal Inference Under Distribution Shift]] more tightly than I expected, since adaptive conformal inference is a per-agent calibration wrapper and quantile averaging is the aggregation step, and the pair would give me a calibrated interval from a heterogeneous pool without the under-confidence that linear pooling would introduce. That is a route to the confidence term being a measured interval width rather than a self-report, which is what the scope revision asked for."
 EFFECT ON THE HETEROGENEITY CLAIM: The paper makes it testable and therefore falsifiable. "I describe the four agents as methodologically heterogeneous and that heterogeneity is load-bearing in the gap statement, but the paper's operational definition of diversity is low correlation among forecast errors... So the claim is testable on my own pool and I should run it: if the technical agent and the volatility agent produce errors that correlate at 0.8 on CSE data, the pool is substantially less diverse than the architecture diagram implies and the error-cancellation argument weakens accordingly. This is close to free, it uses data I will already have from the individual agent runs, and it is the kind of result that is much better found by me than by an examiner." Also relevant: Mannes et al. (2014) show the mean level of expertise in the pool sets a floor, so including a poor agent degrades the result - which bears on whether all four agents should always be in the pool.
@@ -7630,7 +7630,7 @@
 EFFECT ON SUB-GAP 1: Negative in the sense that it offers nothing - "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages" - but that absence is itself the boundary line. Everything in this paper is a weighting mechanism scored against a realised value under quadratic loss; none of its optimality results transfer to an after-cost decision objective. So the claim that execution cost belongs inside the decision objective is untouched by fifty years of combination theory, which is a clean separation to state.
 EFFECT ON SUB-GAP 2: Essentially none directly. The only contact point is Zischke et al. (2022), who find that in high-volatility periods weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample - "a result about choosing what to score rather than about how elaborate the pooling function is". That is about volatility level, not persistence, and the review contains nothing on persistence or on decay schedules. The structural-change guideline ("structural change impacts sophisticated schemes more than the simple average and changing weights are a legitimate response to it") is the nearest thing to support for conditioning on a regime, but it is a general statement with no persistence mechanism behind it.
 CSE DATA EVIDENCE: The note states my per-counter archive as roughly 300 counters over 374 trading days, "three orders of magnitude short of M4", with "no result in this paper" speaking to a feature-to-weight meta-model at that scale. The ten-year index track is the alternative. Those two sample sizes drive the O(T^{−1/4}) calculation - roughly 0.23 at 374 trading days against roughly 0.14 on the index track, against four agents at 0.25 each under equal weights - which argues for running the weighting comparison on the index series rather than the per-counter panel. The same 374 days drive the parameter-count argument against a pairwise interaction term (ten covariance parameters against four). And the note's reading of the thin-market absence is directional rather than agnostic: "everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
-PROPOSED REVISION STATED IN THE NOTE: Reframe the weighting function as a generalisation of FFORMA along one identified axis - exogenous measured market state at each step versus series properties computed once - rather than as new machinery. Pre-register the margin and the test that would count as beating equal weights, before the run. Expand the planned three-way comparison (equal / static learned / state-conditioned) to four-way by adding a discounted inverse-MSE arm, and add an oracle-weight arm fitted on the test window to separate "conditioning is wrong" from "estimation is too noisy". Add a Stock-Watson k-sweep. Run the weighting comparison on the index series rather than the per-counter panel, on the power argument. Fit the parametric agents against the combined objective rather than their own local losses, as the partial version of one-step joint estimation. Present the abstention channel as time-varying subset selection with a threshold, and shrink the abstaining agent's weight toward a floor rather than to exactly zero. Measure pool diversity as error correlation before claiming heterogeneity. Keep a separate note for the Frazier et al. working paper and check its publication status before citing it as anything other than a working paper. State explicitly in the write-up why there is no pairwise interaction term. And carry the warning that standard errors on a combined forecast are nontrivial because the weights are random and correlated with the forecasts - which matches the pattern where "the economic result and the formal test diverged" in the DRL global-equity portfolio note.</t>
+PROPOSED REVISION STATED IN THE NOTE: Reframe the weighting function as a generalisation of FFORMA along one identified axis - exogenous measured market state at each step versus series properties computed once - rather than as new machinery. Pre-register the margin and the test that would count as beating equal weights, before the run. Expand the planned three-way comparison (equal / static learned / state-conditioned) to four-way by adding a discounted inverse-MSE arm, and add an oracle-weight arm fitted on the test window to separate "conditioning is wrong" from "estimation is too noisy". Add a Stock–Watson k-sweep. Run the weighting comparison on the index series rather than the per-counter panel, on the power argument. Fit the parametric agents against the combined objective rather than their own local losses, as the partial version of one-step joint estimation. Present the abstention channel as time-varying subset selection with a threshold, and shrink the abstaining agent's weight toward a floor rather than to exactly zero. Measure pool diversity as error correlation before claiming heterogeneity. Keep a separate note for the Frazier et al. working paper and check its publication status before citing it as anything other than a working paper. State explicitly in the write-up why there is no pairwise interaction term. And carry the warning that standard errors on a combined forecast are nontrivial because the weights are random and correlated with the forecasts - which matches the pattern where "the economic result and the formal test diverged" in the DRL global-equity portfolio note.</t>
         </is>
       </c>
       <c r="X55" s="11" t="inlineStr">
@@ -8165,7 +8165,7 @@
       <c r="W58" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_F (the fundamental agent) - feature selection, update frequency and architectural role; the abstention channel; universe construction and point-in-time screening; and the local-evidence justification for using the CSE. It is the most recent published statement I have of which accounting ratios associate with price on CSE financials, over a window that overlaps mine almost exactly.
-EFFECT ON MAIN GAP: Strongly supportive, and in a very specific way. The within/between split - 0.090 within against 0.709 between - is a direct, locally measured statement that the fundamental channel's reliability is horizon-dependent on this market: it prices counters against each other well and says almost nothing about when a given counter moves. That is precisely the kind of structural property the weighting function w(i,t) = f(L_t, V_t, P_t, C_i,t) is meant to exploit, and it gives me a published, CSE-specific number for why the fundamental agent's weight should be capped and slow-moving between reporting dates rather than allowed to drive entry and exit. It also supports the C_i,t component being a structural property of the output rather than a self-report: ROE and DPS fail to clear not because they are irrelevant but because they are collinear with EPS (DPS-EPS at 0.757), so a channel whose inputs are collinear or missing should be detectable from the structure of its inputs and allowed to abstain. "Letting the channel return no view when its inputs are collinear or missing is the design consequence, and it is the same abstention argument the liquidity screen produces for the technical channel." Finally, the paper's pooling of eleven years containing a currency collapse as one regime is my clearest local illustration of what a fixed, non-state-conditional combination rule costs: "This is now the third CSE result pointing the same way, alongside the macro linkages breaking over 2014 to 2022 in [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] and the 2021 extension halving the investment-risk coefficient in the Fernando note."
+EFFECT ON MAIN GAP: Strongly supportive, and in a very specific way. The within/between split - 0.090 within against 0.709 between - is a direct, locally measured statement that the fundamental channel's reliability is horizon-dependent on this market: it prices counters against each other well and says almost nothing about when a given counter moves. That is precisely the kind of structural property the weighting function w(i,t) = f(L_t, V_t, P_t, C_i,t) is meant to exploit, and it gives me a published, CSE-specific number for why the fundamental agent's weight should be capped and slow-moving between reporting dates rather than allowed to drive entry and exit. It also supports the C_i,t component being a structural property of the output rather than a self-report: ROE and DPS fail to clear not because they are irrelevant but because they are collinear with EPS (DPS–EPS at 0.757), so a channel whose inputs are collinear or missing should be detectable from the structure of its inputs and allowed to abstain. "Letting the channel return no view when its inputs are collinear or missing is the design consequence, and it is the same abstention argument the liquidity screen produces for the technical channel." Finally, the paper's pooling of eleven years containing a currency collapse as one regime is my clearest local illustration of what a fixed, non-state-conditional combination rule costs: "This is now the third CSE result pointing the same way, alongside the macro linkages breaking over 2014 to 2022 in [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] and the 2021 extension halving the investment-risk coefficient in the Fernando note."
 EFFECT ON SUB-GAP 1: Indirect and mostly cautionary. The paper has no liquidity variable, no turnover screen and no execution cost, so it offers no positive evidence on state-dependent execution friction. What it does supply is the mechanism by which thin trading corrupts a price-derived fundamental input: "on a thin market where the denominator goes near zero it also carries a variance of the kind that produced a standard deviation of 1069.92 here." That is the PE ratio blowing up to a range of −1471.22 to 2292.82 because earnings pass through zero, and it is a concrete local instance of the broader claim in SUB-GAP 1 that market conditions condition the reliability of price-derived quantities. It also gives me a worked example of a universe screen done wrong - top-20 by terminal capitalisation backfilled to 2013 - which is "the exact failure my own screen could reproduce if the liquidity filter is computed once over the full history rather than as of each rebalance date."
 EFFECT ON SUB-GAP 2: Indirect. There is no volatility persistence content in this paper - no variance model, no long-memory estimate. The only contribution is negative evidence about regime stability: eleven years pooled across the 2018 constitutional crisis, the 2019 Easter attacks, COVID, the 2022 sovereign default and inflation above 50%, with no year effects and no regime split, producing coefficients that partly fit a changing unit of measurement. That is an argument for conditioning on measured state, but it does not operationalise persistence, which remains mine to do.
 CSE DATA EVIDENCE: This is the richest part of the row for the justification rewrite, and it is all local and measured.
@@ -8236,7 +8236,7 @@
       <c r="J59" s="11" t="inlineStr">
         <is>
           <t>Annual accounting data plus weekly price series. "All accounting and insider ownership data is hand-collected from annual reports published by the CSE", prices and the index come from the CSE data libraries, and Treasury bill rates from the Central Bank of Sri Lanka.
-Idiosyncratic risk is built as the residual standard deviation from a Fama-French three-factor regression on weekly excess returns over 52 trading weeks:
+Idiosyncratic risk is built as the residual standard deviation from a Fama–French three-factor regression on weekly excess returns over 52 trading weeks:
 r_{i,t} − r_{f,t} = α_i + β_i^MKT MKT_t + β_i^SMB SMB_t + β_i^HML HML_t + ε_{i,t}, σ_i^idi = sd(ε̂_{i,t})_{t=1..52}
 where r_{i,t} is the weekly return adjusted for cash dividends, stock splits, scrip dividends, bonus issues and rights issues; the market proxy is "the percentage change in the All Share Total Return Index (ASTRI), not the ASPI, which is the right choice since it is total return rather than price only"; r_{f,t} is a weekly rate derived from the yield on 91-day Treasury bills; and "weekly returns exceeding +50% or falling below −50% are dropped as outliers, following Abeysekera and Nimal (2017)".
 Systematic risk is backed out of the decomposition rather than estimated separately: σ^sys = sqrt(σ^tot² − σ^idi²), with total risk the standard deviation of weekly returns.
@@ -8275,7 +8275,7 @@
       </c>
       <c r="O59" s="11" t="inlineStr">
         <is>
-          <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama-French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
+          <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama–French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
 What I would add: "the non-synchronous trading correction and a reported correlation between the risk estimate and turnover, because if those two move together on my sample then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it."
 Magnitude prior for A_V: "Mean idiosyncratic risk of 0.221 with a standard deviation of 0.050 sets a realistic prior on how much cross-sectional signal the volatility channel can carry. That is a narrow spread, and a one standard deviation move being worth 2.02 percentage points of investment is a real-economy effect rather than a trading one, so I should not expect the cross-sectional volatility ranking on CSE counters to separate firms as cleanly as it does on a US sample."</t>
         </is>
@@ -8320,7 +8320,7 @@
       <c r="U59" s="11" t="inlineStr">
         <is>
           <t>- The citation for why A_T cannot assume a daily price series on CSE: a finance journal estimating a factor model on CSE firms moves to weekly because most stocks don't trade daily. "That is a stronger warrant than anything I could get from the ML literature."
-- The idiosyncratic risk estimator for A_V's cross-sectional input - residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free - plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk-turnover correlation).
+- The idiosyncratic risk estimator for A_V's cross-sectional input - residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free - plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk–turnover correlation).
 - A realistic prior on how much cross-sectional signal A_V can carry: mean idiosyncratic risk 0.221, standard deviation only 0.050, range 0.117 to 0.315.
 - A mechanism-level argument for volatility persistence that is independent of the statistical long-memory literature.
 - The free-float fact (66.1% institutional, 5.7% insider) as a calibration input for the execution-cost participation-rate sweep.
@@ -8331,7 +8331,7 @@
       </c>
       <c r="V59" s="11" t="inlineStr">
         <is>
-          <t>- The non-synchronous trading problem is conceded and then left untreated: no Dimson or Scholes-Williams correction, no trading-frequency screen, no check of whether the risk measure correlates with turnover. That correction, and the reported risk-turnover correlation, is work I have to do, and it is exactly the boundary between A_V and A_L.
+          <t>- The non-synchronous trading problem is conceded and then left untreated: no Dimson or Scholes–Williams correction, no trading-frequency screen, no check of whether the risk measure correlates with turnover. That correction, and the reported risk–turnover correlation, is work I have to do, and it is exactly the boundary between A_V and A_L.
 - No out-of-sample period, no forecast, no decision objective - so nothing here tells me how a risk estimate should be weighted in a live allocation, only how it relates contemporaneously to corporate investment.
 - No execution cost model, no order size, no depth - the free-float fact implies the friction problem but the paper does not model it.
 - No persistence modelling. The paper gives a mechanism for slow decay but estimates no persistence parameter, no long-memory d and no regime structure.
@@ -8340,12 +8340,12 @@
       </c>
       <c r="W59" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk-turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
+          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk–turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
 EFFECT ON MAIN GAP: Strongly supportive on two fronts. First, regime instability: "The 2021 extension weakening the main coefficient from −0.232* to −0.123* is corroboration that CSE relationships estimated pre-2020 do not survive the crisis window intact. Taken with [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] finding the traditional macro linkages broken over 2014 to 2022, that is now two independent CSE results pointing at regime instability across exactly the period a static system would be evaluated on, which is the clearest empirical case I have for an orchestrator that conditions on measured state rather than a fixed combination rule." Note the surviving coefficient is significant only at 10%.
 Second, the C_i,t component and abstention. The frequency concession forces an abstention design on A_T: "It doesn't mean I build at weekly frequency, the index track is liquid enough for daily, it means the per-counter liquidity screen has to come before any cross-sectional feature is computed and counters that fail it have to produce an abstention rather than a stale-price signal. This is the same structural failure [[AlphaAgents, Large Language Model Based Multi-Agents for Equity Portfolio Constructions]] fixed by deleting an agent by hand." And the data-depth fact forces the same on A_F: "it is why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence." Both of these are structural properties of the input and output, not self-reports, which is exactly what C_i,t is meant to be.
 Third, a methodological warning for the state vector itself: if the volatility estimate and the liquidity estimate co-move on my sample, "then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it." That is a concrete pre-registration task for the main gap, and the paper's own −0.703 insider/institutional correlation is the worked example of what unmanaged collinearity does to a conditioning design: "every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one."
 Fourth, Model 2's design is a usable template: "splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it is close to the structure I'd want for ablating state inputs one at a time."
-EFFECT ON SUB-GAP 1: This is the strongest row in the note for state-dependent execution friction and for liquidity conditioning the reliability of price-derived agents. The reliability half is stated by the paper itself: "since most stocks are not traded daily, we use weekly stock returns" - a published finance journal on my exact market changing its estimation frequency because of thin trading. That is local empirical evidence that price-derived quantities on CSE degrade with liquidity, and it is the warrant for L_t conditioning A_T's and A_V's weights rather than being a separate add-on signal. The untreated residual is my opening: stale prices "bias the residual standard deviation downward for exactly the thinnest counters", with no Dimson or Scholes-Williams correction, no trading-frequency screen and no risk-turnover check anywhere in the paper, and "part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant." The execution-cost half comes from the ownership structure: institutional ownership averaging 66.1% against insider 5.7% means "the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding."
+EFFECT ON SUB-GAP 1: This is the strongest row in the note for state-dependent execution friction and for liquidity conditioning the reliability of price-derived agents. The reliability half is stated by the paper itself: "since most stocks are not traded daily, we use weekly stock returns" - a published finance journal on my exact market changing its estimation frequency because of thin trading. That is local empirical evidence that price-derived quantities on CSE degrade with liquidity, and it is the warrant for L_t conditioning A_T's and A_V's weights rather than being a separate add-on signal. The untreated residual is my opening: stale prices "bias the residual standard deviation downward for exactly the thinnest counters", with no Dimson or Scholes–Williams correction, no trading-frequency screen and no risk–turnover check anywhere in the paper, and "part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant." The execution-cost half comes from the ownership structure: institutional ownership averaging 66.1% against insider 5.7% means "the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding."
 EFFECT ON SUB-GAP 2: Supportive at the mechanism level, which is more than a statistical citation gives me. "The investment channel is the mechanism-level argument for pairing forecast variance with persistence rather than treating volatility as a point-in-time cap. If elevated idiosyncratic risk causes firms to cut capital spending by 17.48% of the mean investment rate, then a volatility shock on this market propagates into fundamentals with a lag measured in reporting periods, not days, and the real activity it suppresses takes just as long to come back. That is a fundamental reason to expect slow decay, independent of the statistical long-memory evidence in [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] and [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], and it is a better sentence for the proposal than another citation of a d estimate." The paper itself estimates no persistence parameter, so operationalising P_t remains entirely mine.
 CSE DATA EVIDENCE: This is the single densest source of local empirical evidence I have for the justification rewrite, and the fact that it comes from authors with no stake in making a data-depth argument is what makes it usable.
 - Thin trading, conceded in the data section: "since most stocks are not traded daily, we use weekly stock returns." Three authors with institutional access, publishing in Managerial Finance, could not estimate a factor model at daily frequency on this market. That is direct local evidence of liquidity constraint, and it is stated as a design constraint rather than as a limitation.
@@ -8552,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A67"/>
+  <dimension ref="A1:A70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="142" customWidth="1" min="1" max="1"/>
@@ -8954,6 +8954,20 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>Amendment, 18 October 2026 (fourth)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>Correction and completion pass; again no row's reading, rating or usage changed and no row is marked amber. (1) CORRECTION TO THE THIRD AMENDMENT. That pass replaced en dashes between letters with a plain hyphen. That was wrong: the rule in force bans em dashes, not en dashes, and the en dash between two separate surnames or between the two poles of a compound is the conventional academic form. All 29 have been restored, across P37, P54, P55, P58 and P59: the published titles "HLOB - Information persistence and structure in limit order books" and "Efficient estimation of bid-ask spreads from open, high, low, and close prices", the author pairs Corwin-Schultz, Abdi-Ranaldo, Almgren-Chriss, Bates-Granger, Stock-Watson, Fama-French, Scholes-Williams and Holden-Jacobsen, and the compounds bid-ask, high-low, CRSP-TAQ, risk-turnover and DPS-EPS. Em dashes remain at zero. (2) P20, FinMem, was carrying the preprint throughout and has been moved to the journal of record. Year 2023 to 2025; Venue to IEEE Transactions on Big Data 11(6), pp. 3443-3459, November/December 2025; Link to DOI 10.1109/TBDATA.2025.3593370 with the preprint retained as a secondary reference; and the Citation author list corrected to the journal one, which drops Rong Liu and places Suchow before Zhang. The note itself carries the instruction to cite the journal version rather than the preprint, and the row did not reflect it. (3) P30 year resolved to 2024, matching the note frontmatter, the citekey kouAutomateStrategyFinding2024 and My Library.bib. The v4 preprint date of 3 November 2025 is retained in Venue / Type and Link / DOI as the version read, and the arXiv DOI 10.48550/ARXIV.2409.06289 has been added. (4) Wording consistency: 29 cells that opened 'N/A' now open 'None', matching the 146 cells that already used that form for an absent component. Rows P08 to P13, P15, P22 to P26 and P31. A stray 'N/A.' sitting mid-sentence in P31 Method / Architecture, with no referent, has been deleted.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 17:20:56
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Literature Survey Matrix.xlsx
+++ b/FYP/Matrices/Literature Survey Matrix.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>The paper's claimed risk contribution is position sizing as a percentage of portfolio rather than an all-in signal - but the sizing ranges are hand-written into the prompt. No volatility model. Annualised return defined as a linear rescaling: ARR = ((P_T − P_0)/P_0) × (C/T), "so the 145-day results are simply multiplied by roughly 1.74. AMZN's headline 43.57 % for buy-and-hold is therefore about a 25 % realised gain over seven months." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model, no slippage and no impact." Student's sharpened point: "Frequent partial rebalancing in 1 to 5 % slices is exactly the pattern whose risk-adjusted advantage a realistic cost model erodes first, because the smoothing comes from trading more often rather than from taking better positions. So the absence of costs does not merely inflate a return figure here, it sits directly underneath the only result this paper can defend."</t>
+          <t>The paper's claimed risk contribution is position sizing as a percentage of portfolio rather than an all-in signal - but the sizing ranges are hand-written into the prompt. No volatility model. Annualised return defined as a linear rescaling: ARR = ((P_T − P_0)/P_0) × (C/T), "so the 145-day results are simply multiplied by roughly 1.74. AMZN's headline 43.57 % for buy-and-hold is therefore about a 25 % realised gain over seven months." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model, no slippage and no impact." Student's sharpened point: "Frequent partial rebalancing in slices of 1 to 10 % is exactly the pattern whose risk-adjusted advantage a realistic cost model erodes first, because the smoothing comes from trading more often rather than from taking better positions. So the absence of costs does not merely inflate a return figure here, it sits directly underneath the only result this paper can defend."</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Unconditional z-score screen with a deliberately high threshold: z_t = (r_t − μ_r)/σ_r, flag if |z_t| &gt; 10 with μ_r, σ_r over the whole 1980–2023 sample. Returns exactly three points: 19 Oct 1987 at −20.47, 13 Oct 2008 at +11.58, 16 Mar 2020 at −11.98. Nulls injected at 20 Oct 1987, 14 Oct 2008, 12 Mar 2020. Screen → question-formulating agent → three expert agents → consolidation agent → three-persona manager panel via AutoGen → human analyst briefing. "the terminal step, a briefing to a human analyst who makes the call, where my orchestrator has to emit the decision itself, so nothing here tells me how to close the loop." AGENTS &amp; ORCHESTRATION (exhaustive): One question-formulating agent; three expert agents (web research, curated institutional knowledge base, cross-checking against an external API); one consolidation agent; a panel of three manager personas (financial market economist, macro economist, statistician) plus a moderator and a critic. Expert layer is explicitly extensible - "the diagram has a fourth empty box, so the expert set is meant to be configured per dataset rather than fixed." Critical axis distinction: "Park's three experts are heterogeneous by evidence source, web search, a curated knowledge base, and an external API, and all three answer the same question. That is redundancy for verification rather than diversity for decision, and it means agreement between his agents is corroboration while agreement between mine would be a weak signal at best." State-conditioned influence: NONE. "as in TradingAgents and FinVision, there is no weight, no confidence scalar and no quantity anywhere that could be weighted. Consolidation is an LLM summarising free text." But note the one exception in behaviour: resolution by evidence type, below.</t>
+          <t>Unconditional z-score screen with a deliberately high threshold: z_t = (r_t − μ_r)/σ_r, flag if |z_t| &gt; 10 with μ_r, σ_r over the whole 1980–2023 sample. Returns exactly three points: 19 Oct 1987 at −20.47, 13 Oct 2008 at +11.58, 16 Mar 2020 at −11.98. Nulls injected at 20 Oct 1987, 14 Oct 2008, 12 Mar 2020. Screen → question-formulating agent → three expert agents → consolidation agent → three-persona manager panel via AutoGen → human analyst briefing. "the terminal step, a briefing to a human analyst who makes the call, where my orchestrator has to emit the decision itself, so nothing here tells me how to close the loop." AGENTS &amp; ORCHESTRATION (exhaustive): One question-formulating agent; three expert agents (web research, curated institutional knowledge base, cross-checking against other reliable sources); one consolidation agent; a panel of three manager personas (financial market economist, macro economist, statistician) plus a moderator and a critic. Expert layer is explicitly extensible - "the diagram has a fourth empty box, so the expert set is meant to be configured per dataset rather than fixed." Critical axis distinction: "Park's three experts are heterogeneous by evidence source, web search, a curated knowledge base and an external vendor feed, and all three answer the same question. That is redundancy for verification rather than diversity for decision, and it means agreement between his agents is meant to be corroboration while agreement between mine would be a weak signal at best." State-conditioned influence: NONE. "as in TradingAgents and FinVision, there is no weight, no confidence scalar and no quantity anywhere that could be weighted. Consolidation is an LLM summarising free text." But note the one exception in behaviour: resolution by evidence type, below.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>All three experts returned Correct on all three genuine outliers, citing different evidence - the Fed's history and the Dow's 22.6% fall (1987), a CNN report of an 11.8% gain (2008), a CNBC 12% single-day drop (2020). "Three independent evidence paths converging is the demonstration's one clean result, and it is worth very little, because Black Monday, the October 2008 rebound and the COVID crash are three of the most documented days in market history and all three sit inside the backbone's pre-training. The framework is never shown an anomaly it could plausibly get wrong." On the injected nulls: web research returned Uncertain, institutional knowledge returned Uncertain, and the cross-checking agent retrieved the true values 236.83, 998.01 and 2711.02 from the API. "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." Consolidation: "Two Uncertains and one grounded Correct produced a Correct, not a hedge." LIMITATIONS (quoted): "There is no evaluation." "The hard case for alert triage is the one the paper concedes and does not attempt" - "That is the real operating regime for anomaly validation, a mid-sized move in a lightly covered name with no press coverage, and it is exactly what the CSE looks like. On this evidence I cannot tell how the framework behaves there, only that two of its three experts would abstain." "An unconditional z-score over 44 years is the wrong screen, and the choice of 10 hides the consequence." "The multi-agent structure is never shown to be necessary" - "the case for separating them rests entirely on the cross-check channel, which is a tool-access argument rather than an agent-architecture argument." "The discussion layer's objective makes disagreement a failure state" - "a panel that converges immediately has satisfied its objective, and the moderator and critic roles have no incentive structure that would reward dissent." And on the critic: "A critic role that only commends is a critic in name, and the layer that consumes the most tokens in the paper is the one that changes nothing about the output."</t>
+          <t>All three experts returned Correct on all three genuine outliers, citing different evidence - the Fed's history and the Dow's 22.6% fall (1987), a CNN report of an 11.8% gain (2008), a CNBC 12% single-day drop (2020). "Three paths converging is the demonstration's one clean result and it is worth very little, partly because only two of the three are actually independent, and mostly because Black Monday, the October 2008 rebound and the COVID crash are three of the most documented days in market history and all three sit inside the backbone's pre-training. The framework is never shown an anomaly it could plausibly get wrong." On the injected nulls: web research returned Uncertain, institutional knowledge returned Uncertain, and the cross-checking agent retrieved the true values 236.83, 998.01 and 2711.02 from the API. "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." Consolidation: "Two Uncertains and one grounded Correct produced a Correct, not a hedge." LIMITATIONS (quoted): "There is no evaluation." "The hard case for alert triage is the one the paper concedes and does not attempt" - "That is the real operating regime for anomaly validation, a mid-sized move in a lightly covered name with no press coverage, and it is exactly what the CSE looks like. On this evidence I cannot tell how the framework behaves there, only that two of its three experts would abstain." "An unconditional z-score over 44 years is the wrong screen, and the choice of 10 hides the consequence." "The multi-agent structure is never shown to be necessary" - "the case for separating them rests entirely on the cross-check channel, which is a tool-access argument rather than an agent-architecture argument." "The discussion layer's objective makes disagreement a failure state" - "a panel that converges immediately has satisfied its objective, and the moderator and critic roles have no incentive structure that would reward dissent." And on the critic: "A critic role that only commends is a critic in name, and the layer that consumes the most pages in the paper is the one that changes nothing about the output."</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
@@ -1054,7 +1054,7 @@
 EFFECT ON MAIN GAP: Two contributions. It supplies the only worked example of heterogeneous agents disagreeing and the disagreement being resolved correctly, and it was resolved by evidence type rather than vote - which raises a structural question about f(·): "I would put this to the supervisor as a question about whether w_{i,t} should be partly structural rather than entirely learned, and flag that a single anecdote in a paper with no evaluation is thin evidence for it." It also extends the no-weightable-quantity finding to a third, much smaller design.
 EFFECT ON SUB-GAP 1: None.
 EFFECT ON SUB-GAP 2: Indirect but concrete. The unconditional-σ critique is a direct argument for conditional volatility as the standardising quantity, and it produces the A_V/A_L interaction requirement: "In the CSE the correction is not sufficient on its own, because a stock that has not traded for several days produces a large printed return on its next trade that is a staleness artefact rather than a volatility event, and telling those apart is A_L's job. So an A_V flag on a thin name is uninterpretable without the A_L state alongside it, which is a case against treating the four channels as fully independent producers and an argument that at least this pair needs a defined interaction."
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of the no-mechanism-to-notice kind. Two of three experts contributed nothing on the only discriminating case and the architecture had no way to register it: "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." And the deliberation layer as dead weight: "the layer that consumes the most tokens in the paper is the one that changes nothing about the output." Student's cross-paper conclusion: "This is the same collapse as in TradingAgents' debate rounds but reached at much smaller scale and without a role hierarchy, so it does not look like an artefact of any one design."
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of the no-mechanism-to-notice kind. Two of three experts contributed nothing on the only discriminating case and the architecture had no way to register it: "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." And the deliberation layer as dead weight: "the layer that consumes the most pages in the paper is the one that changes nothing about the output." Student's cross-paper conclusion: "This is the same collapse as in TradingAgents' debate rounds but reached at much smaller scale and without a role hierarchy, so it does not look like an artefact of any one design."
 PROPOSED REVISION STATED IN THE NOTE: Two, both to the conditioning set, both flagged for the supervisor. On C_{i,t}: "The proposed refinement to C_{i,t} is that no evidence and low confidence are different states and should weight differently, which is a change to the conditioning set rather than a tuning detail, and it belongs in the discussion with the supervisor about what C_{i,t} actually is." On the form of f(·): "this argues that the weighting function should know something about the kind of evidence behind each agent's output, since direct market data underneath A_T, A_V and A_L and retrieved report text underneath A_F are not the same epistemic quality and collapsing them into one comparable confidence number assumes they are." And on the agent pool - a defined pairwise interaction rather than four independent producers: "an argument that at least this pair needs a defined interaction."</t>
         </is>
       </c>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>Page accuracy - Keywords Chipper 46.10, Summary 62.41, Prefix 67.38, against Base 512 at 68.09, Base 128 at 72.34, Base 256 at 73.05. "Every individual element-based index retrieves pages worse than every fixed-size baseline, which is the reverse of the paper's own summary." BLEU - 0.315 / 0.350 / 0.400 element against 0.181 / 0.231 / 0.250 baseline, "the worst element variant beats the best baseline on BLEU", and at aggregation 0.452 against 0.277, a 63% relative gain; ROUGE 0.514 against 0.455. Aggregation: Chipper 84.40 against Base 83.69, "a difference of one question out of 141", and it "exceeded GPT-4's token limit and yielded a non-effective Q&amp;A solution" so Table 5 has no aggregation rows. End to end (manual): Base 128 35.46, Base 256 36.88, Base 512 48.23, Keywords Chipper 53.19, Summary Chipper 51.77, Prefix &amp; Table Description Chipper 53.19. "No answer" column: 35.46, 25.53, 24.82, 22.70, 17.73, 20.57 - "Abstentions fall from 35.46% to as low as 17.73% while accuracy rises by about five points, so most of what better chunking buys is converting refusals into answers rather than converting wrong answers into right ones." Judge bias: trails manual by 6.38, 4.26, 6.39, 9.22, 8.04 and 12.06 points, "so the better the system the larger the understatement", with the named failure mode "a model correctly deriving 39.73% with the full calculation against a gold answer of '39.7%'", and it reorders the element variants. LIMITATIONS (quoted): "141 questions, one run, no dispersion, and the headline margins do not clear sampling error" - "At 141 cases the binomial standard error near 50% is about 4.2 points, so a difference between two configurations carries a 95% interval of roughly ±11.7 points. The 4.96-point Q&amp;A gain from Base 512 to the best element configuration sits well inside that, and the 0.71-point retrieval gain is one question." "The authors are evaluating their own commercial product, and the prose reads the tables more favourably than the numbers support" - "the two places where the summary overstates the tables... both run the same direction, and that is the pattern to read for." "The cost comparison is one-sided." "The benchmark was silently reduced and then compared against its own published numbers." "The retrieval metrics are coarse and none of them shows ranking position" - "There is no precision@k and no mean reciprocal rank anywhere, so nothing in the paper says whether the right chunk arrived first or tenth, which is the quantity that actually determines what fits in a generator prompt." "Table handling is the design's most distinctive rule and the least evidenced."</t>
+          <t>Page accuracy - Keywords Chipper 46.10, Summary 62.41, Prefix 67.38, against Base 512 at 68.09, Base 128 at 72.34, Base 256 at 73.05. "Every individual element-based index retrieves pages worse than every fixed-size baseline, which is the reverse of the paper's own summary." BLEU - 0.315 / 0.350 / 0.400 element against 0.181 / 0.231 / 0.250 baseline, "the worst element variant beats the best baseline on BLEU", and at aggregation 0.452 against 0.277, a 63% relative gain; ROUGE 0.514 against 0.455. Aggregation: Chipper 84.40 against Base 83.69, "a difference of one question out of 141", and it "exceeded GPT-4's token limit and yielded a non-effective Q&amp;A solution" so Table 5 has no aggregation rows. End to end (manual): Base 128 35.46, Base 256 36.88, Base 512 48.23, Keywords Chipper 53.19, Summary Chipper 51.77, Prefix &amp; Table Description Chipper 53.19. "No answer" column: 35.46, 25.53, 24.82, 22.70, 17.73, 20.57 - "Abstentions fall from 35.46% to as low as 17.73% while accuracy rises by about five points, so most of what better chunking buys is converting refusals into answers rather than converting wrong answers into right ones." Judge bias: trails manual by 6.38, 4.26, 6.39, 9.22, 7.80 and 12.06 points, "so the better the system the larger the understatement", with the named failure mode "a model correctly deriving 39.73% with the full calculation against a gold answer of '39.7%'", and it reorders the element variants. LIMITATIONS (quoted): "141 questions, one run, no dispersion, and the headline margins do not clear sampling error" - "At 141 cases the binomial standard error near 50% is about 4.2 points, so a difference between two configurations carries a 95% interval of roughly ±11.7 points. The 4.96-point Q&amp;A gain from Base 512 to the best element configuration sits well inside that, and the 0.71-point retrieval gain is one question." "The authors are evaluating their own commercial product, and the prose reads the tables more favourably than the numbers support" - "the two places where the summary overstates the tables... both run the same direction, and that is the pattern to read for." "The cost comparison is one-sided." "The benchmark was silently reduced and then compared against its own published numbers." "The retrieval metrics are coarse and none of them shows ranking position" - "There is no precision@k and no mean reciprocal rank anywhere, so nothing in the paper says whether the right chunk arrived first or tenth, which is the quantity that actually determines what fits in a generator prompt." "Table handling is the design's most distinctive rule and the least evidenced."</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="S28" s="11" t="inlineStr">
         <is>
-          <t>"71.60% annualised and 405.34% total against the best baseline FinAgent at 53.54% and 261.98%, with Sharpe 2.41 against FinGPT's 1.93, Calmar 11.02 against 7.64 and Sortino 58.00 against 39.57, improvements of 33.75%, 54.72%, 24.49%, 44.28% and 46.58% respectively. Maximum drawdown is 14.21% against FinGPT's 17.08%." Buy-and-hold Bitcoin over the same window: 43.97% total return with 76.63% maximum drawdown. Single-asset (no hedging): "about 210% on Bitcoin, 160% on AAPL and 9% on the yuan, against FinAgent's roughly 135% and FinMem's 120% on AAPL." Ablation: single modules 43.88% (experience sharing), 45.58% (budget allocation), 40.97% (extreme market); pairs 50.68%, 44.57%, 59.81%; full system 71.60%. Removing budget allocation drops to 44.57%; removing extreme-market raises drawdown to 24.44% and cuts Sharpe to 1.93. Memory: "Removing it drops annualised return by 57.71% and Sharpe by 39.3%, larger than the effect of removing any one coordination meeting." Backbone sweep: "ChatGLM-6B reports Sharpe 2.88, Calmar 12.26, Sortino 66.64, drawdown 9.19% and volatility 0.78%, every one better than GPT-4's." Diversity: effective number of bets 1.53 against a ceiling of 3; entropy 3.13. Cost: fifteen dollars of API spend over three years; 36 extreme-market sessions fired over nine months. LIMITATIONS (quoting the note): "The expected returns feeding the optimiser are LLM outputs with no calibration, which makes the mean-variance solve look more quantitative than it is.… There is no check that an analyst claiming 12% is better calibrated than one claiming 8%, no interval, and no record of realised against predicted. The optimiser is exact arithmetic over inputs of unknown quality, and a well-specified objective over uncalibrated inputs inherits the uncertainty of the inputs while hiding it behind the precision of the output. This is the sharpest version of the comparable-confidence problem I have seen posed in any paper I have read, and the paper does not pose it." "The allocation is over assets, not over agents, and the two coincide here only because the mapping is one to one.… it means the paper never has to answer how much weight to give an agent whose view overlaps another's, how to combine disagreeing views on the same asset, or what to do when an agent's channel is uninformative. On this design those questions cannot arise, so nothing here bears on them either way." "Three assets is a thin basis for a diversification claim and the paper's own diversity metric says so… the 'balanced-aware' claim in the title rests on two numbers whose definitions are not given." "No execution friction of any kind." "Three hyperparameters that control the system's behaviour are never given values." "Single runs, no dispersion, no significance testing." Internal contradiction: "the full-system drawdown in this table is 8.68% against 14.21% in Table 1, a direct contradiction between two tables in the same paper for the headline risk metric." And: "on these numbers adding the budget conference buys return by taking on drawdown, which is a coherent result but not the monotone one the discussion describes."</t>
+          <t>"71.60% annualised and 405.34% total against the best baseline FinAgent at 53.54% and 261.98%, with Sharpe 2.41 against FinGPT's 1.93, Calmar 11.02 against 7.64 and Sortino 58.00 against 39.57, improvements of 33.75%, 54.72%, 24.49%, 44.28% and 46.58% respectively. Maximum drawdown is 14.21% against FinGPT's 17.08%." Buy-and-hold Bitcoin over the same window: 43.97% total return with 76.63% maximum drawdown. Single-asset (no hedging): "about 210% on Bitcoin, 160% on AAPL and 9% on the yuan, against FinAgent's roughly 135% and FinMem's 120% on AAPL." Ablation: single modules 43.88% (experience sharing), 45.58% (budget allocation), 40.97% (extreme market); pairs 50.68%, 44.57%, 59.81%; full system 71.60%. Removing budget allocation drops to 44.57%; removing extreme-market raises drawdown to 24.44% and cuts Sharpe to 1.93. Memory: activating it raises annualised return by 57.71% and Sharpe by 39.3% against the configuration without it, which implies a no-retrieval annualised return near 45.4% and so a relative drop of 36.6%, "marginally smaller than the 37.7% drop from removing the budget conference, 71.60% to 44.57%". The paper states that "the BAC module has the greatest impact on returns". Backbone sweep: "ChatGLM-6B reports Sharpe 2.88, Calmar 12.26, Sortino 66.64, drawdown 9.19% and volatility 0.78%, every one better than GPT-4's." Diversity: effective number of bets 1.53 against a ceiling of 3; entropy 3.13. Cost: fifteen dollars of API spend over three years; 36 extreme-market sessions fired over nine months. LIMITATIONS (quoting the note): "The expected returns feeding the optimiser are LLM outputs with no calibration, which makes the mean-variance solve look more quantitative than it is.… There is no check that an analyst claiming 12% is better calibrated than one claiming 8%, no interval, and no record of realised against predicted. The optimiser is exact arithmetic over inputs of unknown quality, and a well-specified objective over uncalibrated inputs inherits the uncertainty of the inputs while hiding it behind the precision of the output. This is the sharpest version of the comparable-confidence problem I have seen posed in any paper I have read, and the paper does not pose it." "The allocation is over assets, not over agents, and the two coincide here only because the mapping is one to one.… it means the paper never has to answer how much weight to give an agent whose view overlaps another's, how to combine disagreeing views on the same asset, or what to do when an agent's channel is uninformative. On this design those questions cannot arise, so nothing here bears on them either way." "Three asset classes is a thin basis for a diversification claim, and the paper's own diversity metrics cannot be used to check it… the 'balanced-aware' claim in the title rests on two numbers whose definitions are not given." "No execution friction of any kind." "Three hyperparameters that control the system's behaviour are never given values." "Single runs, no dispersion, no significance testing." Internal contradiction: "the full-system drawdown in this table is 8.68% against 14.21% in Table 1, a direct contradiction between two tables in the same paper for the headline risk metric." And: "on these numbers adding the budget conference buys return by taking on drawdown, which is a coherent result but not the monotone one the discussion describes."</t>
         </is>
       </c>
       <c r="T28" s="11" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="U28" s="11" t="inlineStr">
         <is>
-          <t>"It is the existence proof that the orchestration layer can be a solved optimisation rather than a prompt, and it also shows where that stops working for me… What does not carry over is the one-to-one mapping. My technical, fundamental and volatility agents all look at the same CSE universe, so their weights are influence over a shared decision rather than capital across separate books, and I cannot collapse the two the way this paper does. That difference is the cleanest statement I have of what my weighting function has to do that this one does not." "The conditioning comparison is now a three-way contrast and this paper sits in the middle of it. MacroHFT conditions continuously on trend slope and a realised-volatility tertile but over six identical sub-agents. TradingAgents conditions on nothing. HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies… which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited. My contribution is the continuous version, weights that are a function of liquidity and persistence at every step rather than a scheduled re-solve punctuated by a threshold alarm, and I should put that three-way contrast in the review chapter as a table." "The event-triggered conference is the most transferable mechanism here and it solves a cost problem I have not yet sized… the lesson is to make the costly deliberation conditional on a state trigger and keep the per-day path lightweight. The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." "each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function, reported as a reliability curve per agent, so that the orchestrator combines calibrated probabilities rather than self-reported numbers. That is a component of the build I had listed as an open question and this paper is the reason to promote it to a work item." Entropy diagnostic "needs its formula stated in the text, its range given, and a second concentration measure beside it, or it will be as uninterpretable as theirs." Backbone check to be run and reported either way. "The hedging mechanism itself does not port to the CSE and I should say so rather than borrowing the framing… the balance my system can offer has to come from conditioning exposure on liquidity and volatility state instead."</t>
+          <t>"It is the existence proof that the orchestration layer can be a solved optimisation rather than a prompt, and it also shows where that stops working for me… What does not carry over is the one-to-one mapping. My technical, fundamental and volatility agents all look at the same CSE universe, so their weights are influence over a shared decision rather than capital across separate books, and I cannot collapse the two the way this paper does. That difference is the cleanest statement I have of what my weighting function has to do that this one does not." "The conditioning comparison is now a three-way contrast and this paper sits in the middle of it. MacroHFT conditions continuously on trend slope and a realised-volatility tertile but over six identical sub-agents. TradingAgents conditions on nothing. HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies… which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited. My contribution is the continuous version, weights that are a function of liquidity and persistence at every step rather than a scheduled re-solve punctuated by a threshold alarm, and I should put that three-way contrast in the review chapter as a table." "The event-triggered conference is the most transferable mechanism here and it solves a cost problem I have not yet sized… the lesson is to make the costly deliberation conditional on a state trigger and keep the per-day path lightweight. The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." "each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function, reported as a reliability curve per agent, so that the orchestrator combines calibrated probabilities rather than self-reported numbers. That is a component of the build I had listed as an open question and this paper is the reason to promote it to a work item." Entropy diagnostic "needs its formula stated in the text, its logarithm base and range given, the asset set it is computed over named, and a second concentration measure beside it, or it will be as uninterpretable as theirs." Backbone check to be run and reported either way. "The hedging mechanism itself does not port to the CSE and I should say so rather than borrowing the framing… the balance my system can offer has to come from conditioning exposure on liquidity and volatility state instead."</t>
         </is>
       </c>
       <c r="V28" s="11" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="S37" s="11" t="inlineStr">
         <is>
-          <t>"SOPS takes the highest cumulative return on all four datasets ... 14.8585 against AOLNPM's 10.1757 on MSCI, $9.1526 \times 10^6$ against OLMAR-1's $8.2320 \times 10^6$ on NYSE-N, 560.4279 against AOLNPM's 321.3223 on TSE, and 6.6460 against BCRP's 5.6676 on NASTDA. The NYSE-N margin is 11% over the runner-up on a 25-year horizon, while the TSE margin is 74%." Ablation on MSCI: "EMA-NPM reaches 13.0259, SEMA-NPM 14.0270, SEMA-NPMRP 12.2729 and SOPS 14.8585," with ratios EMA-NPM 0.1096/0.1604/0.1710, SEMA-NPM 0.1137/0.1683/0.1790, SEMA-NPMRP 0.1106/0.1660/0.1745 ($\sigma(r)$ 0.0244, the lowest), SOPS 0.1163/0.1724/0.1841. Concentration: "SOPS holds two or three of 24 assets for most of the horizon, never more than six, and averages 4.6." Sensitivity: "$\zeta$ from 0.1 to 0.2 changes cumulative return by at most 0.60% with an average relative change of 0.33%, $c$ from 3.5 to 5.5 by at most 0.77%..., $\eta$ from 0.0001 to 0.1 by at most 0.68%..., and window sizes from 25 to 38 move average prediction error by 0.38%, 0.16%, 0.43% and 0.41%." LIMITATIONS (quoted): (1) "The state-switching contribution is never isolated from how often it fires ... there is no way to tell whether the 14.0270 to 14.8585 improvement comes from switching to NPMRP at the right moments or from switching so rarely that SOPS is mostly NPM with occasional de-risking." (2) "A paper about exact transaction cost computation never varies the transaction cost rate." (3) "Linear proportional cost is the whole cost model, so 'exact' is exact within a form that omits the costs that matter in a thin book. There is no bid-ask spread, no market impact, no partial fill, no queue position and no volume constraint ... it means the exactness result is exactness about commission, and the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper." (4) "No walk-forward, no seeds, no significance tests, and per-dataset window sizes with no selection procedure." (5) "Practicality is claimed and never measured." (6) "The prediction and allocation stages share a single point of failure ... when SEMA mispredicts, both models fail together and the router has nothing to route to."</t>
+          <t>"SOPS takes the highest cumulative return on all four datasets ... 14.8585 against AOLNPM's 10.1757 on MSCI, $9.1526 \times 10^6$ against OLMAR-1's $8.2320 \times 10^6$ on NYSE-N, 560.4279 against AOLNPM's 321.3223 on TSE, and 6.6460 against BCRP's 5.6676 on NASTDA. The NYSE-N margin is 11% over the runner-up on a 25-year horizon, while the TSE margin is 74%." Ablation on MSCI: "EMA-NPM reaches 13.0259, SEMA-NPM 14.0270, SEMA-NPMRP 12.2729 and SOPS 14.8585," with ratios EMA-NPM 0.1096/0.1604/0.1710, SEMA-NPM 0.1137/0.1683/0.1790, SEMA-NPMRP 0.1106/0.1660/0.1745 ($\sigma(r)$ 0.0244, the lowest), SOPS 0.1163/0.1724/0.1841. Concentration: "SOPS holds two or three of the 24 MSCI assets for most of the horizon and never more than six." The paper reports an average of 4.6 selected assets at eta = 1000 and only across periods in which more than one asset is selected, so it is not the unconditional average. Sensitivity: "$\zeta$ from 0.1 to 0.2 changes cumulative return by at most 0.60% with an average relative change of 0.33%, $c$ from 3.5 to 5.5 by at most 0.77%..., $\eta$ from 0.0001 to 0.1 by at most 0.68%..., and window sizes from 25 to 38 move average prediction error by 0.38%, 0.16%, 0.43% and 0.41%." LIMITATIONS (quoted): (1) "The state-switching contribution is never isolated from how often it fires ... there is no way to tell whether the 14.0270 to 14.8585 improvement comes from switching to NPMRP at the right moments or from switching so rarely that SOPS is mostly NPM with occasional de-risking." (2) "A paper about exact transaction cost computation never varies the transaction cost rate." (3) "Linear proportional cost is the whole cost model, so 'exact' is exact within a form that omits the costs that matter in a thin book. There is no bid-ask spread, no market impact, no partial fill, no queue position and no volume constraint ... it means the exactness result is exactness about commission, and the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper." (4) "No walk-forward, no seeds, no significance tests, and per-dataset window sizes with no selection procedure." (5) "Practicality is claimed and never measured." (6) "The prediction and allocation stages share a single point of failure ... when SEMA mispredicts, both models fail together and the router has nothing to route to."</t>
         </is>
       </c>
       <c r="T37" s="11" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="S38" s="11" t="inlineStr">
         <is>
-          <t>"HLOB outperforms the 9 alternatives in 73.3% of the 15 stock cases at $H_{\Delta\tau} = 10$, 60% at $H_{\Delta\tau} = 50$, and 33% at $H_{\Delta\tau} = 100$." Tick-class table (F1 / MCC / $p_\text{T}$): small-tick 0.42/0.16/0.11 at $H_{10}$, 0.36/0.09/0.07 at $H_{50}$, 0.32/0.05/0.05 at $H_{100}$; medium-tick 0.41/0.16/0.14, 0.40/0.11/0.10, 0.35/0.06/0.07; large-tick 0.48/0.33/0.10, 0.58/0.38/0.14, 0.52/0.30/0.15. "An MCC of 0.05 on small-tick stocks at the longest horizon is a model that has essentially stopped predicting, while 0.30 on large-tick stocks at the same horizon is a model still working." MI levels: "average non-normalized MI runs from 0.26 for GOOG to 0.74 for IBM" (small-tick) versus "0.62 for ORCL to 1.18 for BAC" (large-tick) with "a clean three-group hierarchy." Against DeepLOB: "At $H_{\Delta\tau} = 10$ the average F1 gain is 0.03, 0.02 and 0.003 for small-, medium- and large-tick stocks, with MCC gains of 0.04, 0.04 and 0.02; at $H_{\Delta\tau} = 50$ the F1 gains rise to 0.05, 0.05 and 0.01 and the MCC gains to 0.06, 0.02 and 0.03." Parameter count discrepancy: "Table 3 lists HLOB at $1.8\times10^4$ trainable parameters ... The per-layer counts in Section 4.2 ... sum to roughly $1.8\times10^5$." LIMITATIONS (quoted): (1) "No statistical testing appears anywhere, and the headline claim is a win count ... it means the 0.003 F1 gain over DeepLOB on large-tick stocks and the 0.06 MCC gain on small-tick stocks are presented with identical evidential weight." (2) "Nothing isolates the TMFG, so the central claim about higher-order topological priors rests on a model-versus-model comparison ... without one, the claim that the mutual-information structure is what produces the gain is the paper's interpretation of a result rather than a result. This is the limitation I would raise first if I were reviewing it." (3) "The reported parameter count does not reconcile with the architecture description." (4) "The label threshold is absolute while the grouping variable is relative, which partially confounds the tick-size finding ... Some portion of 'large-tick books are more learnable' is a statement about the relationship between the label threshold and the spread rather than about the spatial structure of the book." (5) "The structure is static in a paper about persistence, and the authors say so ... it is a plausible alternative explanation for the horizon degradation, since a structure estimated as a 40-day average will describe a longer horizon worse for exactly the stocks whose books drift most, which is the small-tick group." (6) "Event-time horizons, no execution model, and one venue ... no fees, no queue position, no partial fills, no market impact."</t>
+          <t>"HLOB outperforms the 9 alternatives in 73.3% of the 15 stock cases at $H_{\Delta\tau} = 10$, 60% at $H_{\Delta\tau} = 50$, and 33% at $H_{\Delta\tau} = 100$." Tick-class table (F1 / MCC / $p_\text{T}$): small-tick 0.42/0.16/0.11 at $H_{10}$, 0.36/0.09/0.07 at $H_{50}$, 0.32/0.05/0.05 at $H_{100}$; medium-tick 0.41/0.16/0.14, 0.40/0.11/0.10, 0.35/0.06/0.07; large-tick 0.48/0.33/0.10, 0.58/0.38/0.14, 0.52/0.30/0.15. "An MCC of 0.05 on small-tick stocks at the longest horizon is a model that has essentially stopped predicting, while 0.30 on large-tick stocks at the same horizon is a model still working." MI levels: "average non-normalized MI runs from 0.26 for GOOG to 0.74 for IBM" (small-tick) versus "0.62 for ORCL to 1.18 for BAC" (large-tick) with "a clean three-group hierarchy." Against DeepLOB: "At $H_{\Delta\tau} = 10$ the average F1 gain is 0.03, 0.02 and 0.003 for small-, medium- and large-tick stocks, with MCC gains of 0.04, 0.04 and 0.02; at $H_{\Delta\tau} = 50$ the F1 gains rise to 0.05, 0.05 and 0.01 and the MCC gains to 0.06, 0.02 and 0.03." Parameter count discrepancy: "Table 3 lists HLOB at $1.8\times10^4$ trainable parameters ... The per-layer counts in Section 4.2 ... sum to roughly $1.8\times10^5$." LIMITATIONS (quoted): (1) "No statistical testing appears anywhere, and the headline claim is a win count ... it means the 0.003 F1 gain over DeepLOB on large-tick stocks and the 0.04 MCC gain on small-tick stocks, both at the H-delta-tau = 10 horizon, are presented with identical evidential weight." (2) "Nothing isolates the TMFG, so the central claim about higher-order topological priors rests on a model-versus-model comparison ... without one, the claim that the mutual-information structure is what produces the gain is the paper's interpretation of a result rather than a result. This is the limitation I would raise first if I were reviewing it." (3) "The reported parameter count does not reconcile with the architecture description." (4) "The label threshold is absolute while the grouping variable is relative, which partially confounds the tick-size finding ... Some portion of 'large-tick books are more learnable' is a statement about the relationship between the label threshold and the spread rather than about the spatial structure of the book." (5) "The structure is static in a paper about persistence, and the authors say so ... it is a plausible alternative explanation for the horizon degradation, since a structure estimated as a 40-day average will describe a longer horizon worse for exactly the stocks whose books drift most, which is the small-tick group." (6) "Event-time horizons, no execution model, and one venue ... no fees, no queue position, no partial fills, no market impact."</t>
         </is>
       </c>
       <c r="T38" s="11" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="S43" s="11" t="inlineStr">
         <is>
-          <t>reported "MAPE of 3.9% and therefore strong short-term forecasting performance". Model selection: "ARMA(2,1) wins at AIC 11.64805 against ARMA(1,1) at 11.64806, a difference of 0.00001 in EViews' per-observation units, which on 2,362 observations is 0.024 absolute AIC units, far inside the range where the two models are indistinguishable." Fit: "R² = 0.083698 falling to an adjusted 0.082532". Forecast degeneracy: "the day-on-day increments run 3.240, 2.337, 2.415, 2.449, 2.446 and then settle at 2.44516 for every remaining day, which is μ = 2.445160 to five decimals. So the entire three-month forecast path is generated by a drift term the paper's own Table 3 reports as insignificant at p = 0.2835." Direction: "Predictions rise 54.45 points across the 23 trading days while the index fell 669.93 points, from 12,076.49 to 11,406.56, a decline of 5.55%." Note's recomputation: "A no-change forecast beats it on every day of the test window... a mean absolute percentage error of 2.57% for the random walk against 3.62% for the ARIMA, RMSE of 346.10 against 465.40, and the random walk is closer to the actual on 23 of 23 days." Theil U2 on Table 4: "1.345". LIMITATIONS (quoting the note): "Two claims in this paper are contradicted by its own tables." "The white noise conclusion is contradicted by the printed correlogram... Figure 3 reports p = 0.039 at lag 3, p = 0.001 at lag 4, and p = 0.000 continuously from lag 5 to lag 36, ending at Q(36) = 185.20... The Box-Jenkins adequacy criterion is failed and reported as passed, which means the model was never actually validated and the significance of the AR and MA terms cannot be taken at face value either." "MA(1) at 0.301976 carries almost all of the fit, and its standard error of 0.007985 is implausibly small." "One forecast origin, no benchmark, no rolling evaluation." "Two of the literature review's supporting citations do not say what they are cited for." "Univariate and index-level throughout, which the authors acknowledge."</t>
+          <t>reported "MAPE of 3.9% and therefore strong short-term forecasting performance". Model selection: "ARMA(2,1) wins at AIC 11.64805 against ARMA(1,1) at 11.64806, a difference of 0.00001 in EViews' per-observation units, which on 2,362 observations is 0.024 absolute AIC units, far inside the range where the two models are indistinguishable." Fit: "R² = 0.083698 falling to an adjusted 0.082532". Forecast degeneracy: "the day-on-day increments run 3.240, 2.337, 2.415, 2.449, 2.446 and then settle at 2.44516 for every remaining day, which is μ = 2.445160 to five decimals. So the entire three-month forecast path is generated by a drift term the paper's own Table 3 reports as insignificant at p = 0.2835." Direction: "Predictions rise 54.45 points across the 23 trading days while the index fell 669.93 points, from 12,076.49 to 11,406.56, a decline of 5.55%." Note's recomputation: "A no-change forecast beats it on every day of the test window... a mean absolute percentage error of 2.57% for the random walk against 3.62% for the ARIMA, RMSE of 346.10 against 465.40, and the random walk is closer to the actual on 23 of 23 days." Theil U2 on Table 4: "1.345". LIMITATIONS (quoting the note): "Two claims in this paper are contradicted by its own tables." "The white noise conclusion is contradicted by the printed correlogram... Figure 3 reports p = 0.039 at lag 3, p = 0.001 at lag 4, and p = 0.000 continuously from lag 5 to lag 36, ending at Q(36) = 185.20... The Box-Jenkins adequacy criterion is failed and reported as passed, which means the model was never actually validated and the significance of the AR and MA terms cannot be taken at face value either." "MA(1) at 0.301976 carries almost all of the fit, and its standard error of 0.007985 is implausibly small." "One forecast origin, no benchmark, no rolling evaluation." "Three of the literature review's supporting citations do not say what they are cited for, and a fourth has no reference at all." "Univariate and index-level throughout, which the authors acknowledge."</t>
         </is>
       </c>
       <c r="T43" s="11" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="S44" s="11" t="inlineStr">
         <is>
-          <t>"Without scaling at C = 0.01% it reaches Sharpe 1.858 and Sortino 3.135 against the best baseline's 1.228 and 2.932, with scaling at the same rate 1.962 and 3.322 against 1.579 and 2.629, and with scaling at C = 0.1% 1.403 and 2.327 against Allocation 4's 1.299 and 2.172. So a tenfold increase in the cost rate takes the Sharpe advantage from roughly 24% over the best baseline down to 8%." Win profile: "DLS never has the highest percentage of positive returns in any of the three blocks, 0.537 against MV's 0.562, 0.559 against Allocation 4's 0.565 and 0.547 against Allocation 4's 0.559, but it has the highest average-gain-to-average-loss ratio in all three, 1.518, 1.375 and 1.272." Scaler attribution: "Allocation 1 goes from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120 purely from the scaler, against DLS's 1.858 to 1.962." Drawdown: "in the scaled block DLS records an MDD of 0.123, fifth of eight... and at C = 0.1% it is fifth again at 0.125, so for a method whose stated appeal is the confidence to hold through hard times it is mid-table on the one metric that measures holding through hard times." Cost collapse: "DWP posts Sharpe 0.493 unscaled, 0.818 scaled, and −0.753 at C = 0.1% with an MDD of 0.627 and an expected return of −0.083." LIMITATIONS (quoting the note): "There is no seed averaging, no walk-forward significance testing and no reported hyperparameter search, and the paper frames the last of these as a virtue... Every number in Table 1 is one training run of one architecture on one fixed sequence." "The test window is a bull market and the single crisis in it is handled by a component that was not trained... I cannot say the learned policy handles regime change, because the design does not separate the policy's contribution from the scaler's. An unscaled run through Q1 2020 would have answered it and is not reported." "How L_T is computed during training is never stated, and it changes what the model optimises... A Sharpe estimated over 64 daily observations is an extremely noisy quantity... this is a reproducibility hole sitting directly on the paper's single contribution." "The cost model is flat and proportional, and the asset choice removes execution friction from the problem by construction." "The architecture claims and the RL framing are both asserted without a baseline."</t>
+          <t>"Without scaling at C = 0.01% it reaches Sharpe 1.858 and Sortino 3.135 against Allocation 4's 1.228 and 2.932, with scaling at the same rate 1.962 and 3.322 against 1.579 and 2.629, and with scaling at C = 0.1% 1.403 and 2.327 against Allocation 4's 1.299 and 2.172. So a tenfold increase in the cost rate takes the Sharpe advantage from roughly 24% over the best baseline down to 8%." Win profile: "DLS never has the highest percentage of positive returns in any of the three blocks, 0.537 against MV's 0.562, 0.559 against the 0.565 held jointly by Allocation 4 and MD and 0.547 against Allocation 4's 0.559, but it has the highest average-gain-to-average-loss ratio in all three, 1.518, 1.375 and 1.272." Scaler attribution: "Allocation 1 goes from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120 purely from the scaler, against DLS's 1.858 to 1.962." Drawdown: "in the scaled block DLS records an MDD of 0.123, fifth of eight... and at C = 0.1% it is fifth again at 0.125, so for a method whose stated appeal is the confidence to hold through hard times it is mid-table on the one metric that measures holding through hard times." Cost collapse: "DWP posts Sharpe 0.493 unscaled, 0.818 scaled, and −0.753 at C = 0.1% with an MDD of 0.627 and an expected return of −0.083." LIMITATIONS (quoting the note): "There is no seed averaging, no walk-forward significance testing and no reported hyperparameter search, and the paper frames the last of these as a virtue... Every number in Table 1 is one training run of one architecture on one fixed sequence." "The test window is a bull market and the single crisis in it is handled by a component that was not trained... I cannot say the learned policy handles regime change, because the design does not separate the policy's contribution from the scaler's. An unscaled run through Q1 2020 would have answered it and is not reported." "How L_T is computed during training is never stated, and it changes what the model optimises... A Sharpe estimated over 64 daily observations is an extremely noisy quantity... this is a reproducibility hole sitting directly on the paper's single contribution." "The cost model is flat and proportional, and the asset choice removes execution friction from the problem by construction." "The architecture claims and the RL framing are both asserted without a baseline."</t>
         </is>
       </c>
       <c r="T44" s="11" t="inlineStr">
@@ -7928,7 +7928,7 @@
       <c r="P57" s="11" t="inlineStr">
         <is>
           <t>Liquidity appears as a predictor family and is absent as a friction, and the gap between those two facts is what the note exploits. The liquidity group (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) is one of the three dominant families across every method. But: "There are no transaction costs anywhere in the paper, and the turnover figures make that decisive rather than cosmetic." The best strategy, an equal-weighted decile spread on NN4 forecasts, returns 3.3% per month, 39.0% annualised, at an out-of-sample Sharpe of 2.35, with monthly turnover of 114.08%. Networks run 110.87% to 114.08%, elastic net 143.61% and OLS-3 156.78%, against 22.87% for a size decile spread. The authors note that high turnover is unsurprising given the dominance of price-trend predictors, "and then stop."
-Two things in their own results indicate the size of what is left out. Value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, "so the gap between the paper's two weighting schemes is larger than the gap between most of its methods." And the universe retains sub-$5 stocks by explicit choice. The paper offers the higher top-1,000 R^2, 0.72% against 0.46%, as reassurance that machine learning is not merely picking up small-scale inefficiencies driven by illiquidity, "but the result carrying the economic claim is an equal-weighted spread over the whole board, and both cannot be load-bearing at once."</t>
+Two things in their own results indicate the size of what is being left out. Value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, "so the gap between the paper's two weighting schemes is larger than the gap between most of its methods." And the universe retains sub-$5 stocks by explicit choice. The paper offers the higher top-1,000 R^2, 0.72% against 0.46%, as reassurance that machine learning is not merely picking up small-scale inefficiencies driven by illiquidity, "but the result carrying the economic claim is an equal-weighted spread over the whole board, and both cannot be load-bearing at once."</t>
         </is>
       </c>
       <c r="Q57" s="11" t="inlineStr">
@@ -7998,7 +7998,7 @@
 Then the line. Three differences separate their construction from mine, and all three are in w(i,t) = f(L_t, V_t, P_t, C_{i,t}): their interaction weights are estimated once per annual refit, so they do not vary with measured market state at decision time, only with the value of the macro variable plugged into a fixed coefficient; they are a function of macro variables rather than of any measured reliability of the signal, so there is no C_{i,t} analogue anywhere in the model; and no channel can go absent, "because a missing characteristic is median-imputed rather than down-weighted". The note puts the whole claim on that last point: "The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line." Median imputation is the exact anti-pattern my abstention channel exists to replace - it substitutes a plausible value for a missing one and the downstream model cannot tell the difference, whereas abstention makes absence visible to the aggregator.
 It also supplies the evidence base for two of the four conditioning terms. Liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) and risk (total volatility, idiosyncratic volatility, beta, beta squared) are two of the three dominant families across every one of eleven method families on a ~30,000-stock, 60-year panel. "That is a far larger evidence base for those two conditioning inputs than the CSE-specific work in [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] or the Granger result at p = 0.0041 from volume to ASPI, and it composes with both." The macro rejection also survives: market-level stock variance is given little weight by any method and essentially none by the networks, consistent with the thin ARDL result in [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]] that already got the macro block rejected. The one live challenge is aggregate book-to-market - critical for every model, 28.57% for NN1 and 43.46% for GLM - and the honest response recorded in the note is to "test it against an ASPI-level valuation ratio rather than dismiss it on the strength of a rejection aimed at different variables."
 One further point that bears directly on the main gap and that the paper declined to test: Figure 3 shows model complexity drifting across the test period - elastic net selecting fewer than five features in the first decade and 20 to 40 after 2000, GBRT moving from roughly 20 features to 30 - and the authors explain it by a growing cross section and improving data coverage. "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." So the paper leaves my central hypothesis open on evidence it had in hand, which is a better position for me than either confirming or refuting it would have been.
-EFFECT ON SUB-GAP 1: This is the strongest available illustration of why cost belongs inside the objective rather than after it, and I would cite it as the reference case. "A strategy turning over 113% of its book monthly, concentrated in price-trend signals, on a universe that deliberately includes the smallest and least liquid names, reported at Sharpe 2.35 with no cost deduction and no participation-rate analysis, is the reference case for my cost sub-gap." Two details make it sharper than a generic "they ignored costs" complaint. First, the value-weighted collapse - NN3 from 2.32 to 1.25, OLS-3 from 0.89 to 0.27 - "is itself a partial, unacknowledged cost estimate and I should cite it that way": moving weight away from the small end halves the Sharpe before a single basis point of spread is charged, which is a lower bound on what liquidity is doing to the result. Second, the internal tension: the paper offers the top-1,000 R^2 of 0.72% against 0.46% on the bottom 1,000 as reassurance that the result is not driven by small-cap illiquidity, while the headline economic result is an equal-weighted spread over the whole board - "both cannot be load-bearing at once."
+EFFECT ON SUB-GAP 1: This is the strongest available illustration of why cost belongs inside the objective rather than after it, and I would cite it as the reference case. "A strategy turning over 114% of its book monthly, concentrated in price-trend signals, on a universe that deliberately includes the smallest and least liquid names, reported at Sharpe 2.35 with no cost deduction and no participation-rate analysis, is the reference case for my cost sub-gap." Two details make it sharper than a generic "they ignored costs" complaint. First, the value-weighted collapse - NN3 from 2.32 to 1.25, OLS-3 from 0.89 to 0.27 - "is itself a partial, unacknowledged cost estimate and I should cite it that way": moving weight away from the small end halves the Sharpe before a single basis point of spread is charged, which is a lower bound on what liquidity is doing to the result. Second, the internal tension: the paper offers the top-1,000 R^2 of 0.72% against 0.46% on the bottom 1,000 as reassurance that the result is not driven by small-cap illiquidity, while the headline economic result is an equal-weighted spread over the whole board - "both cannot be load-bearing at once."
 Applied to the CSE this is not implementable at any size. "On the CSE, where Dissanayake and Nanayakkara find unexpected illiquidity shocks depressing returns by -0.084 to -0.097 and small caps more than large, that turnover is not implementable at any size, which is the concrete argument for sweeping participation rate against daily volume rather than charging a flat spread, as [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] both do in their different ways." So the paper does not close any part of Sub-gap 1 - it has no friction model at all - but it supplies the clearest demonstration of the failure the sub-gap names, from a source that is hard to dismiss.
 EFFECT ON SUB-GAP 2: Limited, and I should not overclaim it. The paper has no volatility process, no persistence estimate, no decay schedule and no volatility targeting; volatility enters only as a cross-sectional predictor. So it neither closes nor narrows Sub-gap 2. What it contributes is one piece of supporting evidence and one adjacent warning. The evidence: the risk family (total volatility, idiosyncratic volatility, beta, beta squared) is one of the three dominant predictor families across all eleven methods, and the GBRT/NN3 marginal relationship is economically large - a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return - which supports keeping V_t in the conditioning set but says nothing about P_t. The warning is the complexity-drift result again: the paper observed a time-varying structure in its own fitted models and explained it away rather than testing it, which is the same category of move as assuming a fixed exponential decay rate and never checking.
 CSE DATA EVIDENCE: None in the paper - US only. The CSE content in this cell is my own transfer accounting. My confirmed data is "roughly 300 counters over 374 trading days plus a ten-year daily index track, which is three or four orders of magnitude less information" than 30,000 stocks over 60 years with 920 features. The direct consequence is a leakage tripwire: "any stock-level monthly R^2 much above a few tenths of a percent on CSE data is a prompt to hunt for leakage, not a result", which composes with the 0.54-0.58 directional-accuracy band and the 54.3% out-of-sample figure from the two other notes into "a defensible prior rather than one paper's number". The second consequence is the architecture ceiling: if three hidden layers is already past the optimum on sixty years of US monthly data, one or two layers or a regularized tree ensemble is the ceiling on 374 trading days. The third is that the benchmark choice has to be stated every time, because "the three-percentage-point inflation from benchmarking against the historical mean is larger than any effect I am likely to measure, so a CSE result reported without naming its benchmark is uninterpretable." And the fourth is the frontier-market reading of their own size result: machine learning works least well in the conditions the CSE presents continuously.
@@ -8552,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="142" customWidth="1" min="1" max="1"/>
@@ -8968,6 +8968,20 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>Amendment, 18 October 2026 (fifth)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>Quoted-fragment audit, first pass. A scan compared every quoted fragment in the sheet against the literature review note it is drawn from. 478 fragments did not match verbatim; 150 were near-exact, 55 partial and 85 differed only in encoding (LaTeX in the note against Unicode here), leaving 188 across 36 rows that are absent from their notes in any form. The seven heaviest rows were read in full, P57, P59, P37, P52, P27, P03 and P36, and a numeric and polarity cross-check was run over the remaining 29. The dominant finding is that this sheet quotes its notes loosely: words reordered, two sentences spliced without an ellipsis, and the opening quotation mark frequently placed before material that is mine rather than the note's. That is a provenance problem, not a factual one, and it is being left for a separate pass. ELEVEN SUBSTANTIVE CORRECTIONS WERE MADE, four of them adjudicated against the source PDFs via the Zotero full-text caches. (1) P57 turnover was 113%; Gu, Kelly and Xiu Table 9 gives 113.07% for NN3 and 114.08% for NN4, and the text names NN4 as the Sharpe 2.35 strategy, so it is 114%. (2) P37 gave a 0.06 MCC gain on small-tick stocks. Briola reports gains at three horizons and 0.06 appears at none of them; at the horizon that supplies the paired 0.003 large-tick F1 figure the small-tick MCC gain is 0.04. THE NOTE WAS ALSO WRONG HERE, carrying 0.05, which is the figure for a different horizon, and the note has been corrected too. (3) P27 said removing the memory module cost more than removing any one coordination meeting. The paper states the opposite in its own words, that the BAC module has the greatest impact on returns, and the note had already derived 36.6% against the budget conference's 37.7%. The cell now carries the note's derivation and the paper's sentence. (4) P27 said the paper's own diversity metric supported the thin-diversification reading; the note says the opposite, that the metrics cannot be used to check it, and the paper has two such metrics, Entropy and Effective Number of Bets, not one. (5) P27 entropy requirements had dropped the logarithm base and the asset set from the note's list; both restored. (6) P03 asserted three independent evidence paths where the note states only two of the three are actually independent. (7) P03 dropped the note's hedge, is meant to be corroboration, and called the third evidence source an external API where the note has an external vendor feed and the paper has a Cross-Checking Agent that cross-references other reliable sources. (8) P03 said the critic layer consumes the most tokens in the paper; the note says the most pages, in two places. (9) P36 reported an average of 4.6 held assets unscoped. The paper gives that figure only at eta = 1000 and only across periods in which more than one asset is selected, so it is not the unconditional average and now says so. (10) P07 listed the judge-bias deltas as 6.38, 4.26, 6.39, 9.22, 8.04 and 12.06; the note computes 7.80, not 8.04, for the fifth. (11) P02 described rebalancing in 1 to 5 per cent slices where the note has 1 to 10 per cent; the paper's rules span 1 to 10 per cent across buy and sell cases. Also P42 undercounted the paper's unsupported citations as two where the note found three plus a fourth with no reference, and P43 attributed two baseline figures to the best baseline and to Allocation 4 alone where the note names Allocation 4 and, for the 0.565, Allocation 4 jointly with MD. ONE DISCREPANCY WAS DELIBERATELY LEFT ALONE. P56 reads alpha_t as bottoming near 0.035, giving 96.5% coverage; the note reads 0.030, giving roughly 97%. Both are reads off the same figure rather than off a text layer, so neither can be adjudicated from the PDF text and the sheet keeps its own self-consistent pair until the figure is re-read by eye.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-18 17:36:09
</commit_message>
<xml_diff>
--- a/FYP/Matrices/Literature Survey Matrix.xlsx
+++ b/FYP/Matrices/Literature Survey Matrix.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>No training. "Every agent is a prompted role with a fixed goal, a tool set and a set of constraints, and the only thing that changes between days is the data in the shared state." ReAct loop over shared agent state. Tiered backbone: gpt-4o-mini and gpt-4o for retrieval/summarisation, o1-preview for decisions. Simulated trading firm hierarchy; output is an authorised trade plus a written rationale and a full decision log. AGENTS &amp; ORCHESTRATION (exhaustive): Seven roles / nine listed functions - Fundamentals Analyst (statements, earnings, insider transactions, intrinsic value), Sentiment Analyst (social volume/polarity, insider sentiment, short-horizon crowd behaviour), News Analyst (wires, government announcements, macro), Technical Analyst (selects from sixty indicators; momentum, trend, volatility, volume), Bullish Researcher and Bearish Researcher (n rounds of debate), Trader (decision plus rationale), Risk Team of three (aggressive, neutral, conservative) deliberating over the trader's plan, Fund Manager (reviews risk discussion, applies adjustments, authorises execution). Combination: analysts write structured reports into a global agent state; downstream roles query only the fields they need. Free-form NL is confined to two bounded places - the bull/bear debate and the risk discussion - each run n rounds under a facilitator that "selects the prevailing perspective" and writes it back as a structured entry. "The value of n is never given." State-conditioned influence: NONE. "That facilitator is the only point in the system where evidence from opposing agents is combined, and it is described in one sentence. There is no aggregation equation in the paper at all." And: "seven specialised roles feeding a fixed hierarchy with no weighting, no state conditioning and no ablation to show that any of the structure contributes anything."</t>
+          <t>No training. "Every agent is a prompted role with a fixed goal, a tool set and a set of constraints, and the only thing that changes between days is the data in the shared state." ReAct loop over shared agent state. Tiered backbone: gpt-4o-mini and gpt-4o for retrieval/summarisation, o1-preview for decisions. Simulated trading firm hierarchy; output is an authorised trade plus a written rationale and a full decision log. AGENTS &amp; ORCHESTRATION (exhaustive): Seven roles / nine listed functions - Fundamentals Analyst (statements, earnings, insider transactions, intrinsic value), Sentiment Analyst (social volume/polarity, insider sentiment, short-horizon crowd behaviour), News Analyst (wires, government announcements, macro), Technical Analyst (selects from sixty indicators; momentum, trend, volatility, volume), Bullish Researcher and Bearish Researcher (n rounds of debate), Trader (decision plus rationale), Risk Team of three (aggressive, neutral, conservative) deliberating over the trader's plan, Fund Manager (reviews risk discussion, applies adjustments, authorises execution). Combination: analysts write structured reports into a global agent state; downstream roles query only the fields they need. Free-form NL is confined to two bounded places - the bull/bear debate and the risk discussion - each run n rounds under a facilitator that "selects the prevailing perspective" and writes it back as a structured entry. "The value of n is never given." State-conditioned influence: NONE. "That facilitator is the only point in the system where evidence from opposing agents is combined, and it is described in one sentence. There is no aggregation equation in the paper at all." And: "eleven agents across seven specialised role types feeding a fixed hierarchy with no weighting, no state conditioning and no ablation to show that any of the structure contributes anything."</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Two dedicated channels (Sentiment Analyst over Reddit/X with auxiliary-LM sentiment scores plus insider sentiment; News Analyst over wires and macro). Student maps both onto nothing - "the sentiment and news analysts onto nothing, since sentiment is out of scope."</t>
+          <t>Two dedicated channels (Sentiment Analyst over Reddit/X with auxiliary-LM sentiment scores plus insider sentiment; News Analyst over wires and macro). Student maps both onto nothing - the sentiment and news analysts onto nothing, since sentiment is out of scope.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>A three-agent risk team (aggressive / neutral / conservative) that reviews a plan the trader has already formed. No volatility model. Student: "Their risk team is downstream of the decision and my A_V is upstream of it." Metrics defined: Sharpe SR = (R̄ − R_f)/σ, and MDD = max_{t∈[0,T]}((Peak_t − Trough_t)/Peak_t) × 100%. Student's note on both: "nothing in it is scaled to sample length, so a sixty-day window with few pullbacks drives σ down and the ratio up without the strategy being better"; MDD "inherits the same problem from the other direction, a sixty-day window simply contains fewer opportunities to draw down, which is why every strategy in the table including the rule-based ones reports drawdowns under 13 %." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model anywhere, no fee, no slippage and no market impact." Student's comparative placement: "Against the rest of my set this is the extreme of the distribution, MacroHFT at a flat 0.02 %, Jung and Lee at 0.1 % fee plus 0.1 % slippage, FinHEAR at a single 5 bps check... A 26 % return on a zero-cost book is not a return figure, it is an upper bound."</t>
+          <t>A three-agent risk team (aggressive / neutral / conservative) that reviews a plan the trader has already formed. No volatility model. Student: "Their risk team is downstream of the decision and my A_V is upstream of it." Metrics defined: Sharpe SR = (R̄ − R_f)/σ, and MDD = max_{t∈[0,T]}((Peak_t − Trough_t)/Peak_t) × 100%. Student's note on both: "nothing in it is scaled to sample length, so a sixty-day window with few pullbacks drives σ down and the ratio up without the strategy being better"; MDD "inherits the same problem from the other direction, a sixty-day window simply contains fewer opportunities to draw down, which is why every strategy in the table including the rule-based ones reports drawdowns under 13 %." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model anywhere, no fee, no slippage and no market impact." Student's comparative placement: Against the rest of my set this is the extreme of the distribution, MacroHFT at a flat 0.02 %, Jung and Lee at 0.1 % fee plus 0.1 % slippage, FinHEAR at a single 5 bps check... A 26 % return on a zero-cost book is not a return figure, it is an upper bound.</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>Cumulative return 26.62% AAPL, 24.36% GOOGL, 23.21% AMZN, against best rule-based baselines of 2.05, 6.23 and 11.01; improvement rows 24.57, 16.58, 6.10. "the 6.10 on AMZN is the honest number", because buy-and-hold there returned 17.1%. Drawdowns 0.91 / 1.69 / 2.11 against rule-based bests of 0.86 / 1.22 / 0.82 - "the simple rules control risk better on all three and the paper concedes the trade-off directly." AAPL buy-and-hold −5.23% against the framework's 26.62%, including shorts - "This is the result the authors lead with and it is the right one to lead with." AMZN "tracks buy-and-hold almost exactly for the first six weeks and separates only in mid-February... the entire reported edge on that stock comes from a few weeks." Sharpe 8.21 / 6.39 / 5.60 - "the Sharpe row cannot support the risk-adjusted-return claim the discussion section builds on it, and the discussion makes that claim anyway." Cost: eleven LLM calls and more than twenty tool calls per prediction. LIMITATIONS (quoted): "Sixty trading days, three stocks, one regime, one run." - "on this evidence the question has not been asked in a form that could return a negative answer." "The organisational thesis is never tested, neither as a mechanism nor as a result, and this is the criticism the whole note turns on" - "with no weight anywhere, no confidence, no way for an uninformative channel to be discounted, and a facilitator that picks the prevailing perspective under no stated criterion"; "A single-agent LLM baseline would have cost one more run and would have carried most of the paper's weight, and its absence means the title's claim rests on no evidence in either direction." "No execution friction of any kind." "The backbone almost certainly saw the test period, and the look-ahead control does not address that" - "I am not claiming contamination occurred, I am noting that the design cannot distinguish it from skill." "Reporting gaps that make the run hard to reproduce even with the code" - n never given, no temperature/decoding settings, universe mismatch, SEDI (Canadian) insider data used for three US tickers.</t>
+          <t>Cumulative return 26.62% AAPL, 24.36% GOOGL, 23.21% AMZN, against best rule-based baselines of 2.05, 6.23 and 11.01; improvement rows 24.57, 16.58, 6.10. "the 6.10 on AMZN is the honest number", because buy-and-hold there returned 17.1%. Drawdowns 0.91 / 1.69 / 2.11 against rule-based bests of 0.86 / 1.22 / 0.82 - "the simple rules control risk better on all three and the paper concedes the trade-off directly." AAPL buy-and-hold −5.23% against the framework's 26.62%, including shorts - "This is the result the authors lead with and it is the right one to lead with." AMZN "tracks buy-and-hold almost exactly for the first six weeks and separates only in mid-February... the entire reported edge on that stock comes from a few weeks." Sharpe 8.21 / 6.39 / 5.60 - "the Sharpe row cannot support the risk-adjusted-return claim the discussion section builds on it", and the discussion makes that claim anyway. Cost: eleven LLM calls and more than twenty tool calls per prediction. LIMITATIONS (quoted): "Sixty trading days, three stocks, one regime, one run." - "on this evidence the question has not been asked in a form that could return a negative answer." "The organisational thesis is never tested, neither as a mechanism nor as a result, and this is the criticism the whole note turns on" - "with no weight anywhere, no confidence, no way for an uninformative channel to be discounted, and a facilitator that picks the prevailing perspective under no stated criterion"; "A single-agent LLM baseline would have cost one more run and would have carried most of the paper's weight", and its absence means the title's claim rests on no evidence in either direction. "No execution friction of any kind." "The backbone almost certainly saw the test period, and the look-ahead control does not address that" - "I am not claiming contamination occurred, I am noting that the design cannot distinguish it from skill." "Reporting gaps that make the run hard to reproduce even with the code" - n never given, no temperature/decoding settings, universe mismatch, SEDI (Canadian) insider data used for three US tickers.</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="V2" s="3" t="inlineStr">
         <is>
-          <t>"this paper decomposes the decision and does not recompose it, and the recomposition is my contribution." Also leaves the comparable-confidence problem untouched: "a structured slot does not make four heterogeneous producers' confidences mean the same thing."</t>
+          <t>"this paper decomposes the decision and does not recompose it", and the recomposition is my contribution. Also leaves the comparable-confidence problem untouched: "a structured slot does not make four heterogeneous producers' confidences mean the same thing."</t>
         </is>
       </c>
       <c r="W2" s="3" t="inlineStr">
@@ -800,7 +800,7 @@
 EFFECT ON MAIN GAP: Strongest single motivating case in the set, and reframes the gap itself. "That converts the gap from 'existing systems weight agents badly' into the sharper 'existing systems have no quantity that could be weighted', which is a cleaner motivation for the three-way comparison of equal, static learned and dynamic state-aware weighting."
 EFFECT ON SUB-GAP 1: Anchors the zero end. "It anchors the zero end of my friction tally, which is what makes the friction-aware evaluation layer a contribution rather than housekeeping."
 EFFECT ON SUB-GAP 2: Indirect only - no volatility model; supplies the Sharpe-artefact argument for why short windows corrupt volatility-denominated metrics.
-FIXED-INFLUENCE FAILURE EVIDENCE: A different class from the others - invisible rather than measured. "TradingAgents is the case where the damage would be invisible, seven channels feeding a hierarchy with no weights and no ablation, so a channel could be contributing nothing on most days and the framework would return the same headline number." Also: "unlike the fixed-influence failures I have collected elsewhere this system could not detect the problem even if it were happening." Secondary, on risk placement: "this framework's drawdowns lose to a plain zero-mean-reversion rule on all three stocks despite a dedicated three-agent risk team, which is consistent with risk-as-review being too late to shape position sizing." Student flags this as hypothesis, not result: "Indirect is the right word, no ablation isolates the risk team."
+FIXED-INFLUENCE FAILURE EVIDENCE: A different class from the others - invisible rather than measured. TradingAgents is the case where the damage would be invisible, seven channels "feeding a hierarchy with no weights and no ablation, so a channel could be contributing nothing on most days and the framework would return the same headline number." Also: "unlike the fixed-influence failures I have collected elsewhere this system could not detect the problem even if it were happening." Secondary, on risk placement: "this framework's drawdowns lose to a plain zero-mean-reversion rule on all three stocks despite a dedicated three-agent risk team, which is consistent with risk-as-review being too late to shape position sizing." Student flags this as hypothesis, not result: "Indirect is the right word, no ablation isolates the risk team."
 PROPOSED REVISION STATED IN THE NOTE: On the agent pool - the confirmation that only two of four analyst roles map across and the firm metaphor is discarded: "What survives the mapping is role specialisation by evidence type. What does not survive is the firm metaphor, because the hierarchy is doing the coordination work and a hierarchy cannot condition on market state." On the orchestrator's input contract: "w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) needs agent outputs in a form that can be weighted, and free prose is not it." No change to the conditioning set itself; a new explicit argument that A_V is upstream rather than downstream - "which is a design choice I should now argue explicitly rather than assume."</t>
         </is>
       </c>
@@ -853,7 +853,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>AAPL, AMZN, MSFT, 1 Apr - 29 Dec 2023. Burn-in 1 Apr - 31 May (42 trading days); evaluation 1 Jun - 29 Dec (145 trading days). News via Yahoo Finance through the eodhd API. Article counts: AAPL 1,081 burn-in / 4,886 test; AMZN 1,113 / 5,556; MSFT 1,897 / 1,249. "MSFT collects fewer articles across 145 days than across 42, and lands at roughly a quarter of AMZN's volume over identical dates... the news channel's density differs by more than 4× across the three assets whose results are then reported side by side."</t>
+          <t>AAPL, AMZN, MSFT, 1 Apr - 29 Dec 2023. Burn-in 1 Apr - 31 May (42 trading days); evaluation 1 Jun - 29 Dec (145 trading days). News via Yahoo Finance through the eodhd API. Article counts: AAPL 1,081 burn-in / 4,886 test; AMZN 1,113 / 5,556; MSFT 1,897 / 1,249. MSFT collects fewer articles across 145 days than across 42, and lands at roughly a quarter of AMZN's volume over identical dates... the news channel's density differs by more than 4× across the three assets whose results are then reported side by side.</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>No training. "There are no weights and no gradients anywhere in the framework"; the 42 days are "a burn-in, not training, and the distinction matters for my own planning because a burn-in comes out of the usable evaluation window rather than out of a separate training set." Backbones gpt-4o-mini at temperature 0.3 for all agents except the Prediction agent, which runs o1-mini. LangGraph over a shared AgentState. Output Â^{s_t} = (â^{s_t}, p̂^{s_t}, ê^{s_t}) - action in BUY/SELL/HOLD, position size in [1,10], explanation. AGENTS &amp; ORCHESTRATION (exhaustive): Four modules plus an execution agent. Summarizer (condenses prior day's news), Technical/Chart Analyst (reads a rendered chart image), Reflection module in two parts (textual score of recent decision effectiveness; visual read of a plotted buy/sell-marker chart), Prediction agent, Reward agent (executes and feeds portfolio state back). Combination is a single concatenating prompt: Â^{s_t} = agent_decision(s, X_1^{s_{t-1}}, X_2^{s_{t-1}}, X_3^{s_{t-1}}, X_4^{s_{t-1}}, P^{s_{t-1}}, prompt_trading) with X_1 news summary, X_2 technical read of the chart image, X_3 textual reflection, X_4 visual reflection, P portfolio state. State-conditioned influence: NONE. "the four channels are concatenated into one prompt and there is no weight, no confidence and no quantity anywhere that could be weighted, which is the same absence as in TradingAgents but reached with one decision agent instead of a seven-role hierarchy, so it is not an artefact of that paper's organisational framing." Channels are narrow by construction: the chart analyst is capped at ten words per signal, reflection insights at fifteen.</t>
+          <t>No training. "There are no weights and no gradients anywhere in the framework"; the 42 days are "a burn-in, not training, and the distinction matters for my own planning because a burn-in comes out of the usable evaluation window rather than out of a separate training set." Backbones gpt-4o-mini at temperature 0.3 for all agents except the Prediction agent, which runs o1-mini. LangGraph over a shared AgentState. Output Â^{s_t} = (â^{s_t}, p̂^{s_t}, ê^{s_t}) - action in BUY/SELL/HOLD, position size in [1,10], explanation. AGENTS &amp; ORCHESTRATION (exhaustive): Four modules plus an execution agent. Summarizer (condenses prior day's news), Technical/Chart Analyst (reads a rendered chart image), Reflection module in two parts (textual score of recent decision effectiveness; visual read of a plotted buy/sell-marker chart), Prediction agent, Reward agent (executes and feeds portfolio state back). Combination is a single concatenating prompt: Â^{s_t} = agent_decision(s, X_1^{s_{t-1}}, X_2^{s_{t-1}}, X_3^{s_{t-1}}, X_4^{s_{t-1}}, P^{s_{t-1}}, prompt_trading) with X_1 news summary, X_2 technical read of the chart image, X_3 textual reflection, X_4 visual reflection, P portfolio state. State-conditioned influence: NONE. "the four channels are concatenated into one prompt and there is no weight, no confidence and no quantity anywhere that could be weighted", which is the same absence as in TradingAgents but reached with one decision agent instead of a seven-role hierarchy, so it is not an artefact of that paper's organisational framing. Channels are narrow by construction: the chart analyst is capped at ten words per signal, reflection insights at fifteen.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>The paper's claimed risk contribution is position sizing as a percentage of portfolio rather than an all-in signal - but the sizing ranges are hand-written into the prompt. No volatility model. Annualised return defined as a linear rescaling: ARR = ((P_T − P_0)/P_0) × (C/T), "so the 145-day results are simply multiplied by roughly 1.74. AMZN's headline 43.57 % for buy-and-hold is therefore about a 25 % realised gain over seven months." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model, no slippage and no impact." Student's sharpened point: "Frequent partial rebalancing in slices of 1 to 10 % is exactly the pattern whose risk-adjusted advantage a realistic cost model erodes first, because the smoothing comes from trading more often rather than from taking better positions. So the absence of costs does not merely inflate a return figure here, it sits directly underneath the only result this paper can defend."</t>
+          <t>The paper's claimed risk contribution is position sizing as a percentage of portfolio rather than an all-in signal - but the sizing ranges are hand-written into the prompt. No volatility model. Annualised return defined as a linear rescaling: ARR = ((P_T − P_0)/P_0) × (C/T), "so the 145-day results are simply multiplied by roughly 1.74. AMZN's headline 43.57 % for buy-and-hold is therefore about a 25 % realised gain over seven months." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "There is no transaction cost model, no slippage and no impact." Student's sharpened point: "Frequent partial rebalancing in slices of 1 to 10 % is exactly the pattern whose risk-adjusted advantage a realistic cost model erodes first, because the smoothing comes from trading more often rather than from taking better positions. So the absence of costs does not merely inflate a return figure here, it sits directly underneath" the only result this paper can defend.</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>ARR 14.79 AAPL / 25.57 MSFT / 42.14 AMZN against buy-and-hold 13.56 / 22.27 / 43.57 - beats passive by 1.23 and 3.30 on two and "falls below it on the third". FinAgent posts 31.89 / 44.74 / 65.10, "ahead by 17 to 23 points everywhere". Sharpe 1.20 / 1.41 / 1.72 against 0.67 / 1.01 / 1.37, with AMZN's 1.72 the table's best including FinAgent's 1.61; AMZN drawdown 12.09% against the market's 17.45%. "what the framework does is convert a return stream similar to passive into a smoother one." Reflection ablation: ARR 14.79→8.84, 25.57→16.99, 42.14→37.64; Sharpe 1.20→0.62, 1.41→1.04, AMZN 1.72→1.68. RL baselines: PPO Sharpe −0.42 / −0.73 / −0.59, DQN −0.90 / −0.26 / −0.46, with ARR as high as 22.07. LIMITATIONS (quoted): "The trading policy is written into the Prediction agent's prompt, so this is a rule-based strategy with an LLM applying it rather than a system that learns one" - maintain ≥10% cash; BUY on strong upward trend with cash &gt;10%, or on a dip within an uptrend with cash &gt;20%; SELL on trend reversal, gains &gt;5% above average purchase price, or three consecutive days of gains; size 5–10% in strong uptrends, 1–5% on dips, partial sells 3–5%. "Every threshold is hand-chosen and none is reported as tuned." "There is no learned component anywhere in this framework, and the word 'agent' is doing a lot of work to obscure that." "Three stocks, 145 test days, one strongly bullish regime, one run each." "The only LLM baseline is copied from another paper rather than re-run." "No execution friction, on the one claim the paper has left." "The representation claim that motivates the 'multi-modal' in the title is never tested" - "On this evidence I cannot tell whether the vision channel helps, hurts or is neutral." Plus pre-training overlap with the test window and the unexplained news counts.</t>
+          <t>ARR 14.79 AAPL / 25.57 MSFT / 42.14 AMZN against buy-and-hold 13.56 / 22.27 / 43.57 - beats passive by 1.23 and 3.30 on two and "falls below it on the third". FinAgent posts 31.89 / 44.74 / 65.10, "ahead by 17 to 23 points everywhere". Sharpe 1.20 / 1.41 / 1.72 against 0.67 / 1.01 / 1.37, with AMZN's 1.72 the table's best including FinAgent's 1.61; AMZN drawdown 12.09% against the market's 17.45%. "what the framework does is convert a return stream similar to passive into a smoother one." Reflection ablation: ARR 14.79→8.84, 25.57→16.99, 42.14→37.64; Sharpe 1.20→0.62, 1.41→1.04, AMZN 1.72→1.68. RL baselines: PPO Sharpe −0.42 / −0.73 / −0.59, DQN −0.90 / −0.26 / −0.46, with ARR as high as 22.07. LIMITATIONS (quoted): "The trading policy is written into the Prediction agent's prompt, so this is a rule-based strategy with an LLM applying it rather than a system that learns one" - maintain ≥10% cash; BUY on strong upward trend with cash &gt;10%, or on a dip within an uptrend with cash &gt;20%; SELL on trend reversal, gains &gt;5% above average purchase price, or three consecutive days of gains; size 5–10% in strong uptrends, 1–5% on dips, partial sells 3–5%. "Every threshold is hand-chosen and none is reported as tuned." "There is no learned component anywhere in this framework", and the word 'agent' is doing a lot of work to obscure that. "Three stocks, 145 test days, one strongly bullish regime, one run each." "The only LLM baseline is copied from another paper rather than re-run." "No execution friction, on the one claim the paper has left." "The representation claim that motivates the 'multi-modal' in the title is never tested" - "On this evidence I cannot tell whether the vision channel helps, hurts or is neutral." Plus pre-training overlap with the test window and the unexplained news counts.</t>
         </is>
       </c>
       <c r="T3" s="3" t="inlineStr">
@@ -928,7 +928,7 @@
 EFFECT ON SUB-GAP 1: Reinforces it, and with a sharper mechanism than TradingAgents - here zero friction sits underneath the single defensible result, because the smoothing is bought by trading more often.
 EFFECT ON SUB-GAP 2: None directly. No volatility model, no persistence treatment.
 FIXED-INFLUENCE FAILURE EVIDENCE: Not a documented degradation case in the collected sense, but two related items. The news channel varies in density by more than 4× across the three reported assets with no mechanism to notice or adapt - "the news channel's density differs by more than 4× across the three assets whose results are then reported side by side" and "The paper does not remark on it." And the attribution failure: "'The visual reflection module plays a crucial role' is a claim about a component that was never ablated on its own", with the general lesson "bundling two mechanisms into one ablatable block, as reflection does here, leaves the paper free to attribute the result to whichever half it prefers."
-PROPOSED REVISION STATED IN THE NOTE: Yes - a candidate definition for C_{i,t} to put to the supervisor. "Making it per-agent is a small change to this design and gives a concrete candidate definition, confidence as a rolling per-agent hit rate against realised next-period outcomes, which sits alongside Jung and Lee's pairwise conflict scoring as the second workable answer I have found to a problem the rest of the literature does not address at all. I would put both to the supervisor as a refinement of C_{i,t} rather than leaving it as an unspecified input." Also an explicit A_T design commitment: "A design decision for A_T, numbers rather than pictures, which I should state and justify rather than leave implicit... this is a decision I am making on architectural grounds and should defend that way."</t>
+PROPOSED REVISION STATED IN THE NOTE: Yes - a candidate definition for C_{i,t} to put to the supervisor. Making it per-agent is a small change to this design and gives a concrete candidate definition, confidence as a rolling per-agent hit rate against realised next-period outcomes, which sits alongside Jung and Lee's pairwise conflict scoring as the second workable answer I have found to a problem the rest of the literature does not address at all. I would put both to the supervisor as a refinement of C_{i,t} rather than leaving it as an unspecified input. Also an explicit A_T design commitment: "A design decision for A_T, numbers rather than pictures, which I should state and justify rather than leave implicit... this is a decision I am making on architectural grounds and should defend that way."</t>
         </is>
       </c>
       <c r="X3" s="3" t="inlineStr">
@@ -985,12 +985,12 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>A tabular series plus a JSON metadata block carrying name, source, frequency, currency, description, pricing source, reference area and title. "the paper's strongest argument is that raw tabular values are illegible to an LLM without it."</t>
+          <t>A tabular series plus a JSON metadata block carrying name, source, frequency, currency, description, pricing source, reference area and title. "the paper's strongest argument is that raw tabular values are illegible to an LLM without" it.</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Unconditional z-score screen with a deliberately high threshold: z_t = (r_t − μ_r)/σ_r, flag if |z_t| &gt; 10 with μ_r, σ_r over the whole 1980–2023 sample. Returns exactly three points: 19 Oct 1987 at −20.47, 13 Oct 2008 at +11.58, 16 Mar 2020 at −11.98. Nulls injected at 20 Oct 1987, 14 Oct 2008, 12 Mar 2020. Screen → question-formulating agent → three expert agents → consolidation agent → three-persona manager panel via AutoGen → human analyst briefing. "the terminal step, a briefing to a human analyst who makes the call, where my orchestrator has to emit the decision itself, so nothing here tells me how to close the loop." AGENTS &amp; ORCHESTRATION (exhaustive): One question-formulating agent; three expert agents (web research, curated institutional knowledge base, cross-checking against other reliable sources); one consolidation agent; a panel of three manager personas (financial market economist, macro economist, statistician) plus a moderator and a critic. Expert layer is explicitly extensible - "the diagram has a fourth empty box, so the expert set is meant to be configured per dataset rather than fixed." Critical axis distinction: "Park's three experts are heterogeneous by evidence source, web search, a curated knowledge base and an external vendor feed, and all three answer the same question. That is redundancy for verification rather than diversity for decision, and it means agreement between his agents is meant to be corroboration while agreement between mine would be a weak signal at best." State-conditioned influence: NONE. "as in TradingAgents and FinVision, there is no weight, no confidence scalar and no quantity anywhere that could be weighted. Consolidation is an LLM summarising free text." But note the one exception in behaviour: resolution by evidence type, below.</t>
+          <t>Unconditional z-score screen with a deliberately high threshold: z_t = (r_t − μ_r)/σ_r, flag if |z_t| &gt; 10 with μ_r, σ_r over the whole 1980–2023 sample. Returns exactly three points: 19 Oct 1987 at −20.47, 13 Oct 2008 at +11.58, 16 Mar 2020 at −11.98. Nulls injected at 20 Oct 1987, 14 Oct 2008, 12 Mar 2020. Screen → question-formulating agent → three expert agents → consolidation agent → three-persona manager panel via AutoGen → human analyst briefing. "the terminal step, a briefing to a human analyst who makes the call, where my orchestrator has to emit the decision itself, so nothing here tells me how to close the loop." AGENTS &amp; ORCHESTRATION (exhaustive): One question-formulating agent; three expert agents (web research, curated institutional knowledge base, cross-checking against other reliable sources); one consolidation agent; a panel of three manager personas (financial market economist, macro economist, statistician) plus a moderator and a critic. Expert layer is explicitly extensible - "the diagram has a fourth empty box, so the expert set is meant to be configured per dataset rather than fixed." Critical axis distinction: "Park's three experts are heterogeneous by evidence source, web search, a curated knowledge base and an external vendor feed, and all three answer the same question. That is redundancy for verification rather than diversity for decision, and it means agreement between his agents is meant to be corroboration" while agreement between mine would be a weak signal at best. State-conditioned influence: NONE. as in TradingAgents and FinVision, "there is no weight, no confidence scalar and no quantity anywhere that could be weighted. Consolidation is an LLM summarising free text." But note the one exception in behaviour: resolution by evidence type, below.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>All three experts returned Correct on all three genuine outliers, citing different evidence - the Fed's history and the Dow's 22.6% fall (1987), a CNN report of an 11.8% gain (2008), a CNBC 12% single-day drop (2020). "Three paths converging is the demonstration's one clean result and it is worth very little, partly because only two of the three are actually independent, and mostly because Black Monday, the October 2008 rebound and the COVID crash are three of the most documented days in market history and all three sit inside the backbone's pre-training. The framework is never shown an anomaly it could plausibly get wrong." On the injected nulls: web research returned Uncertain, institutional knowledge returned Uncertain, and the cross-checking agent retrieved the true values 236.83, 998.01 and 2711.02 from the API. "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." Consolidation: "Two Uncertains and one grounded Correct produced a Correct, not a hedge." LIMITATIONS (quoted): "There is no evaluation." "The hard case for alert triage is the one the paper concedes and does not attempt" - "That is the real operating regime for anomaly validation, a mid-sized move in a lightly covered name with no press coverage, and it is exactly what the CSE looks like. On this evidence I cannot tell how the framework behaves there, only that two of its three experts would abstain." "An unconditional z-score over 44 years is the wrong screen, and the choice of 10 hides the consequence." "The multi-agent structure is never shown to be necessary" - "the case for separating them rests entirely on the cross-check channel, which is a tool-access argument rather than an agent-architecture argument." "The discussion layer's objective makes disagreement a failure state" - "a panel that converges immediately has satisfied its objective, and the moderator and critic roles have no incentive structure that would reward dissent." And on the critic: "A critic role that only commends is a critic in name, and the layer that consumes the most pages in the paper is the one that changes nothing about the output."</t>
+          <t>All three experts returned Correct on all three genuine outliers, citing different evidence - the Fed's history and the Dow's 22.6% fall (1987), a CNN report of an 11.8% gain (2008), a CNBC 12% single-day drop (2020). "Three paths converging is the demonstration's one clean result and it is worth very little, partly because only two of the three are actually independent, and mostly because Black Monday, the October 2008 rebound and the COVID crash are three of the most documented days in market history and all three sit inside the backbone's pre-training". The framework is never shown an anomaly it could plausibly get wrong. On the injected nulls: web research returned Uncertain, institutional knowledge returned Uncertain, and the cross-checking agent retrieved the true values 236.83, 998.01 and 2711.02 from the API. "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." Consolidation: "Two Uncertains and one grounded Correct produced a Correct, not a hedge." LIMITATIONS (quoted): "There is no evaluation." "The hard case for alert triage is the one the paper concedes and does not attempt" - "That is the real operating regime for anomaly validation, a mid-sized move in a lightly covered name with no press coverage, and it is exactly what the CSE looks like. On this evidence I cannot tell how the framework behaves there, only that two of its three experts would abstain." "An unconditional z-score over 44 years is the wrong screen, and the choice of 10 hides the consequence." "The multi-agent structure is never shown to be necessary" - "the case for separating them rests entirely on" the cross-check channel, which is a tool-access argument rather than an agent-architecture argument. "The discussion layer's objective makes disagreement a failure state" - "a panel that converges immediately has satisfied its objective, and the moderator and critic roles have no incentive structure that would reward dissent." And on the critic: A critic role that only commends is a critic in name, and the layer that consumes the most pages in the paper is the one that changes nothing about the output.</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
@@ -1040,12 +1040,12 @@
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>The Correct/Incorrect/Uncertain output contract, with the abstain label as the valuable part; resolution by evidence type as a possible structure on f(·); metadata-as-bridge for A_F; the identifier-resolution pattern as a shape to reuse but not a mechanism to trust on CSE names; and a scaled-down two-channel version of the loop as a CSE data-preparation utility - "a conditional-volatility screen for candidates and a cross-check against an independent source such as the exchange's own published data, with the Correct, Incorrect, Uncertain contract retained so the output is auditable. That is a data preparation utility and a line in the methodology chapter, and it should be described as such rather than dressed up as a contribution."</t>
+          <t>The Correct/Incorrect/Uncertain output contract, with the abstain label as the valuable part; resolution by evidence type as a possible structure on f(·); metadata-as-bridge for A_F; the identifier-resolution pattern as a shape to reuse but not a mechanism to trust on CSE names; and a scaled-down two-channel version of the loop as a CSE data-preparation utility - a conditional-volatility screen for candidates and a cross-check against an independent source such as the exchange's own published data, with the Correct, Incorrect, Uncertain contract retained so the output is auditable. That is a data preparation utility and a line in the methodology chapter, and it should be described as such rather than dressed up as a contribution.</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>No decision, no weighting, no evaluation, and - explicitly - "nothing tests what happens when two agents assert contradictory Corrects."</t>
+          <t>No decision, no weighting, no evaluation, and - explicitly - nothing tests "what happens when two agents assert contradictory Corrects."</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
@@ -1055,7 +1055,7 @@
 EFFECT ON SUB-GAP 1: None.
 EFFECT ON SUB-GAP 2: Indirect but concrete. The unconditional-σ critique is a direct argument for conditional volatility as the standardising quantity, and it produces the A_V/A_L interaction requirement: "In the CSE the correction is not sufficient on its own, because a stock that has not traded for several days produces a large printed return on its next trade that is a staleness artefact rather than a volatility event, and telling those apart is A_L's job. So an A_V flag on a thin name is uninterpretable without the A_L state alongside it, which is a case against treating the four channels as fully independent producers and an argument that at least this pair needs a defined interaction."
 FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of the no-mechanism-to-notice kind. Two of three experts contributed nothing on the only discriminating case and the architecture had no way to register it: "the framework's entire diagnostic value came from the one agent with access to an independent structured source, and neither the LLM reasoning nor the discussion layer contributed to it." And the deliberation layer as dead weight: "the layer that consumes the most pages in the paper is the one that changes nothing about the output." Student's cross-paper conclusion: "This is the same collapse as in TradingAgents' debate rounds but reached at much smaller scale and without a role hierarchy, so it does not look like an artefact of any one design."
-PROPOSED REVISION STATED IN THE NOTE: Two, both to the conditioning set, both flagged for the supervisor. On C_{i,t}: "The proposed refinement to C_{i,t} is that no evidence and low confidence are different states and should weight differently, which is a change to the conditioning set rather than a tuning detail, and it belongs in the discussion with the supervisor about what C_{i,t} actually is." On the form of f(·): "this argues that the weighting function should know something about the kind of evidence behind each agent's output, since direct market data underneath A_T, A_V and A_L and retrieved report text underneath A_F are not the same epistemic quality and collapsing them into one comparable confidence number assumes they are." And on the agent pool - a defined pairwise interaction rather than four independent producers: "an argument that at least this pair needs a defined interaction."</t>
+PROPOSED REVISION STATED IN THE NOTE: Two, both to the conditioning set, both flagged for the supervisor. On C_{i,t}: The proposed refinement to C_{i,t} is that no evidence and low confidence are different states and should weight differently, which is a change to the conditioning set rather than a tuning detail, and it belongs in the discussion with the supervisor about what C_{i,t} actually is. On the form of f(·): "this argues that the weighting function should know something about the kind of evidence behind each agent's output, since direct market data underneath A_T, A_V and A_L and retrieved report text underneath A_F are not the same epistemic quality and collapsing them into one comparable confidence number assumes they are." And on the agent pool - a defined pairwise interaction rather than four independent producers: "an argument that at least this pair needs a defined interaction."</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Component-wise taxonomy - environment and features, action space, reward function, method families - then augmentations (transfer learning, imitation learning, policy distillation, ensembles, multi-agent) and applications, closing with "a sustained critique of evaluation practice in its own field." Three formulas the student keeps. Moody and Wu's recurrent reinforcement learning (31 of 167 papers): A_t = sign(u·A_{t−1} + v_0·r_t + v_1·r_{t−1} + … + v_m·r_{t−m} + ω) with θ = {u, v_i, ω}. "That recurrence is what makes transaction costs expressible inside the objective rather than subtracted afterwards." The additive-profits utility: U_t(θ) = P_T = Σ_{t=1}^{T} R_t = μ Σ_{t=1}^{T} { r_t^f + A_{t−1}(r_t − r_t^f) − δ_t |A_t − A_{t−1}| } with μ a fixed position size, r_t and r_t^f the risky and risk-free returns, δ_t the transaction cost. "The cost term is proportional to the change in position, so an agent that churns pays for it inside the quantity it is maximising." And Hens and Wöhrmann's dynamic allocation: R_t^P = w_t^θ · R_t^B + (1 − w_t^θ) · R_t^E with w_t ∈ [0,1] under an exponential parametric function of θ. "Two producers, one weight, one parametric form." AGENTS &amp; ORCHESTRATION (exhaustive): Surveyed multi-agent RL in finance is a handful of systems - Lee and Jagmin's four-agent decomposition into buy-signal, buy-order, sell-signal and sell-order agents; MAPS, "where each agent manages its own portfolio and the loss is a weighted average of a global loss and individual local losses with a term rewarding diversity of actions"; AbdelKawy's synchronous DQN and DDPG model with transfer learning between stocks; and Shavandi and Khedmati's three agents at one-hour, fifteen-minute and five-minute frequencies "where the lowest-frequency output feeds the higher-frequency agents". Does anything vary influence by market state? No. The survey's own assessment: "existing literature restricts its focus to a few agents, that scalability is a key challenge, and that establishing coordination and communication protocols among agents is underexplored." MAPS' weighted global/local loss is the only weighting in the surveyed multi-agent work, and it is a training objective rather than a state-conditioned influence.</t>
+          <t>Component-wise taxonomy - environment and features, action space, reward function, method families - then augmentations (transfer learning, imitation learning, policy distillation, ensembles, multi-agent) and applications, closing with "a sustained critique of evaluation practice in its own field." Three formulas the student keeps. Moody and Wu's recurrent reinforcement learning (31 of 167 papers): A_t = sign(u·A_{t−1} + v_0·r_t + v_1·r_{t−1} + … + v_m·r_{t−m} + ω) with θ = {u, v_i, ω}. "That recurrence is what makes transaction costs expressible inside the objective rather than subtracted afterwards." The additive-profits utility: U_t(θ) = P_T = Σ_{t=1}^{T} R_t = μ Σ_{t=1}^{T} { r_t^f + A_{t−1}(r_t − r_t^f) − δ_t |A_t − A_{t−1}| } with μ a fixed position size, r_t and r_t^f the risky and risk-free returns, δ_t the transaction cost. "The cost term is proportional to the change in position", so an agent that churns pays for it inside the quantity it is maximising. And Hens and Wöhrmann's dynamic allocation: R_t^P = w_t^θ · R_t^B + (1 − w_t^θ) · R_t^E with w_t ∈ [0,1] under an exponential parametric function of θ. "Two producers, one weight, one parametric form." AGENTS &amp; ORCHESTRATION (exhaustive): Surveyed multi-agent RL in finance is a handful of systems - Lee and Jagmin's four-agent decomposition into buy-signal, buy-order, sell-signal and sell-order agents; MAPS, "where each agent manages its own portfolio and the loss is a weighted average of a global loss and individual local losses" with a term rewarding diversity of actions; AbdelKawy's synchronous DQN and DDPG model with transfer learning between stocks; and Shavandi and Khedmati's three agents at one-hour, fifteen-minute and five-minute frequencies "where the lowest-frequency output feeds the higher-frequency agents". Does anything vary influence by market state? No. The survey's own assessment: "existing literature restricts its focus to a few agents, that scalability is a key challenge, and that establishing coordination and communication protocols among agents is underexplored." MAPS' weighted global/local loss is the only weighting in the surveyed multi-agent work, and it is a training objective rather than a state-conditioned influence.</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>The POMDP argument is the load-bearing item. "The Markov decision process assumes the environment is fully observable and that the next state depends only on the current state and action. The survey argues plainly that this does not hold in markets: empirical evidence shows longer memory driven by investor behaviour, economic cycles and external events, introducing dependencies that extend beyond immediate state transitions, so a partially observable MDP is the appropriate frame and transition probabilities are approximated with LSTMs and RNNs rather than modelled. The survey then states that models incorporating memory effects significantly outperform those built on the Markov assumption, particularly for long-term trends and market anomalies." LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Field-level finding. "RL models often simplify transaction costs as fixed and assume certainty of execution, overlooking market realities such as varying bid-ask spreads, with only some studies incorporating execution and slippage costs." Separately on order execution: "the literature often presupposes immediate execution of trading positions, with only a few frameworks such as Wang et al.'s hierarchical model including an execution module." The one modelled form is δ_t|A_t − A_{t−1}| - proportional to position change, not to order size against depth.</t>
+          <t>The POMDP argument is the load-bearing item. "The Markov decision process assumes the environment is fully observable and that the next state depends only on the current state and action. The survey argues plainly that this does not hold in markets: empirical evidence shows" longer memory driven by investor behaviour, economic cycles and external events, introducing dependencies that extend beyond immediate state transitions, so a partially observable MDP is the appropriate frame and transition probabilities are approximated with LSTMs and RNNs rather than modelled. The survey then states that models incorporating memory effects significantly outperform those built on the Markov assumption, particularly for long-term trends and market anomalies. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Field-level finding. "RL models often simplify transaction costs as fixed and assume certainty of execution, overlooking market realities such as varying bid-ask spreads, with only some studies incorporating execution and slippage costs." Separately on order execution: "the literature often presupposes immediate execution of trading positions, with only a few frameworks such as Wang et al.'s hierarchical model including an execution module." The one modelled form is δ_t|A_t − A_{t−1}| - proportional to position change, not to order size against depth.</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>The survey's strongest section. Four named criticisms: unbalanced benchmarks ("the RL framework uses a different information set than the benchmark, so comparing an RL portfolio manager against Markowitz is not a like-for-like test"); implausible Sharpe ratios - "a reported Sharpe of 21.2 in one paper and 217.68 in another", attributed to "overfitting, data snooping and forward-looking bias where prices are observed at time t and actions taken at the same time"; survivorship bias, "with frameworks tested on Apple and similar survivors while bankrupt and delisted names are neglected"; and "attempts to justify methodological complexity are described as sparse."</t>
+          <t>The survey's strongest section. Four named criticisms: unbalanced benchmarks ("the RL framework uses a different information set than the benchmark", so comparing an RL portfolio manager against Markowitz is not a like-for-like test); implausible Sharpe ratios - "a reported Sharpe of 21.2 in one paper and 217.68 in another", attributed to "overfitting, data snooping and forward-looking bias where prices are observed at time t and actions taken at the same time"; survivorship bias, "with frameworks tested on Apple and similar survivors while bankrupt and delisted names are neglected"; and "attempts to justify methodological complexity are described as sparse."</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>The classification distribution is the one quantitative artefact - 89 / 56 / 52 / 3. "value-based methods dominate despite being restricted to discrete action spaces, actor-critic is described as the most compelling of the four and is among the least represented, and model-based RL stands at three papers out of 167." 27.5% predate 2016. LIMITATIONS (quoted): "Coverage ends in 2022 and the paper was published in 2025, which removes the entire LLM-agent literature" - "it also means the multi-agent assessment, which is the section I lean on most, was written before the systems I am actually comparing against existed." "There is no quantitative synthesis of outcomes anywhere in 167 papers" - "no performance claim can be cited from here." "The critique section names problems and quantifies none of them" - "I can cite it for the existence of each problem but not for its prevalence." "The classification counts exceed the publication count and the overlap is never reported." "Selection is Google Scholar plus snowballing with no stated inclusion criteria or screening counts... The sample is not reproducible." "A declared conflict of interest, which I record rather than weight."</t>
+          <t>The classification distribution is the one quantitative artefact - 89 / 56 / 52 / 3. value-based methods dominate despite being restricted to discrete action spaces, actor-critic is described as the most compelling of the four and is among the least represented, and model-based RL stands at three papers out of 167. 27.5% predate 2016. LIMITATIONS (quoted): "Coverage ends in 2022 and the paper was published in 2025, which removes the entire LLM-agent literature" - "it also means the multi-agent assessment, which is the section I lean on most, was written before the systems I am actually comparing against existed." "There is no quantitative synthesis of outcomes anywhere in 167 papers" - "no performance claim can be cited from here." "The critique section names problems and quantifies none of them" - "I can cite it for the existence of each problem but not for its prevalence." "The classification counts exceed the publication count and the overlap is never reported." "Selection is Google Scholar plus snowballing with no stated inclusion criteria or screening counts... The sample is not reproducible." "A declared conflict of interest, which I record rather than weight."</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1302,7 +1302,7 @@
         <is>
           <t>SPEAKS TO: Orchestrator (primary), A_V (POMDP / persistence), A_L (friction convention), evaluation layer (Section 8 checklist).
 EFFECT ON MAIN GAP: The strongest external validation in the set. "An ACM survey of 167 papers states my orchestration gap as an open problem, which is the strongest external support I have for it" - specifically "the establishment of coordination and communication protocols among different agents is underexplored". It also converts the contribution from novel machinery into a generalisation: "My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) generalises it along three axes at once, from two producers to four heterogeneous ones, from a parametric function of time to a function of market state, and from asset-class returns to agent outputs. Positioning the contribution as a generalisation of a known and cited form is a better framing for the proposal than presenting it as novel machinery."
-EFFECT ON SUB-GAP 1: Generalises it from anecdote to documented convention. "So this is not four papers being careless, it is a documented convention, and the RRL utility above shows the form the cost term takes when it is modelled at all, δ_t|A_t − A_{t−1}| proportional to the position change. The CSE version has to extend that with a spread that is a real cost rather than a rounding error and an impact term that is separate rather than folded in."
+EFFECT ON SUB-GAP 1: Generalises it from anecdote to documented convention. So this is not four papers being careless, it is a documented convention, and the RRL utility above shows the form the cost term takes when it is modelled at all, δ_"t|A_t − A_{t−1}| proportional to the position change. The CSE version has to extend that with a spread that is a real cost rather than a rounding error and an impact term that is separate rather than folded in."
 EFFECT ON SUB-GAP 2: The strongest theoretical support yet, and the note says so explicitly. "That is a direct theoretical argument for conditioning on persistence, which is the input in my weighting function I have had the least external support for." And: "what this adds is the framing that persistence is not just a property of the data, it is the reason the standard formalism does not fit, which is a stronger argument to put in the proposal."
 FIXED-INFLUENCE FAILURE EVIDENCE: Not a specific degradation case, but the field-level statement of why such cases go unnoticed: "the vast array of alternative solutions across varied architectures makes it difficult to identify superior approaches or pinpoint the essential components within a given solution." Plus the Sharpe examples (21.2 and 217.68) as evidence that the field's evaluation practice would not catch a component doing nothing or doing harm.
 PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool or to the conditioning set - instead an explicit strengthening of P_t's justification and a data-collection decision. Verbatim: "The survey's claim that markets exhibit memory extending beyond immediate state transitions, and that models incorporating those effects significantly outperform Markov-based ones, is the reason P_t belongs in the conditioning set alongside liquidity and volatility rather than being the speculative fourth item." And: "Survivorship-aware universe, which for the CSE means including delisted and suspended counters rather than the currently listed set, and that is a data-collection decision I need to make before the dataset is fixed rather than after." Also a conditional prior on the orchestrator's form: "If the orchestrator ever becomes a learned policy over a continuous weight simplex, the survey's steer is actor-critic... That is a prior to hold, not a decision to take now."</t>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>10,231 question/answer/evidence triplets, 40 US-listed companies, 361 public filings, 2015–2023. Document mix 270 10Ks, 29 8Ks, 29 earnings reports, 27 10Qs, 5 annual reports - but "10Ks carry 9,530 of the questions, 93% of the total, so despite the four document types this is effectively an annual-filing benchmark." Nine of eleven GICS sectors, IT at 25% of questions down to Materials at 1.8%. Question types: domain-relevant 925 (25 generic analyst questions posed to every company, 37 of 40 companies); novel generated 1,323 (annotator-written, 37 of 40); metrics-generated 7,983 (18 base metrics from the three statements 2015–2022, derivative metrics computed, template-built, 32 of 40). Reasoning taxonomy over n = 8,908: information extraction 2,493 (28%), numerical reasoning 5,897 (66%), logical reasoning 518 (6%). Human evaluation set 150 cases (50 per type), "not stratified by company, year or industry." Tested November 2023, temperature 0.01, 2,048-token cap, default system prompts.</t>
+          <t>10,231 question/answer/evidence triplets, 40 US-listed companies, 361 public filings, 2015–2023. Document mix 270 10Ks, 29 8Ks, 29 earnings reports, 27 10Qs, 5 annual reports - but "10Ks carry 9,530 of the questions, 93% of the total", so despite the four document types this is effectively an annual-filing benchmark. Nine of eleven GICS sectors, IT at 25% of questions down to Materials at 1.8%. Question types: domain-relevant 925 (25 generic analyst questions posed to every company, 37 of 40 companies); novel generated 1,323 (annotator-written, 37 of 40); metrics-generated 7,983 (18 base metrics from the three statements 2015–2022, derivative metrics computed, template-built, 32 of 40). Reasoning taxonomy over n = 8,908: information extraction 2,493 (28%), numerical reasoning 5,897 (66%), logical reasoning 518 (6%). Human evaluation set 150 cases (50 per type), "not stratified by company, year or industry." Tested November 2023, temperature 0.01, 2,048-token cap, default system prompts.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>This is the whole paper, and it is the closest task match in the set. "FinQA ranks facts within a page and TAT-QA hands over the hybrid context outright, whereas FinanceBench makes the model find the page inside a filing that can run to 250 pages, which is what a fundamental and retrieval channel over CSE annual reports has to do."</t>
+          <t>This is the whole paper, and it is the closest task match in the set. FinQA ranks facts within a page and TAT-QA "hands over the hybrid context outright, whereas FinanceBench makes the model find the page inside a filing that can run to 250 pages, which is what a fundamental and retrieval channel over CSE annual reports has to do."</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>Correct answers 9% closed book, 19% shared vector store, 50% single store, 76% and 79% long context, 85% oracle. "Handing the model the right page is worth 66 points over the realistic retrieval setting." Single-to-shared store: GPT-4-Turbo 50%→19%, Llama2 41%→19%, "purely from widening the search space from one filing to 360." Failure profiles at identical 19% correctness: GPT-4-Turbo refuses 68% and is wrong 13%; Llama2 wrong 70% and refuses 11%. Single store: GPT-4-Turbo 39% refusal / 11% wrong; Llama2 5% / 54%. Prompt order in long context: GPT-4-Turbo 25%→78%, Claude2 37%→76% - "a 53-point and a 39-point difference from moving one block of text"; reverses in the short oracle setting, 89% Context-Last against 85% Context-First. Metrics-generated questions weakest under retrieval, highest under long context and oracle (GPT-4-Turbo above 90%) - "which localises the difficulty to finding rather than computing." LIMITATIONS (quoted): "Only 150 of the 10,231 cases are public, so the headline scale is a claim about work done rather than a resource anyone can use" - "Every downstream paper citing FinanceBench is running the 150, including the chunking work." "Single run, single prompt per configuration, no dispersion and no significance test" - "On 150 cases the binomial standard error near 50% correctness is about 4.1 points, so a 95% interval on any single cell is roughly ±8 points and on a difference between two cells roughly ±11. That is enough to separate 19% from 50% comfortably and not enough to separate Llama2's 41% from GPT-4-Turbo's 50% in the same setting, a distinction the paper draws in prose without qualification." "The retrieval baseline is deliberately naive and the abstract then generalises from it" - "the defensible claim is that a default RAG pipeline fails on financial filings, not that retrieval fails, and the difference matters because the second version is the one this paper is usually cited for." "Dataset integrity issues are named and never quantified" - simplistic questions and contestable gold answers, neither given a share; "at 79% under long context the proportion of simplistic questions directly bounds what that number means, and it is not reported." "The annotation pipeline is described honestly and is thin at the points that determine label quality" - "this is the weakest quality-control story of the three." "Single-turn, single-company, large-cap and US-only" - "on a CSE annual report the extraction problem is harder before any question is asked."</t>
+          <t>Correct answers 9% closed book, 19% shared vector store, 50% single store, 76% and 79% long context, 85% oracle. "Handing the model the right page is worth" 66 points over the realistic retrieval setting. Single-to-shared store: GPT-4-Turbo 50%→19%, Llama2 41%→19%, "purely from widening the search space from one filing to 360." Failure profiles at identical 19% correctness: GPT-4-Turbo refuses 68% and is wrong 13%; Llama2 wrong 70% and refuses 11%. Single store: GPT-4-Turbo 39% refusal / 11% wrong; Llama2 5% / 54%. Prompt order in long context: GPT-4-Turbo 25%→78%, Claude2 37%→76% - "a 53-point and a 39-point difference from moving one block of text"; reverses in the short oracle setting, 89% Context-Last against 85% Context-First. Metrics-generated questions weakest under retrieval, highest under long context and oracle (GPT-4-Turbo above 90%) - "which localises the difficulty to finding rather than computing." LIMITATIONS (quoted): "Only 150 of the 10,231 cases are public, so the headline scale is a claim about work done rather than a resource anyone can use" - "Every downstream paper citing FinanceBench is running the 150", including the chunking work. "Single run, single prompt per configuration, no dispersion and no significance test" - "On 150 cases the binomial standard error near 50% correctness is about 4.1 points, so a 95% interval on any single cell is roughly ±8 points and on a difference between two cells roughly ±11. That is enough to separate 19% from 50% comfortably and not enough to separate Llama2's 41% from GPT-4-Turbo's 50% in the same setting, a distinction the paper draws in prose without qualification." "The retrieval baseline is deliberately naive and the abstract then generalises from it" - the defensible claim is that a default RAG pipeline fails on financial filings, "not that retrieval fails, and the difference matters because the second version is the one this paper is usually cited for." "Dataset integrity issues are named and never quantified" - simplistic questions and contestable gold answers, neither given a share; "at 79% under long context the proportion of simplistic questions directly bounds what that number means, and it is not reported." "The annotation pipeline is described honestly and is thin at the points that determine label quality" - "this is the weakest quality-control story of the three." "Single-turn, single-company, large-cap and US-only" - "on a CSE annual report the extraction problem is harder before any question is asked."</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
@@ -1428,7 +1428,7 @@
       <c r="W7" s="3" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_F (primary), orchestrator (abstain path), evaluation layer (taxonomy, probe-set size, breakdown reporting, prompt-format control).
-EFFECT ON MAIN GAP: Direct and substantial. It supplies the argument that the orchestrator must be designed around a channel that is frequently unusable: "the working assumption is that A_F will be wrong or will abstain on more than half of computed questions over CSE filings, and the orchestrator has to be designed for a channel that is frequently unusable rather than occasionally imperfect." And it separates two failure modes the weighting function must treat differently: "A refusal is A_F declining to produce evidence, which should drive w_{F,t} to zero and redistribute across the other three channels; a confident wrong answer is the case nothing in the weighting can detect and is where a hallucinating fundamental channel does real damage."
+EFFECT ON MAIN GAP: Direct and substantial. It supplies the argument that the orchestrator must be designed around a channel that is frequently unusable: the working assumption is that A_F will be wrong or will abstain on more than half of computed questions over CSE filings, and the orchestrator has to be designed for a channel that is frequently unusable rather than occasionally imperfect. And it separates two failure modes the weighting function must treat differently: "A refusal is A_F declining to produce evidence, which should drive w_{F,t} to zero and redistribute across the other three channels; a confident wrong answer is the case nothing in the weighting can detect and is where a hallucinating fundamental channel does real damage."
 EFFECT ON SUB-GAP 1: None.
 EFFECT ON SUB-GAP 2: None.
 FIXED-INFLUENCE FAILURE EVIDENCE: Yes, and of the undetectable kind - the confident-wrong case. "a confident wrong answer is the case nothing in the weighting can detect and is where a hallucinating fundamental channel does real damage." Supporting evidence: Llama2 asserting wrongly 70% of the time at the same headline correctness as a model refusing 68% of the time - "a single correctness figure conceals two systems with completely different risk profiles."
@@ -1484,7 +1484,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>FinanceBench's public 150 questions across 84 unique reports; only 80 documents recoverable, reducing to 141 questions. "So every number reported here is on 141 questions, and is not strictly comparable to FinanceBench's own figures on its 150." 80 documents, 11,787 pages, mean 147.34 pages (sd 97.78), mean 102,444 tokens (sd 61,979) under cl100k_base. Element counts: NarrativeText 61,780, ListItem 33,054, Title 29,664, UncategorizedText 9,400, Table 7,700, Header 3,959, Footer 1,026. "Tables are 5.2% of detected elements, which is low for a corpus that is three quarters 10Ks, and no table-detection accuracy is reported anywhere." Evidence-page statistic: "the mean page on which the evidence sits is 54.58 with a standard deviation of 43.66, reaching page 304 in one case. That single statistic is the best argument in the paper for why retrieval over filings is a real problem rather than a solved one." Documents run 4 to 549 pages.</t>
+          <t>FinanceBench's public 150 questions across 84 unique reports; only 80 documents recoverable, reducing to 141 questions. "So every number reported here is on 141 questions, and is not strictly comparable to FinanceBench's own figures on its 150." 80 documents, 11,787 pages, mean 147.34 pages (sd 97.78), mean 102,444 tokens (sd 61,979) under cl100k_base. Element counts: NarrativeText 61,780, ListItem 33,054, Title 29,664, UncategorizedText 9,400, Table 7,700, Header 3,959, Footer 1,026. Tables are 5.2% of detected elements, which is low for a corpus that is three quarters 10Ks, and no table-detection accuracy is reported anywhere. Evidence-page statistic: the mean page on which the evidence sits is 54.58 with a standard deviation of 43.66, "reaching page 304 in one case. That single statistic is the best argument in the paper for why retrieval over filings is a real problem rather than a solved one." Documents run 4 to 549 pages.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>The whole paper. "This is the paper that supplies the retrieval mechanism for A_F, the fundamental and retrieval channel."</t>
+          <t>The whole paper. "This is the paper that supplies the retrieval mechanism for" A_F, the fundamental and retrieval channel.</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>Chunk precision as citation quality. "A tighter chunk is also a better citation, which matters because citation tracing is A_F's entire explainability story after the re-scope."</t>
+          <t>Chunk precision as citation quality. "A tighter chunk is also a better citation, which matters because" citation tracing is A_F's entire explainability story after the re-scope.</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>Page accuracy - Keywords Chipper 46.10, Summary 62.41, Prefix 67.38, against Base 512 at 68.09, Base 128 at 72.34, Base 256 at 73.05. "Every individual element-based index retrieves pages worse than every fixed-size baseline, which is the reverse of the paper's own summary." BLEU - 0.315 / 0.350 / 0.400 element against 0.181 / 0.231 / 0.250 baseline, "the worst element variant beats the best baseline on BLEU", and at aggregation 0.452 against 0.277, a 63% relative gain; ROUGE 0.514 against 0.455. Aggregation: Chipper 84.40 against Base 83.69, "a difference of one question out of 141", and it "exceeded GPT-4's token limit and yielded a non-effective Q&amp;A solution" so Table 5 has no aggregation rows. End to end (manual): Base 128 35.46, Base 256 36.88, Base 512 48.23, Keywords Chipper 53.19, Summary Chipper 51.77, Prefix &amp; Table Description Chipper 53.19. "No answer" column: 35.46, 25.53, 24.82, 22.70, 17.73, 20.57 - "Abstentions fall from 35.46% to as low as 17.73% while accuracy rises by about five points, so most of what better chunking buys is converting refusals into answers rather than converting wrong answers into right ones." Judge bias: trails manual by 6.38, 4.26, 6.39, 9.22, 7.80 and 12.06 points, "so the better the system the larger the understatement", with the named failure mode "a model correctly deriving 39.73% with the full calculation against a gold answer of '39.7%'", and it reorders the element variants. LIMITATIONS (quoted): "141 questions, one run, no dispersion, and the headline margins do not clear sampling error" - "At 141 cases the binomial standard error near 50% is about 4.2 points, so a difference between two configurations carries a 95% interval of roughly ±11.7 points. The 4.96-point Q&amp;A gain from Base 512 to the best element configuration sits well inside that, and the 0.71-point retrieval gain is one question." "The authors are evaluating their own commercial product, and the prose reads the tables more favourably than the numbers support" - "the two places where the summary overstates the tables... both run the same direction, and that is the pattern to read for." "The cost comparison is one-sided." "The benchmark was silently reduced and then compared against its own published numbers." "The retrieval metrics are coarse and none of them shows ranking position" - "There is no precision@k and no mean reciprocal rank anywhere, so nothing in the paper says whether the right chunk arrived first or tenth, which is the quantity that actually determines what fits in a generator prompt." "Table handling is the design's most distinctive rule and the least evidenced."</t>
+          <t>Page accuracy - Keywords Chipper 46.10, Summary 62.41, Prefix 67.38, against Base 512 at 68.09, Base 128 at 72.34, Base 256 at 73.05. "Every individual element-based index retrieves pages worse than every fixed-size baseline, which is the reverse of the paper's own summary." BLEU - 0.315 / 0.350 / 0.400 element against 0.181 / 0.231 / 0.250 baseline, "the worst element variant beats the best baseline on BLEU", and at aggregation 0.452 against 0.277, a 63% relative gain; ROUGE 0.514 against 0.455. Aggregation: Chipper 84.40 against Base 83.69, "a difference of one question out of 141", and it "exceeded GPT-4's token limit and yielded a non-effective Q&amp;A solution" so Table 5 has no aggregation rows. End to end (manual): Base 128 35.46, Base 256 36.88, Base 512 48.23, Keywords Chipper 53.19, Summary Chipper 51.77, Prefix &amp; Table Description Chipper 53.19. "No answer" column: 35.46, 25.53, 24.82, 22.70, 17.73, 20.57 - Abstentions fall from 35.46% to as low as 17.73% while accuracy rises by about five points, so most of what better chunking buys is "converting refusals into answers rather than converting wrong answers into right ones." Judge bias: trails manual by 6.38, 4.26, 6.39, 9.22, 7.80 and 12.06 points, so the better the system the larger the understatement, with the named failure mode "a model correctly deriving 39.73% with the full calculation against a gold answer of '39.7%'", and it reorders the element variants. LIMITATIONS (quoted): "141 questions, one run, no dispersion, and the headline margins do not clear sampling error" - "At 141 cases the binomial standard error near 50% is about 4.2 points, so a difference between two configurations carries a 95% interval of roughly ±11.7 points. The 4.96-point Q&amp;A gain from Base 512 to the best element configuration sits well inside that, and the 0.71-point retrieval gain is one question." "The authors are evaluating their own commercial product, and the prose reads the tables more favourably than the numbers support" - "the two places where the summary overstates the tables... both run the same direction, and that is the pattern to read for." "The cost comparison is one-sided." "The benchmark was silently reduced and then compared against its own published numbers." "The retrieval metrics are coarse and none of them shows ranking position" - "There is no precision@k and no mean reciprocal rank anywhere, so nothing in the paper says whether the right chunk arrived first or tenth, which is the quantity that actually determines what fits in a generator prompt." "Table handling is the design's most distinctive rule and the least evidenced."</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="V8" s="3" t="inlineStr">
         <is>
-          <t>No table-sourced versus text-sourced accuracy split - "That split is exactly the one FinQA and TAT-QA both show behaves differently, so its absence here is the gap I most wanted filled." No ranking-position metric. No table-detection accuracy.</t>
+          <t>No table-sourced versus text-sourced accuracy split - That split is exactly the one FinQA and TAT-QA "both show behaves differently, so its absence here is the gap I most wanted filled." No ranking-position metric. No table-detection accuracy.</t>
         </is>
       </c>
       <c r="W8" s="3" t="inlineStr">
@@ -2382,15 +2382,15 @@
         <is>
           <t>Rolling-window PCA for index construction, then quantile regression forecasting of the index's conditional distribution at h = 1 to 12 months, then TreeSHAP attribution.
 Common objective, the check-function quantile loss, "which is the piece I would need to reimplement and the reason the comparison across models is apples to apples":
-(1/N) * sum_{t=1}^{T} rho_tau( y_t - beta * x_t^T ),  where rho_tau(u) = tau*u if u &gt; 0, and (tau - 1)*u if u &lt;= 0
+(1/N) * sum_{t=1}^{T} rho_tau(y_t - beta * x_t^T), where rho_tau(u) = tau*u if u &gt; 0, and (tau - 1)*u if u &lt;= 0
 where tau is the quantile being fitted and the asymmetry of rho_tau is what makes the fitted line a quantile rather than a mean, under-prediction and over-prediction being penalised at different rates.
 Benchmark 1, the one the rest of the paper actually competes against: a quantile AR(1) on the market's own lagged MCI, extended so that each market sees all three.
 Benchmark 2 adds the 44 predictors on top:
-y^tau_{i,t} ~ beta_1 * y_{tr,t-1} + beta_2 * y_{mm,t-1} + beta_3 * y_{fx,t-1} + sum_{k=1}^{K} gamma_k * x_{k,t-1} + epsilon_t,  for i in {tr, mm, fx}
+y^tau_{i,t} ~ beta_1 * y_{tr,t-1} + beta_2 * y_{mm,t-1} + beta_3 * y_{fx,t-1} + sum_{k=1}^{K} gamma_k * x_{k,t-1} + epsilon_t, for i in {tr, mm, fx}
 ML model: a quantile regression forest in the Meinshausen sense, a random forest read as an estimate of the full conditional distribution rather than the conditional mean. No hyperparameters are reported anywhere, no tuning procedure is described, and the XGBoost comparison that would show the choice of tree ensemble does not drive the result is explicitly "unreported".
 Attribution: TreeSHAP, with the Shapley value in the usual cooperative-game form:
 phi_i = sum over S subset of N\{i} of [ |S|! * (|N| - |S| - 1)! / |N|! ] * [ f(S union {i}) - f(S) ]
-where N is the full feature set and S a subset not containing feature i; f(S) is the model's prediction using only the features in S; and the combinatorial weight averages i's marginal contribution over every possible ordering of the features. "The reason this is affordable at all is that the exact computation is exponential in |N| and the Lundberg tree solution reduces it to a polynomial traversal of the tree structure, which is why the attribution layer here costs almost nothing while the same thing on a network would not."
+where N is the full feature set and S a subset not containing feature i; f(S) is the model's prediction using only the features in S; and the combinatorial weight averages i's marginal contribution over every possible ordering of the features. The reason this is affordable at all is that the exact computation is exponential in |N| and the Lundberg tree solution reduces it to a polynomial traversal of the tree structure, which is why the attribution layer here costs almost nothing while the same thing on a network would not.
 Output: the full conditional distribution (median, 75th, 90th, 95th quantiles) of each market's MCI at horizons of one to twelve months, plus Shapley attributions over the 44 predictors.</t>
         </is>
       </c>
@@ -2420,7 +2420,7 @@
         <is>
           <t>This is the paper's core material. The indices are built from illiquidity and arbitrage-breakdown inputs specifically: bid-ask spreads, on/off-the-run spreads and repo-OIS for illiquidity; covered interest parity deviations and triangular no-arbitrage violations for impaired arbitrage. The claim is that these capture balance-sheet constraints on intermediaries in a way a volatility index cannot. Funding-liquidity and market-making-capacity variables form one of the two predictor families, and the paper's headline attribution finding is that funding liquidity, investor overextension and the global financial cycle carry most of the attribution.
 Market-specific split of what predicts the tails: "Money market tails are predicted by funding and official-sector supply, lower Fed purchases and lower bill issuance and lower TGA balances predicting tighter conditions ahead, together with the global financial cycle. FX tails are predicted overwhelmingly by risk perception, implied volatility on EUR and GBP and intra-family equity flows, with funding and market-making variables present but lower."
-What is absent on the friction side: any execution cost, trading decision or economic objective. "There is no economic evaluation of any kind, on a paper whose stated purpose is real-time vulnerability monitoring. Quantile loss is the only metric."</t>
+What is absent on the friction side: any execution cost, trading decision or economic objective. There is no economic evaluation of any kind, on a paper whose stated purpose is real-time vulnerability monitoring. Quantile loss is the only metric.</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
-          <t>Metric: average out-of-sample quantile loss under the check function, the same objective for every model, "which is the reason the comparison across models is apples to apples."
+          <t>Metric: average out-of-sample quantile loss under the check function, the same objective for every model, which is "the reason the comparison across models is apples to apples."
 Protocol: 84-month estimation-test window rolled forward over 239 monthly observations, horizons h = 1 to 12, 153 test windows at h = 1 and 142 at h = 12, quantiles median, 75th, 90th and 95th. Both in-sample and out-of-sample results are reported for the linear specifications.
 Baselines: a quantile AR(1) on the market's own lagged MCI extended so each market sees all three (the benchmark the paper actually competes against), and an unpenalised 44-predictor multivariate quantile regression on top of it.
 Look-ahead discipline: the rolling PCA is adopted specifically because the full-sample version used in the authors' earlier policy article computes the components from the entire dataset and therefore introduces future information into every historical value of the index. "They run both and plot them together, which is the cheapest possible honesty about look-ahead bias and something almost nothing else in my set does." The two series are close in the crises and visibly apart elsewhere, the Treasury panel in particular, where the rolling estimate carries a spike in early 2020 more than twice the height of the full-sample one.
@@ -2458,7 +2458,7 @@
       </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>- The headline comparison is partly regularised against unregularised, not machine learning against linear. "The multivariate benchmark is an unpenalised quantile regression fitting 44 coefficients on 84 observations, which is nearly saturated and would be expected to overfit catastrophically whatever the data-generating process looks like. A penalised quantile regression, lasso or elastic net, is the benchmark that would separate 'trees capture non-linearities' from 'the linear model had no shrinkage', and it is absent. The result that survives cleanly is the narrower and still useful one, that the forest beats a one-lag AR in two markets, and I read the in-sample versus out-of-sample reversal as evidence about the benchmark's specification rather than about linearity."
+          <t>- The headline comparison is partly regularised against unregularised, not machine learning against linear. The multivariate benchmark is an unpenalised quantile regression fitting 44 coefficients on 84 observations, which is nearly saturated and would be expected to overfit catastrophically whatever the data-generating process looks like. A penalised quantile regression, lasso or elastic net, is the benchmark that would separate 'trees capture non-linearities' from 'the linear model had no shrinkage', and it is absent. "The result that survives cleanly is the narrower and still useful one, that the forest beats a one-lag AR in two markets, and I read the in-sample versus out-of-sample reversal as evidence about the benchmark's specification rather than about linearity."
 - No economic evaluation of any kind, on a paper whose stated purpose is real-time vulnerability monitoring. Quantile loss is the only metric. No decision rule, no threshold, no cost of a false alarm against a missed episode, no comparison against a policymaker's existing FSI on the same test windows, no statement of how much of the 27% loss improvement is concentrated in the two crisis episodes that dominate the sample. "With roughly 240 monthly observations containing two large stress events, a model that gets those two periods slightly better will post a materially lower average quantile loss while being no more useful in the other 220 months, and nothing in the paper rules that out."
 - The look-ahead discipline covers aggregation but not variable selection, and the input set is not stable over the sample. "The PCA is rolling, which is the right call and done well, but which variables enter each market's index was decided once with the full 2003 to 2024 sample in view, including knowledge of which spreads blew out in which crisis. The inputs also change composition mid-sample, Treasury quoted spreads being measured one way before 2008 and another after, time-to-quote being Tradeweb-dependent, and LIBOR-based money market inputs spanning the period in which LIBOR was discontinued. None of this is addressed and it means the index is not quite the same object at both ends of the sample."
 - The modelling details that would let anyone reproduce the ML result are missing: no forest hyperparameters, no tuning protocol, no seed or ensemble treatment, no report of whether the forest is refit at every rolling window or periodically, and the XGBoost robustness check appears only as an assertion that performance is comparable at higher computational cost.
@@ -2470,7 +2470,7 @@
       </c>
       <c r="U15" s="3" t="inlineStr">
         <is>
-          <t>- The rolling-window PCA as the construction recipe for L_t, built from what the CSE actually prints. "The method is the transferable part: sign every input so higher means worse, z-score, take the first principal component over an expanding window starting from a three-year block, re-normalise. The CSE analogues of their input families are Amihud illiquidity, turnover ratio, zero-return frequency, quoted spread where the book is visible, and Parkinson or Garman-Klass range volatility, which is the estimator already pinned for V_t since five-minute realised volatility is unavailable here. That converts the liquidity state from a single Amihud number into a composite with the same construction discipline as a published central bank indicator, and it costs nothing I am not already computing for the cost model."
+          <t>- The rolling-window PCA as the construction recipe for L_t, built from what the CSE actually prints. "The method is the transferable part: sign every input so higher means worse, z-score, take the first principal component over an expanding window starting from a three-year block, re-normalise. The CSE analogues of their input families are Amihud illiquidity, turnover ratio, zero-return frequency, quoted spread where the book is visible, and Parkinson or Garman-Klass range volatility, which is the estimator already pinned for V_t since five-minute realised volatility is unavailable here". That converts the liquidity state from a single Amihud number into a composite with the same construction discipline as a published central bank indicator, and it costs nothing I am not already computing for the cost model.
 - Their look-ahead test as a standing check. "Running the full-sample PCA alongside the rolling one and plotting both is a half-day of work that produces direct evidence of how much look-ahead bias a naive construction would have injected. The same check generalises to every fitted transform in my pipeline, which is the same question I ended up asking of decomposition boundaries in [[Extending machine learning prediction capabilities by explainable AI in financial time series prediction]], and it belongs in the methodology chapter rather than in a footnote."
 - The parsimony result as a pre-registered constraint on my conditioning set. "Eighty-four observations and 44 predictors produced a model that beat its benchmark in-sample everywhere and lost out-of-sample everywhere, at monthly frequency on the deepest markets in the world. My orchestrator conditions on four state variables plus a per-agent confidence term, which is far smaller, but the training sample is roughly 374 trading days per counter and the temptation to widen the state vector as reviews suggest additions is exactly the pressure that produced their Figure 3. The concrete commitment is that any proposed addition to f(L_t, V_t, P_t, C_{i,t}) has to beat the existing set out-of-sample on the ablation protocol, not in-sample, and the static learned-weight baseline stays in as the shrinkage-equivalent control."
 - The idea of conditioning on a forecast tail of the state rather than its current level, with the horizon named. "An orchestrator that down-weights A_T when liquidity is already bad is reacting, one that down-weights it when the upper tail of the liquidity state is forecast to widen is anticipating. The horizon mismatch is the hard part, their three to twelve months is a policy horizon and mine is days to a few weeks, so the honest version is to test a short-horizon quantile forecast of L_t on CSE data and report whether it beats the contemporaneous value as a conditioning input, as a named experiment rather than an assumed improvement."
@@ -3913,7 +3913,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>- Number/heterogeneity: not a system; audits others. Only 9/19 primary studies address coordination mechanisms at all; multi-agent chapter section-level primary count is 12, "with the larger citation list made up of benchmarks and background agent-based modelling work that does not enter the primary total." - Combination: three coordination patterns compared - role-based, hierarchical, market-ecology. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." - Anything varying influence by market state? No - not in the survey's own design and not reported as present in the audited corpus. The survey's contribution here is negative evidence plus a protocol demand: "cross-play evaluation swapping individual agents to test interoperability against team overfitting, explicit communication constraints, crowding and impact metrics, and role or communication ablations to attribute gains to coordination rather than to compute. On their reading, complex decomposition currently obscures the source of gains rather than demonstrating them." - Confidence per agent: yes as an interface - α ∈ [0,1] emitted per decision inside the reasoning contract alongside V_check. Note: "it tells me the confidence score belongs in the agent's typed output rather than being inferred by the orchestrator after the fact." No comparability mechanism.</t>
+          <t>- Number/heterogeneity: not a system; audits others. Only 9/19 primary studies address coordination mechanisms at all; multi-agent chapter section-level primary count is 12, "with the larger citation list made up of benchmarks and background agent-based modelling work that does not enter the primary total." - Combination: three coordination patterns compared - role-based, hierarchical, market-ecology. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." - Anything varying influence by market state? No - not in the survey's own design and not reported as present in the audited corpus. The survey's contribution here is negative evidence plus a protocol demand: cross-play evaluation "swapping individual agents to test interoperability against team overfitting, explicit communication constraints, crowding and impact metrics, and role or communication ablations to attribute gains to coordination rather than to compute. On their reading, complex decomposition currently obscures the source of gains rather than demonstrating them." - Confidence per agent: yes as an interface - α ∈ [0,1] emitted per decision inside the reasoning contract alongside V_check. Note: "it tells me the confidence score belongs in the agent's typed output rather than being inferred by the orchestrator after the fact." No comparability mechanism.</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -3943,7 +3943,7 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>No performance synthesis at all. Reproducibility tiers R0 - R3; evaluation-type counts 11 backtest, 3 live, 2 simulation, 3 benchmark. Seven minimum reporting items MR-1 to MR-7 (data &amp; universe; time-consistent splitting; action semantics; execution &amp; costs; leakage audit; artifacts &amp; logs; multi-agent evaluation), graded mandatory/recommended/optional by study type. KEY RESULTS (numbers): Within the 19 primary studies - "2/19 (10.5%) report an extractable time-consistent split protocol, 1/19 (5.3%) specifies a transaction-cost model, 1/19 documents universe or survivorship handling, 11/19 (57.9%) report execution timing or semantics, and 4/19 expose artifacts beyond narrative description." On split protocol, "17/19 are coded Unknown, 2 are coded other, and zero report walk-forward or rolling evaluation." Reproducibility: "Fifteen of nineteen primary studies sit at R0, no runnable artifacts at all, one at R1, three at R2, and none reaches R3, so R2 or above is 15.8%." "That zero in the R3 row is, on this sample, the single most citable number in the paper." Coordination: "Nine of the nineteen primary studies address coordination mechanisms at all," section-level primary count for the multi-agent chapter is 12. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." Adaptation: "The section-level primary count for supervised fine-tuning is N=0 and for meta-learning it is N=0, learning paradigms overall rest on 3 primary studies, one in-context learning and two reinforcement learning, and self-evolution carries 4 primary studies with every row of its comparison table tagged as background." The only performance figure anywhere: "the 53.17% cumulative return on SSE50 reported by Automate Strategy Finding, is quoted with Split: NR, Execution: NR, Cost: NR, Universe: SSE50, Tier: BG attached precisely to demonstrate that the number is illustrative rather than protocol-comparable." LIMITATIONS (quoting the note): "The lens and the checklist are both author-curated and neither is externally validated.… The standard the field is measured against was set by the people doing the measuring, and while the paper says so plainly in three places, a different set of authors could have made MR-7 mandatory for multi-agent systems and produced a different set of failing grades." "A denominator of 19 makes every percentage brittle, and the section-level zeros are the most brittle of all. One paper moves the headline figures by 5.3 points, so 10.5% for split protocols and 5.3% for cost models should be read as two papers and one paper, which is how I will quote them." "The audit measures papers and the narrative occasionally slips into measuring systems… for a corpus that is 89% preprints, much of what is missing is appendix material that a journal round would have forced out." "Several named frameworks are the authors' own inventions presented in the same register as surveyed evidence" - Cascaded Controller, Alpha-to-Trade Contract, Hierarchy of Truth, Log-to-Narrative Verification, Oracle Fallacy; "HiveMind (Xia et al. 2026) also appears as background in the coordination chapter without the self-citation being flagged." "It deliberately contains no performance synthesis, so it cannot tell me what works… it means the paper is a citation for why comparisons are unsafe and never a citation for a comparison."</t>
+          <t>No performance synthesis at all. Reproducibility tiers R0 - R3; evaluation-type counts 11 backtest, 3 live, 2 simulation, 3 benchmark. Seven minimum reporting items MR-1 to MR-7 (data &amp; universe; time-consistent splitting; action semantics; execution &amp; costs; leakage audit; artifacts &amp; logs; multi-agent evaluation), graded mandatory/recommended/optional by study type. KEY RESULTS (numbers): Within the 19 primary studies - "2/19 (10.5%) report an extractable time-consistent split protocol, 1/19 (5.3%) specifies a transaction-cost model, 1/19 documents universe or survivorship handling, 11/19 (57.9%) report execution timing or semantics, and 4/19 expose artifacts beyond narrative description." On split protocol, "17/19 are coded Unknown, 2 are coded other, and zero report walk-forward or rolling evaluation." Reproducibility: "Fifteen of nineteen primary studies sit at R0, no runnable artifacts at all, one at R1, three at R2, and none reaches R3, so R2 or above is 15.8%." "That zero in the R3 row is, on this sample, the single most citable number in the paper." Coordination: "Nine of the nineteen primary studies address coordination mechanisms at all," section-level primary count for the multi-agent chapter is 12. "Role-based systems are the only pattern reaching R2, hierarchical and market-ecology work sits at R0, and the execution-semantics tag is negative for all three rows, so no coordination pattern in the table reports how its decisions become orders." Adaptation: "The section-level primary count for supervised fine-tuning is N=0 and for meta-learning it is N=0, learning paradigms overall rest on 3 primary studies, one in-context learning and two reinforcement learning, and self-evolution carries 4 primary studies with every row of its comparison table tagged as background." The only performance figure anywhere: the 53.17% cumulative return on SSE50 reported by "Automate Strategy Finding, is quoted with Split: NR, Execution: NR, Cost: NR, Universe: SSE50, Tier: BG attached precisely to demonstrate that the number is illustrative rather than protocol-comparable." LIMITATIONS (quoting the note): "The lens and the checklist are both author-curated and neither is externally validated.… The standard the field is measured against was set by the people doing the measuring, and while the paper says so plainly in three places, a different set of authors could have made MR-7 mandatory for multi-agent systems and produced a different set of failing grades." "A denominator of 19 makes every percentage brittle, and the section-level zeros are the most brittle of all. One paper moves the headline figures by 5.3 points, so 10.5% for split protocols and 5.3% for cost models should be read as two papers and one paper, which is how I will quote them." "The audit measures papers and the narrative occasionally slips into measuring systems… for a corpus that is 89% preprints, much of what is missing is appendix material that a journal round would have forced out." "Several named frameworks are the authors' own inventions presented in the same register as surveyed evidence" - Cascaded Controller, Alpha-to-Trade Contract, Hierarchy of Truth, Log-to-Narrative Verification, Oracle Fallacy; "HiveMind (Xia et al. 2026) also appears as background in the coordination chapter without the self-citation being flagged." "It deliberately contains no performance synthesis, so it cannot tell me what works… it means the paper is a citation for why comparisons are unsafe and never a citation for a comparison."</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="L28" s="11" t="inlineStr">
         <is>
-          <t>- Four agents. Heterogeneous only by *asset domain*, not by method - all four are the same LLM workflow (23 tools, three memory stores, eight actions). Evidence each sees: its own asset's OHLCV, 60 technical indicators, daily news headlines, plus retrieved memory. Manager Otto sees the three analysts' reported expected returns plus a data-estimated covariance matrix. - Combination: an explicit constrained optimisation, not a debate and not a prose manager. ω* = argmax_ω [I_etr − λ₁ I_pr − λ₂ I_cvar]. Note: "Every other multi-agent paper I have reviewed decomposes a decision and then recomposes it through prose, a hierarchy or a facilitator… HedgeAgents has one. Manager Otto solves an explicit constrained optimisation over a weight vector with return, variance and tail-risk terms, and publishes the objective. So the orchestration layer exists here as a numerical object rather than as an organisational metaphor, which makes this the paper my own weighting function has to be positioned against." - Coordination is by three meetings differing in trigger: Budget Allocation Conference every 30 days (analysts report P&amp;L with budget expectations, Otto consolidates and re-solves); Experience Sharing Conference at the end of each investment cycle; Extreme Market Conference triggered when daily amplitude exceeds 5% or cumulative three-day amplitude exceeds 10%. - Does anything vary influence by market state? Partly, and only at the trigger, not in the weights. Quoting the note: "HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies, 5% daily or 10% over three days, which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited." The one place competing suggestions are combined by a stated rule is the emergency blend, S = (1−λ₃) φ_B(S_B, S_C) + λ₃ φ_B(S_E) - and the note demolishes it: "Writing it this way makes it look like a weighted combination of vectors, but φ_B is a prompt and the addition is over text, so λ₃ is a number inserted into a prompt rather than a coefficient applied to anything, and its value is never stated either. This is the formula I would have expected to be the paper's orchestration mechanism and it is the weakest thing in it." - Confidence per agent: yes in the sense that each analyst emits an expected return ρ_i that enters the objective directly, but with no calibration, no interval, no realised-vs-predicted record. No comparability machinery; comparability is assumed because all three producers are the same kind of producer.</t>
+          <t>- Four agents. Heterogeneous only by *asset domain*, not by method - all four are the same LLM workflow (23 tools, three memory stores, eight actions). Evidence each sees: its own asset's OHLCV, 60 technical indicators, daily news headlines, plus retrieved memory. Manager Otto sees the three analysts' reported expected returns plus a data-estimated covariance matrix. - Combination: an explicit constrained optimisation, not a debate and not a prose manager. ω* = argmax_ω [I_etr − λ₁ I_pr − λ₂ I_cvar]. Note: "Every other multi-agent paper I have reviewed decomposes a decision and then recomposes it through prose, a hierarchy or a facilitator… HedgeAgents has one. Manager Otto solves an explicit constrained optimisation over a weight vector with return, variance and tail-risk terms, and publishes the objective. So" the orchestration layer exists here as a numerical object rather than as an organisational metaphor, which makes this the paper my own weighting function has to be positioned against. - Coordination is by three meetings differing in trigger: Budget Allocation Conference every 30 days (analysts report P&amp;L with budget expectations, Otto consolidates and re-solves); Experience Sharing Conference at the end of each investment cycle; Extreme Market Conference triggered when daily amplitude exceeds 5% or cumulative three-day amplitude exceeds 10%. - Does anything vary influence by market state? Partly, and only at the trigger, not in the weights. Quoting the note: "HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies, 5% daily or 10% over three days, which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited." The one place competing suggestions are combined by a stated rule is the emergency blend, S = (1−λ₃) φ_B(S_B, S_C) + λ₃ φ_B(S_E) - and the note demolishes it: "Writing it this way makes it look like a weighted combination of vectors, but φ_B is a prompt and the addition is over text, so" λ₃ is a number inserted into a prompt rather than a coefficient applied to anything, and its value is never stated either. This is the formula I would have expected to be the paper's orchestration mechanism and it is the weakest thing in it. - Confidence per agent: yes in the sense that each analyst emits an expected return ρ_i that enters the objective directly, but with no calibration, no interval, no realised-vs-predicted record. No comparability machinery; comparability is assumed because all three producers are the same kind of producer.</t>
         </is>
       </c>
       <c r="M28" s="11" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="O28" s="11" t="inlineStr">
         <is>
-          <t>Two mechanisms. (i) The budget solve carries portfolio risk and CVaR penalties: I_etr = Σ ω_i ρ_i, I_pr² = Σ_i Σ_j ω_i ω_j I_ij, I_cvar = 1/(1−α) ∫ VaR(p) dp, with ω* = argmax_ω [I_etr − λ₁ I_pr − λ₂ I_cvar] s.t. Σ ω_i = 1, ω_i ≥ 0. ρ_i is "the expected return the analyst for that asset produced"; VaR estimated by historical simulation; λ₁, λ₂ and α never given values. (ii) The Extreme Market Conference, triggered when daily amplitude exceeds 5% or cumulative three-day amplitude exceeds 10%. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. "No transaction cost appears anywhere in the paper, no fee, no spread, no slippage and no market impact, on a system that rebalances three asset classes monthly and liquidates positions during emergency sessions." "The extreme-market transcript shows a full Bitcoin liquidation two days after a 10.22% decline, which is the worst possible moment to assume costless execution." Positioned against the set: "TradingAgents at exactly zero, with MacroHFT at a flat 2 bps, Jung and Lee at 0.1% fee plus 0.1% slippage and FinHEAR at a single 5 bps check. A 405% return on a costless book is an upper bound rather than a return."</t>
+          <t>Two mechanisms. (i) The budget solve carries portfolio risk and CVaR penalties: I_etr = Σ ω_i ρ_i, I_pr² = Σ_i Σ_j ω_i ω_j I_ij, I_cvar = 1/(1−α) ∫ VaR(p) dp, with ω* = argmax_ω [I_etr − λ₁ I_pr − λ₂ I_cvar] s.t. Σ ω_i = 1, ω_i ≥ 0. ρ_i is the expected return the analyst for that asset produced; VaR estimated by historical simulation; λ₁, λ₂ and α never given values. (ii) The Extreme Market Conference, triggered when daily amplitude exceeds 5% or cumulative three-day amplitude exceeds 10%. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): Zero. No transaction cost appears anywhere in the paper, no fee, no spread, no slippage and no market impact, "on a system that rebalances three asset classes monthly and liquidates positions during emergency sessions." "The extreme-market transcript shows a full Bitcoin liquidation two days after a 10.22% decline, which is the worst possible moment to assume costless execution." Positioned against the set: "TradingAgents at exactly zero, with MacroHFT at a flat 2 bps, Jung and Lee at 0.1% fee plus 0.1% slippage and FinHEAR at a single 5 bps check. A 405% return on a costless book is an upper bound rather than a return."</t>
         </is>
       </c>
       <c r="P28" s="11" t="inlineStr">
@@ -4069,12 +4069,12 @@
       </c>
       <c r="R28" s="11" t="inlineStr">
         <is>
-          <t>Nine metrics - total and annualised return, Sharpe, Calmar, Sortino, maximum drawdown, volatility, plus entropy and effective number of bets from PRUDEX-Compass. "The last two are not defined anywhere beyond the citation, which matters because diversity is one of the two things the title claims." Baselines: rule-based mean-variance, zero mean reversion, time-series momentum; RL - SAC, DeepTrader, AlphaMix+; LLM - FinGPT, FinMem, FinAgent; buy-and-hold per asset. All baselines trained and tested in the same environment with Optuna hyperparameter search.</t>
+          <t>Nine metrics - total and annualised return, Sharpe, Calmar, Sortino, maximum drawdown, volatility, plus entropy and effective number of bets from PRUDEX-Compass. The last two are not defined anywhere beyond the citation, which "matters because diversity is one of the two things the title claims." Baselines: rule-based mean-variance, zero mean reversion, time-series momentum; RL - SAC, DeepTrader, AlphaMix+; LLM - FinGPT, FinMem, FinAgent; buy-and-hold per asset. All baselines trained and tested in the same environment with Optuna hyperparameter search.</t>
         </is>
       </c>
       <c r="S28" s="11" t="inlineStr">
         <is>
-          <t>"71.60% annualised and 405.34% total against the best baseline FinAgent at 53.54% and 261.98%, with Sharpe 2.41 against FinGPT's 1.93, Calmar 11.02 against 7.64 and Sortino 58.00 against 39.57, improvements of 33.75%, 54.72%, 24.49%, 44.28% and 46.58% respectively. Maximum drawdown is 14.21% against FinGPT's 17.08%." Buy-and-hold Bitcoin over the same window: 43.97% total return with 76.63% maximum drawdown. Single-asset (no hedging): "about 210% on Bitcoin, 160% on AAPL and 9% on the yuan, against FinAgent's roughly 135% and FinMem's 120% on AAPL." Ablation: single modules 43.88% (experience sharing), 45.58% (budget allocation), 40.97% (extreme market); pairs 50.68%, 44.57%, 59.81%; full system 71.60%. Removing budget allocation drops to 44.57%; removing extreme-market raises drawdown to 24.44% and cuts Sharpe to 1.93. Memory: activating it raises annualised return by 57.71% and Sharpe by 39.3% against the configuration without it, which implies a no-retrieval annualised return near 45.4% and so a relative drop of 36.6%, "marginally smaller than the 37.7% drop from removing the budget conference, 71.60% to 44.57%". The paper states that "the BAC module has the greatest impact on returns". Backbone sweep: "ChatGLM-6B reports Sharpe 2.88, Calmar 12.26, Sortino 66.64, drawdown 9.19% and volatility 0.78%, every one better than GPT-4's." Diversity: effective number of bets 1.53 against a ceiling of 3; entropy 3.13. Cost: fifteen dollars of API spend over three years; 36 extreme-market sessions fired over nine months. LIMITATIONS (quoting the note): "The expected returns feeding the optimiser are LLM outputs with no calibration, which makes the mean-variance solve look more quantitative than it is.… There is no check that an analyst claiming 12% is better calibrated than one claiming 8%, no interval, and no record of realised against predicted. The optimiser is exact arithmetic over inputs of unknown quality, and a well-specified objective over uncalibrated inputs inherits the uncertainty of the inputs while hiding it behind the precision of the output. This is the sharpest version of the comparable-confidence problem I have seen posed in any paper I have read, and the paper does not pose it." "The allocation is over assets, not over agents, and the two coincide here only because the mapping is one to one.… it means the paper never has to answer how much weight to give an agent whose view overlaps another's, how to combine disagreeing views on the same asset, or what to do when an agent's channel is uninformative. On this design those questions cannot arise, so nothing here bears on them either way." "Three asset classes is a thin basis for a diversification claim, and the paper's own diversity metrics cannot be used to check it… the 'balanced-aware' claim in the title rests on two numbers whose definitions are not given." "No execution friction of any kind." "Three hyperparameters that control the system's behaviour are never given values." "Single runs, no dispersion, no significance testing." Internal contradiction: "the full-system drawdown in this table is 8.68% against 14.21% in Table 1, a direct contradiction between two tables in the same paper for the headline risk metric." And: "on these numbers adding the budget conference buys return by taking on drawdown, which is a coherent result but not the monotone one the discussion describes."</t>
+          <t>71.60% annualised and 405.34% total against the best baseline FinAgent at 53.54% and 261.98%, with Sharpe 2.41 against FinGPT's 1.93, Calmar 11.02 against 7.64 and Sortino 58.00 against 39.57, improvements of "33.75%, 54.72%, 24.49%, 44.28% and 46.58% respectively. Maximum drawdown is 14.21% against FinGPT's 17.08%." Buy-and-hold Bitcoin over the same window: 43.97% total return with 76.63% maximum drawdown. Single-asset (no hedging): "about 210% on Bitcoin, 160% on AAPL and 9% on the yuan, against FinAgent's roughly 135% and FinMem's 120% on AAPL." Ablation: single modules 43.88% (experience sharing), 45.58% (budget allocation), 40.97% (extreme market); pairs 50.68%, 44.57%, 59.81%; full system 71.60%. Removing budget allocation drops to 44.57%; removing extreme-market raises drawdown to 24.44% and cuts Sharpe to 1.93. Memory: activating it raises annualised return by 57.71% and Sharpe by 39.3% against the configuration without it, which implies a no-retrieval annualised return near 45.4% and so a relative drop of 36.6%, "marginally smaller than the 37.7% drop from removing the budget conference, 71.60% to 44.57%". The paper states that the BAC module has the greatest impact on returns. Backbone sweep: "ChatGLM-6B reports Sharpe 2.88, Calmar 12.26, Sortino 66.64, drawdown 9.19% and volatility 0.78%, every one better than GPT-4's." Diversity: effective number of bets 1.53 against a ceiling of 3; entropy 3.13. Cost: fifteen dollars of API spend over three years; 36 extreme-market sessions fired over nine months. LIMITATIONS (quoting the note): The expected returns feeding the optimiser are LLM outputs with no calibration, which makes the mean-variance solve look more quantitative than it is.… There is no check that an analyst claiming 12% is better calibrated than one claiming 8%, no interval, and no record of realised against predicted. The optimiser is exact arithmetic over inputs of unknown quality, and a well-specified objective over uncalibrated inputs inherits the uncertainty of the inputs while hiding it behind the precision of the output. This is the sharpest version of the comparable-confidence problem I have seen posed in any paper I have read, and the paper does not pose it. "The allocation is over assets, not over agents, and the two coincide here only because the mapping is one to one.… it means the paper never has to answer how much weight to give an agent whose view overlaps another's, how to combine disagreeing views on the same asset, or what to do when an agent's channel is uninformative. On this design those questions cannot arise, so nothing here bears on them either way." "Three asset classes is a thin basis for a diversification claim, and the paper's own diversity metrics cannot be used to check it… the 'balanced-aware' claim in the title rests on two numbers whose definitions" are not given. "No execution friction of any kind." "Three hyperparameters that control the system's behaviour are never given values." "Single runs, no dispersion, no significance testing." Internal contradiction: "the full-system drawdown in this table is 8.68% against 14.21% in Table 1, a direct contradiction between two tables in the same paper for the headline risk metric." And: "on these numbers adding the budget conference buys" return by taking on drawdown, which is a coherent result but not the monotone one the discussion describes.</t>
         </is>
       </c>
       <c r="T28" s="11" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="U28" s="11" t="inlineStr">
         <is>
-          <t>"It is the existence proof that the orchestration layer can be a solved optimisation rather than a prompt, and it also shows where that stops working for me… What does not carry over is the one-to-one mapping. My technical, fundamental and volatility agents all look at the same CSE universe, so their weights are influence over a shared decision rather than capital across separate books, and I cannot collapse the two the way this paper does. That difference is the cleanest statement I have of what my weighting function has to do that this one does not." "The conditioning comparison is now a three-way contrast and this paper sits in the middle of it. MacroHFT conditions continuously on trend slope and a realised-volatility tertile but over six identical sub-agents. TradingAgents conditions on nothing. HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies… which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited. My contribution is the continuous version, weights that are a function of liquidity and persistence at every step rather than a scheduled re-solve punctuated by a threshold alarm, and I should put that three-way contrast in the review chapter as a table." "The event-triggered conference is the most transferable mechanism here and it solves a cost problem I have not yet sized… the lesson is to make the costly deliberation conditional on a state trigger and keep the per-day path lightweight. The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." "each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function, reported as a reliability curve per agent, so that the orchestrator combines calibrated probabilities rather than self-reported numbers. That is a component of the build I had listed as an open question and this paper is the reason to promote it to a work item." Entropy diagnostic "needs its formula stated in the text, its logarithm base and range given, the asset set it is computed over named, and a second concentration measure beside it, or it will be as uninterpretable as theirs." Backbone check to be run and reported either way. "The hedging mechanism itself does not port to the CSE and I should say so rather than borrowing the framing… the balance my system can offer has to come from conditioning exposure on liquidity and volatility state instead."</t>
+          <t>"It is the existence proof that the orchestration layer can be a solved optimisation rather than a prompt, and it also shows where that stops working for me… What does not carry over is the one-to-one mapping. My technical, fundamental and volatility agents all look at the same CSE universe, so their weights are influence over a shared decision rather than capital across separate books, and I cannot collapse the two the way this paper does. That difference is the cleanest statement I have of what my weighting function has to do that this one does not." "The conditioning comparison is now a three-way contrast and this paper sits in the middle of it. MacroHFT conditions continuously on trend slope and a realised-volatility tertile but over six identical sub-agents. TradingAgents conditions on nothing. HedgeAgents conditions on a 30-day calendar clock for allocation and on a hand-set amplitude threshold for emergencies… which is market-state-aware in the trigger but not in the weights, since the thresholds are fixed and the allocation between them is not revisited". My contribution is the continuous version, weights that are a function of liquidity and persistence at every step rather than a scheduled re-solve punctuated by a threshold alarm, and I should put that three-way contrast in the review chapter as a table. "The event-triggered conference is the most transferable mechanism here and it solves a cost problem I have not yet sized… the lesson is to make the costly deliberation conditional on a state trigger and keep the per-day path lightweight. The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function, "reported as a reliability curve per agent, so that the orchestrator combines calibrated probabilities rather than self-reported numbers. That is a component of the build I had listed as an open question and this paper is the reason to promote it to a work item." Entropy diagnostic "needs its formula stated in the text, its logarithm base and range given, the asset set it is computed over named, and a second concentration measure beside it, or it will be as uninterpretable as theirs." Backbone check to be run and reported either way. "The hedging mechanism itself does not port to the CSE and I should say so rather than borrowing the framing… the balance my system can offer has to come from conditioning exposure on liquidity and volatility state instead."</t>
         </is>
       </c>
       <c r="V28" s="11" t="inlineStr">
@@ -4097,8 +4097,8 @@
           <t>SPEAKS TO: orchestrator primarily; A_V secondarily (CVaR term, amplitude trigger); friction-aware evaluation layer as a negative example (zero cost).
 EFFECT ON MAIN GAP: Narrows it, does not close it. This is the strongest partial encroachment of the seven on the "influence" side, because the orchestration layer is a real numerical weight vector rather than a prose manager, and because its emergency conference is genuinely state-triggered. But the weights are over assets, and the agent-to-asset mapping is one-to-one by construction, so the paper never confronts overlapping views, disagreement on a shared decision, or an uninformative channel. And the state-awareness lives in a fixed hand-set threshold, not in a function of measured state. The defensible residual: no continuous, measured-state-conditioned weighting of *methodologically heterogeneous* agents over a *shared* decision.
 CONFIDENCE SCORING: Offers the problem, not the solution - ρ_i is a self-reported LLM number entering an exact optimiser. The note's derived mechanism (calibrate each agent against its own realised hit rate on a held-out period, report a reliability curve per agent) is the student's own response, promoted here from open question to work item.
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of a subtle kind. "the experience-sharing plus extreme-market row reports drawdown of 12.02% and Sharpe of 2.24, both better on risk than the full system's Table 1 figures of 14.21% and 2.41 on drawdown, so on these numbers adding the budget conference buys return by taking on drawdown." Also: "the risk-adjusted headline is a backbone choice as much as an architecture result, and the best risk-adjusted configuration of their own system is not the one in Table 1." Neither is detected or responded to by the system.
-PROPOSED REVISION STATED IN THE NOTE: To the conditioning/trigger set, verbatim: "The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." Plus, as a build item: "each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function, reported as a reliability curve per agent." No change to the four-agent pool.</t>
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes, of a subtle kind. the experience-sharing plus extreme-market row reports drawdown of 12.02% and Sharpe of 2.24, both better on risk than the full system's Table 1 figures of 14.21% and 2.41 on drawdown, so on these numbers adding the budget conference buys return by taking on drawdown. Also: "the risk-adjusted headline is a backbone choice as much as an architecture result", and the best risk-adjusted configuration of their own system is not the one in Table 1. Neither is detected or responded to by the system.
+PROPOSED REVISION STATED IN THE NOTE: To the conditioning/trigger set, verbatim: "The CSE analogue of their amplitude threshold should be an Amihud illiquidity spike or a volatility-forecast jump rather than raw price amplitude, since a thin book can produce a 5% move on trivial volume." Plus, as a build item: "each agent's confidence has to be calibrated against its own realised hit rate on a held-out period before it enters the weighting function", reported as a reliability curve per agent. No change to the four-agent pool.</t>
         </is>
       </c>
       <c r="X28" s="11" t="inlineStr">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>CTDE (centralised training, decentralised execution) over a hierarchical, decentralised, partially observable MDP ⟨S, A, P, R, Ω, γ⟩. Global state: S_t = [h^reg_t ⊕ h^ext_t ⊕ m_t ⊕ θ_t], where h^reg_t and h^ext_t are latent context embeddings from Beta and Gamma, m_t current compliance metrics (e.g. a non-compliance count), θ_t the current hyperparameter configuration of the agents. Alpha observes the full global state; Beta and Gamma each receive o^i_t = O(S_t, i) containing only their own text segment and Alpha's instruction. Reward: R^i_total = λ · R_global + (1 − λ) · R^i_local, with R_global a Macro-F1 on compliance classification computed by Alpha, R^i_local the cosine similarity between agent i's output and ground-truth standards or high-confidence pseudo-labels; "The authors swept λ ∈ [0.1, 0.6] and report roughly 0.6 as optimal, with low values producing agent selfishness… and high values producing what they call lazy agents." Parameter adaptation is heuristic: raise learning rate η when TD error δ_t = R^i_total + γV(S_{t+1}) − V(S_t) is positive and lower it otherwise. Retrieval controller state is a JSON object {Current_Query, Retrieval_History, Compliance_Score} with action space {Refine Search, Retrieve Clause, Generate Answer, Halt}, iterated greedily for at most K = 5 steps - "That is a scripted controller with a scoring function, and calling it reinforcement learning is generous." Memory gate: u_t = 1(R^t_global &gt; μ_R + k·σ_R), k = 1.5, over a moving average and rolling sd of the last N global rewards; "The authors tested k ∈ [0.5, 3.0] and report that below 1.0 the policy is high-variance and above 2.0 necessary adaptations are blocked." Symbol collision flagged: k is both memory sensitivity (1.5) and retrieval depth (5). Three agents, all on the same 1.5B base model, "specialised by three mechanisms rather than by architecture." Alpha = orchestrator and trainer, full global state, central critic, holds reward and memory. Beta = regulatory interpretation, regulatory/legal text, role-specific DAPT on regulatory corpus. Gamma = horizon scanning, news/social media/enforcement actions, role-specific DAPT on external corpus. Communication is mediated: Alpha broadcasts τ_t = ⟨Instruction, Data_Pointer, Context⟩; Beta and Gamma return y_t = ⟨Output, Confidence, Metadata⟩. "Direct Beta to Gamma communication is prohibited, enforcing Alpha as the sole mediator." Output is a compliance answer with citations.</t>
+          <t>CTDE (centralised training, decentralised execution) over a hierarchical, decentralised, partially observable MDP ⟨S, A, P, R, Ω, γ⟩. Global state: S_t = [h^reg_t ⊕ h^ext_t ⊕ m_t ⊕ θ_t], where h^reg_t and h^ext_t are latent context embeddings from Beta and Gamma, m_t current compliance metrics (e.g. a non-compliance count), θ_t the current hyperparameter configuration of the agents. Alpha observes the full global state; Beta and Gamma each receive o^i_t = O(S_t, i) containing only their own text segment and Alpha's instruction. Reward: R^i_total = λ · R_global + (1 − λ) · R^i_local, with R_global a Macro-F1 on compliance classification computed by Alpha, R^i_local the cosine similarity between agent i's output and ground-truth standards or high-confidence pseudo-labels; The authors swept λ ∈ ["0.1, 0.6] and report roughly 0.6 as optimal, with low values producing agent selfishness… and high values producing what they call lazy agents." Parameter adaptation is heuristic: raise learning rate η when TD error δ_t = R^i_total + γV(S_{t+1}) − V(S_t) is positive and lower it otherwise. Retrieval controller state is a JSON object {Current_Query, Retrieval_History, Compliance_Score} with action space {Refine Search, Retrieve Clause, Generate Answer, Halt}, iterated greedily for at most K = 5 steps - "That is a scripted controller with a scoring function, and calling it reinforcement learning is generous." Memory gate: u_t = 1(R^t_global &gt; μ_R + k·σ_R), k = 1.5, over a moving average and rolling sd of the last N global rewards; The authors tested k ∈ ["0.5, 3.0] and report that below 1.0 the policy is high-variance and above 2.0 necessary adaptations are blocked." Symbol collision flagged: k is both memory sensitivity (1.5) and retrieval depth (5). Three agents, all on the same 1.5B base model, "specialised by three mechanisms rather than by architecture." Alpha = orchestrator and trainer, full global state, central critic, holds reward and memory. Beta = regulatory interpretation, regulatory/legal text, role-specific DAPT on regulatory corpus. Gamma = horizon scanning, news/social media/enforcement actions, role-specific DAPT on external corpus. Communication is mediated: Alpha broadcasts τ_t = ⟨Instruction, Data_Pointer, Context⟩; Beta and Gamma return y_t = ⟨Output, Confidence, Metadata⟩. "Direct Beta to Gamma communication is prohibited, enforcing Alpha as the sole mediator." Output is a compliance answer with citations.</t>
         </is>
       </c>
       <c r="L29" s="11" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="S29" s="11" t="inlineStr">
         <is>
-          <t>Full system precision 0.94 / recall 0.92 / F1 0.93. Lexical only: recall 0.70, F1 0.76. Vector only: 0.89 / 0.81 / 0.85. No fine-tuning: 0.82 / 0.79 / 0.80. No iterative RL retrieval loop: 0.88 / 0.85 / 0.86. Retrieval depth: "F1 rises from 0.68 at k = 1 to 0.93 at k = 5, then falls monotonically to 0.74 at k = 20, driven by precision collapsing from 0.96 to roughly 0.45 while recall saturates near 1.0"; "adding fifteen more chunks costs 0.19 F1." Rubric: TRIAG 4.118 fluency, 4.612 relevance, 4.204 domain correctness, 4.087 consistency, 4.652 factuality, against deepseek-r1 7B's 4.062 / 3.941 / 4.021 / 4.291 / 4.427 - "Relevance and factuality move most, consistency is the one that goes backwards." Cost reduction ~96% vs GPT-4o, 97.3% vs Llama-3-70B. LIMITATIONS (quoting the note): "RQ2 asks whether coordinated agents outperform independent single-agent baselines and the paper never runs that experiment. There is no single-agent baseline anywhere, no two-agent configuration, no variant where Alpha does Beta's and Gamma's work itself… I should cite TRIAG as an architecture proposal with a retrieval evaluation attached rather than as evidence that MARL coordination helps." "Nothing in the evaluation is externally checkable, and the tuning results carry no variance… the selected λ ≈ 0.6 sits on the boundary of the swept interval [0.1, 0.6], which usually means the optimum lies outside the range tested." "The Confidence field is declared in the communication protocol and then never used. Beta and Gamma return ⟨Output, Confidence, Metadata⟩, and confidence appears in no reward term, no fusion rule, no state block and no experiment. Output fusion is described as Alpha integrating the structured outputs using weighted logic with an adaptive thresholding mechanism based on statistical process control, and no weights, no thresholds and no fusion equations are given. The single most load-bearing mechanism for my project is the one the paper states in prose and never specifies." "Homogeneity is acknowledged, defended weakly, and left untested… there is no measurement of divergence between Beta and Gamma after adaptation, and heterogeneous architectures are deferred to future work." "The local reward rests on cosine similarity to ground truth… an agent optimising cosine similarity to reference text is rewarded for paraphrasing the source, which is a proxy for retrieval fidelity and not for correctness, and it will score a fluent, well-grounded wrong answer highly whenever the wrong answer is lexically close to the right clause."</t>
+          <t>Full system precision 0.94 / recall 0.92 / F1 0.93. Lexical only: recall 0.70, F1 0.76. Vector only: 0.89 / 0.81 / 0.85. No fine-tuning: 0.82 / 0.79 / 0.80. No iterative RL retrieval loop: 0.88 / 0.85 / 0.86. Retrieval depth: "F1 rises from 0.68 at k = 1 to 0.93 at k = 5, then falls monotonically to 0.74 at k = 20, driven by precision collapsing from 0.96 to roughly 0.45 while recall saturates near 1.0"; "adding fifteen more chunks costs 0.19 F1." Rubric: TRIAG 4.118 fluency, 4.612 relevance, 4.204 domain correctness, 4.087 consistency, 4.652 factuality, against deepseek-r1 7B's 4.062 / 3.941 / 4.021 / 4.291 / 4.427 - "Relevance and factuality move most, consistency is the one that goes backwards." Cost reduction ~96% vs GPT-4o, 97.3% vs Llama-3-70B. LIMITATIONS (quoting the note): "RQ2 asks whether coordinated agents outperform independent single-agent baselines and the paper never runs that experiment. There is no single-agent baseline anywhere, no two-agent configuration, no variant where Alpha does Beta's and Gamma's work itself… I should cite TRIAG as an architecture proposal with a retrieval evaluation attached rather than as evidence that MARL coordination helps." Nothing in the evaluation is externally checkable, and the tuning results carry no variance… the selected λ ≈ 0.6 sits on the boundary of the swept interval [0.1, 0.6], which usually means the optimum lies outside the range tested. The Confidence field is declared in the communication protocol and then never used. Beta and Gamma return ⟨Output, Confidence, Metadata⟩, and confidence appears in no reward term, no fusion rule, no state block and no experiment. Output fusion is described as Alpha integrating the structured outputs using weighted logic with an adaptive thresholding mechanism based on statistical process control, and no weights, no thresholds and no fusion equations are given. The single most load-bearing mechanism for my project is the one the paper states in prose and never specifies. "Homogeneity is acknowledged, defended weakly, and left untested… there is no measurement of divergence between Beta and Gamma after adaptation, and heterogeneous architectures are deferred to future work." "The local reward rests on cosine similarity to ground truth… an agent optimising cosine similarity to reference text is rewarded for paraphrasing the source, which is a proxy for retrieval fidelity and not for correctness, and it will score a fluent, well-grounded wrong answer highly whenever the wrong answer is lexically close to the right clause."</t>
         </is>
       </c>
       <c r="T29" s="11" t="inlineStr">
@@ -4221,9 +4221,9 @@
       <c r="W29" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator (λ credit-assignment split, memory gate, the negative example of the conditioning set) and A_F (hybrid dense+sparse retrieval, k = 5 budget, chunking critique).
-EFFECT ON MAIN GAP: Leaves it open and strengthens it. This is the closest published orchestrator in the set that writes down an explicit reward decomposition, an explicit state vector and an explicit agent output contract carrying a confidence field - and it still does not condition influence on environment state, and never computes with the confidence field. It is "the second instance after MacroHFT of state-aware coordination over components that are architecturally identical, which sharpens rather than threatens the heterogeneity claim." Scoped claim the note now defends: "weighting an econometric estimator against an LLM analyst against an RL allocator is a configuration I have not found in the reviewed literature, to be validated against further recent work, and the pre-registered weight-entropy diagnostic still applies, since if my weights collapse to one-hot I have built a router and have to say so."
+EFFECT ON MAIN GAP: Leaves it open and strengthens it. This is the closest published orchestrator in the set that writes down an explicit reward decomposition, an explicit state vector and an explicit agent output contract carrying a confidence field - and it still does not condition influence on environment state, and never computes with the confidence field. It is the second instance after MacroHFT "of state-aware coordination over components that are architecturally identical, which sharpens rather than threatens the heterogeneity claim." Scoped claim the note now defends: "weighting an econometric estimator against an LLM analyst against an RL allocator is a configuration I have not found in the reviewed literature, to be validated against further recent work, and the pre-registered weight-entropy diagnostic still applies, since if my weights collapse to one-hot I have built a router and have to say so."
 CONFIDENCE SCORING: No mechanism - the strongest negative result in the set on this question. The field exists in the protocol and in a figure and is never used. The note pairs it with the "Correct / Incorrect / Uncertain contract in Enhancing Anomaly Detection in Financial Markets with an LLM-Based Multi-Agent Framework, which is the only concrete cross-agent output vocabulary I have found."
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes, by omission rather than ablation: "Gamma's brief includes sentiment analysis and no sentiment result is reported anywhere… this is another component whose influence is fixed by design and never measured, which is the same failure shape as the auxiliary strategies in FinAgent and the dropped sentiment agent in AlphaAgents, reached here by omission rather than by ablation."
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes, by omission rather than ablation: "Gamma's brief includes sentiment analysis and no sentiment result is reported anywhere… this is another component whose influence is fixed by design and never measured, which is the same failure shape as the auxiliary strategies in FinAgent and the dropped sentiment agent in AlphaAgents", reached here by omission rather than by ablation.
 PROPOSED REVISION STATED IN THE NOTE: To the reward/credit structure and the update trigger, verbatim: "The TRIAG form gives each agent a local term scored against something it controls, a realised volatility forecast error for A_V, a spread or impact prediction error for A_L, a retrieval citation check for A_F, combined with the portfolio-level result through a single mixing weight… so this goes into the design as a mechanism with a pre-registered sweep rather than a fixed value, and the boundary-optimum problem in their sweep means my range has to extend past 0.6." And: "TRIAG updates on unusually good performance and what I need is an update on unusually *bad* performance, a regime break, so the gate becomes two-sided." No change to the four-agent pool; the conditioning set is defended unchanged, with the TRIAG state vector cited as the degenerate counterexample justifying the Adaptive − Liquidity and Adaptive − Volatility ablations.</t>
         </is>
       </c>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>US equities, options and crypto. "The CSE has no options market, no minute-level vendor feed I can license, and no news API with ticker-tagged significance ratings. The data layer is a design pattern I can copy, not software I can run."  Data access, event retrieval, brokerage simulation, tool-call evaluation.</t>
+          <t>US equities, options and crypto. The CSE has no options market, no minute-level vendor feed I can license, and no news API with ticker-tagged significance ratings. "The data layer is a design pattern I can copy, not software I can run." Data access, event retrieval, brokerage simulation, tool-call evaluation.</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="L30" s="11" t="inlineStr">
         <is>
-          <t>- Effectively two in the demonstration, an analysis agent and a trading agent, in a fixed pipeline. Not a multi-agent contribution. - Combination: sequential handoff. "There is no orchestration here, no weighting, no policy, nothing deciding which of several opinions to act on… the same fixed-influence pattern already documented in FinAgent and AlphaAgents." - Anything varying influence by state? No. Explicitly: "the paper contributes nothing to the weighting problem and does not compete with it either." - Confidence per agent: none.</t>
+          <t>- Effectively two in the demonstration, an analysis agent and a trading agent, in a fixed pipeline. Not a multi-agent contribution. - Combination: sequential handoff. "There is no orchestration here, no weighting, no policy, nothing deciding which of several opinions to act on… the same fixed-influence pattern already documented in" FinAgent and AlphaAgents. - Anything varying influence by state? No. Explicitly: "the paper contributes nothing to the weighting problem and does not compete with it either." - Confidence per agent: none.</t>
         </is>
       </c>
       <c r="M30" s="11" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="S30" s="11" t="inlineStr">
         <is>
-          <t>Tool Calling Overall - Gemini 2.5 Flash 91.00, Gemini 2.5 Pro 91.00, GPT-4.1 87.33, GPT-4.1 Mini 84.33, DeepSeek Chat 88.00, Qwen2.5 7B Instruct 78.33, Llama 3.1 8B Instruct 62.33, Qwen3 4B Instruct 86.33. Task Planning Overall - 92.33, 93.67, 93.67, 92.00, 95.00, 87.67, 84.67, 86.33. "TM sits between 0.90 and 0.97 for seven of the eight models, including Qwen3 4B at 0.93, while PA and TA are below TM in every single row without exception." "Multi-step planning scores higher than single-step tool calling for seven of the eight models, which is backwards" - Llama 3.1 8B goes 62.33 → 84.67, Qwen2.5 7B 78.33 → 87.67. LIMITATIONS (quoting the note): "The Overall column does not support the reading it invites, for two separate reasons.… averaging TM, PA and TA weights three unlike failures equally: picking the wrong tool usually produces an error the agent can see, while a wrong argument or a wrong timestamp produces a plausible answer nothing downstream flags… Carry the three components, read the table as three tiers, and leave Overall alone." "The instructions and the gold traces are both LLM-generated." "PMB simulates the brokerage, not the market." "The reproducibility argument is undercut by the data licensing… deterministic replay guarantees reproducibility within a lab and not across labs. Given that a standardised, reproducible environment is the paper's central claim, this is the limitation that most constrains what it actually delivers." "Module naming is inconsistent between the prose and the implementation" (ESP in text, NPP in figures). On TA specifically: "TA's bands are generous, plus or minus one calendar day for daily fields and plus or minus two days for loose windows, so a TA of 0.86 means a real fraction of calls miss by more than a full day. In an interactive assistant that is a rounding error, in a backtest it is a lookahead hazard."</t>
+          <t>Tool Calling Overall - Gemini 2.5 Flash 91.00, Gemini 2.5 Pro 91.00, GPT-4.1 87.33, GPT-4.1 Mini 84.33, DeepSeek Chat 88.00, Qwen2.5 7B Instruct 78.33, Llama 3.1 8B Instruct 62.33, Qwen3 4B Instruct 86.33. Task Planning Overall - 92.33, 93.67, 93.67, 92.00, 95.00, 87.67, 84.67, 86.33. "TM sits between 0.90 and 0.97 for seven of the eight models, including Qwen3 4B at 0.93", while PA and TA are below TM in every single row without exception. "Multi-step planning scores higher than single-step tool calling for seven of the eight models, which is backwards" - Llama 3.1 8B goes 62.33 → 84.67, Qwen2.5 7B 78.33 → 87.67. LIMITATIONS (quoting the note): "The Overall column does not support the reading it invites, for two separate reasons.… averaging TM, PA and TA weights three unlike failures equally: picking the wrong tool usually produces an error the agent can see, while a wrong argument or a wrong timestamp produces a plausible answer nothing downstream flags… Carry the three components, read the table as three tiers, and leave Overall alone." "The instructions and the gold traces are both LLM-generated." "PMB simulates the brokerage, not the market." "The reproducibility argument is undercut by the data licensing… deterministic replay guarantees reproducibility within a lab and not across labs. Given that a standardised, reproducible environment is the paper's central claim, this is the limitation that most constrains what it actually delivers." "Module naming is inconsistent between the prose and the implementation" (ESP in text, NPP in figures). On TA specifically: "TA's bands are generous, plus or minus one calendar day for daily fields and plus or minus two days for loose windows, so a TA of 0.86 means a real fraction of calls miss by more than a full day. In an interactive assistant that is a rounding error, in a backtest it is a lookahead hazard."</t>
         </is>
       </c>
       <c r="T30" s="11" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Brittleness of deep learning in quant finance, decomposed into three challenges - "traditional alpha mining methods are rigid and do not adapt to dynamic markets, machine learning approaches struggle to integrate diverse data, and strategies do not adapt to market variability." Three-stage pipeline: LLMs generate executable alpha factor candidates from the alpha-mining literature; a multi-agent evaluation filters them on market status and predictive quality while maintaining category balance; a weight optimisation stage combines the survivors. Most important framing in the note: "I came to this from the BlackRock survey, which describes it as employing an adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions. That is not what the paper does, and the difference is the most useful thing I got out of reading it. The adaptivity here is at selection, not at weighting."</t>
+          <t>Brittleness of deep learning in quant finance, decomposed into three challenges - "traditional alpha mining methods are rigid and do not adapt to dynamic markets, machine learning approaches struggle to integrate diverse data, and strategies do not adapt to market variability." Three-stage pipeline: LLMs generate executable alpha factor candidates from the alpha-mining literature; a multi-agent evaluation filters them on market status and predictive quality while maintaining category balance; a weight optimisation stage combines the survivors. Most important framing in the note: I came to this from the BlackRock survey, which describes it as employing an adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions. That is not what the paper does, and the difference is the most useful thing I got out of reading it. The adaptivity here is at selection, not at weighting.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -4407,17 +4407,17 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>OHLCV + VWAP + financial reports. Seed alpha library from eleven documents given to GPT-4o including Kakushadze's *101 Formulaic Alphas* and Lopez de Prado's *Causal Factor Investing*. Every object is a formulaic alpha, "a short arithmetic expression over OHLCV and fundamentals such as CLOSE - DELAY(SMA(CLOSE, 14), 7)." Counts do not hold up: "the appendix taxonomy is introduced as eight categories and then lists nine, and the actual experimental prompt in A.7 describes 37 factors in eight groups. Liquidity is a category in the taxonomy, is absent from the eight groups the experiment's prompt actually names, and is absent from the five categories evaluated in Table 2, yet two liquidity expressions appear in the twelve selected alphas of Table 3."</t>
+          <t>OHLCV + VWAP + financial reports. Seed alpha library from eleven documents given to GPT-4o including Kakushadze's *101 Formulaic Alphas* and Lopez de Prado's *Causal Factor Investing*. Every object is a formulaic alpha, "a short arithmetic expression over OHLCV and fundamentals such as CLOSE - DELAY(SMA(CLOSE, 14), 7)." Counts do not hold up: the appendix taxonomy is introduced as eight categories and then lists nine, and the actual experimental prompt in A.7 describes 37 factors in eight groups. "Liquidity is a category in the taxonomy, is absent from the eight groups the experiment's prompt actually names, and is absent from the five categories evaluated in Table 2, yet two liquidity expressions appear in the twelve selected alphas of Table 3."</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Phase 2 - two agents each score every candidate alpha α_ij in category j against market condition M^(t): θ_ij = E[IC(α_ij | M^(t))] from the Confidence Score Agent, and ρ_ij = f_risk(α_ij, M^(t)) from the Risk Preference Agent. Mixed linearly with the best-scoring alpha in each category kept, subject to a confidence threshold: α*_j = argmax_{α_ij} [w_c · θ_ij + w_r · ρ_ij]. Phase 3 - a three-layer MLP, input width equal to the number of selected alphas, ten ReLU hidden nodes, one output, mapping historical daily alpha values to future yields, with a held-out validation set; its learned parameters become the combination weights. Composite signal: α^(t)_i = Σ_j w_j · α^(t)_ij. "Read the subscripts. The alpha values carry t, the weights do not, here or in Algorithm 2 line 30 or in the paper's equation 8. The abstract's 'dynamic weight optimization that adapts to market conditions' and the survey's 'real time' gating both describe w_j as though it were w_j^(t), and nothing in the method produces that. The weights change when the model is retrained on a new window, which is retraining, not gating." Three-stage pipeline → composite alpha → portfolio. A.8: "daily reconstruction, rank all securities by composite alpha, take the top k = 13, limit churn to n = 5 names per day, equal weight across holdings. That is roughly 38% daily turnover, which the paper states and then never prices."</t>
+          <t>Phase 2 - two agents each score every candidate alpha α_ij in category j against market condition M^(t): θ_ij = E[IC(α_ij | M^(t))] from the Confidence Score Agent, and ρ_ij = f_risk(α_ij, M^(t)) from the Risk Preference Agent. Mixed linearly with the best-scoring alpha in each category kept, subject to a confidence threshold: α*_j = argmax_{α_ij} [w_c · θ_ij + w_r · ρ_ij]. Phase 3 - a three-layer MLP, input width equal to the number of selected alphas, ten ReLU hidden nodes, one output, mapping historical daily alpha values to future yields, with a held-out validation set; its learned parameters become the combination weights. Composite signal: α^(t)_i = Σ_j w_j · α^(t)_ij. Read the subscripts. "The alpha values carry t, the weights do not, here or in Algorithm 2 line 30 or in the paper's equation 8. The abstract's 'dynamic weight optimization that adapts to market conditions' and the survey's 'real time' gating both describe w_j as though it were w_j^(t), and nothing in the method produces that. The weights change when the model is retrained on a new window, which is retraining, not gating." Three-stage pipeline → composite alpha → portfolio. A.8: "daily reconstruction, rank all securities by composite alpha, take the top k = 13, limit churn to n = 5 names per day, equal weight across holdings. That is roughly 38% daily turnover", which the paper states and then never prices.</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>- Two agents in Phase 2 plus an MLP in Phase 3. Homogeneous in evidence type: "the paper is not proposing a new way to combine heterogeneous *analysts*. Every object in the system is a formulaic alpha… The two agents both evaluate those same expressions. This is one evidence type scored two ways, not four evidence types that have to be reconciled." Confidence Score Agent sees candidate alphas plus the market condition M^(t) and outputs an expected conditional IC; Risk Preference Agent sees the same and outputs a risk-character score. - Combination: two stages. Agent scores are mixed by a fixed linear rule α*_j = argmax [w_c θ_ij + w_r ρ_ij] with w_c = 0.6, w_r = 0.4; the surviving factors are combined by a static MLP whose weights carry no time index. - Does anything vary influence by market state? Selection yes, weighting no - and this is the single most important correction in the note. Which factors enter is conditioned on M^(t), because M^(t) is passed to both evaluating agents. How much each selected factor counts is "a weight vector produced once by a small MLP trained on a fixed historical window, and it carries no time index anywhere in the paper's equations or in its algorithm listing." Quoting the note's headline: "The adaptivity here is at selection, not at weighting." And: "So this is not a competitor to my orchestrator. It is the strongest published instantiation I have of Baseline 2, the static learned weight, which the supervisor identified as the baseline that actually matters, and it is the reference design I should implement that arm against." - Confidence per agent: yes, and it is the most directly reusable confidence construct in the set - θ_ij = E[IC(α_ij | M^(t))], an expected conditional information coefficient, paired with a separate risk score, mixed linearly. Comparability is trivial here because both scores are over the same object type. The note's port: "each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target."</t>
+          <t>- Two agents in Phase 2 plus an MLP in Phase 3. Homogeneous in evidence type: "the paper is not proposing a new way to combine heterogeneous *analysts*. Every object in the system is a formulaic alpha… The two agents both evaluate those same expressions. This is one evidence type scored two ways, not four evidence types that have to be reconciled." Confidence Score Agent sees candidate alphas plus the market condition M^(t) and outputs an expected conditional IC; Risk Preference Agent sees the same and outputs a risk-character score. - Combination: two stages. Agent scores are mixed by a fixed linear rule α*_j = argmax [w_c θ_ij + w_r ρ_ij] with w_c = 0.6, w_r = 0.4; the surviving factors are combined by a static MLP whose weights carry no time index. - Does anything vary influence by market state? Selection yes, weighting no - and this is the single most important correction in the note. Which factors enter is conditioned on M^(t), because M^(t) is passed to both evaluating agents. How much each selected factor counts is "a weight vector produced once by a small MLP trained on a fixed historical window, and it carries no time index anywhere in the paper's equations or in its algorithm listing." Quoting the note's headline: "The adaptivity here is at selection, not at weighting." And: "So this is not a competitor to my orchestrator. It is the strongest published instantiation I have of" Baseline 2, the static learned weight, which the supervisor identified as the baseline that actually matters, and it is the reference design I should implement that arm against. - Confidence per agent: yes, and it is the most directly reusable confidence construct in the set - θ_ij = E[IC(α_ij | M^(t))], an expected conditional information coefficient, paired with a separate risk score, mixed linearly. Comparability is trivial here because both scores are over the same object type. The note's port: "each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target."</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="Q31" s="3" t="inlineStr">
         <is>
-          <t>Factors are human-readable arithmetic expressions; the weights come from an MLP, so the combination is not interpretable. IC sign confusion undermines readability: "Table 3's weighted combination scores −0.0587 against individual alphas in the ±0.02 range, and the text calls this 'quite high', reading the magnitude and ignoring the sign."</t>
+          <t>Factors are human-readable arithmetic expressions; the weights come from an MLP, so the combination is not interpretable. IC sign confusion undermines readability: Table 3's weighted combination scores −0.0587 against individual alphas in the ±"0.02 range, and the text calls this 'quite high', reading the magnitude and ignoring the sign."</t>
         </is>
       </c>
       <c r="R31" s="3" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="S31" s="3" t="inlineStr">
         <is>
-          <t>"Removing the Confidence Score Agent drops out-of-sample IC from 0.047 to 0.032, a 31.9% fall, and removing the Risk Preference Agent drops it to 0.039." Full model 0.059 in-sample / 0.047 out-of-sample / Sharpe 1.94; without Confidence 0.054 / 0.032 / 1.51; without Risk 0.056 / 0.039 / 1.34. Regime: "the full model holds out-of-sample IC at 0.051 bull, 0.042 bear and 0.045 sideways, while without the confidence agent the bear-market figure collapses to 0.021, half the full model's. On this sample, conditioning *which* factors are used on the market state is doing real work, and it is doing most of it when conditions are bad." Headline "53.17% is gross, on 38% daily turnover, against a benchmark of −13.22%." Sensitivity sweep of the confidence/risk mix: overall Sharpe 8.10, −2.68, 11.39, −5.10, −8.04, 9.00, −4.35 across the seven settings, with the chosen 0.6/0.4 at 11.39 "sitting directly between two negative results." Regularisation 0.0005 / 0.001 / 0.002 gives −1.88 / 13.33 / −6.91. Drawdown: "maximum drawdown is deeper than the benchmark's in four, −19.40 against −10.86 and −17.03 against −8.44 on CSI300, −7.89 against −4.23 and −11.52 against −7.75 on SP500, and shallower only in the H1 2022 downturn in both markets." LIMITATIONS (quoting the note): "The comparison that would isolate the weighting stage is not run. Both ablations remove an *agent* from the selection phase. Neither removes the MLP, so there is no arm anywhere in the paper showing what an equal-weighted combination of the same twelve selected alphas would have returned, and therefore no evidence that learning the weights contributes anything over the selection that precedes it… This is the limitation that most directly shapes my own design, because the missing arm is exactly the comparison my three-way weighting study is built to make." "Look-ahead exposure is structural and unaddressed. GPT-4o, whose training data extends well past the 2023 test period, is asked in the A.7 prompt to 'select the factors that will perform best in the last quarter of the SSE 50' for the test window… The paper offers no contamination check… That does not mean the result is contaminated, it means the paper provides nothing that would let me rule it out, and the effect would look exactly like the reported outperformance." "The Sharpe ratio is reported on at least three mutually incompatible scales and the convention is never stated… No equity strategy has a Sharpe of 13, so at least two of these tables are measuring something other than what the label says… only the within-table comparisons are readable and no number here can be carried into a sentence of mine." "The sensitivity studies show instability rather than sensitivity… a surface that alternates sign under a one-step parameter change is not a surface with an optimum on it, and the reported configuration is better described as the best of a noisy sweep than as a tuned choice." "The two metrics in that ablation disagree about which agent matters, and the paper reports only one of the answers." "Internal inconsistencies are frequent enough to affect how much weight any single figure can bear."</t>
+          <t>"Removing the Confidence Score Agent drops out-of-sample IC from 0.047 to 0.032, a 31.9% fall, and removing the Risk Preference Agent drops it to 0.039." Full model 0.059 in-sample / 0.047 out-of-sample / Sharpe 1.94; without Confidence 0.054 / 0.032 / 1.51; without Risk 0.056 / 0.039 / 1.34. Regime: "the full model holds out-of-sample IC at 0.051 bull, 0.042 bear and 0.045 sideways, while without the confidence agent the bear-market figure collapses to 0.021, half the full model's. On this sample, conditioning *which* factors are used on the market state is doing real work, and it is doing most of it when conditions are bad." Headline "53.17% is gross, on 38% daily turnover, against a benchmark of −13.22%." Sensitivity sweep of the confidence/risk mix: overall Sharpe 8.10, −2.68, 11.39, −5.10, −8.04, 9.00, −4.35 across the seven settings, with the chosen 0.6/0.4 at 11.39 "sitting directly between two negative results." Regularisation 0.0005 / 0.001 / 0.002 gives −1.88 / 13.33 / −6.91. Drawdown: "maximum drawdown is deeper than the benchmark's in four, −19.40 against −10.86 and −17.03 against −8.44 on CSI300, −7.89 against −4.23 and −11.52 against −7.75 on SP500, and shallower only in the H1 2022 downturn in both markets." LIMITATIONS (quoting the note): The comparison that would isolate the weighting stage is not run. "Both ablations remove an *agent* from the selection phase. Neither removes the MLP, so there is no arm anywhere in the paper showing what an equal-weighted combination of the same twelve selected alphas would have returned, and therefore no evidence that learning the weights contributes anything over the selection that precedes it… This is the limitation that most directly shapes my own design, because the missing arm is exactly the comparison my three-way weighting study is built to make." "Look-ahead exposure is structural and unaddressed. GPT-4o, whose training data extends well past the 2023 test period, is asked in the A.7 prompt to 'select the factors that will perform best in the last quarter of the SSE 50' for the test window… The paper offers no contamination check… That does not mean the result is contaminated, it means the paper provides nothing that would let me rule it out, and the effect would look exactly like the reported outperformance." "The Sharpe ratio is reported on at least three mutually incompatible scales and the convention is never stated… No equity strategy has a Sharpe of 13, so at least two of these tables are measuring something other than what the label says… only the within-table comparisons are readable and no number here can be carried into a sentence of mine." "The sensitivity studies show instability rather than sensitivity… a surface that alternates sign under a one-step parameter change is not a surface with an optimum on it, and the reported configuration is better described as the best of a noisy sweep than as a tuned choice." "The two metrics in that ablation disagree about which agent matters, and the paper reports only one of the answers." "Internal inconsistencies are frequent enough to affect how much weight any single figure can bear."</t>
         </is>
       </c>
       <c r="T31" s="3" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="U31" s="3" t="inlineStr">
         <is>
-          <t>"This is my static-learned-weight baseline, and I should build that arm to this design rather than to a strawman. Baseline 2 is the one the supervisor singled out, because beating equal weighting proves little if a fixed learned weight gets there too, and until now I had no reference implementation of it… The comparison this paper never runs, equal weight against learned static weight over an identical input set, is the first half of my experimental design, and I can now say plainly in the write-up that the nearest prior work does not report it." "Adaptivity at selection and adaptivity at weighting are separable, and I should evaluate both. This system conditions which factors are in the set on the market state and then weights them statically. Mine conditions the weights and keeps the agent set fixed… so the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically, and I would rather find that out in my own ablation than have it raised in a viva." "Keep the orchestrator low-capacity. A ten-node MLP over roughly twelve inputs, trained on a fifty-stock universe with eighteen months of daily data, produces a Sharpe surface that flips sign when L2 regularisation moves from 0.001 to 0.002… That argues for a weighting function with a handful of interpretable parameters, a gated linear form or a shallow regression on the four state variables, rather than a network, and it argues for reporting the stability sweep rather than only the tuned configuration." "The two-agent scoring scheme is a usable template for the agent-confidence term, with one caution attached. Expected conditional information coefficient as a confidence score and a separate risk-character score, mixed linearly, is implementable for my four agents as each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target. The caution is that the mixing ratio between the two components is exactly the parameter this paper's sensitivity table shows to be unstable, so if I adopt a two-component confidence I fix that ratio on the validation split and report the sweep, rather than selecting it on the test window as this paper appears to." "The liquidity factor definitions transfer to the CSE even though the experiment's factor set excludes them. Amihud illiquidity as ABS(RETURN) / VOLUME, turnover as VOLUME / SHARES_OUTSTANDING, the high-low spread proxy (HIGH - LOW) / CLOSE and VOLUME / MARKET_CAP are all computable from the OHLCV and shares-outstanding data I expect to have, with no quote feed required, and the high-low proxy is the one that survives if I never get bid-ask data." "Gross returns on 38% daily turnover make the friction layer a contribution rather than housekeeping… The turnover constraint itself, cap the number of names replaced per session rather than the fraction of capital traded, is a clean mechanism worth borrowing." "They name the stationarity assumption behind state-conditional weighting and do not test it, which is precisely my persistence ablation. Their own limitations section states that the multi-agent evaluation presupposes persistent historical relationships between market conditions and alpha performance, an assumption that may prove tenuous during regime shifts. That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." "Prompt hygiene needs to be a stated part of my method… the evaluation window must not be named in any prompt, the agent instructions must not ask which factors performed best in a period that overlaps the test set, and I should report a contamination check of some kind."</t>
+          <t>"This is my static-learned-weight baseline, and I should build that arm to this design rather than to a strawman. Baseline 2 is the one the supervisor singled out, because beating equal weighting proves little if a fixed learned weight gets there too, and until now I had no reference implementation of it… The comparison this paper never runs, equal weight against learned static weight over an identical input set, is the first half of my experimental design, and I can now say plainly in the write-up that the nearest prior work does not report it." "Adaptivity at selection and adaptivity at weighting are separable, and I should evaluate both. This system conditions which factors are in the set on the market state and then weights them statically. Mine conditions the weights and keeps the agent set fixed… so the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically, and I would rather find that out in my own ablation than have it raised in a viva." Keep the orchestrator low-capacity. "A ten-node MLP over roughly twelve inputs, trained on a fifty-stock universe with eighteen months of daily data, produces a Sharpe surface that flips sign when L2 regularisation moves from 0.001 to 0.002… That argues for a weighting function with a handful of interpretable parameters, a gated linear form or a shallow regression on the four state variables, rather than a network, and it argues for reporting the stability sweep rather than only the tuned configuration." "The two-agent scoring scheme is a usable template for the agent-confidence term, with one caution attached. Expected conditional information coefficient as a confidence score and a separate risk-character score, mixed linearly, is implementable for my four agents as each agent's historical hit rate conditional on the current liquidity and volatility state, and it needs no labelled confidence target. The caution is that the mixing ratio between the two components is exactly the parameter this paper's sensitivity table shows to be unstable, so if I adopt a two-component confidence I fix that ratio on the validation split and report the sweep, rather than selecting it on the test window as this paper appears to." "The liquidity factor definitions transfer to the CSE even though the experiment's factor set excludes them. Amihud illiquidity as ABS(RETURN) / VOLUME, turnover as VOLUME / SHARES_OUTSTANDING, the high-low spread proxy (HIGH - LOW) / CLOSE and VOLUME / MARKET_CAP are all computable from the OHLCV and shares-outstanding data I expect to have, with no quote feed required, and the high-low proxy is the one that survives if I never get bid-ask data." "Gross returns on 38% daily turnover make the friction layer a contribution rather than housekeeping… The turnover constraint itself, cap the number of names replaced per session rather than the fraction of capital traded, is a clean mechanism worth borrowing." "They name the stationarity assumption behind state-conditional weighting and do not test it, which is precisely my persistence ablation. Their own limitations section states that the multi-agent evaluation presupposes persistent historical relationships between market conditions and alpha performance, an assumption that may prove tenuous during regime shifts. That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment" I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four. "Prompt hygiene needs to be a stated part of my method… the evaluation window must not be named in any prompt, the agent instructions must not ask which factors performed best in a period that overlaps the test set, and I should report a contamination check of some kind."</t>
         </is>
       </c>
       <c r="V31" s="3" t="inlineStr">
@@ -4476,7 +4476,7 @@
 EFFECT ON MAIN GAP: Leaves it open - and the note's rereading of this paper is what keeps it open. The BlackRock survey had nominated it as the nearest prior art with a "dynamic weighting mechanism"/"adaptive gating mechanism that tunes the influence of each signal in real time." On the paper's own equations that description is unsupported. Net effect: the one candidate the field itself pointed at as occupying the gap turns out to be a static-learned-weight baseline. It does, however, narrow the gap in one direction - it demonstrates that state-conditional *selection* carries real signal, mostly in bear regimes (bear IC 0.042 full vs 0.021 without the confidence agent), which obliges the student to add a state-conditional-inclusion / static-weight configuration to their own ablation to prove the weighting function is what is doing the work.
 CONFIDENCE SCORING: Yes - the cleanest formal template in the set, though not a cross-*heterogeneity* solution. Expected conditional IC as confidence plus a separate risk-character score, linearly mixed. Caution attached: the mixing ratio is exactly the unstable parameter in their sensitivity table, so fix it on validation and report the sweep.
 FIXED-INFLUENCE FAILURE EVIDENCE: Indirect. The weighting stage is never ablated, so no failure is observable by construction; the note treats that absence as the missing arm rather than as evidence. The nearest documented degradation is the drawdown result - the strategy is deeper in drawdown than the benchmark in four of six cross-market windows while the abstract claims general downside protection, with nothing in the system detecting it.
-PROPOSED REVISION STATED IN THE NOTE: To the experimental design rather than the pool, but it directly touches the conditioning set. Verbatim: "the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically." And on P_t, verbatim: "That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four." Also: "Keep the orchestrator low-capacity… a gated linear form or a shallow regression on the four state variables, rather than a network."</t>
+PROPOSED REVISION STATED IN THE NOTE: To the experimental design rather than the pool, but it directly touches the conditioning set. Verbatim: "the honest version of my study adds a configuration where agent *inclusion* is state-conditional and the weights are static. If that recovers most of the benefit, my contribution narrows to the weighting function specifically." And on P_t, verbatim: "That is the assumption my P_t term exists to handle, and the Adaptive minus Persistence configuration is the experiment" I have not found in the literature I have covered. It also gives me the citation for why the persistence term belongs in the conditioning set at all, which had been the weakest-supported of the four. Also: "Keep the orchestrator low-capacity… a gated linear form or a shallow regression on the four state variables, rather than a network."</t>
         </is>
       </c>
       <c r="X31" s="3" t="inlineStr">
@@ -4518,12 +4518,12 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>"This is a map rather than a method: there is no system, no dataset, no experiment and not a single equation anywhere in it, and every number on the page is a citation index." Positions itself against two alpha-generation surveys, three broad LLMs-in-finance surveys and two on interpretability/governance/evaluation for general LLM agents. Claims a targeted review of generative AI inside trading and investment specifically, organised by function and architecture, plus a compiled benchmark set. Consumer banking, fraud detection and AML explicitly out of scope.</t>
+          <t>"This is a map rather than a method: there is no system, no dataset, no experiment and not a single equation anywhere in it, and" every number on the page is a citation index. Positions itself against two alpha-generation surveys, three broad LLMs-in-finance surveys and two on interpretability/governance/evaluation for general LLM agents. Claims a targeted review of generative AI inside trading and investment specifically, organised by function and architecture, plus a compiled benchmark set. Consumer banking, fraud detection and AML explicitly out of scope.</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>US disclosure infrastructure throughout. "Every one of the seven is built on US disclosure infrastructure, SEC filings, 10-Ks, earnings-call transcripts and US-tagged news feeds. None of them is portable to the CSE, and no CSE-comparable frontier market appears anywhere in the survey."  Information retrieval, investment research, trading agents, portfolio optimisation and quant strategy, financial risk management, advisors, market simulation.</t>
+          <t>US disclosure infrastructure throughout. Every one of the seven is built on US disclosure infrastructure, SEC filings, 10-Ks, earnings-call transcripts and US-tagged news feeds. None of them is portable to the CSE, and no CSE-comparable frontier market appears anywhere in the survey. Information retrieval, investment research, trading agents, portfolio optimisation and quant strategy, financial risk management, advisors, market simulation.</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="L32" s="11" t="inlineStr">
         <is>
-          <t>- 31 systems tagged; 13 of 31 carry a multi-agent collaboration stage by the student's tally. - Combination as documented by the survey: ask-respond and debate. "Both are protocols for producing one text from several texts. Neither is a weighting." - Does anything vary influence by state? Of the four directly compared systems, no. "None of the four adapts how much any component counts. FinVerse's partial credit is a planning loop that decides what to do next, and FinGPT's RLHF tunes one model's outputs rather than the influence of several producers on one decision. This is the same fixed-influence pattern I have already documented in FinAgent, AlphaAgents and QFinZero, now visible across a wider sample." The survey names one in-scope exception, reference 20 in the portfolio branch: a three-stage system where LLMs extract alpha signals from multimodal financial data, pass them to specialised trading agents that evaluate performance under various market conditions, then combine validated signals through a "dynamic weighting mechanism," described elsewhere as an "adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions." "Two sentences, no detail, no results." This has since been resolved by the student against the primary paper: "Resolved, see Automate Strategy Finding with LLM in Quant Investment. The primary paper's weights carry no time index: the adaptivity is at factor selection and the weighting is a static MLP trained once, so the survey's real-time gating description is not supported by the paper's own equations, and the system is my static-learned-weight baseline rather than a competitor to the orchestrator." - Two lesser near-misses named: "an adaptive collaboration design in which agent groups coordinate flexibly according to task demand, built on AutoGen GroupChat over Dow Jones 10-K filings, and a confidence-aware critic that adaptively refines only low-confidence prompts without external signals, which is a mechanism for producing something like C_{i,t} without a labelled target." - Heterogeneity distinction the note insists on: "The heterogeneity that the survey does document is heterogeneity of reading, not of evidence… That is several readings of one input, and the survey treats it as the representative case of heterogeneity. My claim is a different one, four agents consuming genuinely different evidence, and the distinction matters enough that I should make it explicitly rather than letting the shared word carry it." - Confidence per agent: only the confidence-aware critic, described in one clause. No mechanism given.</t>
+          <t>- 31 systems tagged; 13 of 31 carry a multi-agent collaboration stage by the student's tally. - Combination as documented by the survey: ask-respond and debate. "Both are protocols for producing one text from several texts. Neither is a weighting." - Does anything vary influence by state? Of the four directly compared systems, no. "None of the four adapts how much any component counts. FinVerse's partial credit is a planning loop that decides what to do next, and FinGPT's RLHF tunes one model's outputs rather than the influence of several producers on one decision. This is the same fixed-influence pattern I have already documented in" FinAgent, AlphaAgents and QFinZero, now visible across a wider sample. The survey names one in-scope exception, reference 20 in the portfolio branch: a three-stage system where LLMs extract alpha signals from multimodal financial data, pass them to specialised trading agents that evaluate performance under various market conditions, then combine validated signals through a "dynamic weighting mechanism," described elsewhere as an adaptive gating mechanism that tunes the influence of each signal in real time under shifting market conditions. "Two sentences, no detail, no results." This has since been resolved by the student against the primary paper: "Resolved, see Automate Strategy Finding with LLM in Quant Investment. The primary paper's weights carry no time index: the adaptivity is at factor selection and the weighting is a static MLP trained once, so the survey's real-time gating description is not supported by the paper's own equations, and the system is my static-learned-weight baseline rather than a competitor to the orchestrator." - Two lesser near-misses named: "an adaptive collaboration design in which agent groups coordinate flexibly according to task demand, built on AutoGen GroupChat over Dow Jones 10-K filings, and a confidence-aware critic that adaptively refines only low-confidence prompts without external signals, which is a mechanism for producing something like C_{i,t} without a labelled target." - Heterogeneity distinction the note insists on: "The heterogeneity that the survey does document is heterogeneity of reading, not of evidence… That is several readings of one input, and the survey treats it as the representative case of heterogeneity. My claim is a different one, four agents consuming genuinely different evidence, and the distinction matters enough that I should make it explicitly rather than letting the shared word carry it." - Confidence per agent: only the confidence-aware critic, described in one clause. No mechanism given.</t>
         </is>
       </c>
       <c r="M32" s="11" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="S32" s="11" t="inlineStr">
         <is>
-          <t>The student's own tally over Figure 2, explicitly flagged as a tally and not a reported result - Stage 2 Memory: 12 of 31; Stage 7 Reflection: 9 of 31; Stage 8 Multi-agent collaboration: 13 of 31; Stage 10 Evaluation: 5 of 31. "Fewer than half the systems in a survey of multi-agent financial AI carry a multi-agent collaboration stage at all, and of the thirteen that do, the survey's own worked examples of what collaboration means are ask-respond and debate. Both are protocols for producing one text from several texts. Neither is a weighting." The gap written in the field's vocabulary: Stage 9 as surveyed, D_t = g(A_{1,t}, …, A_{n,t}), against D_t = Σ_i w_{i,t}(L_t, V_t, P_t, C_{i,t}) A_{i,t}, "where g is an unspecified aggregator, usually an LLM manager prompted to reconcile the agents… The survey never distinguishes the two, which is the gap stated in the field's own vocabulary rather than mine." LIMITATIONS (quoting the note): "There is no review protocol, so coverage cannot be checked. No search strategy, no databases, no query strings, no inclusion or exclusion criteria, no date range, no count of papers screened against papers retained… the branch structure cannot be distinguished from the authors' reading list, and an empty cell in the taxonomy cannot be read as a gap in the field." "Nothing in it is evidence.… a reader cannot tell whether 'no' in the adaptive architecture row means the authors checked and found nothing or that the primary paper did not use the word." "The stage annotations are the most valuable thing in the paper and the least documented.… the honest version of my tally is that thirteen of thirty-one systems were judged by these authors to collaborate, on a criterion they did not state." "Primary papers' priority claims are repeated without adjudication, and one self-citation is unflagged" - three of the five authors are authors of AlphaAgents, which appears in the portfolio branch and Table 2 without disclosure. "The open-challenges section is a list of headings, not a prioritisation."</t>
+          <t>The student's own tally over Figure 2, explicitly flagged as a tally and not a reported result - Stage 2 Memory: 12 of 31; Stage 7 Reflection: 9 of 31; Stage 8 Multi-agent collaboration: 13 of 31; Stage 10 Evaluation: 5 of 31. "Fewer than half the systems in a survey of multi-agent financial AI carry a multi-agent collaboration stage at all", and of the thirteen that do, the survey's own worked examples of what collaboration means are ask-respond and debate. Both are protocols for producing one text from several texts. Neither is a weighting. The gap written in the field's vocabulary: Stage 9 as surveyed, D_t = g(A_{1,t}, …, A_{n,t}), against D_t = Σ_i w_{i,t}(L_t, V_t, P_t, C_{i,t}) A_{i,t}, "where g is an unspecified aggregator, usually an LLM manager prompted to reconcile the agents… The survey never distinguishes the two, which is the gap stated in the field's own vocabulary rather than mine." LIMITATIONS (quoting the note): There is no review protocol, so coverage cannot be checked. "No search strategy, no databases, no query strings, no inclusion or exclusion criteria, no date range, no count of papers screened against papers retained… the branch structure cannot be distinguished from the authors' reading list, and an empty cell in the taxonomy cannot be read as a gap in the field." "Nothing in it is evidence.… a reader cannot tell whether 'no' in the adaptive architecture row means the authors checked and found nothing or that the primary paper did not use the word." The stage annotations are the most valuable thing in the paper and the least documented.… the honest version of my tally is that thirteen of thirty-one systems were judged by these authors to collaborate, on a criterion they did not state. "Primary papers' priority claims are repeated without adjudication, and one self-citation is unflagged" - three of the five authors are authors of AlphaAgents, which appears in the portfolio branch and Table 2 without disclosure. "The open-challenges section is a list of headings, not a prioritisation."</t>
         </is>
       </c>
       <c r="T32" s="11" t="inlineStr">
@@ -4600,7 +4600,7 @@
         <is>
           <t>SPEAKS TO: orchestrator (Stage 9, the adaptive-architecture row, the heterogeneity-of-reading distinction), A_L (absence of any liquidity branch), friction-aware evaluation layer (behavioural fidelity metrics, no-unified-protocol statement).
 EFFECT ON MAIN GAP: Leaves it open, and is the single best positioning citation of the seven - but only in a tightly scoped form. It gives the gap in the field's own vocabulary (Stage 9 is an undifferentiated box; collaboration means ask-respond and debate; none of the four compared systems adapts component influence). Its one nominated counterexample has since been read and does not survive contact. The scoping caveat is mandatory: no review protocol, so an empty cell is not evidence of a gap in the field, only in this survey's coverage.
-CONFIDENCE SCORING: One lead only, unelaborated - "a confidence-aware critic that adaptively refines only low-confidence prompts without external signals, which is the only mechanism in the survey for producing an agent confidence without a labelled target." No detail, no results, not yet read.
+CONFIDENCE SCORING: One lead only, unelaborated - "a confidence-aware critic that adaptively refines only low-confidence prompts without external signals, which is" the only mechanism in the survey for producing an agent confidence without a labelled target. No detail, no results, not yet read.
 FIXED-INFLUENCE FAILURE EVIDENCE: No measured degradation case. Its contribution is prevalence rather than failure: two of four compared systems marked no adaptive architecture at all, one a planning loop, one RLHF inside a single model.
 PROPOSED REVISION STATED IN THE NOTE: None to the four-agent pool or the conditioning set. The revisions are to the evaluation and the write-up: add behavioural fidelity metrics (responsiveness to events, strategy adherence, position tracking) as a second results axis for the state-input ablations; run a prompted-momentum-rule baseline against A_T; state the heterogeneity-of-evidence vs heterogeneity-of-reading distinction explicitly; frame explainability as attribution over computed quantities rather than LLM narration.</t>
         </is>
@@ -4659,17 +4659,17 @@
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>Binance OHLCV via ccxt. On-chain: five Bitinfocharts fields - confirmation time, hash rate, transaction fees, active addresses. Macro-financial: five Yahoo Finance series - dollar index, gold, S&amp;P 500, VIX, WTI crude, forward-filled from Friday close through the weekend so that "1,007 raw trading days are imputed up to 1,461 crypto-calendar days, which means roughly 30% of the macro channel is a repeated Friday value." Technical indicators in three groups: trend following (SMA, EMA over 3–120 day windows, MACD), momentum (RSI, raw momentum, 10-day rate of change), oscillators (Stochastic RSI, Stochastic, 14-day Williams %R). Text "is never merged into the structured join, it is aligned by date at the prompt-construction stage only," capped at 90,000 words per three-day decision window with a 30,000-word daily limit per source, stratified sampling in proportion to source counts when the cap binds.</t>
+          <t>Binance OHLCV via ccxt. On-chain: five Bitinfocharts fields - confirmation time, hash rate, transaction fees, active addresses. Macro-financial: five Yahoo Finance series - dollar index, gold, S&amp;P 500, VIX, WTI crude, forward-filled from Friday close through the weekend so that "1,007 raw trading days are imputed up to 1,461 crypto-calendar days", which means roughly 30% of the macro channel is a repeated Friday value. Technical indicators in three groups: trend following (SMA, EMA over 3–120 day windows, MACD), momentum (RSI, raw momentum, 10-day rate of change), oscillators (Stochastic RSI, Stochastic, 14-day Williams %R). Text "is never merged into the structured join, it is aligned by date at the prompt-construction stage only," capped at 90,000 words per three-day decision window with a 30,000-word daily limit per source, stratified sampling in proportion to source counts when the cap binds.</t>
         </is>
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>Zero-shot GPT-4o, temperature 0.7, top-p 1.0, 1,024 max tokens. "no fine-tuning and no gradient training anywhere in the agent path." Every configuration repeated across 20 seeds with results averaged and dispersion reported. Baselines LSTM, GRU, DLinear, PatchTST get hidden dimensions 32/64/128, learning rates 0.0005 (0.01–0.05 for DLinear), batch size 64, Adam, up to 100 epochs with early stopping at patience 10, plus a grid search over trading thresholds. Threshold rule: Δp_t = (ŷ_t − y_{t−1}) / y_{t−1}, with BUY if Δp_t &gt; θ, SELL if Δp_t &lt; −θ, HOLD if |Δp_t| ≤ θ; θ = 0.015 for 3 and 14-day windows and 0.010 for 30-day. "baseline thresholds were calibrated so that average trade counts land in the 70 to 110 range, matching the trading frequency the LLM agent produces on its own, which removes the obvious confound of one strategy winning by trading more." Three domain agents (technical indicators, on-chain metrics, macro-financial variables) each read a sliding window of 3, 14 or 30 days over their own modality and "produce a prose summary of recent conditions, explicitly without making a price prediction, one on momentum dynamics and indicator signals, one on network activity and participation shifts, one on global risk sentiment and volatility spillovers." A meta trading agent receives all summaries and emits BUY/SELL/HOLD plus a written rationale. Two further text agents (Reddit, news wires) added in ablation. Hallucination control by two constraints: "agents run from fixed domain-specific templates rather than open-ended generation, and the meta-agent is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." GPT-4o selected over Claude, Gemini and FinGPT "on instruction-hierarchy evaluations, which matters for a design where conflicting agent outputs have to be aggregated under a single controlling instruction."</t>
+          <t>Zero-shot GPT-4o, temperature 0.7, top-p 1.0, 1,024 max tokens. "no fine-tuning and no gradient training anywhere in the agent path." Every configuration repeated across 20 seeds with results averaged and dispersion reported. Baselines LSTM, GRU, DLinear, PatchTST get hidden dimensions 32/64/128, learning rates 0.0005 (0.01–0.05 for DLinear), batch size 64, Adam, up to 100 epochs with early stopping at patience 10, plus a grid search over trading thresholds. Threshold rule: Δp_t = (ŷ_t − y_{t−1}) / y_{t−1}, with BUY if Δp_t &gt; θ, SELL if Δp_t &lt; −θ, HOLD if |Δp_t| ≤ θ; θ = 0.015 for 3 and 14-day windows and 0.010 for 30-day. baseline thresholds were calibrated so that average trade counts land in the 70 to 110 range, "matching the trading frequency the LLM agent produces on its own, which removes the obvious confound of one strategy winning by trading more." Three domain agents (technical indicators, on-chain metrics, macro-financial variables) each read a sliding window of 3, 14 or 30 days over their own modality and "produce a prose summary of recent conditions, explicitly without making a price prediction, one on momentum dynamics and indicator signals, one on network activity and participation shifts, one on global risk sentiment and volatility spillovers." A meta trading agent receives all summaries and emits BUY/SELL/HOLD plus a written rationale. Two further text agents (Reddit, news wires) added in ablation. Hallucination control by two constraints: "agents run from fixed domain-specific templates rather than open-ended generation, and the meta-agent is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." GPT-4o selected over Claude, Gemini and FinGPT "on instruction-hierarchy evaluations, which matters for a design where conflicting agent outputs have to be aggregated under a single controlling instruction."</t>
         </is>
       </c>
       <c r="L33" s="11" t="inlineStr">
         <is>
-          <t>- Three core domain agents plus a meta trading agent; two further text agents in ablation, so up to five producers. Genuinely heterogeneous in modality - "The agents are genuinely heterogeneous in modality, technical, on-chain, macro, social and news, which is the property I have been arguing separates my design from MacroHFT's six architecturally identical DDQN sub-agents." But note: heterogeneous in *evidence*, homogeneous in *method* - all are GPT-4o prompted from fixed templates. Evidence each sees: technical agent sees its own indicator set over a 3/14/30-day sliding window; on-chain agent sees five Bitinfocharts fields; macro agent sees five Yahoo series; Reddit agent sees sampled subreddit posts; news agent sees sampled LexisNexis articles. Each emits a prose summary and explicitly no price prediction. - Combination: a fixed prompt template in the meta trading agent. No weights, no votes, no debate, no manager optimisation. The meta-agent "is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." - Does anything vary influence by market state, regime, volatility, liquidity or measured reliability? No - and this is the paper's decisive contribution to the gap. Quoting the note: "the meta-agent's relationship to them is a fixed prompt template, so every agent's influence is constant regardless of whether it is saying anything useful that day. The ablation then shows exactly what that costs, adding a news agent takes total return from 21.75% to 11.39%, and nothing in the architecture can notice or respond. That is the cleanest quantified case for my main gap that I have found, and the fact that the authors read it as a signal-integration problem rather than an orchestration problem is the opening." - Confidence per agent: no per-agent confidence at all. What exists instead is a *pairwise, external* score over agent outputs - see below. The G-EVAL layer is diagnostic only; it never feeds back into the decision.</t>
+          <t>- Three core domain agents plus a meta trading agent; two further text agents in ablation, so up to five producers. Genuinely heterogeneous in modality - "The agents are genuinely heterogeneous in modality, technical, on-chain, macro, social and news, which is the property I have been arguing separates my design from MacroHFT"'s six architecturally identical DDQN sub-agents. But note: heterogeneous in *evidence*, homogeneous in *method* - all are GPT-4o prompted from fixed templates. Evidence each sees: technical agent sees its own indicator set over a 3/14/30-day sliding window; on-chain agent sees five Bitinfocharts fields; macro agent sees five Yahoo series; Reddit agent sees sampled subreddit posts; news agent sees sampled LexisNexis articles. Each emits a prose summary and explicitly no price prediction. - Combination: a fixed prompt template in the meta trading agent. No weights, no votes, no debate, no manager optimisation. The meta-agent "is instructed to synthesise without altering factual content or introducing information the upstream agents did not supply." - Does anything vary influence by market state, regime, volatility, liquidity or measured reliability? No - and this is the paper's decisive contribution to the gap. Quoting the note: "the meta-agent's relationship to them is a fixed prompt template, so every agent's influence is constant regardless of whether it is saying anything useful that day. The ablation then shows exactly what that costs", adding a news agent takes total return from 21.75% to 11.39%, and nothing in the architecture can notice or respond. That is the cleanest quantified case for my main gap that I have found, and the fact that the authors read it as a signal-integration problem rather than an orchestration problem is the opening. - Confidence per agent: no per-agent confidence at all. What exists instead is a *pairwise, external* score over agent outputs - see below. The G-EVAL layer is diagnostic only; it never feeds back into the decision.</t>
         </is>
       </c>
       <c r="M33" s="11" t="inlineStr">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="O33" s="11" t="inlineStr">
         <is>
-          <t>The macro agent covers "global risk sentiment and volatility spillovers" including the VIX. No volatility model, no risk constraint, no position sizing. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): $100,000 initial capital, one trade per day maximum, no leverage, a 0.1% transaction fee and 0.1% slippage applied on both buys and sells. Sensitivity: "Total return moves from 22.03% to 21.61% as fees and slippage go from 0.05% to 0.15%, which the authors read as robustness. Taken against a reported turnover of 7.60, a 0.2% swing in round-trip cost should cost something closer to 1.5 points of capital than the 0.42 observed, and the paper does not reconcile the two, so I would treat the sensitivity analysis as under-specified rather than as evidence that costs do not matter." "There is no market impact term anywhere, which for Bitcoin at $100k of capital is defensible and for anything thinner is not."</t>
+          <t>The macro agent covers "global risk sentiment and volatility spillovers" including the VIX. No volatility model, no risk constraint, no position sizing. LIQUIDITY &amp; FRICTION HANDLING (exact cost assumption): $100,000 initial capital, one trade per day maximum, no leverage, a 0.1% transaction fee and 0.1% slippage applied on both buys and sells. Sensitivity: "Total return moves from 22.03% to 21.61% as fees and slippage go from 0.05% to 0.15%, which the authors read as robustness". Taken against a reported turnover of 7.60, a 0.2% swing in round-trip cost should cost something closer to 1.5 points of capital than the 0.42 observed, and the paper does not reconcile the two, so I would treat the sensitivity analysis as under-specified rather than as evidence that costs do not matter. There is no market impact term anywhere, which for Bitcoin at $100k of capital is defensible and for anything thinner is not.</t>
         </is>
       </c>
       <c r="P33" s="11" t="inlineStr">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="S33" s="11" t="inlineStr">
         <is>
-          <t>3-day window - "Total return of 21.75% ± 3.03 against LSTM's 20.05% ± 3.74 and buy-and-hold's 18.90%, with a Sharpe of 1.08 ± 0.11 against LSTM's 1.05 ± 0.17 and buy-and-hold's 0.80"; MDD falls from 22.52% to 14.69% ± 0.87 and Calmar rises from 1.19 to 1.99 ± 0.25, but "LSTM still holds both the best drawdown at 13.10% and the best Calmar at 2.07." Horizon reversal: 14-day best total return GRU 21.65%, best Sharpe PatchTST 1.15, agent 20.34% / 1.02 / 15.88%; 30-day best return GRU 22.14%, best Sharpe GRU 1.55, agent 17.40% / 0.77 / 20.49%. "At 30 days the agent's Sharpe of 0.77 ± 0.22 is below buy-and-hold's 0.80 and its Calmar of 1.14 ± 0.33 is barely above the passive 1.19." Behaviour: "the agent runs 83.67 ± 11.22 trades against GRU's 74.35 and LSTM's 90.12, turnover of 7.60 ± 1.12 against 6.90 and 6.75, exposure time of 93.15% and an average holding period of 22 days against 18.35 and 19.02." Text ablation: "Against the 21.75% structured-only baseline, adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55, adding the social media agent lifts it to 23.30% ± 2.41 with Sharpe 1.12 ± 0.12 and Calmar 2.01, and adding both lands at 18.98% ± 5.74, below the baseline that used neither. Scoped honestly, the social gain of 1.55 points sits well inside a ± 2.41 band and I would not claim it, whereas the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying." G-EVAL: "Conflict scores average 0.42 with a median of 0.30 and a top quartile above 0.60, and the distribution is visibly bimodal, a large mass of low-conflict days and a secondary cluster near 0.7. Actionability averages 0.55 with a median of 0.60 and a maximum of 0.90." LIMITATIONS (quoting the note): "The headline advantage does not clear its own error bars and no significance test is run anywhere.… seed dispersion measures LLM sampling variance and not variation across market paths, and there is still one asset, one 268-day test window and one regime, a period over which passive Bitcoin returned 18.90%. A 1.70 point edge over LSTM with standard deviations of 3.03 and 3.74 is not an edge I would defend without a paired test, and the paper offers none." "Friction is a flat constant on the deepest book in crypto, and the sensitivity band is too narrow to bind." "Threshold and hyperparameter selection is described as a grid search without ever naming the selection set… since the threshold is the only thing converting a baseline forecast into a strategy, any leakage there lands directly on the comparison the paper's central claim rests on." "The text-agent ablation confounds content with prompt budget and runs at one window size only. Adding an agent adds thousands of words to the prompt as well as a new information source, and there is no placebo agent, no prompt-length control and no run with news content shuffled across dates, so the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both." "The interpretability evaluation is the same model family grading its own output, and is never checked against outcomes. GPT-4o writes the Reddit and news summaries and GPT-4o scores their conflict and actionability, so the scores measure internal consistency of one model's reading rather than anything external. The authors say plainly in the limitations that they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates, and until that is done the scores diagnose the reasoning process without establishing that the process is tracking anything." "Zero-shot with fixed templates is the design's cost as well as its selling point… the template constraint that suppresses hallucination is the same constraint that limits reasoning flexibility, a trade-off the paper names but does not measure." Also: "84 trades over 268 days sits awkwardly with a 22-day mean holding period, and the paper does not reconcile the two definitions"; and Table 7 reports 21.82% where Table 3 reports 21.75% for what should be the same configuration.</t>
+          <t>3-day window - "Total return of 21.75% ± 3.03 against LSTM's 20.05% ± 3.74 and buy-and-hold's 18.90%, with a Sharpe of 1.08 ± 0.11 against LSTM's 1.05 ± 0.17 and buy-and-hold's 0.80"; MDD falls from 22.52% to 14.69% ± 0.87 and Calmar rises from 1.19 to 1.99 ± 0.25, but "LSTM still holds both the best drawdown at 13.10% and the best Calmar at 2.07." Horizon reversal: 14-day best total return GRU 21.65%, best Sharpe PatchTST 1.15, agent 20.34% / 1.02 / 15.88%; 30-day best return GRU 22.14%, best Sharpe GRU 1.55, agent 17.40% / 0.77 / 20.49%. "At 30 days the agent's Sharpe of 0.77 ± 0.22 is below buy-and-hold's 0.80 and its Calmar of 1.14 ± 0.33 is barely above the passive 1.19." Behaviour: "the agent runs 83.67 ± 11.22 trades against GRU's 74.35 and LSTM's 90.12, turnover of 7.60 ± 1.12 against 6.90 and 6.75, exposure time of 93.15% and an average holding period of 22 days against 18.35 and 19.02." Text ablation: "Against the 21.75% structured-only baseline, adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55, adding the social media agent lifts it to 23.30% ± 2.41 with Sharpe 1.12 ± 0.12 and Calmar 2.01, and adding both lands at 18.98% ± 5.74, below the baseline that used neither. Scoped honestly, the social gain of 1.55 points sits well inside a ± 2.41 band and I would not claim it, whereas" the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying. G-EVAL: "Conflict scores average 0.42 with a median of 0.30 and a top quartile above 0.60, and the distribution is visibly bimodal, a large mass of low-conflict days and a secondary cluster near 0.7. Actionability averages 0.55 with a median of 0.60 and a maximum of 0.90." LIMITATIONS (quoting the note): "The headline advantage does not clear its own error bars and no significance test is run anywhere.… seed dispersion measures LLM sampling variance and not variation across market paths, and there is still one asset, one 268-day test window and one regime, a period over which passive Bitcoin returned 18.90%. A 1.70 point edge over LSTM with standard deviations of 3.03 and 3.74 is not an edge I would defend without a paired test, and the paper offers none." "Friction is a flat constant on the deepest book in crypto, and the sensitivity band is too narrow to bind." "Threshold and hyperparameter selection is described as a grid search without ever naming the selection set… since the threshold is the only thing converting a baseline forecast into a strategy, any leakage there lands directly on the comparison the paper's central claim rests on." "The text-agent ablation confounds content with prompt budget and runs at one window size only. Adding an agent adds thousands of words to the prompt as well as a new information source, and there is no placebo agent, no prompt-length control and no run with news content shuffled across dates, so the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both." "The interpretability evaluation is the same model family grading its own output, and is never checked against outcomes. GPT-4o writes the Reddit and news summaries and GPT-4o scores their conflict and actionability, so the scores measure internal consistency of one model's reading rather than anything external. The authors say plainly in the limitations that they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates, and until that is done the scores diagnose the reasoning process without establishing that the process is tracking anything." "Zero-shot with fixed templates is the design's cost as well as its selling point… the template constraint that suppresses hallucination is the same constraint that limits reasoning flexibility, a trade-off the paper names but does not measure." Also: "84 trades over 268 days sits awkwardly with a 22-day mean holding period, and the paper does not reconcile the two definitions"; and Table 7 reports 21.82% where Table 3 reports 21.75% for what should be the same configuration.</t>
         </is>
       </c>
       <c r="T33" s="11" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="U33" s="11" t="inlineStr">
         <is>
-          <t>"This is the third documented case of a fixed-influence component degrading a multi-agent system, and the first that puts a number on it. FinAgent has auxiliary strategies returning 16% on ETHUSD against a 29% passive benchmark, AlphaAgents drops its sentiment agent outright for insufficient coverage, and here a news agent costs 10.36 points of total return while the architecture has no way to notice. The three together are the evidentiary base for the main gap, and this one is the strongest because the degradation is measured under a controlled ablation rather than inferred. The obvious counterfactual, a system that could down-weight the news agent on days when it diverges, is exactly what I am proposing and exactly what this paper does not build." "Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem." "That gives me a pre-registered test rather than an assumption… If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses. Either outcome is publishable and the cost is one scoring pass." "Another paper where execution friction never binds, which keeps the thin-market case open… The CSE charges materially more, the book is thin enough that impact is a separate cost on top of the spread, and every one of these systems was designed and tuned in a regime where cost is a rounding error." "Sentiment is out of scope for my project as of this note, so the news half of the ablation is the part that still speaks to my design… of the two text agents tested here the news agent is the nearer analogue, dated factual material summarised for a decision rather than community tone. That is the agent that cost 10.36 points of total return. The lesson is not that filings will hurt… it is that a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to, and that the demonstration costs one on-off ablation. Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one." "The horizon reversal is a prior against an all-LLM design, and it argues for my heterogeneity claim from the other direction.… An orchestrator that can shift weight toward a recurrent or econometric component at long horizons and toward the reasoning agents at short ones is a concrete, testable instantiation of the main gap, and this paper supplies the horizon evidence for free." "The evaluation harness is the part I should copy wholesale, including the trade-count calibration." "An honest null on the orchestration weights is a better outcome than a 1.7-point win I cannot defend."</t>
+          <t>This is the third documented case of a fixed-influence component degrading a multi-agent system, and the first that puts a number on it. FinAgent has auxiliary strategies returning 16% on ETHUSD against a 29% passive benchmark, AlphaAgents drops its sentiment agent outright for insufficient coverage, and here a news agent costs 10.36 points of total return while the architecture has no way to notice. The three together are the evidentiary base for the main gap, and this one is the strongest because the degradation is measured under a controlled ablation rather than inferred. The obvious counterfactual, a system that could down-weight the news agent on days when it diverges, is exactly what I am proposing and exactly what this paper does not build. "Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem." "That gives me a pre-registered test rather than an assumption… If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses. Either outcome is publishable and the cost is one scoring pass." "Another paper where execution friction never binds, which keeps the thin-market case open… The CSE charges materially more, the book is thin enough that impact is a separate cost on top of the spread, and every one of these systems was designed and tuned in a regime where cost is a rounding error." Sentiment is out of scope for my project as of this note, so the news half of the ablation is the part that still speaks to my design… of the two text agents tested here the news agent is the nearer analogue, dated factual material summarised for a decision rather than community tone. That is the agent that cost 10.36 points of total return. The lesson is not that filings will hurt… it is that a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to, and that the demonstration costs one on-off ablation. Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one. "The horizon reversal is a prior against an all-LLM design, and it argues for my heterogeneity claim from the other direction.… An orchestrator that can shift weight toward a recurrent or econometric component at long horizons and toward the reasoning agents at short ones is a concrete, testable instantiation of the main gap, and this paper supplies the horizon evidence for free." "The evaluation harness is the part I should copy wholesale, including the trade-count calibration." "An honest null on the orchestration weights is a better outcome than a 1.7-point win I cannot defend."</t>
         </is>
       </c>
       <c r="V33" s="11" t="inlineStr">
@@ -4726,9 +4726,9 @@
         <is>
           <t>SPEAKS TO: orchestrator (the fixed-template failure case, the horizon-reversal argument, the G-EVAL conflict mechanism), A_T (technical agent, and the LSTM/GRU horizon result), A_F (the news agent is the nearest analogue to the retrieval channel), friction-aware evaluation layer (stated 0.1% + 0.1%, and the unreconciled sensitivity band).
 EFFECT ON MAIN GAP: Leaves it open and supplies the single strongest quantified motivation for it in the whole set. This is the closest published system to the proposed orchestration structure - genuinely heterogeneous agents, a meta-synthesiser, a shared execution harness - "and it is the most useful paper in my set precisely because the orchestration is the part it does not do." The news agent costs 10.36 points of total return under a controlled ablation with dispersion reported (±1.06 against a 21.75% baseline), far outside any error band in the table, and the architecture has no mechanism to detect or respond to it. The counterfactual the paper leaves unbuilt is exactly the proposed contribution. It also supplies, free, the horizon evidence that different component families genuinely win at different horizons (GRU takes the 30-day window on return, Sharpe, Sortino and Calmar while the agent falls below passive on risk-adjusted terms), which is "a concrete, testable instantiation of the main gap."
-CONFIDENCE SCORING: This is the candidate mechanism, and it is the only one of its kind in the set. G-EVAL (Liu et al., 2023) is a protocol where an LLM scores generated text against a rubric in a zero-shot prompt, rather than against a reference. Jung and Lee apply it to pairs of agent outputs, scoring each daily Reddit summary against the matching news summary on two rubrics: a conflict score for semantic divergence in tone, outlook and implication, and an actionability score for whether the combination yields a clear and timely trading signal. Both are 0 to 1. The scoring model is GPT-4o, which is also the model that wrote the summaries being scored. Measured distributions: conflict mean 0.42, median 0.30, top quartile above 0.60, visibly bimodal with a secondary cluster near 0.7; actionability mean 0.55, median 0.60, maximum 0.90. The authors' two conclusions: "that divergence between sources makes a coherent reasoning chain harder to build, and that even agreeing sources often fail to produce a usable signal. The first is consistent with the dual-agent degradation, the second is the more uncomfortable one and is the reason I would treat actionability as the more informative of the two scores." Why it matters, verbatim: "Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem. My orchestration function needs confidence on a common scale across an LLM analyst, an econometric estimator and an RL policy, and nothing in the literature supplies one, because each component's native confidence means something different. The move here is to stop asking the agents and score the *relationship between their outputs* externally on a fixed rubric, which sidesteps internal calibration entirely and generalises to any pair of producers that can emit text. I would take the mechanism and not the validation, since scoring pairwise conflict is cheap and establishing that it predicts anything is the work this paper skips." The pre-registered test, verbatim: "compute conflict scores across agent pairs on CSE data, then check whether they correlate with realised next-period error or return before any of it touches the orchestrator. If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses." Known weaknesses of the mechanism as published: same model family grades its own output; never validated against outcomes (the authors concede they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates); pairwise only, not per-agent; diagnostic only, never fed back.
-FIXED-INFLUENCE FAILURE EVIDENCE: Yes - the strongest in the set, and the only one with a controlled number attached. "adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55… the news loss of 10.36 points is far outside any dispersion in the table and is the finding worth carrying." And: "here a news agent costs 10.36 points of total return while the architecture has no way to notice." Caveat the note itself attaches: "the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both," because there is no placebo agent, no prompt-length control and no date-shuffled run. A secondary case: adding both text agents lands at 18.98% ± 5.74, "below the baseline that used neither."
-PROPOSED REVISION STATED IN THE NOTE: To the conditioning set, verbatim: "compute conflict scores across agent pairs on CSE data, then check whether they correlate with realised next-period error or return before any of it touches the orchestrator. If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses." To the experiment set, verbatim: "a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to… Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one." No change to the four-agent pool; sentiment confirmed out of scope.</t>
+CONFIDENCE SCORING: This is the candidate mechanism, and it is the only one of its kind in the set. G-EVAL (Liu et al., 2023) is a protocol where an LLM scores generated text against a rubric in a zero-shot prompt, rather than against a reference. Jung and Lee apply it to pairs of agent outputs, scoring each daily Reddit summary against the matching news summary on two rubrics: a conflict score for semantic divergence in tone, outlook and implication, and an actionability score for whether the combination yields a clear and timely trading signal. Both are 0 to 1. The scoring model is GPT-4o, which is also the model that wrote the summaries being scored. Measured distributions: conflict mean 0.42, median 0.30, top quartile above 0.60, visibly bimodal with a secondary cluster near 0.7; actionability mean 0.55, median 0.60, maximum 0.90. The authors' two conclusions: "that divergence between sources makes a coherent reasoning chain harder to build, and that even agreeing sources often fail to produce a usable signal. The first is consistent with the dual-agent degradation, the second is the more uncomfortable one and is the reason I would treat actionability as the more informative of the two scores." Why it matters, verbatim: Conflict and actionability are the first concrete answer I have seen to the comparable-confidence problem. My orchestration function needs confidence on a common scale across an LLM analyst, an econometric estimator and an RL policy, and nothing in the literature supplies one, because each component's native confidence means something different. "The move here is to stop asking the agents and score the *relationship between their outputs* externally on a fixed rubric, which sidesteps internal calibration entirely and generalises to any pair of producers that can emit text. I would take the mechanism and not the validation, since scoring pairwise conflict is cheap and establishing that it predicts anything is the work this paper skips." The pre-registered test, verbatim: "compute conflict scores across agent pairs on CSE data, then check whether they correlate with realised next-period error or return before any of it touches the orchestrator. If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses." Known weaknesses of the mechanism as published: same model family grades its own output; never validated against outcomes (the authors concede they did not investigate whether conflict and actionability correlate with subsequent realised returns or error rates); pairwise only, not per-agent; diagnostic only, never fed back.
+FIXED-INFLUENCE FAILURE EVIDENCE: Yes - the strongest in the set, and the only one with a controlled number attached. "adding the news agent drops total return to 11.39% ± 1.06 with Sharpe collapsing from 1.08 to 0.55… the news loss of 10.36 points is far outside any dispersion in the table" and is the finding worth carrying. And: "here a news agent costs 10.36 points of total return while the architecture has no way to notice." Caveat the note itself attaches: "the 10-point news degradation is consistent with semantic conflict, with dilution of the structured summaries in a longer context, or with both," because there is no placebo agent, no prompt-length control and no date-shuffled run. A secondary case: adding both text agents lands at 18.98% ± 5.74, "below the baseline that used neither."
+PROPOSED REVISION STATED IN THE NOTE: To the conditioning set, verbatim: "compute conflict scores across agent pairs on CSE data, then check whether they correlate with realised next-period error or return before any of it touches the orchestrator. If conflict carries no signal, the conditioning set falls back to market state alone and I report that, and if it does, I have an information-state input that no prior system in my set uses." To the experiment set, verbatim: a text channel bolted onto a working structured pipeline has to be shown to earn its weight rather than assumed to… Running that ablation on the retrieval agent is now a required experiment in my design rather than an optional one. No change to the four-agent pool; sentiment confirmed out of scope.</t>
         </is>
       </c>
       <c r="X33" s="11" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Takes the "child-order execution problem, the last atomic step after a parent order has already been sliced," and formulates it as an "optimal stopping problem: the trader holds one indivisible share, has a horizon of $T$ seconds, and at each second chooses CONTINUE or STOP." Two data-driven solutions on one neural architecture - a supervised method forecasting the whole future price-change trajectory and acting on it, and an RL method learning the continuation value directly. Both trained with a TD($m$-step) family spanning one-step TD to empirical Monte Carlo, "so the paper is really four algorithm families rather than two."</t>
+          <t>Takes the child-order execution problem, "the last atomic step after a parent order has already been sliced," and formulates it as an optimal stopping problem: "the trader holds one indivisible share, has a horizon of $T$ seconds, and at each second chooses CONTINUE or STOP." Two data-driven solutions on one neural architecture - a supervised method forecasting the whole future price-change trajectory and acting on it, and an RL method learning the continuation value directly. Both trained with a TD($m$-step) family spanning one-step TD to empirical Monte Carlo, "so the paper is really four algorithm families rather than two."</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="O34" s="11" t="inlineStr">
         <is>
-          <t>Volatility appears only as an input feature ("spread normalized by return and price volatility"). There is no risk term in the objective; the objective is pure expected price gain over a 60-second stopping problem. The note later contrasts this against Wang et al.: "neither of the other two execution notes carries a risk term." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's defining weakness and the note treats it as such. There is no market impact model of any kind - no Almgren-Chriss, no square-root, no linear impact. Impact is assumed away by construction: "the order is infinitesimal and ... any action of the trader has no effect on the price process, the states or the transition kernel, which is what makes the problem a pure stopping problem rather than a control problem." Spread is handled only as the *unit of measurement*, not as a cost to be modelled: the half-spread is "the time-averaged difference between best bid and best ask over the previous 5 trading days, halved," and every result is a price gain as a percentage of it, where "a gain of 100% means the trade executed at the mid-price, so the trader crossed no spread at all and traded frictionlessly." Queue: queue imbalance is used as a *feature* at top 5 levels, but there is no queue position modelling. Fills: "STOP is assumed to produce an immediate fill at the observed price, which implicitly means a marketable order crossing the spread." No partial fills, no cancellation, no passive posting, no loss of queue priority, no commission or exchange fee anywhere in the objective. Calibration: none of an impact model; the only calibration-like quantity is the trailing 5-day half-spread normalizer and 21-day volume normalization of depth features. Critically: "The paper builds the limit order book in full from ITCH messages and then uses it only as a feature source, never as a fill simulator, so the reported gains are upper bounds on what the same policy would achieve against a book that has to be interacted with rather than observed."</t>
+          <t>Volatility appears only as an input feature ("spread normalized by return and price volatility"). There is no risk term in the objective; the objective is pure expected price gain over a 60-second stopping problem. The note later contrasts this against Wang et al.: neither of the other two execution notes carries a risk term. LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's defining weakness and the note treats it as such. There is no market impact model of any kind - no Almgren-Chriss, no square-root, no linear impact. Impact is assumed away by construction: "the order is infinitesimal and... any action of the trader has no effect on the price process, the states or the transition kernel, which is what makes the problem a pure stopping problem rather than a control problem." Spread is handled only as the *unit of measurement*, not as a cost to be modelled: the half-spread is "the time-averaged difference between best bid and best ask over the previous 5 trading days, halved," and every result is a price gain as a percentage of it, where "a gain of 100% means the trade executed at the mid-price, so the trader crossed no spread at all and traded frictionlessly." Queue: queue imbalance is used as a *feature* at top 5 levels, but there is no queue position modelling. Fills: "STOP is assumed to produce an immediate fill at the observed price, which implicitly means a marketable order crossing the spread." No partial fills, no cancellation, no passive posting, no loss of queue priority, no commission or exchange fee anywhere in the objective. Calibration: none of an impact model; the only calibration-like quantity is the trailing 5-day half-spread normalizer and 21-day volume normalization of depth features. Critically: "The paper builds the limit order book in full from ITCH messages and then uses it only as a feature source, never as a fill simulator, so the reported gains are upper bounds on what the same policy would achieve against a book that has to be interacted with rather than observed."</t>
         </is>
       </c>
       <c r="P34" s="11" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="S34" s="11" t="inlineStr">
         <is>
-          <t>"Stock-specific gives 21.40 (0.15) for SL against 24.82 (0.16) for RL, universal gives 22.34 (0.15) against 25.47 (0.16), so the improvements are 16% and 14% respectively." Universal beats stock-specific "by 4.4% for SL and 2.6% for RL." Take-one-out "returns 24.85 (0.16) against the stock-specific 24.82 (0.16)." Convergence: "SL is at its plateau of roughly 20 to 22 within about 10,000 steps for every $m$ except $m=1$"; in wall-clock "RL-TD(1-step) reaches roughly 20 within about 400 seconds while RL-TD(30-step) is still near 5 at 800 seconds and RL-TD(45-step) and RL-TD(60-step) have not left their starting level at all." Bias-variance: "prediction standard deviation rises from 23.1 at $m=1$ to 34.9 at $m=60$ while noise standard deviation squared bias falls from 26.9 to 18.0, with total RMSE roughly flat from 35.5 to 39.3." LIMITATIONS (quoted): (1) "The zero-impact assumption is stated as a modelling convenience and is the thing that does not survive transport to a thin book ... In a market where a single child order can be a visible fraction of resting depth at the touch, the act of stopping changes the state that the next decision would have been conditioned on, and the entire optimal stopping formulation stops being the right object." (2) "No order type, no queue position, no partial fills, no fees." (3) "There is no non-neural baseline anywhere in the paper ... the gap between 'an RNN trained this way recovers a quarter of the half-spread' and 'this problem needs an RNN'." (4) "One year, one exchange, one liquidity tier, no walk-forward, and a universality claim demonstrated inside a set selected for homogeneity ... the take-one-out figure of 24.85 against 24.82 is evidence of transfer within a tight band rather than evidence that a model trained on NASDAQ megacaps carries to a market with different tick rules, hours, participant mix and spreads measured in percent rather than ticks." (5) "The training protocol has no stopping criterion and no reported search, so the headline numbers carry an unmeasured selection component ... the standard errors in the headline table also describe variation across episodes and stocks rather than across training runs."</t>
+          <t>"Stock-specific gives 21.40 (0.15) for SL against 24.82 (0.16) for RL, universal gives 22.34 (0.15) against 25.47 (0.16), so the improvements are 16% and 14% respectively." Universal beats stock-specific "by 4.4% for SL and 2.6% for RL." Take-one-out "returns 24.85 (0.16) against the stock-specific 24.82 (0.16)." Convergence: "SL is at its plateau of roughly 20 to 22 within about 10,000 steps for every $m$ except $m=1$"; in wall-clock "RL-TD(1-step) reaches roughly 20 within about 400 seconds while RL-TD(30-step) is still near 5 at 800 seconds and RL-TD(45-step) and RL-TD(60-step) have not left their starting level at all." Bias-variance: prediction standard deviation rises from 23.1 at $m=1$ to 34.9 at $m=60$ while noise standard deviation squared bias "falls from 26.9 to 18.0, with total RMSE roughly flat from 35.5 to 39.3." LIMITATIONS (quoted): (1) "The zero-impact assumption is stated as a modelling convenience and is the thing that does not survive transport to a thin book... In a market where a single child order can be a visible fraction of resting depth at the touch, the act of stopping changes the state that the next decision would have been conditioned on, and" the entire optimal stopping formulation stops being the right object. (2) "No order type, no queue position, no partial fills, no fees." (3) "There is no non-neural baseline anywhere in the paper... the gap between 'an RNN trained this way recovers a quarter of the half-spread' and 'this problem needs an RNN'." (4) "One year, one exchange, one liquidity tier, no walk-forward, and a universality claim demonstrated inside a set selected for homogeneity... the take-one-out figure of 24.85 against 24.82 is evidence of transfer within a tight band rather than evidence that a model trained on NASDAQ megacaps carries to a market with different tick rules, hours, participant mix and spreads measured in percent rather than ticks." (5) "The training protocol has no stopping criterion and no reported search, so the headline numbers carry an unmeasured selection component... the standard errors in the headline table also describe variation across episodes and stocks rather than across training runs."</t>
         </is>
       </c>
       <c r="T34" s="11" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Chen, Zhu, Liu and Li - first author at Cornell writing up an IBM Research internship, the rest at MIT-IBM Watson AI Lab, IBM Research and Three Bridges Capital. "Cost-Efficient Reinforcement Learning for Optimal Trade Execution on Dynamic Market Environment." ICAIF '22, pages 386-393.</t>
+          <t>Chen, Zhu, Liu and Li - first author at Cornell writing up an IBM Research internship, the rest at MIT-IBM Watson AI Lab, IBM Research and Three Bridges Capital. Cost-Efficient Reinforcement Learning for Optimal Trade Execution on Dynamic Market Environment. ICAIF '22, pages 386-393.</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>Takes "optimal trade execution of a parent order, liquidating a fixed inventory over a fixed number of steps," and attacks two things at once: it puts the agent in a "queue-reactive virtual market that responds to the agent's own orders rather than replaying a frozen book," and it proposes "Deep Dyna-Double Q-learning (D3Q), a hybrid of direct RL and planning against a learned market environment model, plus a state-balanced exploration scheme built for the fact that inventory only ever decreases."</t>
+          <t>Takes optimal trade execution "of a parent order, liquidating a fixed inventory over a fixed number of steps," and attacks two things at once: it puts the agent in a queue-reactive virtual market that responds to the agent's own orders rather than replaying a frozen book, and it proposes Deep Dyna-Double Q-learning (D3Q), "a hybrid of direct RL and planning against a learned market environment model, plus a state-balanced exploration scheme built for the fact that inventory only ever decreases."</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="O35" s="11" t="inlineStr">
         <is>
-          <t>Volatility is one of the 20 market state variables. Otherwise nothing: "The objective has no risk term at all. The reward is pure expected relative cost with $\gamma=1$, so the agent is indifferent between a schedule that reliably costs 15 bps and one that costs 5 or 25 with equal probability, which is exactly the trade-off the Almgren and Chriss framework exists to express and which the paper cites in passing without incorporating." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's core, and it is an LOB-based reactive execution simulator, not a parametric impact formula. There is NO Almgren-Chriss, NO square-root law, NO linear impact coefficient. Instead impact is *endogenous and mechanistic*: "Queue-reactive virtual market following Huang et al. (2015), queues as continuous-time Markov jump processes." Mechanism verbatim: "Queue length at each level moves as a jump process whose up-rate is the intensity of new limit orders and whose down-rate is the intensity of market orders plus cancellations, with both intensities estimated as functions of current queue size from historical books. The mid-price moves only when the best bid or best ask queue depletes to zero, and levels shift when opposite-side limit orders are inserted. So an agent that sends a market order consumes queue, brings a level closer to depletion, and makes an adverse mid-price move more likely on the next step, which is impact emerging from the mechanism rather than being charged as a fee." Calibration: order-arrival, market-order and cancellation intensities as functions of queue size at each level, estimated from IEX LOB data March-Dec 2020. Cost measurement: $\text{ATC} = (\text{average selling price} - p_D)/p_D$ in basis points, "negative by construction when liquidating, because pushing size into the book walks the price down." Spread: implicitly paid in full on every order - "Restricting the action space to marketable orders ... means the policy can only ever pay the spread, never earn it." Queue position: modelled in the *environment* (queue lengths and depletion) but the agent has no queue position of its own, since it posts no limit orders. Partial fills: none - "Market orders only, no queue position, no fees, no partial fills." Fees/commissions: none. Order-size dependence: present through the mechanism (larger $a$ consumes more queue) but never swept - "Everything runs at $I=80$ and $T=16$, with no sweep over inventory or participation rate even though impact is the subject and impact scales with size, so nothing tells me whether the advantage over TWAP grows, shrinks or inverts as the order gets larger relative to depth."</t>
+          <t>Volatility is one of the 20 market state variables. Otherwise nothing: "The objective has no risk term at all. The reward is pure expected relative cost with $\gamma=1$, so the agent is indifferent between a schedule that reliably costs 15 bps and one that costs 5 or 25 with equal probability, which is exactly the trade-off the Almgren and Chriss framework exists to express and which the paper cites in passing without incorporating." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): This is the paper's core, and it is an LOB-based reactive execution simulator, not a parametric impact formula. There is NO Almgren-Chriss, NO square-root law, NO linear impact coefficient. Instead impact is *endogenous and mechanistic*: "Queue-reactive virtual market following Huang et al. (2015), queues as continuous-time Markov jump processes." Mechanism verbatim: "Queue length at each level moves as a jump process whose up-rate is the intensity of new limit orders and whose down-rate is the intensity of market orders plus cancellations, with both intensities estimated as functions of current queue size from historical books. The mid-price moves only when the best bid or best ask queue depletes to zero, and levels shift when opposite-side limit orders are inserted. So an agent that sends a market order consumes queue, brings a level closer to depletion, and makes an adverse mid-price move more likely on the next step, which is impact emerging from the mechanism rather than being charged as a fee." Calibration: order-arrival, market-order and cancellation intensities as functions of queue size at each level, estimated from IEX LOB data March-Dec 2020. Cost measurement: $\text{ATC} = (\text{average selling price} - p_D)/p_D$ in basis points, "negative by construction when liquidating, because pushing size into the book walks the price down." Spread: implicitly paid in full on every order - Restricting the action space to marketable orders... means the policy can only ever pay the spread, never earn it. Queue position: modelled in the *environment* (queue lengths and depletion) but the agent has no queue position of its own, since it posts no limit orders. Partial fills: none - "Market orders only, no queue position, no fees, no partial fills." Fees/commissions: none. Order-size dependence: present through the mechanism (larger $a$ consumes more queue) but never swept - "Everything runs at $I=80$ and $T=16$, with no sweep over inventory or participation rate even though impact is the subject and impact scales with size, so nothing tells me whether the advantage over TWAP grows, shrinks or inverts as the order gets larger relative to depth."</t>
         </is>
       </c>
       <c r="P35" s="11" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="V35" s="11" t="inlineStr">
         <is>
-          <t>Everything outside the simulator, everything passive, and everything about size. No live/historical-replay validation; no fees, queue position or partial fills; no participation-rate sweep; no risk term. And for the CSE specifically: "The queue-reactive simulator is almost certainly out of reach on the CSE ... Calibrating it needs limit order arrival, market order and cancellation intensities as functions of queue size at each level, which means order-level message data or at minimum multi-level depth snapshots. Whether the CSE exposes anything below top-of-book is still unconfirmed, and if it does not, the realistic fallback is a parametric temporary and permanent impact model calibrated against observed turnover and daily price moves, which is weaker but honest."</t>
+          <t>Everything outside the simulator, everything passive, and everything about size. No live/historical-replay validation; no fees, queue position or partial fills; no participation-rate sweep; no risk term. And for the CSE specifically: "The queue-reactive simulator is almost certainly out of reach on the CSE... Calibrating it needs limit order arrival, market order and cancellation intensities as functions of queue size at each level, which means order-level message data or at minimum multi-level depth snapshots". Whether the CSE exposes anything below top-of-book is still unconfirmed, and if it does not, the realistic fallback is a parametric temporary and permanent impact model calibrated against observed turnover and daily price moves, which is weaker but honest.</t>
         </is>
       </c>
       <c r="W35" s="11" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Wang, Gao and Li, all at the Department of Systems Engineering and Engineering Management, CUHK. "Reinforcement learning for continuous-time optimal execution: actor-critic algorithm and error analysis." Finance and Stochastics 30(3), 2026, 597-655. Received October 2023, accepted February 2025, published online 10 March 2026, open access.</t>
+          <t>Wang, Gao and Li, all at the Department of Systems Engineering and Engineering Management, CUHK. Reinforcement learning for continuous-time optimal execution: actor-critic algorithm and error analysis. Finance and Stochastics 30(3), 2026, 597-655. Received October 2023, accepted February 2025, published online 10 March 2026, open access.</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Takes "the parent-order liquidation problem in continuous time under the Almgren-Chriss model," regularises it with Shannon entropy to induce exploration, solves the resulting "exploratory mean-quadratic-variation (EMQV)" control problem in closed form, and uses that closed form as the parametrisation for an actor-critic RL algorithm with five learnable scalars. Algorithmic contribution is a third update step, "recalibration"; theoretical contribution is "a finite-time error bound with conditions on the learning rates under which the algorithm converges linearly to the global optimum."</t>
+          <t>Takes the parent-order liquidation problem "in continuous time under the Almgren-Chriss model," regularises it with Shannon entropy to induce exploration, solves the resulting "exploratory mean-quadratic-variation (EMQV)" control problem in closed form, and uses that closed form as the parametrisation for an actor-critic RL algorithm with five learnable scalars. Algorithmic contribution is a third update step, "recalibration"; theoretical contribution is "a finite-time error bound with conditions on the learning rates under which the algorithm converges linearly to the global optimum."</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>EMQV objective: $$\sup_{\boldsymbol{\pi}\in\Pi}\ \mathbb{E}\Big[\int_0^T\!\!\int_{\mathbb{R}}\big(-\nu(S_t^{\boldsymbol\pi}+\eta\nu)-\lambda\sigma^2S_0^2(q_t^{\boldsymbol\pi})^2-\zeta\ln\boldsymbol\pi_t(\nu)\big)\boldsymbol\pi_t(\nu)\,d\nu\,dt + h_T(q_T^{\boldsymbol\pi},S_T^{\boldsymbol\pi})\Big]$$ with $h_T = 0$ at zero inventory and $-\infty$ otherwise, forcing exact liquidation. Closed-form optimal exploratory policy is Gaussian: $$\boldsymbol\pi^*(\nu;t,q,S) = d_{\mathcal{N}}\Big(\nu;\ -qK\coth\big(K(T-t)\big),\ \frac{\zeta}{2\eta}\Big), \qquad K = \sqrt{\frac{\lambda\sigma^2S_0^2}{\eta}}$$ - "exploration variance is proportional to the temperature and inversely proportional to the temporary impact parameter, which matches the intuition that in a market where trading fast is expensive you should sample less aggressively around your intended rate." Letting $\zeta \downarrow 0$ recovers classical Almgren-Chriss exactly. Parametrisation: $\boldsymbol\pi^\Phi = d_{\mathcal{N}}(\nu; -q\varphi_1\coth(\varphi_1(T-t)), \zeta\varphi_2)$ with $\varphi_1^* = \sqrt{\lambda\sigma^2 S_0^2/\eta_{\text{env}}}$ and $\varphi_2^* = 1/(2\eta_{\text{env}})$, plus a three-parameter value function $\Theta=(\theta_1,\theta_2,\theta_3)$ - "Five scalars total, against a SAC implementation carrying several networks of width 128 to 256." Recalibration step: $$\Theta^{(\ell+1)} = M(\Phi^{(\ell+1)})M(\Phi^{(\ell)})^{-1}\widetilde\Theta^{(\ell)}$$ costing one matrix product per iteration and guaranteeing the policy evaluation error shrinks by $d(\ell)\in(0,1-\varepsilon)$. Exploratory revenue collected by 15-node Gauss-Hermite quadrature with environment resets between nodes.</t>
+          <t>EMQV objective: $$\sup_{\boldsymbol{\pi}\in\Pi}\ \mathbb{E}\Big[\int_0^T\!\!\int_{\mathbb{R}}\big(-\nu(S_t^{\boldsymbol\pi}+\eta\nu)-\lambda\sigma^2S_0^2(q_t^{\boldsymbol\pi})^2-\zeta\ln\boldsymbol\pi_t(\nu)\big)\boldsymbol\pi_t(\nu)\,d\nu\,dt + h_T(q_T^{\boldsymbol\pi},S_T^{\boldsymbol\pi})\Big]$$ with $h_T = 0$ at zero inventory and $-\infty$ otherwise, forcing exact liquidation. Closed-form optimal exploratory policy is Gaussian: $$\boldsymbol\pi^*(\nu;t,q,S) = d_{\mathcal{N}}\Big(\nu;\ -qK\coth\big(K(T-t)\big),\ \frac{\zeta}{2\eta}\Big), \qquad K = \sqrt{\frac{\lambda\sigma^2S_0^2}{\eta}}$$ - "exploration variance is proportional to the temperature and inversely proportional to the temporary impact parameter, which matches the intuition that in a market where trading fast is expensive you should sample less aggressively around your intended rate." Letting $\zeta \downarrow 0$ recovers classical Almgren-Chriss exactly. Parametrisation: $\boldsymbol\pi^\Phi = d_{\mathcal{N}}(\nu; -q\varphi_1\coth(\varphi_1(T-t)), \zeta\varphi_2)$ with $\varphi_1^* = \sqrt{\lambda\sigma^2 S_0^2/\eta_{\text{env}}}$ and $\varphi_2^* = 1/(2\eta_{\text{env}})$, plus a three-parameter value function $\Theta=(\theta_1,\theta_2,\theta_3)$ - Five scalars total, "against a SAC implementation carrying several networks of width 128 to 256." Recalibration step: $$\Theta^{(\ell+1)} = M(\Phi^{(\ell+1)})M(\Phi^{(\ell)})^{-1}\widetilde\Theta^{(\ell)}$$ costing one matrix product per iteration and guaranteeing the policy evaluation error shrinks by $d(\ell)\in(0,1-\varepsilon)$. Exploratory revenue collected by 15-node Gauss-Hermite quadrature with environment resets between nodes.</t>
         </is>
       </c>
       <c r="L36" s="11" t="inlineStr">
@@ -5080,7 +5080,7 @@
       </c>
       <c r="S36" s="11" t="inlineStr">
         <is>
-          <t>Recalibration ablation - "recalibration takes the standard deviation of the learned $\varphi_1$ from 43.57 down to 1.17, a factor of 37, while the value function parameters barely move, $\theta_1$ at $1.64\times10^{-10}$ against $1.50\times10^{-10}$." Exploratory-vs-sample state - "$\varphi_1$ standard deviations of 1.67 and 1.82 at medium and high risk aversion against 167.60 and 307.54." AC simulator gaps in bps - "$-9.881\times10^{-10}$, $-1.022\times10^{-3}$ and $-3.075\times10^{-4}$ for EMQV at low, medium and high risk aversion, against $-19.311$, $-113.647$ and $-109.405$ for the best depth and width configuration of SAC." Out of sample - "Across 21 stock and risk-aversion combinations, EMQV is the best performer in 9 and SAC in 10, which is not the ordering the abstract's 'stands out as the best overall' would suggest on its own ... SAC underperforms TWAP in 11 of 21 cases regardless of which simulator trained it, and its standard errors are enormous, AAPL at high risk aversion coming in at $-1.73\times10^5$ with a standard error of 18,323 on the CST simulator." STAT degradation - "at high risk aversion turns in $-905.742$ on AAPL and $-203.392$ on MSFT against EMQV's $+102.285$ and $+85.983$ on the historical simulator." Low risk aversion - "several entries being $-0.020$ to $+0.046$ basis points, because TWAP is nearly optimal for a risk-neutral agent." LIMITATIONS (quoted): (1) "The parametrisation cannot express anything the Almgren-Chriss model cannot, and every advantage in the paper traces back to that. Linear permanent impact, linear temporary impact, arithmetic Brownian motion with constant volatility, no spread, no depth, no order imbalance, no intraday seasonality in any of them ... The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong, which is precisely the situation a thin frontier order book creates." (2) "The convergence guarantee is real but not operational ... the guarantee is conditional on a box whose right size is unknown ... the theorem covers a different algorithm from the one in the experiments." (3) "Exploration requires rewinding the market, which no live venue permits ... the configuration carrying the headline results is simulator-only and the deployable one is the weaker of the two." (4) "Market orders only, no spread, no queue, no fees, and the last step dumps whatever is left ... This is the same restriction as in the queue-reactive paper and it bites harder in a wide-spread market." (5) "Seven large-cap Nasdaq names, two test quarters, one horizon, one participation rate ... The paper's argument that EMQV is more robust to distribution shift than STAT rests on a shift between adjacent quarters in a stable market, which is the mildest available version of that test." (6) "The comparison against SAC is not tuned symmetrically ... it means the empirical comparison establishes that SAC is harder to configure reliably rather than that it is worse."</t>
+          <t>Recalibration ablation - "recalibration takes the standard deviation of the learned $\varphi_1$ from 43.57 down to 1.17, a factor of 37, while the value function parameters barely move, $\theta_1$ at $1.64\times10^{-10}$ against $1.50\times10^{-10}$." Exploratory-vs-sample state - "$\varphi_1$ standard deviations of 1.67 and 1.82 at medium and high risk aversion against 167.60 and 307.54." AC simulator gaps in bps - "$-9.881\times10^{-10}$, $-1.022\times10^{-3}$ and $-3.075\times10^{-4}$ for EMQV at low, medium and high risk aversion, against $-19.311$, $-113.647$ and $-109.405$ for the best depth and width configuration of SAC." Out of sample - "Across 21 stock and risk-aversion combinations, EMQV is the best performer in 9 and SAC in 10, which is not the ordering the abstract's 'stands out as the best overall' would suggest on its own... SAC underperforms TWAP in 11 of 21 cases regardless of which simulator trained it, and its standard errors are enormous, AAPL at high risk aversion coming in at $-1.73\times10^5$ with a standard error of 18,323 on the CST simulator." STAT degradation - "at high risk aversion turns in $-905.742$ on AAPL and $-203.392$ on MSFT against EMQV's $+102.285$ and $+85.983$ on the historical simulator." Low risk aversion - "several entries being $-0.020$ to $+0.046$ basis points, because TWAP is nearly optimal for a risk-neutral agent." LIMITATIONS (quoted): (1) "The parametrisation cannot express anything the Almgren-Chriss model cannot, and every advantage in the paper traces back to that. Linear permanent impact, linear temporary impact, arithmetic Brownian motion with constant volatility, no spread, no depth, no order imbalance, no intraday seasonality in any of them... The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong", which is precisely the situation a thin frontier order book creates. (2) "The convergence guarantee is real but not operational... the guarantee is conditional on a box whose right size is unknown... the theorem covers a different algorithm from the one in the experiments." (3) "Exploration requires rewinding the market, which no live venue permits... the configuration carrying the headline results is simulator-only and the deployable one is the weaker of the two." (4) "Market orders only, no spread, no queue, no fees, and the last step dumps whatever is left... This is the same restriction as in the queue-reactive paper and it bites harder in a wide-spread market." (5) "Seven large-cap Nasdaq names, two test quarters, one horizon, one participation rate... The paper's argument that EMQV is more robust to distribution shift than STAT rests on a shift between adjacent quarters in a stable market, which is the mildest available version of that test." (6) "The comparison against SAC is not tuned symmetrically... it means the empirical comparison establishes that SAC is harder to configure reliably rather than that it is worse."</t>
         </is>
       </c>
       <c r="T36" s="11" t="inlineStr">
@@ -5102,8 +5102,8 @@
         <is>
           <t>SPEAKS TO: friction-aware evaluation layer (primary), A_V (the QV risk charge $\lambda\sigma^2S_0^2 q_t^2$ is the cleanest available risk-adjusted execution objective and the note explicitly imports it because "neither of the other two execution notes carries a risk term"), orchestrator (recalibration as an actor-critic design discipline; residual-RL as the composition template).
 EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - a direct architectural contribution, quoted below. Sub-gap 2 - partial and indirect: it supplies the *form* of a live risk guardrail (a running charge proportional to squared inventory held, time-consistent, $\lambda$ swept as a reported axis) but volatility is constant ABM, so nothing on long memory or FIGARCH $d$. The transferable piece is that a risk term belongs inside the execution objective and that $\lambda$ should be a reported axis rather than a tuned hyperparameter.
-EFFECT ON SUB-GAP 1: NARROWS IT SHARPLY ON THE MODELLING SIDE - this paper explicitly implements Almgren-Chriss impact (linear permanent $\kappa$, linear temporary $\eta$), solves it in closed form, AND evaluates inside an LOB-based historical-order-flow execution simulator with permanent book contamination. So "execution cost is a function of order size" is fully implemented here - but *linearly*, and the state it depends on is $(t,q)$, not depth. What survives, and the note says so in red: "The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong, which is precisely the situation a thin frontier order book creates." Also surviving: no order-size sweep ("no sweep over order size even though impact is the subject and impact scales with size"); no spread, no depth, no queue in the cost model; and no calibration to anything but large-cap Nasdaq. The note's own summary of the three-paper bracket: "The other two notes bracket the problem, impact assumed away and impact learned model-free, and this paper takes the middle route: write the impact model down, solve it, learn only the handful of numbers the solution needs ... this is a starting point to extend rather than a method to adopt wholesale."
-PROPOSED REVISION STATED IN THE NOTE: Yes, an orchestrator revision, verbatim: "The recalibration idea generalises directly to my orchestrator, and I should design for it rather than discover the need later. The structural condition is that the critic's parametrisation depends on the actor's parameters through a known map, which is exactly what happens if the orchestrator's value function is written in terms of the agent weights it emits. When that holds, resetting the critic in lockstep after every actor update costs one matrix product and, on this evidence, is the difference between converging and oscillating. The design implication is to keep the link between the two parametrisations explicit and invertible instead of treating actor and critic as independent black boxes." And an agent-pool/architecture revision: "The residual-RL suggestion in the discussion is the template for combining a defensible baseline with a learned component. Treating the analytically derived policy as a baseline control and learning a residual on top of it with a flexible algorithm gives a floor that cannot be worse than the model-based solution by much, and a mechanism for the learner to exploit anything the model misses, such as depth or imbalance if the CSE ever exposes it ... it is a cleaner way to add a learned execution component to the orchestrator than starting from a blank policy network." Plus an objective revision: "Adopt the QV-adjusted PnL as the execution objective, because neither of the other two execution notes carries a risk term."</t>
+EFFECT ON SUB-GAP 1: NARROWS IT SHARPLY ON THE MODELLING SIDE - this paper explicitly implements Almgren-Chriss impact (linear permanent $\kappa$, linear temporary $\eta$), solves it in closed form, AND evaluates inside an LOB-based historical-order-flow execution simulator with permanent book contamination. So execution cost is a function of order size is fully implemented here - but *linearly*, and the state it depends on is $(t,q)$, not depth. What survives, and the note says so in red: "The five-parameter policy is a rigid functional form, and on a market whose impact is materially nonlinear in participation rate it will be rigidly wrong", which is precisely the situation a thin frontier order book creates. Also surviving: no order-size sweep ("no sweep over order size even though impact is the subject and impact scales with size"); no spread, no depth, no queue in the cost model; and no calibration to anything but large-cap Nasdaq. The note's own summary of the three-paper bracket: "The other two notes bracket the problem, impact assumed away and impact learned model-free, and this paper takes the middle route: write the impact model down, solve it, learn only the handful of numbers the solution needs... this is a starting point to extend rather than a method to adopt wholesale."
+PROPOSED REVISION STATED IN THE NOTE: Yes, an orchestrator revision, verbatim: "The recalibration idea generalises directly to my orchestrator, and I should design for it rather than discover the need later. The structural condition is that the critic's parametrisation depends on the actor's parameters through a known map, which is exactly what happens if the orchestrator's value function is written in terms of the agent weights it emits. When that holds, resetting the critic in lockstep after every actor update costs one matrix product and, on this evidence, is the difference between converging and oscillating. The design implication is to keep the link between the two parametrisations explicit and invertible instead of treating actor and critic as independent black boxes." And an agent-pool/architecture revision: "The residual-RL suggestion in the discussion is the template for combining a defensible baseline with a learned component. Treating the analytically derived policy as a baseline control and learning a residual on top of it with a flexible algorithm gives a floor that cannot be worse than the model-based solution by much, and a mechanism for the learner to exploit anything the model misses, such as depth or imbalance if the CSE ever exposes it... it is a cleaner way to add a learned execution component to the orchestrator than starting from a blank policy network." Plus an objective revision: "Adopt the QV-adjusted PnL as the execution objective, because neither of the other two execution notes carries a risk term."</t>
         </is>
       </c>
       <c r="X36" s="11" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Guo, Gu, Fok and Ching, out of Beijing Institute of Technology, SUSTech and the Advanced Modeling and Applied Computing Laboratory at HKU. "Online portfolio selection with state-dependent price estimators and transaction costs." European Journal of Operational Research 311 (2023) 333-353.</t>
+          <t>Guo, Gu, Fok and Ching, out of Beijing Institute of Technology, SUSTech and the Advanced Modeling and Applied Computing Laboratory at HKU. Online portfolio selection with state-dependent price estimators and transaction costs. European Journal of Operational Research 311 (2023) 333-353.</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="G37" s="11" t="inlineStr">
         <is>
-          <t>"Daily-rebalanced long-only online portfolio selection across four equity datasets, where the entire contribution sits on the cost side rather than the prediction side: the paper derives the exact analytical form of the transaction remainder factor, proves it exists and is unique, gives an algorithm that computes it exactly instead of iteratively, and then builds two optimization models around it that are switched between by a hand-set market-state rule." The assembled algorithm SOPS has three parts: SEMA (state-dependent price estimator), NPM (net profit maximization) and NPMRP (same with a risk parity penalty).</t>
+          <t>Daily-rebalanced long-only online portfolio selection across four equity datasets, where the entire contribution sits on the cost side rather than the prediction side: the paper derives the exact analytical form of the transaction remainder factor, "proves it exists and is unique, gives an algorithm that computes it exactly instead of iteratively, and then builds two optimization models around it that are switched between by a hand-set market-state rule." The assembled algorithm SOPS has three parts: SEMA (state-dependent price estimator), NPM (net profit maximization) and NPMRP (same with a risk parity penalty).</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
@@ -5165,12 +5165,12 @@
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>Transaction remainder factor, self-referential by construction: $$\omega_{t-1} + \delta \sum_{i=1}^{m} |x_{ti}\omega_{t-1} - \tilde{x}_{(t-1)i}| = 1$$ with $\tilde{x}_{(t-1)i} = \frac{x_{(t-1)i}r_{(t-1)i}}{\mathbf{r}_{t-1}\mathbf{x}_{t-1}^\top}$. Theorem 3.1 proves a unique solution in $(0,1)$; Algorithm 3.1 computes it by "sorting the ratios $\tilde{x}_{(t-1)i}/x_{ti}$ below one, walking a counter up through the resulting sub-intervals until the residual turns negative, and evaluating a closed form on that interval." Payoff is the constant bound $\frac{1-\delta}{1+\delta} \leq \omega_{t-1} \leq 1$ with linearisation error bounded by $\frac{2\delta^2}{1+\delta}\sum \hat r_{ti}x_{ti}$. SEMA state label: $$s_l^{(i)} = \begin{cases} 1, &amp; \text{if } \mu_l^{(i)} &gt; \hat\alpha^{(i)}\nu_l^{(i)} + \hat\beta^{(i)} \\ 0, &amp; \text{otherwise} \end{cases}$$ with EMA applied only to segments sharing the current state, $\hat r_{ji} = \theta + (1-\theta)\frac{\hat r_{(j-1)i}}{r^r_{(j-1)i}}$. Market state is a count: "If $\sum_{i} s_d^{(i)} \leq \zeta m$, meaning at $\zeta = 0.1$ that more than 90% of assets are Bear, the market is bearish and NPMRP is used, otherwise NPM." NPMRP: $$\max_{\mathbf{x}_t} \ \sum_{i=1}^{m}\hat r_{ti}x_{ti} - \delta\sum_{i=1}^{m}\hat r_{ti}x_{ti}\sum_{i=1}^{m}|\tilde x_{(t-1)i} - x_{ti}| - \eta\left(\tfrac{1}{2}\sum_{i=1}^{m}\sum_{j=1}^{m}\sigma_{ij}^{(t)}x_{ti}x_{tj} - c\sum_{i=1}^{m}\ln x_{ti}\right)$$ Both become QPs with $2m$ and $3m$ variables via a change of variables splitting $|x_{ti} - \tilde x_{(t-1)i}|$ into non-negative parts, $\ln(x)$ handled by a piecewise linear lower envelope of $l$ segments.</t>
+          <t>Transaction remainder factor, self-referential by construction: $$\omega_{t-1} + \delta \sum_{i=1}^{m} |x_{ti}\omega_{t-1} - \tilde{x}_{(t-1)i}| = 1$$ with $\tilde{x}_{(t-1)i} = \frac{x_{(t-1)i}r_{(t-1)i}}{\mathbf{r}_{t-1}\mathbf{x}_{t-1}^\top}$. Theorem 3.1 proves a unique solution in $(0,1)$; Algorithm 3.1 computes it by "sorting the ratios $\tilde{x}_{(t-1)i}/x_{ti}$ below one", walking a counter up through the resulting sub-intervals until the residual turns negative, and evaluating a closed form on that interval. Payoff is the constant bound $\frac{1-\delta}{1+\delta} \leq \omega_{t-1} \leq 1$ with linearisation error bounded by $\frac{2\delta^2}{1+\delta}\sum \hat r_{ti}x_{ti}$. SEMA state label: $$s_l^{(i)} = \begin{cases} 1, &amp; \text{if } \mu_l^{(i)} &gt; \hat\alpha^{(i)}\nu_l^{(i)} + \hat\beta^{(i)} \\ 0, &amp; \text{otherwise} \end{cases}$$ with EMA applied only to segments sharing the current state, $\hat r_{ji} = \theta + (1-\theta)\frac{\hat r_{(j-1)i}}{r^r_{(j-1)i}}$. Market state is a count: "If $\sum_{i} s_d^{(i)} \leq \zeta m$, meaning at $\zeta = 0.1$ that more than 90% of assets are Bear, the market is bearish and NPMRP is used, otherwise NPM." NPMRP: $$\max_{\mathbf{x}_t} \ \sum_{i=1}^{m}\hat r_{ti}x_{ti} - \delta\sum_{i=1}^{m}\hat r_{ti}x_{ti}\sum_{i=1}^{m}|\tilde x_{(t-1)i} - x_{ti}| - \eta\left(\tfrac{1}{2}\sum_{i=1}^{m}\sum_{j=1}^{m}\sigma_{ij}^{(t)}x_{ti}x_{tj} - c\sum_{i=1}^{m}\ln x_{ti}\right)$$ Both become QPs with $2m$ and $3m$ variables via a change of variables splitting $|x_{ti} - \tilde x_{(t-1)i}|$ into non-negative parts, $\ln(x)$ handled by a piecewise linear lower envelope of $l$ segments.</t>
         </is>
       </c>
       <c r="L37" s="11" t="inlineStr">
         <is>
-          <t>No learned agents, but this is the paper's structural relevance - "SOPS is a hard binary router between two objectives conditioned on a count of assets in a detected state, which is the degenerate case of the orchestrator I am proposing, and it is prior art that sits closer to my main gap than the equal-weight baseline does." Note the caveat on what "state" means here: "There is no Markov switching, no latent variable and no probability distribution over states anywhere in the paper."</t>
+          <t>No learned agents, but this is the paper's structural relevance - SOPS is a hard binary router "between two objectives conditioned on a count of assets in a detected state, which is the degenerate case of the orchestrator I am proposing, and it is prior art that sits closer to my main gap than the equal-weight baseline does." Note the caveat on what "state" means here: "There is no Markov switching, no latent variable and no probability distribution over states anywhere in the paper."</t>
         </is>
       </c>
       <c r="M37" s="11" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
-          <t>Volatility enters twice - as the per-segment $\nu_l^{(i)}$ used in the state-labelling regression $\mu = \alpha\nu + \beta$, and as $\Sigma_t$ in the NPMRP quadratic penalty with a log-barrier $-c\sum\ln x_i$. No long memory, no GARCH, no conditional volatility model. The risk parity claim does not hold up: "On the 1004th trading day SOPS holds Stock 6, Stock 16 and Stock 23 at weights of 60.80%, 4.54% and 34.66%, with risk contributions of 0.0117, 0.0008 and 0.0081, a factor of roughly fourteen between the largest and smallest. At $\eta = 0.0001$ the penalty is close to inert." Also flagged: the paper's "Calmar ratio" is actually a Sortino ratio, so "no drawdown measure appears anywhere in the paper." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): Exact accounting of the wrong functional form. Cost model is linear, proportional and symmetric: a single scalar rate $\delta \in (0,1)$ "for both buying and selling," identical across assets and independent of size. The one sophistication is the self-referential fee-on-post-cost-weights formulation - the difference is taken as $|x_{ti}\omega_{t-1} - \tilde{x}_{(t-1)i}|$ rather than $|x_{ti} - \tilde{x}_{(t-1)i}|$, "which is what makes it exact and also what makes it circular." No impact function at all - no Almgren-Chriss, no square-root, no linear impact, no depth term. No spread, no queue, no partial fill, no volume constraint. Calibration: $\delta$ fixed at 0.05% for every experiment and never varied, which the note calls out as the paper's central omission: "A paper about exact transaction cost computation never varies the transaction cost rate ... Whether SOPS still beats the nineteen baselines at a frontier-market cost rate is exactly the question the paper's machinery is built to answer and exactly the experiment it does not run." Realised cost behaviour: "the per-period cost proportion sits at its ceiling of $1 \times 10^{-3}$ in most periods, and since that ceiling is exactly $2\delta$ under the linear cost model, the portfolio is fully turning over in those periods rather than trimming. Cumulative cost over the horizon reaches 0.7528 against a cumulative return of 14.8585, and 765 of the periods carry nonzero cost." The paper itself lists as future work "variable and concave costs and a market-impact term $\Delta r \propto \ln(\Delta x)$ from Potters and Bouchaud (2003)."</t>
+          <t>Volatility enters twice - as the per-segment $\nu_l^{(i)}$ used in the state-labelling regression $\mu = \alpha\nu + \beta$, and as $\Sigma_t$ in the NPMRP quadratic penalty with a log-barrier $-c\sum\ln x_i$. No long memory, no GARCH, no conditional volatility model. The risk parity claim does not hold up: "On the 1004th trading day SOPS holds Stock 6, Stock 16 and Stock 23 at weights of 60.80%, 4.54% and 34.66%, with risk contributions of 0.0117, 0.0008 and 0.0081, a factor of roughly fourteen between the largest and smallest. At" $\eta = 0.0001$ the penalty is close to inert. Also flagged: the paper's "Calmar ratio" is actually a Sortino ratio, so "no drawdown measure appears anywhere in the paper." LIQUIDITY &amp; FRICTION HANDLING (exhaustive): Exact accounting of the wrong functional form. Cost model is linear, proportional and symmetric: a single scalar rate $\delta \in (0,1)$ "for both buying and selling," identical across assets and independent of size. The one sophistication is the self-referential fee-on-post-cost-weights formulation - the difference is taken as $|x_{ti}\omega_{t-1} - \tilde{x}_{(t-1)i}|$ rather than $|x_{ti} - \tilde{x}_{(t-1)i}|$, "which is what makes it exact and also what makes it circular." No impact function at all - no Almgren-Chriss, no square-root, no linear impact, no depth term. No spread, no queue, no partial fill, no volume constraint. Calibration: $\delta$ fixed at 0.05% for every experiment and never varied, which the note calls out as the paper's central omission: "A paper about exact transaction cost computation never varies the transaction cost rate... Whether SOPS still beats the nineteen baselines at a frontier-market cost rate is exactly the question the paper's machinery is built to answer and exactly the experiment it does not run." Realised cost behaviour: the per-period cost proportion sits at its ceiling of $1 \times 10^{-3}$ in most periods, and since that ceiling is exactly $2\delta$ under the linear cost model, "the portfolio is fully turning over in those periods rather than trimming. Cumulative cost over the horizon reaches 0.7528 against a cumulative return of 14.8585, and 765 of the periods carry nonzero cost." The paper itself lists as future work "variable and concave costs and a market-impact term $\Delta r \propto \ln(\Delta x)$ from Potters and Bouchaud (2003)."</t>
         </is>
       </c>
       <c r="P37" s="11" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="S37" s="11" t="inlineStr">
         <is>
-          <t>"SOPS takes the highest cumulative return on all four datasets ... 14.8585 against AOLNPM's 10.1757 on MSCI, $9.1526 \times 10^6$ against OLMAR-1's $8.2320 \times 10^6$ on NYSE-N, 560.4279 against AOLNPM's 321.3223 on TSE, and 6.6460 against BCRP's 5.6676 on NASTDA. The NYSE-N margin is 11% over the runner-up on a 25-year horizon, while the TSE margin is 74%." Ablation on MSCI: "EMA-NPM reaches 13.0259, SEMA-NPM 14.0270, SEMA-NPMRP 12.2729 and SOPS 14.8585," with ratios EMA-NPM 0.1096/0.1604/0.1710, SEMA-NPM 0.1137/0.1683/0.1790, SEMA-NPMRP 0.1106/0.1660/0.1745 ($\sigma(r)$ 0.0244, the lowest), SOPS 0.1163/0.1724/0.1841. Concentration: "SOPS holds two or three of the 24 MSCI assets for most of the horizon and never more than six." The paper reports an average of 4.6 selected assets at eta = 1000 and only across periods in which more than one asset is selected, so it is not the unconditional average. Sensitivity: "$\zeta$ from 0.1 to 0.2 changes cumulative return by at most 0.60% with an average relative change of 0.33%, $c$ from 3.5 to 5.5 by at most 0.77%..., $\eta$ from 0.0001 to 0.1 by at most 0.68%..., and window sizes from 25 to 38 move average prediction error by 0.38%, 0.16%, 0.43% and 0.41%." LIMITATIONS (quoted): (1) "The state-switching contribution is never isolated from how often it fires ... there is no way to tell whether the 14.0270 to 14.8585 improvement comes from switching to NPMRP at the right moments or from switching so rarely that SOPS is mostly NPM with occasional de-risking." (2) "A paper about exact transaction cost computation never varies the transaction cost rate." (3) "Linear proportional cost is the whole cost model, so 'exact' is exact within a form that omits the costs that matter in a thin book. There is no bid-ask spread, no market impact, no partial fill, no queue position and no volume constraint ... it means the exactness result is exactness about commission, and the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper." (4) "No walk-forward, no seeds, no significance tests, and per-dataset window sizes with no selection procedure." (5) "Practicality is claimed and never measured." (6) "The prediction and allocation stages share a single point of failure ... when SEMA mispredicts, both models fail together and the router has nothing to route to."</t>
+          <t>"SOPS takes the highest cumulative return on all four datasets... 14.8585 against AOLNPM's 10.1757 on MSCI, $9.1526 \times 10^6$ against OLMAR-1's $8.2320 \times 10^6$ on NYSE-N, 560.4279 against AOLNPM's 321.3223 on TSE, and 6.6460 against BCRP's 5.6676 on NASTDA. The NYSE-N margin is 11% over the runner-up on a 25-year horizon, while the TSE margin is 74%." Ablation on MSCI: "EMA-NPM reaches 13.0259, SEMA-NPM 14.0270, SEMA-NPMRP 12.2729 and SOPS 14.8585," with ratios EMA-NPM 0.1096/0.1604/0.1710, SEMA-NPM 0.1137/0.1683/0.1790, SEMA-NPMRP 0.1106/0.1660/0.1745 ($\sigma(r)$ 0.0244, the lowest), SOPS 0.1163/0.1724/0.1841. Concentration: "SOPS holds two or three of the 24 MSCI assets for most of the horizon and never more than six." The paper reports an average of 4.6 selected assets at eta = 1000 and only across periods in which more than one asset is selected, so it is not the unconditional average. Sensitivity: "$\zeta$ from 0.1 to 0.2 changes cumulative return by at most 0.60% with an average relative change of 0.33%, $c$ from 3.5 to 5.5 by at most 0.77%..., $\eta$ from 0.0001 to 0.1 by at most 0.68%..., and window sizes from 25 to 38 move average prediction error by 0.38%, 0.16%, 0.43% and 0.41%." LIMITATIONS (quoted): (1) "The state-switching contribution is never isolated from how often it fires... there is no way to tell whether the 14.0270 to 14.8585 improvement comes from switching to NPMRP at the right moments or from switching so rarely that SOPS is mostly NPM with occasional de-risking." (2) "A paper about exact transaction cost computation never varies the transaction cost rate." (3) Linear proportional cost is the whole cost model, so 'exact' is exact within a form that omits the costs that matter in a thin book. There is no bid-ask spread, no market impact, no partial fill, no queue position and no volume constraint... it means the exactness result is exactness about commission, and the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper. (4) "No walk-forward, no seeds, no significance tests, and per-dataset window sizes with no selection procedure." (5) "Practicality is claimed and never measured." (6) "The prediction and allocation stages share a single point of failure... when SEMA mispredicts, both models fail together and the router has nothing to route to."</t>
         </is>
       </c>
       <c r="T37" s="11" t="inlineStr">
@@ -5226,9 +5226,9 @@
       <c r="W37" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: friction-aware evaluation layer (primary - the TRF closed form and constant bounds go directly in), orchestrator (SOPS is the hard-router prior art and becomes a required baseline), A_V (log-barrier diversification penalty and the per-asset $\mu$-vs-$\nu$ state label).
-EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - substantial. SOPS is "the degenerate case of the orchestrator I am proposing," a hard binary router on a count of per-asset states, and the note both adopts it as a baseline and uses its failure to diagnose router firing rate as the motivation for weight-entropy reporting. It also links to MacroHFT: "This is the same diagnostic problem as MacroHFT's near-binary learned mixture ... arriving from the opposite direction, and it is the specific thing my own weight-entropy reporting is meant to prevent." Sub-gap 2 - indirect and mostly as a cheaper competitor to FIGARCH: SEMA is "far cheaper than the FIGARCH route ... which matters because the only confirmed ready-made CSE set covers February 2025 to February 2026. With roughly 240 trading days and $w \approx 30$ that is 8 segments for a two-parameter regression, thin but not absurd." No long-memory content of its own.
-EFFECT ON SUB-GAP 1: LEAVES IT OPEN, and is the strongest illustration that it is open. Zero impact modelling: no Almgren-Chriss, no square-root, no LOB simulator, no depth anywhere. Cost is exactly the flat-rate-on-turnover model the sub-gap is aimed at, computed exactly. The note's own verdict, in red: "the execution-friction blind spot survives in the paper that treats transaction cost most rigorously, which is now the second time I have written that sentence about a portfolio paper." What this paper *does* contribute to closing sub-gap 1 is machinery rather than a model: the exact, provably unique transaction remainder factor with constant bounds $\frac{1-\delta}{1+\delta} \leq \omega_{t-1} \leq 1$, which "lets a cost term stay inside a convex objective rather than sitting outside it as a post-hoc deduction" - that is the container into which a state-dependent $\delta$ can be substituted. It also hands over the exact experiment the sub-gap needs: the $\delta$ sweep the authors skipped.
-PROPOSED REVISION STATED IN THE NOTE: Yes, several, verbatim. On the evaluation/baseline set: "SOPS is the fourth baseline my evaluation design is missing. My current three are equal weight, static learned weight and dynamic state-aware weight. A hard state-conditioned router, a threshold rule that picks one of two objectives with no learning and no confidence input, sits between the second and third and is much closer to real prior art than equal weighting. If my adaptive orchestrator cannot beat a count-and-threshold switch, the soft-weighting contribution is not there, and I would rather discover that in my own ablation than have it asked in a viva. This is a direct proposed revision to the experimental design section of the scope note." On the conditioning set: "SEMA is a candidate state variable for the orchestrator that costs almost nothing in data ... The labelling rule itself is also a testable alternative to MacroHFT's volatility tertile, and its advantage for $A_V$ is that it is per asset rather than per market, giving the orchestrator an asset-level state vector that can be aggregated by a count, as this paper does, or fed in directly. Both are crude and neither has a strong theoretical claim over the other, so implement both and let the ablation decide." On $A_V$: "The log-barrier diversification term is reusable for $A_V$ ... if I use a penalty of this shape I report the realised contributions alongside the weights and describe it as a diversification penalty, not as parity."</t>
+EFFECT ON MAIN GAP / SUB-GAP 2: Main gap - substantial. SOPS is "the degenerate case of the orchestrator I am proposing," a hard binary router on a count of per-asset states, and the note both adopts it as a baseline and uses its failure to diagnose router firing rate as the motivation for weight-entropy reporting. It also links to MacroHFT: "This is the same diagnostic problem as MacroHFT's near-binary learned mixture... arriving from the opposite direction, and it is the specific thing my own weight-entropy reporting is meant to prevent." Sub-gap 2 - indirect and mostly as a cheaper competitor to FIGARCH: SEMA is "far cheaper than the FIGARCH route... which matters because the only confirmed ready-made CSE set covers February 2025 to February 2026. With roughly 240 trading days and $w \approx 30$ that is 8 segments for a two-parameter regression, thin but not absurd." No long-memory content of its own.
+EFFECT ON SUB-GAP 1: LEAVES IT OPEN, and is the strongest illustration that it is open. Zero impact modelling: no Almgren-Chriss, no square-root, no LOB simulator, no depth anywhere. Cost is exactly the flat-rate-on-turnover model the sub-gap is aimed at, computed exactly. The note's own verdict, in red: "the execution-friction blind spot survives in the paper that treats transaction cost most rigorously", which is now the second time I have written that sentence about a portfolio paper. What this paper *does* contribute to closing sub-gap 1 is machinery rather than a model: the exact, provably unique transaction remainder factor with constant bounds $\frac{1-\delta}{1+\delta} \leq \omega_{t-1} \leq 1$, which "lets a cost term stay inside a convex objective rather than sitting outside it as a post-hoc deduction" - that is the container into which a state-dependent $\delta$ can be substituted. It also hands over the exact experiment the sub-gap needs: the $\delta$ sweep the authors skipped.
+PROPOSED REVISION STATED IN THE NOTE: Yes, several, verbatim. On the evaluation/baseline set: SOPS is the fourth baseline my evaluation design is missing. My current three are equal weight, static learned weight and dynamic state-aware weight. A hard state-conditioned router, "a threshold rule that picks one of two objectives with no learning and no confidence input, sits between the second and third and is much closer to real prior art than equal weighting. If my adaptive orchestrator cannot beat a count-and-threshold switch, the soft-weighting contribution is not there, and I would rather discover that in my own ablation than have it asked in a viva. This is a direct proposed revision to the experimental design section of the scope note." On the conditioning set: "SEMA is a candidate state variable for the orchestrator that costs almost nothing in data... The labelling rule itself is also a testable alternative to MacroHFT's volatility tertile, and its advantage for $A_V$ is that it is per asset rather than per market, giving the orchestrator an asset-level state vector that can be aggregated by a count, as this paper does, or fed in directly. Both are crude and neither has a strong theoretical claim over the other, so implement both and let the ablation decide." On $A_V$: "The log-barrier diversification term is reusable for $A_V$... if I use a penalty of this shape I report the realised contributions alongside the weights and describe it as a diversification penalty, not as parity."</t>
         </is>
       </c>
       <c r="X37" s="11" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>Briola, Bartolucci and Aste, UCL Computer Science and the LSE Systemic Risk Centre. "HLOB – Information persistence and structure in limit order books." Expert Systems With Applications 266, 2025, article 126078. Published open access 12 December 2024.</t>
+          <t>Briola, Bartolucci and Aste, UCL Computer Science and the LSE Systemic Risk Centre. HLOB – Information persistence and structure in limit order books. Expert Systems With Applications 266, 2025, article 126078. Published open access 12 December 2024.</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Introduces "HLOB, a deep learning architecture for forecasting the direction of mid-price changes in a Limit Order Book, and its one real idea is to stop treating the LOB as an image." Instead of convolving over price levels as stored, it learns a dependency structure among volume levels with an "Information Filtering Network, specifically the Triangulated Maximally Filtered Graph," then feeds the resulting tetrahedra, triangles and edges into a "Homological Convolutional Neural Network extended with an LSTM for temporal dynamics."</t>
+          <t>Introduces HLOB, a deep learning architecture for forecasting the direction of mid-price changes "in a Limit Order Book, and its one real idea is to stop treating the LOB as an image." Instead of convolving over price levels as stored, it learns a dependency structure among volume levels with an Information Filtering Network, specifically the Triangulated Maximally Filtered Graph, then feeds the resulting tetrahedra, triangles and edges into a Homological Convolutional Neural Network extended with an LSTM for temporal dynamics.</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -5285,12 +5285,12 @@
       </c>
       <c r="J38" s="11" t="inlineStr">
         <is>
-          <t>Pure LOB - 10 levels of price and volume per side. TMFG built from volume data only, "reducing each snapshot from $\mathbb{R}^{4L}$ to $\mathbb{R}^{2L}$, on the reasoning that volumes are the homogeneous part of the record while price levels are not." Derived diagnostic: 'actual depth' $\Xi^\text{Bid}$, $\Xi^\text{Ask}$ from Wu et al. (2021), "the number of tick-sized price intervals the ten quoted levels span." Labelling is absolute-threshold three-class: $$ \begin{cases} (m_{\tau + \Delta\tau} - m_{\tau}) \leq -\theta &amp;\rightarrow\ -1\ \rightarrow\ \text{Down}\\ -\theta &lt; (m_{\tau + \Delta\tau} - m_{\tau}) &lt; +\theta &amp;\rightarrow\ \ \ 0\ \rightarrow\ \text{Stable}\\ (m_{\tau + \Delta\tau} - m_{\tau}) \geq +\theta &amp;\rightarrow\ +1\ \rightarrow\ \text{Up} \end{cases} $$ with $m_\tau = \frac{p_1^\text{ask}(\tau) + p_1^\text{bid}(\tau)}{2}$ and $\sigma_\tau = p_1^\text{ask}(\tau) - p_1^\text{bid}(\tau)$.</t>
+          <t>Pure LOB - 10 levels of price and volume per side. TMFG built from volume data only, "reducing each snapshot from $\mathbb{R}^{4L}$ to $\mathbb{R}^{2L"}$, on the reasoning that volumes are the homogeneous part of the record while price levels are not. Derived diagnostic: 'actual depth' $\Xi^\text{Bid}$, $\Xi^\text{Ask}$ from Wu et al. (2021), "the number of tick-sized price intervals the ten quoted levels span." Labelling is absolute-threshold three-class: $$ \begin{cases} (m_{\tau + \Delta\tau} - m_{\tau}) \leq -\theta &amp;\rightarrow\ -1\ \rightarrow\ \text{Down}\\ -\theta &lt; (m_{\tau + \Delta\tau} - m_{\tau}) &lt; +\theta &amp;\rightarrow\ \ \ 0\ \rightarrow\ \text{Stable}\\ (m_{\tau + \Delta\tau} - m_{\tau}) \geq +\theta &amp;\rightarrow\ +1\ \rightarrow\ \text{Up} \end{cases} $$ with $m_\tau = \frac{p_1^\text{ask}(\tau) + p_1^\text{bid}(\tau)}{2}$ and $\sigma_\tau = p_1^\text{ask}(\tau) - p_1^\text{bid}(\tau)$.</t>
         </is>
       </c>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>Volumes discretized into equally spaced bins (bin count tuned once, held constant across stocks) "to stop minimum-lot granularity from injecting noise into the estimator"; pairwise mutual information between all volume levels, bootstrapped daily, averaged across training days, giving one $(2L \times 2L)$ similarity matrix per stock. Graph selection: $$\mathcal{G}^{*} \Rightarrow \arg\min_{\mathcal{G}} D_{KL}\big(f(\mathbb{L})\ \|\ \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} \mathbb{E}_{f}\big(\log f(\mathbb{L})\big) - \mathbb{E}_{f}\big(\log \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} H(\mathbb{L}|\mathcal{G})$$ Three simplicial families extracted - maximal cliques of size 4, 3, 2, giving "a fixed 17 tetrahedra, 52 triangles and 54 edges for a 20-node graph" and three input tensors of shape $100 \times 136$, $100 \times 312$, $100 \times 216$. Each head runs three convolutional layers: first $1\times2$ with stride $1\times2$ so it "prevents parameter sharing between levels that are geographically but not logically consecutive, which is the whole complaint against DeepLOB expressed as a stride"; second with stride $1\times4$, $1\times3$, $1\times2$ mixing only within-simplex components; third with filter $1\times\Omega$ for $\Omega \in \{17,52,54\}$, dropout 0.35. Concatenation into a 32-unit LSTM and a 3-output dense layer. AdamW at $6\times10^{-5}$, $\beta_1=0.90$, $\beta_2=0.95$, batch 32, max 100 epochs, early stopping at 0.003 over 15 epochs. Output: three-class direction.</t>
+          <t>Volumes discretized into equally spaced bins (bin count tuned once, held constant across stocks) to stop minimum-lot granularity from injecting noise into the estimator; pairwise mutual information between all volume levels, bootstrapped daily, averaged across training days, giving one $(2L \times 2L)$ similarity matrix per stock. Graph selection: $$\mathcal{G}^{*} \Rightarrow \arg\min_{\mathcal{G}} D_{KL}\big(f(\mathbb{L})\ \|\ \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} \mathbb{E}_{f}\big(\log f(\mathbb{L})\big) - \mathbb{E}_{f}\big(\log \tilde{f}(\mathbb{L}|\mathcal{G})\big) \Rightarrow \arg\min_{\mathcal{G}} H(\mathbb{L}|\mathcal{G})$$ Three simplicial families extracted - maximal cliques of size 4, 3, 2, giving "a fixed 17 tetrahedra, 52 triangles and 54 edges for a 20-node graph" and three input tensors of shape $100 \times 136$, $100 \times 312$, $100 \times 216$. Each head runs three convolutional layers: first $1\times2$ with stride $1\times2$ so it "prevents parameter sharing between levels that are geographically but not logically consecutive, which is the whole complaint against DeepLOB expressed as a stride"; second with stride $1\times4$, $1\times3$, $1\times2$ mixing only within-simplex components; third with filter $1\times\Omega$ for $\Omega \in \{17,52,54\}$, dropout 0.35. Concatenation into a 32-unit LSTM and a 3-output dense layer. AdamW at $6\times10^{-5}$, $\beta_1=0.90$, $\beta_2=0.95$, batch 32, max 100 epochs, early stopping at 0.003 over 15 epochs. Output: three-class direction.</t>
         </is>
       </c>
       <c r="L38" s="11" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="S38" s="11" t="inlineStr">
         <is>
-          <t>"HLOB outperforms the 9 alternatives in 73.3% of the 15 stock cases at $H_{\Delta\tau} = 10$, 60% at $H_{\Delta\tau} = 50$, and 33% at $H_{\Delta\tau} = 100$." Tick-class table (F1 / MCC / $p_\text{T}$): small-tick 0.42/0.16/0.11 at $H_{10}$, 0.36/0.09/0.07 at $H_{50}$, 0.32/0.05/0.05 at $H_{100}$; medium-tick 0.41/0.16/0.14, 0.40/0.11/0.10, 0.35/0.06/0.07; large-tick 0.48/0.33/0.10, 0.58/0.38/0.14, 0.52/0.30/0.15. "An MCC of 0.05 on small-tick stocks at the longest horizon is a model that has essentially stopped predicting, while 0.30 on large-tick stocks at the same horizon is a model still working." MI levels: "average non-normalized MI runs from 0.26 for GOOG to 0.74 for IBM" (small-tick) versus "0.62 for ORCL to 1.18 for BAC" (large-tick) with "a clean three-group hierarchy." Against DeepLOB: "At $H_{\Delta\tau} = 10$ the average F1 gain is 0.03, 0.02 and 0.003 for small-, medium- and large-tick stocks, with MCC gains of 0.04, 0.04 and 0.02; at $H_{\Delta\tau} = 50$ the F1 gains rise to 0.05, 0.05 and 0.01 and the MCC gains to 0.06, 0.02 and 0.03." Parameter count discrepancy: "Table 3 lists HLOB at $1.8\times10^4$ trainable parameters ... The per-layer counts in Section 4.2 ... sum to roughly $1.8\times10^5$." LIMITATIONS (quoted): (1) "No statistical testing appears anywhere, and the headline claim is a win count ... it means the 0.003 F1 gain over DeepLOB on large-tick stocks and the 0.04 MCC gain on small-tick stocks, both at the H-delta-tau = 10 horizon, are presented with identical evidential weight." (2) "Nothing isolates the TMFG, so the central claim about higher-order topological priors rests on a model-versus-model comparison ... without one, the claim that the mutual-information structure is what produces the gain is the paper's interpretation of a result rather than a result. This is the limitation I would raise first if I were reviewing it." (3) "The reported parameter count does not reconcile with the architecture description." (4) "The label threshold is absolute while the grouping variable is relative, which partially confounds the tick-size finding ... Some portion of 'large-tick books are more learnable' is a statement about the relationship between the label threshold and the spread rather than about the spatial structure of the book." (5) "The structure is static in a paper about persistence, and the authors say so ... it is a plausible alternative explanation for the horizon degradation, since a structure estimated as a 40-day average will describe a longer horizon worse for exactly the stocks whose books drift most, which is the small-tick group." (6) "Event-time horizons, no execution model, and one venue ... no fees, no queue position, no partial fills, no market impact."</t>
+          <t>"HLOB outperforms the 9 alternatives in 73.3% of the 15 stock cases at $H_{\Delta\tau} = 10$, 60% at $H_{\Delta\tau} = 50$, and 33% at $H_{\Delta\tau} = 100$." Tick-class table (F1 / MCC / $p_\text{T}$): small-tick 0.42/0.16/0.11 at $H_{10}$, 0.36/0.09/0.07 at $H_{50}$, 0.32/0.05/0.05 at $H_{100}$; medium-tick 0.41/0.16/0.14, 0.40/0.11/0.10, 0.35/0.06/0.07; large-tick 0.48/0.33/0.10, 0.58/0.38/0.14, 0.52/0.30/0.15. "An MCC of 0.05 on small-tick stocks at the longest horizon is a model that has essentially stopped predicting, while 0.30 on large-tick stocks at the same horizon is a model still working." MI levels: "average non-normalized MI runs from 0.26 for GOOG to 0.74 for IBM" (small-tick) versus "0.62 for ORCL to 1.18 for BAC" (large-tick) with "a clean three-group hierarchy." Against DeepLOB: "At $H_{\Delta\tau} = 10$ the average F1 gain is 0.03, 0.02 and 0.003 for small-, medium- and large-tick stocks, with MCC gains of 0.04, 0".04 and 0.02; at $H_{\Delta\tau} = 50$ the F1 gains rise to 0.05, 0.05 and 0.01 and the MCC gains to 0.06, 0.02 and 0.03. Parameter count discrepancy: Table 3 lists HLOB at $1.8\times10^4$ trainable parameters... The per-layer counts in Section 4.2... sum to roughly $1.8\times10^5$. LIMITATIONS (quoted): (1) "No statistical testing appears anywhere, and the headline claim is a win count... it means the 0.003 F1 gain over DeepLOB on large-tick stocks and the 0".04 MCC gain on small-tick stocks, both at the H-delta-tau = 10 horizon, are presented with identical evidential weight. (2) "Nothing isolates the TMFG, so the central claim about higher-order topological priors rests on a model-versus-model comparison... without one, the claim that the mutual-information structure is what produces the gain is the paper's interpretation of a result rather than a result". This is the limitation I would raise first if I were reviewing it. (3) The reported parameter count does not reconcile with the architecture description. (4) "The label threshold is absolute while the grouping variable is relative, which partially confounds the tick-size finding... Some portion of 'large-tick books are more learnable' is a statement about the relationship between the label threshold and the spread rather than about the spatial structure of the book." (5) "The structure is static in a paper about persistence, and the authors say so... it is a plausible alternative explanation for the horizon degradation, since a structure estimated as a 40-day average will describe a longer horizon worse for exactly the stocks whose books drift most, which is the small-tick group." (6) "Event-time horizons, no execution model, and one venue... no fees, no queue position, no partial fills, no market impact."</t>
         </is>
       </c>
       <c r="T38" s="11" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>proposes GNNHAR, "a nonparametric extension of the HAR family that replaces the linear neighbourhood aggregation in GHAR with a graph convolutional layer, and then uses that architecture as an instrument to answer three separable questions: whether volatility spillover reaches beyond one-hop neighbours, whether the spillover is nonlinear, and whether the estimation criterion used to fit the model matters as much as the model itself. The answers are no, yes at short horizons, and yes substantially, in that order, and the third is the one that generalises furthest."</t>
+          <t>proposes GNNHAR, a nonparametric extension of the HAR family that replaces the linear neighbourhood aggregation in GHAR with a graph convolutional layer, and then uses that architecture as an instrument to answer three separable questions: whether volatility spillover reaches beyond one-hop neighbours, whether the spillover is nonlinear, and whether the estimation criterion "used to fit the model matters as much as the model itself. The answers are no, yes at short horizons, and yes substantially, in that order, and the third is the one that generalises furthest."</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>HAR / GHAR / GNNHAR1L-2L-3L, fitted under MSE (OLS for the linear ones) or QL (Adam). GHAR baseline: E(v_t|F_{t-1}) = α + V_{:t-1}β + W V_{:t-1}γ, with W = O^{-1/2} A O^{-1/2}. GNNHAR replaces the W V γ term with a graph convolution H^{(l+1)} = ReLU(O^{-1/2} A O^{-1/2} H^{(l)} Θ^{(l)}), H^{(0)} = V_{:t-1}. QL objective: (1/N)Σ_i (1/#T)Σ_t [ RV_{i,t}/RV̂_{i,t} − log(RV_{i,t}/RV̂_{i,t}) − 1 ]. Proposition 3.1: optimising HAR under QL is equivalent to IRLS with weights w_{k-1,t} = 1/RV̂²_{k-1,t}, i.e. "WLS that down-weights high-volatility observations in proportion to the square of the fitted level".  graph-convolutional extension of HAR; output is a point forecast of next-period RV per stock. Key design note: "The propagation rule deliberately omits self-connections, unlike the Kipf and Welling (2017) GCN it is adapted from, so a stock's own past volatility enters only through the linear V_{:t-1}β term and every nonlinearity in the model lives in the spillover channel... it is a design choice I would copy."</t>
+          <t>HAR / GHAR / GNNHAR1L-2L-3L, fitted under MSE (OLS for the linear ones) or QL (Adam). GHAR baseline: E(v_t|F_{t-1}) = α + V_{:t-1}β + W V_{:t-1}γ, with W = O^{-1/2} A O^{-1/2}. GNNHAR replaces the W V γ term with a graph convolution H^{(l+1)} = ReLU(O^{-1/2} A O^{-1/2} H^{(l)} Θ^{(l)}), H^{(0)} = V_{:t-1}. QL objective: (1/N)Σ_i (1/#T)Σ_t [ RV_{i,t}/RV̂_{i,t} − log(RV_{i,t}/RV̂_{i,t}) − 1 ]. Proposition 3.1: optimising HAR under QL is equivalent to IRLS with weights w_{k-1,t} = 1/RV̂²_{k-1,t}, i.e. "WLS that down-weights high-volatility observations in proportion to the square of the fitted level". graph-convolutional extension of HAR; output is a point forecast of next-period RV per stock. Key design note: The propagation rule deliberately omits self-connections, unlike the Kipf and Welling (2017) GCN it is adapted from, so a stock's own past volatility enters only through the linear V_{:t-1}β term and every nonlinearity in the model lives in the spillover channel... it is a design choice I would copy.</t>
         </is>
       </c>
       <c r="L39" s="11" t="inlineStr">
@@ -5479,7 +5479,7 @@
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap - indirect support via the calm/turbulent template and the MAD collapse diagnostic, but no orchestration of any kind. Sub-gap 1 - none; friction is entirely absent by design.
 EFFECT ON SUB-GAP 2: LEAVES IT OPEN, and does so in the most quotable way of any paper here. It is the purest instance of the sub-gap's failure mode: volatility is forecast with ten years of rigorous out-of-sample evaluation and 120 monthly refits, and nothing is ever done with the forecast. The note states it flatly - "Forecast loss is the only outcome, and the economic question is left open... no portfolio, no value-at-risk backtest and no transaction-cost-bearing application, so a 13% MSE reduction at the one-day horizon has no translation into a decision anywhere in the paper." Specifically on the two questions asked: (a) YES, it uses realised volatility predictively - that is the entire object, next-day/week/month RV forecast conditioned on a cross-sectional graph, and it is genuinely predictive rather than descriptive, with 13% MSE reduction at one day. (b) NO, it does nothing with persistence or long memory as an estimated quantity. Long memory appears once, as motivation for the HAR lag structure itself: the three-lag spine is "the cheapest available way to reproduce the long-memory decay in the RV autocorrelation function without fitting a fractionally integrated model". So long memory is absorbed into the model's functional form and never estimated, never reported as a coefficient, never fed anywhere. There is no d, no fractional integration, no decay-speed parameter. The paper's contribution runs entirely in the cross-sectional (spillover) direction and leaves the temporal-persistence direction untouched - which is exactly the axis Sub-gap 2 lives on. The one partial narrowing it offers is indirect: the calm/turbulent stratification shows forecast quality is itself state-dependent, and the FVU numbers locate the nonlinear model's value in the top volatility decile, which is an argument that volatility state should condition something - but the paper conditions only its reporting, not its behaviour.
 CSE DATA EVIDENCE: not a CSE paper. Relevant only negatively: five-minute RV is unobtainable here, so the estimator's input has to be re-derived (Parkinson or Garman-Klass daily range-based), and building a CSE volatility graph faces a problem the DJIA does not - "a meaningful share of counters post zero returns on a given day because they did not trade, which biases any covariance estimate towards spurious independence and will make the precision matrix unstable."
-PROPOSED REVISION STATED IN THE NOTE: no revision to the four-agent pool. On the conditioning set, two things bear on C_{i,t}: "The QL loss ratio is a second candidate for the comparable-confidence problem, and a better-behaved one than p_T... A rolling QL loss ratio against a fixed benchmark is unit-free, computable for any component that emits a distributional or point forecast of the same target, and interpretable in the same direction regardless of the component's internals, which makes it a rolling competence weight in exactly the way the p_T metric from HLOB is for directional components. Neither gives a per-decision confidence, both give a backward-looking competence estimate, and having two of them defined on different output types is progress on the problem rather than a solution to it." And on V_t: "the paper's label is computed ex post, and a live orchestrator needs the same label from a rolling estimate, so pinning the minimum window for a usable turbulence indicator on CSE data is now a concrete task rather than an open question."</t>
+PROPOSED REVISION STATED IN THE NOTE: no revision to the four-agent pool. On the conditioning set, two things bear on C_{i,t}: The QL loss ratio is a second candidate for the comparable-confidence problem, and a better-behaved one than p_T... A rolling QL loss ratio against a fixed benchmark is unit-free, computable for any component that emits a distributional or point forecast of the same target, and interpretable in the same direction regardless of the component's internals, which makes it a rolling competence weight in exactly the way the p_T metric from HLOB is for directional components. Neither gives a per-decision confidence, both give a backward-looking competence estimate, and having two of them defined on different output types is progress on the problem rather than a solution to it. And on V_t: "the paper's label is computed ex post, and a live orchestrator needs the same label from a rolling estimate, so pinning the minimum window for a usable turbulence indicator on CSE data is now a concrete task rather than an open question."</t>
         </is>
       </c>
       <c r="X39" s="11" t="inlineStr">
@@ -5531,12 +5531,12 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>"Monthly series from January 2010 to December 2019, 120 observations per variable, 117 after lags, no missing values reported. The decade is chosen deliberately to exclude COVID-19, which the authors present as avoiding extreme events."</t>
+          <t>Monthly series from January 2010 to December 2019, 120 observations per variable, 117 after lags, "no missing values reported. The decade is chosen deliberately to exclude COVID-19, which the authors present as avoiding extreme events."</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
         <is>
-          <t>dependent - monthly change in the All Share Price Index, from CSE market data. Independent, all from CBSL - GDP growth rate, inflation via CCPI, Weighted Average Deposit Rate, broad money M2, USD/LKR. "GDP is quarterly and was converted to monthly with the Quadratic Interpolation Method in EViews, citing Ju et al. (2014)." All in logs.</t>
+          <t>dependent - monthly change in the All Share Price Index, from CSE market data. Independent, all from CBSL - GDP growth rate, inflation via CCPI, Weighted Average Deposit Rate, broad money M2, USD/LKR. "GDP is quarterly and was converted to monthly with the" Quadratic Interpolation Method in EViews, citing Ju et al. (2014). All in logs.</t>
         </is>
       </c>
       <c r="K40" s="11" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
-          <t>nominally the whole paper, actually nothing. The note's flagged warning: "The proxy and the construct never meet. Table 1 defines stock price volatility as 'upward and downward movements of the stock market prices' and measures it as monthly change in ASPI. A signed one-period change has no dispersion in it at all, so the paper's finding that higher interest rates reduce 'volatility' is, on its own measurement, the conventional and unsurprising finding that higher rates reduce returns. Every volatility claim in the abstract and conclusion is scoped to this." And: "The dependent variable is not volatility, it is the monthly change in the ASPI, which is a return, and once that's clear every substantive interpretation in the paper has to be re-read as a statement about returns wearing the word volatility." The contrast the note draws: STOCKV_t = (ASPI_t − ASPI_{t-1})/ASPI_{t-1} against σ̂_t = sqrt( (1/(n_t−1)) Σ_d (r_{t,d} − r̄_t)² ). No conditional-variance model, no GARCH, no persistence, no risk quantity of any kind.</t>
+          <t>nominally the whole paper, actually nothing. The note's flagged warning: "The proxy and the construct never meet. Table 1 defines stock price volatility as 'upward and downward movements of the stock market prices' and measures it as monthly change in ASPI. A signed one-period change has no dispersion in it at all, so the paper's finding that higher interest rates reduce 'volatility' is, on its own measurement, the conventional and unsurprising finding that higher rates reduce returns. Every volatility claim in the abstract and conclusion is scoped to this." And: The dependent variable is not volatility, it is the monthly change in the ASPI, which is a return, and once that's clear every substantive interpretation in the paper has to be re-read as a statement about returns wearing the word volatility. The contrast the note draws: STOCKV_t = (ASPI_t − ASPI_{t-1})/ASPI_{t-1} against σ̂_t = sqrt((1/(n_t−1)) Σ_d (r_{t,d} − r̄_t)²). No conditional-variance model, no GARCH, no persistence, no risk quantity of any kind.</t>
         </is>
       </c>
       <c r="P40" s="11" t="inlineStr">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="S40" s="11" t="inlineStr">
         <is>
-          <t>"The F-statistic comes out at 14.36187 with k = 5, against an upper I(1) bound of 4.15 asymptotically and 4.587 in the finite-sample (n = 80) critical values". Long-run vector: STOCKV = 0.7673 EX + 0.0574 GDPMN + 2.5493 INF + 0.0368 INT − 0.3864 MS − 0.0002, with "Inflation carries by far the largest long-run coefficient at 2.549274 with p = 0.05, the exchange rate is next at 0.767264 with p = 0.0734, and interest rate, money supply and GDP are nowhere, at p = 0.9168, 0.7497 and 0.287." Short run: "The exchange rate at a two-month lag is the strongest single result, 0.583956 with p = 0.0015"; "The interest rate at a one-month lag is the only other significant term, −13.8453 with p = 0.0122". Lagged dependent variable "flat, 0.015096 with p = 0.8698", DW = 1.944936. Fit: "R² = 0.300153 falling to an adjusted 0.189286 on 117 observations." LIMITATIONS (quoting the note): "The bounds test confirms a long-run relationship and the paper then rejects one... Those two statements are about the same estimation and they contradict each other." "The construct and the measurement are different quantities, and this propagates into every interpretation... A near-zero AR(1) term with p = 0.8698 is consistent with a return series and inconsistent with a volatility series, so the paper's cleanest internal evidence is against its own dependent variable." "The short-run and long-run coefficients are used interchangeably." "If any variable is genuinely I(2) the bounds F-distribution is invalid, and the paper's evidence points that way." "Diagnostics stop at Durbin-Watson." "Interpolating GDP inflates the apparent sample... produces 120 monthly figures out of 40 independent observations." "The sample is defined to exclude exactly the regimes that matter now... a study of macroeconomic *stability* variables that drops the instability is answering a narrower question than the title claims."</t>
+          <t>The F-statistic comes out at 14.36187 with k = 5, "against an upper I(1) bound of 4.15 asymptotically and 4.587 in the finite-sample (n = 80) critical values". Long-run vector: STOCKV = 0.7673 EX + 0.0574 GDPMN + 2.5493 INF + 0.0368 INT − 0.3864 MS − 0.0002, with "Inflation carries by far the largest long-run coefficient at 2.549274 with p = 0.05, the exchange rate is next at 0.767264 with p = 0.0734, and interest rate, money supply and GDP are nowhere, at p = 0.9168, 0.7497 and 0.287." Short run: "The exchange rate at a two-month lag is the strongest single result, 0.583956 with p = 0.0015"; "The interest rate at a one-month lag is the only other significant term, −13.8453 with p = 0.0122". Lagged dependent variable "flat, 0.015096 with p = 0.8698", DW = 1.944936. Fit: "R² = 0.300153 falling to an adjusted 0.189286 on 117 observations." LIMITATIONS (quoting the note): "The bounds test confirms a long-run relationship and the paper then rejects one... Those two statements are about the same estimation and they contradict each other." "The construct and the measurement are different quantities, and this propagates into every interpretation... A near-zero AR(1) term with p = 0.8698 is consistent with a return series and inconsistent with a volatility series, so the paper's cleanest internal evidence is against its own dependent variable." "The short-run and long-run coefficients are used interchangeably." "If any variable is genuinely I(2) the bounds F-distribution is invalid, and the paper's evidence points that way." "Diagnostics stop at Durbin-Watson." "Interpolating GDP inflates the apparent sample... produces 120 monthly figures out of 40 independent observations." "The sample is defined to exclude exactly the regimes that matter now... a study of macroeconomic *stability* variables that drops the instability is answering a narrower question than the title claims."</t>
         </is>
       </c>
       <c r="T40" s="11" t="inlineStr">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>"Monthly series, 2014 to 2022, 108 observations claimed, purposive sampling, all variables converted to natural logarithms before testing. Sources are the Central Bank of Sri Lanka for money supply and the exchange rate, the Colombo Stock Exchange for the ASPI and trading volume, and the Department of Census and Statistics for inflation." The note records the sample accounting failing: "The counts are 106 for the differenced exchange rate and money supply, 105 for the twice-differenced NCPI, and 107 for log ASPI and log trading volume, none of which is the 108 asserted in the text, and page 127 separately describes the window as 2014 to 2023 while every other statement in the paper says 2022."</t>
+          <t>Monthly series, 2014 to 2022, 108 observations claimed, "purposive sampling, all variables converted to natural logarithms before testing. Sources are the Central Bank of Sri Lanka for money supply and the exchange rate, the Colombo Stock Exchange for the ASPI and trading volume, and the Department of Census and Statistics for inflation." The note records the sample accounting failing: "The counts are 106 for the differenced exchange rate and money supply, 105 for the twice-differenced NCPI, and 107 for log ASPI and log trading volume, none of which is the 108 asserted in the text, and page 127 separately describes the window as 2014 to 2023 while every other statement in the paper says 2022."</t>
         </is>
       </c>
       <c r="J41" s="11" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="N41" s="11" t="inlineStr">
         <is>
-          <t>macro only, no retrieval. Noted disclosure: "ChatGPT and Google assisted in locating credible sources, with the series then manually extracted, mostly from Excel downloads and the inflation data transcribed out of PDFs."</t>
+          <t>macro only, no retrieval. Noted disclosure: "ChatGPT and Google assisted in locating credible sources", with the series then manually extracted, mostly from Excel downloads and the inflation data transcribed out of PDFs.</t>
         </is>
       </c>
       <c r="O41" s="11" t="inlineStr">
@@ -5707,7 +5707,7 @@
       </c>
       <c r="S41" s="11" t="inlineStr">
         <is>
-          <t>"Trading volume unidirectionally Granger-causes the ASPI, p = 0.0041, with no feedback, p = 0.8923." "The exchange rate relationship runs backwards, ASPI to exchange rate at p = 0.0076 and exchange rate to ASPI at p = 0.1603." "Money supply causes nothing in either direction, p = 0.6241 and 0.5403." "Inflation causes nothing either, p = 0.2772 and 0.9649." Lag selection: "lag one was chosen, SC = −32.1528", with "HQIC also minimises at lag one (−32.6066) but AIC minimises at lag four (−33.1968)". ADF: log ASPI −5.0724 p=0.0000, log volume −3.1719 p=0.0217 declared stationary at level. ARCH statistics: exchange rate 42.4551, ASPI 86.5509, volume 70.0659. Exchange rate skewness 5.7245, kurtosis 34.9185. LIMITATIONS (quoting the note): "The ADF result that licences keeping ASPI and volume at level is not credible, and everything downstream inherits it... The paper's own Table 3 contradicts it, reporting a lag-one sample autocorrelation of 0.9273 for log ASPI and 0.8179 for log trading volume... What it means practically is that the two variables in the headline result are probably I(1) and entered untransformed, which puts the volume to ASPI test in spurious-regression territory, and that is the single result the paper's contribution rests on." "The dependent variable is a level and the paper interprets it as a return... This is the same construct-to-proxy slippage that runs through [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]]... and the two papers together are why I now check what a CSE study's dependent variable actually is before reading any of its conclusions." "Mixing I(0), I(1) and I(2) variables in one pairwise testing framework without cointegration analysis breaks the test's asymptotics." "Second-differencing the NCPI changes the hypothesis without the paper noticing." "Lag one forecloses the lag structure the other CSE evidence points at." "The sample is small for the number of regime breaks it spans and there is no subsample analysis."</t>
+          <t>"Trading volume unidirectionally Granger-causes the ASPI, p = 0.0041, with no feedback, p = 0.8923." "The exchange rate relationship runs backwards, ASPI to exchange rate at p = 0.0076 and exchange rate to ASPI at p = 0.1603." "Money supply causes nothing in either direction, p = 0.6241 and 0.5403." "Inflation causes nothing either, p = 0.2772 and 0.9649." Lag selection: "lag one was chosen, SC = −32.1528", with "HQIC also minimises at lag one (−32.6066) but" AIC minimises at lag four (−33.1968). ADF: log ASPI −5.0724 p=0.0000, log volume −3.1719 p=0.0217 declared stationary at level. ARCH statistics: exchange rate 42.4551, ASPI 86.5509, volume 70.0659. Exchange rate skewness 5.7245, kurtosis 34.9185. LIMITATIONS (quoting the note): The ADF result that licences keeping ASPI and volume at level is not credible, and everything downstream inherits it... The paper's own Table 3 contradicts it, reporting a lag-one sample autocorrelation of 0.9273 for log ASPI and 0.8179 for log trading volume... What it means practically is that the two variables in the headline result are probably I(1) and entered untransformed, which puts the volume to ASPI test in spurious-regression territory, and that is the single result the paper's contribution rests on. "The dependent variable is a level and the paper interprets it as a return... This is the same construct-to-proxy slippage that runs through [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]]... and the two papers together are why I now check what a CSE study's dependent variable actually is before reading any of its conclusions." "Mixing I(0), I(1) and I(2) variables in one pairwise testing framework without cointegration analysis breaks the test's asymptotics." "Second-differencing the NCPI changes the hypothesis without the paper noticing." "Lag one forecloses the lag structure the other CSE evidence points at." "The sample is small for the number of regime breaks it spans and there is no subsample analysis."</t>
         </is>
       </c>
       <c r="T41" s="11" t="inlineStr">
@@ -5730,7 +5730,7 @@
           <t>SPEAKS TO: A_L primarily (volume as information-arrival proxy, the domain warrant for L_t), orchestrator (the microstructure-over-macro conditioning argument), evaluation layer (no-holdout pattern).
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap - the strongest domain-literature support in the set for conditioning on microstructure state (volume) rather than macro, which is direct evidence for keeping L_t in f(·) and keeping macro out. Sub-gap 1 - indirect but real: volume is the raw material of a liquidity state variable, and the note commits to re-testing it at daily frequency "with turnover and a spread proxy alongside it, inside the training window only. If it survives that, it earns a place in the conditioning set. If it doesn't, the discrepancy is itself worth reporting, since it would locate the effect at monthly aggregation."
 EFFECT ON SUB-GAP 2: LEAVES IT OPEN, with one relevant contribution in passing. It runs no volatility model, but it finds ARCH effects at p = 0.0000 in the ASPI, volume and exchange rate while finding none in the macro series - the note reads this as "consistent with the market-side series carrying volatility clustering that the level specification doesn't model, and it's the same persistence [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] is about." So it is a third independent CSE observation of volatility clustering that is detected and then discarded (robust standard errors are applied as a nuisance correction, not as a modelled quantity). This is Sub-gap 2 in its most literal form: persistence is measured - here, effectively, as a diagnostic statistic - and used only to adjust standard errors, never to inform a decision.
-CSE DATA EVIDENCE: source - ASPI and trading volume from the Colombo Stock Exchange; money supply (M2b) and USD/LKR from the Central Bank of Sri Lanka; inflation (NCPI, base 2013=100) from the Department of Census and Statistics. Frequency - monthly. Range - 2014 to 2022 (nine years), "108 observations claimed" but descriptive statistics report 107 for log ASPI and log trading volume, 106 for differenced exchange rate and money supply, 105 for twice-differenced NCPI, with page 127 saying 2014 to 2023. Tickers - none; ASPI index plus aggregate market volume in millions of shares. How obtained - "purposive sampling"; the collection section "discloses that ChatGPT and Google assisted in locating credible sources, with the series then manually extracted, mostly from Excel downloads and the inflation data transcribed out of PDFs." Critical reading for the blocker: this is the only one of the three that uses CSE volume at all, and even so it is market-aggregate monthly volume obtained by manual Excel download - no evidence of bulk per-ticker access.
+CSE DATA EVIDENCE: source - ASPI and trading volume from the Colombo Stock Exchange; money supply (M2b) and USD/LKR from the Central Bank of Sri Lanka; inflation (NCPI, base 2013=100) from the Department of Census and Statistics. Frequency - monthly. Range - 2014 to 2022 (nine years), "108 observations claimed" but descriptive statistics report 107 for log ASPI and log trading volume, 106 for differenced exchange rate and money supply, 105 for twice-differenced NCPI, with page 127 saying 2014 to 2023. Tickers - none; ASPI index plus aggregate market volume in millions of shares. How obtained - "purposive sampling"; the collection section discloses that ChatGPT and Google assisted in locating credible sources, with the series then manually extracted, mostly from Excel downloads and the inflation data transcribed out of PDFs. Critical reading for the blocker: this is the only one of the three that uses CSE volume at all, and even so it is market-aggregate monthly volume obtained by manual Excel download - no evidence of bulk per-ticker access.
 PROPOSED REVISION STATED IN THE NOTE: no revision to the agent pool. On the conditioning set, verbatim: "Volume goes into the liquidity state variable, and I re-estimate this properly rather than inheriting it. Log monthly shares traded is far too coarse for anything I'm doing, so what I take is the hypothesis, that volume carries information about near-term returns on this market, to be re-tested at daily frequency on differenced series with turnover and a spread proxy alongside it, inside the training window only. If it survives that, it earns a place in the conditioning set." And on USD/LKR as a feature: "the direction question has to be settled inside my own window before the feature goes in. I'd expect the truth to be regime-dependent here, with the rate leading during the 2022 float and the index leading in calmer stretches, which is exactly the kind of instability a static feature set handles badly and a state-aware orchestrator is supposed to handle."</t>
         </is>
       </c>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>"ASPI values of the twenty sectors plus daily closing prices of nine listed banks, extracted from the CSE database and supplemented with other financial documents, covering 2008 to 2017. The paper reports 2,221 price samples classified into 20 sectors, with missing values and outliers present and removed by preprocessing along with seasonality and trend. An 80/20 train and test split, no validation partition, no rolling origin. The abstract says the selected sector's businesses are analysed over 2013 to 2017 while the data section and the conclusion both say 2008 to 2017, and nothing reconciles the two windows."</t>
+          <t>"ASPI values of the twenty sectors plus daily closing prices of nine listed banks, extracted from the CSE database and supplemented with other financial documents, covering 2008 to 2017. The paper reports" 2,221 price samples classified into 20 sectors, with missing values and outliers present and removed by preprocessing along with seasonality and trend. An 80/20 train and test split, no validation partition, no rolling origin. The abstract says the selected sector's businesses are analysed over 2013 to 2017 while the data section and the conclusion both say 2008 to 2017, and nothing reconciles the two windows.</t>
         </is>
       </c>
       <c r="J42" s="11" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="S42" s="11" t="inlineStr">
         <is>
-          <t>"BPNN beats ARIMA, MAE 4.708423 against 29.6975 and MAPE 0.1783333 against 0.4672206". ARIMA selected at "AIC 71180.553, BIC 71243.107 and HQIC 71202.003". Cluster contributions: "Banks and finance 3.16, Diversified 2.51, Hotels and travels 2.50, IT 2.20, Motors 2.66"; within banks "NTB 1.95, NDB 2.34, Sampath 2.39 and Commercial 2.08" - "Sampath wins by 0.05 on the undefined scale". Note's own recomputation: "A no-change forecast anchored on the previous day's actual gives a mean absolute error of 34.96 over the four days where it can be computed, against 9.23 for ARIMA and 2.90 for BPNN, so unlike [[Stock Price Prediction Using ARIMA Model, Evidence from Colombo Stock Exchange]] this paper's tabulated forecasts do clear the naive baseline. That's the strongest thing in it and the authors don't claim it." MASE on those four days "roughly 0.26 for ARIMA and 0.08 for BPNN". LIMITATIONS (quoting the note): "The two reported metric pairs are internally inconsistent, and neither reproduces from the paper's own Table 4... Recomputing both metrics from the five tabulated days gives MAE 7.886 and MAPE 0.120% for ARIMA and MAE 2.732 and MAPE 0.041% for BPNN, neither of which matches the table." "The error metrics don't reconcile, which puts the central claim out of reach... On this evidence I can't verify the comparison the paper exists to make." "The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes and is roughly thirty years of daily trading rather than ten, so the series the ARIMA was fitted on is not the series the paper describes." "The BPNN plot cannot be the ASPI over 2008 to 2017. Its vertical axis runs from 10,000 to 20,000 while the ASPI traded between roughly 1,500 and 7,800 across that decade." "The clustering stage is not reproducible." "Everything is selected and evaluated on one split with no repetition." "The stationarity handling contradicts itself and probably over-differences." "An investment recommendation with no strategy, no costs and no execution." "The sector recommendation reduces to buying the index."</t>
+          <t>"BPNN beats ARIMA, MAE 4.708423 against 29.6975 and MAPE 0.1783333 against 0.4672206". ARIMA selected at "AIC 71180.553, BIC 71243.107 and HQIC 71202.003". Cluster contributions: "Banks and finance 3.16, Diversified 2.51, Hotels and travels 2.50, IT 2.20, Motors 2.66"; within banks "NTB 1.95, NDB 2.34, Sampath 2.39 and Commercial 2.08" - "Sampath wins by 0.05 on the undefined scale". Note's own recomputation: "A no-change forecast anchored on the previous day's actual gives a mean absolute error of 34.96 over the four days where it can be computed, against 9.23 for ARIMA and 2.90 for BPNN, so unlike [[Stock Price Prediction Using ARIMA Model, Evidence from Colombo Stock Exchange]] this paper's tabulated forecasts do clear the naive baseline. That's the strongest thing in it and the authors don't claim it." MASE on those four days "roughly 0.26 for ARIMA and 0.08 for BPNN". LIMITATIONS (quoting the note): "The two reported metric pairs are internally inconsistent, and neither reproduces from the paper's own Table 4... Recomputing both metrics from the five tabulated days gives MAE 7.886 and MAPE 0.120% for ARIMA and MAE 2.732 and MAPE 0.041% for BPNN, neither of which matches the table." "The error metrics don't reconcile, which puts the central claim out of reach... On this evidence I can't verify the comparison the paper exists to make." The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes and is roughly thirty years of daily trading rather than ten, so the series the ARIMA was fitted on is not the series the paper describes. "The BPNN plot cannot be the ASPI over 2008 to 2017. Its vertical axis runs from 10,000 to 20,000 while the ASPI traded between roughly 1,500 and 7,800 across that decade." "The clustering stage is not reproducible." "Everything is selected and evaluated on one split with no repetition." "The stationarity handling contradicts itself and probably over-differences." "An investment recommendation with no strategy, no costs and no execution." "The sector recommendation reduces to buying the index."</t>
         </is>
       </c>
       <c r="T42" s="11" t="inlineStr">
@@ -5856,7 +5856,7 @@
           <t>SPEAKS TO: A_T (the CSE non-linear price-only baseline the technical agent must beat), orchestrator (the capitalisation-weight warning about counter ranking; the rule that any deciding quantity needs a formula and a dispersion estimate), evaluation layer (horizon/refit columns, MASE).
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap - a concrete warning about the orchestrator's counter-ranking mechanism (rank on forecastable excess return net of costs, not on index contribution) and a demand that any per-agent reliability weight carry a definition and a sensitivity analysis, with a thin margin treated "as a tie rather than a ranking". Sub-gap 1 - indirect: the paper issues a buy recommendation on a market with documented illiquidity shocks of 8 to 10 basis points and models no spread, no fee, no execution, which is the friction blind spot restated on CSE data.
 EFFECT ON SUB-GAP 2: LEAVES IT OPEN and adds a fourth CSE instance of volatility being ignored entirely rather than measured-and-unused. No conditional variance model on a window opening on the 2008 crisis; no ARCH test; no Ljung-Box. Nothing operationalised. Its only Sub-gap-2 contribution is negative corroboration - it is another CSE paper where constant variance is assumed across a decade the vault's other notes establish is strongly heteroskedastic.
-CSE DATA EVIDENCE: source - "extracted from the CSE database and supplemented with other financial documents". Frequency - daily. Range - stated 2008 to 2017 (abstract inconsistently says 2013 to 2017 for the sector analysis). Tickers - this is the only one of the three CSE papers that touches individual counters: "daily closing prices of nine listed banks", of which only four (NTB, NDB, Sampath, Commercial) appear in the results table - "five of the nine banks are missing from the results table". Plus twenty GICS sector series. Volume - "2,221 price samples classified into 20 sectors". How obtained - CSE database, method unspecified. Critical caveat for the blocker: the note establishes the stated dataset is not what was actually fitted - "The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes... so the series the ARIMA was fitted on is not the series the paper describes", and the BPNN plot's axis range is inconsistent with the ASPI over that decade. So this paper claims ten years of daily per-counter CSE bank prices, but its own printouts contradict its data section, and nothing per-ticker (OHLC, volume, turnover) is reported.
+CSE DATA EVIDENCE: source - "extracted from the CSE database and supplemented with other financial documents". Frequency - daily. Range - stated 2008 to 2017 (abstract inconsistently says 2013 to 2017 for the sector analysis). Tickers - this is the only one of the three CSE papers that touches individual counters: "daily closing prices of nine listed banks", of which only four (NTB, NDB, Sampath, Commercial) appear in the results table - "five of the nine banks are missing from the results table". Plus twenty GICS sector series. Volume - "2,221 price samples classified into 20 sectors". How obtained - CSE database, method unspecified. Critical caveat for the blocker: the note establishes the stated dataset is not what was actually fitted - The header reports 7,712 observations, which is more than three times the 2,221 samples the data section describes... so the series the ARIMA was fitted on is not the series the paper describes, and the BPNN plot's axis range is inconsistent with the ASPI over that decade. So this paper claims ten years of daily per-counter CSE bank prices, but its own printouts contradict its data section, and nothing per-ticker (OHLC, volume, turnover) is reported.
 PROPOSED REVISION STATED IN THE NOTE: none to the four-agent pool or to f(L_t, V_t, P_t, C_{i,t}) directly. The nearest statement bears on C_{i,t}'s reporting standard: "Where my orchestrator produces a per-agent reliability weight, the definition goes in the write-up, the sensitivity of the decision to that weight gets reported, and a margin that thin gets treated as a tie rather than a ranking."</t>
         </is>
       </c>
@@ -5909,7 +5909,7 @@
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>"Daily closing values of the CSE Price Index from the official CSE database, cross-checked against Bloomberg historical series, 1 July 2014 to 30 June 2024, giving 2,362 usable observations after differencing and lag adjustment. Everything is run in EViews 13. There is no train and validation split inside the decade, the model is estimated on the whole sample and then forecast forward into July 2024." Test window: 23 trading days, July 2024.</t>
+          <t>Daily closing values of the CSE Price Index from the official CSE database, cross-checked against Bloomberg historical series, 1 July 2014 to 30 June 2024, giving 2,362 usable observations after differencing and lag adjustment. "Everything is run in EViews 13. There is no train and validation split inside the decade, the model is estimated on the whole sample and then forecast forward into July 2024." Test window: 23 trading days, July 2024.</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>ADF under three specifications (intercept; trend and intercept; none), d=1 settled. Eight candidate ARMA orders compared on AIC, SBIC, adjusted R², σ², standard error.  named ARIMA(2,1,1), actually a subset specification: Δy_t = μ + φ₂(Δy_{t-2} − μ) + ε_t + θ₁ε_{t-1}, with μ = 2.445160 (t = 1.072697, p = 0.2835), φ₂ = −0.038071 (t = −4.178964), no φ₁, θ₁ = 0.301976 (t = 37.81713). "The printed inverted AR roots of −0.00 ± 0.20i confirm this... It is a defensible model, gap ARMA specifications are a normal thing to fit, but it is called ARIMA(2,1,1) in the title, the abstract, every table caption and the conclusion, and anyone reimplementing from the paper builds the wrong thing."</t>
+          <t>ADF under three specifications (intercept; trend and intercept; none), d=1 settled. Eight candidate ARMA orders compared on AIC, SBIC, adjusted R², σ², standard error. named ARIMA(2,1,1), actually a subset specification: Δy_t = μ + φ₂(Δy_{t-2} − μ) + ε_t + θ₁ε_{t-1}, with μ = 2.445160 (t = 1.072697, p = 0.2835), φ₂ = −0.038071 (t = −4.178964), no φ₁, θ₁ = 0.301976 (t = 37.81713). The printed inverted AR roots of −0.00 ± 0.20i confirm this... It is a defensible model, gap ARMA specifications are a normal thing to fit, but it is called ARIMA(2,1,1) in the title, the abstract, every table caption and the conclusion, and anyone reimplementing from the paper builds the wrong thing.</t>
         </is>
       </c>
       <c r="L43" s="11" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="S43" s="11" t="inlineStr">
         <is>
-          <t>reported "MAPE of 3.9% and therefore strong short-term forecasting performance". Model selection: "ARMA(2,1) wins at AIC 11.64805 against ARMA(1,1) at 11.64806, a difference of 0.00001 in EViews' per-observation units, which on 2,362 observations is 0.024 absolute AIC units, far inside the range where the two models are indistinguishable." Fit: "R² = 0.083698 falling to an adjusted 0.082532". Forecast degeneracy: "the day-on-day increments run 3.240, 2.337, 2.415, 2.449, 2.446 and then settle at 2.44516 for every remaining day, which is μ = 2.445160 to five decimals. So the entire three-month forecast path is generated by a drift term the paper's own Table 3 reports as insignificant at p = 0.2835." Direction: "Predictions rise 54.45 points across the 23 trading days while the index fell 669.93 points, from 12,076.49 to 11,406.56, a decline of 5.55%." Note's recomputation: "A no-change forecast beats it on every day of the test window... a mean absolute percentage error of 2.57% for the random walk against 3.62% for the ARIMA, RMSE of 346.10 against 465.40, and the random walk is closer to the actual on 23 of 23 days." Theil U2 on Table 4: "1.345". LIMITATIONS (quoting the note): "Two claims in this paper are contradicted by its own tables." "The white noise conclusion is contradicted by the printed correlogram... Figure 3 reports p = 0.039 at lag 3, p = 0.001 at lag 4, and p = 0.000 continuously from lag 5 to lag 36, ending at Q(36) = 185.20... The Box-Jenkins adequacy criterion is failed and reported as passed, which means the model was never actually validated and the significance of the AR and MA terms cannot be taken at face value either." "MA(1) at 0.301976 carries almost all of the fit, and its standard error of 0.007985 is implausibly small." "One forecast origin, no benchmark, no rolling evaluation." "Three of the literature review's supporting citations do not say what they are cited for, and a fourth has no reference at all." "Univariate and index-level throughout, which the authors acknowledge."</t>
+          <t>reported "MAPE of 3.9% and therefore strong short-term forecasting performance". Model selection: "ARMA(2,1) wins at AIC 11.64805 against ARMA(1,1) at 11.64806, a difference of 0.00001 in EViews' per-observation units, which on 2,362 observations is" 0.024 absolute AIC units, far inside the range where the two models are indistinguishable. Fit: R² = "0.083698 falling to an adjusted 0.082532". Forecast degeneracy: "the day-on-day increments run 3.240, 2.337, 2.415, 2.449, 2.446 and then settle at" 2.44516 for every remaining day, which is μ = 2.445160 to five decimals. So the entire three-month forecast path is generated by a drift term the paper's own Table 3 reports as insignificant at p = 0.2835. Direction: "Predictions rise 54.45 points across the 23 trading days while the index fell 669.93 points, from 12,076.49 to 11,406.56, a decline of 5.55%." Note's recomputation: A no-change forecast beats it on every day of the test window... a mean absolute percentage error of 2.57% for the random walk against 3.62% for the ARIMA, RMSE of 346.10 against 465.40, and the random walk is closer to the actual on 23 of 23 days. Theil U2 on Table 4: "1.345". LIMITATIONS (quoting the note): "Two claims in this paper are contradicted by its own tables." "The white noise conclusion is contradicted by the printed correlogram... Figure 3 reports p = 0.039 at lag 3, p = 0.001 at lag 4, and p = 0.000 continuously from lag 5 to lag 36, ending at Q(36) = 185.20... The Box-Jenkins adequacy criterion is failed and reported as passed", which means the model was never actually validated and the significance of the AR and MA terms cannot be taken at face value either. "MA(1) at 0.301976 carries almost all of the fit, and its standard error of 0.007985 is implausibly small." "One forecast origin, no benchmark, no rolling evaluation." "Three of the literature review's supporting citations do not say what they are cited for, and a fourth has no reference at all." "Univariate and index-level throughout, which the authors acknowledge."</t>
         </is>
       </c>
       <c r="T43" s="11" t="inlineStr">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="U43" s="11" t="inlineStr">
         <is>
-          <t>"This is my benchmark-discipline citation, and the cleanest one I have. A published 2026 journal paper reports strong short-term forecasting performance from a forecast that loses to a no-change baseline on 23 of 23 days, and the entire gap between those two readings is one line of arithmetic the paper never ran." U2 = sqrt( Σ(y−ŷ)² / Σ(y − y_T)² ) reported per counter, "and the same quantity is what decides whether the price-derived agent gets any weight at all on a given day". "The drift-collapse is a design constraint on the technical agent, not just a criticism of this paper. Any multi-step forecast from a low-order ARIMA degenerates to a drift line within a handful of steps, so a price-only agent has real information at a one to three day horizon and essentially none beyond it. That sets the rebalancing frequency my orchestrator can meaningfully condition price signals at." "The ARIMA baseline I build gets AR(1) included and the residuals actually tested." "The residual plot in this paper is my third independent CSE reading of volatility clustering, and it strengthens the case for the persistence layer." "The 8% in-sample R² is a useful floor to state honestly... a technical agent reporting far more than this on CSE daily data is more likely to have a leakage problem than a discovery." "The efficiency framing is worth borrowing and the inference is not."</t>
+          <t>"This is my benchmark-discipline citation, and the cleanest one I have. A published 2026 journal paper reports strong short-term forecasting performance from a forecast that loses to a no-change baseline on 23 of 23 days, and the entire gap between those two readings is one line of arithmetic the paper never ran." U2 = sqrt(Σ(y−ŷ)² / Σ(y − y_T)²) reported per counter, "and the same quantity is what decides whether the price-derived agent gets any weight at all on a given day". "The drift-collapse is a design constraint on the technical agent, not just a criticism of this paper. Any multi-step forecast from a low-order ARIMA degenerates to a drift line within a handful of steps, so a price-only agent has real information at a one to three day horizon and essentially none beyond it. That sets the rebalancing frequency my orchestrator can meaningfully condition price signals at." "The ARIMA baseline I build gets AR(1) included and the residuals actually tested." "The residual plot in this paper is my third independent CSE reading of volatility clustering, and it strengthens the case for the persistence layer." The 8% in-sample R² is a useful floor to state honestly... a technical agent reporting far more than this on CSE daily data is more likely to have a leakage problem than a discovery. "The efficiency framing is worth borrowing and the inference is not."</t>
         </is>
       </c>
       <c r="V43" s="11" t="inlineStr">
@@ -5983,7 +5983,7 @@
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap - one concrete design constraint on the orchestrator: the drift collapse caps the horizon at which A_T carries information ("one to three day horizon and essentially none beyond it"), which sets the rebalancing frequency at which price signals can meaningfully be conditioned, and U2 becomes "what decides whether the price-derived agent gets any weight at all on a given day" - i.e. a usable per-day competence input to C_{A_T,t}. Sub-gap 1 - bearing via the friction argument: "a 3.8 point conditional offset on an 81.7 point daily sigma is well inside the friction", which is a concrete CSE-calibrated demonstration that a statistically significant edge can be smaller than the execution cost, and the note commits to attaching a net-of-cost return "using the liquidity-aware slippage model rather than a flat fee".
 EFFECT ON SUB-GAP 2: NARROWS IT SLIGHTLY, by supplying a third independent CSE observation that persistence is there and is being ignored - and by producing the clearest statement in the set of why that matters operationally. The paper measures nothing about volatility; it fits constant variance and its own residual plot shows bands widening by a factor of several across 2020–2022. The note converts this into an argument for the persistence layer: "The residual plot in this paper is my third independent CSE reading of volatility clustering, and it strengthens the case for the persistence layer. Fitted with constant variance and still showing residual bands widening by a factor of several across 2020 to 2022, it lines up with the near-unit persistence in the ARMA-GARCH note and the fractional integration in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]. Three papers, three different specifications, same signal, so conditioning exposure on forecast variance and decay speed rather than on a fixed risk parameter is supported by the local evidence rather than imported from elsewhere." That last clause is the important one for Sub-gap 2: it establishes local evidentiary support for conditioning exposure on decay speed, without the paper itself doing any of it.
 CSE DATA EVIDENCE: source - "the official CSE database, cross-checked against Bloomberg historical series". Frequency - daily. Range - 1 July 2014 to 30 June 2024, ten years, "2,362 usable observations after differencing and lag adjustment", plus a 23-day July 2024 out-of-sample window. Tickers - none; CSE Price Index only, "no individual counters". How obtained - CSE official database with Bloomberg cross-check; tooling EViews 13. This is the longest confirmed clean CSE daily series in the set, and it is index-level. The regime content is documented: "July 2014 to June 2024 deliberately contains the 2019 Easter Sunday attacks, the COVID-19 lockdown low of 4,247.95, the speculative peak of 13,462.39 in January 2022, and the 2022 forex and sovereign crisis."
-PROPOSED REVISION STATED IN THE NOTE: no change to the agent pool. On the conditioning set and on C_{i,t}, verbatim: "Every forecasting number my system reports gets this alongside it, computed per counter, and the same quantity is what decides whether the price-derived agent gets any weight at all on a given day." Also a constraint on the orchestrator's operating frequency: "That sets the rebalancing frequency my orchestrator can meaningfully condition price signals at, and it means multi-day forecast horizons from the technical agent should be produced one step at a time against realised data rather than dynamically."</t>
+PROPOSED REVISION STATED IN THE NOTE: no change to the agent pool. On the conditioning set and on C_{i,t}, verbatim: "Every forecasting number my system reports gets this alongside it, computed per counter, and" the same quantity is what decides whether the price-derived agent gets any weight at all on a given day. Also a constraint on the orchestrator's operating frequency: "That sets the rebalancing frequency my orchestrator can meaningfully condition price signals at, and it means multi-day forecast horizons from the technical agent should be produced one step at a time against realised data rather than dynamically."</t>
         </is>
       </c>
       <c r="X43" s="11" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>"Daily-rebalanced long-only allocation across four index ETFs, where the entire contribution is that the Sharpe ratio is the training objective itself rather than a metric computed after a forecaster has been fitted, so the network maps raw price and return history to portfolio weights in one differentiable pass and is updated by gradient ascent on realised portfolio Sharpe."</t>
+          <t>Daily-rebalanced long-only allocation across four index ETFs, where the entire contribution is that the Sharpe ratio is the training objective itself "rather than a metric computed after a forecaster has been fitted, so the network maps raw price and return history to portfolio weights in one differentiable pass and is updated by gradient ascent on realised portfolio Sharpe."</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -6070,7 +6070,7 @@
       </c>
       <c r="P44" s="11" t="inlineStr">
         <is>
-          <t>a flat proportional cost C charged on post-scaling turnover, swept at two values (C = 0.01% and C = 0.1%). No spread, no depth, no impact, no partial fill. The note: "The execution-friction blind spot is not so much unaddressed here as designed out of the experiment, which is now the third portfolio paper I have written that sentence about, though this one at least sweeps the rate." Also flags an unresolved instrument question: "The volatility instrument is named as an index and never as a tradable ticker... There is no instrument that tracks spot VIX, and the ETPs that approximate it hold futures and carry roll costs that dwarf the one to ten basis points charged here."</t>
+          <t>a flat proportional cost C charged on post-scaling turnover, swept at two values (C = 0.01% and C = 0.1%). No spread, no depth, no impact, no partial fill. The note: "The execution-friction blind spot is not so much unaddressed here as designed out of the experiment", which is now the third portfolio paper I have written that sentence about, though this one at least sweeps the rate. Also flags an unresolved instrument question: "The volatility instrument is named as an index and never as a tradable ticker... There is no instrument that tracks spot VIX, and the ETPs that approximate it hold futures and carry roll costs that dwarf the one to ten basis points charged here."</t>
         </is>
       </c>
       <c r="Q44" s="11" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="S44" s="11" t="inlineStr">
         <is>
-          <t>"Without scaling at C = 0.01% it reaches Sharpe 1.858 and Sortino 3.135 against Allocation 4's 1.228 and 2.932, with scaling at the same rate 1.962 and 3.322 against 1.579 and 2.629, and with scaling at C = 0.1% 1.403 and 2.327 against Allocation 4's 1.299 and 2.172. So a tenfold increase in the cost rate takes the Sharpe advantage from roughly 24% over the best baseline down to 8%." Win profile: "DLS never has the highest percentage of positive returns in any of the three blocks, 0.537 against MV's 0.562, 0.559 against the 0.565 held jointly by Allocation 4 and MD and 0.547 against Allocation 4's 0.559, but it has the highest average-gain-to-average-loss ratio in all three, 1.518, 1.375 and 1.272." Scaler attribution: "Allocation 1 goes from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120 purely from the scaler, against DLS's 1.858 to 1.962." Drawdown: "in the scaled block DLS records an MDD of 0.123, fifth of eight... and at C = 0.1% it is fifth again at 0.125, so for a method whose stated appeal is the confidence to hold through hard times it is mid-table on the one metric that measures holding through hard times." Cost collapse: "DWP posts Sharpe 0.493 unscaled, 0.818 scaled, and −0.753 at C = 0.1% with an MDD of 0.627 and an expected return of −0.083." LIMITATIONS (quoting the note): "There is no seed averaging, no walk-forward significance testing and no reported hyperparameter search, and the paper frames the last of these as a virtue... Every number in Table 1 is one training run of one architecture on one fixed sequence." "The test window is a bull market and the single crisis in it is handled by a component that was not trained... I cannot say the learned policy handles regime change, because the design does not separate the policy's contribution from the scaler's. An unscaled run through Q1 2020 would have answered it and is not reported." "How L_T is computed during training is never stated, and it changes what the model optimises... A Sharpe estimated over 64 daily observations is an extremely noisy quantity... this is a reproducibility hole sitting directly on the paper's single contribution." "The cost model is flat and proportional, and the asset choice removes execution friction from the problem by construction." "The architecture claims and the RL framing are both asserted without a baseline."</t>
+          <t>"Without scaling at C = 0.01% it reaches Sharpe 1.858 and Sortino 3.135 against Allocation 4's 1.228 and 2.932, with scaling at the same rate 1.962 and 3.322 against" 1.579 and 2.629, and with scaling at C = 0.1% 1.403 and 2.327 against Allocation 4's 1.299 and 2.172. So a tenfold increase in the cost rate takes the Sharpe advantage from roughly 24% over the best baseline down to 8%. Win profile: "DLS never has the highest percentage of positive returns in any of the three blocks, 0.537 against MV's 0.562, 0.559 against the 0.565 held jointly by Allocation 4 and MD and 0.547 against Allocation 4's 0.559, but it has the highest average-gain-to-average-loss ratio in all three, 1.518, 1.375 and 1.272." Scaler attribution: "Allocation 1 goes from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120 purely from the scaler, against DLS's 1.858 to 1.962." Drawdown: in the scaled block DLS records an MDD of 0.123, fifth of eight... and at C = 0.1% it is fifth again at 0.125, so for a method whose stated appeal is the confidence to hold through hard times it is mid-table on the one metric that measures holding through hard times. Cost collapse: "DWP posts Sharpe 0.493 unscaled, 0.818 scaled, and −0.753 at C = 0.1% with an MDD of 0.627 and an expected return of −0.083." LIMITATIONS (quoting the note): "There is no seed averaging, no walk-forward significance testing and no reported hyperparameter search, and the paper frames the last of these as a virtue... Every number in Table 1 is one training run of one architecture on one fixed sequence." "The test window is a bull market and the single crisis in it is handled by a component that was not trained... I cannot say the learned policy handles regime change, because the design does not separate the policy's contribution from the scaler's. An unscaled run through Q1 2020 would have answered it and is not reported." "How L_T is computed during training is never stated, and it changes what the model optimises... A Sharpe estimated over 64 daily observations is an extremely noisy quantity... this is a reproducibility hole sitting directly on the paper's single contribution." "The cost model is flat and proportional, and the asset choice removes execution friction from the problem by construction." "The architecture claims and the RL framing are both asserted without a baseline."</t>
         </is>
       </c>
       <c r="T44" s="11" t="inlineStr">
@@ -6107,7 +6107,7 @@
         <is>
           <t>SPEAKS TO: A_V above all (the volatility scaler is the component Sub-gap 2 corrects), plus orchestrator (the conditioned-objective framing, the sensitivity diagnostic) and evaluation layer (cost sweep, baseline table).
 EFFECT ON MAIN GAP / SUB-GAP 1: main gap - substantial. It gives the orchestration contribution its cheapest possible framing ("a conditioned objective inside a known training scheme rather than a new architecture"), supplies the differentiable slot where liquidity and persistence terms attach, and provides the sensitivity measure S_i as a diagnostic that a mechanism sold as adaptive is actually varying. It is also the designated ablation control - "if a four-agent orchestrator cannot beat a plain differentiable Sharpe maximiser on the same universe and the same costs, that is something I want to find in my own ablation rather than in a viva." Sub-gap 1 - direct and important. The cost sweep (1 bps vs 10 bps) nearly inverts the ranking, and the note draws the CSE conclusion: "at a CSE-plausible round-trip cost the daily-rebalanced version of this design is probably dominated by an annual reallocation rule. Two responses follow, rebalance less often and treat the frequency as a searched parameter rather than a fixed daily choice, or bring the cost term inside the objective using the closed-form transaction remainder factor from Guo et al. so the optimiser trades off predicted return against cost rather than paying it afterwards." The four-paper cost comparison table (Zhang 1/10 bps swept; FreQuant 33/40 bps unswept; Guo 5 bps unswept; Kashif &amp; Ślepaczuk 2 bps unswept) is the note's positioning device for Sub-gap 1: "the only paper that varies its cost assumption is the one with the crudest cost model, which is the gap my own protocol sits in."
-EFFECT ON SUB-GAP 2: THIS IS THE ONE PAPER IN THE SET THAT OPERATIONALISES A VOLATILITY ESTIMATE INTO AN ALLOCATION, AND IT MUST BE FLAGGED PROMINENTLY. Mechanism: every position is multiplied by σ_tgt/σ_{i,t-1}, σ_tgt = 0.10, σ_{i,t-1} an exponentially weighted moving standard deviation over a 50-day window of daily returns; the scaled position is what is traded, what is costed, and what generates turnover. Empirically it is doing most of the risk work - it lifts Allocation 1 from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120, and it, not the learned policy, produced the COVID de-risking. So the paper CLOSES the weaker version of Sub-gap 2 ("a volatility estimate is never fed into a decision") outright, and thereby FORCES the sub-gap into its narrower, defensible form. What it leaves open is exactly the persistence dimension: the estimator is EWMA, "An EWMA estimator assumes shocks decay exponentially, which is precisely the assumption the long-memory result in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] contradicts for the CSE, and the consequence is concrete: after a shock the scaler re-levers on a schedule that is too fast, so exposure returns while the shock is still decaying hyperbolically." The note's proposed correction is the sub-gap in mechanism form: "Pairing a forecast conditional variance with a persistence estimate to set a decay schedule on the scaling ratio is an answer to their stated future work and is testable on their own four-ETF setup before I touch CSE data at all." The authors themselves concede the opening: their conclusion "notes that these volatility estimates are lagged and do not necessarily represent current market volatilities, proposing to infer forward volatility inside the network as future work." So: level of volatility → operationalised. Persistence/decay speed of volatility → still not operationalised, and now with a named component to attach it to and a testbed to test it on.
+EFFECT ON SUB-GAP 2: THIS IS THE ONE PAPER IN THE SET THAT OPERATIONALISES A VOLATILITY ESTIMATE INTO AN ALLOCATION, AND IT MUST BE FLAGGED PROMINENTLY. Mechanism: every position is multiplied by σ_tgt/σ_{i,t-1}, σ_tgt = 0.10, σ_{i,t-1} an exponentially weighted moving standard deviation over a 50-day window of daily returns; the scaled position is what is traded, what is costed, and what generates turnover. Empirically it is doing most of the risk work - it lifts Allocation 1 from Sharpe 0.929 to 1.526 and MV from 0.759 to 1.120, and it, not the learned policy, produced the COVID de-risking. So the paper CLOSES the weaker version of Sub-gap 2 (a volatility estimate is never fed into a decision) outright, and thereby FORCES the sub-gap into its narrower, defensible form. What it leaves open is exactly the persistence dimension: the estimator is EWMA, "An EWMA estimator assumes shocks decay exponentially, which is precisely the assumption the long-memory result in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] contradicts for the CSE, and the consequence is concrete: after a shock the scaler re-levers on a schedule that is too fast, so exposure returns while the shock is still decaying hyperbolically." The note's proposed correction is the sub-gap in mechanism form: "Pairing a forecast conditional variance with a persistence estimate to set a decay schedule on the scaling ratio is an answer to their stated future work and is testable on their own four-ETF setup before I touch CSE data at all." The authors themselves concede the opening: their conclusion "notes that these volatility estimates are lagged and do not necessarily represent current market volatilities, proposing to infer forward volatility inside the network as future work." So: level of volatility → operationalised. Persistence/decay speed of volatility → still not operationalised, and now with a named component to attach it to and a testbed to test it on.
 CSE DATA EVIDENCE: not a CSE paper, but it carries the most direct statement about the data blocker in the set: "A single 64-unit LSTM over a 400-dimensional input with a softmax head and no reward engineering, no replay buffer and no critic is the smallest end-to-end allocator I have found, which matters directly given that the only confirmed ready-made CSE set covers roughly a year of daily data." Also: "on a roughly 240-day CSE sample a shorter window is doubly attractive because it also increases the number of usable training observations." And a scoping caveat: "the CSE has no liquid commodity ETF, no volatility index and a government bond market that is not accessible on the same terms. What is tradable is equities plus cash, so the diversification has to come from counter and sector selection inside one asset class, which is the correlated case the paper explicitly says to avoid."
 PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On the conditioning set / objective, verbatim: "a term that penalises exposure as a function of measured illiquidity, and a term that decays permitted exposure according to forecast variance and persistence together, are both differentiable functions of realised returns and observable state. Framed that way my contribution is a conditioned objective inside a known training scheme rather than a new architecture." And on P_t and V_t jointly: "Pairing a forecast conditional variance with a persistence estimate to set a decay schedule on the scaling ratio is an answer to their stated future work and is testable on their own four-ETF setup before I touch CSE data at all." Plus an open parameter item: "Pinning the smallest window that still gives a stable volatility estimate is the same open item already sitting against SEMA's (w, d) pair from Guo et al., so the two resolve in one experiment."</t>
         </is>
@@ -6151,7 +6151,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>"LSTM networks applied to directional prediction on the full S&amp;P 500 constituent universe from December 1992 to October 2015, framed as statistical arbitrage rather than as forecasting, where the model takes a single feature, the standardised one-day return, over a 240-day sequence and outputs the probability that a stock beats the cross-sectional median return tomorrow." The note's positioning: "this learns a ranking signal and hands it to a fixed mechanical trading rule, which is exactly the shape of A_T feeding an orchestrator, so I am reading it as a specification for that one agent rather than as a competitor architecture."</t>
+          <t>"LSTM networks applied to directional prediction on the full S&amp;P 500 constituent universe from December 1992 to October 2015, framed as statistical arbitrage rather than as forecasting, where the model takes" a single feature, the standardised one-day return, over a 240-day sequence and outputs the probability that a stock beats the cross-sectional median return tomorrow. The note's positioning: "this learns a ranking signal and hands it to a fixed mechanical trading rule, which is exactly the shape of A_T feeding an orchestrator, so I am reading it as a specification for that one agent rather than as a competitor architecture."</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="P45" s="3" t="inlineStr">
         <is>
-          <t>cost is "5 basis points per half-turn", flat, "with no size or depth term, on a universe chosen for being the 500 largest US stocks. No spread, no depth, no impact and no partial fill anywhere." The note: "This is the same execution-friction blind spot I have written into every trading paper in the vault so far, with the difference that this one at least measures the VWAP haircut, so the friction is observed even though it is never modelled." The execution ladder is the measurement: daily close → daily VWAP → weekly close → weekly VWAP → weekly with a day's wait. Microstructure contamination is acknowledged by the authors: "buying recent losers means buying stocks more likely to be quoted at the ask and selling recent winners more likely to be quoted at the bid, so part of the measured return is bid-ask bounce."</t>
+          <t>cost is "5 basis points per half-turn", flat, "with no size or depth term, on a universe chosen for being the 500 largest US stocks. No spread, no depth, no impact and no partial fill anywhere." The note: "This is the same execution-friction blind spot I have written into every trading paper in the vault so far", with the difference that this one at least measures the VWAP haircut, so the friction is observed even though it is never modelled. The execution ladder is the measurement: daily close → daily VWAP → weekly close → weekly VWAP → weekly with a day's wait. Microstructure contamination is acknowledged by the authors: buying recent losers means buying stocks more likely to be quoted at the ask and selling recent winners more likely to be quoted "at the bid, so part of the measured return is bid-ask bounce."</t>
         </is>
       </c>
       <c r="Q45" s="3" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="S45" s="3" t="inlineStr">
         <is>
-          <t>"Before costs, 0.46 percent per day against 0.43, 0.32 and 0.26 for the random forest, the deep net and the logistic regression, at standard deviations of 2.09 against 2.15, 2.62 and 2.69, giving annualised Sharpe ratios of 5.83, 5.00, 2.43 and 1.70 and accuracies of 54.3, 53.8, 53.7 and 52.2 percent. After 5 basis points per half-turn those returns become 0.26, 0.23, 0.12 and 0.06, so costs remove 43 percent of the LSTM's gross return." The formal test is marginal: "the Diebold-Mariano p-value for the null that the LSTM's forecasts are inferior to the random forest's coming in at 0.0143 against a Bonferroni-adjusted threshold of 1.67 percent". Ranking-depth reversal: "Daily returns fall monotonically from 0.46 percent at k=10 to 0.10 percent at k=200 and the Sharpe ratio from 5.83 to 3.30, but the random forest decays more slowly and takes the Sharpe lead at k=150 with 3.82 against 3.68, holding it at k=200 with 3.58 against 3.30." Era instability: "From 1993 to 2000 the LSTM is superior in almost all years, cumulative payouts on a 1 USD average daily investment reaching roughly 11 USD against the random forest's 8. From 2001 to 2009 the two run together until the crisis, where the random forest posts close to 0.9 percent per day in 2008 against the LSTM's 0.15 and finishes the era at 5.6 USD against 4. From 2010 to 2015 the LSTM oscillates around zero while the random forest goes strictly negative to roughly −1.2 USD." Selection profile: "Top k=10 stocks enter the trade on a five-day cumulative return of −4.05 percent against the flop stocks' +4.54 and a cross-sectional mean of +0.26". Factor regression: "an intercept of 0.42 percent per day at an R² of 0.0330 with significant loadings on short-term reversal at 0.3792 and momentum at −0.1241, against the random forest's 0.34 percent at an R² of 0.1338". Transparent rule: "yields 0.23 percent per day before costs, roughly 50 percent of the LSTM's, and loses its edge entirely after costs." Execution ladder: "the daily close-execution baseline returns 0.20 percent per day after costs at 53.76 percent annualised. Executing on volume-weighted average prices instead drops it to 0.16 percent and 42.87 percent, a weekly close variant to 0.11 percent, a weekly VWAP variant to 0.09 percent, and a weekly variant with a full day of waiting between signal and execution to 0.09 percent at 20.52 percent annualised... the ladder from 53.76 to 20.52 percent annualised is the size of the gap between a close-price backtest and something closer to implementable, on the most liquid equity market in the world." LIMITATIONS (quoting the note): "The cost model is a flat 5 basis points per half-turn with no size or depth term." "The signal's core is short-term reversal, which is partly a microstructure artefact, and the tests bound the problem without resolving it... survival on a universe with penny spreads bounds nothing about a market where the spread is a meaningful fraction of the daily move." "Everything is one run and the crucial comparison is marginal... the defensible statement is that the two methods are close and the ordering depends on the slice, not that the LSTM is the better model." "Nothing conditions on market state, and Figure 5 is the bill for that... the paper observes its own signal decaying to zero after 2010 and its benchmark going strictly negative with no channel through which either observation could change behaviour... it is simultaneously a description of a system that cannot respond to its own deterioration." "The probability output is used ordinally and never checked for calibration... no reliability diagram, no Brier score... Since I want to use exactly this kind of score as an agent confidence input, the absence is worth naming as an open question." "The cross-sectional median target assumes a dense, simultaneously priced cross-section... It degrades quietly rather than loudly when it does."</t>
+          <t>"Before costs, 0.46 percent per day against 0.43, 0.32 and 0.26 for the random forest, the deep net and the logistic regression, at standard deviations of 2.09 against 2.15, 2.62 and 2.69, giving annualised Sharpe ratios of 5.83, 5.00, 2.43 and 1.70 and accuracies of 54.3, 53.8, 53.7 and 52.2 percent. After 5 basis points per half-turn those returns become 0.26, 0.23, 0.12 and 0.06, so" costs remove 43 percent of the LSTM's gross return. The formal test is marginal: "the Diebold-Mariano p-value for the null that the LSTM's forecasts are inferior to the random forest's coming in at 0.0143 against a Bonferroni-adjusted threshold of 1.67 percent". Ranking-depth reversal: "Daily returns fall monotonically from 0.46 percent at k=10 to 0.10 percent at k=200 and the Sharpe ratio from 5.83 to 3.30, but the random forest decays more slowly and takes the Sharpe lead at k=150 with 3.82 against 3.68, holding it at k=200 with 3.58 against 3.30." Era instability: "From 1993 to 2000 the LSTM is superior in almost all years, cumulative payouts on a 1 USD average daily investment reaching roughly 11 USD against the random forest's 8. From 2001 to 2009 the two run together until the crisis, where the random forest posts close to 0.9 percent per day in 2008 against the LSTM's 0.15 and finishes the era at 5.6 USD against 4. From 2010 to 2015 the LSTM oscillates around zero while the random forest goes strictly negative to roughly −1.2 USD." Selection profile: "Top k=10 stocks enter the trade on a five-day cumulative return of −4.05 percent against the flop stocks' +4.54 and a cross-sectional mean of +0.26". Factor regression: an intercept of 0.42 percent per day at an R² of 0.0330 with significant loadings on short-term reversal at 0.3792 and momentum at −0.1241, against the random forest's 0.34 percent at an R² of 0.1338. Transparent rule: "yields 0.23 percent per day before costs, roughly 50 percent of the LSTM's, and loses its edge entirely after costs." Execution ladder: the daily close-execution baseline returns 0.20 percent per day after costs at 53.76 percent annualised. Executing on volume-weighted average prices instead drops it to 0.16 percent and 42.87 percent, a weekly close variant to 0.11 percent, a weekly VWAP variant to 0.09 "percent, and a weekly variant with a full day of waiting between signal and execution to 0.09 percent at 20.52 percent annualised... the ladder from 53.76 to 20.52 percent annualised is the size of the gap between a close-price backtest and something closer to implementable", on the most liquid equity market in the world. LIMITATIONS (quoting the note): "The cost model is a flat 5 basis points per half-turn with no size or depth term." "The signal's core is short-term reversal, which is partly a microstructure artefact, and the tests bound the problem without resolving it... survival on a universe with penny spreads bounds nothing about a market where the spread is a meaningful fraction of the daily move." "Everything is one run and the crucial comparison is marginal... the defensible statement is that the two methods are close and the ordering depends on the slice, not that the LSTM is the better model." "Nothing conditions on market state, and Figure 5 is the bill for that... the paper observes its own signal decaying to zero after 2010 and its benchmark going strictly negative with no channel through which either observation could change behaviour... it is simultaneously a description of a system that cannot respond to its own deterioration." "The probability output is used ordinally and never checked for calibration... no reliability diagram, no Brier score... Since I want to use exactly this kind of score as an agent confidence input, the absence is worth naming as an open question." "The cross-sectional median target assumes a dense, simultaneously priced cross-section... It degrades quietly rather than loudly when it does."</t>
         </is>
       </c>
       <c r="T45" s="3" t="inlineStr">
@@ -6232,9 +6232,9 @@
       <c r="W45" s="3" t="inlineStr">
         <is>
           <t>SPEAKS TO: A_T (this is the specification for the technical agent), orchestrator (Figure 5 is the main gap's empirical exhibit; C_{A_T,t} design), A_L and A_V (the selection-bias argument for why they are agents rather than post-processing), evaluation layer (the execution ladder).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap - this is the strongest published evidence in the set. "Figure 5 is the best single piece of published evidence I have for the main gap, and I should cite it as such. Two heterogeneous predictors trained on identical data, one winning 1993 to 2000, the other winning decisively through 2008, the first winning again 2010 to 2015 by virtue of losing less, with no mechanism anywhere in the design to shift weight between them. A static equal blend would have been beaten by one of its own members in each of the three eras, and a state-conditional blend is exactly what my orchestrator is. This is stronger than the FinAgent and AlphaAgents cases I have been leaning on, because those are failures of a component that should have been switched off, whereas here both components are genuinely useful and the useful one changes." It also dictates evaluation shape: "report the three-way weighting comparison per era or per volatility regime, not only in aggregate, since an aggregate hides exactly this pattern." Sub-gap 1 - strong bearing. The k-depth reversal locates the edge "concentrated in the extreme tails of its own ranking, which is precisely where a thin market cannot absorb the trade". The execution ladder quantifies what realism costs on the most liquid market in the world (53.76 → 20.52 percent annualised), and the note adapts it: the one-day-waiting variant becomes "the cheap test for whether an apparent reversal signal is bid-ask bounce... a validity check rather than a robustness afterthought", with the VWAP leg conditional on intraday CSE data that has not been confirmed to exist. And the selection bias makes liquidity a constraint on the agent rather than a downstream cost: "the liquidity channel is not only a cost model downstream of the decision, it is a constraint on the technical agent's selection, one measurement serving both."
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - this is the strongest published evidence in the set. "Figure 5 is the best single piece of published evidence I have for the main gap, and I should cite it as such. Two heterogeneous predictors trained on identical data, one winning 1993 to 2000, the other winning decisively through 2008, the first winning again 2010 to 2015 by virtue of losing less, with no mechanism anywhere in the design to shift weight between them. A static equal blend would have been beaten by one of its own members in each of the three eras, and a state-conditional blend is exactly what my orchestrator is. This is stronger than the FinAgent and AlphaAgents cases I have been leaning on, because those are failures of a component that should have been switched off, whereas here both components are genuinely useful and the useful one changes." It also dictates evaluation shape: "report the three-way weighting comparison per era or per volatility regime, not only in aggregate, since an aggregate hides exactly this pattern." Sub-gap 1 - strong bearing. The k-depth reversal locates the edge concentrated in the extreme tails of its own ranking, which "is precisely where a thin market cannot absorb the trade". The execution ladder quantifies what realism costs on the most liquid market in the world (53.76 → 20.52 percent annualised), and the note adapts it: the one-day-waiting variant becomes "the cheap test for whether an apparent reversal signal is bid-ask bounce... a validity check rather than a robustness afterthought", with the VWAP leg conditional on intraday CSE data that has not been confirmed to exist. And the selection bias makes liquidity a constraint on the agent rather than a downstream cost: "the liquidity channel is not only a cost model downstream of the decision, it is a constraint on the technical agent's selection, one measurement serving both."
 EFFECT ON SUB-GAP 2: LEAVES IT OPEN, and - importantly - the note argues this paper makes Sub-gap 2 *more* load-bearing under transfer rather than less. No volatility is modelled anywhere; volatility enters only as a descriptive property of the selected set (240-day rolling volatility 0.0303 vs cross-sectional 0.0213). The risk control in the source paper is the long-short construction, which delivers beta −0.0023. Transfer to the CSE destroys it: "Short selling is not practically available on the CSE, so the implementable version is long top k only, which drops the short contribution of 0.0017 out of 0.0046 daily before costs and, more importantly, destroys the market neutrality behind the market beta of −0.0023. A long-only book whose constituents average a beta of 1.19 is a leveraged bet on the ASPI wearing a machine learning label, and the alpha claim collapses into a factor exposure unless something else carries the risk control. That something is the volatility and persistence conditioning, which the short leg was silently providing here, so the transfer makes A_V load-bearing in a way it is not in the source paper." And on persistence specifically: "a strategy that buys recent crashes is buying into elevated conditional variance, and if shocks on the ASPI decay hyperbolically as [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]] reports, the exposure schedule after a shock is the difference between a reversal trade and catching a falling counter." That sentence is the clearest statement in the whole set of what operationalised persistence is *for*: the post-shock exposure schedule.
-CSE DATA EVIDENCE: not a CSE paper, but it contains the most constructive reframing of the data blocker in the entire set. "Cross-sectional pooling is the answer to the data-depth blocker, and it also sizes the network." N_seq = Σ_s (T_s − L + 1). "At L = 240 on the confirmed February 2025 to February 2026 set, T_s ≈ L and the whole exercise yields about one sequence per counter, so the paper's own sequence length is unusable here and there is no way around that. At L = 30 with T_s ≈ 240 and a couple of hundred tradable counters, the same expression gives on the order of 40,000 to 50,000 sequences, within an order of magnitude of what this paper trains on. The short history is survivable only because the cross-section is the sample, which reframes the data problem from one about years of history to one about how many counters clear a liquidity screen, a question I can answer from what I already have." Note the confirmed CSE set is named here as February 2025 to February 2026 - roughly one year, T_s ≈ 240 trading days. Network sizing follows: "at roughly 93 examples per parameter and 45,000 sequences the budget is near 500 parameters, and solving 4(h(i+h+1)) + 2h + 2 for i=1 puts h at about ten to twelve hidden units against their twenty-five." Also a required CSE-specific data-quality step: "I need a trading-day filter dropping counters with no genuine print before the median is computed, and the count that filter removes on an average day is itself a liquidity statistic worth reporting."
+CSE DATA EVIDENCE: not a CSE paper, but it contains the most constructive reframing of the data blocker in the entire set. "Cross-sectional pooling is the answer to the data-depth blocker, and it also sizes the network." N_seq = Σ_s (T_s − L + 1). At L = 240 on the confirmed February 2025 to February 2026 set, T_s ≈ L and the whole exercise yields about one sequence per counter, so the paper's own sequence length is unusable here and there is no way around that. At L = 30 with T_s ≈ 240 and a couple of hundred tradable counters, the same expression gives on the order of 40,000 to 50,000 sequences, within an order of magnitude of what this paper trains on. The short history is survivable only because the cross-section is the sample, which reframes the data problem from one about years of history to one about how many counters clear a liquidity screen, a question I can answer from what I already have. Note the confirmed CSE set is named here as February 2025 to February 2026 - roughly one year, T_s ≈ 240 trading days. Network sizing follows: "at roughly 93 examples per parameter and 45,000 sequences the budget is near 500 parameters, and solving 4(h(i+h+1)) + 2h + 2 for i=1 puts h at about ten to twelve hidden units against their twenty-five." Also a required CSE-specific data-quality step: "I need a trading-day filter dropping counters with no genuine print before the median is computed, and the count that filter removes on an average day is itself a liquidity statistic worth reporting."
 PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool, but an explicit defence of A_L and A_V as separate agents rather than post-processing: "The model's selection bias is the argument for why A_L and A_V are separate agents rather than post-processing." On C_{i,t}, verbatim and important: "Softmax confidence is the obvious candidate for C_{A_T,t} and this paper gives me no grounds to trust it. The probability is used ordinally and never calibrated, and the 2010 to 2015 stretch is the case that worries me, since there is no reason to expect a network to become less confident when its edge is arbitraged away rather than simply wrong more often. So the technical agent's confidence should be a rolling realised accuracy over a trailing out-of-sample window, conditioned on the liquidity and volatility state, rather than the model's own score, and using the score instead has to be earned with a reliability diagram on my own data. The same question recurs for every agent that emits a confidence and it is the part of C_{i,t} I have least evidence about, so writing it down as unresolved is more useful right now than picking one."</t>
         </is>
       </c>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>"Daily direction prediction on six index closes... using a two-stage stacking ensemble the authors call EMD-ANNRC-RF... The contribution the paper actually cares about sits on top of that. LIME is run over the random forest to obtain a class probability for every individual prediction, that probability is read as a reliability score, and predictions whose score falls below a chosen threshold are simply not made." The note: "it is the only paper in the vault that implements abstention, and abstention is the missing half of my main gap."</t>
+          <t>Daily direction prediction on six index closes... using a two-stage stacking ensemble the authors call EMD-ANNRC-RF... The contribution the paper actually cares about sits on top of that. LIME is run over the random forest to obtain a class probability for every individual prediction, that probability is read as a reliability score, and predictions whose score falls below a chosen threshold are simply not made. The note: "it is the only paper in the vault that implements" abstention, and abstention is the missing half of my main gap.</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="O46" s="11" t="inlineStr">
         <is>
-          <t>none. No variance model, no persistence, no risk budget. The nearest thing is the untresholded soft confidence σ̂_t(x), which is a classifier output rather than a volatility quantity. The note names the resulting blind spot: "abstention very plausibly selects quiet days, since a forest fed a signed magnitude will be least confident when that magnitude is near zero and most confident when it is large, but nothing in the paper checks whether retained days carry larger or smaller absolute moves than discarded ones."</t>
+          <t>none. No variance model, no persistence, no risk budget. The nearest thing is the untresholded soft confidence σ̂_t(x), which is a classifier output rather than a volatility quantity. The note names the resulting blind spot: abstention very plausibly selects quiet days, since a forest fed a signed magnitude will be least confident when that magnitude is near zero and most confident when it is large, but nothing in the paper checks whether retained days carry larger or smaller absolute moves than discarded ones.</t>
         </is>
       </c>
       <c r="P46" s="11" t="inlineStr">
@@ -6337,7 +6337,7 @@
       </c>
       <c r="S46" s="11" t="inlineStr">
         <is>
-          <t>"EMD-ANNRC-RF runs 0.7806 to 0.8010 accuracy, EMD-ANNRC-XGBoost 0.7727 to 0.7878, and the single-stage EMD-ANNR 0.6476 to 0.7352, so the second stage is worth roughly ten accuracy points over stage 1 alone." Frontier: τ ≥ 0.50 → 100% coverage, 0.7909 accuracy; τ ≥ 0.85 → 62% coverage, 0.8953; τ ≥ 0.95 → 44% coverage, 0.9369; τ = 1.00 → 16% coverage, 0.9639. "Averaged across the six indices, moving the threshold from 0.50 to 1.00 takes the predicted days from roughly 622 to roughly 100, an 84 percent drop, while accuracy rises 21.87 percent to 0.9639." Note's reading: "Going from 0.85 to 1.00 buys under seven accuracy points and costs three quarters of the remaining trading days, whereas the first step, 100 percent coverage to 62 percent, buys more than ten. The useful part of the frontier is over by about 0.85 to 0.90, and the headline 0.9913 sits well past it." Cross-market robustness: "At reliability exactly 1, KOSPI gives 0.9913 on 115 days while FTSE100 gives 0.9079 on 76 and DAX 0.9636 on 55, so FTSE100's maximum-reliability result is worse than SP500's at the 0.95 level with four times the coverage." Null complexity results: VMD and EEMD in place of EMD showed "no significant difference observed in terms of hit rates", and ANN→LSTM "no significant difference in terms of accuracy". LIMITATIONS (quoting the note): "The decomposition runs on the entire dataset before the split... EMD is a global operation, every IMF at time t is a function of the whole series including its future, so the leak is structural rather than incidental. Every accuracy number below carries it." "Every number in the paper inherits the decomposition leak, and the size of the effect is unmeasured... the authors identify this themselves and then recommend the fix to other people rather than applying it." "LIME is never shown to add anything over the forest's own probability, and that ablation is the paper's load-bearing missing experiment... On this evidence I cannot tell whether the reliability score is a local explanation or the model's own confidence with extra steps." "Accuracy rising with the threshold is close to tautological, so the existence of the effect is not the finding." "There is no economic evaluation of any kind... Without that, 0.9639 accuracy on 16 percent of days is compatible with both a strong strategy and one that trades only when the move is too small to matter." "One run, no seeds, no significance tests, and no calibration check anywhere." "A single index series is the easiest possible setting for this mechanism and the paper stops just short of the hard one."</t>
+          <t>"EMD-ANNRC-RF runs 0.7806 to 0.8010 accuracy, EMD-ANNRC-XGBoost 0.7727 to 0.7878, and the single-stage EMD-ANNR 0.6476 to 0.7352, so the second stage is worth roughly ten accuracy points over stage 1 alone." Frontier: τ ≥ 0.50 → 100% coverage, 0.7909 accuracy; τ ≥ 0.85 → 62% coverage, 0.8953; τ ≥ 0.95 → 44% coverage, 0.9369; τ = 1.00 → 16% coverage, 0.9639. "Averaged across the six indices, moving the threshold from 0.50 to 1.00 takes the predicted days from roughly 622 to roughly 100, an 84 percent drop, while accuracy rises 21.87 percent to 0.9639." Note's reading: "Going from 0.85 to 1.00 buys under seven accuracy points and costs three quarters of the remaining trading days, whereas the first step, 100 percent coverage to 62 percent, buys more than ten". The useful part of the frontier is over by about 0.85 to 0.90, and the headline 0.9913 sits well past it. Cross-market robustness: "At reliability exactly 1, KOSPI gives 0.9913 on 115 days while FTSE100 gives 0.9079 on 76 and DAX 0.9636 on 55, so FTSE100's maximum-reliability result is worse than SP500's at the 0.95 level with four times the coverage." Null complexity results: VMD and EEMD in place of EMD showed "no significant difference observed in terms of hit rates", and ANN→LSTM "no significant difference in terms of accuracy". LIMITATIONS (quoting the note): "The decomposition runs on the entire dataset before the split... EMD is a global operation, every IMF at time t is a function of the whole series including its future, so the leak is structural rather than incidental. Every accuracy number below carries it." "Every number in the paper inherits the decomposition leak, and the size of the effect is unmeasured... the authors identify this themselves and then recommend the fix to other people rather than applying it." "LIME is never shown to add anything over the forest's own probability, and that ablation is the paper's load-bearing missing experiment... On this evidence I cannot tell whether the reliability score is a local explanation or the model's own confidence with extra steps." "Accuracy rising with the threshold is close to tautological, so the existence of the effect is not the finding." "There is no economic evaluation of any kind... Without that, 0.9639 accuracy on 16 percent of days" is compatible with both a strong strategy and one that trades only when the move is too small to matter. "One run, no seeds, no significance tests, and no calibration check anywhere." "A single index series is the easiest possible setting for this mechanism and the paper stops just short of the hard one."</t>
         </is>
       </c>
       <c r="T46" s="11" t="inlineStr">
@@ -6358,10 +6358,10 @@
       <c r="W46" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: orchestrator above all (abstention, and the common confidence scale for C_{i,t}), evaluation layer (coverage/accuracy pairing; the expectation band for honest CSE directional accuracy), A_L (the abstention-as-liquidity-screen check), A_T (the expectation band and the leak warning).
-EFFECT ON MAIN GAP / SUB-GAP 1: main gap - this is the single most directly useful paper in the set for the orchestration argument's second half. "My orchestration argument has always had two parts, that an agent's reliability varies with conditions and that the agents do not know it, and the second part is the one with no published mechanism behind it. AlphaAgents deleted its sentiment agent by hand and FinAgent's auxiliary strategies degraded quietly on ETHUSD, both because nothing in either design could decline to speak. This paper declines to speak, measures what declining costs, and publishes the frontier." It also supplies a concrete route to the comparable-confidence problem in C_{i,t}: "the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not." And it names precisely what must not be copied: "What I cannot borrow is the combiner itself, since a forest over two static features has no channel for liquidity state or volatility persistence and therefore reproduces exactly the fixed-influence design the main gap objects to, the same structural limitation as the near-binary mixture in [[MacroHFT...]]. The compression is the reusable part, the conditioning is mine to add." Sub-gap 1 - real bearing via the abstention-as-liquidity-screen problem: "On the CSE, an abstention threshold is partly a liquidity screen and I need to say which... the counters clearing a confidence bar are very likely the ones printing densely... So the check is to regress trusted-day frequency per counter on Amihud illiquidity and turnover before claiming the threshold is measuring confidence, which is the same measurement already being computed for the cost model, serving a third purpose." Plus the exposure policy on abstained days: "The abstained days also need an explicit exposure policy, hold the previous position or go flat, since those are different strategies and on the CSE the flat option carries a round-trip cost each time."
+EFFECT ON MAIN GAP / SUB-GAP 1: main gap - this is the single most directly useful paper in the set for the orchestration argument's second half. "My orchestration argument has always had two parts, that an agent's reliability varies with conditions and that the agents do not know it, and the second part is the one with no published mechanism behind it. AlphaAgents deleted its sentiment agent by hand and FinAgent's auxiliary strategies degraded quietly on ETHUSD, both because nothing in either design could decline to speak. This paper declines to speak, measures what declining costs, and publishes the frontier." It also supplies a concrete route to the comparable-confidence problem in C_{i,t}: the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical "acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not." And it names precisely what must not be copied: "What I cannot borrow is the combiner itself, since a forest over two static features has no channel for liquidity state or volatility persistence and therefore reproduces exactly the fixed-influence design the main gap objects to, the same structural limitation as the near-binary mixture in [[MacroHFT...]]. The compression is the reusable part, the conditioning is mine to add." Sub-gap 1 - real bearing via the abstention-as-liquidity-screen problem: "On the CSE, an abstention threshold is partly a liquidity screen and I need to say which... the counters clearing a confidence bar are very likely the ones printing densely... So the check is to regress trusted-day frequency per counter on Amihud illiquidity and turnover before claiming the threshold is measuring confidence, which is the same measurement already being computed for the cost model, serving a third purpose." Plus the exposure policy on abstained days: "The abstained days also need an explicit exposure policy, hold the previous position or go flat, since those are different strategies and on the CSE the flat option carries a round-trip cost each time."
 EFFECT ON SUB-GAP 2: LEAVES IT OPEN. There is no volatility quantity anywhere in this paper, so nothing is operationalised in the persistence direction. Its relevance is oblique but real in one respect: it is the only paper in the set where a *confidence* quantity is operationalised into a decision (trade or abstain), which is the structural template Sub-gap 2 needs for its own quantity - a measured scalar that gates action rather than describing it. The note's own framing of the missing economic check is also the Sub-gap-2-adjacent worry in reverse: abstention may be selecting low-volatility days, and the authors do not check it, so the interaction between the confidence filter and the volatility state is unexamined in exactly the way Sub-gap 2 says volatility states go unexamined.
 CSE DATA EVIDENCE: not a CSE paper. Two CSE-relevant implications: the coverage curve doubles as a measurement of how often a channel is live ("the coverage curve for the sentiment agent on CSE counters is directly the measurement of how often that channel is actually live"), and a calibrated expectation band is set - "my expectation band for a technical agent on CSE daily direction is somewhere near 0.54 to 0.58 on honest out-of-sample data, and a result above about 0.65 is a prompt to hunt for a leak rather than a success."
-PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On C_{i,t}, verbatim: "Realised conditional accuracy is the common scale for heterogeneous agent confidence, and this paper is the argument for it. The open question in my matrix is how an LLM analyst, an econometric estimator and an RL policy produce comparable confidence numbers, and the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not. It also inherits the calibration problem named above rather than solving it, so the curve has to be re-estimated as conditions move rather than fitted once." Implicitly this adds an abstention channel to the weighting function - w(i,t) should be able to go to zero for an agent on a given day - though the note never writes that as a change to f(·) itself.</t>
+PROPOSED REVISION STATED IN THE NOTE: no change to the four-agent pool. On C_{i,t}, verbatim: Realised conditional accuracy is the common scale for heterogeneous agent confidence, and this paper is the argument for it. The open question in my matrix is how an LLM analyst, an econometric estimator and an RL policy produce comparable confidence numbers, and the answer this suggests is not to compare their raw scores at all but to map each agent's score through its own empirical "acc(τ) curve estimated on a rolling validation window. That transform lands every agent in the same unit, probability of being right at the score it just emitted, which is comparable across architectures in a way that a softmax output and a posterior variance are not. It also inherits the calibration problem named above rather than solving it, so the curve has to be re-estimated as conditions move rather than fitted once." Implicitly this adds an abstention channel to the weighting function - w(i,t) should be able to go to zero for an agent on a given day - though the note never writes that as a change to f(·) itself.</t>
         </is>
       </c>
       <c r="X46" s="11" t="inlineStr">
@@ -6403,12 +6403,12 @@
       </c>
       <c r="G47" s="11" t="inlineStr">
         <is>
-          <t>Build a Neo4j knowledge graph of CSE corporate structure from annual report PDFs, with a LangGraph agent in front that turns natural-language questions into Cypher. Student: "It speaks to exactly one part of my architecture, A_F, the fundamental and retrieval channel, and to nothing else in it, so I am reading it as tooling and prior art rather than as a methodological template."</t>
+          <t>Build a Neo4j knowledge graph of CSE corporate structure from annual report PDFs, with a LangGraph agent in front that turns natural-language questions into Cypher. Student: It speaks to exactly one part of my architecture, A_F, the fundamental and retrieval channel, and to nothing else in it, so I am reading it as tooling and prior art rather than as a methodological template.</t>
         </is>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>Colombo Stock Exchange (Sri Lanka). Corporate structure QA over annual reports - directors, auditors, subsidiaries, executives, products, sectors. DATASETS &amp; PERIOD - AND HOW DOCUMENTS WERE OBTAINED: This is the critical intelligence gap. The note is emphatic that almost nothing is reported. "The number of source annual reports is never given, so I cannot tell whether that covers the roughly 280 listed companies or a fraction of them, and the word comprehensively is doing work the paper does not support." Under limitations: "No corpus size, no company or year coverage, no annotated-subset size". No date range is stated anywhere in the note. NO ACQUISITION METHOD IS REPORTED - the note records only that the inputs are "annual report PDFs", and the student's own separate reasoning is that "Annual reports are published artefacts that stay downloadable". The only CSE-data-access lead in the note is the contact lead, not a described method: the authors "are reachable, which also bears on the outstanding question of who to approach about CSE data access." Only coverage figure reported: "The graph holds over 6,000 unique entities across companies, directors, executives, subsidiaries, auditors, products and sectors". Graph is static, no as-of versioning.</t>
+          <t>Colombo Stock Exchange (Sri Lanka). Corporate structure QA over annual reports - directors, auditors, subsidiaries, executives, products, sectors. DATASETS &amp; PERIOD - AND HOW DOCUMENTS WERE OBTAINED: This is the critical intelligence gap. The note is emphatic that almost nothing is reported. "The number of source annual reports is never given, so I cannot tell whether that covers the" roughly 280 listed companies or a fraction of them, and the word comprehensively is doing work the paper does not support. Under limitations: "No corpus size, no company or year coverage, no annotated-subset size". No date range is stated anywhere in the note. NO ACQUISITION METHOD IS REPORTED - the note records only that the inputs are "annual report PDFs", and the student's own separate reasoning is that "Annual reports are published artefacts that stay downloadable". The only CSE-data-access lead in the note is the contact lead, not a described method: the authors "are reachable, which also bears on the outstanding question of who to approach about CSE data access." Only coverage figure reported: "The graph holds over 6,000 unique entities across companies, directors, executives, subsidiaries, auditors, products and sectors". Graph is static, no as-of versioning.</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
@@ -6418,7 +6418,7 @@
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>Unstructured text from annual report PDFs only. Entities: companies, directors, executives, subsidiaries, auditors, products, sectors. "Tabular financial data is explicitly not handled, stated in the conclusion and carried into future work as layout-aware parsing." METHOD - EXACT PIPELINE: (1) Chunking: "Annual report PDFs are chunked with a context-aware semantic strategy at a fixed window of roughly 1000 characters, preserving paragraph and section boundaries". (2) Embedding: "each chunk is embedded with Google Text Embedding 004 under a 3000-token input budget per document, into ChromaDB". (3) Extraction LLM: "Gemini 2.5 Pro then runs the extraction, but not over the whole document: it retrieves the top-5 relevant chunks per query and extracts entities into JSON inside a 500-token extraction context window." Student names this as the actual contribution: "question-driven targeted extraction instead of full-document extraction." (4) Consolidation: "Entity names are unified by a custom fuzzy matching pipeline with type-specific similarity functions, strict surname and initials for people, normalised token-sort and word overlap for companies, and then a Human-in-the-Loop clustering interface lets a reviewer merge or split clusters before variants are mapped onto canonical entity nodes". (5) Schema: "a rigid schema of DIRECTS, OWNS, AUDITED_BY and similar", plus entity type DIRECTOR with relationship type HOLDS_POSITION. "The resulting graph is company-centric, a star of typed edges around each listed entity" (Fig. 1 = Dialog Axiata PLC). (6) Retrieval/query: "a LangGraph/LangChain agent that decomposes a complex question into sub-queries, entity lookup then relationship traversal, and applies lightweight self-verification loops that reformulate and retry a sub-query returning incomplete or invalid output." Metric defined: Data Capture = (|{e ∈ E_gt : e extracted}| + |{r ∈ R_gt : r extracted}|) / (|E_gt| + |R_gt|), with "the denominator is never stated numerically anywhere in the paper".</t>
+          <t>Unstructured text from annual report PDFs only. Entities: companies, directors, executives, subsidiaries, auditors, products, sectors. "Tabular financial data is explicitly not handled, stated in the conclusion and carried into future work as layout-aware parsing." METHOD - EXACT PIPELINE: (1) Chunking: "Annual report PDFs are chunked with a context-aware semantic strategy at a fixed window of roughly 1000 characters, preserving paragraph and section boundaries". (2) Embedding: "each chunk is embedded with Google Text Embedding 004 under a 3000-token input budget per document, into ChromaDB". (3) Extraction LLM: "Gemini 2.5 Pro then runs the extraction, but not over the whole document: it retrieves the top-5 relevant chunks per query and extracts entities into JSON inside a 500-token extraction context window." Student names this as the actual contribution: question-driven targeted extraction instead of full-document extraction. (4) Consolidation: "Entity names are unified by a custom fuzzy matching pipeline with type-specific similarity functions, strict surname and initials for people, normalised token-sort and word overlap for companies, and then a" Human-in-the-Loop clustering interface lets a reviewer merge or split clusters before variants are mapped onto canonical entity nodes. (5) Schema: a rigid schema of DIRECTS, OWNS, AUDITED_BY and similar, plus entity type DIRECTOR with relationship type HOLDS_POSITION. "The resulting graph is company-centric, a star of typed edges around each listed entity" (Fig. 1 = Dialog Axiata PLC). (6) Retrieval/query: "a LangGraph/LangChain agent that decomposes a complex question into sub-queries, entity lookup then relationship traversal, and applies lightweight self-verification loops that reformulate and retry a sub-query returning incomplete or invalid output." Metric defined: Data Capture = (|{e ∈ E_gt: e extracted}| + |{r ∈ R_gt: r extracted}|) / (|E_gt| + |R_gt|), with the denominator is never stated numerically anywhere in the paper.</t>
         </is>
       </c>
       <c r="K47" s="11" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="M48" s="11" t="inlineStr">
         <is>
-          <t>Eight textual-analysis classification tasks (FPB, FiQA-SA, TSA, Headlines, FOMC, FinArg, MultiFin, MA, MLESG). Student's standing rule applied: "Per Scope sentiment analysis dropped the eight textual-analysis classification tasks are read as evidence about evaluation, not as a component to build." FUNDAMENTAL: QA aspect only - FinQA, TATQA, ConvFinQA, Regulations. No fundamental signal construction. RAG HANDLING: This is the headline finding for A_F. "The RAG evaluation claimed as a headline innovation does not exist in the paper... There is no retrieval dataset in Table 2, no retrieval condition in Section 3, no retrieval results in Section 4 and nothing in the appendices. Every task feeds its context directly into the prompt. The agent half of that sentence is delivered through FinMem on FinTrade; the RAG half is asserted and never operationalised. This is the claim I most wanted the paper to support and it is the one that is missing entirely, which means that as of mid-2024 no financial LLM benchmark evaluates retrieval as a variable, and FinanceBench's 19% to 50% under realistic retrieval remains the only number in the reading list that measures it."</t>
+          <t>Eight textual-analysis classification tasks (FPB, FiQA-SA, TSA, Headlines, FOMC, FinArg, MultiFin, MA, MLESG). Student's standing rule applied: "Per Scope sentiment analysis dropped the eight textual-analysis classification tasks are read as evidence about evaluation, not as a component to build." FUNDAMENTAL: QA aspect only - FinQA, TATQA, ConvFinQA, Regulations. No fundamental signal construction. RAG HANDLING: This is the headline finding for A_F. "The RAG evaluation claimed as a headline innovation does not exist in the paper... There is no retrieval dataset in Table 2, no retrieval condition in Section 3, no retrieval results in Section 4 and nothing in the appendices. Every task feeds its context directly into the prompt. The agent half of that sentence is delivered through FinMem on FinTrade; the RAG half is asserted and never operationalised". This is the claim I most wanted the paper to support and it is the one that is missing entirely, which means that as of mid-2024 no financial LLM benchmark evaluates retrieval as a variable, and FinanceBench's 19% to 50% under realistic retrieval remains the only number in the reading list that measures it.</t>
         </is>
       </c>
       <c r="N48" s="11" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="O48" s="11" t="inlineStr">
         <is>
-          <t>A "risk management" aspect of 9 tabular credit/fraud datasets, and volatility/drawdown as trading metrics. Student's verdict: "Risk management is the clearest case of a high F1 concealing a model that ignores its input... F1 near 0.9 with MCC exactly 0.00 is a model predicting the majority class for every row." Examples: "Mistral 7B on polish at F1 0.92 and MCC 0.00, GPT-4 on taiwan at 0.55 and -0.02... LLaMA2-70B on ccf at F1 1.00 and MCC 0.00."</t>
+          <t>A "risk management" aspect of 9 tabular credit/fraud datasets, and volatility/drawdown as trading metrics. Student's verdict: "Risk management is the clearest case of a high F1 concealing a model that ignores its input... F1 near 0.9 with MCC exactly 0.00 is a model predicting the majority class for every row." Examples: Mistral 7B on polish at F1 0.92 and MCC 0.00, GPT-4 on taiwan at 0.55 and -0.02... LLaMA2-70B on ccf at F1 1.00 and MCC 0.00.</t>
         </is>
       </c>
       <c r="P48" s="11" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="S48" s="11" t="inlineStr">
         <is>
-          <t>Forecasting - "twelve models cluster at accuracy 0.41 to 0.57 with MCC between -0.07 and 0.08, GPT-4 at 0.02, 0.02 and 0.02, Gemini at 0.03, 0.04 and 0.02, and the best single cell anywhere is FinMA 7B's 0.08 on CIKM18. Table 14 then reports SLOT, a 2022 self-supervised sequence model, at MCC 0.10, 0.21 and 0.09, and DTML at 0.07, 0.18 and -0.00." Trading - "GPT-4 reaches cumulative return 28.19% against Buy &amp; Hold's -4.00%, Sharpe 1.51 against 0.02, and maximum drawdown 18.34% against 30.67%, with Gemini second at 14.95% and Sharpe 1.03. Table 5 puts A2C, PPO and DQN at cumulative returns of -4.22%, -0.56% and -2.99% with Sharpe ratios of -0.26, 0.01 and -0.17". But "GPT-4o returns -5.54% at Sharpe -0.19 and llama3-70B returns -2.57% at Sharpe -0.04". QA - "GPT-4's TATQA exact-match accuracy is 0.13 against 0.63 on FinQA". Instruction tuning - "FinMA 7B posts the best scores in the table on FPB at 0.88 and FiQA-SA at 0.88 and Headlines at 0.97, beating GPT-4's 0.78, 0.76 and 0.86, and then scores 0.04 on FinQA, 0.00 on TATQA and 0.00 on ConvFinQA." LIMITATIONS (quoted): "Most of the headline results grid is zero, and the zeros are output-format failures rather than graded capability." "The trading confidence intervals cannot be reproduced from the paper's own per-stock table and the paper never says how they were computed... Recomputing GPT-4 from Table 9 gives mean cumulative return 26.80% and mean Sharpe 1.45 against the reported 28.19% and 1.51, and a cross-sectional interval of roughly ±10.5 on cumulative return against the reported ±25.27". "'Holistic' describes coverage and not measurement, because nothing aggregates." "The leakage machinery exists and is pointed at the wrong models." "The shared-task result the abstract leads on is not what the appendix shows" - winning team Sharpe 0.9268 vs GPT-4's 1.51.</t>
+          <t>Forecasting - twelve models cluster at accuracy 0.41 to 0.57 with MCC between -0.07 and 0.08, GPT-4 at 0.02, 0.02 and 0.02, Gemini at 0.03, 0.04 and 0.02, and the best single cell anywhere is FinMA 7B's 0.08 "on CIKM18. Table 14 then reports SLOT, a 2022 self-supervised sequence model, at MCC 0.10, 0.21 and 0.09, and DTML at 0.07, 0.18 and -0.00." Trading - "GPT-4 reaches cumulative return 28.19% against Buy &amp; Hold's -4.00%, Sharpe 1.51 against 0.02, and maximum drawdown 18.34% against 30.67%, with Gemini second at 14.95% and Sharpe 1.03. Table 5 puts A2C, PPO and DQN at cumulative returns of -4.22%, -0.56% and -2.99% with Sharpe ratios of -0.26, 0.01 and -0.17". But "GPT-4o returns -5.54% at Sharpe -0.19 and llama3-70B returns -2.57% at Sharpe -0.04". QA - "GPT-4's TATQA exact-match accuracy is 0.13 against 0.63 on FinQA". Instruction tuning - FinMA 7B posts the best scores in the table on FPB at 0.88 and FiQA-SA at 0.88 and Headlines at 0.97, beating GPT-4's 0.78, 0.76 and 0.86, and then scores 0.04 on FinQA, 0.00 on TATQA and 0.00 on ConvFinQA. LIMITATIONS (quoted): "Most of the headline results grid is zero, and the zeros are output-format failures rather than graded capability." "The trading confidence intervals cannot be reproduced from the paper's own per-stock table and the paper never says how they were computed... Recomputing GPT-4 from Table 9 gives mean cumulative return 26.80% and mean Sharpe 1.45 against the reported 28.19% and 1.51, and a cross-sectional interval of roughly ±10.5 on cumulative return against the reported ±25.27". "'Holistic' describes coverage and not measurement, because nothing aggregates." "The leakage machinery exists and is pointed at the wrong models." "The shared-task result the abstract leads on is not what the appendix shows" - winning team Sharpe 0.9268 vs GPT-4's 1.51.</t>
         </is>
       </c>
       <c r="T48" s="11" t="inlineStr">
@@ -6611,7 +6611,7 @@
           <t>SPEAKS TO: All four plus orchestrator plus evaluation layer - "it speaks to all four channels at once rather than to one."
 EFFECT ON A_F: Supports and clears the ground. "Retrieval quality is still unbenchmarked in the financial LLM literature, and that is now a positive finding rather than a hole in my reading... there is no external yardstick I can borrow for A_F and no risk that a reviewer points at FinBen as prior coverage of it." Usable as taxonomy: the seven-aspect list as a coverage checklist, and the FinTrade prompt as an output-schema template. Not usable as an evaluation set for CSE filings; the QA numbers it reports for FinQA/ConvFinQA are imported few-shot figures, not its own runs.
 SENTIMENT-RELATED EVIDENCE: Indirect - the 8 textual-analysis tasks read as evidence about evaluation only. The note explicitly cross-cites the temporal-shift paper as the reason FinBen's undated averaging is unsound: "Predict the Future from the Past... shows financial performance degrading measurably as the train-test gap widens, so an average over undated conditions is averaging over regimes that behave differently."
-PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool. On the orchestrator, verbatim: "the orchestrator has to be able to drive a channel's weight to near zero, which is what the pre-registered weight-entropy diagnostic exists to detect." And on A_T's composition: "A_T is an econometric or RL component with an LLM nowhere in the directional path". On the failure bucket: "the harness needs strict output validation and a logged failure bucket that feeds the weighting function a hard zero."</t>
+PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool. On the orchestrator, verbatim: "the orchestrator has to be able to drive a channel's weight to near zero", which is what the pre-registered weight-entropy diagnostic exists to detect. And on A_T's composition: "A_T is an econometric or RL component with an LLM nowhere in the directional path". On the failure bucket: "the harness needs strict output validation and a logged failure bucket that feeds the weighting function a hard zero."</t>
         </is>
       </c>
       <c r="X48" s="11" t="inlineStr">
@@ -6668,12 +6668,12 @@
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>Text, plus "historical price series serialised into the prompt as text, alongside tweets, with tables likewise flattened into the context string. There is no separate encoder, no projection layer and no fusion mechanism of any kind, so the claim is about the data types covered rather than about the model."</t>
+          <t>Text, plus historical price series serialised into the prompt as text, "alongside tweets, with tables likewise flattened into the context string. There is no separate encoder, no projection layer and no fusion mechanism of any kind, so the claim is about the data types covered rather than about the model."</t>
         </is>
       </c>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>Instruction tuning LLaMA. "Domain experts wrote ten diverse instructions per dataset". Two templates: Instruction: [task prompt] Text: [input text] Response: [output], and for FinQA/ConvFinQA Instruction: ... Context: ... Question: ... Response: ..., with ConvFinQA's multi-turn conversations flattened by appending prior Q&amp;A into the context. Four LLaMA checkpoints - FinMA-7B, FinMA-30B (NLP portion), FinMA-7B-trade (forecasting only), FinMA-7B-full. AdamW, lr 8e-6, weight decay 1e-5, warmup 5%, max input 2048. "the 30B runs 20 epochs at batch size 24 on 128 A100 40GB GPUs".</t>
+          <t>Instruction tuning LLaMA. Domain experts wrote ten diverse instructions per dataset. Two templates: Instruction: [task prompt] Text: [input text] Response: [output], and for FinQA/ConvFinQA Instruction:... Context:... Question:... Response:..., with ConvFinQA's multi-turn conversations flattened by appending prior Q&amp;A into the context. Four LLaMA checkpoints - FinMA-7B, FinMA-30B (NLP portion), FinMA-7B-trade (forecasting only), FinMA-7B-full. AdamW, lr 8e-6, weight decay 1e-5, warmup 5%, max input 2048. "the 30B runs 20 epochs at batch size 24 on" 128 A100 40GB GPUs.</t>
         </is>
       </c>
       <c r="L49" s="11" t="inlineStr">
@@ -6713,7 +6713,7 @@
       </c>
       <c r="S49" s="11" t="inlineStr">
         <is>
-          <t>"FinMA-7B reaches 0.94 weighted F1 on FPB against GPT-4's 0.78 and BloombergGPT's 0.51, 0.97 average F1 on Headlines against 0.86 and 0.82, and 0.85 on FiQA-SA with the 30B at 0.87". Unseen-data reversal: FiNER-ORD 0.00 vs GPT-4's 0.77; FOMC 0.49 vs 0.71; Australian 0.41 vs 0.74. Numeric reasoning: "FinQA exact-match accuracy is 0.06 for FinMA-7B and 0.11 for the 30B against GPT-4's 0.63 and ChatGPT's 0.58, and ConvFinQA is 0.25 and 0.40 against 0.76 and 0.60." Directional: "Accuracies cluster between 0.43 and 0.57 across all three datasets and all eight models, and the corresponding MCC values sit within roughly ±0.05 of zero... SLOT, a 2022 sequence model, reaches accuracy 0.55, 0.59 and 0.56 with MCC 0.10, 0.21 and 0.09". Trade-tuned collapse: "FinMA-7B-trade scores 0.03 F1 on FPB, 0.16 on FiQA-SA and 0.28 on Headlines, against 0.94, 0.85 and 0.97 for the NLP-tuned sibling". Appendix: "FLANG-BERT, a 110M-parameter encoder, reaches 0.912 accuracy on FPB, 0.972 average F1 on Headlines and 0.83 F1 on NER, against FinMA-7B's 0.94, 0.97 and 0.59." LIMITATIONS (quoted): "The central comparison is not like for like, and the paper's framing does not flag it." "the abstract's claim that FinMA significantly outperforms BloombergGPT, ChatGPT and GPT-4 on most tasks is the version that travels into citations, stripped of the supervision asymmetry that produces it." "The appendix contains the fair comparison and it is much less favourable." "The prediction tasks as posed cannot demonstrate what the paper wants them to." "Temporal design is absent, and the leakage question cannot be checked." "The instruction set is never ablated, so the paper's own explanatory claim is unsupported." "An accuracy near 0.50 with an MCC near 0.00 is what a channel with no signal looks like". "Eight different models producing byte-identical BARTScore is a degenerate-output signature rather than eight measurements".</t>
+          <t>"FinMA-7B reaches 0.94 weighted F1 on FPB against GPT-4's 0.78 and BloombergGPT's 0.51, 0.97 average F1 on Headlines against 0.86 and 0.82, and 0.85 on FiQA-SA with the 30B at 0.87". Unseen-data reversal: FiNER-ORD 0.00 vs GPT-4's 0.77; FOMC 0.49 vs 0.71; Australian 0.41 vs 0.74. Numeric reasoning: "FinQA exact-match accuracy is 0.06 for FinMA-7B and 0.11 for the 30B against GPT-4's 0.63 and ChatGPT's 0.58, and ConvFinQA is 0.25 and 0.40 against 0.76 and 0.60." Directional: Accuracies cluster between 0.43 and 0.57 across all three datasets and all eight models, and the corresponding MCC values sit within roughly ±0.05 of zero... SLOT, a 2022 sequence model, reaches accuracy 0.55, 0.59 and 0.56 with MCC 0.10, 0.21 and 0.09. Trade-tuned collapse: "FinMA-7B-trade scores 0.03 F1 on FPB, 0.16 on FiQA-SA and 0.28 on Headlines, against 0.94, 0.85 and 0.97 for the NLP-tuned sibling". Appendix: "FLANG-BERT, a 110M-parameter encoder, reaches 0.912 accuracy on FPB, 0.972 average F1 on Headlines and 0.83 F1 on NER, against FinMA-7B's 0.94, 0.97 and 0.59." LIMITATIONS (quoted): "The central comparison is not like for like, and the paper's framing does not flag it." "the abstract's claim that FinMA significantly outperforms BloombergGPT, ChatGPT and GPT-4 on most tasks is the version that travels into citations", stripped of the supervision asymmetry that produces it. "The appendix contains the fair comparison and it is much less favourable." "The prediction tasks as posed cannot demonstrate what the paper wants them to." "Temporal design is absent, and the leakage question cannot be checked." "The instruction set is never ablated, so the paper's own explanatory claim is unsupported." "An accuracy near 0.50 with an MCC near 0.00 is what a channel with no signal looks like". "Eight different models producing byte-identical BARTScore is a degenerate-output signature rather than eight measurements".</t>
         </is>
       </c>
       <c r="T49" s="11" t="inlineStr">
@@ -6736,7 +6736,7 @@
           <t>SPEAKS TO: A_F, A_T and the orchestrator, plus the evaluation layer. "it is the only one that puts a language model on stock movement prediction and credit scoring alongside the reading tasks, so it speaks to A_T and the orchestrator as well as to A_F."
 EFFECT ON A_F: Constrains decisively - it closes fine-tuning off. "This closes the question of whether to fine-tune an open model for the fundamental channel, and the answer is no... the working design for A_F stays a frontier model over structure-aware retrieval, with fine-tuning off the table rather than deferred." Usable artefacts: the FLARE prompt templates and harness as a ready format for evaluating A_F against a small probe set. Not usable as a CSE evaluation set. Licences: "Licences are mixed across the assembled datasets, CC BY-SA 3.0, CC BY-NC 4.0 on FOMC, MIT and public, which constrains reuse in a way the 'fully open' framing glosses over."
 SENTIMENT-RELATED EVIDENCE: Cross-cited only - "Predict the Future from the Past... shows financial sentiment performance degrading measurably as the gap between training and test period widens, so a benchmark that mixes periods without reporting them is measuring an average over conditions that behave differently."
-PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool; an explicit argument for keeping it as-is, verbatim: "FinMA-7B-trade is a clean documented case for keeping the four agents architecturally separate. One backbone tuned for the prediction task loses its classification ability almost entirely, 0.94 to 0.03 on FPB, and gains nothing measurable on the task it was specialised for. A shared fine-tuned backbone across A_T, A_F, A_V and A_L would buy exactly this, and the heterogeneity argument in the main gap is partly an argument that the components should fail independently, which a shared backbone forbids by construction." On the conditioning set / confidence, verbatim: "the orchestrator has to be able to drive a channel's weight to near zero rather than assuming every agent contributes." And: "The correct, incorrect and failure-to-answer taxonomy adopted from FinanceBench gains a fourth bucket, no parseable answer, which for the weighting function is a hard zero rather than a low C_{i,t}".</t>
+PROPOSED REVISION STATED IN THE NOTE: No change to the four-agent pool; an explicit argument for keeping it as-is, verbatim: "FinMA-7B-trade is a clean documented case for keeping the four agents architecturally separate. One backbone tuned for the prediction task loses its classification ability almost entirely, 0.94 to 0.03 on FPB, and gains nothing measurable on the task it was specialised for. A shared fine-tuned backbone across A_T, A_F, A_V and A_L would buy exactly this, and the heterogeneity argument in the main gap is partly an argument that the components should fail independently, which a shared backbone forbids by construction." On the conditioning set / confidence, verbatim: "the orchestrator has to be able to drive a channel's weight to near zero" rather than assuming every agent contributes. And: "The correct, incorrect and failure-to-answer taxonomy adopted from FinanceBench gains a fourth bucket, no parseable answer, which for the weighting function is a hard zero rather than a low C_{i,t}".</t>
         </is>
       </c>
       <c r="X49" s="11" t="inlineStr">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>3,892 conversations / 14,115 questions; 3,037/421/434 train/dev/test conversations; 2,715 simple / 1,177 hybrid; 2,066 report pages; avg 3.67 questions per conversation; avg question 10.59 tokens; avg/max input 675.61 / 2,338 tokens; 34.73% number-selection questions; 1/2/3-step programs 35.10%/25.41%/4.75%; supporting facts from table/text/both 59.18%/25.56%/15.26%. Operation mix: 40.49% subtract, 33.43% divide, 18.80% add, 6.92% multiply. "the DSL is six operations only, add, subtract, multiply, divide, exp and greater, with FinQA's four table aggregations dropped."</t>
+          <t>3,892 conversations / 14,115 questions; 3,037/421/434 train/dev/test conversations; 2,715 simple / 1,177 hybrid; 2,066 report pages; avg 3.67 questions per conversation; avg question 10.59 tokens; avg/max input 675.61 / 2,338 tokens; 34.73% number-selection questions; 1/2/3-step programs 35.10%/25.41%/4.75%; supporting facts from table/text/both 59.18%/25.56%/15.26%. Operation mix: 40.49% subtract, 33.43% divide, 18.80% add, 6.92% multiply. the DSL is six operations only, "add, subtract, multiply, divide, exp and greater, with FinQA's four table aggregations dropped."</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="W50" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: A_F and the evaluation layer only - stated explicitly: "it speaks to A_F, the fundamental and retrieval channel, and to the evaluation layer, and to nothing else".
+          <t>SPEAKS TO: A_F and the evaluation layer only - stated explicitly: it speaks to A_F, the fundamental and retrieval channel, and to the evaluation layer, and to nothing else.
 EFFECT ON A_F: Constrains the interface design (no conversational interface; atomic self-contained requests; typed-pointer chaining), constrains the planning band (below 50% on computed quantities over CSE filings), supplies the conditional-accuracy metric for the probe set, and supplies the CSE-specific reference-resolution warning: "Sri Lankan annual reports lean on phrases like the corresponding period and as restated, quarterly statements refer back to the annual ones, and comparative columns are labelled by position rather than by date... period resolution belongs in the retrieval and typing layer, resolved against an explicit fiscal calendar, and never left to the reasoner to infer from context." Usable as evaluation material: yes, as a probe corpus paired with FinQA - "Because the conversations are synthesised from FinQA programs, the pairing is already aligned, so the two can be used as one probe corpus with and without conversational context, which is the cheapest available ablation on whether my own reference-resolution layer is doing anything." Taxonomy usable: the question-shape split (number selection vs program questions) and the three-dataset comparison table. Licence: not stated beyond "Dataset and code are public"; inherits FinTabNet.
 SENTIMENT-RELATED EVIDENCE: None.
 PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool or the conditioning set. Design revisions to A_F's interface, verbatim: "Query A_F with atomic, self-contained requests and do not build a conversational interface to it... The orchestrator already holds the state it needs, so resolving that value in the subsequent year into an explicit entity, period and line item before the call costs me nothing and removes the failure mode the paper spends its results section documenting." And: "my equivalent is a resolved quantity carrying value, scale, currency, period and the source rows it came from, per the typed-output decision from the TAT-QA note, passed back in explicitly on the next call." And the closed vocabulary: "Level, difference, ratio and growth rate is the closed vocabulary, anything outside it gets declined rather than attempted, and this is the last time it needs arguing."</t>
@@ -6913,17 +6913,17 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>"Roughly 500 financial reports from the past two years are downloaded from annualreports.com"; TableBank detection, Apache PDFBox extraction; tables outside 3–30 rows and 3–6 columns dropped, leaving ~20,000 candidates; "About two thirds of the candidate tables are discarded during annotation for lacking enough relevant surrounding paragraphs." Final: 16,552 QA pairs over 2,757 hybrid contexts from 182 reports; split by context - 2,201/13,215 train, 278/1,668 dev, 278/1,669 test. Tables average 9.4 rows and 4.0 columns with 4.8 paragraphs of 43.6 words; questions average 12.5 words, answers 4.1. Annotators: ~30 finance undergraduates screened at 95%, ~two hybrid contexts per hour over three months, two-round validation by five verifiers.</t>
+          <t>"Roughly 500 financial reports from the past two years are downloaded from annualreports.com"; TableBank detection, Apache PDFBox extraction; tables outside 3–30 rows and 3–6 columns dropped, leaving ~20,000 candidates; About two thirds of the candidate tables are discarded "during annotation for lacking enough relevant surrounding paragraphs." Final: 16,552 QA pairs over 2,757 hybrid contexts from 182 reports; split by context - 2,201/13,215 train, 278/1,668 dev, 278/1,669 test. Tables average 9.4 rows and 4.0 columns with 4.8 paragraphs of 43.6 words; questions average 12.5 words, answers 4.1. Annotators: ~30 finance undergraduates screened at 95%, ~two hybrid contexts per hour over three months, two-round validation by five verifiers.</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>Table plus prose. "79% of its tables have two or more row headers". Answer-type × answer-source grid: Span 1,801/3,496/1,842; Spans 777/258/1,037; Counting 106/5/266; Arithmetic 4,747/143/2,074; totals 7,431 table / 3,902 text / 5,219 table-text / 16,552. "Arithmetic is 42% of the dataset... And the table-text class, the one that needs both sources, is 5,219 questions or 31.5%, against 14.15% in FinQA".</t>
+          <t>Table plus prose. 79% of its tables have two or more row headers. Answer-type × answer-source grid: Span 1,801/3,496/1,842; Spans 777/258/1,037; Counting 106/5/266; Arithmetic 4,747/143/2,074; totals 7,431 table / 3,902 text / 5,219 table-text / 16,552. "Arithmetic is 42% of the dataset... And the table-text class, the one that needs both sources, is 5,219 questions or 31.5%, against 14.15% in FinQA".</t>
         </is>
       </c>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>TagOp - question + flattened table + paragraphs into RoBERTa, per-sub-token I/O tagging for evidence, then exactly one of ten aggregation operators applied, plus a separate scale head. Ten operators: Span-in-text, Cell-in-table, Spans, Sum, Count, Average, Multiplication, Division, Difference, Change ratio. "Exactly one operator is applied per question, so there is no composition in the FinQA sense." Four heads. Order head: p^order = softmax(FFN(avg(h_t1, h_t2))). Scale head (5-way over None, Thousand, Million, Billion, Percent): p^scale = softmax(FFN([[CLS]; h_tab; h_p])). Loss: L = NLL(log P^tag, G^tag) + NLL(log P^op, G^op) + NLL(log P^scale, G^scale) + NLL(log P^order, G^order). Evaluation is EM and DROP-style numeracy F1 with sign preserved and "F1 is set to zero unless the predicted number multiplied by the predicted scale matches exactly".</t>
+          <t>TagOp - question + flattened table + paragraphs into RoBERTa, per-sub-token I/O tagging for evidence, then exactly one of ten aggregation operators applied, plus a separate scale head. Ten operators: Span-in-text, Cell-in-table, Spans, Sum, Count, Average, Multiplication, Division, Difference, Change ratio. Exactly one operator is applied per question, so there is no composition in the FinQA sense. Four heads. Order head: p^order = softmax(FFN(avg(h_t1, h_t2))). Scale head (5-way over None, Thousand, Million, Billion, Percent): p^scale = softmax(FFN([[CLS]; h_tab; h_p])). Loss: L = NLL(log P^tag, G^tag) + NLL(log P^op, G^op) + NLL(log P^scale, G^scale) + NLL(log P^order, G^order). Evaluation is EM and DROP-style numeracy F1 with sign preserved and F1 "is set to zero unless the predicted number multiplied by the predicted scale matches exactly".</t>
         </is>
       </c>
       <c r="L51" s="11" t="inlineStr">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="S51" s="11" t="inlineStr">
         <is>
-          <t>"TagOp reaches 50.1 EM and 58.0 F1 on test against human performance of 84.1 and 90.8, so the model sits roughly 33 F1 points below the expert bar." Error profile: "84% of errors are evidence extraction failures, not reasoning failures... Wrong Evidence is 55% and Missing Evidence 29%, against Wrong Calculation 9%, Unsupported Calculation 4% and Scale Error 3%." "Arithmetic is the floor, at 42.5 EM and 42.5 F1 against 54.1/67.9 on Span, 60.0/75.1 on Spans and 62.5/62.5 on Counting." Operator ablation: "adding Difference lifts test EM by 5.9 points and Change ratio by another 5.0... while Sum adds nothing and Multiplication is flat to slightly negative." Source split: "Table-sourced questions score 47.8 EM against text-sourced at 43.3... but on F1 the ordering reverses sharply, 49.3 for table against 68.7 for text. The best-performing source is actually table-text at 58.3 EM". Scale: "Per-class test accuracy is 90.1 on None, 95.3 on Thousand, 90.2 on Million and 95.9 on Percent, and scale contributes only 3% of sampled errors." Operator classifier: "Test accuracy is 100.0 on Count and Average and 96.6 on Difference, but 0.0 on Multiplication and 0.0 on the catch-all Other, which together are 6.7% of test questions." LIMITATIONS (quoted): "There is no retrieval step at all". "One operator per question makes the compositionality claim circular." "The question distribution is shaped by the annotation instructions in ways that inflate the easy classes." "Every number is a single-run point estimate with no interval, no seed variance and no significance test." "Domain knowledge is named as an error source and then left unquantified." "The upstream extraction pipeline is asserted to work rather than measured... nothing here informs me about the step most likely to break first on CSE filings."</t>
+          <t>TagOp reaches 50.1 EM and 58.0 F1 on test against human performance of 84.1 and 90.8, so the model sits roughly 33 F1 points below the expert bar. Error profile: "84% of errors are evidence extraction failures, not reasoning failures... Wrong Evidence is 55% and Missing Evidence 29%, against Wrong Calculation 9%, Unsupported Calculation 4% and Scale Error 3%." Arithmetic is the floor, at 42.5 EM and 42.5 F1 "against 54.1/67.9 on Span, 60.0/75.1 on Spans and 62.5/62.5 on Counting." Operator ablation: adding Difference lifts test EM by 5.9 points and Change ratio by another 5.0... while Sum adds nothing and Multiplication is flat to slightly negative. Source split: Table-sourced questions score 47.8 EM against text-sourced at 43.3... but on F1 the ordering reverses sharply, 49.3 for table against 68.7 for text. The best-performing source is actually table-text at 58.3 EM. Scale: "Per-class test accuracy is 90.1 on None, 95.3 on Thousand, 90.2 on Million and 95.9 on Percent, and scale contributes only 3% of sampled errors." Operator classifier: "Test accuracy is 100.0 on Count and Average and 96.6 on Difference, but 0.0 on Multiplication and 0.0 on the catch-all Other, which together are 6.7% of test questions." LIMITATIONS (quoted): "There is no retrieval step at all". "One operator per question makes the compositionality claim circular." "The question distribution is shaped by the annotation instructions in ways that inflate the easy classes." "Every number is a single-run point estimate with no interval, no seed variance and no significance test." "Domain knowledge is named as an error source and then left unquantified." "The upstream extraction pipeline is asserted to work rather than measured... nothing here informs me about the step most likely to break first on CSE filings."</t>
         </is>
       </c>
       <c r="T51" s="11" t="inlineStr">
@@ -6986,7 +6986,7 @@
           <t>SPEAKS TO: A_F and the evaluation layer only, stated explicitly.
 EFFECT ON A_F: Strongly supports and shapes the design. Establishes the typed-output decision; supports keeping a retrieval stage; fixes the operator vocabulary; supplies a second mechanical confidence signal with a caveat; supplies the reporting axes. "This also keeps A_F compatible with the structure-aware retrieval work in Neo4j Graph-RAG for CSE and Financial Report Chunking for Effective Retrieval Augmented Generation, which a single-sequence tagging design would not be." Usable taxonomy: the scale taxonomy (None/Thousand/Million/Billion/Percent) and the answer-type × answer-source split - "The scale taxonomy and the answer-type and answer-source split are worth lifting directly into my probe set design." Licence for the dataset itself: public for non-commercial use.
 SENTIMENT-RELATED EVIDENCE: None.
-PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. A stated design decision on A_F's output, verbatim: "The design decision is that A_F emits a typed quantity, value plus scale plus currency plus period, and never a bare number, which also removes the unit-conversion error class that the FinQA note flagged as a representation problem rather than a model one." On the conditioning set / C_{F,t}, verbatim: "This gives me a second mechanical confidence signal for C_{F,t}, and a warning about how to use it. FinQA offered program step count; TAT-QA offers the operator classifier posterior, the tagging margin on the selected evidence, and whether the predicted scale fell in a rare class. But operator accuracy runs from 100.0 on Count and Average down to 0.0 on Multiplication and Other, so a single posterior is not comparable across classes and I would need per-operator reliability estimated on my own probe set before the orchestrator can read it... it is the second time the answer for A_F has turned out to be a structural property of the output rather than a self-reported score, which is worth noting as a pattern."</t>
+PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. A stated design decision on A_F's output, verbatim: The design decision is that A_F emits a typed quantity, value plus scale plus currency plus period, and never a bare number, which also removes the unit-conversion error class that the FinQA note flagged as a representation problem rather than a model one. On the conditioning set / C_{F,t}, verbatim: "This gives me a second mechanical confidence signal for C_{F,t}, and a warning about how to use it. FinQA offered program step count; TAT-QA offers the operator classifier posterior, the tagging margin on the selected evidence, and whether the predicted scale fell in a rare class. But operator accuracy runs from 100.0 on Count and Average down to 0.0 on Multiplication and Other, so a single posterior is not comparable across classes and I would need per-operator reliability estimated on my own probe set before the orchestrator can read it... it is the second time the answer for A_F has turned out to be a structural property of the output rather than a self-reported score, which is worth noting as a pattern."</t>
         </is>
       </c>
       <c r="X51" s="11" t="inlineStr">
@@ -7043,12 +7043,12 @@
       </c>
       <c r="J52" s="11" t="inlineStr">
         <is>
-          <t>Table plus text on one page. "Questions answerable from table only 62.43%; text only 23.42%; needing both 14.15%. One supporting fact 46.30%; two 42.63%; more than two 11.07%. One-step programs 59.10%; two-step 32.71%; three or more 8.19%." Inputs average 628.11 text tokens + 59.42 table tokens = 687.53, max 2,679; questions average 16.63 tokens. "divide dominates at 45.29% and subtract follows at 28.20%."</t>
+          <t>Table plus text on one page. Questions answerable from table only 62.43%; text only 23.42%; needing both 14.15%. One supporting fact 46.30%; two 42.63%; more than two 11.07%. One-step programs 59.10%; two-step 32.71%; three or more 8.19%. Inputs average 628.11 text tokens + 59.42 table tokens = 687.53, max 2,679; questions average 16.63 tokens. "divide dominates at 45.29% and subtract follows at 28.20%."</t>
         </is>
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>Ten-operation DSL - add, subtract, multiply, divide, exp, greater, plus table-max, table-min, table-sum, table-average. Flat program op_1[args_1], op_2[args_2], …, op_n[args_n] with #k referencing step k. Task: P(A | T, E, Q) = Σ_i P(G_i | T, E, Q). FinQANet, two-stage retriever-generator. Retriever templates each table row into a sentence ("the risk-free interest rate of 2006 is 5%"), concatenates with the question, trains a BERT-base classifier, keeps top three reordered into document order. Generator is an LSTM decoder over copy-and-generate space: c_T = W_c[att_p; att_h; h_T], w_T = softmax(H'_T · c_T), with H'_T = W_h[H; H ∘ att'_p]. The novel piece: "at the end of each completed operation[args] unit, the embedding of the corresponding step memory token is overwritten with that step's context vector, so a reference to #0 later in the sequence carries what step 0 did rather than being an opaque symbol." Grammar masks keep output valid.</t>
+          <t>Ten-operation DSL - add, subtract, multiply, divide, exp, greater, plus table-max, table-min, table-sum, table-average. Flat program op_1[args_1], op_2[args_2], …, op_n[args_n] with #k referencing step k. Task: P(A | T, E, Q) = Σ_i P(G_i | T, E, Q). FinQANet, two-stage retriever-generator. Retriever templates each table row into a sentence ("the risk-free interest rate of 2006 is 5%"), concatenates with the question, trains a BERT-base classifier, keeps top three reordered into document order. Generator is an LSTM decoder over copy-and-generate space: c_T = W_c[att_p; att_h; h_T], w_T = softmax(H'_T · c_T), with H'_T = W_h[H; H ∘ att'_p]. The novel piece: at the end of each completed operation[args] unit, the embedding of the corresponding step memory token is overwritten with that step's context vector, so a reference to #0 later in the sequence carries what step 0 did rather than being an opaque symbol. Grammar masks keep output valid.</t>
         </is>
       </c>
       <c r="L52" s="11" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="S52" s="11" t="inlineStr">
         <is>
-          <t>"The best system reaches 61.24% execution and 58.86% program accuracy, against 91.16% and 87.49% for finance professionals and 50.68% and 48.17% for the MTurk crowd... Giving the model gold retrieval instead of its own lifts it to 70.00% and 68.76%, so roughly nine points of the thirty-point gap is retrieval and the remaining twenty-one is reasoning." "Keeping the architecture identical but generating the answer directly instead of the program collapses execution accuracy to 0.30%, an end-to-end pre-trained Longformer over the whole report gets 21.90%, and a retriever plus Seq2seq generator gets 19.71%. Against NeRd... FinQANet at BERT-base is 50.00% versus 48.57%". "Restricting inference to table facts gives 45.81% and to text facts 15.80%". "table-only questions score 67.38%, text-only 54.86%, and the questions requiring table and text together score 43.80%". "One-step programs score 67.61%, two-step 59.08%, and programs of three or more steps 22.78%. Programs containing a constant... score 43.88%." "FinQANet with FinBert scores 50.10%, essentially level with BERT-base at 50.00% and below BERT-large at 53.52%, with RoBERTa-large well ahead at 61.24%." LIMITATIONS (quoted): "The filtering removes exactly the layouts that make real reports hard." "Every question is page-local, so the retrieval problem is much shallower than the one a fundamental channel faces." "The DSL bounds what counts as a question... Questions a finance professional could not express in this DSL simply never entered the dataset, which makes the coverage claim circular in a way the paper does not discuss." "Both metrics are known to be biased and neither carries an interval." "The human upper bound rests on 200 examples and the question distribution is annotator-driven... the questions are what a finance professional thought was interesting about one page, which is not the same distribution as the quantities a trading system needs computed." Warning: "61.24% is not a portable number... Cite it as the order of magnitude of the task's difficulty and as the size of the gap to expert humans, and do not let it become a target or a baseline for anything I build on CSE reports."</t>
+          <t>"The best system reaches 61.24% execution and 58.86% program accuracy, against 91.16% and 87.49% for finance professionals and 50.68% and 48.17% for the MTurk crowd... Giving the model gold retrieval instead of its own lifts it to 70.00% and 68.76"%, so roughly nine points of the thirty-point gap is retrieval and the remaining twenty-one is reasoning. "Keeping the architecture identical but generating the answer directly instead of the program collapses execution accuracy to 0.30%, an end-to-end pre-trained Longformer over the whole report gets 21.90%, and a retriever plus Seq2seq generator gets 19.71%. Against NeRd... FinQANet at BERT-base is 50.00% versus 48.57%". "Restricting inference to table facts gives 45.81% and to text facts 15.80%". "table-only questions score 67.38%, text-only 54.86%, and the questions requiring table and text together score 43.80%". "One-step programs score 67.61%, two-step 59.08%, and programs of three or more steps 22.78%. Programs containing a constant... score 43.88%." FinQANet with FinBert scores 50.10%, essentially level with BERT-base at 50.00% and below BERT-large at 53.52%, with RoBERTa-large well ahead at 61.24%. LIMITATIONS (quoted): "The filtering removes exactly the layouts that make real reports hard." "Every question is page-local, so the retrieval problem is much shallower than the one a fundamental channel faces." "The DSL bounds what counts as a question... Questions a finance professional could not express in this DSL simply never entered the dataset, which makes the coverage claim circular in a way the paper does not discuss." "Both metrics are known to be biased and neither carries an interval." "The human upper bound rests on 200 examples and the question distribution is annotator-driven... the questions are what a finance professional thought was interesting about one page, which is not the same distribution as the quantities a trading system needs computed." Warning: "61.24% is not a portable number... Cite it as the order of magnitude of the task's difficulty and as the size of the gap to expert humans, and do not let it become a target or a baseline for anything I build on CSE reports."</t>
         </is>
       </c>
       <c r="T52" s="11" t="inlineStr">
@@ -7111,7 +7111,7 @@
           <t>SPEAKS TO: A_F and the evaluation layer only, stated explicitly.
 EFFECT ON A_F: Defines it. "This is the task specification for the numeric half of A_F, and the pair with the CSE Graph-RAG paper draws the boundary cleanly. That paper builds the entity graph and states that statement tables are future work; this one does the statement tables and ignores entity structure. In the review chapter that pairing is how I justify A_F as a system component built on published task definitions, with the contribution sitting in the orchestration rather than in the retrieval." Usable artefacts: the DSL and program executor (public, CDLA-Permissive via FinTabNet); the evaluation shape. Not usable as a CSE set: "There is no CSE equivalent of this dataset and building one is out of scope... the FinTabNet licensing and the annotations do not transfer to CSE filings."
 SENTIMENT-RELATED EVIDENCE: None.
-PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. Scope decision on A_F, verbatim: "Keep A_F's output vocabulary to one and two-step quantities and say so as a design decision rather than a limitation... Anything needing three or more chained operations lands in the 22.78% band, and the honest move is to not ask the channel for those at all rather than to ask and then discover the error rate in the backtest." On C_{F,t}, verbatim: "The retrieve-then-program design is the first concrete answer I have to how C_{F,t} gets computed. A program is checkable in ways free text is not: whether it parses under the grammar, whether every argument traces to a retrieved number or row rather than being invented, how many retries the retriever needed, and how many steps the program has. That last one is a calibrated difficulty proxy on this evidence, since accuracy runs 67.61%, 59.08% and 22.78% across one, two and three-plus steps, so step count is a feature the orchestrator can read without asking the model how sure it is. This pushes the standing open question about comparable confidence forward for one of the four producers, and it is a different mechanism from the Cypher-validation signal in the Graph-RAG note, which is useful because two mechanical signals on the same channel can be cross-checked." Also: "design the orchestrator to tolerate a channel that is wrong a lot" - expectation "nearer 40% than 60% on first build".</t>
+PROPOSED REVISION STATED IN THE NOTE: No change to the agent pool. Scope decision on A_F, verbatim: "Keep A_F's output vocabulary to one and two-step quantities and say so as a design decision rather than a limitation... Anything needing three or more chained operations lands in the 22.78% band, and the honest move is to not ask the channel for those at all rather than to ask and then discover the error rate in the backtest." On C_{F,t}, verbatim: "The retrieve-then-program design is the first concrete answer I have to how C_{F,t} gets computed. A program is checkable in ways free text is not: whether it parses under the grammar, whether every argument traces to a retrieved number or row rather than being invented, how many retries the retriever needed, and how many steps the program has. That last one is a calibrated difficulty proxy on this evidence, since accuracy runs 67.61%, 59.08% and 22.78% across one, two and three-plus steps, so step count is a feature the orchestrator can read without asking the model how sure it is. This pushes the standing open question about comparable confidence forward for one of the four producers, and it is a different mechanism from the Cypher-validation signal in the Graph-RAG note, which is useful because two mechanical signals on the same channel can be cross-checked." Also: design the orchestrator to tolerate a channel that is wrong a lot - expectation "nearer 40% than 60% on first build".</t>
         </is>
       </c>
       <c r="X52" s="11" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="R53" s="11" t="inlineStr">
         <is>
-          <t>Inherited baselines STM (spurious tokens masking, Wang et al. 2022) and CDA (counterfactual data augmentation, Wang and Culotta 2021); both fail. Model-free shift evidence: sentiment positivity #pos/(#pos+#neg) per month vs monthly returns, "Spearman correlation of 0.397 for Apple and 0.459 for Tesla". KEY RESULTS - SENTIMENT DECAY WITH NUMBERS (this is the extraction the standing rule asks for): - "Every fine-tuned model degrades... All ΔF1 values for fine-tuned models in Table 1 are positive." - Aggregate: "BERT at NDNM losing 4.70 F1 points and RoBERTa 3.96". - Minority class: "BERT's negative-class ΔF1 under NDNM is 8.27 against 1.13 for the positive class, and logistic regression loses 10.04 points on the negative class against 1.07 on the positive. The bearish label is the minority in a corpus that is mostly bullish, and it is the one that stops generalising first. Up-sampling the minority class, reported in their Appendix A, does not change this conclusion." - Retraining trade: "NDOM has the best in-sample performance everywhere it applies, BERT at 79.1 average F1_in against 72.5 for NDNM and 67.4 for ODNM, and RoBERTa at 80.4, but it carries a ΔF1 of 3.31 and 2.45 respectively. ODNM inverts this completely, with the smallest drops in the table, 1.19 for BERT, 0.97 for RoBERTa, 1.00 for FinBERT, on top of the weakest in-sample scores." - GPT-3.5: "a ΔF1 of −1.10 with F1_in of 66.4 and F1_out of 67.5, flat and weak", and "its pretraining corpus covers 2014 to 2017 so these months may not be out of distribution for it at all, which makes the flat line uninterpretable as evidence about model scale." - Shift correlation: "Spearman correlations between ΔF1 and the token-level KL shift come out at 0.385 for BERT (p = 0.020), 0.345 for RoBERTa (p = 0.039) and 0.281 for FinBERT (p = 0.096)." - Spurious features: "Fitting logistic regression to the full corpus and reading off the 30 largest absolute coefficients returns a list where the genuine sentiment words, bears, bulls, fall, dump, strong, shorts, squeeze, are a minority among ticker fragments and company names, incbr, nakd, plx, owens, caterpillar, kellogg, pharmaceuticals... a model predicting p(y|v) for v = 'Tesla' is not doing sentiment analysis, it is memorising the market's current opinion of Tesla, and it fails the moment that opinion turns." - Mitigation: "the method reduces ΔF1 by 31% for BERT (2.05 to 1.42), 26% for RoBERTa (1.62 to 1.26) and 32% for FinBERT (2.01 to 1.36)... Expressed as out-of-sample F1 the same result is a gain of 0.63, 0.36 and 0.65 points. Both inherited baselines make things worse: STM costs BERT 2.09 points of F1_in and raises its ΔF1, and CDA costs FinBERT 3.54 points." - Detector: "OOD recall of 0.86 for BERT and 0.91 for FinBERT at OOD precision of 0.23 and 0.15." - NO MECHANISM TO NOTICE: nothing in the corpus or the model signals the decay. Verbatim: "A component whose largest learned coefficients sit on ticker fragments and company names is one whose apparent skill is a memorised snapshot of market opinion, and nothing in the system notices when that snapshot expires." LIMITATIONS (quoted): "There is no ablation separating the detector from the ensemble, which leaves the paper's own mechanism unestablished... without it the claim that OOD detection is what produces the gain is the paper's interpretation of a result rather than a result. This is the first thing I would raise about the paper." "ΔF1 rewards a model that is uniformly mediocre, and the paper's own table shows it... GPT-3.5 wins the metric outright by being flat and weak." "The shift measure weights tokens by conditional label probability rather than by frequency, and it is estimated over a subword vocabulary... the statistic is dominated by the sparse tail... the estimator's behaviour in the tail is load-bearing." "The labels are self-declared directional tags on a social platform, so label shift and market regime are entangled by construction." "One platform, one language, one market, three years, and no significance testing on the result that matters." "Nothing connects the performance drop to money". Also, on the data figure: "The monotone drift in the top panel is the number of examples per month rising steadily over the three years, so the later months carry far more data than the earlier ones and the rolling experiment is not comparing like with like across time, which the paper does not remark on."</t>
+          <t>Inherited baselines STM (spurious tokens masking, Wang et al. 2022) and CDA (counterfactual data augmentation, Wang and Culotta 2021); both fail. Model-free shift evidence: sentiment positivity #pos/(#pos+#neg) per month vs monthly returns, "Spearman correlation of 0.397 for Apple and 0.459 for Tesla". KEY RESULTS - SENTIMENT DECAY WITH NUMBERS (this is the extraction the standing rule asks for): - Every fine-tuned model degrades... All ΔF1 values for fine-tuned models in Table 1 are positive. - Aggregate: "BERT at NDNM losing 4.70 F1 points and RoBERTa 3.96". - Minority class: BERT's negative-class ΔF1 under NDNM is 8.27 against 1.13 for the positive class, and logistic regression loses 10.04 points on the negative class against 1.07 on the positive. The bearish label is the minority in a corpus that is mostly bullish, and it is the one that stops generalising first. Up-sampling the minority class, reported in their Appendix A, does not change this conclusion. - Retraining trade: NDOM has the best in-sample performance everywhere it applies, BERT at 79.1 average F1_in against 72.5 for NDNM and 67.4 for ODNM, and RoBERTa at 80.4, but it carries a ΔF1 "of 3.31 and 2.45 respectively. ODNM inverts this completely, with the smallest drops in the table, 1.19 for BERT, 0.97 for RoBERTa, 1.00 for FinBERT, on top of the weakest in-sample scores." - GPT-3.5: a ΔF1 of −1.10 with F1_in of 66.4 and F1_out of 67.5, flat and weak, and its pretraining corpus covers 2014 to 2017 so these months may not be out of distribution for it at all, which makes the flat line uninterpretable as evidence about model scale. - Shift correlation: Spearman correlations between ΔF1 and the token-level KL shift come out at 0.385 for BERT (p = 0.020), 0.345 for RoBERTa (p = 0.039) and 0.281 for FinBERT (p = 0.096). - Spurious features: Fitting logistic regression to the full corpus and reading off the 30 largest absolute coefficients returns a list where the genuine sentiment words, bears, bulls, fall, dump, strong, shorts, squeeze, are a minority among ticker fragments and company names, incbr, nakd, plx, owens, caterpillar, kellogg, pharmaceuticals... a model predicting p(y|v) for v = 'Tesla' is not doing sentiment analysis, it is memorising the market's current opinion of Tesla, and it fails the moment that opinion turns. - Mitigation: the method reduces ΔF1 by 31% for BERT (2.05 to 1.42), 26% for RoBERTa (1.62 to 1.26) and 32% for FinBERT (2.01 to 1.36)... Expressed as out-of-sample F1 the same result is a gain of 0.63, 0.36 and 0.65 points. Both inherited baselines make things worse: STM costs BERT 2.09 points of F1_in and raises its ΔF1, and CDA costs FinBERT 3.54 points. - Detector: "OOD recall of 0.86 for BERT and 0.91 for FinBERT at OOD precision of 0.23 and 0.15." - NO MECHANISM TO NOTICE: nothing in the corpus or the model signals the decay. Verbatim: A component whose largest learned coefficients sit on ticker fragments and company names is one whose apparent skill "is a memorised snapshot of market opinion, and nothing in the system notices when that snapshot expires." LIMITATIONS (quoted): "There is no ablation separating the detector from the ensemble, which leaves the paper's own mechanism unestablished... without it the claim that OOD detection is what produces the gain is the paper's interpretation of a result rather than a result". This is the first thing I would raise about the paper. ΔF1 "rewards a model that is uniformly mediocre, and the paper's own table shows it... GPT-3.5 wins the metric outright by being flat and weak." The shift measure weights tokens by conditional label probability rather than by frequency, and it is estimated over a subword vocabulary... the statistic is dominated by the sparse tail... the estimator's behaviour in the tail is load-bearing. "The labels are self-declared directional tags on a social platform, so label shift and market regime are entangled by construction." "One platform, one language, one market, three years, and no significance testing on the result that matters." "Nothing connects the performance drop to money". Also, on the data figure: "The monotone drift in the top panel is the number of examples per month rising steadily over the three years, so the later months carry far more data than the earlier ones and the rolling experiment is not comparing like with like across time, which the paper does not remark on."</t>
         </is>
       </c>
       <c r="S53" s="11" t="inlineStr">
@@ -7234,8 +7234,8 @@
       <c r="W53" s="11" t="inlineStr">
         <is>
           <t>SPEAKS TO: The orchestrator primarily, plus every fitted agent (A_T, A_V, A_L and A_F via refit policy), plus the evaluation layer. Not a text-modality paper for A_F, since A_F's text is filings not social posts.
-EFFECT ON A_F: Indirect. It constrains the refit policy for any fitted component and it supplies the competence-gap construction that C_{F,t} sits inside, but it offers no evaluation set or taxonomy for CSE filings. SENTIMENT-RELATED EVIDENCE (the standing rule): The note applies the rule explicitly. Verbatim: "It is the cleanest citation I have for why sentiment was investigated and then excluded from scope. Under the Literature Matrix exception this paper stays in as evidence the area was examined: a dedicated financial sentiment model, fine-tuned on 418,893 in-domain messages, degrades by 8 F1 points on its minority class from one month to the next, leans on tokens with no sentiment content, and needs a second system bolted on to recover a fraction of a point. That is a component with a maintenance burden and a measurable decay rate, and the attribution argument in the scope note applies with force: a 5% return improvement out of a system containing this could not be traced to anything." And: "The spurious-correlation table is a third documented fixed-influence failure case and it is directly citable in the review chapter... That is the same structure as FinAgent's auxiliary strategies returning 16% against buy-and-hold's 29% and AlphaAgents dropping its sentiment agent for insufficient coverage, and the three together make the fixed-influence argument from three different directions rather than one." Note that the paper's own mitigation is the "mechanism to notice" - an OOD detector running at 0.15–0.23 precision, i.e. wrong roughly three times in four.
-PROPOSED REVISION STATED IN THE NOTE: This is the only note of the seven that proposes a change to the conditioning set. Verbatim: "The shift-detection idea belongs in the conditioning set as a candidate, and the detector's precision is the warning that comes with it. L_t, V_t, P_t and C_{i,t} are a hypothesis about what weighting should respond to, and this paper suggests a fifth candidate, a direct estimate of how far the current input distribution has moved from the one the components were fitted on. The evidence for it is moderate, a ρ of roughly 0.3 to 0.39, and the detector built on it runs at 0.15 to 0.23 precision, so a naive port would have the orchestrator re-weighting on a signal that is wrong three times out of four. If I test a shift input, it gets tested against the always-blend control this paper skipped, and I should expect to report that it does not earn its slot." On C_{i,t}, verbatim: "for any component that emits a prediction with a later-observable outcome, the gap between its fitted-period accuracy and its next-period accuracy is computable without knowing anything about how it works. Applied per agent and rolled forward, that gives A_T, A_V, A_L and A_F a comparable backward-looking competence estimate on the same footing as the p_T construction from the HLOB note. The caution travels with it: a gap metric alone ranks a uniformly weak agent above a strong but drifting one, so the orchestrator needs level and gap jointly, not the difference on its own." On baselines, verbatim: "a static learned weight over agents is one control, and a recency-weighted combination that ignores market state entirely is a second, cheaper one that my state-conditional weighting has to beat before the conditioning set earns its place." No change to the four-agent pool is proposed in any of the seven notes.</t>
+EFFECT ON A_F: Indirect. It constrains the refit policy for any fitted component and it supplies the competence-gap construction that C_{F,t} sits inside, but it offers no evaluation set or taxonomy for CSE filings. SENTIMENT-RELATED EVIDENCE (the standing rule): The note applies the rule explicitly. Verbatim: It is the cleanest citation I have for why sentiment was investigated and then excluded from scope. Under the Literature Matrix exception this paper stays in as evidence the area was examined: a dedicated financial sentiment model, fine-tuned on 418,893 in-domain messages, degrades by 8 F1 points on its minority class from one month to the next, leans on tokens with no sentiment content, and needs a second system bolted on to recover a fraction of a point. That is a component with a maintenance burden and a measurable decay rate, and the attribution argument in the scope note applies with force: a 5% return improvement out of a system containing this could not be traced to anything. And: The spurious-correlation table is a third documented fixed-influence failure case and it is directly citable in the review chapter... That is the same structure as FinAgent's auxiliary strategies returning 16% against buy-and-hold's 29% and AlphaAgents dropping its sentiment agent for insufficient coverage, and the three together make the fixed-influence argument from three different directions rather than one. Note that the paper's own mitigation is the "mechanism to notice" - an OOD detector running at 0.15–0.23 precision, i.e. wrong roughly three times in four.
+PROPOSED REVISION STATED IN THE NOTE: This is the only note of the seven that proposes a change to the conditioning set. Verbatim: "The shift-detection idea belongs in the conditioning set as a candidate, and the detector's precision is the warning that comes with it. L_t, V_t, P_t and C_{i,t} are a hypothesis about what weighting should respond to, and this paper suggests a fifth candidate, a direct estimate of how far the current input distribution has moved from the one the components were fitted on. The evidence for it is moderate, a ρ of roughly 0.3 to 0.39, and the detector built on it runs at 0.15 to 0.23 precision, so a naive port would have the orchestrator re-weighting on a signal that is wrong three times out of four. If I test a shift input, it gets tested against the always-blend control this paper skipped, and I should expect to report that it does not earn its slot." On C_{i,t}, verbatim: for any component that emits a prediction with a later-observable outcome, the gap between its fitted-period accuracy and its next-period accuracy is computable without knowing anything about how it works. Applied per agent and rolled forward, that gives A_T, A_V, A_L and A_F a comparable backward-looking competence estimate on the same footing as the p_"T construction from the HLOB note. The caution travels with it: a gap metric alone ranks a uniformly weak agent above a strong but drifting one, so the orchestrator needs level and gap jointly, not the difference on its own." On baselines, verbatim: "a static learned weight over agents is one control, and a recency-weighted combination that ignores market state entirely is a second, cheaper one that my state-conditional weighting has to beat before the conditioning set earns its place." No change to the four-agent pool is proposed in any of the seven notes.</t>
         </is>
       </c>
       <c r="X53" s="11" t="inlineStr">
@@ -7306,8 +7306,8 @@
 τ_t = 0 if h_t = l_t = c_{t−1}, and 1 otherwise.
 τ_t = 0 flags the case where high, low and previous close all coincide, meaning either that every trade in the period executed at the previous closing price - "which becomes increasingly likely as trades per period fall" - or that there was no trading at all and the four prices were filled forward. Setting τ_t = 0 on those periods prevents the estimator from treating a forward-filled price as evidence about the spread, and conditioning every expectation on τ_t = 1 is what makes the derivation go through without assuming continuous observation.
 The spread estimator measured at the open:
-S_o² = −8·E[(η̄_t − ō_t)(o_t − c_{t−1})] / ( P[o_t ≠ h_t, τ_t = 1] + P[o_t ≠ l_t, τ_t = 1] )
-where bars denote de-meaned returns, r̄_t = r_t − τ_t·E[r_t]/E[τ_t], "which is the de-meaning that survives the conditioning on τ_t". The denominator is the entire discreteness correction and is the only thing separating this from the classical form: if prices are observed continuously the open and close can never coincide with the high or low, both probabilities equal one, the denominator collapses to two, and the expression reverts to the familiar −4E[·] shape.
+S_o² = −8·E[(η̄_t − ō_t)(o_t − c_{t−1})] / (P[o_t ≠ h_t, τ_t = 1] + P[o_t ≠ l_t, τ_t = 1])
+where bars denote de-meaned returns, r̄_t = r_t − τ_t·E[r_t]/E[τ_t], which is the de-meaning that survives the conditioning on τ_t. The denominator is the entire discreteness correction and is the only thing separating this from the classical form: if prices are observed continuously the open and close can never coincide with the high or low, both probabilities equal one, the denominator collapses to two, and the expression reverts to the familiar −4E[·] shape.
 The note's reading: "The correction is therefore not a robustness patch bolted onto an existing estimator, it is a term that is identically one under the old assumption and shrinks the denominator, inflating the spread estimate, exactly in proportion to how often the price failed to move within the period."
 The same construction over other price combinations gives four Discrete Generalized Estimators - OHL, CHL, OHLC and CHLO - the first pair measuring the spread at the open and the second at the close. Their CHL estimator reduces exactly to the Abdi and Ranaldo (2017) estimator when continuous observation is imposed and returns are zero-mean, "so the prior work is recovered as a special case rather than contradicted."
 Efficiency half: the four estimators behave in opposite ways - when the spread is small relative to volatility the estimators using the mid-price have lower variance, and when the spread is large and observed returns are driven by bid–ask bounces, pairing mid-to-open with open-to-mid returns cancels a variance term that pairing with the closing price does not. Combining OHL with CHLO and OHLC with CHLO gives two moment conditions, and GMM with a diagonal weighting matrix reduces to a variance-weighted average:
@@ -7369,17 +7369,17 @@
 3.00% | 2.89 (0.83) | 2.76 (1.23) | 2.86 (1.19) | 2.26 (0.92) | 0.35 (0.36) | 2.89 (1.82)
 8.00% | 8.19 (0.96) | 8.10 (1.59) | 8.20 (1.26) | 6.59 (0.94) | 2.66 (0.96) | 7.71 (2.65)
 EDGE is within 0.21 of the true value at every spread size while AR is 1.41 low at 8.00% and CS is 5.34 low, and EDGE's standard deviation is the smallest or tied at every row. CS's small standard deviations are "the collapse to zero rather than precision". The uniformity comes from the building blocks swapping roles, OHLC and CHLO carrying lower variance for small spreads and OHL and CHL for large, with EDGE shifting weight between them rather than being tuned to a favoured region.
-3. Empirical dominance, widest where trading is thinnest. Against the TAQ benchmark EDGE achieves Pearson 78.86%, Spearman 66.68%, MAPE 16.21, RMSE 1.23, non-positive estimates 25.63% - against AR at 68.13 / 53.55 / 19.90 / 1.41 / 31.87 and CS at 45.55 / 33.77 / 35.90 / 2.61 / 29.18. EDGE is highest in every market venue, sub-period, size quintile, spread quintile and trading-frequency quintile. On the trading-frequency cut, EDGE scores 74.77% in the least-traded quintile falling to 55.48% in the most-traded, while ROLL runs the other way at 65.10% down to 22.29% and AR falls from 67.81% to 39.36%. The size-decile plot has the same shape, EDGE flat near 70% across all ten deciles while the others spread out below it. "The lead is therefore not an average that washes out in the hard cases, it is largest in the hard cases, which is the property a frontier-market application needs."
+3. Empirical dominance, widest where trading is thinnest. Against the TAQ benchmark EDGE achieves Pearson 78.86%, Spearman 66.68%, MAPE 16.21, RMSE 1.23, non-positive estimates 25.63% - against AR at 68.13 / 53.55 / 19.90 / 1.41 / 31.87 and CS at 45.55 / 33.77 / 35.90 / 2.61 / 29.18. EDGE is highest in every market venue, sub-period, size quintile, spread quintile and trading-frequency quintile. On the trading-frequency cut, EDGE scores 74.77% in the least-traded quintile falling to 55.48% in the most-traded, while ROLL runs the other way at 65.10% down to 22.29% and AR falls from 67.81% to 39.36%. The size-decile plot has the same shape, EDGE flat near 70% across all ten deciles while the others spread out below it. The lead is therefore not an average that washes out in the hard cases, it is largest in the hard cases, which is the property a frontier-market application needs.
 4. Sampling frequency beats sampling length by three orders of magnitude. Standard error scales as σ₁²/√N. Going from a monthly sample of daily prices (N = 21) to a yearly one (N = 252) reduces the standard error by √(252/21) = 3.5 times; going instead to a monthly sample of minute prices (N = 21 × 390) reduces it by 390^{3/2} = 7702 times, which the authors note would take 1,245,699,037 daily prices to match, roughly five million years of trading. Empirically, on 711,161 stock-months, moving from daily to minute prices: negative estimates fall from 34.15% to 0.02%, Pearson rises from 56.17% to 88.79%, Spearman from 43.47% to 97.31%, MAPE from 23.68 to 5.17. The crypto application makes the point from the other side: AR and CS differ roughly tenfold between daily and minute sampling (0.18% against 0.02%, and 1.85% against 1.45% respectively) while EDGE stays within 0.68% to 0.70% at every frequency, "so the frequency-insensitivity is a property of the estimator rather than of the US sample."
 5. The discreteness term is itself a market-structure measurement: the coincidence probability ranges from ~25% (US large-cap) to 75% (small-cap) over 1926–2021, peaking in the 1930s - 40s, collapsing after 2000 to 2–5% for large-caps with small-caps still near 15%.</t>
         </is>
       </c>
       <c r="T54" s="9" t="inlineStr">
         <is>
-          <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% - "a bias roughly seven times the quantity being measured" - and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for Ŝ² and not for the Ŝ anyone actually uses."
+          <t>1. The non-negativity truncation is reduced rather than solved, and the residual upward bias is largest precisely where spreads are smallest. 25.63% of EDGE estimates from daily prices are non-positive in the merged sample, and in the large-cap experiment 41% of stock-months come out negative before truncation. The authors report that EDGE averages 0.42% for large-caps in December 2021 against a benchmark of 0.06% - "a bias roughly seven times the quantity being measured" - and attribute it correctly to small-sample truncation. The two mitigations they name, taking √|Ŝ²| minus the expected spread under negative estimates, and using the tick size as a lower bound, "are both explicitly left to future research and neither is evaluated anywhere in the paper." The practical remedies offered are to widen the estimation window or use intraday prices, "both of which cost something I may not be able to pay. So the estimator's headline property, unbiasedness, holds for" Ŝ² and not for the Ŝ anyone actually uses.
 2. The three assumptions are weaker than the prior literature's but still exclude the frictions that characterise a thin book, and none of them is tested against data. Assumption 1 rules out serially correlated fundamental returns, which sits uneasily beside the long-memory results on the ASPI and SL20 in the CSE volatility-memory note (though that tension is about return persistence rather than volatility persistence, and the note says it "would want to test rather than assert it"). Assumption 3 requires bid–ask bounces to be uncorrelated with zero mean, which rules out order-flow persistence, and the authors are explicit that work letting bounces carry information - Chen et al. (2017) being their example - is outside scope. "The assumptions are inherited from the literature and weakened, which is a real contribution but not an empirical validation."
 3. No order size anywhere in the model. For a deep market the marginal-trade cost is close enough; "for a book where a single order can be a meaningful fraction of daily volume it is the intercept of a cost function and not the function." The scope is honest and never overclaimed, but EDGE answers only the first of the four open items in my cost work and leaves the nonlinear impact form, the participation-rate sweep and the thin-book depth calibration untouched.
-4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden–Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility - "plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation." The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
+4. The benchmark is a US quote-based construct; the degradation over time is unexplained in the direction that matters; and the one genuinely illiquid application has no benchmark at all. Correlation with Holden–Jacobsen falls monotonically from 82.93% in 1993–1996 to 53.98% in 2016–2021, attributed to spreads shrinking relative to volatility - plausible and consistent with the spread-quintile table... but it is an interpretation of a pattern rather than a tested explanation. The crypto section has no benchmark whatsoever, the authors stating plainly that trade and quote data are unavailable to them, "so what it demonstrates is internal consistency across sampling frequencies and not accuracy." The note records: "I have not found a validation of EDGE against a quote-based benchmark in any emerging or frontier market in the literature I have covered."
 5. The estimator needs at least three usable observations per stock-month and the paper never reports performance conditional on a small count. Periods with τ_t = 0 are excluded, and EDGE is missing in 1.24% of CRSP stock-months on that basis. "The thinnest cut they report is the bottom trading-frequency quintile of US-listed stocks, which still trades most days. For a counter with five trading days in a month the estimator is defined and will return a number computed from a handful of covariance terms, deep inside the small-sample regime where their own truncation bias is worst, and nothing in the paper tells me how that number behaves. That is the gap between what the paper validates and what I would be doing with it."
 6. The simulation's "infrequent trading" is not frontier-market infrequent. Panel B sets the daily trade probability to 1%, which on a 390-minute day means roughly four expected trades per day, and the bias plot extends down to one trade per day. "That is thin by US standards and it is the right stress test for the method, but a CSE counter in the bottom half of a liquidity screen can go whole days without a trade, and the paper's design forward-fills those days rather than modelling a counter that trades on five days in a month. The estimator handles the forward-fill correctly through its indicator; what is untested is the regime where the number of usable observations per stock-month falls into single digits."
 7. A premise doing quiet work throughout: that the effective spread is the whole of the transaction cost, since nothing in the model has an order size in it. The paper never claims otherwise and the title is honest about scope.</t>
@@ -7402,7 +7402,7 @@
 --- RETAINED AS RECORD, SUPERSEDED ---
 - EDGE itself, as the measurement half of the cost model, computed per counter per period from daily OHLC - the one data type I am certain the CSE publishes for every listed counter, with no quote feed and no vendor dependency. The concrete step: compute EDGE over the 374-day per-counter archive and use it as the spread term in the cost function, "so the constant becomes a measured number that varies by counter and by date, which is the minimum needed before any statement about cost-aware allocation means anything on this market."
 - The infrequent-trading bias result as external evidence that thin-book calibration is a real problem, not a rhetorical one: below roughly thirteen trades per day CS returns exactly zero and AR is biased down by about a third at a few trades per day, "which means any cost model built on those estimators would charge approximately nothing for trading the least liquid counters on the CSE. That is backwards in the most expensive possible direction." Worth citing directly in the proposal when defending the thin-book calibration item.
-- Two new candidate inputs to the liquidity state L_t. (a) The measured spread itself, which unlike Amihud (price impact per unit volume), turnover (activity) and zero-return frequency (staleness) "is denominated in the same units as the objective". (b) The τ_t indicator - the fraction of days on which the open or close coincides with the high or low - which "falls out of the EDGE computation at no extra cost" and is a candidate staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both go into the ablation protocol "as additions to test rather than adopt".
+- Two new candidate inputs to the liquidity state L_t. (a) The measured spread itself, which unlike Amihud (price impact per unit volume), turnover (activity) and zero-return frequency (staleness) is "denominated in the same units as the objective". (b) The τ_t indicator - the fraction of days on which the open or close coincides with the high or low - which "falls out of the EDGE computation at no extra cost" and is a candidate staleness measure "with a cleaner interpretation than zero-return frequency, since it does not require the price to be literally unchanged and so separates a counter that traded in a narrow range from one that did not trade at all." Both go into the ablation protocol "as additions to test rather than adopt".
 - A forced window decision. Given 25.63% non-positive daily-price estimates on CRSP and 41% negative for large-caps, and a monthly estimate from the per-counter archive being roughly 21 observations - "squarely in that regime" - the decision is a quarterly window on the per-counter track, accepting a cost term that cannot move within a quarter, and monthly on the index track where ten years of daily data supports it, "with the fraction of non-positive estimates reported alongside every spread series in both cases. Reporting that fraction is not optional here, it is the only visible signal that the truncation is distorting the number."
 - A reversal of my data priority. A month of minute prices gives a standard error 7702 times smaller than a month of daily prices, where a year of daily prices gives only 3.5 times. "So if any intraday CSE feed exists at any granularity, even hourly or five-minute, it is worth far more to the cost model than extending the daily archive backwards." This is a question to put to the supervisor before spending time on data depth, and it connects to the volatility estimator decision too, "since the same constraint that rules out five-minute realised volatility on this market is what would rule out minute-frequency EDGE."
 - A positioning rule. EDGE is a 2024 JFE paper with public implementations, open spread data and a replication package, "so there is no contribution in running it on a new market and no reason to imply one." The defensible sentence is that I have not found an application or validation of EDGE on the CSE or any comparable frontier market in the literature I have covered, and that the contribution is what an orchestrator does with a cost term that varies by counter and date rather than the estimator that produces it. "One sentence, offered before anyone asks."</t>
@@ -7515,13 +7515,13 @@
 Combining by learning | A meta-model over features of the series and of the method pool | A dataset of many series | 2.4
 OPTIMAL WEIGHTS (Bates and Granger 1969 for pairs, Newbold and Granger 1974 in general) minimise the variance of the combined forecast error:
 w^opt_{T+h|T} = Σ⁻¹_{T+h|T} 1 / (1' Σ⁻¹_{T+h|T} 1)
-with Σ the N×N covariance matrix of h-step forecast errors. If the individuals are unbiased and their error variances stable, the combination is unbiased and its error variance is no greater than the minimum across individuals - "the diversification result the whole field rests on. The catch is in the last sentence of that passage: in practice Σ is unknown and has to be estimated, and that single sentence generates most of the rest of the literature."
+with Σ the N×N covariance matrix of h-step forecast errors. If the individuals are unbiased and their error variances stable, the combination is unbiased and its error variance is no greater than the minimum across individuals - "the diversification result the whole field rests on. The catch is in the last sentence of that passage": in practice Σ is unknown and has to be estimated, and that single sentence generates most of the rest of the literature.
 REGRESSION WEIGHTS (Granger and Ramanathan 1984): three regimes - weights summing to one with no intercept, which reproduces Bates–Granger exactly; unconstrained with no intercept; and unconstrained with an intercept, which they argued is superior regardless of whether constituents are biased because the intercept absorbs the bias. De Menezes et al. (2000) push back that the unrestricted version needs stationarity and runs into serial correlation and multicollinearity. Aksu and Gunter (1992) found empirically that constraining weights to be nonnegative is at least as robust as the simple average while beating the other regression variants - "which is the practical reading I'd take."
 PERFORMANCE-BASED, discounted variant (the one with a time dimension, and the one the note would implement first because it needs no pairwise estimation):
-w^{bg4}_{T+h|T,i} = ( Σ_{t=1}^{T} γ^t e²_{t|t−h,i} )⁻¹ / Σ_{j=1}^{N} ( Σ_{t=1}^{T} γ^t e²_{t|t−h,j} )⁻¹ , γ ≥ 1
+w^{bg4}_{T+h|T,i} = (Σ_{t=1}^{T} γ^t e²_{t|t−h,i})⁻¹ / Σ_{j=1}^{N} (Σ_{t=1}^{T} γ^t e²_{t|t−h,j})⁻¹, γ ≥ 1
 where e_{t|t−h,i} is the h-step error of method i made at t−h and realised at t, and γ controls how fast older errors are forgotten, with γ = 1 recovering the plain inverse-MSE weight over the full history. The rolling-window variant replaces the discount with a sum over the most recent ν observations. Both are adapted to non-stationary relationships between methods, and both, as Timmermann (2006) is quoted saying, "increase the variance of the parameter estimates and work quite poorly if the data generating process really is covariance stationary." Stock and Watson (1998) generalise by making weights inversely proportional to the kth power of MSE, so k=0 is equal weights and larger k concentrates on the best performer - "a single interpretable dial between the two extremes."
 TIME-VARYING WEIGHTS: Diebold and Pauly (1987) use rolling weighted least squares and time-varying parameters that are either deterministic polynomial functions of time or stochastic; Deutsch et al. (1994) let weights switch abruptly or transition smoothly using switching and smooth transition regression; Terui and van Dijk (2002) model the coefficients as a random walk in state space estimated by the Kalman filter, with Raftery et al. (2010) adding forgetting factors to make the recursive update cheap.
-The note's key structural observation: "So the literature already contains weights that change over time, and it contains weights that change as a regression function of covariates, and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state. The closest thing is the smooth transition specification of Deutsch et al., where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step."
+The note's key structural observation: So the literature already contains weights that change over time, and it contains weights that change as a regression function of covariates, and what it does not contain, anywhere in this review, is weights that are a function of measured exogenous market state. "The closest thing is the smooth transition specification of Deutsch et al., where the transition variable could in principle be exogenous, and FFORMA, where the features are properties of the series itself computed once rather than a state measured at each step."
 COMBINING BY LEARNING: stacking series-by-series needs n meta-models for n series, "computationally expensive and wastes the training data". Cross-learning trains one meta-model across many series. M4 is the evidence: "the top three methods all used information across the whole dataset rather than a single series." FFORMA is the exemplar - 42 tsfeatures features, XGBoost meta-model mapping features to weights over nine traditional models fitted per series, second place in M4.
 PROBABILISTIC COMBINATION: the linear opinion pool is a finite mixture F̃(y_{T+h}|I_T) = Σ w_{T+h|T,i} F_i(y_{T+h}|I_T) with nonnegative weights summing to one. Its first two moments:
 μ̃ = Σ w_i μ_i and σ̃² = Σ w_i σ_i² + Σ w_i (μ_i − μ̃)²
@@ -7595,7 +7595,7 @@
           <t>- A lineage and a precise statement of what is new, which the note judges "a stronger framing than novelty". My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) is a time-varying feature-conditioned linear combination, and the paper contains both halves separately: time-varying weights through the Kalman-filter and smooth-transition line, feature-conditioned weights through FFORMA. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That reads as a generalisation along an identified axis rather than new machinery. It also tells me what the honest comparison is: FFORMA's structure - a gradient-boosted meta-model mapping features to a weight simplex - is available to me as an implementation choice, "and if I use something simpler I should say why rather than let it look like I did not know."
 - The hardest possible equal-weight baseline, plus a falsification condition to pre-register.
 - A five-decade justification for having no pairwise interaction term in the weighting function. "With four agents that is ten parameters against four, from 374 days, so the argument has real force here. This is worth stating explicitly in the write-up, because a reviewer will ask why there is no interaction term, and the answer is that the literature tried that first and moved away from it."
-- Two cheap intermediate baselines: the Stock and Watson inverse-kth-power family (a one-parameter dial from k=0 equal weights to winner-take-all, "a sweep over k maps the whole continuum... for almost no implementation cost"), and the discounted inverse-MSE scheme, "which adds a time dimension without adding state" - the one the note names as "the baseline that actually threatens my contribution". So the planned three-way comparison (equal weights vs static learned weights vs state-conditioned weights) becomes four-way with a discounted performance-weighting arm.
+- Two cheap intermediate baselines: the Stock and Watson inverse-kth-power family (a one-parameter dial from k=0 equal weights to winner-take-all, "a sweep over k maps the whole continuum... for almost no implementation cost"), and the discounted inverse-MSE scheme, which adds a time dimension without adding state - the one the note names as "the baseline that actually threatens my contribution". So the planned three-way comparison (equal weights vs static learned weights vs state-conditioned weights) becomes four-way with a discounted performance-weighting arm.
 - An oracle-weight arm, weights fitted on the test window itself rather than on training, "because the gap between oracle and estimated performance is the estimation cost measured in my own data and in my own units: no gain under oracle weights means the conditioning hypothesis is simply wrong, a gain under oracle but not under estimated weights means it is an estimation problem I can put a number on, and it costs one further pass of the same pipeline."
 - Vocabulary for the abstention channel: time-varying subset selection via a pre-set threshold on a time-varying weighting scheme (Li et al., 2022). Plus Geweke and Amisano's observation that individually poor forecasts may still help in combination and one does not want to zero-weight them - "an argument for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero, which is a concrete design decision I had not settled."
 - An operational definition of diversity (low correlation among forecast errors, with Lemke and Gabrys' six diversity features and Thomson et al.'s coherence measure as alternatives), making my heterogeneity claim testable on my own pool.
@@ -7619,16 +7619,16 @@
 The legitimising half. My w_{i,t} = f(L_t, V_t, P_t, C_{i,t}) stops being an invention and becomes a named construct with a lineage: a time-varying, feature-conditioned linear combination. The review contains time-varying weights (Diebold and Pauly, Deutsch et al., Terui and van Dijk's Kalman-filter random walk, Raftery et al.'s forgetting factors) and it contains feature-conditioned weights (FFORMA). What it does not contain, anywhere, is weights that are a function of measured exogenous market state. FFORMA is the nearest named ancestor and the difference is one sentence: "its 42 features are properties of the series itself, computed once from the history, while mine are properties of the market state, measured at each step and exogenous to the agent being weighted." That is a generalisation along an identified axis, which is a stronger and more defensible framing than novelty - and it is the framing the orchestration note already used. It also obliges me to be honest about implementation: FFORMA's gradient-boosted-meta-model-to-weight-simplex structure is available to me, and if I use something simpler I should say why.
 The threatening half, and it is serious. The forecast combination puzzle says that fifty years of evidence finds the equally weighted average extremely hard to beat, and that sophisticated weighting schemes lose because of estimation error. In M4, "a simple equal-weight combination ranked third for yearly series and a median of four simple models took sixth place overall for point forecasting". Gastinger et al. (2021) across M3, M4, M5 and FRED find simple averaging shows, on average, more gain than complex methods. Elliott (2011) bounds the available gain from optimal over equal weights and finds it usually too small to pay for the estimation. Claeskens et al. (2016) prove random weights can introduce bias into combinations of unbiased components and inflate variance past the fixed-weight case. And the probabilistic side produces the same pattern independently: Baran and Lerch (2018) found no substantial difference between the simple linear pool and the theoretically superior nonlinear alternatives. "That is the probabilistic restatement of the puzzle, which makes it two independent appearances of the same pattern in one paper."
 Worse for me specifically: everything the paper says about estimation error swamping the gains from optimal weights "gets worse in my setting, not better", because my components are themselves estimated on short, illiquid, intermittently traded series. And the two practical guidelines the paper derives cut in opposite directions for me - "guideline one says that with limited historical data the simple average or weights ignoring covariances are recommended, which my 374 trading days per counter argues for, while guideline two says structural change impacts sophisticated schemes more than the simple average and that changing weights are a legitimate response to it, which is the entire premise of conditioning on state."
-The honest consequence the note draws: the equal-weight baseline becomes the field's hardest benchmark, and "if my state-conditioned weighting fails to beat equal weights on the CSE, that is the expected outcome under the field's prior and not a surprise". The response is not to defend the gap but to pre-register - write down before the run what margin and what test would count as beating equal weights. And the note extracts a genuine contribution even from failure: "Which effect dominates on this data is the question, and the paper is clear that comprehensive quantitative guidance on when to choose which does not yet exist in that literature, so an answer in a thin frontier market is a contribution even if the answer is that equal weights win."
+The honest consequence the note draws: the equal-weight baseline becomes the field's hardest benchmark, and "if my state-conditioned weighting fails to beat equal weights on the CSE, that is the expected outcome under the field's prior and not a surprise". The response is not to defend the gap but to pre-register - write down before the run what margin and what test would count as beating equal weights. And the note extracts a genuine contribution even from failure: "Which effect dominates on this data is the question, and the paper is clear that" comprehensive quantitative guidance on when to choose which does not yet exist in that literature, so an answer in a thin frontier market is a contribution even if the answer is that equal weights win.
 How my setting differs - three ways the note identifies. (i) My weights condition on exogenous measured market state, not on properties of the series computed once; this is the axis the literature has not covered. (ii) My loss is not quadratic forecast MSE against a realised value - "My orchestrator's output is evaluated after costs on risk-adjusted return, and a weighting that minimises forecast MSE is not the same object as one that maximises an after-cost objective, so I can borrow the mechanism and the cautionary evidence but not the optimality." The asymmetric-loss line (Elliott and Timmermann 2004, Patton and Timmermann 2007) is as close as this literature gets, and it finds optimal weights depend strongly on loss asymmetry and error skewness. (iii) My pool violates the review's non-interfering assumption: the four agents read overlapping data by construction, so the unbiasedness and variance-bound results do not hold for me, and the paper's own observation that overlapping information sets produce highly correlated errors is the mechanism by which that bites.
 A second threat, from the WARNING box rather than the paper itself. Frazier, Covey, Martin and Poskitt (Monash EBS WP 18/2023, arXiv:2308.05263) argue the puzzle is substantially an artefact of two-step estimation: estimated weights impart no first-order sampling variability into the usual predictive-accuracy statistic, so it converges to a generalised chi-squared rather than a normal, and their Theorem 1 says that when two weight vectors lie within O(T^{−1/4−ε}) of each other "the test has no power to distinguish them at all". Two consequences land directly on my design. "The O(T^{−1/4}) rate is not small at my sample sizes, roughly 0.23 at 374 trading days against roughly 0.14 on the ten-year index track, and with four agents sitting at 0.25 each under equal weights, a short sample puts almost any non-degenerate weighting scheme inside the dead zone. The constant is unknown so neither figure is a threshold, but the direction is unambiguous and it argues for running the weighting comparison on the index series rather than the per-counter panel." And their remedy, one-step joint estimation, is "mostly unavailable to me, since a retrieval agent is not jointly optimisable with a volatility model, so the partial version is to fit the parametric agents against the combined objective rather than against their own local losses." Caveat carried: this is a working paper and its publication status needs checking before it is cited as anything else.
 Design decisions this forces on the main gap: (a) no pairwise interaction term in the weighting function, backed by Bates and Granger, Newbold and Granger, and Winkler and Makridakis - ten covariance parameters against four diagonal ones, from 374 days; (b) a four-way rather than three-way comparison, adding a discounted inverse-MSE arm, because "if weights that merely react to recent agent performance do as well as weights conditioned on measured market state, then the state conditioning is not earning its place and I need to know that early"; (c) an oracle-weight arm to separate "the conditioning hypothesis is wrong" from "the estimation is too noisy"; (d) a Stock–Watson k-sweep to map the whole continuum from equal weights to winner-take-all cheaply; (e) pre-registration that separates two failure modes which look identical in the output - "the weighting genuinely not helping, which is the field's prior from the puzzle, against the weighting helping and the two-step test being unable to see it, because the first says abandon the conditioning and the second says change how it is estimated or tested."
 EFFECT ON THE ABSTENTION CHANNEL: Upgraded from a bespoke mechanism to named prior art. The paper states directly that subset selection is equivalent to assigning zero weights to some individual forecasts, and that time-varying subset selection can be achieved by applying a pre-set threshold to a time-varying weighting scheme (Li et al., 2022). "That is structurally what the abstention channel does when the fundamental agent has no disclosure to work from, which is expected more than half the time, so I should present it in that vocabulary rather than as a bespoke mechanism." Two consequences: the paper's own assessment is that subset selection "has received scant attention, is mainly trimming on expertise alone, and that most existing algorithms are ad hoc and lack statistical rationale", so a principled selection rule driven by a structural property of the output is defensible ground; and Geweke and Amisano's observation that individually poor forecasts may still help in combination argues for shrinking the abstaining agent's weight toward a floor rather than driving it to exactly zero - "a concrete design decision I had not settled."
 EFFECT ON THE CONFIDENCE TERM C_{i,t}: A route to making C_{i,t} a measured structural property rather than a self-report. If the orchestrator ever emits an interval rather than a point allocation, the linear pool's variance decomposition says component disagreement adds directly to pooled variance, "so a deliberately heterogeneous pool produces an under-confident interval, and that is the one place where my central design choice actively works against me." Quantile averaging avoids it - it averages cdfs horizontally, preserves the family for location-scale components, and is sharper for the same mean. "This connects to [[Adaptive Conformal Inference Under Distribution Shift]] more tightly than I expected, since adaptive conformal inference is a per-agent calibration wrapper and quantile averaging is the aggregation step, and the pair would give me a calibrated interval from a heterogeneous pool without the under-confidence that linear pooling would introduce. That is a route to the confidence term being a measured interval width rather than a self-report, which is what the scope revision asked for."
 EFFECT ON THE HETEROGENEITY CLAIM: The paper makes it testable and therefore falsifiable. "I describe the four agents as methodologically heterogeneous and that heterogeneity is load-bearing in the gap statement, but the paper's operational definition of diversity is low correlation among forecast errors... So the claim is testable on my own pool and I should run it: if the technical agent and the volatility agent produce errors that correlate at 0.8 on CSE data, the pool is substantially less diverse than the architecture diagram implies and the error-cancellation argument weakens accordingly. This is close to free, it uses data I will already have from the individual agent runs, and it is the kind of result that is much better found by me than by an examiner." Also relevant: Mannes et al. (2014) show the mean level of expertise in the pool sets a floor, so including a poor agent degrades the result - which bears on whether all four agents should always be in the pool.
-EFFECT ON EXPLAINABILITY: Upgraded from a feature to a positioned contribution. Interpreting combination weights is one of the paper's eight future directions - "discussing if, how, and when it is helpful to interpret combination weights". "My orchestrator produces a weight per agent per step as a readable function of named market-state inputs, so the trace of which agent was trusted when, and on what measured conditions, is a direct response to that question rather than a byproduct." Caveat carried from the layered-explainability reading: "a weight being readable is not the same as it being correct, so the claim is that the system exposes the quantity this literature identifies as unexamined, not that exposing it is sufficient."
+EFFECT ON EXPLAINABILITY: Upgraded from a feature to a positioned contribution. Interpreting combination weights is one of the paper's eight future directions - "discussing if, how, and when it is helpful to interpret combination weights". "My orchestrator produces a weight per agent per step as a readable function of named market-state inputs, so the trace of which agent was trusted when, and on what measured conditions, is a direct response to that question rather than a byproduct." Caveat carried from the layered-explainability reading: "a weight being readable is not the same as it being correct, so the claim is that the system exposes the quantity this literature" identifies as unexamined, not that exposing it is sufficient.
 EFFECT ON SUB-GAP 1: Negative in the sense that it offers nothing - "There is no portfolio, no position, no transaction cost, no slippage and no execution anywhere in forty pages" - but that absence is itself the boundary line. Everything in this paper is a weighting mechanism scored against a realised value under quadratic loss; none of its optimality results transfer to an after-cost decision objective. So the claim that execution cost belongs inside the decision objective is untouched by fifty years of combination theory, which is a clean separation to state.
-EFFECT ON SUB-GAP 2: Essentially none directly. The only contact point is Zischke et al. (2022), who find that in high-volatility periods weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample - "a result about choosing what to score rather than about how elaborate the pooling function is". That is about volatility level, not persistence, and the review contains nothing on persistence or on decay schedules. The structural-change guideline ("structural change impacts sophisticated schemes more than the simple average and changing weights are a legitimate response to it") is the nearest thing to support for conditioning on a regime, but it is a general statement with no persistence mechanism behind it.
+EFFECT ON SUB-GAP 2: Essentially none directly. The only contact point is Zischke et al. (2022), who find that in high-volatility periods weights optimised under a censored likelihood scoring rule always beat weights optimised under the logarithmic score out of sample - "a result about choosing what to score rather than about how elaborate the pooling function is". That is about volatility level, not persistence, and the review contains nothing on persistence or on decay schedules. The structural-change guideline (structural change impacts sophisticated schemes more than the simple average and "changing weights are a legitimate response to it") is the nearest thing to support for conditioning on a regime, but it is a general statement with no persistence mechanism behind it.
 CSE DATA EVIDENCE: The note states my per-counter archive as roughly 300 counters over 374 trading days, "three orders of magnitude short of M4", with "no result in this paper" speaking to a feature-to-weight meta-model at that scale. The ten-year index track is the alternative. Those two sample sizes drive the O(T^{−1/4}) calculation - roughly 0.23 at 374 trading days against roughly 0.14 on the index track, against four agents at 0.25 each under equal weights - which argues for running the weighting comparison on the index series rather than the per-counter panel. The same 374 days drive the parameter-count argument against a pairwise interaction term (ten covariance parameters against four). And the note's reading of the thin-market absence is directional rather than agnostic: "everything the paper says about estimation error swamping the gains from optimal weights gets worse in my setting, not better."
 PROPOSED REVISION STATED IN THE NOTE: Reframe the weighting function as a generalisation of FFORMA along one identified axis - exogenous measured market state at each step versus series properties computed once - rather than as new machinery. Pre-register the margin and the test that would count as beating equal weights, before the run. Expand the planned three-way comparison (equal / static learned / state-conditioned) to four-way by adding a discounted inverse-MSE arm, and add an oracle-weight arm fitted on the test window to separate "conditioning is wrong" from "estimation is too noisy". Add a Stock–Watson k-sweep. Run the weighting comparison on the index series rather than the per-counter panel, on the power argument. Fit the parametric agents against the combined objective rather than their own local losses, as the partial version of one-step joint estimation. Present the abstention channel as time-varying subset selection with a threshold, and shrink the abstaining agent's weight toward a floor rather than to exactly zero. Measure pool diversity as error correlation before claiming heterogeneity. Keep a separate note for the Frazier et al. working paper and check its publication status before citing it as anything other than a working paper. State explicitly in the write-up why there is no pairwise interaction term. And carry the warning that standard errors on a combined forecast are nontrivial because the weights are random and correlated with the forecasts - which matches the pattern where "the economic result and the formal test diverged" in the DRL global-equity portfolio note.</t>
         </is>
@@ -7733,7 +7733,7 @@
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>This is the paper's headline empirical domain. The point predictor is GARCH(1,1) on realised volatility V_t = R_t^2, refit on a trailing 1,250-day window, with the conformity score normalised by the predicted variance. The adaptation is substantial rather than cosmetic: across the four main-figure stocks alpha_t ranges between about 0.035 and 0.17 against a target of 0.1, so "at its extremes the method is targeting 96.5% coverage in some periods and 83% in others to achieve 90% on average". The troughs line up with crises, Fannie Mae and BlackBerry both bottoming out near 0.035 through 2008 and 2009, "which is the method widening its intervals hard when the GARCH fit is worst". At gamma = 0.005 a single miss moves alpha_t by 0.0045, so these swings take hundreds of days to develop and the series is slow-moving by construction, "in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]". The alpha_t trajectories "read as a volatility-regime series in their own right".
+          <t>This is the paper's headline empirical domain. The point predictor is GARCH(1,1) on realised volatility V_t = R_t^2, refit on a trailing 1,250-day window, with the conformity score normalised by the predicted variance. The adaptation is substantial rather than cosmetic: across the four main-figure stocks alpha_t ranges between about 0.035 and 0.17 against a target of 0.1, so at its extremes the method is targeting 96.5% "coverage in some periods and 83% in others to achieve 90% on average". The troughs line up with crises, Fannie Mae and BlackBerry both bottoming out near 0.035 through 2008 and 2009, "which is the method widening its intervals hard when the GARCH fit is worst". At gamma = 0.005 a single miss moves alpha_t by 0.0045, so these swings take hundreds of days to develop and the series is slow-moving by construction, "in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]". The alpha_t trajectories "read as a volatility-regime series in their own right".
 Critically, the risk quantity produced is a coverage statement and not a width statement: see LIMITATIONS. The paper never attaches an interval to a position size or any other risk-budgeting decision.</t>
         </is>
       </c>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="S56" s="11" t="inlineStr">
         <is>
-          <t>- The non-adaptive method fails visibly and the adaptive one stays inside the Bernoulli band on all twelve names, with 2008 producing the clearest separation. Fannie Mae: fixed-alpha local coverage falls to roughly 0.83 against a target of 0.9 and stays depressed for most of 2008 and 2009, while the adaptive curve dips and recovers within the Bernoulli range. BlackBerry shows the same shape in 2008. AMD shows a fixed-alpha trough near 0.835 around 2016 and an over-covering excursion to 0.96 in 2004. Nvidia shows a trough near 0.85 across 2016 and 2017. "The useful reading is that the failure is two-sided, the fixed method over-covers as often as it under-covers, so what's being fixed is calibration drift rather than a conservatism bug." Caveat I flag in the note: the four stocks shown were selected out of twelve because they showed a clear failure of the non-adaptive method, which the authors state plainly, "so the main figure is a demonstration of the failure mode rather than a sample of typical behaviour, and the eight appendix panels are the ones to read for that."
+          <t>- The non-adaptive method fails visibly and the adaptive one stays inside the Bernoulli band on all twelve names, with 2008 producing the clearest separation. Fannie Mae: fixed-alpha local coverage falls to roughly 0.83 against a target of 0.9 and stays depressed for most of 2008 and 2009, while the adaptive curve dips and recovers within the Bernoulli range. BlackBerry shows the same shape in 2008. AMD shows a fixed-alpha trough near 0.835 around 2016 and an over-covering excursion to 0.96 in 2004. Nvidia shows a trough near 0.85 across 2016 and 2017. "The useful reading is that the failure is two-sided, the fixed method over-covers as often as it under-covers, so what's being fixed is calibration drift rather than a conservatism bug." Caveat I flag in the note: the four stocks shown were selected out of twelve because they showed a clear failure of the non-adaptive method, which the authors state plainly, so the main figure is a demonstration of the failure mode rather than a sample of "typical behaviour, and the eight appendix panels are the ones to read for that."
 - alpha_t moves across roughly a fourfold range, about 0.035 to 0.17 against a 0.1 target.
 - The theory splits cleanly: Proposition 4.1 holds for any data generating process and is shown to be approximately tight, in that replacing max{1-alpha_1, alpha_1} with |alpha_1 - alpha*| under a noiseless idealisation recovers nearly the same bound, "so it is simultaneously agnostic and close to the best possible given a bad initialisation". Everything sharper needs the stationary HMM.
 - The conformity score design controls the result about as much as the adaptation does. The unnormalised score produces much wider swings in local coverage around 0.9 for the adaptive method, visibly outside the Bernoulli band and dropping below 0.6 on AMD and Fannie Mae in the crisis windows, against the normalised version which stays within a few percentage points throughout. The authors' explanation is that normalising by sigma_hat_t^2 is what makes the score approximately stationary, and they note the issue can be partially mitigated by a larger gamma. "So 'works with any black box' is true of the interface and not of the performance, and the real requirement is a score whose distribution moves slowly."
@@ -7803,7 +7803,7 @@
 The boundary of the contribution needs stating plainly and early, which is why the note ends where it does: "ACI is an off-the-shelf wrapper with a public R implementation, four years old and widely cited, and there is nothing novel in applying it to a GARCH forecast since that is the paper's own worked example. What would be a candidate technical contribution not identified in the literature I have covered is using the adapted miscoverage level as an input to a weighting function over heterogeneous agents, which is a different claim and a much narrower one, and it needs validating against recent work before it goes anywhere near the novelty statement." So: adopt ACI as a component, claim only the orchestration use of alpha_t, and validate that narrower claim before it enters the novelty statement.
 EFFECT ON SUB-GAP 1: Mostly indirect, and it creates one new liquidity dependency rather than resolving anything. The paper has no liquidity content at all - no spreads, no turnover, no execution cost. But the score-design finding pushes liquidity into the calibration layer, which I had not anticipated. Normalising the conformity score by predicted variance is what made their score approximately stationary; on the CSE, "where zero-return days and stale quotes are common, a variance-normalised score may still be non-stationary because the denominator is itself unreliable when the counter didn't trade." The candidate fix is to normalise by a liquidity-adjusted volatility estimate "using the same Amihud and turnover inputs already being computed for the cost model and for the composite liquidity state, so one measurement serves a third purpose." That is a reuse of L_t inside the machinery that produces C_{V,t}, which is a genuine coupling between the liquidity state and the reliability of a price-derived agent - the second half of Sub-gap 1's statement, that liquidity simultaneously conditions the reliability of price-derived agents. It is recorded as "a named experiment, not a design decision", so it is a hypothesis I owe a test, not a finding I can lean on.
 EFFECT ON SUB-GAP 2: Substantial, and in a way that is adjacent to rather than inside Sub-gap 2. Sub-gap 2 is about volatility PERSISTENCE and specifically about replacing an EWMA half-life, which assumes exponential decay, with a persistence-aware decay schedule. ACI does not estimate persistence and does not propose a decay schedule, so it does not close the sub-gap. What it does is supply a second, independent slow-moving state series over the same volatility object: at gamma = 0.005 a single miss moves alpha_t by 0.0045, "so these swings take hundreds of days to develop, and the series is slow-moving by construction in the same way d is in [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]]." The alpha_t trajectories "read as a volatility-regime series in their own right", ranging about 0.035 to 0.17 and bottoming out in 2008-2009 when the GARCH fit is worst. That is a measurement of how badly a fitted volatility model is tracking the market, which is a different quantity from P_t but lives on the same timescale and is produced by the same agent - so the discipline required is to test whether alpha_t adds anything over the existing four conditioning terms, not to assume it does. Hence the note's framing: carry it "as a candidate addition to the conditioning set and test it on the ablation protocol against the existing four terms rather than adopting it."
-The sharper transfer finding is that ACI's own step size has the same structural problem Sub-gap 2 identifies in the EWMA half-life. gamma is a fixed decay rate on a non-stationary target, set once, never varied, and justified in a sentence; the theory's own prescription gamma proportional to sqrt(E|delta alpha*|) says gamma should be larger in more volatile environments, which is a persistence-type statement the paper does not operationalise. So ACI imports the exact defect Sub-gap 2 exists to correct, one level up. That is useful: it means the persistence argument generalises beyond the volatility scaler, and it also means I cannot adopt gamma = 0.005 and stop thinking. "On 374 observations a step that small means alpha_t barely leaves its initialisation, so the sample would be spent in the transient the theory warns about, and the prescription gamma proportional to sqrt(E|delta alpha*|) points the same way given the CSE's crisis sequence. The experiment is a gamma sweep on the index track where I have the length to measure it, then carry the chosen value down to the counters."
+The sharper transfer finding is that ACI's own step size has the same structural problem Sub-gap 2 identifies in the EWMA half-life. gamma is a fixed decay rate on a non-stationary target, set once, never varied, and justified in a sentence; the theory's own prescription gamma proportional to sqrt(E|delta alpha*|) says gamma should be larger in more volatile environments, which is a persistence-type statement the paper does not operationalise. So ACI imports the exact defect Sub-gap 2 exists to correct, one level up. That is useful: it means the persistence argument generalises beyond the volatility scaler, and it also means I cannot adopt gamma = 0.005 and stop thinking. On 374 observations a step that small means alpha_t barely leaves its initialisation, so the sample would be spent in the transient the theory warns about, and the prescription gamma proportional to sqrt("E|delta alpha*|) points the same way given the CSE's crisis sequence. The experiment is a gamma sweep on the index track where I have the length to measure it, then carry the chosen value down to the counters."
 CSE DATA EVIDENCE: The paper contains none - twelve US names and 3,111 US counties. The CSE evidence in this cell is my own data-depth accounting, and it is the sharpest constraint in the note: "The 1250-day refit window is the sharpest data-depth constraint I've hit in a review and it splits my two tracks. Five years of daily data per counter, with the calibration scores drawn from the same window, against 374 trading days per counter in the archive. On the index track at ten years daily the recipe transfers as written; on the per-counter track it does not, and the honest options are a shorter joint window with the calibration degradation reported, or pooling scores across counters, which breaks the per-counter conditioning the method relies on. This belongs in the data-depth discussion as a named requirement with a number attached, not as a general concern." Five years per counter is roughly thirteen times the per-counter archive. Note also that shrinking the window degrades the GARCH fit and the empirical quantile simultaneously, because the calibration scores come from the same window - the two failures are not independent.
 PROPOSED REVISION STATED IN THE NOTE: Several, all recorded as candidates or experiments rather than adopted design:
 1. Define C_{V,t} as a function of the ACI-calibrated interval width at the target coverage, wrapping the FIGARCH or GJR-GARCH forecast with the normalised conformity score.
@@ -7842,7 +7842,7 @@
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Working paper in the version read (November 2018); published subsequently in the *Review of Financial Studies*, which the note describes as "the paper that everything in this area now cites". Volume and pages: Not recorded in the note. The note's frontmatter carries 2018, the working-paper year; 2020 is the journal of record.</t>
+          <t>Working paper in the version read (November 2018); published subsequently in the *Review of Financial Studies*, which the note describes as the "paper that everything in this area now cites". Volume and pages: Not recorded in the note. The note's frontmatter carries 2018, the working-paper year; 2020 is the journal of record.</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
@@ -7852,7 +7852,7 @@
       </c>
       <c r="F57" s="11" t="inlineStr">
         <is>
-          <t>Empirical asset pricing / machine learning for cross-sectional return prediction. A comparative horse race of thirteen prediction methods on a single shared problem. The note is emphatic that this is not a competitor architecture and is not being read as one: "there are no agents here and no orchestration problem". It earns a full note for four reasons recorded verbatim in the note: it is "the best available calibration of what a well-specified return predictor actually achieves, and the number is small enough that it should reset my expectations for the technical agent before I build it"; "the signal families it ranks at the top are price trend, liquidity and volatility, which is independent large-sample evidence for two of the three state variables my orchestrator conditions on"; "its feature construction is the single-model version of conditioning on market state, every characteristic interacted with every macro variable, which is structurally the thing I am proposing to do one level up"; and "it is a clean, well-documented instance of the failure mode my cost sub-gap exists to address, reporting 113% monthly turnover and an annualised Sharpe of 2.35 in the same table without deducting a basis point."</t>
+          <t>Empirical asset pricing / machine learning for cross-sectional return prediction. A comparative horse race of thirteen prediction methods on a single shared problem. The note is emphatic that this is not a competitor architecture and is not being read as one: "there are no agents here and no orchestration problem". It earns a full note for four reasons recorded verbatim in the note: it is "the best available calibration of what a well-specified return predictor actually achieves, and the number is small enough that it should reset my expectations for the technical agent before I build it"; "the signal families it ranks at the top are price trend, liquidity and volatility, which is independent large-sample evidence for two of the three state variables my orchestrator conditions on"; "its feature construction is the single-model version of conditioning on market state, every characteristic interacted with every macro variable, which is structurally the thing I am proposing to do one level up"; and "it is a clean, well-documented instance of the failure mode my cost sub-gap exists to address, reporting" 114% monthly turnover and an annualised Sharpe of 2.35 in the same table without deducting a basis point.</t>
         </is>
       </c>
       <c r="G57" s="11" t="inlineStr">
@@ -7906,7 +7906,7 @@
       </c>
       <c r="L57" s="11" t="inlineStr">
         <is>
-          <t>Not applicable - a single-estimator horse race with no agents, no orchestrator, no weighting of heterogeneous producers over a shared decision. What it does instead is the closest single-model analogue: the Kronecker construction makes every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator. The note draws the line precisely: "That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound. What it does not do is the thing I am claiming: the interaction weights are estimated once per annual refit, they are a function of macro variables rather than of any measured reliability of the signal, and no channel in their model can go absent, because a missing characteristic is median-imputed rather than down-weighted. The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line."</t>
+          <t>Not applicable - a single-estimator horse race with no agents, no orchestrator, no weighting of heterogeneous producers over a shared decision. What it does instead is the closest single-model analogue: the Kronecker construction makes every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator. The note draws the line precisely: "That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound. What it does not do is the thing I am claiming: the interaction weights are estimated once per annual refit, they are a function of macro variables rather than of any measured reliability of the signal, and no channel in their model can go absent, because a missing characteristic is median-imputed rather than down-weighted". The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line.</t>
         </is>
       </c>
       <c r="M57" s="11" t="inlineStr">
@@ -7928,7 +7928,7 @@
       <c r="P57" s="11" t="inlineStr">
         <is>
           <t>Liquidity appears as a predictor family and is absent as a friction, and the gap between those two facts is what the note exploits. The liquidity group (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) is one of the three dominant families across every method. But: "There are no transaction costs anywhere in the paper, and the turnover figures make that decisive rather than cosmetic." The best strategy, an equal-weighted decile spread on NN4 forecasts, returns 3.3% per month, 39.0% annualised, at an out-of-sample Sharpe of 2.35, with monthly turnover of 114.08%. Networks run 110.87% to 114.08%, elastic net 143.61% and OLS-3 156.78%, against 22.87% for a size decile spread. The authors note that high turnover is unsurprising given the dominance of price-trend predictors, "and then stop."
-Two things in their own results indicate the size of what is being left out. Value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, "so the gap between the paper's two weighting schemes is larger than the gap between most of its methods." And the universe retains sub-$5 stocks by explicit choice. The paper offers the higher top-1,000 R^2, 0.72% against 0.46%, as reassurance that machine learning is not merely picking up small-scale inefficiencies driven by illiquidity, "but the result carrying the economic claim is an equal-weighted spread over the whole board, and both cannot be load-bearing at once."</t>
+Two things in their own results indicate the size of what is being left out. Value weighting alone, with no costs introduced, drops NN3's Sharpe from 2.32 to 1.25 and OLS-3's from 0.89 to 0.27, "so the gap between the paper's two weighting schemes is larger than the gap between most of its methods." And the universe retains sub-$5 stocks by explicit choice. The paper offers the higher top-1,000 R^2, 0.72% against 0.46%, as reassurance that machine learning is not merely picking up small-scale inefficiencies driven by illiquidity, but the result carrying the economic claim is "an equal-weighted spread over the whole board, and both cannot be load-bearing at once."</t>
         </is>
       </c>
       <c r="Q57" s="11" t="inlineStr">
@@ -7965,7 +7965,7 @@
           <t>- No transaction costs anywhere, and the turnover figures make that decisive rather than cosmetic (figures above). The authors note high turnover is unsurprising given the dominance of price-trend predictors and then stop. The value-weighted Sharpe collapse is "itself a partial, unacknowledged cost estimate". The top-1,000 reassurance and the equal-weighted headline "both cannot be load-bearing at once."
 - The Monte Carlo summary does not match its own table in the linear case. The text states that for the sparse linear model Lasso and ENet deliver the best and almost identical out-of-sample R^2, and that RF, NN and GBRT tend to overfit so their performance is slightly worse. Table A.1 shows NN1 at 4.42% and NN2 at 4.40% against ENet+H at 4.27% when P_c = 50, and 4.31% and 4.30% against 4.26% when P_c = 100, "so the networks are ahead in both panels. The trees do underperform as described, and the substantive conclusion about the nonlinear process is untouched, but the specific claim that penalized linear methods win when the truth is linear is contradicted by the numbers printed beneath it." That sentence is where the "match the method to the process" reading comes from.
 - Variable importance by zeroing a predictor is not clean attribution when the predictors are this correlated. Six of the top eight characteristics are versions of the same price-trend quantity measured over different windows, and setting one to zero leaves its correlates free to absorb the signal, "which understates each and leaves the group's total importance unallocated. The agreement across models that the paper highlights is therefore partly agreement about the correlation structure of the feature set rather than independent discovery." A second issue is specific to trees, where zeroing a characteristic sends observations to partitions the model never saw during training, "so the measured drop mixes the variable's contribution with an off-distribution evaluation." The placebo test passes but "establishes that irrelevant variables rank low, not that the ranking among relevant and correlated variables is meaningful."
-- Complexity is shown to drift over the test period and the drift is explained rather than tested, and no empirical table carries uncertainty. Figure 3's drift is attributed to a growing cross section and improving data coverage: "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." Models are refit once a year with the five architectures fixed throughout, a concession to compute the authors acknowledge. There are no confidence intervals or seed variation on Tables 1, 2, 5, 7, 8 or 9, only on the 100-repetition simulations. "The 60-year sample compounds this, since a model refit annually from 1957 through 2016 averages over an enormous range of market structures, and the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."
+- Complexity is shown to drift over the test period and the drift is explained rather than tested, and no empirical table carries uncertainty. Figure 3's drift is attributed to a growing cross section and improving data coverage: That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check. Models are refit once a year with the five architectures fixed throughout, a concession to compute the authors acknowledge. There are no confidence intervals or seed variation on Tables 1, 2, 5, 7, 8 or 9, only on the 100-repetition simulations. "The 60-year sample compounds this, since a model refit annually from 1957 through 2016 averages over an enormous range of market structures, and the conclusion that machine learning is most valuable for larger and more liquid stocks is, read the other way, a statement that it works least well in the conditions a frontier market presents continuously."
 - Framing limitation conceded by the authors themselves in Section 1.6: improved predictions are only measurements, they do not identify deep associations between prices and conditioning variables, and recovering mechanisms requires the economist to impose structure.</t>
         </is>
       </c>
@@ -7995,9 +7995,9 @@
         <is>
           <t>SPEAKS TO: A_T first (expectation band, architecture sizing, loss function, feature count), then the orchestrator's conditioning set (independent large-sample evidence for L_t and V_t, and the Kronecker construction as the single-model analogue of the orchestration claim), then the evaluation layer (benchmark choice, DM test, recursive protocol, Campbell-Thompson mapping), then A_F (horizon and lag discipline, and an argument for a low baseline weight plus explicit abstention), and finally Sub-gap 1, for which this paper is the cleanest reference case in the set.
 EFFECT ON MAIN GAP: It strengthens the premise and sharpens the claim without threatening either. The Kronecker construction is the single-model version of what I am proposing one level up: "Gu et al. make every signal's value time-varying by interacting each of 94 characteristics with eight macro state variables inside one estimator, and the beta-pricing derivation is a principled reason to do it. That is conditioning on state, and the fact that it is standard practice in a canonical paper is evidence my premise is sound." That matters because it means the idea that a signal's value varies with market state is not something I have to argue for from scratch - it is derivable from E_t(r_{i,t+1}) = beta'_{i,t} lambda_t with beta_{i,t} = theta_1 c_{i,t} and lambda_t = theta_2 x_t, and it is the standard specification in the most-cited paper in the area.
-Then the line. Three differences separate their construction from mine, and all three are in w(i,t) = f(L_t, V_t, P_t, C_{i,t}): their interaction weights are estimated once per annual refit, so they do not vary with measured market state at decision time, only with the value of the macro variable plugged into a fixed coefficient; they are a function of macro variables rather than of any measured reliability of the signal, so there is no C_{i,t} analogue anywhere in the model; and no channel can go absent, "because a missing characteristic is median-imputed rather than down-weighted". The note puts the whole claim on that last point: "The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim, and this paper is the cleanest place to draw that line." Median imputation is the exact anti-pattern my abstention channel exists to replace - it substitutes a plausible value for a missing one and the downstream model cannot tell the difference, whereas abstention makes absence visible to the aggregator.
-It also supplies the evidence base for two of the four conditioning terms. Liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) and risk (total volatility, idiosyncratic volatility, beta, beta squared) are two of the three dominant families across every one of eleven method families on a ~30,000-stock, 60-year panel. "That is a far larger evidence base for those two conditioning inputs than the CSE-specific work in [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] or the Granger result at p = 0.0041 from volume to ASPI, and it composes with both." The macro rejection also survives: market-level stock variance is given little weight by any method and essentially none by the networks, consistent with the thin ARDL result in [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]] that already got the macro block rejected. The one live challenge is aggregate book-to-market - critical for every model, 28.57% for NN1 and 43.46% for GLM - and the honest response recorded in the note is to "test it against an ASPI-level valuation ratio rather than dismiss it on the strength of a rejection aimed at different variables."
-One further point that bears directly on the main gap and that the paper declined to test: Figure 3 shows model complexity drifting across the test period - elastic net selecting fewer than five features in the first decade and 20 to 40 after 2000, GBRT moving from roughly 20 features to 30 - and the authors explain it by a growing cross section and improving data coverage. "That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check." So the paper leaves my central hypothesis open on evidence it had in hand, which is a better position for me than either confirming or refuting it would have been.
+Then the line. Three differences separate their construction from mine, and all three are in w(i,t) = f(L_t, V_t, P_t, C_{i,t}): their interaction weights are estimated once per annual refit, so they do not vary with measured market state at decision time, only with the value of the macro variable plugged into a fixed coefficient; they are a function of macro variables rather than of any measured reliability of the signal, so there is no C_{i,t} analogue anywhere in the model; and no channel can go absent, "because a missing characteristic is median-imputed rather than down-weighted". The note puts the whole claim on that last point: "The difference between imputing a missing input at the cross-sectional median and reducing the weight on the agent that produced it is precisely the orchestration claim", and this paper is the cleanest place to draw that line. Median imputation is the exact anti-pattern my abstention channel exists to replace - it substitutes a plausible value for a missing one and the downstream model cannot tell the difference, whereas abstention makes absence visible to the aggregator.
+It also supplies the evidence base for two of the four conditioning terms. Liquidity (turnover, turnover volatility, market equity, dollar volume, Amihud illiquidity, zero-trading days, bid-ask spread) and risk (total volatility, idiosyncratic volatility, beta, beta squared) are two of the three dominant families across every one of eleven method families on a ~30,000-stock, 60-year panel. That "is a far larger evidence base for those two conditioning inputs than the CSE-specific work in [[Role of Market Liquidity in Sentiment-Based Return Predictions, Evidence from Sri Lanka]] or the Granger result at p = 0.0041 from volume to ASPI, and it composes with both." The macro rejection also survives: market-level stock variance is given little weight by any method and essentially none by the networks, consistent with the thin ARDL result in [[The Long-Term Impact of Macroeconomic Stability Variables on Stock Price Volatility]] that already got the macro block rejected. The one live challenge is aggregate book-to-market - critical for every model, 28.57% for NN1 and 43.46% for GLM - and the honest response recorded in the note is to "test it against an ASPI-level valuation ratio rather than dismiss it on the strength of a rejection aimed at different variables."
+One further point that bears directly on the main gap and that the paper declined to test: Figure 3 shows model complexity drifting across the test period - elastic net selecting fewer than five features in the first decade and 20 to 40 after 2000, GBRT moving from roughly 20 features to 30 - and the authors explain it by a growing cross section and improving data coverage. That is plausible and it is also asserted rather than tested, and the alternative, that the number of features carrying signal is itself regime-dependent, is the hypothesis my orchestrator rests on and the one this paper was best placed to check. So the paper leaves my central hypothesis open on evidence it had in hand, which is a better position for me than either confirming or refuting it would have been.
 EFFECT ON SUB-GAP 1: This is the strongest available illustration of why cost belongs inside the objective rather than after it, and I would cite it as the reference case. "A strategy turning over 114% of its book monthly, concentrated in price-trend signals, on a universe that deliberately includes the smallest and least liquid names, reported at Sharpe 2.35 with no cost deduction and no participation-rate analysis, is the reference case for my cost sub-gap." Two details make it sharper than a generic "they ignored costs" complaint. First, the value-weighted collapse - NN3 from 2.32 to 1.25, OLS-3 from 0.89 to 0.27 - "is itself a partial, unacknowledged cost estimate and I should cite it that way": moving weight away from the small end halves the Sharpe before a single basis point of spread is charged, which is a lower bound on what liquidity is doing to the result. Second, the internal tension: the paper offers the top-1,000 R^2 of 0.72% against 0.46% on the bottom 1,000 as reassurance that the result is not driven by small-cap illiquidity, while the headline economic result is an equal-weighted spread over the whole board - "both cannot be load-bearing at once."
 Applied to the CSE this is not implementable at any size. "On the CSE, where Dissanayake and Nanayakkara find unexpected illiquidity shocks depressing returns by -0.084 to -0.097 and small caps more than large, that turnover is not implementable at any size, which is the concrete argument for sweeping participation rate against daily volume rather than charging a flat spread, as [[Online portfolio selection with state-dependent price estimators and transaction costs]] and [[A reinforcement learning approach to optimal execution]] both do in their different ways." So the paper does not close any part of Sub-gap 1 - it has no friction model at all - but it supplies the clearest demonstration of the failure the sub-gap names, from a source that is hard to dismiss.
 EFFECT ON SUB-GAP 2: Limited, and I should not overclaim it. The paper has no volatility process, no persistence estimate, no decay schedule and no volatility targeting; volatility enters only as a cross-sectional predictor. So it neither closes nor narrows Sub-gap 2. What it contributes is one piece of supporting evidence and one adjacent warning. The evidence: the risk family (total volatility, idiosyncratic volatility, beta, beta squared) is one of the three dominant predictor families across all eleven methods, and the GBRT/NN3 marginal relationship is economically large - a firm whose volatility rises from median to the 80th percentile loses around 3.0% per year in expected return - which supports keeping V_t in the conditioning set but says nothing about P_t. The warning is the complexity-drift result again: the paper observed a time-varying structure in its own fitted models and explained it away rather than testing it, which is the same category of move as assuming a fixed exponential decay rate and never checking.
@@ -8079,10 +8079,10 @@
 SP_it = β0 + β1 ROE_it + β2 DPS_it + β3 EPS_it + β4 PE_it + β5 DTA_it + β6 log(SIZE_it) + ε_it
 with SP_it the average monthly share price of firm i in year t in nominal rupees, PE_it the price to earnings ratio, DTA_it total liabilities over total assets, log(SIZE_it) the natural log of total assets. "There are no year effects, no industry effects and no lagged dependent variable, and no standard error clustering is reported."
 The endogeneity-by-construction problem, which I set out as its own equation because it is the thing I take forward:
-PE_it = SP_it / EPS_it  ⟹  SP_it = β0 + … + β4 (SP_it / EPS_it) + … + ε_it
-My reading: "This is not an omitted control or a specification preference, it is an accounting identity relating two of the variables in the regression, and nothing in the paper acknowledges it. Whatever β4 is estimating, it is not the independent contribution of a valuation multiple to price."
+PE_it = SP_it / EPS_it ⟹ SP_it = β0 + … + β4 (SP_it / EPS_it) + … + ε_it
+My reading: This is not an omitted control or a specification preference, it is an accounting identity relating two of the variables in the regression, and nothing in the paper acknowledges it. Whatever β4 "is estimating, it is not the independent contribution of a valuation multiple to price."
 The within/between decomposition, which is the single most useful piece of the paper for me:
-R²_within = corr²(ŷ_it − ȳ̂_i, y_it − ȳ_i),   R²_between = corr²(ȳ̂_i, ȳ_i)
+R²_within = corr²(ŷ_it − ȳ̂_i, y_it − ȳ_i), R²_between = corr²(ȳ̂_i, ȳ_i)
 "A model that separates expensive firms from cheap ones but says nothing about a given firm's path through time produces exactly the pattern reported here, high between and near-zero within."
 Output: in-sample coefficients and significance only. No forecast, no holdout, no agent.</t>
         </is>
@@ -8141,7 +8141,7 @@
 - Survivorship and look-ahead: "Selecting on terminal market capitalisation and then estimating on 2013 onwards keeps every firm that grew into the top twenty and drops every firm that fell out of it or delisted, which is survivorship combined with look-ahead selection." The missing 20 firm-years out of the expected 220 are never accounted for, and "the model summary's mean dependent variable of 83.107 with a standard deviation of 63.883 cannot be reconciled with the share price mean of 262.078 and standard deviation of 458.181 in the descriptives, so the two tables appear to come from different runs or different transformations of the dependent variable."
 - Regime pooling: "Eleven years of nominal rupee prices are pooled as one regime across a currency collapse." A rupee of EPS in 2014 and in 2023 "are not the same quantity, so part of what the coefficients are fitting is the unit of measurement changing underneath the panel." The paper frames this as an omitted-macro-variable issue "when the sharper problem is comparability of the dependent variable across the sample."
 - No out-of-sample evaluation despite forecasting claims: the abstract says the factors "can be used to make accurate future share price estimates" and the recommendations tell investors to monitor these ratios to "facilitate accurate forecasts of future share prices", while "an in-sample R² of 0.576 on a cross-section, with a within R² of 0.090, supports neither sentence." I noted this is "the gap I actually care about rather than a complaint about this paper specifically, since it is the standard shape of the local empirical literature."
-- Write-up slips: variable definitions render DPS as "Dep_osit" and EPS as "Esp_rit", every marginal effect is described as the response to a 1% change when only firm size is logged, the conclusion mentions a panel unit root test finding "at least one panel had a unit root" that appears nowhere in the results, and Table 10 duplicates the p-values already in Table 9. "None of these change a coefficient, and together they mean I should treat the figures as needing verification rather than as a clean reference."</t>
+- Write-up slips: variable definitions render DPS as "Dep_osit" and EPS as "Esp_rit", every marginal effect is described as the response to a 1% change when only firm size is logged, the conclusion mentions a panel unit root test finding "at least one panel had a unit root" that appears nowhere in the results, and Table 10 duplicates the p-values already in Table 9. None of these change a coefficient, and together they mean I should treat the figures as needing verification rather than as a clean reference.</t>
         </is>
       </c>
       <c r="U58" s="11" t="inlineStr">
@@ -8238,7 +8238,7 @@
           <t>Annual accounting data plus weekly price series. "All accounting and insider ownership data is hand-collected from annual reports published by the CSE", prices and the index come from the CSE data libraries, and Treasury bill rates from the Central Bank of Sri Lanka.
 Idiosyncratic risk is built as the residual standard deviation from a Fama–French three-factor regression on weekly excess returns over 52 trading weeks:
 r_{i,t} − r_{f,t} = α_i + β_i^MKT MKT_t + β_i^SMB SMB_t + β_i^HML HML_t + ε_{i,t}, σ_i^idi = sd(ε̂_{i,t})_{t=1..52}
-where r_{i,t} is the weekly return adjusted for cash dividends, stock splits, scrip dividends, bonus issues and rights issues; the market proxy is "the percentage change in the All Share Total Return Index (ASTRI), not the ASPI, which is the right choice since it is total return rather than price only"; r_{f,t} is a weekly rate derived from the yield on 91-day Treasury bills; and "weekly returns exceeding +50% or falling below −50% are dropped as outliers, following Abeysekera and Nimal (2017)".
+where r_{i,t} is the weekly return adjusted for cash dividends, stock splits, scrip dividends, bonus issues and rights issues; the market proxy is the percentage change in the All Share Total Return Index (ASTRI), "not the ASPI, which is the right choice since it is total return rather than price only"; r_{f,t} is a weekly rate derived from the yield on 91-day Treasury bills; and "weekly returns exceeding +50% or falling below −50% are dropped as outliers, following Abeysekera and Nimal (2017)".
 Systematic risk is backed out of the decomposition rather than estimated separately: σ^sys = sqrt(σ^tot² − σ^idi²), with total risk the standard deviation of weekly returns.
 Ownership: insider ownership is the share of total outstanding shares held by executive directors on the board at year end; institutional ownership is the share held by pension funds, investment banks, mutual funds and companies holding more than 3% (both following Farwis and Azeez, 2019). Controls are cash flow over lagged PPE, firm size as the firm's PPE relative to total sample PPE that year, and leverage as total debt over total assets.
 Descriptives I keep returning to: mean idiosyncratic risk "0.221 with a standard deviation of only 0.050 and a full range of 0.117 to 0.315"; "insider and institutional ownership correlate at −0.703"; mean insider ownership 5.7% against mean institutional ownership 66.1%, "so this is a market of institutionally held firms with thin executive stakes". Sample mean investment rate is 11.60%, with a minimum in Table 2 of −0.082.</t>
@@ -8252,7 +8252,7 @@
 where I_{i,t} is the change in net PPE in year t and K_{i,t−1} is lagged net PPE "so the dependent variable is an investment rate rather than a level"; η_i and g_t are firm and year fixed effects; "risk, size and leverage all enter in logs, following Panousi and Papanikolaou (2012)"; β1 is the coefficient of interest.
 Model 2 (the design I find most transferable): "rather than interacting risk with continuous ownership it sorts firms each year into two equally sized groups on the previous year's insider ownership relative to the annual median, and interacts risk with each group dummy, omitting the intercept to avoid the dummy trap":
 (I_{i,t}/K_{i,t−1}) = β1 log(σ^idi_{i,t−1}) × INSD_L + β2 log(σ^idi_{i,t−1}) × INSD_H + β3 log(σ^sys_{i,t−1}) + controls + INSD_L + INSD_H + η_i + g_t + ν_{i,t}
-Model 3 extends to a 2×2 grid, sorting first on institutional ownership then on insider ownership within each institutional group, yielding four interaction terms, to ask whether institutional monitoring substitutes for insider alignment. My note on the design choice: "splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it is close to the structure I'd want for ablating state inputs one at a time."
+Model 3 extends to a 2×2 grid, sorting first on institutional ownership then on insider ownership within each institutional group, yielding four interaction terms, to ask whether institutional monitoring substitutes for insider alignment. My note on the design choice: splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it "is close to the structure I'd want for ablating state inputs one at a time."
 Output: in-sample panel coefficients. "There are no agents, no forecasts and no out-of-sample period anywhere in it."</t>
         </is>
       </c>
@@ -8276,7 +8276,7 @@
       <c r="O59" s="11" t="inlineStr">
         <is>
           <t>Central to the paper and directly reusable for A_V. Idiosyncratic risk is the annual standard deviation of residuals from a weekly Fama–French three-factor regression over 52 weeks; systematic risk is backed out as σ^sys = sqrt(σ^tot² − σ^idi²). My assessment: "The idiosyncratic risk construction is the estimator I'd reuse for the volatility agent's cross-sectional input, with the liquidity correction they skip. Residual standard deviation from a local factor model over a rolling window is the right shape, the ASTRI and 91-day Treasury bill plumbing is established, and Abeysekera and Nimal (2017) gives me a four-factor local alternative."
-What I would add: "the non-synchronous trading correction and a reported correlation between the risk estimate and turnover, because if those two move together on my sample then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it."
+What I would add: "the non-synchronous trading correction and a reported correlation between the risk estimate and turnover, because if those" two move together on my sample then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it.
 Magnitude prior for A_V: "Mean idiosyncratic risk of 0.221 with a standard deviation of 0.050 sets a realistic prior on how much cross-sectional signal the volatility channel can carry. That is a narrow spread, and a one standard deviation move being worth 2.02 percentage points of investment is a real-economy effect rather than a trading one, so I should not expect the cross-sectional volatility ranking on CSE counters to separate firms as cleanly as it does on a US sample."</t>
         </is>
       </c>
@@ -8285,7 +8285,7 @@
           <t>The paper has no liquidity variable, no turnover screen and no execution cost model, but it makes two liquidity-relevant concessions that I treat as primary evidence.
 First, the frequency concession, which I flagged as an important callout: "Weekly, not daily, and the paper says why in one sentence: 'since most stocks are not traded daily, we use weekly stock returns.' That is a finance journal on my exact market conceding the non-synchronous trading problem in the data section rather than the limitations section. Every frequency decision I make downstream has to answer to it."
 Second, the free-float consequence: "Mean institutional ownership of 66.1% against insider ownership of 5.7% is a free-float fact with a liquidity consequence. Two thirds of shares held by institutions means the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding. This is cheap to check on my own data and I should check it before setting the sweep range."
-Third, the untreated bias: "Weekly returns reduce the problem relative to daily but they do not eliminate it on a market where the paper itself says most stocks don't trade daily, and stale prices bias the residual standard deviation downward for exactly the thinnest counters. There is no Dimson or Scholes-Williams correction, no reported trading-frequency screen, and no check of whether the idiosyncratic risk measure correlates with turnover." The ±50% weekly return trim "is a sensible outlier rule and it is also a reminder of what the raw series looks like."</t>
+Third, the untreated bias: "Weekly returns reduce the problem relative to daily but they do not eliminate it on a market where the paper itself says most stocks don't trade daily, and stale prices bias the residual standard deviation downward for exactly the thinnest counters. There is no Dimson or Scholes-Williams correction, no reported trading-frequency screen, and no check of whether the idiosyncratic risk measure correlates with turnover." The ±50% weekly return trim is a sensible outlier rule and it is also a reminder of what the raw series looks like.</t>
         </is>
       </c>
       <c r="Q59" s="11" t="inlineStr">
@@ -8309,17 +8309,17 @@
       </c>
       <c r="T59" s="11" t="inlineStr">
         <is>
-          <t>- "The moderation results, which are the paper's contribution, rest on very few firms." 59 unique firms and 297 firm-years for insider tests, 54 firms and 278 for institutional tests, and after propensity score matching "64 and 76 observations respectively, all of this carrying firm fixed effects, year fixed effects and category dummies. At those sample sizes firm fixed effects consume a large share of the degrees of freedom and the matched-sample estimates in particular are being asked to do more than the data can support. The authors are not hiding any of this, the counts are in every table, but the write-up treats the matched results as confirmation when at 64 observations they are closer to a consistency check."
-- "The −0.703 correlation between insider and institutional ownership makes the 2×2 grid structurally unbalanced, and the insignificant cells are where that bites. Two variables correlating that strongly cannot produce four well-populated quadrants from 278 observations, so the high-insider-high-institutional cell is thin by construction, and every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one. The substitution story the paper tells could be right, but the evidence for it is one significant cell and three insignificant ones, and the design can't separate a genuine null from low power."
+          <t>- "The moderation results, which are the paper's contribution, rest on very few firms." 59 unique firms and 297 firm-years for insider tests, 54 firms and 278 for institutional tests, and after propensity score matching 64 and 76 observations respectively, all of this carrying firm fixed effects, year fixed effects and category dummies. At those sample sizes firm fixed effects consume a large share of the degrees of freedom and the matched-sample estimates in particular are being asked to do more than the data can support. The authors are not hiding any of this, the counts are in every table, but the write-up treats the matched results as confirmation when at 64 observations they are closer to a consistency check.
+- The −0.703 correlation between insider and institutional ownership makes the 2×2 "grid structurally unbalanced, and the insignificant cells are where that bites. Two variables correlating that strongly cannot produce four well-populated quadrants from 278 observations, so the high-insider-high-institutional cell is thin by construction, and every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one. The substitution story the paper tells could be right, but the evidence for it is one significant cell and three insignificant ones, and the design can't separate a genuine null from low power."
 - "Non-synchronous trading is handled by moving to weekly data and then not mentioned again… stale prices bias the residual standard deviation downward for exactly the thinnest counters. There is no Dimson or Scholes-Williams correction, no reported trading-frequency screen, and no check of whether the idiosyncratic risk measure correlates with turnover. That matters because firm size is a control and size correlates with liquidity, so part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant."
-- "The investment measure is a net quantity doing the work of a gross one. The change in net PPE nets out depreciation and disposals, so a firm that holds capex constant while an existing asset base ages records a falling investment rate, and a firm that sells a property records a negative one, which is why the minimum in Table 2 is −0.082. Capex is reported separately in Sri Lankan annual reports and the paper hand-collects everything else, so this is a choice rather than a constraint, inherited from Panousi and Papanikolaou for comparability, and it leaves the dependent variable noisier than the framing suggests."
+- "The investment measure is a net quantity doing the work of a gross one. The change in net PPE nets out depreciation and disposals, so a firm that holds capex constant while an existing asset base ages records a falling investment rate, and a firm that sells a property records a negative one, which is why the minimum in Table 2 is −0.082". Capex is reported separately in Sri Lankan annual reports and the paper hand-collects everything else, so this is a choice rather than a constraint, inherited from Panousi and Papanikolaou for comparability, and it leaves the dependent variable noisier than the framing suggests.
 - "Alignment against entrenchment is inferred from a sign pattern rather than tested. Nothing in the design observes managerial risk preference, wealth concentration or the project set, so the mechanism is read off the direction of an interaction coefficient… which is a reasonable inference and not a test. The authors say as much in their conclusion, where they note the underlying mechanisms warrant further exploration."
 - "The 2018 cutoff is well-argued and the extension quietly undercuts the argument for it. SLFRS 16 changing lease recognition in 2019 genuinely contaminates PPE, and that justifies the main sample. But the extended analysis to 2021 then runs straight through SLFRS 16, the Easter attacks and COVID with no adjustment to the PPE measure and no regime split, and reports the result as consistent, so the paper ends up both claiming the break is serious enough to truncate the sample and treating a sample that spans it as corroborating evidence."</t>
         </is>
       </c>
       <c r="U59" s="11" t="inlineStr">
         <is>
-          <t>- The citation for why A_T cannot assume a daily price series on CSE: a finance journal estimating a factor model on CSE firms moves to weekly because most stocks don't trade daily. "That is a stronger warrant than anything I could get from the ML literature."
+          <t>- The citation for why A_T cannot assume a daily price series on CSE: a finance journal estimating a factor model on CSE firms moves to weekly because most stocks don't trade daily. That is a stronger warrant than anything I could get from the ML literature.
 - The idiosyncratic risk estimator for A_V's cross-sectional input - residual standard deviation from a local factor model over a rolling window, with ASTRI as market proxy and the 91-day Treasury bill as risk-free - plus the explicit list of what I must add that they skip (non-synchronous trading correction, reported risk–turnover correlation).
 - A realistic prior on how much cross-sectional signal A_V can carry: mean idiosyncratic risk 0.221, standard deviation only 0.050, range 0.117 to 0.315.
 - A mechanism-level argument for volatility persistence that is independent of the statistical long-memory literature.
@@ -8340,16 +8340,16 @@
       </c>
       <c r="W59" s="11" t="inlineStr">
         <is>
-          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk–turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution."
+          <t>SPEAKS TO: All four agents, but asymmetrically. A_T (frequency and liquidity screening before any cross-sectional feature is computed), A_V (the idiosyncratic risk estimator and a prior on its cross-sectional spread), A_L (the free-float consequence for depth, and the risk–turnover collinearity question), and A_F (the extraction-cost constraint and the SLFRS 16 break). It also speaks directly to the orchestrator's conditioning design and to the abstention channel. The note's framing: "What makes it worth a full note rather than a paragraph is that it is the most careful treatment of CSE firm-level data I have found, and in the course of being careful it concedes three things about this market that my own design has to absorb: that" weekly returns are used because most CSE stocks are not traded daily, that usable ownership data exists for roughly a third of the firms that have usable accounting data, and that the headline relationship weakens substantially once the sample is extended through 2021. Those are constraints on the technical, volatility and fundamental channels respectively, stated by authors who had no reason to be making a point about data depth, which is exactly why I trust them more than I'd trust the same claim in a methods section arguing for its own contribution.
 EFFECT ON MAIN GAP: Strongly supportive on two fronts. First, regime instability: "The 2021 extension weakening the main coefficient from −0.232* to −0.123* is corroboration that CSE relationships estimated pre-2020 do not survive the crisis window intact. Taken with [[The Relationship between Macroeconomic Variables, Trading Volume and Stock Returns, Granger Causality Evidence from the Colombo Stock Exchange]] finding the traditional macro linkages broken over 2014 to 2022, that is now two independent CSE results pointing at regime instability across exactly the period a static system would be evaluated on, which is the clearest empirical case I have for an orchestrator that conditions on measured state rather than a fixed combination rule." Note the surviving coefficient is significant only at 10%.
-Second, the C_i,t component and abstention. The frequency concession forces an abstention design on A_T: "It doesn't mean I build at weekly frequency, the index track is liquid enough for daily, it means the per-counter liquidity screen has to come before any cross-sectional feature is computed and counters that fail it have to produce an abstention rather than a stale-price signal. This is the same structural failure [[AlphaAgents, Large Language Model Based Multi-Agents for Equity Portfolio Constructions]] fixed by deleting an agent by hand." And the data-depth fact forces the same on A_F: "it is why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence." Both of these are structural properties of the input and output, not self-reports, which is exactly what C_i,t is meant to be.
-Third, a methodological warning for the state vector itself: if the volatility estimate and the liquidity estimate co-move on my sample, "then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it." That is a concrete pre-registration task for the main gap, and the paper's own −0.703 insider/institutional correlation is the worked example of what unmanaged collinearity does to a conditioning design: "every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one."
-Fourth, Model 2's design is a usable template: "splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it is close to the structure I'd want for ablating state inputs one at a time."
+Second, the C_i,t component and abstention. The frequency concession forces an abstention design on A_T: "It doesn't mean I build at weekly frequency, the index track is liquid enough for daily, it means the per-counter liquidity screen has to come before any cross-sectional feature is computed and counters that fail it have to produce an abstention rather than a stale-price signal. This is the same structural failure [[AlphaAgents, Large Language Model Based Multi-Agents for Equity Portfolio Constructions]] fixed by deleting an agent by hand." And the data-depth fact forces the same on A_F: it is "why the fundamental agent is being designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence." Both of these are structural properties of the input and output, not self-reports, which is exactly what C_i,t is meant to be.
+Third, a methodological warning for the state vector itself: if the volatility estimate and the liquidity estimate co-move on my sample, then the volatility agent and the liquidity agent are partly measuring the same thing and the orchestrator's state vector has a collinearity problem I need to know about before I start weighting on it. That is a concrete pre-registration task for the main gap, and the paper's own −0.703 insider/institutional correlation is the worked example of what unmanaged collinearity does to a conditioning design: "every coefficient the paper reads as 'no effect' is in a cell that would struggle to detect one."
+Fourth, Model 2's design is a usable template: splitting at the median annually and reading the group-specific slope rather than a single interaction coefficient is a cleaner way of asking a conditioning question than a continuous interaction would be, and it "is close to the structure I'd want for ablating state inputs one at a time."
 EFFECT ON SUB-GAP 1: This is the strongest row in the note for state-dependent execution friction and for liquidity conditioning the reliability of price-derived agents. The reliability half is stated by the paper itself: "since most stocks are not traded daily, we use weekly stock returns" - a published finance journal on my exact market changing its estimation frequency because of thin trading. That is local empirical evidence that price-derived quantities on CSE degrade with liquidity, and it is the warrant for L_t conditioning A_T's and A_V's weights rather than being a separate add-on signal. The untreated residual is my opening: stale prices "bias the residual standard deviation downward for exactly the thinnest counters", with no Dimson or Scholes–Williams correction, no trading-frequency screen and no risk–turnover check anywhere in the paper, and "part of what the size coefficient absorbs may be measurement error in the risk variable rather than an investment determinant." The execution-cost half comes from the ownership structure: institutional ownership averaging 66.1% against insider 5.7% means "the tradeable float is a fraction of market capitalisation, so order size against available depth is worse than a capitalisation-based estimate would suggest, and the participation-rate sweep in the execution cost work needs to be calibrated against float rather than shares outstanding."
-EFFECT ON SUB-GAP 2: Supportive at the mechanism level, which is more than a statistical citation gives me. "The investment channel is the mechanism-level argument for pairing forecast variance with persistence rather than treating volatility as a point-in-time cap. If elevated idiosyncratic risk causes firms to cut capital spending by 17.48% of the mean investment rate, then a volatility shock on this market propagates into fundamentals with a lag measured in reporting periods, not days, and the real activity it suppresses takes just as long to come back. That is a fundamental reason to expect slow decay, independent of the statistical long-memory evidence in [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] and [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], and it is a better sentence for the proposal than another citation of a d estimate." The paper itself estimates no persistence parameter, so operationalising P_t remains entirely mine.
+EFFECT ON SUB-GAP 2: Supportive at the mechanism level, which is more than a statistical citation gives me. The investment channel is the mechanism-level argument for pairing forecast variance with persistence rather than treating volatility as a point-in-time cap. If elevated idiosyncratic risk causes firms to cut capital spending by 17.48% of the mean investment rate, then a volatility shock on this market propagates into fundamentals with a lag measured in reporting periods, not days, and the real activity it suppresses takes just as long to come back. That is a fundamental reason to expect slow decay, independent of the statistical long-memory evidence in [[The effect of COVID-19 on long memory in returns and volatility of cryptocurrency and stock markets]] and [[Modeling Long-Term Volatility Memory Dynamics in the Colombo Stock Exchange]], and it is a better sentence for the proposal than another citation of a d estimate. The paper itself estimates no persistence parameter, so operationalising P_t remains entirely mine.
 CSE DATA EVIDENCE: This is the single densest source of local empirical evidence I have for the justification rewrite, and the fact that it comes from authors with no stake in making a data-depth argument is what makes it usable.
 - Thin trading, conceded in the data section: "since most stocks are not traded daily, we use weekly stock returns." Three authors with institutional access, publishing in Managerial Finance, could not estimate a factor model at daily frequency on this market. That is direct local evidence of liquidity constraint, and it is stated as a design constraint rather than as a limitation.
-- Heterogeneous trading activity: the ±50% weekly return trim following Abeysekera and Nimal (2017) is itself "a reminder of what the raw series looks like" - a market where weekly moves beyond ±50% occur often enough to need a documented rule.
+- Heterogeneous trading activity: the ±50% weekly return trim following Abeysekera and Nimal (2017) is itself a reminder of what the raw series looks like - a market where weekly moves beyond ±50% occur often enough to need a documented rule.
 - Universe depth: 167 unique firms with usable accounting data, 1,226 firm-years over 2010–2018, after excluding financials, utilities, energy and telecoms, firm-years with missing variables, and negative book values. Ownership data available only from 2011 and only for 59 firms (insider) and 54 firms (institutional) - "usable ownership data exists for roughly a third of the firms that have usable accounting data". After propensity score matching, 64 and 76 observations.
 - Ownership concentration and free float: mean institutional ownership 66.1%, mean insider ownership 5.7%, correlating at −0.703. "This is a market of institutionally held firms with thin executive stakes." Two thirds of shares in institutional hands is a free-float constraint with a direct depth consequence.
 - Family control: family firms are 33% of firm-years, identified by hand from annual reports and executive biographies following Anderson and Reeb (2003).
@@ -8360,7 +8360,7 @@
 - Documented accounting break: SLFRS 16 changed lease recognition in 2019 and contaminates PPE - a structural break in CSE fundamentals sitting inside my 1 July 2014 to 30 June 2024 index track.
 - Fundamental extraction cost: all accounting figures, insider stakes, board composition, CEO duality and family-firm status were pulled out of CSE annual report PDFs by hand over nine years, by authors with institutional access and every incentive to keep the sample large.
 - Correct survivorship handling exists in the local literature: "Both listed and delisted firms are retained, which is a deliberate survivorship-bias control and more than most of the local literature does."
-PROPOSED REVISION STATED IN THE NOTE: (1) A per-counter liquidity screen must run before any cross-sectional feature is computed, and counters failing it must emit an abstention rather than a stale-price signal - A_T does not get to assume a daily series on this market. (2) A_V reuses this idiosyncratic risk construction (residual standard deviation from a local factor model over a rolling window, ASTRI market proxy, 91-day Treasury bill risk-free, with Abeysekera and Nimal (2017) as a four-factor local alternative) but adds the non-synchronous trading correction they skip and reports the correlation between the risk estimate and turnover, to establish whether A_V and A_L are partly measuring the same thing before any weighting is set on them. (3) The cross-sectional volatility ranking's expected separating power on CSE counters should be "pinned down on my own data before the agent's influence weight is allowed to swing much on it", given the 0.221/0.050 spread. (4) Any PPE-derived or lease-sensitive fundamental feature must either avoid the affected line items or carry an explicit SLFRS 16 break control, "with the choice stated in the methodology - I'd rather find this now than discover it in an ablation". (5) The execution-cost participation-rate sweep must be calibrated against free float rather than shares outstanding, and this is to be checked on my own data "before setting the sweep range". (6) A_F is designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence. (7) The volatility-persistence argument in the proposal is to be made at the mechanism level - investment suppression propagating through reporting periods - rather than by another citation of a long-memory d estimate.</t>
+PROPOSED REVISION STATED IN THE NOTE: (1) A per-counter liquidity screen must run before any cross-sectional feature is computed, and counters failing it must emit an abstention rather than a stale-price signal - A_T does not get to assume a daily series on this market. (2) A_V reuses this idiosyncratic risk construction (residual standard deviation from a local factor model over a rolling window, ASTRI market proxy, 91-day Treasury bill risk-free, with Abeysekera and Nimal (2017) as a four-factor local alternative) but adds the non-synchronous trading correction they skip and reports the correlation between the risk estimate and turnover, to establish whether A_V and A_L are partly measuring the same thing before any weighting is set on them. (3) The cross-sectional volatility ranking's expected separating power on CSE counters should be pinned down on my own data before the agent's influence weight is allowed to swing much on it, given the 0.221/0.050 spread. (4) Any PPE-derived or lease-sensitive fundamental feature must either avoid the affected line items or carry an explicit SLFRS 16 break control, with the choice stated in the methodology - I'd rather find this now than discover it in an ablation. (5) The execution-cost participation-rate sweep must be calibrated against free float rather than shares outstanding, and this is to be checked on my own data "before setting the sweep range". (6) A_F is designed for a channel that is frequently absent rather than occasionally imperfect, with abstention as the structural consequence. (7) The volatility-persistence argument in the proposal is to be made at the mechanism level - investment suppression propagating through reporting periods - rather than by another citation of a long-memory d estimate.</t>
         </is>
       </c>
       <c r="X59" s="11" t="inlineStr">
@@ -8454,7 +8454,7 @@
         <is>
           <t>What the paper did: news was scraped from a public economic-news blog with a pagination loop after the CSE's own announcement feed was found not rich enough to train a usable classifier, giving over 4,000 articles from 2012 to 2019. Labels were derived mechanically rather than annotated: each article was joined to the quantitative data by publication date under the assumption that news published on day t-1 moves the trend on day t, and inherited that next day's up or down label. Five classifiers were compared (Decision Tree, Naive Bayes, SVM, Random Forest, a simple ANN), tuned over CountVectorizer n-gram range, stop-word removal and TfidfTransformer settings, and Multinomial Naive Bayes was selected on 10-fold cross-validation accuracy of 0.95 (+/-0.02), tied with SVM at 0.95 (+/-0.03) against Decision Tree and Random Forest at 0.88. The text predictions then enter the weighted vote one term per article.
 My reading of that 0.95: it "is not evidence of predictive skill, and the hybrid result demonstrates that. Those labels were assigned mechanically from the next day's price direction, and 10-fold CV shuffles articles that are temporally adjacent and frequently cover the same event, so articles sharing a day share a label and overlapping vocabulary and the classifier can recover the day rather than the direction. The test that matters is the one the paper itself runs: a component scoring 0.95 in isolation contributes about four accuracy points to a joint decision in which it holds most of the weight. Those two numbers cannot both be measuring the same thing."
-Scope statement: this component is out of scope for my project. The sentiment agent was removed from my architecture by the supervisor's scope decision (see [[Scope sentiment analysis dropped]]), and my note states the consequence directly: "the only reading available to me since sentiment is out of scope and the text half is not something I'll rebuild." This row is retained in the matrix as evidence about the CSE and about fixed-weight combination, not as a design input. Per the scope rules the text channel is cited as a fixed-influence failure case, not as a component to rebuild.</t>
+Scope statement: this component is out of scope for my project. The sentiment agent was removed from my architecture by the supervisor's scope decision (see [[Scope sentiment analysis dropped]]), and my note states the consequence directly: "the only reading available to me since sentiment is out of scope" and the text half is not something I'll rebuild. This row is retained in the matrix as evidence about the CSE and about fixed-weight combination, not as a design input. Per the scope rules the text channel is cited as a fixed-influence failure case, not as a component to rebuild.</t>
         </is>
       </c>
       <c r="N60" s="11" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="T60" s="11" t="inlineStr">
         <is>
-          <t>- The weights were selected on the data the result is reported on. Table IV is headed as a holdout measurement and reports both the equal-weight and finalised instances on it, and the finalised ratio was found by changing the weights until performance was at its best. There is no third partition separating weight selection from reporting, so 0.5837 is an in-sample figure for the one parameter the paper's contribution turns on. "The 54% to 58% improvement is therefore not independently evidenced, and with the walk-forward machinery already built, holding out a separate window for the combination step would have cost very little."
+          <t>- The weights were selected on the data the result is reported on. Table IV is headed as a holdout measurement and reports both the equal-weight and finalised instances on it, and the finalised ratio was found by changing the weights until performance was at its best. There is no third partition separating weight selection from reporting, so 0.5837 is an in-sample figure for the one parameter the paper's contribution turns on. "The 54% to 58% improvement is therefore not independently evidenced", and with the walk-forward machinery already built, holding out a separate window for the combination step would have cost very little.
 - The disrupted-data problem that motivates the paper is never handled in the methodology. Non-trading days on thin counters are named in the abstract as the reason a CSE-specific model is needed, then treated only by a general statement that missing values were handled. On a lookback of four days the choice between dropping, forward-filling and zero-filling changes what the window contains. AGAL is the counter most likely to have gaps, "which makes the omission load-bearing rather than cosmetic."
 - No baseline of any kind, and no backtest. Majority-class rate and persistence are not computed and class balance is not reported. No position, fee, spread or return, so the claim that at 58% accuracy "the users will always receive an overall gain" does not follow.
 - Three counters, one of them trained differently, and no liquidity screen. JKH, CTC and AGAL described as powerful counters with no stated selection criterion. CTC was trained unnormalised with a different parameter set, "so cross-counter comparison is not available even in principle, and the trend-classification result in Table IV is reported as a single number without saying which counter or counters produced it."
@@ -8552,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A73"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="142" customWidth="1" min="1" max="1"/>
@@ -8982,6 +8982,20 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="15" t="inlineStr">
+        <is>
+          <t>Amendment, 18 October 2026 (sixth)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>Provenance pass, completing the quoted-fragment audit begun in the fifth amendment. Every quoted span in the sheet was matched word by word against the literature review note its row links, ignoring case, punctuation and the LaTeX-against-Unicode difference. A span that did not appear in its note was repaired by one of three mechanical rules, never by rewriting: where a run of at least eight words at the END of the span was verbatim in the note, the OPENING quotation mark was moved forward to the start of that run, so my own lead-in prose is no longer presented as the note speaking; where a run at the START was verbatim, the CLOSING mark was moved back; and where neither held, both marks were removed, leaving the text exactly as it was but no longer attributed. Matching was done on whole words so a boundary can never fall inside one, and a move was refused when it would have opened a quotation on a conjunction or preposition, those being unquoted instead. RESULT: 79 opening marks moved, 95 closing marks moved, 101 spans unquoted, across 175 cells and then 4 more on a second pass to convergence. Every one of the 1,621 quoted spans now in the sheet is verbatim in the note it is drawn from, and the scan reports nothing outstanding. VERIFICATION: the sheet was diffed against its pre-pass state. Across all 59 rows the only words that left the sheet are the six deliberate factual corrections listed below; the pass itself removed 202 quotation marks and not one word. Spacing before punctuation fell from 72 occurrences to 32 and doubled spaces from 37 to 28, so the pass left the text cleaner rather than scarred. Quote parity is even in every cell, no cell is empty, and the autofilter, freeze pane and the P54 amber fill are untouched. TWO FURTHER FACTUAL CORRECTIONS surfaced while doing it. (1) P01 described the framework as seven specialised roles; the note says eleven agents across seven specialised role types, and the cell now matches. (2) P57 carried a SECOND instance of the 113% turnover error, in Research Stream, which the fifth amendment had not caught; it is now 114% in both places. WHAT THIS PASS DELIBERATELY DID NOT DO: it did not make any paraphrase verbatim and it did not check whether an unquoted span is a fair restatement of the note. It establishes only that nothing in quotation marks is now claiming to be the note when it is not.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>